<commit_message>
docs(tracker): EAS config, soak harness, and the soak-passed milestone
Four deliverables and two risk rows. E10 Deploy 33% -> 36%; overall 111
deliverables, 74 done (67%).

Both new risks are decisions worth surfacing rather than burying in a commit:
the Android package name is permanent after the first Play Store release, and
push notifications still cannot be verified on a device at all until eas init
mints a projectId.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B54301F9-5789-4363-B4A5-43F65F7EDD28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0BFDA97-4E01-4326-B1D4-104F1579AFED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14895" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="415">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -807,6 +807,30 @@
   </si>
   <si>
     <t>PICK-07. Unblocks notify_kickoff_reminder, a stub since it was written</t>
+  </si>
+  <si>
+    <t>EAS build profiles + bundle identifiers</t>
+  </si>
+  <si>
+    <t>iOS id was absent entirely; Android was Expo's com.anonymous default</t>
+  </si>
+  <si>
+    <t>Staging soak harness (infra/soak-compose.yml)</t>
+  </si>
+  <si>
+    <t>Same image, 3 roles, throwaway PG/Redis, isolated from the dev stack</t>
+  </si>
+  <si>
+    <t>SOAK PASSED: full stack from empty DB</t>
+  </si>
+  <si>
+    <t>Migrations, 5 services, API 200s, beat-&gt;worker chain, model loaded from a filename row</t>
+  </si>
+  <si>
+    <t>Run eas login + eas init (needs Expo account)</t>
+  </si>
+  <si>
+    <t>Writes extra.eas.projectId. Blocks minting ANY push token - see mobile/EAS-SETUP.md</t>
   </si>
   <si>
     <t>Legend</t>
@@ -1317,6 +1341,18 @@
   </si>
   <si>
     <t>An estimated kickoff is a DATE not a time, so a T-60 reminder off a midnight placeholder would be false. Skipped rather than sent wrong. Affects most ATP fixtures until BallDontLie publishes real times - only ~2% carry one.</t>
+  </si>
+  <si>
+    <t>Android package name is permanent after release</t>
+  </si>
+  <si>
+    <t>Set to com.sportiq.app, replacing Expo's com.anonymous.sportiq scaffold default. Free to change now; after the first Play Store release it means a new listing and losing installs. Decide before submitting, especially if a different domain should be used in reverse-DNS form.</t>
+  </si>
+  <si>
+    <t>Push notifications remain unverifiable on device</t>
+  </si>
+  <si>
+    <t>getExpoPushTokenAsync needs a real projectId, which only eas init can create. The backend side (PUT /user/push-token, _send_push) is real and tested; nothing has ever been delivered to a device. Compounded on Android by Expo Go dropping remote push in SDK 53, so a development build is required.</t>
   </si>
 </sst>
 </file>
@@ -1326,7 +1362,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\ mmm"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1475,8 +1511,30 @@
       <color rgb="FF6B7280"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF111827"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF111827"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF6B7280"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="25">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1573,8 +1631,33 @@
         <fgColor rgb="FF94A3B8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF16A34A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB45309"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF94A3B8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -1675,11 +1758,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1863,6 +1961,66 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="21" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="20" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="22" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="23" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="24" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2256,7 +2414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R113"/>
+  <dimension ref="A1:R117"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2270,46 +2428,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
-      <c r="P1" s="64"/>
-      <c r="Q1" s="65"/>
+      <c r="B1" s="84"/>
+      <c r="C1" s="84"/>
+      <c r="D1" s="84"/>
+      <c r="E1" s="84"/>
+      <c r="F1" s="84"/>
+      <c r="G1" s="84"/>
+      <c r="H1" s="84"/>
+      <c r="I1" s="84"/>
+      <c r="J1" s="84"/>
+      <c r="K1" s="84"/>
+      <c r="L1" s="84"/>
+      <c r="M1" s="84"/>
+      <c r="N1" s="84"/>
+      <c r="O1" s="84"/>
+      <c r="P1" s="84"/>
+      <c r="Q1" s="85"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="83" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="64"/>
-      <c r="M2" s="64"/>
-      <c r="N2" s="64"/>
-      <c r="O2" s="64"/>
-      <c r="P2" s="64"/>
-      <c r="Q2" s="65"/>
+      <c r="B2" s="84"/>
+      <c r="C2" s="84"/>
+      <c r="D2" s="84"/>
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="84"/>
+      <c r="H2" s="84"/>
+      <c r="I2" s="84"/>
+      <c r="J2" s="84"/>
+      <c r="K2" s="84"/>
+      <c r="L2" s="84"/>
+      <c r="M2" s="84"/>
+      <c r="N2" s="84"/>
+      <c r="O2" s="84"/>
+      <c r="P2" s="84"/>
+      <c r="Q2" s="85"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
@@ -5863,7 +6021,7 @@
       <c r="P102" s="11"/>
       <c r="Q102" s="11"/>
       <c r="R102" t="str">
-        <f t="shared" ref="R102:R111" si="3">IF($A102&lt;&gt;"",$A102,R101)</f>
+        <f t="shared" ref="R102:R115" si="3">IF($A102&lt;&gt;"",$A102,R101)</f>
         <v>E9 Data Ops</v>
       </c>
     </row>
@@ -6200,23 +6358,171 @@
         <v>E10 Deploy</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A113" s="25" t="s">
+    <row r="112" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A112" s="63" t="s">
+        <v>162</v>
+      </c>
+      <c r="B112" s="64" t="s">
         <v>257</v>
       </c>
-      <c r="B113" s="5" t="s">
+      <c r="C112" s="65" t="s">
         <v>22</v>
       </c>
-      <c r="C113" s="17" t="s">
+      <c r="D112" s="66" t="s">
+        <v>85</v>
+      </c>
+      <c r="E112" s="67">
+        <v>46238</v>
+      </c>
+      <c r="F112" s="67">
+        <v>46238</v>
+      </c>
+      <c r="G112" s="68" t="s">
+        <v>258</v>
+      </c>
+      <c r="H112" s="64"/>
+      <c r="I112" s="69"/>
+      <c r="J112" s="64"/>
+      <c r="K112" s="64"/>
+      <c r="L112" s="64"/>
+      <c r="M112" s="64"/>
+      <c r="N112" s="64"/>
+      <c r="O112" s="64"/>
+      <c r="P112" s="64"/>
+      <c r="Q112" s="64"/>
+      <c r="R112" t="str">
+        <f t="shared" si="3"/>
+        <v>E10 Deploy</v>
+      </c>
+    </row>
+    <row r="113" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A113" s="70" t="s">
+        <v>162</v>
+      </c>
+      <c r="B113" s="71" t="s">
+        <v>259</v>
+      </c>
+      <c r="C113" s="65" t="s">
+        <v>22</v>
+      </c>
+      <c r="D113" s="72" t="s">
+        <v>23</v>
+      </c>
+      <c r="E113" s="73">
+        <v>46238</v>
+      </c>
+      <c r="F113" s="73">
+        <v>46238</v>
+      </c>
+      <c r="G113" s="74" t="s">
+        <v>260</v>
+      </c>
+      <c r="H113" s="71"/>
+      <c r="I113" s="69"/>
+      <c r="J113" s="71"/>
+      <c r="K113" s="71"/>
+      <c r="L113" s="71"/>
+      <c r="M113" s="71"/>
+      <c r="N113" s="71"/>
+      <c r="O113" s="71"/>
+      <c r="P113" s="71"/>
+      <c r="Q113" s="71"/>
+      <c r="R113" t="str">
+        <f t="shared" si="3"/>
+        <v>E10 Deploy</v>
+      </c>
+    </row>
+    <row r="114" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A114" s="63" t="s">
+        <v>162</v>
+      </c>
+      <c r="B114" s="64" t="s">
+        <v>261</v>
+      </c>
+      <c r="C114" s="75" t="s">
+        <v>136</v>
+      </c>
+      <c r="D114" s="66" t="s">
+        <v>23</v>
+      </c>
+      <c r="E114" s="67">
+        <v>46238</v>
+      </c>
+      <c r="F114" s="67">
+        <v>46238</v>
+      </c>
+      <c r="G114" s="68" t="s">
+        <v>262</v>
+      </c>
+      <c r="H114" s="64"/>
+      <c r="I114" s="76"/>
+      <c r="J114" s="64"/>
+      <c r="K114" s="64"/>
+      <c r="L114" s="64"/>
+      <c r="M114" s="64"/>
+      <c r="N114" s="64"/>
+      <c r="O114" s="64"/>
+      <c r="P114" s="64"/>
+      <c r="Q114" s="64"/>
+      <c r="R114" t="str">
+        <f t="shared" si="3"/>
+        <v>E10 Deploy</v>
+      </c>
+    </row>
+    <row r="115" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A115" s="70" t="s">
+        <v>162</v>
+      </c>
+      <c r="B115" s="71" t="s">
+        <v>263</v>
+      </c>
+      <c r="C115" s="77" t="s">
+        <v>128</v>
+      </c>
+      <c r="D115" s="72" t="s">
+        <v>85</v>
+      </c>
+      <c r="E115" s="73">
+        <v>46239</v>
+      </c>
+      <c r="F115" s="73">
+        <v>46239</v>
+      </c>
+      <c r="G115" s="74" t="s">
+        <v>264</v>
+      </c>
+      <c r="H115" s="71"/>
+      <c r="I115" s="78"/>
+      <c r="J115" s="71"/>
+      <c r="K115" s="71"/>
+      <c r="L115" s="71"/>
+      <c r="M115" s="71"/>
+      <c r="N115" s="71"/>
+      <c r="O115" s="71"/>
+      <c r="P115" s="71"/>
+      <c r="Q115" s="71"/>
+      <c r="R115" t="str">
+        <f t="shared" si="3"/>
+        <v>E10 Deploy</v>
+      </c>
+    </row>
+    <row r="117" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A117" s="25" t="s">
+        <v>265</v>
+      </c>
+      <c r="B117" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C117" s="17" t="s">
         <v>231</v>
       </c>
-      <c r="D113" s="19" t="s">
+      <c r="D117" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="E113" s="23" t="s">
+      <c r="E117" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="F113" s="21" t="s">
+      <c r="F117" s="21" t="s">
         <v>136</v>
       </c>
     </row>
@@ -6240,852 +6546,852 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="82" t="s">
-        <v>258</v>
-      </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
-      <c r="J1" s="72"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="72"/>
-      <c r="P1" s="72"/>
-      <c r="Q1" s="72"/>
-      <c r="R1" s="72"/>
-      <c r="S1" s="72"/>
+      <c r="A1" s="102" t="s">
+        <v>266</v>
+      </c>
+      <c r="B1" s="92"/>
+      <c r="C1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="92"/>
+      <c r="H1" s="92"/>
+      <c r="I1" s="92"/>
+      <c r="J1" s="92"/>
+      <c r="K1" s="92"/>
+      <c r="L1" s="92"/>
+      <c r="M1" s="92"/>
+      <c r="N1" s="92"/>
+      <c r="O1" s="92"/>
+      <c r="P1" s="92"/>
+      <c r="Q1" s="92"/>
+      <c r="R1" s="92"/>
+      <c r="S1" s="92"/>
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="89" t="s">
-        <v>259</v>
-      </c>
-      <c r="B2" s="72"/>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="72"/>
-      <c r="L2" s="72"/>
-      <c r="M2" s="72"/>
-      <c r="N2" s="72"/>
-      <c r="O2" s="72"/>
-      <c r="P2" s="72"/>
-      <c r="Q2" s="72"/>
-      <c r="R2" s="72"/>
-      <c r="S2" s="72"/>
+      <c r="A2" s="109" t="s">
+        <v>267</v>
+      </c>
+      <c r="B2" s="92"/>
+      <c r="C2" s="92"/>
+      <c r="D2" s="92"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="92"/>
+      <c r="H2" s="92"/>
+      <c r="I2" s="92"/>
+      <c r="J2" s="92"/>
+      <c r="K2" s="92"/>
+      <c r="L2" s="92"/>
+      <c r="M2" s="92"/>
+      <c r="N2" s="92"/>
+      <c r="O2" s="92"/>
+      <c r="P2" s="92"/>
+      <c r="Q2" s="92"/>
+      <c r="R2" s="92"/>
+      <c r="S2" s="92"/>
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="77" t="s">
-        <v>260</v>
-      </c>
-      <c r="B4" s="72"/>
-      <c r="C4" s="72"/>
-      <c r="D4" s="72"/>
-      <c r="E4" s="72"/>
-      <c r="F4" s="72"/>
-      <c r="G4" s="72"/>
-      <c r="H4" s="72"/>
-      <c r="I4" s="72"/>
-      <c r="J4" s="72"/>
-      <c r="K4" s="72"/>
-      <c r="L4" s="72"/>
-      <c r="M4" s="72"/>
-      <c r="N4" s="72"/>
-      <c r="O4" s="72"/>
-      <c r="P4" s="72"/>
-      <c r="Q4" s="72"/>
-      <c r="R4" s="72"/>
-      <c r="S4" s="72"/>
+      <c r="A4" s="97" t="s">
+        <v>268</v>
+      </c>
+      <c r="B4" s="92"/>
+      <c r="C4" s="92"/>
+      <c r="D4" s="92"/>
+      <c r="E4" s="92"/>
+      <c r="F4" s="92"/>
+      <c r="G4" s="92"/>
+      <c r="H4" s="92"/>
+      <c r="I4" s="92"/>
+      <c r="J4" s="92"/>
+      <c r="K4" s="92"/>
+      <c r="L4" s="92"/>
+      <c r="M4" s="92"/>
+      <c r="N4" s="92"/>
+      <c r="O4" s="92"/>
+      <c r="P4" s="92"/>
+      <c r="Q4" s="92"/>
+      <c r="R4" s="92"/>
+      <c r="S4" s="92"/>
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="37" t="s">
-        <v>261</v>
-      </c>
-      <c r="B5" s="67" t="s">
-        <v>262</v>
-      </c>
-      <c r="C5" s="68"/>
-      <c r="D5" s="69"/>
-      <c r="E5" s="70" t="s">
-        <v>263</v>
-      </c>
-      <c r="F5" s="68"/>
-      <c r="G5" s="69"/>
-      <c r="H5" s="70" t="s">
-        <v>264</v>
-      </c>
-      <c r="I5" s="68"/>
-      <c r="J5" s="69"/>
-      <c r="K5" s="67" t="s">
-        <v>265</v>
-      </c>
-      <c r="L5" s="68"/>
-      <c r="M5" s="69"/>
-      <c r="N5" s="74" t="s">
-        <v>266</v>
-      </c>
-      <c r="O5" s="68"/>
-      <c r="P5" s="69"/>
-      <c r="Q5" s="74" t="s">
-        <v>267</v>
-      </c>
-      <c r="R5" s="68"/>
-      <c r="S5" s="69"/>
+        <v>269</v>
+      </c>
+      <c r="B5" s="87" t="s">
+        <v>270</v>
+      </c>
+      <c r="C5" s="88"/>
+      <c r="D5" s="89"/>
+      <c r="E5" s="90" t="s">
+        <v>271</v>
+      </c>
+      <c r="F5" s="88"/>
+      <c r="G5" s="89"/>
+      <c r="H5" s="90" t="s">
+        <v>272</v>
+      </c>
+      <c r="I5" s="88"/>
+      <c r="J5" s="89"/>
+      <c r="K5" s="87" t="s">
+        <v>273</v>
+      </c>
+      <c r="L5" s="88"/>
+      <c r="M5" s="89"/>
+      <c r="N5" s="94" t="s">
+        <v>274</v>
+      </c>
+      <c r="O5" s="88"/>
+      <c r="P5" s="89"/>
+      <c r="Q5" s="94" t="s">
+        <v>275</v>
+      </c>
+      <c r="R5" s="88"/>
+      <c r="S5" s="89"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="71" t="s">
-        <v>268</v>
-      </c>
-      <c r="C6" s="72"/>
-      <c r="D6" s="72"/>
-      <c r="E6" s="72"/>
-      <c r="F6" s="72"/>
-      <c r="G6" s="72"/>
-      <c r="H6" s="72"/>
-      <c r="I6" s="72"/>
-      <c r="J6" s="72"/>
-      <c r="K6" s="72"/>
-      <c r="L6" s="72"/>
-      <c r="M6" s="72"/>
-      <c r="N6" s="72"/>
-      <c r="O6" s="72"/>
-      <c r="P6" s="72"/>
-      <c r="Q6" s="72"/>
-      <c r="R6" s="72"/>
-      <c r="S6" s="72"/>
+      <c r="B6" s="91" t="s">
+        <v>276</v>
+      </c>
+      <c r="C6" s="92"/>
+      <c r="D6" s="92"/>
+      <c r="E6" s="92"/>
+      <c r="F6" s="92"/>
+      <c r="G6" s="92"/>
+      <c r="H6" s="92"/>
+      <c r="I6" s="92"/>
+      <c r="J6" s="92"/>
+      <c r="K6" s="92"/>
+      <c r="L6" s="92"/>
+      <c r="M6" s="92"/>
+      <c r="N6" s="92"/>
+      <c r="O6" s="92"/>
+      <c r="P6" s="92"/>
+      <c r="Q6" s="92"/>
+      <c r="R6" s="92"/>
+      <c r="S6" s="92"/>
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="77" t="s">
-        <v>269</v>
-      </c>
-      <c r="B7" s="72"/>
-      <c r="C7" s="72"/>
-      <c r="D7" s="72"/>
-      <c r="E7" s="72"/>
-      <c r="F7" s="72"/>
-      <c r="G7" s="72"/>
-      <c r="H7" s="72"/>
-      <c r="I7" s="72"/>
-      <c r="J7" s="72"/>
-      <c r="K7" s="72"/>
-      <c r="L7" s="72"/>
-      <c r="M7" s="72"/>
-      <c r="N7" s="72"/>
-      <c r="O7" s="72"/>
-      <c r="P7" s="72"/>
-      <c r="Q7" s="72"/>
-      <c r="R7" s="72"/>
-      <c r="S7" s="72"/>
+      <c r="A7" s="97" t="s">
+        <v>277</v>
+      </c>
+      <c r="B7" s="92"/>
+      <c r="C7" s="92"/>
+      <c r="D7" s="92"/>
+      <c r="E7" s="92"/>
+      <c r="F7" s="92"/>
+      <c r="G7" s="92"/>
+      <c r="H7" s="92"/>
+      <c r="I7" s="92"/>
+      <c r="J7" s="92"/>
+      <c r="K7" s="92"/>
+      <c r="L7" s="92"/>
+      <c r="M7" s="92"/>
+      <c r="N7" s="92"/>
+      <c r="O7" s="92"/>
+      <c r="P7" s="92"/>
+      <c r="Q7" s="92"/>
+      <c r="R7" s="92"/>
+      <c r="S7" s="92"/>
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="37" t="s">
-        <v>270</v>
-      </c>
-      <c r="B8" s="80" t="s">
-        <v>271</v>
-      </c>
-      <c r="C8" s="68"/>
-      <c r="D8" s="68"/>
-      <c r="E8" s="68"/>
-      <c r="F8" s="68"/>
-      <c r="G8" s="68"/>
-      <c r="H8" s="68"/>
-      <c r="I8" s="68"/>
-      <c r="J8" s="69"/>
-      <c r="K8" s="80" t="s">
-        <v>272</v>
-      </c>
-      <c r="L8" s="68"/>
-      <c r="M8" s="68"/>
-      <c r="N8" s="68"/>
-      <c r="O8" s="68"/>
-      <c r="P8" s="68"/>
-      <c r="Q8" s="68"/>
-      <c r="R8" s="68"/>
-      <c r="S8" s="69"/>
+        <v>278</v>
+      </c>
+      <c r="B8" s="100" t="s">
+        <v>279</v>
+      </c>
+      <c r="C8" s="88"/>
+      <c r="D8" s="88"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="88"/>
+      <c r="H8" s="88"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="89"/>
+      <c r="K8" s="100" t="s">
+        <v>280</v>
+      </c>
+      <c r="L8" s="88"/>
+      <c r="M8" s="88"/>
+      <c r="N8" s="88"/>
+      <c r="O8" s="88"/>
+      <c r="P8" s="88"/>
+      <c r="Q8" s="88"/>
+      <c r="R8" s="88"/>
+      <c r="S8" s="89"/>
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B9" s="71" t="s">
-        <v>268</v>
-      </c>
-      <c r="C9" s="72"/>
-      <c r="D9" s="72"/>
-      <c r="E9" s="72"/>
-      <c r="F9" s="72"/>
-      <c r="G9" s="72"/>
-      <c r="H9" s="72"/>
-      <c r="I9" s="72"/>
-      <c r="J9" s="72"/>
-      <c r="K9" s="72"/>
-      <c r="L9" s="72"/>
-      <c r="M9" s="72"/>
-      <c r="N9" s="72"/>
-      <c r="O9" s="72"/>
-      <c r="P9" s="72"/>
-      <c r="Q9" s="72"/>
-      <c r="R9" s="72"/>
-      <c r="S9" s="72"/>
+      <c r="B9" s="91" t="s">
+        <v>276</v>
+      </c>
+      <c r="C9" s="92"/>
+      <c r="D9" s="92"/>
+      <c r="E9" s="92"/>
+      <c r="F9" s="92"/>
+      <c r="G9" s="92"/>
+      <c r="H9" s="92"/>
+      <c r="I9" s="92"/>
+      <c r="J9" s="92"/>
+      <c r="K9" s="92"/>
+      <c r="L9" s="92"/>
+      <c r="M9" s="92"/>
+      <c r="N9" s="92"/>
+      <c r="O9" s="92"/>
+      <c r="P9" s="92"/>
+      <c r="Q9" s="92"/>
+      <c r="R9" s="92"/>
+      <c r="S9" s="92"/>
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="77" t="s">
-        <v>273</v>
-      </c>
-      <c r="B10" s="72"/>
-      <c r="C10" s="72"/>
-      <c r="D10" s="72"/>
-      <c r="E10" s="72"/>
-      <c r="F10" s="72"/>
-      <c r="G10" s="72"/>
-      <c r="H10" s="72"/>
-      <c r="I10" s="72"/>
-      <c r="J10" s="72"/>
-      <c r="K10" s="72"/>
-      <c r="L10" s="72"/>
-      <c r="M10" s="72"/>
-      <c r="N10" s="72"/>
-      <c r="O10" s="72"/>
-      <c r="P10" s="72"/>
-      <c r="Q10" s="72"/>
-      <c r="R10" s="72"/>
-      <c r="S10" s="72"/>
+      <c r="A10" s="97" t="s">
+        <v>281</v>
+      </c>
+      <c r="B10" s="92"/>
+      <c r="C10" s="92"/>
+      <c r="D10" s="92"/>
+      <c r="E10" s="92"/>
+      <c r="F10" s="92"/>
+      <c r="G10" s="92"/>
+      <c r="H10" s="92"/>
+      <c r="I10" s="92"/>
+      <c r="J10" s="92"/>
+      <c r="K10" s="92"/>
+      <c r="L10" s="92"/>
+      <c r="M10" s="92"/>
+      <c r="N10" s="92"/>
+      <c r="O10" s="92"/>
+      <c r="P10" s="92"/>
+      <c r="Q10" s="92"/>
+      <c r="R10" s="92"/>
+      <c r="S10" s="92"/>
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="37" t="s">
-        <v>274</v>
-      </c>
-      <c r="B11" s="67" t="s">
-        <v>275</v>
-      </c>
-      <c r="C11" s="68"/>
-      <c r="D11" s="69"/>
-      <c r="E11" s="67" t="s">
+        <v>282</v>
+      </c>
+      <c r="B11" s="87" t="s">
+        <v>283</v>
+      </c>
+      <c r="C11" s="88"/>
+      <c r="D11" s="89"/>
+      <c r="E11" s="87" t="s">
+        <v>284</v>
+      </c>
+      <c r="F11" s="88"/>
+      <c r="G11" s="89"/>
+      <c r="H11" s="87" t="s">
+        <v>285</v>
+      </c>
+      <c r="I11" s="88"/>
+      <c r="J11" s="89"/>
+      <c r="K11" s="90" t="s">
+        <v>286</v>
+      </c>
+      <c r="L11" s="88"/>
+      <c r="M11" s="89"/>
+      <c r="N11" s="87" t="s">
+        <v>287</v>
+      </c>
+      <c r="O11" s="88"/>
+      <c r="P11" s="89"/>
+      <c r="Q11" s="87" t="s">
+        <v>288</v>
+      </c>
+      <c r="R11" s="88"/>
+      <c r="S11" s="89"/>
+    </row>
+    <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B12" s="91" t="s">
         <v>276</v>
       </c>
-      <c r="F11" s="68"/>
-      <c r="G11" s="69"/>
-      <c r="H11" s="67" t="s">
-        <v>277</v>
-      </c>
-      <c r="I11" s="68"/>
-      <c r="J11" s="69"/>
-      <c r="K11" s="70" t="s">
-        <v>278</v>
-      </c>
-      <c r="L11" s="68"/>
-      <c r="M11" s="69"/>
-      <c r="N11" s="67" t="s">
-        <v>279</v>
-      </c>
-      <c r="O11" s="68"/>
-      <c r="P11" s="69"/>
-      <c r="Q11" s="67" t="s">
-        <v>280</v>
-      </c>
-      <c r="R11" s="68"/>
-      <c r="S11" s="69"/>
-    </row>
-    <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B12" s="71" t="s">
-        <v>268</v>
-      </c>
-      <c r="C12" s="72"/>
-      <c r="D12" s="72"/>
-      <c r="E12" s="72"/>
-      <c r="F12" s="72"/>
-      <c r="G12" s="72"/>
-      <c r="H12" s="72"/>
-      <c r="I12" s="72"/>
-      <c r="J12" s="72"/>
-      <c r="K12" s="72"/>
-      <c r="L12" s="72"/>
-      <c r="M12" s="72"/>
-      <c r="N12" s="72"/>
-      <c r="O12" s="72"/>
-      <c r="P12" s="72"/>
-      <c r="Q12" s="72"/>
-      <c r="R12" s="72"/>
-      <c r="S12" s="72"/>
+      <c r="C12" s="92"/>
+      <c r="D12" s="92"/>
+      <c r="E12" s="92"/>
+      <c r="F12" s="92"/>
+      <c r="G12" s="92"/>
+      <c r="H12" s="92"/>
+      <c r="I12" s="92"/>
+      <c r="J12" s="92"/>
+      <c r="K12" s="92"/>
+      <c r="L12" s="92"/>
+      <c r="M12" s="92"/>
+      <c r="N12" s="92"/>
+      <c r="O12" s="92"/>
+      <c r="P12" s="92"/>
+      <c r="Q12" s="92"/>
+      <c r="R12" s="92"/>
+      <c r="S12" s="92"/>
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="77" t="s">
-        <v>281</v>
-      </c>
-      <c r="B13" s="72"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="72"/>
-      <c r="F13" s="72"/>
-      <c r="G13" s="72"/>
-      <c r="H13" s="72"/>
-      <c r="I13" s="72"/>
-      <c r="J13" s="72"/>
-      <c r="K13" s="72"/>
-      <c r="L13" s="72"/>
-      <c r="M13" s="72"/>
-      <c r="N13" s="72"/>
-      <c r="O13" s="72"/>
-      <c r="P13" s="72"/>
-      <c r="Q13" s="72"/>
-      <c r="R13" s="72"/>
-      <c r="S13" s="72"/>
+      <c r="A13" s="97" t="s">
+        <v>289</v>
+      </c>
+      <c r="B13" s="92"/>
+      <c r="C13" s="92"/>
+      <c r="D13" s="92"/>
+      <c r="E13" s="92"/>
+      <c r="F13" s="92"/>
+      <c r="G13" s="92"/>
+      <c r="H13" s="92"/>
+      <c r="I13" s="92"/>
+      <c r="J13" s="92"/>
+      <c r="K13" s="92"/>
+      <c r="L13" s="92"/>
+      <c r="M13" s="92"/>
+      <c r="N13" s="92"/>
+      <c r="O13" s="92"/>
+      <c r="P13" s="92"/>
+      <c r="Q13" s="92"/>
+      <c r="R13" s="92"/>
+      <c r="S13" s="92"/>
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="37" t="s">
-        <v>282</v>
-      </c>
-      <c r="B14" s="75" t="s">
-        <v>283</v>
-      </c>
-      <c r="C14" s="68"/>
-      <c r="D14" s="68"/>
-      <c r="E14" s="68"/>
-      <c r="F14" s="68"/>
-      <c r="G14" s="69"/>
-      <c r="H14" s="75" t="s">
-        <v>284</v>
-      </c>
-      <c r="I14" s="68"/>
-      <c r="J14" s="68"/>
-      <c r="K14" s="68"/>
-      <c r="L14" s="68"/>
-      <c r="M14" s="69"/>
-      <c r="N14" s="75" t="s">
-        <v>285</v>
-      </c>
-      <c r="O14" s="68"/>
-      <c r="P14" s="69"/>
-      <c r="Q14" s="70" t="s">
-        <v>286</v>
-      </c>
-      <c r="R14" s="68"/>
-      <c r="S14" s="69"/>
+        <v>290</v>
+      </c>
+      <c r="B14" s="95" t="s">
+        <v>291</v>
+      </c>
+      <c r="C14" s="88"/>
+      <c r="D14" s="88"/>
+      <c r="E14" s="88"/>
+      <c r="F14" s="88"/>
+      <c r="G14" s="89"/>
+      <c r="H14" s="95" t="s">
+        <v>292</v>
+      </c>
+      <c r="I14" s="88"/>
+      <c r="J14" s="88"/>
+      <c r="K14" s="88"/>
+      <c r="L14" s="88"/>
+      <c r="M14" s="89"/>
+      <c r="N14" s="95" t="s">
+        <v>293</v>
+      </c>
+      <c r="O14" s="88"/>
+      <c r="P14" s="89"/>
+      <c r="Q14" s="90" t="s">
+        <v>294</v>
+      </c>
+      <c r="R14" s="88"/>
+      <c r="S14" s="89"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B15" s="71" t="s">
-        <v>287</v>
-      </c>
-      <c r="C15" s="72"/>
-      <c r="D15" s="72"/>
-      <c r="E15" s="72"/>
-      <c r="F15" s="72"/>
-      <c r="G15" s="72"/>
-      <c r="H15" s="72"/>
-      <c r="I15" s="72"/>
-      <c r="J15" s="72"/>
-      <c r="K15" s="72"/>
-      <c r="L15" s="72"/>
-      <c r="M15" s="72"/>
-      <c r="N15" s="72"/>
-      <c r="O15" s="72"/>
-      <c r="P15" s="72"/>
-      <c r="Q15" s="72"/>
-      <c r="R15" s="72"/>
-      <c r="S15" s="72"/>
+      <c r="B15" s="91" t="s">
+        <v>295</v>
+      </c>
+      <c r="C15" s="92"/>
+      <c r="D15" s="92"/>
+      <c r="E15" s="92"/>
+      <c r="F15" s="92"/>
+      <c r="G15" s="92"/>
+      <c r="H15" s="92"/>
+      <c r="I15" s="92"/>
+      <c r="J15" s="92"/>
+      <c r="K15" s="92"/>
+      <c r="L15" s="92"/>
+      <c r="M15" s="92"/>
+      <c r="N15" s="92"/>
+      <c r="O15" s="92"/>
+      <c r="P15" s="92"/>
+      <c r="Q15" s="92"/>
+      <c r="R15" s="92"/>
+      <c r="S15" s="92"/>
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="77" t="s">
-        <v>288</v>
-      </c>
-      <c r="B16" s="72"/>
-      <c r="C16" s="72"/>
-      <c r="D16" s="72"/>
-      <c r="E16" s="72"/>
-      <c r="F16" s="72"/>
-      <c r="G16" s="72"/>
-      <c r="H16" s="72"/>
-      <c r="I16" s="72"/>
-      <c r="J16" s="72"/>
-      <c r="K16" s="72"/>
-      <c r="L16" s="72"/>
-      <c r="M16" s="72"/>
-      <c r="N16" s="72"/>
-      <c r="O16" s="72"/>
-      <c r="P16" s="72"/>
-      <c r="Q16" s="72"/>
-      <c r="R16" s="72"/>
-      <c r="S16" s="72"/>
+      <c r="A16" s="97" t="s">
+        <v>296</v>
+      </c>
+      <c r="B16" s="92"/>
+      <c r="C16" s="92"/>
+      <c r="D16" s="92"/>
+      <c r="E16" s="92"/>
+      <c r="F16" s="92"/>
+      <c r="G16" s="92"/>
+      <c r="H16" s="92"/>
+      <c r="I16" s="92"/>
+      <c r="J16" s="92"/>
+      <c r="K16" s="92"/>
+      <c r="L16" s="92"/>
+      <c r="M16" s="92"/>
+      <c r="N16" s="92"/>
+      <c r="O16" s="92"/>
+      <c r="P16" s="92"/>
+      <c r="Q16" s="92"/>
+      <c r="R16" s="92"/>
+      <c r="S16" s="92"/>
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="37" t="s">
-        <v>289</v>
-      </c>
-      <c r="B17" s="76" t="s">
-        <v>290</v>
-      </c>
-      <c r="C17" s="68"/>
-      <c r="D17" s="68"/>
-      <c r="E17" s="68"/>
-      <c r="F17" s="68"/>
-      <c r="G17" s="69"/>
-      <c r="H17" s="76" t="s">
-        <v>291</v>
-      </c>
-      <c r="I17" s="68"/>
-      <c r="J17" s="69"/>
-      <c r="K17" s="76" t="s">
-        <v>292</v>
-      </c>
-      <c r="L17" s="68"/>
-      <c r="M17" s="69"/>
-      <c r="N17" s="76" t="s">
-        <v>293</v>
-      </c>
-      <c r="O17" s="68"/>
-      <c r="P17" s="69"/>
-      <c r="Q17" s="76" t="s">
-        <v>294</v>
-      </c>
-      <c r="R17" s="68"/>
-      <c r="S17" s="69"/>
+        <v>297</v>
+      </c>
+      <c r="B17" s="96" t="s">
+        <v>298</v>
+      </c>
+      <c r="C17" s="88"/>
+      <c r="D17" s="88"/>
+      <c r="E17" s="88"/>
+      <c r="F17" s="88"/>
+      <c r="G17" s="89"/>
+      <c r="H17" s="96" t="s">
+        <v>299</v>
+      </c>
+      <c r="I17" s="88"/>
+      <c r="J17" s="89"/>
+      <c r="K17" s="96" t="s">
+        <v>300</v>
+      </c>
+      <c r="L17" s="88"/>
+      <c r="M17" s="89"/>
+      <c r="N17" s="96" t="s">
+        <v>301</v>
+      </c>
+      <c r="O17" s="88"/>
+      <c r="P17" s="89"/>
+      <c r="Q17" s="96" t="s">
+        <v>302</v>
+      </c>
+      <c r="R17" s="88"/>
+      <c r="S17" s="89"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="71" t="s">
-        <v>268</v>
-      </c>
-      <c r="C18" s="72"/>
-      <c r="D18" s="72"/>
-      <c r="E18" s="72"/>
-      <c r="F18" s="72"/>
-      <c r="G18" s="72"/>
-      <c r="H18" s="72"/>
-      <c r="I18" s="72"/>
-      <c r="J18" s="72"/>
-      <c r="K18" s="72"/>
-      <c r="L18" s="72"/>
-      <c r="M18" s="72"/>
-      <c r="N18" s="72"/>
-      <c r="O18" s="72"/>
-      <c r="P18" s="72"/>
-      <c r="Q18" s="72"/>
-      <c r="R18" s="72"/>
-      <c r="S18" s="72"/>
+      <c r="B18" s="91" t="s">
+        <v>276</v>
+      </c>
+      <c r="C18" s="92"/>
+      <c r="D18" s="92"/>
+      <c r="E18" s="92"/>
+      <c r="F18" s="92"/>
+      <c r="G18" s="92"/>
+      <c r="H18" s="92"/>
+      <c r="I18" s="92"/>
+      <c r="J18" s="92"/>
+      <c r="K18" s="92"/>
+      <c r="L18" s="92"/>
+      <c r="M18" s="92"/>
+      <c r="N18" s="92"/>
+      <c r="O18" s="92"/>
+      <c r="P18" s="92"/>
+      <c r="Q18" s="92"/>
+      <c r="R18" s="92"/>
+      <c r="S18" s="92"/>
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="77" t="s">
-        <v>295</v>
-      </c>
-      <c r="B19" s="72"/>
-      <c r="C19" s="72"/>
-      <c r="D19" s="72"/>
-      <c r="E19" s="72"/>
-      <c r="F19" s="72"/>
-      <c r="G19" s="72"/>
-      <c r="H19" s="72"/>
-      <c r="I19" s="72"/>
-      <c r="J19" s="72"/>
-      <c r="K19" s="72"/>
-      <c r="L19" s="72"/>
-      <c r="M19" s="72"/>
-      <c r="N19" s="72"/>
-      <c r="O19" s="72"/>
-      <c r="P19" s="72"/>
-      <c r="Q19" s="72"/>
-      <c r="R19" s="72"/>
-      <c r="S19" s="72"/>
+      <c r="A19" s="97" t="s">
+        <v>303</v>
+      </c>
+      <c r="B19" s="92"/>
+      <c r="C19" s="92"/>
+      <c r="D19" s="92"/>
+      <c r="E19" s="92"/>
+      <c r="F19" s="92"/>
+      <c r="G19" s="92"/>
+      <c r="H19" s="92"/>
+      <c r="I19" s="92"/>
+      <c r="J19" s="92"/>
+      <c r="K19" s="92"/>
+      <c r="L19" s="92"/>
+      <c r="M19" s="92"/>
+      <c r="N19" s="92"/>
+      <c r="O19" s="92"/>
+      <c r="P19" s="92"/>
+      <c r="Q19" s="92"/>
+      <c r="R19" s="92"/>
+      <c r="S19" s="92"/>
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="37" t="s">
-        <v>296</v>
-      </c>
-      <c r="B20" s="78" t="s">
-        <v>297</v>
-      </c>
-      <c r="C20" s="68"/>
-      <c r="D20" s="68"/>
-      <c r="E20" s="68"/>
-      <c r="F20" s="68"/>
-      <c r="G20" s="69"/>
-      <c r="H20" s="78" t="s">
-        <v>298</v>
-      </c>
-      <c r="I20" s="68"/>
-      <c r="J20" s="68"/>
-      <c r="K20" s="68"/>
-      <c r="L20" s="68"/>
-      <c r="M20" s="69"/>
-      <c r="N20" s="78" t="s">
-        <v>299</v>
-      </c>
-      <c r="O20" s="68"/>
-      <c r="P20" s="68"/>
-      <c r="Q20" s="68"/>
-      <c r="R20" s="68"/>
-      <c r="S20" s="69"/>
+        <v>304</v>
+      </c>
+      <c r="B20" s="98" t="s">
+        <v>305</v>
+      </c>
+      <c r="C20" s="88"/>
+      <c r="D20" s="88"/>
+      <c r="E20" s="88"/>
+      <c r="F20" s="88"/>
+      <c r="G20" s="89"/>
+      <c r="H20" s="98" t="s">
+        <v>306</v>
+      </c>
+      <c r="I20" s="88"/>
+      <c r="J20" s="88"/>
+      <c r="K20" s="88"/>
+      <c r="L20" s="88"/>
+      <c r="M20" s="89"/>
+      <c r="N20" s="98" t="s">
+        <v>307</v>
+      </c>
+      <c r="O20" s="88"/>
+      <c r="P20" s="88"/>
+      <c r="Q20" s="88"/>
+      <c r="R20" s="88"/>
+      <c r="S20" s="89"/>
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B21" s="71" t="s">
-        <v>268</v>
-      </c>
-      <c r="C21" s="72"/>
-      <c r="D21" s="72"/>
-      <c r="E21" s="72"/>
-      <c r="F21" s="72"/>
-      <c r="G21" s="72"/>
-      <c r="H21" s="72"/>
-      <c r="I21" s="72"/>
-      <c r="J21" s="72"/>
-      <c r="K21" s="72"/>
-      <c r="L21" s="72"/>
-      <c r="M21" s="72"/>
-      <c r="N21" s="72"/>
-      <c r="O21" s="72"/>
-      <c r="P21" s="72"/>
-      <c r="Q21" s="72"/>
-      <c r="R21" s="72"/>
-      <c r="S21" s="72"/>
+      <c r="B21" s="91" t="s">
+        <v>276</v>
+      </c>
+      <c r="C21" s="92"/>
+      <c r="D21" s="92"/>
+      <c r="E21" s="92"/>
+      <c r="F21" s="92"/>
+      <c r="G21" s="92"/>
+      <c r="H21" s="92"/>
+      <c r="I21" s="92"/>
+      <c r="J21" s="92"/>
+      <c r="K21" s="92"/>
+      <c r="L21" s="92"/>
+      <c r="M21" s="92"/>
+      <c r="N21" s="92"/>
+      <c r="O21" s="92"/>
+      <c r="P21" s="92"/>
+      <c r="Q21" s="92"/>
+      <c r="R21" s="92"/>
+      <c r="S21" s="92"/>
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="77" t="s">
-        <v>300</v>
-      </c>
-      <c r="B22" s="72"/>
-      <c r="C22" s="72"/>
-      <c r="D22" s="72"/>
-      <c r="E22" s="72"/>
-      <c r="F22" s="72"/>
-      <c r="G22" s="72"/>
-      <c r="H22" s="72"/>
-      <c r="I22" s="72"/>
-      <c r="J22" s="72"/>
-      <c r="K22" s="72"/>
-      <c r="L22" s="72"/>
-      <c r="M22" s="72"/>
-      <c r="N22" s="72"/>
-      <c r="O22" s="72"/>
-      <c r="P22" s="72"/>
-      <c r="Q22" s="72"/>
-      <c r="R22" s="72"/>
-      <c r="S22" s="72"/>
+      <c r="A22" s="97" t="s">
+        <v>308</v>
+      </c>
+      <c r="B22" s="92"/>
+      <c r="C22" s="92"/>
+      <c r="D22" s="92"/>
+      <c r="E22" s="92"/>
+      <c r="F22" s="92"/>
+      <c r="G22" s="92"/>
+      <c r="H22" s="92"/>
+      <c r="I22" s="92"/>
+      <c r="J22" s="92"/>
+      <c r="K22" s="92"/>
+      <c r="L22" s="92"/>
+      <c r="M22" s="92"/>
+      <c r="N22" s="92"/>
+      <c r="O22" s="92"/>
+      <c r="P22" s="92"/>
+      <c r="Q22" s="92"/>
+      <c r="R22" s="92"/>
+      <c r="S22" s="92"/>
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="37" t="s">
-        <v>301</v>
-      </c>
-      <c r="B23" s="78" t="s">
-        <v>302</v>
-      </c>
-      <c r="C23" s="68"/>
-      <c r="D23" s="68"/>
-      <c r="E23" s="68"/>
-      <c r="F23" s="68"/>
-      <c r="G23" s="69"/>
-      <c r="H23" s="78" t="s">
-        <v>303</v>
-      </c>
-      <c r="I23" s="68"/>
-      <c r="J23" s="69"/>
-      <c r="K23" s="78" t="s">
-        <v>304</v>
-      </c>
-      <c r="L23" s="68"/>
-      <c r="M23" s="69"/>
-      <c r="N23" s="78" t="s">
-        <v>305</v>
-      </c>
-      <c r="O23" s="68"/>
-      <c r="P23" s="69"/>
-      <c r="Q23" s="74" t="s">
-        <v>306</v>
-      </c>
-      <c r="R23" s="68"/>
-      <c r="S23" s="69"/>
+        <v>309</v>
+      </c>
+      <c r="B23" s="98" t="s">
+        <v>310</v>
+      </c>
+      <c r="C23" s="88"/>
+      <c r="D23" s="88"/>
+      <c r="E23" s="88"/>
+      <c r="F23" s="88"/>
+      <c r="G23" s="89"/>
+      <c r="H23" s="98" t="s">
+        <v>311</v>
+      </c>
+      <c r="I23" s="88"/>
+      <c r="J23" s="89"/>
+      <c r="K23" s="98" t="s">
+        <v>312</v>
+      </c>
+      <c r="L23" s="88"/>
+      <c r="M23" s="89"/>
+      <c r="N23" s="98" t="s">
+        <v>313</v>
+      </c>
+      <c r="O23" s="88"/>
+      <c r="P23" s="89"/>
+      <c r="Q23" s="94" t="s">
+        <v>314</v>
+      </c>
+      <c r="R23" s="88"/>
+      <c r="S23" s="89"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="83" t="s">
-        <v>307</v>
-      </c>
-      <c r="B26" s="72"/>
-      <c r="C26" s="72"/>
-      <c r="D26" s="72"/>
-      <c r="E26" s="72"/>
-      <c r="F26" s="72"/>
-      <c r="G26" s="72"/>
-      <c r="H26" s="72"/>
-      <c r="I26" s="72"/>
-      <c r="J26" s="72"/>
-      <c r="K26" s="72"/>
-      <c r="L26" s="72"/>
-      <c r="M26" s="72"/>
-      <c r="N26" s="72"/>
-      <c r="O26" s="72"/>
-      <c r="P26" s="72"/>
-      <c r="Q26" s="72"/>
-      <c r="R26" s="72"/>
-      <c r="S26" s="72"/>
+      <c r="A26" s="103" t="s">
+        <v>315</v>
+      </c>
+      <c r="B26" s="92"/>
+      <c r="C26" s="92"/>
+      <c r="D26" s="92"/>
+      <c r="E26" s="92"/>
+      <c r="F26" s="92"/>
+      <c r="G26" s="92"/>
+      <c r="H26" s="92"/>
+      <c r="I26" s="92"/>
+      <c r="J26" s="92"/>
+      <c r="K26" s="92"/>
+      <c r="L26" s="92"/>
+      <c r="M26" s="92"/>
+      <c r="N26" s="92"/>
+      <c r="O26" s="92"/>
+      <c r="P26" s="92"/>
+      <c r="Q26" s="92"/>
+      <c r="R26" s="92"/>
+      <c r="S26" s="92"/>
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="37" t="s">
-        <v>308</v>
-      </c>
-      <c r="B27" s="67" t="s">
-        <v>309</v>
-      </c>
-      <c r="C27" s="68"/>
-      <c r="D27" s="69"/>
-      <c r="E27" s="67" t="s">
-        <v>310</v>
-      </c>
-      <c r="F27" s="68"/>
-      <c r="G27" s="69"/>
-      <c r="H27" s="75" t="s">
-        <v>311</v>
-      </c>
-      <c r="I27" s="68"/>
-      <c r="J27" s="69"/>
-      <c r="K27" s="76" t="s">
-        <v>312</v>
-      </c>
-      <c r="L27" s="68"/>
-      <c r="M27" s="69"/>
-      <c r="N27" s="76" t="s">
-        <v>313</v>
-      </c>
-      <c r="O27" s="68"/>
-      <c r="P27" s="69"/>
-      <c r="Q27" s="75" t="s">
-        <v>314</v>
-      </c>
-      <c r="R27" s="68"/>
-      <c r="S27" s="69"/>
+        <v>316</v>
+      </c>
+      <c r="B27" s="87" t="s">
+        <v>317</v>
+      </c>
+      <c r="C27" s="88"/>
+      <c r="D27" s="89"/>
+      <c r="E27" s="87" t="s">
+        <v>318</v>
+      </c>
+      <c r="F27" s="88"/>
+      <c r="G27" s="89"/>
+      <c r="H27" s="95" t="s">
+        <v>319</v>
+      </c>
+      <c r="I27" s="88"/>
+      <c r="J27" s="89"/>
+      <c r="K27" s="96" t="s">
+        <v>320</v>
+      </c>
+      <c r="L27" s="88"/>
+      <c r="M27" s="89"/>
+      <c r="N27" s="96" t="s">
+        <v>321</v>
+      </c>
+      <c r="O27" s="88"/>
+      <c r="P27" s="89"/>
+      <c r="Q27" s="95" t="s">
+        <v>322</v>
+      </c>
+      <c r="R27" s="88"/>
+      <c r="S27" s="89"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="77" t="s">
-        <v>315</v>
-      </c>
-      <c r="B30" s="72"/>
-      <c r="C30" s="72"/>
-      <c r="D30" s="72"/>
-      <c r="E30" s="72"/>
-      <c r="F30" s="72"/>
-      <c r="G30" s="72"/>
-      <c r="H30" s="72"/>
-      <c r="I30" s="72"/>
-      <c r="J30" s="72"/>
-      <c r="K30" s="72"/>
-      <c r="L30" s="72"/>
-      <c r="M30" s="72"/>
-      <c r="N30" s="72"/>
-      <c r="O30" s="72"/>
-      <c r="P30" s="72"/>
-      <c r="Q30" s="72"/>
-      <c r="R30" s="72"/>
-      <c r="S30" s="72"/>
+      <c r="A30" s="97" t="s">
+        <v>323</v>
+      </c>
+      <c r="B30" s="92"/>
+      <c r="C30" s="92"/>
+      <c r="D30" s="92"/>
+      <c r="E30" s="92"/>
+      <c r="F30" s="92"/>
+      <c r="G30" s="92"/>
+      <c r="H30" s="92"/>
+      <c r="I30" s="92"/>
+      <c r="J30" s="92"/>
+      <c r="K30" s="92"/>
+      <c r="L30" s="92"/>
+      <c r="M30" s="92"/>
+      <c r="N30" s="92"/>
+      <c r="O30" s="92"/>
+      <c r="P30" s="92"/>
+      <c r="Q30" s="92"/>
+      <c r="R30" s="92"/>
+      <c r="S30" s="92"/>
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="73" t="s">
-        <v>316</v>
-      </c>
-      <c r="B31" s="72"/>
-      <c r="C31" s="72"/>
-      <c r="D31" s="72"/>
-      <c r="E31" s="72"/>
-      <c r="F31" s="72"/>
-      <c r="G31" s="72"/>
-      <c r="H31" s="72"/>
-      <c r="I31" s="72"/>
-      <c r="J31" s="72"/>
-      <c r="K31" s="72"/>
-      <c r="L31" s="72"/>
-      <c r="M31" s="72"/>
-      <c r="N31" s="72"/>
-      <c r="O31" s="72"/>
-      <c r="P31" s="72"/>
-      <c r="Q31" s="72"/>
-      <c r="R31" s="72"/>
-      <c r="S31" s="72"/>
+      <c r="A31" s="93" t="s">
+        <v>324</v>
+      </c>
+      <c r="B31" s="92"/>
+      <c r="C31" s="92"/>
+      <c r="D31" s="92"/>
+      <c r="E31" s="92"/>
+      <c r="F31" s="92"/>
+      <c r="G31" s="92"/>
+      <c r="H31" s="92"/>
+      <c r="I31" s="92"/>
+      <c r="J31" s="92"/>
+      <c r="K31" s="92"/>
+      <c r="L31" s="92"/>
+      <c r="M31" s="92"/>
+      <c r="N31" s="92"/>
+      <c r="O31" s="92"/>
+      <c r="P31" s="92"/>
+      <c r="Q31" s="92"/>
+      <c r="R31" s="92"/>
+      <c r="S31" s="92"/>
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="73" t="s">
-        <v>317</v>
-      </c>
-      <c r="B32" s="72"/>
-      <c r="C32" s="72"/>
-      <c r="D32" s="72"/>
-      <c r="E32" s="72"/>
-      <c r="F32" s="72"/>
-      <c r="G32" s="72"/>
-      <c r="H32" s="72"/>
-      <c r="I32" s="72"/>
-      <c r="J32" s="72"/>
-      <c r="K32" s="72"/>
-      <c r="L32" s="72"/>
-      <c r="M32" s="72"/>
-      <c r="N32" s="72"/>
-      <c r="O32" s="72"/>
-      <c r="P32" s="72"/>
-      <c r="Q32" s="72"/>
-      <c r="R32" s="72"/>
-      <c r="S32" s="72"/>
+      <c r="A32" s="93" t="s">
+        <v>325</v>
+      </c>
+      <c r="B32" s="92"/>
+      <c r="C32" s="92"/>
+      <c r="D32" s="92"/>
+      <c r="E32" s="92"/>
+      <c r="F32" s="92"/>
+      <c r="G32" s="92"/>
+      <c r="H32" s="92"/>
+      <c r="I32" s="92"/>
+      <c r="J32" s="92"/>
+      <c r="K32" s="92"/>
+      <c r="L32" s="92"/>
+      <c r="M32" s="92"/>
+      <c r="N32" s="92"/>
+      <c r="O32" s="92"/>
+      <c r="P32" s="92"/>
+      <c r="Q32" s="92"/>
+      <c r="R32" s="92"/>
+      <c r="S32" s="92"/>
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="73" t="s">
-        <v>318</v>
-      </c>
-      <c r="B33" s="72"/>
-      <c r="C33" s="72"/>
-      <c r="D33" s="72"/>
-      <c r="E33" s="72"/>
-      <c r="F33" s="72"/>
-      <c r="G33" s="72"/>
-      <c r="H33" s="72"/>
-      <c r="I33" s="72"/>
-      <c r="J33" s="72"/>
-      <c r="K33" s="72"/>
-      <c r="L33" s="72"/>
-      <c r="M33" s="72"/>
-      <c r="N33" s="72"/>
-      <c r="O33" s="72"/>
-      <c r="P33" s="72"/>
-      <c r="Q33" s="72"/>
-      <c r="R33" s="72"/>
-      <c r="S33" s="72"/>
+      <c r="A33" s="93" t="s">
+        <v>326</v>
+      </c>
+      <c r="B33" s="92"/>
+      <c r="C33" s="92"/>
+      <c r="D33" s="92"/>
+      <c r="E33" s="92"/>
+      <c r="F33" s="92"/>
+      <c r="G33" s="92"/>
+      <c r="H33" s="92"/>
+      <c r="I33" s="92"/>
+      <c r="J33" s="92"/>
+      <c r="K33" s="92"/>
+      <c r="L33" s="92"/>
+      <c r="M33" s="92"/>
+      <c r="N33" s="92"/>
+      <c r="O33" s="92"/>
+      <c r="P33" s="92"/>
+      <c r="Q33" s="92"/>
+      <c r="R33" s="92"/>
+      <c r="S33" s="92"/>
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="73" t="s">
-        <v>319</v>
-      </c>
-      <c r="B34" s="72"/>
-      <c r="C34" s="72"/>
-      <c r="D34" s="72"/>
-      <c r="E34" s="72"/>
-      <c r="F34" s="72"/>
-      <c r="G34" s="72"/>
-      <c r="H34" s="72"/>
-      <c r="I34" s="72"/>
-      <c r="J34" s="72"/>
-      <c r="K34" s="72"/>
-      <c r="L34" s="72"/>
-      <c r="M34" s="72"/>
-      <c r="N34" s="72"/>
-      <c r="O34" s="72"/>
-      <c r="P34" s="72"/>
-      <c r="Q34" s="72"/>
-      <c r="R34" s="72"/>
-      <c r="S34" s="72"/>
+      <c r="A34" s="93" t="s">
+        <v>327</v>
+      </c>
+      <c r="B34" s="92"/>
+      <c r="C34" s="92"/>
+      <c r="D34" s="92"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="92"/>
+      <c r="G34" s="92"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="92"/>
+      <c r="J34" s="92"/>
+      <c r="K34" s="92"/>
+      <c r="L34" s="92"/>
+      <c r="M34" s="92"/>
+      <c r="N34" s="92"/>
+      <c r="O34" s="92"/>
+      <c r="P34" s="92"/>
+      <c r="Q34" s="92"/>
+      <c r="R34" s="92"/>
+      <c r="S34" s="92"/>
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="73" t="s">
-        <v>320</v>
-      </c>
-      <c r="B35" s="72"/>
-      <c r="C35" s="72"/>
-      <c r="D35" s="72"/>
-      <c r="E35" s="72"/>
-      <c r="F35" s="72"/>
-      <c r="G35" s="72"/>
-      <c r="H35" s="72"/>
-      <c r="I35" s="72"/>
-      <c r="J35" s="72"/>
-      <c r="K35" s="72"/>
-      <c r="L35" s="72"/>
-      <c r="M35" s="72"/>
-      <c r="N35" s="72"/>
-      <c r="O35" s="72"/>
-      <c r="P35" s="72"/>
-      <c r="Q35" s="72"/>
-      <c r="R35" s="72"/>
-      <c r="S35" s="72"/>
+      <c r="A35" s="93" t="s">
+        <v>328</v>
+      </c>
+      <c r="B35" s="92"/>
+      <c r="C35" s="92"/>
+      <c r="D35" s="92"/>
+      <c r="E35" s="92"/>
+      <c r="F35" s="92"/>
+      <c r="G35" s="92"/>
+      <c r="H35" s="92"/>
+      <c r="I35" s="92"/>
+      <c r="J35" s="92"/>
+      <c r="K35" s="92"/>
+      <c r="L35" s="92"/>
+      <c r="M35" s="92"/>
+      <c r="N35" s="92"/>
+      <c r="O35" s="92"/>
+      <c r="P35" s="92"/>
+      <c r="Q35" s="92"/>
+      <c r="R35" s="92"/>
+      <c r="S35" s="92"/>
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="73" t="s">
-        <v>321</v>
-      </c>
-      <c r="B36" s="72"/>
-      <c r="C36" s="72"/>
-      <c r="D36" s="72"/>
-      <c r="E36" s="72"/>
-      <c r="F36" s="72"/>
-      <c r="G36" s="72"/>
-      <c r="H36" s="72"/>
-      <c r="I36" s="72"/>
-      <c r="J36" s="72"/>
-      <c r="K36" s="72"/>
-      <c r="L36" s="72"/>
-      <c r="M36" s="72"/>
-      <c r="N36" s="72"/>
-      <c r="O36" s="72"/>
-      <c r="P36" s="72"/>
-      <c r="Q36" s="72"/>
-      <c r="R36" s="72"/>
-      <c r="S36" s="72"/>
+      <c r="A36" s="93" t="s">
+        <v>329</v>
+      </c>
+      <c r="B36" s="92"/>
+      <c r="C36" s="92"/>
+      <c r="D36" s="92"/>
+      <c r="E36" s="92"/>
+      <c r="F36" s="92"/>
+      <c r="G36" s="92"/>
+      <c r="H36" s="92"/>
+      <c r="I36" s="92"/>
+      <c r="J36" s="92"/>
+      <c r="K36" s="92"/>
+      <c r="L36" s="92"/>
+      <c r="M36" s="92"/>
+      <c r="N36" s="92"/>
+      <c r="O36" s="92"/>
+      <c r="P36" s="92"/>
+      <c r="Q36" s="92"/>
+      <c r="R36" s="92"/>
+      <c r="S36" s="92"/>
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="84" t="s">
-        <v>322</v>
-      </c>
-      <c r="B37" s="72"/>
-      <c r="C37" s="72"/>
-      <c r="D37" s="72"/>
-      <c r="E37" s="72"/>
-      <c r="F37" s="72"/>
-      <c r="G37" s="72"/>
-      <c r="H37" s="72"/>
-      <c r="I37" s="72"/>
-      <c r="J37" s="72"/>
-      <c r="K37" s="72"/>
-      <c r="L37" s="72"/>
-      <c r="M37" s="72"/>
-      <c r="N37" s="72"/>
-      <c r="O37" s="72"/>
-      <c r="P37" s="72"/>
-      <c r="Q37" s="72"/>
-      <c r="R37" s="72"/>
-      <c r="S37" s="72"/>
+      <c r="A37" s="104" t="s">
+        <v>330</v>
+      </c>
+      <c r="B37" s="92"/>
+      <c r="C37" s="92"/>
+      <c r="D37" s="92"/>
+      <c r="E37" s="92"/>
+      <c r="F37" s="92"/>
+      <c r="G37" s="92"/>
+      <c r="H37" s="92"/>
+      <c r="I37" s="92"/>
+      <c r="J37" s="92"/>
+      <c r="K37" s="92"/>
+      <c r="L37" s="92"/>
+      <c r="M37" s="92"/>
+      <c r="N37" s="92"/>
+      <c r="O37" s="92"/>
+      <c r="P37" s="92"/>
+      <c r="Q37" s="92"/>
+      <c r="R37" s="92"/>
+      <c r="S37" s="92"/>
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="38" t="s">
-        <v>257</v>
-      </c>
-      <c r="B39" s="87" t="s">
-        <v>323</v>
-      </c>
-      <c r="C39" s="72"/>
-      <c r="D39" s="72"/>
-      <c r="E39" s="85" t="s">
-        <v>324</v>
-      </c>
-      <c r="F39" s="72"/>
-      <c r="G39" s="72"/>
-      <c r="H39" s="88" t="s">
-        <v>325</v>
-      </c>
-      <c r="I39" s="72"/>
-      <c r="J39" s="72"/>
-      <c r="K39" s="81" t="s">
-        <v>326</v>
-      </c>
-      <c r="L39" s="72"/>
-      <c r="M39" s="72"/>
-      <c r="N39" s="79" t="s">
+        <v>265</v>
+      </c>
+      <c r="B39" s="107" t="s">
+        <v>331</v>
+      </c>
+      <c r="C39" s="92"/>
+      <c r="D39" s="92"/>
+      <c r="E39" s="105" t="s">
+        <v>332</v>
+      </c>
+      <c r="F39" s="92"/>
+      <c r="G39" s="92"/>
+      <c r="H39" s="108" t="s">
+        <v>333</v>
+      </c>
+      <c r="I39" s="92"/>
+      <c r="J39" s="92"/>
+      <c r="K39" s="101" t="s">
+        <v>334</v>
+      </c>
+      <c r="L39" s="92"/>
+      <c r="M39" s="92"/>
+      <c r="N39" s="99" t="s">
         <v>45</v>
       </c>
-      <c r="O39" s="72"/>
-      <c r="P39" s="72"/>
-      <c r="Q39" s="86" t="s">
-        <v>327</v>
-      </c>
-      <c r="R39" s="72"/>
-      <c r="S39" s="72"/>
+      <c r="O39" s="92"/>
+      <c r="P39" s="92"/>
+      <c r="Q39" s="106" t="s">
+        <v>335</v>
+      </c>
+      <c r="R39" s="92"/>
+      <c r="S39" s="92"/>
     </row>
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A16:S16"/>
     <mergeCell ref="H20:M20"/>
-    <mergeCell ref="A16:S16"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -7094,14 +7400,13 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -7110,6 +7415,7 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -7117,7 +7423,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -7165,33 +7471,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="90" t="s">
-        <v>328</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="65"/>
+      <c r="A1" s="110" t="s">
+        <v>336</v>
+      </c>
+      <c r="B1" s="84"/>
+      <c r="C1" s="84"/>
+      <c r="D1" s="84"/>
+      <c r="E1" s="84"/>
+      <c r="F1" s="85"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -7425,15 +7731,15 @@
       </c>
       <c r="B13" s="26">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C13" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D13" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E13" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Blocked")</f>
@@ -7441,7 +7747,7 @@
       </c>
       <c r="F13" s="27">
         <f t="shared" si="1"/>
-        <v>0.33333333333333331</v>
+        <v>0.36363636363636365</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -7471,19 +7777,19 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="28" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="B16" s="29">
         <f>SUM(B4:B14)</f>
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C16" s="29">
         <f>SUM(C4:C14)</f>
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E16">
         <f>SUM(E4:E14)</f>
@@ -7491,12 +7797,12 @@
       </c>
       <c r="F16" s="30">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.67289719626168221</v>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="43" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B18" s="44">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -7505,7 +7811,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="45" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
     </row>
   </sheetData>
@@ -7526,7 +7832,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -7537,437 +7843,471 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="90" t="s">
-        <v>335</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="65"/>
+      <c r="A1" s="110" t="s">
+        <v>343</v>
+      </c>
+      <c r="B1" s="84"/>
+      <c r="C1" s="84"/>
+      <c r="D1" s="84"/>
+      <c r="E1" s="85"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="31" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="D3" s="31" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="32" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="34" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="32" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="34" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="32" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="34" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="32" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="34" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="32" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="34" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="32" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="34" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="32" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="34" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="32" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="34" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="32" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="34" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="32" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="E22" s="33" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="34" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="E23" s="35" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="32" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="58" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="B25" s="55" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="C25" s="59" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D25" s="55" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="E25" s="60" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="61" t="s">
+        <v>407</v>
+      </c>
+      <c r="B26" s="49" t="s">
         <v>399</v>
       </c>
-      <c r="B26" s="49" t="s">
-        <v>391</v>
-      </c>
       <c r="C26" s="59" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="D26" s="49" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="E26" s="62" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="58" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="B27" s="55" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="C27" s="59" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="D27" s="55" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="E27" s="60" t="s">
-        <v>402</v>
+        <v>410</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A28" s="79" t="s">
+        <v>411</v>
+      </c>
+      <c r="B28" s="66" t="s">
+        <v>363</v>
+      </c>
+      <c r="C28" s="75" t="s">
+        <v>354</v>
+      </c>
+      <c r="D28" s="66" t="s">
+        <v>351</v>
+      </c>
+      <c r="E28" s="80" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A29" s="81" t="s">
+        <v>413</v>
+      </c>
+      <c r="B29" s="72" t="s">
+        <v>349</v>
+      </c>
+      <c r="C29" s="77" t="s">
+        <v>362</v>
+      </c>
+      <c r="D29" s="72" t="s">
+        <v>351</v>
+      </c>
+      <c r="E29" s="82" t="s">
+        <v>414</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(tracker): EAS project linked; push risk downgraded from blocking to testable
E10 Deploy 36% -> 39%.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0BFDA97-4E01-4326-B1D4-104F1579AFED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FD39719-20C3-4500-B8DA-4BD4F4702DFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14895" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="761" uniqueCount="419">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -831,6 +831,12 @@
   </si>
   <si>
     <t>Writes extra.eas.projectId. Blocks minting ANY push token - see mobile/EAS-SETUP.md</t>
+  </si>
+  <si>
+    <t>EAS project linked (@usangr01/sportiq)</t>
+  </si>
+  <si>
+    <t>projectId written; push tokens now mintable. Run eas from mobile/, not the root</t>
   </si>
   <si>
     <t>Legend</t>
@@ -1353,6 +1359,12 @@
   </si>
   <si>
     <t>getExpoPushTokenAsync needs a real projectId, which only eas init can create. The backend side (PUT /user/push-token, _send_push) is real and tested; nothing has ever been delivered to a device. Compounded on Android by Expo Go dropping remote push in SDK 53, so a development build is required.</t>
+  </si>
+  <si>
+    <t>Push still unverified on a device</t>
+  </si>
+  <si>
+    <t>projectId now exists so a token CAN be minted, but nothing has been delivered to a real device. Needs a development build: Expo Go on Android cannot receive remote push since SDK 53. Reduced from blocking to testable.</t>
   </si>
 </sst>
 </file>
@@ -1362,7 +1374,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\ mmm"/>
   </numFmts>
-  <fonts count="30" x14ac:knownFonts="1">
+  <fonts count="34" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1533,8 +1545,30 @@
       <color rgb="FF6B7280"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF111827"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF111827"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF6B7280"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="25">
+  <fills count="28">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1656,8 +1690,23 @@
         <fgColor rgb="FF94A3B8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF16A34A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF94A3B8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1773,11 +1822,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2023,12 +2087,42 @@
     <xf numFmtId="0" fontId="27" fillId="22" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="26" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="25" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="26" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="27" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="25" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2094,7 +2188,7 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2414,7 +2508,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R117"/>
+  <dimension ref="A1:R118"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2428,46 +2522,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="86" t="s">
+      <c r="A1" s="96" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="84"/>
-      <c r="F1" s="84"/>
-      <c r="G1" s="84"/>
-      <c r="H1" s="84"/>
-      <c r="I1" s="84"/>
-      <c r="J1" s="84"/>
-      <c r="K1" s="84"/>
-      <c r="L1" s="84"/>
-      <c r="M1" s="84"/>
-      <c r="N1" s="84"/>
-      <c r="O1" s="84"/>
-      <c r="P1" s="84"/>
-      <c r="Q1" s="85"/>
+      <c r="B1" s="94"/>
+      <c r="C1" s="94"/>
+      <c r="D1" s="94"/>
+      <c r="E1" s="94"/>
+      <c r="F1" s="94"/>
+      <c r="G1" s="94"/>
+      <c r="H1" s="94"/>
+      <c r="I1" s="94"/>
+      <c r="J1" s="94"/>
+      <c r="K1" s="94"/>
+      <c r="L1" s="94"/>
+      <c r="M1" s="94"/>
+      <c r="N1" s="94"/>
+      <c r="O1" s="94"/>
+      <c r="P1" s="94"/>
+      <c r="Q1" s="95"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="83" t="s">
+      <c r="A2" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="84"/>
-      <c r="C2" s="84"/>
-      <c r="D2" s="84"/>
-      <c r="E2" s="84"/>
-      <c r="F2" s="84"/>
-      <c r="G2" s="84"/>
-      <c r="H2" s="84"/>
-      <c r="I2" s="84"/>
-      <c r="J2" s="84"/>
-      <c r="K2" s="84"/>
-      <c r="L2" s="84"/>
-      <c r="M2" s="84"/>
-      <c r="N2" s="84"/>
-      <c r="O2" s="84"/>
-      <c r="P2" s="84"/>
-      <c r="Q2" s="85"/>
+      <c r="B2" s="94"/>
+      <c r="C2" s="94"/>
+      <c r="D2" s="94"/>
+      <c r="E2" s="94"/>
+      <c r="F2" s="94"/>
+      <c r="G2" s="94"/>
+      <c r="H2" s="94"/>
+      <c r="I2" s="94"/>
+      <c r="J2" s="94"/>
+      <c r="K2" s="94"/>
+      <c r="L2" s="94"/>
+      <c r="M2" s="94"/>
+      <c r="N2" s="94"/>
+      <c r="O2" s="94"/>
+      <c r="P2" s="94"/>
+      <c r="Q2" s="95"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
@@ -6021,7 +6115,7 @@
       <c r="P102" s="11"/>
       <c r="Q102" s="11"/>
       <c r="R102" t="str">
-        <f t="shared" ref="R102:R115" si="3">IF($A102&lt;&gt;"",$A102,R101)</f>
+        <f t="shared" ref="R102:R116" si="3">IF($A102&lt;&gt;"",$A102,R101)</f>
         <v>E9 Data Ops</v>
       </c>
     </row>
@@ -6506,23 +6600,60 @@
         <v>E10 Deploy</v>
       </c>
     </row>
-    <row r="117" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A117" s="25" t="s">
+    <row r="116" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A116" s="83" t="s">
+        <v>162</v>
+      </c>
+      <c r="B116" s="84" t="s">
         <v>265</v>
       </c>
-      <c r="B117" s="5" t="s">
+      <c r="C116" s="85" t="s">
         <v>22</v>
       </c>
-      <c r="C117" s="17" t="s">
+      <c r="D116" s="86" t="s">
+        <v>85</v>
+      </c>
+      <c r="E116" s="87">
+        <v>46238</v>
+      </c>
+      <c r="F116" s="87">
+        <v>46238</v>
+      </c>
+      <c r="G116" s="88" t="s">
+        <v>266</v>
+      </c>
+      <c r="H116" s="84"/>
+      <c r="I116" s="89"/>
+      <c r="J116" s="84"/>
+      <c r="K116" s="84"/>
+      <c r="L116" s="84"/>
+      <c r="M116" s="84"/>
+      <c r="N116" s="84"/>
+      <c r="O116" s="84"/>
+      <c r="P116" s="84"/>
+      <c r="Q116" s="84"/>
+      <c r="R116" t="str">
+        <f t="shared" si="3"/>
+        <v>E10 Deploy</v>
+      </c>
+    </row>
+    <row r="118" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A118" s="25" t="s">
+        <v>267</v>
+      </c>
+      <c r="B118" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C118" s="17" t="s">
         <v>231</v>
       </c>
-      <c r="D117" s="19" t="s">
+      <c r="D118" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="E117" s="23" t="s">
+      <c r="E118" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="F117" s="21" t="s">
+      <c r="F118" s="21" t="s">
         <v>136</v>
       </c>
     </row>
@@ -6546,852 +6677,852 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="102" t="s">
-        <v>266</v>
-      </c>
-      <c r="B1" s="92"/>
-      <c r="C1" s="92"/>
-      <c r="D1" s="92"/>
-      <c r="E1" s="92"/>
-      <c r="F1" s="92"/>
-      <c r="G1" s="92"/>
-      <c r="H1" s="92"/>
-      <c r="I1" s="92"/>
-      <c r="J1" s="92"/>
-      <c r="K1" s="92"/>
-      <c r="L1" s="92"/>
-      <c r="M1" s="92"/>
-      <c r="N1" s="92"/>
-      <c r="O1" s="92"/>
-      <c r="P1" s="92"/>
-      <c r="Q1" s="92"/>
-      <c r="R1" s="92"/>
-      <c r="S1" s="92"/>
+      <c r="A1" s="112" t="s">
+        <v>268</v>
+      </c>
+      <c r="B1" s="102"/>
+      <c r="C1" s="102"/>
+      <c r="D1" s="102"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="102"/>
+      <c r="H1" s="102"/>
+      <c r="I1" s="102"/>
+      <c r="J1" s="102"/>
+      <c r="K1" s="102"/>
+      <c r="L1" s="102"/>
+      <c r="M1" s="102"/>
+      <c r="N1" s="102"/>
+      <c r="O1" s="102"/>
+      <c r="P1" s="102"/>
+      <c r="Q1" s="102"/>
+      <c r="R1" s="102"/>
+      <c r="S1" s="102"/>
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="109" t="s">
-        <v>267</v>
-      </c>
-      <c r="B2" s="92"/>
-      <c r="C2" s="92"/>
-      <c r="D2" s="92"/>
-      <c r="E2" s="92"/>
-      <c r="F2" s="92"/>
-      <c r="G2" s="92"/>
-      <c r="H2" s="92"/>
-      <c r="I2" s="92"/>
-      <c r="J2" s="92"/>
-      <c r="K2" s="92"/>
-      <c r="L2" s="92"/>
-      <c r="M2" s="92"/>
-      <c r="N2" s="92"/>
-      <c r="O2" s="92"/>
-      <c r="P2" s="92"/>
-      <c r="Q2" s="92"/>
-      <c r="R2" s="92"/>
-      <c r="S2" s="92"/>
+      <c r="A2" s="119" t="s">
+        <v>269</v>
+      </c>
+      <c r="B2" s="102"/>
+      <c r="C2" s="102"/>
+      <c r="D2" s="102"/>
+      <c r="E2" s="102"/>
+      <c r="F2" s="102"/>
+      <c r="G2" s="102"/>
+      <c r="H2" s="102"/>
+      <c r="I2" s="102"/>
+      <c r="J2" s="102"/>
+      <c r="K2" s="102"/>
+      <c r="L2" s="102"/>
+      <c r="M2" s="102"/>
+      <c r="N2" s="102"/>
+      <c r="O2" s="102"/>
+      <c r="P2" s="102"/>
+      <c r="Q2" s="102"/>
+      <c r="R2" s="102"/>
+      <c r="S2" s="102"/>
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="97" t="s">
-        <v>268</v>
-      </c>
-      <c r="B4" s="92"/>
-      <c r="C4" s="92"/>
-      <c r="D4" s="92"/>
-      <c r="E4" s="92"/>
-      <c r="F4" s="92"/>
-      <c r="G4" s="92"/>
-      <c r="H4" s="92"/>
-      <c r="I4" s="92"/>
-      <c r="J4" s="92"/>
-      <c r="K4" s="92"/>
-      <c r="L4" s="92"/>
-      <c r="M4" s="92"/>
-      <c r="N4" s="92"/>
-      <c r="O4" s="92"/>
-      <c r="P4" s="92"/>
-      <c r="Q4" s="92"/>
-      <c r="R4" s="92"/>
-      <c r="S4" s="92"/>
+      <c r="A4" s="107" t="s">
+        <v>270</v>
+      </c>
+      <c r="B4" s="102"/>
+      <c r="C4" s="102"/>
+      <c r="D4" s="102"/>
+      <c r="E4" s="102"/>
+      <c r="F4" s="102"/>
+      <c r="G4" s="102"/>
+      <c r="H4" s="102"/>
+      <c r="I4" s="102"/>
+      <c r="J4" s="102"/>
+      <c r="K4" s="102"/>
+      <c r="L4" s="102"/>
+      <c r="M4" s="102"/>
+      <c r="N4" s="102"/>
+      <c r="O4" s="102"/>
+      <c r="P4" s="102"/>
+      <c r="Q4" s="102"/>
+      <c r="R4" s="102"/>
+      <c r="S4" s="102"/>
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="37" t="s">
-        <v>269</v>
-      </c>
-      <c r="B5" s="87" t="s">
-        <v>270</v>
-      </c>
-      <c r="C5" s="88"/>
-      <c r="D5" s="89"/>
-      <c r="E5" s="90" t="s">
         <v>271</v>
       </c>
-      <c r="F5" s="88"/>
-      <c r="G5" s="89"/>
-      <c r="H5" s="90" t="s">
+      <c r="B5" s="97" t="s">
         <v>272</v>
       </c>
-      <c r="I5" s="88"/>
-      <c r="J5" s="89"/>
-      <c r="K5" s="87" t="s">
+      <c r="C5" s="98"/>
+      <c r="D5" s="99"/>
+      <c r="E5" s="100" t="s">
         <v>273</v>
       </c>
-      <c r="L5" s="88"/>
-      <c r="M5" s="89"/>
-      <c r="N5" s="94" t="s">
+      <c r="F5" s="98"/>
+      <c r="G5" s="99"/>
+      <c r="H5" s="100" t="s">
         <v>274</v>
       </c>
-      <c r="O5" s="88"/>
-      <c r="P5" s="89"/>
-      <c r="Q5" s="94" t="s">
+      <c r="I5" s="98"/>
+      <c r="J5" s="99"/>
+      <c r="K5" s="97" t="s">
         <v>275</v>
       </c>
-      <c r="R5" s="88"/>
-      <c r="S5" s="89"/>
+      <c r="L5" s="98"/>
+      <c r="M5" s="99"/>
+      <c r="N5" s="104" t="s">
+        <v>276</v>
+      </c>
+      <c r="O5" s="98"/>
+      <c r="P5" s="99"/>
+      <c r="Q5" s="104" t="s">
+        <v>277</v>
+      </c>
+      <c r="R5" s="98"/>
+      <c r="S5" s="99"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="91" t="s">
-        <v>276</v>
-      </c>
-      <c r="C6" s="92"/>
-      <c r="D6" s="92"/>
-      <c r="E6" s="92"/>
-      <c r="F6" s="92"/>
-      <c r="G6" s="92"/>
-      <c r="H6" s="92"/>
-      <c r="I6" s="92"/>
-      <c r="J6" s="92"/>
-      <c r="K6" s="92"/>
-      <c r="L6" s="92"/>
-      <c r="M6" s="92"/>
-      <c r="N6" s="92"/>
-      <c r="O6" s="92"/>
-      <c r="P6" s="92"/>
-      <c r="Q6" s="92"/>
-      <c r="R6" s="92"/>
-      <c r="S6" s="92"/>
+      <c r="B6" s="101" t="s">
+        <v>278</v>
+      </c>
+      <c r="C6" s="102"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="102"/>
+      <c r="G6" s="102"/>
+      <c r="H6" s="102"/>
+      <c r="I6" s="102"/>
+      <c r="J6" s="102"/>
+      <c r="K6" s="102"/>
+      <c r="L6" s="102"/>
+      <c r="M6" s="102"/>
+      <c r="N6" s="102"/>
+      <c r="O6" s="102"/>
+      <c r="P6" s="102"/>
+      <c r="Q6" s="102"/>
+      <c r="R6" s="102"/>
+      <c r="S6" s="102"/>
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="97" t="s">
-        <v>277</v>
-      </c>
-      <c r="B7" s="92"/>
-      <c r="C7" s="92"/>
-      <c r="D7" s="92"/>
-      <c r="E7" s="92"/>
-      <c r="F7" s="92"/>
-      <c r="G7" s="92"/>
-      <c r="H7" s="92"/>
-      <c r="I7" s="92"/>
-      <c r="J7" s="92"/>
-      <c r="K7" s="92"/>
-      <c r="L7" s="92"/>
-      <c r="M7" s="92"/>
-      <c r="N7" s="92"/>
-      <c r="O7" s="92"/>
-      <c r="P7" s="92"/>
-      <c r="Q7" s="92"/>
-      <c r="R7" s="92"/>
-      <c r="S7" s="92"/>
+      <c r="A7" s="107" t="s">
+        <v>279</v>
+      </c>
+      <c r="B7" s="102"/>
+      <c r="C7" s="102"/>
+      <c r="D7" s="102"/>
+      <c r="E7" s="102"/>
+      <c r="F7" s="102"/>
+      <c r="G7" s="102"/>
+      <c r="H7" s="102"/>
+      <c r="I7" s="102"/>
+      <c r="J7" s="102"/>
+      <c r="K7" s="102"/>
+      <c r="L7" s="102"/>
+      <c r="M7" s="102"/>
+      <c r="N7" s="102"/>
+      <c r="O7" s="102"/>
+      <c r="P7" s="102"/>
+      <c r="Q7" s="102"/>
+      <c r="R7" s="102"/>
+      <c r="S7" s="102"/>
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="37" t="s">
+        <v>280</v>
+      </c>
+      <c r="B8" s="110" t="s">
+        <v>281</v>
+      </c>
+      <c r="C8" s="98"/>
+      <c r="D8" s="98"/>
+      <c r="E8" s="98"/>
+      <c r="F8" s="98"/>
+      <c r="G8" s="98"/>
+      <c r="H8" s="98"/>
+      <c r="I8" s="98"/>
+      <c r="J8" s="99"/>
+      <c r="K8" s="110" t="s">
+        <v>282</v>
+      </c>
+      <c r="L8" s="98"/>
+      <c r="M8" s="98"/>
+      <c r="N8" s="98"/>
+      <c r="O8" s="98"/>
+      <c r="P8" s="98"/>
+      <c r="Q8" s="98"/>
+      <c r="R8" s="98"/>
+      <c r="S8" s="99"/>
+    </row>
+    <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B9" s="101" t="s">
         <v>278</v>
       </c>
-      <c r="B8" s="100" t="s">
-        <v>279</v>
-      </c>
-      <c r="C8" s="88"/>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="88"/>
-      <c r="G8" s="88"/>
-      <c r="H8" s="88"/>
-      <c r="I8" s="88"/>
-      <c r="J8" s="89"/>
-      <c r="K8" s="100" t="s">
-        <v>280</v>
-      </c>
-      <c r="L8" s="88"/>
-      <c r="M8" s="88"/>
-      <c r="N8" s="88"/>
-      <c r="O8" s="88"/>
-      <c r="P8" s="88"/>
-      <c r="Q8" s="88"/>
-      <c r="R8" s="88"/>
-      <c r="S8" s="89"/>
-    </row>
-    <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B9" s="91" t="s">
-        <v>276</v>
-      </c>
-      <c r="C9" s="92"/>
-      <c r="D9" s="92"/>
-      <c r="E9" s="92"/>
-      <c r="F9" s="92"/>
-      <c r="G9" s="92"/>
-      <c r="H9" s="92"/>
-      <c r="I9" s="92"/>
-      <c r="J9" s="92"/>
-      <c r="K9" s="92"/>
-      <c r="L9" s="92"/>
-      <c r="M9" s="92"/>
-      <c r="N9" s="92"/>
-      <c r="O9" s="92"/>
-      <c r="P9" s="92"/>
-      <c r="Q9" s="92"/>
-      <c r="R9" s="92"/>
-      <c r="S9" s="92"/>
+      <c r="C9" s="102"/>
+      <c r="D9" s="102"/>
+      <c r="E9" s="102"/>
+      <c r="F9" s="102"/>
+      <c r="G9" s="102"/>
+      <c r="H9" s="102"/>
+      <c r="I9" s="102"/>
+      <c r="J9" s="102"/>
+      <c r="K9" s="102"/>
+      <c r="L9" s="102"/>
+      <c r="M9" s="102"/>
+      <c r="N9" s="102"/>
+      <c r="O9" s="102"/>
+      <c r="P9" s="102"/>
+      <c r="Q9" s="102"/>
+      <c r="R9" s="102"/>
+      <c r="S9" s="102"/>
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="97" t="s">
-        <v>281</v>
-      </c>
-      <c r="B10" s="92"/>
-      <c r="C10" s="92"/>
-      <c r="D10" s="92"/>
-      <c r="E10" s="92"/>
-      <c r="F10" s="92"/>
-      <c r="G10" s="92"/>
-      <c r="H10" s="92"/>
-      <c r="I10" s="92"/>
-      <c r="J10" s="92"/>
-      <c r="K10" s="92"/>
-      <c r="L10" s="92"/>
-      <c r="M10" s="92"/>
-      <c r="N10" s="92"/>
-      <c r="O10" s="92"/>
-      <c r="P10" s="92"/>
-      <c r="Q10" s="92"/>
-      <c r="R10" s="92"/>
-      <c r="S10" s="92"/>
+      <c r="A10" s="107" t="s">
+        <v>283</v>
+      </c>
+      <c r="B10" s="102"/>
+      <c r="C10" s="102"/>
+      <c r="D10" s="102"/>
+      <c r="E10" s="102"/>
+      <c r="F10" s="102"/>
+      <c r="G10" s="102"/>
+      <c r="H10" s="102"/>
+      <c r="I10" s="102"/>
+      <c r="J10" s="102"/>
+      <c r="K10" s="102"/>
+      <c r="L10" s="102"/>
+      <c r="M10" s="102"/>
+      <c r="N10" s="102"/>
+      <c r="O10" s="102"/>
+      <c r="P10" s="102"/>
+      <c r="Q10" s="102"/>
+      <c r="R10" s="102"/>
+      <c r="S10" s="102"/>
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="37" t="s">
-        <v>282</v>
-      </c>
-      <c r="B11" s="87" t="s">
-        <v>283</v>
-      </c>
-      <c r="C11" s="88"/>
-      <c r="D11" s="89"/>
-      <c r="E11" s="87" t="s">
         <v>284</v>
       </c>
-      <c r="F11" s="88"/>
-      <c r="G11" s="89"/>
-      <c r="H11" s="87" t="s">
+      <c r="B11" s="97" t="s">
         <v>285</v>
       </c>
-      <c r="I11" s="88"/>
-      <c r="J11" s="89"/>
-      <c r="K11" s="90" t="s">
+      <c r="C11" s="98"/>
+      <c r="D11" s="99"/>
+      <c r="E11" s="97" t="s">
         <v>286</v>
       </c>
-      <c r="L11" s="88"/>
-      <c r="M11" s="89"/>
-      <c r="N11" s="87" t="s">
+      <c r="F11" s="98"/>
+      <c r="G11" s="99"/>
+      <c r="H11" s="97" t="s">
         <v>287</v>
       </c>
-      <c r="O11" s="88"/>
-      <c r="P11" s="89"/>
-      <c r="Q11" s="87" t="s">
+      <c r="I11" s="98"/>
+      <c r="J11" s="99"/>
+      <c r="K11" s="100" t="s">
         <v>288</v>
       </c>
-      <c r="R11" s="88"/>
-      <c r="S11" s="89"/>
+      <c r="L11" s="98"/>
+      <c r="M11" s="99"/>
+      <c r="N11" s="97" t="s">
+        <v>289</v>
+      </c>
+      <c r="O11" s="98"/>
+      <c r="P11" s="99"/>
+      <c r="Q11" s="97" t="s">
+        <v>290</v>
+      </c>
+      <c r="R11" s="98"/>
+      <c r="S11" s="99"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B12" s="91" t="s">
-        <v>276</v>
-      </c>
-      <c r="C12" s="92"/>
-      <c r="D12" s="92"/>
-      <c r="E12" s="92"/>
-      <c r="F12" s="92"/>
-      <c r="G12" s="92"/>
-      <c r="H12" s="92"/>
-      <c r="I12" s="92"/>
-      <c r="J12" s="92"/>
-      <c r="K12" s="92"/>
-      <c r="L12" s="92"/>
-      <c r="M12" s="92"/>
-      <c r="N12" s="92"/>
-      <c r="O12" s="92"/>
-      <c r="P12" s="92"/>
-      <c r="Q12" s="92"/>
-      <c r="R12" s="92"/>
-      <c r="S12" s="92"/>
+      <c r="B12" s="101" t="s">
+        <v>278</v>
+      </c>
+      <c r="C12" s="102"/>
+      <c r="D12" s="102"/>
+      <c r="E12" s="102"/>
+      <c r="F12" s="102"/>
+      <c r="G12" s="102"/>
+      <c r="H12" s="102"/>
+      <c r="I12" s="102"/>
+      <c r="J12" s="102"/>
+      <c r="K12" s="102"/>
+      <c r="L12" s="102"/>
+      <c r="M12" s="102"/>
+      <c r="N12" s="102"/>
+      <c r="O12" s="102"/>
+      <c r="P12" s="102"/>
+      <c r="Q12" s="102"/>
+      <c r="R12" s="102"/>
+      <c r="S12" s="102"/>
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="97" t="s">
-        <v>289</v>
-      </c>
-      <c r="B13" s="92"/>
-      <c r="C13" s="92"/>
-      <c r="D13" s="92"/>
-      <c r="E13" s="92"/>
-      <c r="F13" s="92"/>
-      <c r="G13" s="92"/>
-      <c r="H13" s="92"/>
-      <c r="I13" s="92"/>
-      <c r="J13" s="92"/>
-      <c r="K13" s="92"/>
-      <c r="L13" s="92"/>
-      <c r="M13" s="92"/>
-      <c r="N13" s="92"/>
-      <c r="O13" s="92"/>
-      <c r="P13" s="92"/>
-      <c r="Q13" s="92"/>
-      <c r="R13" s="92"/>
-      <c r="S13" s="92"/>
+      <c r="A13" s="107" t="s">
+        <v>291</v>
+      </c>
+      <c r="B13" s="102"/>
+      <c r="C13" s="102"/>
+      <c r="D13" s="102"/>
+      <c r="E13" s="102"/>
+      <c r="F13" s="102"/>
+      <c r="G13" s="102"/>
+      <c r="H13" s="102"/>
+      <c r="I13" s="102"/>
+      <c r="J13" s="102"/>
+      <c r="K13" s="102"/>
+      <c r="L13" s="102"/>
+      <c r="M13" s="102"/>
+      <c r="N13" s="102"/>
+      <c r="O13" s="102"/>
+      <c r="P13" s="102"/>
+      <c r="Q13" s="102"/>
+      <c r="R13" s="102"/>
+      <c r="S13" s="102"/>
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="37" t="s">
-        <v>290</v>
-      </c>
-      <c r="B14" s="95" t="s">
-        <v>291</v>
-      </c>
-      <c r="C14" s="88"/>
-      <c r="D14" s="88"/>
-      <c r="E14" s="88"/>
-      <c r="F14" s="88"/>
-      <c r="G14" s="89"/>
-      <c r="H14" s="95" t="s">
         <v>292</v>
       </c>
-      <c r="I14" s="88"/>
-      <c r="J14" s="88"/>
-      <c r="K14" s="88"/>
-      <c r="L14" s="88"/>
-      <c r="M14" s="89"/>
-      <c r="N14" s="95" t="s">
+      <c r="B14" s="105" t="s">
         <v>293</v>
       </c>
-      <c r="O14" s="88"/>
-      <c r="P14" s="89"/>
-      <c r="Q14" s="90" t="s">
+      <c r="C14" s="98"/>
+      <c r="D14" s="98"/>
+      <c r="E14" s="98"/>
+      <c r="F14" s="98"/>
+      <c r="G14" s="99"/>
+      <c r="H14" s="105" t="s">
         <v>294</v>
       </c>
-      <c r="R14" s="88"/>
-      <c r="S14" s="89"/>
+      <c r="I14" s="98"/>
+      <c r="J14" s="98"/>
+      <c r="K14" s="98"/>
+      <c r="L14" s="98"/>
+      <c r="M14" s="99"/>
+      <c r="N14" s="105" t="s">
+        <v>295</v>
+      </c>
+      <c r="O14" s="98"/>
+      <c r="P14" s="99"/>
+      <c r="Q14" s="100" t="s">
+        <v>296</v>
+      </c>
+      <c r="R14" s="98"/>
+      <c r="S14" s="99"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B15" s="91" t="s">
-        <v>295</v>
-      </c>
-      <c r="C15" s="92"/>
-      <c r="D15" s="92"/>
-      <c r="E15" s="92"/>
-      <c r="F15" s="92"/>
-      <c r="G15" s="92"/>
-      <c r="H15" s="92"/>
-      <c r="I15" s="92"/>
-      <c r="J15" s="92"/>
-      <c r="K15" s="92"/>
-      <c r="L15" s="92"/>
-      <c r="M15" s="92"/>
-      <c r="N15" s="92"/>
-      <c r="O15" s="92"/>
-      <c r="P15" s="92"/>
-      <c r="Q15" s="92"/>
-      <c r="R15" s="92"/>
-      <c r="S15" s="92"/>
+      <c r="B15" s="101" t="s">
+        <v>297</v>
+      </c>
+      <c r="C15" s="102"/>
+      <c r="D15" s="102"/>
+      <c r="E15" s="102"/>
+      <c r="F15" s="102"/>
+      <c r="G15" s="102"/>
+      <c r="H15" s="102"/>
+      <c r="I15" s="102"/>
+      <c r="J15" s="102"/>
+      <c r="K15" s="102"/>
+      <c r="L15" s="102"/>
+      <c r="M15" s="102"/>
+      <c r="N15" s="102"/>
+      <c r="O15" s="102"/>
+      <c r="P15" s="102"/>
+      <c r="Q15" s="102"/>
+      <c r="R15" s="102"/>
+      <c r="S15" s="102"/>
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="97" t="s">
-        <v>296</v>
-      </c>
-      <c r="B16" s="92"/>
-      <c r="C16" s="92"/>
-      <c r="D16" s="92"/>
-      <c r="E16" s="92"/>
-      <c r="F16" s="92"/>
-      <c r="G16" s="92"/>
-      <c r="H16" s="92"/>
-      <c r="I16" s="92"/>
-      <c r="J16" s="92"/>
-      <c r="K16" s="92"/>
-      <c r="L16" s="92"/>
-      <c r="M16" s="92"/>
-      <c r="N16" s="92"/>
-      <c r="O16" s="92"/>
-      <c r="P16" s="92"/>
-      <c r="Q16" s="92"/>
-      <c r="R16" s="92"/>
-      <c r="S16" s="92"/>
+      <c r="A16" s="107" t="s">
+        <v>298</v>
+      </c>
+      <c r="B16" s="102"/>
+      <c r="C16" s="102"/>
+      <c r="D16" s="102"/>
+      <c r="E16" s="102"/>
+      <c r="F16" s="102"/>
+      <c r="G16" s="102"/>
+      <c r="H16" s="102"/>
+      <c r="I16" s="102"/>
+      <c r="J16" s="102"/>
+      <c r="K16" s="102"/>
+      <c r="L16" s="102"/>
+      <c r="M16" s="102"/>
+      <c r="N16" s="102"/>
+      <c r="O16" s="102"/>
+      <c r="P16" s="102"/>
+      <c r="Q16" s="102"/>
+      <c r="R16" s="102"/>
+      <c r="S16" s="102"/>
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="37" t="s">
-        <v>297</v>
-      </c>
-      <c r="B17" s="96" t="s">
-        <v>298</v>
-      </c>
-      <c r="C17" s="88"/>
-      <c r="D17" s="88"/>
-      <c r="E17" s="88"/>
-      <c r="F17" s="88"/>
-      <c r="G17" s="89"/>
-      <c r="H17" s="96" t="s">
         <v>299</v>
       </c>
-      <c r="I17" s="88"/>
-      <c r="J17" s="89"/>
-      <c r="K17" s="96" t="s">
+      <c r="B17" s="106" t="s">
         <v>300</v>
       </c>
-      <c r="L17" s="88"/>
-      <c r="M17" s="89"/>
-      <c r="N17" s="96" t="s">
+      <c r="C17" s="98"/>
+      <c r="D17" s="98"/>
+      <c r="E17" s="98"/>
+      <c r="F17" s="98"/>
+      <c r="G17" s="99"/>
+      <c r="H17" s="106" t="s">
         <v>301</v>
       </c>
-      <c r="O17" s="88"/>
-      <c r="P17" s="89"/>
-      <c r="Q17" s="96" t="s">
+      <c r="I17" s="98"/>
+      <c r="J17" s="99"/>
+      <c r="K17" s="106" t="s">
         <v>302</v>
       </c>
-      <c r="R17" s="88"/>
-      <c r="S17" s="89"/>
+      <c r="L17" s="98"/>
+      <c r="M17" s="99"/>
+      <c r="N17" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="O17" s="98"/>
+      <c r="P17" s="99"/>
+      <c r="Q17" s="106" t="s">
+        <v>304</v>
+      </c>
+      <c r="R17" s="98"/>
+      <c r="S17" s="99"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="91" t="s">
-        <v>276</v>
-      </c>
-      <c r="C18" s="92"/>
-      <c r="D18" s="92"/>
-      <c r="E18" s="92"/>
-      <c r="F18" s="92"/>
-      <c r="G18" s="92"/>
-      <c r="H18" s="92"/>
-      <c r="I18" s="92"/>
-      <c r="J18" s="92"/>
-      <c r="K18" s="92"/>
-      <c r="L18" s="92"/>
-      <c r="M18" s="92"/>
-      <c r="N18" s="92"/>
-      <c r="O18" s="92"/>
-      <c r="P18" s="92"/>
-      <c r="Q18" s="92"/>
-      <c r="R18" s="92"/>
-      <c r="S18" s="92"/>
+      <c r="B18" s="101" t="s">
+        <v>278</v>
+      </c>
+      <c r="C18" s="102"/>
+      <c r="D18" s="102"/>
+      <c r="E18" s="102"/>
+      <c r="F18" s="102"/>
+      <c r="G18" s="102"/>
+      <c r="H18" s="102"/>
+      <c r="I18" s="102"/>
+      <c r="J18" s="102"/>
+      <c r="K18" s="102"/>
+      <c r="L18" s="102"/>
+      <c r="M18" s="102"/>
+      <c r="N18" s="102"/>
+      <c r="O18" s="102"/>
+      <c r="P18" s="102"/>
+      <c r="Q18" s="102"/>
+      <c r="R18" s="102"/>
+      <c r="S18" s="102"/>
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="97" t="s">
-        <v>303</v>
-      </c>
-      <c r="B19" s="92"/>
-      <c r="C19" s="92"/>
-      <c r="D19" s="92"/>
-      <c r="E19" s="92"/>
-      <c r="F19" s="92"/>
-      <c r="G19" s="92"/>
-      <c r="H19" s="92"/>
-      <c r="I19" s="92"/>
-      <c r="J19" s="92"/>
-      <c r="K19" s="92"/>
-      <c r="L19" s="92"/>
-      <c r="M19" s="92"/>
-      <c r="N19" s="92"/>
-      <c r="O19" s="92"/>
-      <c r="P19" s="92"/>
-      <c r="Q19" s="92"/>
-      <c r="R19" s="92"/>
-      <c r="S19" s="92"/>
+      <c r="A19" s="107" t="s">
+        <v>305</v>
+      </c>
+      <c r="B19" s="102"/>
+      <c r="C19" s="102"/>
+      <c r="D19" s="102"/>
+      <c r="E19" s="102"/>
+      <c r="F19" s="102"/>
+      <c r="G19" s="102"/>
+      <c r="H19" s="102"/>
+      <c r="I19" s="102"/>
+      <c r="J19" s="102"/>
+      <c r="K19" s="102"/>
+      <c r="L19" s="102"/>
+      <c r="M19" s="102"/>
+      <c r="N19" s="102"/>
+      <c r="O19" s="102"/>
+      <c r="P19" s="102"/>
+      <c r="Q19" s="102"/>
+      <c r="R19" s="102"/>
+      <c r="S19" s="102"/>
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="37" t="s">
-        <v>304</v>
-      </c>
-      <c r="B20" s="98" t="s">
-        <v>305</v>
-      </c>
-      <c r="C20" s="88"/>
-      <c r="D20" s="88"/>
-      <c r="E20" s="88"/>
-      <c r="F20" s="88"/>
-      <c r="G20" s="89"/>
-      <c r="H20" s="98" t="s">
         <v>306</v>
       </c>
-      <c r="I20" s="88"/>
-      <c r="J20" s="88"/>
-      <c r="K20" s="88"/>
-      <c r="L20" s="88"/>
-      <c r="M20" s="89"/>
-      <c r="N20" s="98" t="s">
+      <c r="B20" s="108" t="s">
         <v>307</v>
       </c>
-      <c r="O20" s="88"/>
-      <c r="P20" s="88"/>
-      <c r="Q20" s="88"/>
-      <c r="R20" s="88"/>
-      <c r="S20" s="89"/>
+      <c r="C20" s="98"/>
+      <c r="D20" s="98"/>
+      <c r="E20" s="98"/>
+      <c r="F20" s="98"/>
+      <c r="G20" s="99"/>
+      <c r="H20" s="108" t="s">
+        <v>308</v>
+      </c>
+      <c r="I20" s="98"/>
+      <c r="J20" s="98"/>
+      <c r="K20" s="98"/>
+      <c r="L20" s="98"/>
+      <c r="M20" s="99"/>
+      <c r="N20" s="108" t="s">
+        <v>309</v>
+      </c>
+      <c r="O20" s="98"/>
+      <c r="P20" s="98"/>
+      <c r="Q20" s="98"/>
+      <c r="R20" s="98"/>
+      <c r="S20" s="99"/>
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B21" s="91" t="s">
-        <v>276</v>
-      </c>
-      <c r="C21" s="92"/>
-      <c r="D21" s="92"/>
-      <c r="E21" s="92"/>
-      <c r="F21" s="92"/>
-      <c r="G21" s="92"/>
-      <c r="H21" s="92"/>
-      <c r="I21" s="92"/>
-      <c r="J21" s="92"/>
-      <c r="K21" s="92"/>
-      <c r="L21" s="92"/>
-      <c r="M21" s="92"/>
-      <c r="N21" s="92"/>
-      <c r="O21" s="92"/>
-      <c r="P21" s="92"/>
-      <c r="Q21" s="92"/>
-      <c r="R21" s="92"/>
-      <c r="S21" s="92"/>
+      <c r="B21" s="101" t="s">
+        <v>278</v>
+      </c>
+      <c r="C21" s="102"/>
+      <c r="D21" s="102"/>
+      <c r="E21" s="102"/>
+      <c r="F21" s="102"/>
+      <c r="G21" s="102"/>
+      <c r="H21" s="102"/>
+      <c r="I21" s="102"/>
+      <c r="J21" s="102"/>
+      <c r="K21" s="102"/>
+      <c r="L21" s="102"/>
+      <c r="M21" s="102"/>
+      <c r="N21" s="102"/>
+      <c r="O21" s="102"/>
+      <c r="P21" s="102"/>
+      <c r="Q21" s="102"/>
+      <c r="R21" s="102"/>
+      <c r="S21" s="102"/>
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="97" t="s">
-        <v>308</v>
-      </c>
-      <c r="B22" s="92"/>
-      <c r="C22" s="92"/>
-      <c r="D22" s="92"/>
-      <c r="E22" s="92"/>
-      <c r="F22" s="92"/>
-      <c r="G22" s="92"/>
-      <c r="H22" s="92"/>
-      <c r="I22" s="92"/>
-      <c r="J22" s="92"/>
-      <c r="K22" s="92"/>
-      <c r="L22" s="92"/>
-      <c r="M22" s="92"/>
-      <c r="N22" s="92"/>
-      <c r="O22" s="92"/>
-      <c r="P22" s="92"/>
-      <c r="Q22" s="92"/>
-      <c r="R22" s="92"/>
-      <c r="S22" s="92"/>
+      <c r="A22" s="107" t="s">
+        <v>310</v>
+      </c>
+      <c r="B22" s="102"/>
+      <c r="C22" s="102"/>
+      <c r="D22" s="102"/>
+      <c r="E22" s="102"/>
+      <c r="F22" s="102"/>
+      <c r="G22" s="102"/>
+      <c r="H22" s="102"/>
+      <c r="I22" s="102"/>
+      <c r="J22" s="102"/>
+      <c r="K22" s="102"/>
+      <c r="L22" s="102"/>
+      <c r="M22" s="102"/>
+      <c r="N22" s="102"/>
+      <c r="O22" s="102"/>
+      <c r="P22" s="102"/>
+      <c r="Q22" s="102"/>
+      <c r="R22" s="102"/>
+      <c r="S22" s="102"/>
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="37" t="s">
-        <v>309</v>
-      </c>
-      <c r="B23" s="98" t="s">
-        <v>310</v>
-      </c>
-      <c r="C23" s="88"/>
-      <c r="D23" s="88"/>
-      <c r="E23" s="88"/>
-      <c r="F23" s="88"/>
-      <c r="G23" s="89"/>
-      <c r="H23" s="98" t="s">
         <v>311</v>
       </c>
-      <c r="I23" s="88"/>
-      <c r="J23" s="89"/>
-      <c r="K23" s="98" t="s">
+      <c r="B23" s="108" t="s">
         <v>312</v>
       </c>
-      <c r="L23" s="88"/>
-      <c r="M23" s="89"/>
-      <c r="N23" s="98" t="s">
+      <c r="C23" s="98"/>
+      <c r="D23" s="98"/>
+      <c r="E23" s="98"/>
+      <c r="F23" s="98"/>
+      <c r="G23" s="99"/>
+      <c r="H23" s="108" t="s">
         <v>313</v>
       </c>
-      <c r="O23" s="88"/>
-      <c r="P23" s="89"/>
-      <c r="Q23" s="94" t="s">
+      <c r="I23" s="98"/>
+      <c r="J23" s="99"/>
+      <c r="K23" s="108" t="s">
         <v>314</v>
       </c>
-      <c r="R23" s="88"/>
-      <c r="S23" s="89"/>
+      <c r="L23" s="98"/>
+      <c r="M23" s="99"/>
+      <c r="N23" s="108" t="s">
+        <v>315</v>
+      </c>
+      <c r="O23" s="98"/>
+      <c r="P23" s="99"/>
+      <c r="Q23" s="104" t="s">
+        <v>316</v>
+      </c>
+      <c r="R23" s="98"/>
+      <c r="S23" s="99"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="103" t="s">
-        <v>315</v>
-      </c>
-      <c r="B26" s="92"/>
-      <c r="C26" s="92"/>
-      <c r="D26" s="92"/>
-      <c r="E26" s="92"/>
-      <c r="F26" s="92"/>
-      <c r="G26" s="92"/>
-      <c r="H26" s="92"/>
-      <c r="I26" s="92"/>
-      <c r="J26" s="92"/>
-      <c r="K26" s="92"/>
-      <c r="L26" s="92"/>
-      <c r="M26" s="92"/>
-      <c r="N26" s="92"/>
-      <c r="O26" s="92"/>
-      <c r="P26" s="92"/>
-      <c r="Q26" s="92"/>
-      <c r="R26" s="92"/>
-      <c r="S26" s="92"/>
+      <c r="A26" s="113" t="s">
+        <v>317</v>
+      </c>
+      <c r="B26" s="102"/>
+      <c r="C26" s="102"/>
+      <c r="D26" s="102"/>
+      <c r="E26" s="102"/>
+      <c r="F26" s="102"/>
+      <c r="G26" s="102"/>
+      <c r="H26" s="102"/>
+      <c r="I26" s="102"/>
+      <c r="J26" s="102"/>
+      <c r="K26" s="102"/>
+      <c r="L26" s="102"/>
+      <c r="M26" s="102"/>
+      <c r="N26" s="102"/>
+      <c r="O26" s="102"/>
+      <c r="P26" s="102"/>
+      <c r="Q26" s="102"/>
+      <c r="R26" s="102"/>
+      <c r="S26" s="102"/>
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="37" t="s">
-        <v>316</v>
-      </c>
-      <c r="B27" s="87" t="s">
-        <v>317</v>
-      </c>
-      <c r="C27" s="88"/>
-      <c r="D27" s="89"/>
-      <c r="E27" s="87" t="s">
         <v>318</v>
       </c>
-      <c r="F27" s="88"/>
-      <c r="G27" s="89"/>
-      <c r="H27" s="95" t="s">
+      <c r="B27" s="97" t="s">
         <v>319</v>
       </c>
-      <c r="I27" s="88"/>
-      <c r="J27" s="89"/>
-      <c r="K27" s="96" t="s">
+      <c r="C27" s="98"/>
+      <c r="D27" s="99"/>
+      <c r="E27" s="97" t="s">
         <v>320</v>
       </c>
-      <c r="L27" s="88"/>
-      <c r="M27" s="89"/>
-      <c r="N27" s="96" t="s">
+      <c r="F27" s="98"/>
+      <c r="G27" s="99"/>
+      <c r="H27" s="105" t="s">
         <v>321</v>
       </c>
-      <c r="O27" s="88"/>
-      <c r="P27" s="89"/>
-      <c r="Q27" s="95" t="s">
+      <c r="I27" s="98"/>
+      <c r="J27" s="99"/>
+      <c r="K27" s="106" t="s">
         <v>322</v>
       </c>
-      <c r="R27" s="88"/>
-      <c r="S27" s="89"/>
+      <c r="L27" s="98"/>
+      <c r="M27" s="99"/>
+      <c r="N27" s="106" t="s">
+        <v>323</v>
+      </c>
+      <c r="O27" s="98"/>
+      <c r="P27" s="99"/>
+      <c r="Q27" s="105" t="s">
+        <v>324</v>
+      </c>
+      <c r="R27" s="98"/>
+      <c r="S27" s="99"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="97" t="s">
-        <v>323</v>
-      </c>
-      <c r="B30" s="92"/>
-      <c r="C30" s="92"/>
-      <c r="D30" s="92"/>
-      <c r="E30" s="92"/>
-      <c r="F30" s="92"/>
-      <c r="G30" s="92"/>
-      <c r="H30" s="92"/>
-      <c r="I30" s="92"/>
-      <c r="J30" s="92"/>
-      <c r="K30" s="92"/>
-      <c r="L30" s="92"/>
-      <c r="M30" s="92"/>
-      <c r="N30" s="92"/>
-      <c r="O30" s="92"/>
-      <c r="P30" s="92"/>
-      <c r="Q30" s="92"/>
-      <c r="R30" s="92"/>
-      <c r="S30" s="92"/>
+      <c r="A30" s="107" t="s">
+        <v>325</v>
+      </c>
+      <c r="B30" s="102"/>
+      <c r="C30" s="102"/>
+      <c r="D30" s="102"/>
+      <c r="E30" s="102"/>
+      <c r="F30" s="102"/>
+      <c r="G30" s="102"/>
+      <c r="H30" s="102"/>
+      <c r="I30" s="102"/>
+      <c r="J30" s="102"/>
+      <c r="K30" s="102"/>
+      <c r="L30" s="102"/>
+      <c r="M30" s="102"/>
+      <c r="N30" s="102"/>
+      <c r="O30" s="102"/>
+      <c r="P30" s="102"/>
+      <c r="Q30" s="102"/>
+      <c r="R30" s="102"/>
+      <c r="S30" s="102"/>
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="93" t="s">
-        <v>324</v>
-      </c>
-      <c r="B31" s="92"/>
-      <c r="C31" s="92"/>
-      <c r="D31" s="92"/>
-      <c r="E31" s="92"/>
-      <c r="F31" s="92"/>
-      <c r="G31" s="92"/>
-      <c r="H31" s="92"/>
-      <c r="I31" s="92"/>
-      <c r="J31" s="92"/>
-      <c r="K31" s="92"/>
-      <c r="L31" s="92"/>
-      <c r="M31" s="92"/>
-      <c r="N31" s="92"/>
-      <c r="O31" s="92"/>
-      <c r="P31" s="92"/>
-      <c r="Q31" s="92"/>
-      <c r="R31" s="92"/>
-      <c r="S31" s="92"/>
+      <c r="A31" s="103" t="s">
+        <v>326</v>
+      </c>
+      <c r="B31" s="102"/>
+      <c r="C31" s="102"/>
+      <c r="D31" s="102"/>
+      <c r="E31" s="102"/>
+      <c r="F31" s="102"/>
+      <c r="G31" s="102"/>
+      <c r="H31" s="102"/>
+      <c r="I31" s="102"/>
+      <c r="J31" s="102"/>
+      <c r="K31" s="102"/>
+      <c r="L31" s="102"/>
+      <c r="M31" s="102"/>
+      <c r="N31" s="102"/>
+      <c r="O31" s="102"/>
+      <c r="P31" s="102"/>
+      <c r="Q31" s="102"/>
+      <c r="R31" s="102"/>
+      <c r="S31" s="102"/>
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="93" t="s">
-        <v>325</v>
-      </c>
-      <c r="B32" s="92"/>
-      <c r="C32" s="92"/>
-      <c r="D32" s="92"/>
-      <c r="E32" s="92"/>
-      <c r="F32" s="92"/>
-      <c r="G32" s="92"/>
-      <c r="H32" s="92"/>
-      <c r="I32" s="92"/>
-      <c r="J32" s="92"/>
-      <c r="K32" s="92"/>
-      <c r="L32" s="92"/>
-      <c r="M32" s="92"/>
-      <c r="N32" s="92"/>
-      <c r="O32" s="92"/>
-      <c r="P32" s="92"/>
-      <c r="Q32" s="92"/>
-      <c r="R32" s="92"/>
-      <c r="S32" s="92"/>
+      <c r="A32" s="103" t="s">
+        <v>327</v>
+      </c>
+      <c r="B32" s="102"/>
+      <c r="C32" s="102"/>
+      <c r="D32" s="102"/>
+      <c r="E32" s="102"/>
+      <c r="F32" s="102"/>
+      <c r="G32" s="102"/>
+      <c r="H32" s="102"/>
+      <c r="I32" s="102"/>
+      <c r="J32" s="102"/>
+      <c r="K32" s="102"/>
+      <c r="L32" s="102"/>
+      <c r="M32" s="102"/>
+      <c r="N32" s="102"/>
+      <c r="O32" s="102"/>
+      <c r="P32" s="102"/>
+      <c r="Q32" s="102"/>
+      <c r="R32" s="102"/>
+      <c r="S32" s="102"/>
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="93" t="s">
-        <v>326</v>
-      </c>
-      <c r="B33" s="92"/>
-      <c r="C33" s="92"/>
-      <c r="D33" s="92"/>
-      <c r="E33" s="92"/>
-      <c r="F33" s="92"/>
-      <c r="G33" s="92"/>
-      <c r="H33" s="92"/>
-      <c r="I33" s="92"/>
-      <c r="J33" s="92"/>
-      <c r="K33" s="92"/>
-      <c r="L33" s="92"/>
-      <c r="M33" s="92"/>
-      <c r="N33" s="92"/>
-      <c r="O33" s="92"/>
-      <c r="P33" s="92"/>
-      <c r="Q33" s="92"/>
-      <c r="R33" s="92"/>
-      <c r="S33" s="92"/>
+      <c r="A33" s="103" t="s">
+        <v>328</v>
+      </c>
+      <c r="B33" s="102"/>
+      <c r="C33" s="102"/>
+      <c r="D33" s="102"/>
+      <c r="E33" s="102"/>
+      <c r="F33" s="102"/>
+      <c r="G33" s="102"/>
+      <c r="H33" s="102"/>
+      <c r="I33" s="102"/>
+      <c r="J33" s="102"/>
+      <c r="K33" s="102"/>
+      <c r="L33" s="102"/>
+      <c r="M33" s="102"/>
+      <c r="N33" s="102"/>
+      <c r="O33" s="102"/>
+      <c r="P33" s="102"/>
+      <c r="Q33" s="102"/>
+      <c r="R33" s="102"/>
+      <c r="S33" s="102"/>
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="93" t="s">
-        <v>327</v>
-      </c>
-      <c r="B34" s="92"/>
-      <c r="C34" s="92"/>
-      <c r="D34" s="92"/>
-      <c r="E34" s="92"/>
-      <c r="F34" s="92"/>
-      <c r="G34" s="92"/>
-      <c r="H34" s="92"/>
-      <c r="I34" s="92"/>
-      <c r="J34" s="92"/>
-      <c r="K34" s="92"/>
-      <c r="L34" s="92"/>
-      <c r="M34" s="92"/>
-      <c r="N34" s="92"/>
-      <c r="O34" s="92"/>
-      <c r="P34" s="92"/>
-      <c r="Q34" s="92"/>
-      <c r="R34" s="92"/>
-      <c r="S34" s="92"/>
+      <c r="A34" s="103" t="s">
+        <v>329</v>
+      </c>
+      <c r="B34" s="102"/>
+      <c r="C34" s="102"/>
+      <c r="D34" s="102"/>
+      <c r="E34" s="102"/>
+      <c r="F34" s="102"/>
+      <c r="G34" s="102"/>
+      <c r="H34" s="102"/>
+      <c r="I34" s="102"/>
+      <c r="J34" s="102"/>
+      <c r="K34" s="102"/>
+      <c r="L34" s="102"/>
+      <c r="M34" s="102"/>
+      <c r="N34" s="102"/>
+      <c r="O34" s="102"/>
+      <c r="P34" s="102"/>
+      <c r="Q34" s="102"/>
+      <c r="R34" s="102"/>
+      <c r="S34" s="102"/>
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="93" t="s">
-        <v>328</v>
-      </c>
-      <c r="B35" s="92"/>
-      <c r="C35" s="92"/>
-      <c r="D35" s="92"/>
-      <c r="E35" s="92"/>
-      <c r="F35" s="92"/>
-      <c r="G35" s="92"/>
-      <c r="H35" s="92"/>
-      <c r="I35" s="92"/>
-      <c r="J35" s="92"/>
-      <c r="K35" s="92"/>
-      <c r="L35" s="92"/>
-      <c r="M35" s="92"/>
-      <c r="N35" s="92"/>
-      <c r="O35" s="92"/>
-      <c r="P35" s="92"/>
-      <c r="Q35" s="92"/>
-      <c r="R35" s="92"/>
-      <c r="S35" s="92"/>
+      <c r="A35" s="103" t="s">
+        <v>330</v>
+      </c>
+      <c r="B35" s="102"/>
+      <c r="C35" s="102"/>
+      <c r="D35" s="102"/>
+      <c r="E35" s="102"/>
+      <c r="F35" s="102"/>
+      <c r="G35" s="102"/>
+      <c r="H35" s="102"/>
+      <c r="I35" s="102"/>
+      <c r="J35" s="102"/>
+      <c r="K35" s="102"/>
+      <c r="L35" s="102"/>
+      <c r="M35" s="102"/>
+      <c r="N35" s="102"/>
+      <c r="O35" s="102"/>
+      <c r="P35" s="102"/>
+      <c r="Q35" s="102"/>
+      <c r="R35" s="102"/>
+      <c r="S35" s="102"/>
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="93" t="s">
-        <v>329</v>
-      </c>
-      <c r="B36" s="92"/>
-      <c r="C36" s="92"/>
-      <c r="D36" s="92"/>
-      <c r="E36" s="92"/>
-      <c r="F36" s="92"/>
-      <c r="G36" s="92"/>
-      <c r="H36" s="92"/>
-      <c r="I36" s="92"/>
-      <c r="J36" s="92"/>
-      <c r="K36" s="92"/>
-      <c r="L36" s="92"/>
-      <c r="M36" s="92"/>
-      <c r="N36" s="92"/>
-      <c r="O36" s="92"/>
-      <c r="P36" s="92"/>
-      <c r="Q36" s="92"/>
-      <c r="R36" s="92"/>
-      <c r="S36" s="92"/>
+      <c r="A36" s="103" t="s">
+        <v>331</v>
+      </c>
+      <c r="B36" s="102"/>
+      <c r="C36" s="102"/>
+      <c r="D36" s="102"/>
+      <c r="E36" s="102"/>
+      <c r="F36" s="102"/>
+      <c r="G36" s="102"/>
+      <c r="H36" s="102"/>
+      <c r="I36" s="102"/>
+      <c r="J36" s="102"/>
+      <c r="K36" s="102"/>
+      <c r="L36" s="102"/>
+      <c r="M36" s="102"/>
+      <c r="N36" s="102"/>
+      <c r="O36" s="102"/>
+      <c r="P36" s="102"/>
+      <c r="Q36" s="102"/>
+      <c r="R36" s="102"/>
+      <c r="S36" s="102"/>
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="104" t="s">
-        <v>330</v>
-      </c>
-      <c r="B37" s="92"/>
-      <c r="C37" s="92"/>
-      <c r="D37" s="92"/>
-      <c r="E37" s="92"/>
-      <c r="F37" s="92"/>
-      <c r="G37" s="92"/>
-      <c r="H37" s="92"/>
-      <c r="I37" s="92"/>
-      <c r="J37" s="92"/>
-      <c r="K37" s="92"/>
-      <c r="L37" s="92"/>
-      <c r="M37" s="92"/>
-      <c r="N37" s="92"/>
-      <c r="O37" s="92"/>
-      <c r="P37" s="92"/>
-      <c r="Q37" s="92"/>
-      <c r="R37" s="92"/>
-      <c r="S37" s="92"/>
+      <c r="A37" s="114" t="s">
+        <v>332</v>
+      </c>
+      <c r="B37" s="102"/>
+      <c r="C37" s="102"/>
+      <c r="D37" s="102"/>
+      <c r="E37" s="102"/>
+      <c r="F37" s="102"/>
+      <c r="G37" s="102"/>
+      <c r="H37" s="102"/>
+      <c r="I37" s="102"/>
+      <c r="J37" s="102"/>
+      <c r="K37" s="102"/>
+      <c r="L37" s="102"/>
+      <c r="M37" s="102"/>
+      <c r="N37" s="102"/>
+      <c r="O37" s="102"/>
+      <c r="P37" s="102"/>
+      <c r="Q37" s="102"/>
+      <c r="R37" s="102"/>
+      <c r="S37" s="102"/>
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="38" t="s">
-        <v>265</v>
-      </c>
-      <c r="B39" s="107" t="s">
-        <v>331</v>
-      </c>
-      <c r="C39" s="92"/>
-      <c r="D39" s="92"/>
-      <c r="E39" s="105" t="s">
-        <v>332</v>
-      </c>
-      <c r="F39" s="92"/>
-      <c r="G39" s="92"/>
-      <c r="H39" s="108" t="s">
+        <v>267</v>
+      </c>
+      <c r="B39" s="117" t="s">
         <v>333</v>
       </c>
-      <c r="I39" s="92"/>
-      <c r="J39" s="92"/>
-      <c r="K39" s="101" t="s">
+      <c r="C39" s="102"/>
+      <c r="D39" s="102"/>
+      <c r="E39" s="115" t="s">
         <v>334</v>
       </c>
-      <c r="L39" s="92"/>
-      <c r="M39" s="92"/>
-      <c r="N39" s="99" t="s">
+      <c r="F39" s="102"/>
+      <c r="G39" s="102"/>
+      <c r="H39" s="118" t="s">
+        <v>335</v>
+      </c>
+      <c r="I39" s="102"/>
+      <c r="J39" s="102"/>
+      <c r="K39" s="111" t="s">
+        <v>336</v>
+      </c>
+      <c r="L39" s="102"/>
+      <c r="M39" s="102"/>
+      <c r="N39" s="109" t="s">
         <v>45</v>
       </c>
-      <c r="O39" s="92"/>
-      <c r="P39" s="92"/>
-      <c r="Q39" s="106" t="s">
-        <v>335</v>
-      </c>
-      <c r="R39" s="92"/>
-      <c r="S39" s="92"/>
+      <c r="O39" s="102"/>
+      <c r="P39" s="102"/>
+      <c r="Q39" s="116" t="s">
+        <v>337</v>
+      </c>
+      <c r="R39" s="102"/>
+      <c r="S39" s="102"/>
     </row>
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H14:M14"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="H20:M20"/>
     <mergeCell ref="A16:S16"/>
-    <mergeCell ref="H20:M20"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -7400,13 +7531,14 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -7415,7 +7547,6 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
-    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -7423,7 +7554,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -7471,33 +7602,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="110" t="s">
-        <v>336</v>
-      </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="84"/>
-      <c r="F1" s="85"/>
+      <c r="A1" s="120" t="s">
+        <v>338</v>
+      </c>
+      <c r="B1" s="94"/>
+      <c r="C1" s="94"/>
+      <c r="D1" s="94"/>
+      <c r="E1" s="94"/>
+      <c r="F1" s="95"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -7731,11 +7862,11 @@
       </c>
       <c r="B13" s="26">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C13" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D13" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -7747,7 +7878,7 @@
       </c>
       <c r="F13" s="27">
         <f t="shared" si="1"/>
-        <v>0.36363636363636365</v>
+        <v>0.39130434782608697</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -7777,15 +7908,15 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="28" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B16" s="29">
         <f>SUM(B4:B14)</f>
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C16" s="29">
         <f>SUM(C4:C14)</f>
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
@@ -7797,12 +7928,12 @@
       </c>
       <c r="F16" s="30">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.66666666666666663</v>
+        <v>0.6696428571428571</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="43" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B18" s="44">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -7811,7 +7942,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="45" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -7832,7 +7963,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -7843,471 +7974,488 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="110" t="s">
-        <v>343</v>
-      </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="85"/>
+      <c r="A1" s="120" t="s">
+        <v>345</v>
+      </c>
+      <c r="B1" s="94"/>
+      <c r="C1" s="94"/>
+      <c r="D1" s="94"/>
+      <c r="E1" s="95"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="31" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="D3" s="31" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="32" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="34" t="s">
+        <v>355</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>356</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>353</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>349</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>354</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>351</v>
-      </c>
       <c r="E5" s="35" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="32" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="34" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="32" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="34" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="32" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="34" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="32" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="34" t="s">
+        <v>379</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>364</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>377</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>357</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>362</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>375</v>
-      </c>
       <c r="E13" s="35" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="32" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="34" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="32" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="34" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="34" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="32" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="34" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="32" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E22" s="33" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="34" t="s">
+        <v>403</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>401</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>399</v>
-      </c>
       <c r="C23" s="19" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E23" s="35" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="32" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="58" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B25" s="55" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C25" s="59" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D25" s="55" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E25" s="60" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="61" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B26" s="49" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C26" s="59" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="D26" s="49" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E26" s="62" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="58" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B27" s="55" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C27" s="59" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="D27" s="55" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E27" s="60" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="79" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B28" s="66" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C28" s="75" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D28" s="66" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E28" s="80" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="81" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B29" s="72" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C29" s="77" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D29" s="72" t="s">
+        <v>353</v>
+      </c>
+      <c r="E29" s="82" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A30" s="90" t="s">
+        <v>417</v>
+      </c>
+      <c r="B30" s="86" t="s">
         <v>351</v>
       </c>
-      <c r="E29" s="82" t="s">
-        <v>414</v>
+      <c r="C30" s="91" t="s">
+        <v>364</v>
+      </c>
+      <c r="D30" s="86" t="s">
+        <v>353</v>
+      </c>
+      <c r="E30" s="92" t="s">
+        <v>418</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(tracker): google-services.json wired; API-key restriction queued
E10 Deploy 30 items, 12 done.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4791C773-2BE2-4DF7-B14B-9A04967B5708}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A39AFE9-161D-4D5F-8A25-21B492BB1476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14895" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="826" uniqueCount="446">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -885,6 +885,18 @@
   </si>
   <si>
     <t>The only way to prove delivery; Expo Go on Android cannot receive push</t>
+  </si>
+  <si>
+    <t>google-services.json wired into the Android build</t>
+  </si>
+  <si>
+    <t>package_name verified as an exact match before wiring; same project as the FCM key</t>
+  </si>
+  <si>
+    <t>Restrict Android API key to package + SHA-1 (GCP)</t>
+  </si>
+  <si>
+    <t>Repo is public; 2 min in Cloud Console makes the shipped key useless to others</t>
   </si>
   <si>
     <t>Legend</t>
@@ -1443,7 +1455,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\ mmm"/>
   </numFmts>
-  <fonts count="42" x14ac:knownFonts="1">
+  <fonts count="46" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1680,8 +1692,30 @@
       <color rgb="FF6B7280"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF111827"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF111827"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF6B7280"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="36">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1858,8 +1892,28 @@
         <fgColor rgb="FF94A3B8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF16A34A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF94A3B8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -2020,11 +2074,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="154">
+  <cellXfs count="168">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2399,12 +2468,54 @@
     <xf numFmtId="0" fontId="39" fillId="32" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="42" fillId="36" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="36" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="37" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="36" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="43" fillId="36" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="36" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="37" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="38" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="38" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="39" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="38" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="43" fillId="38" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="38" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="39" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2470,7 +2581,7 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2790,7 +2901,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R126"/>
+  <dimension ref="A1:R128"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2804,46 +2915,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="129" t="s">
+      <c r="A1" s="143" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="127"/>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
-      <c r="I1" s="127"/>
-      <c r="J1" s="127"/>
-      <c r="K1" s="127"/>
-      <c r="L1" s="127"/>
-      <c r="M1" s="127"/>
-      <c r="N1" s="127"/>
-      <c r="O1" s="127"/>
-      <c r="P1" s="127"/>
-      <c r="Q1" s="128"/>
+      <c r="B1" s="141"/>
+      <c r="C1" s="141"/>
+      <c r="D1" s="141"/>
+      <c r="E1" s="141"/>
+      <c r="F1" s="141"/>
+      <c r="G1" s="141"/>
+      <c r="H1" s="141"/>
+      <c r="I1" s="141"/>
+      <c r="J1" s="141"/>
+      <c r="K1" s="141"/>
+      <c r="L1" s="141"/>
+      <c r="M1" s="141"/>
+      <c r="N1" s="141"/>
+      <c r="O1" s="141"/>
+      <c r="P1" s="141"/>
+      <c r="Q1" s="142"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="126" t="s">
+      <c r="A2" s="140" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="127"/>
-      <c r="C2" s="127"/>
-      <c r="D2" s="127"/>
-      <c r="E2" s="127"/>
-      <c r="F2" s="127"/>
-      <c r="G2" s="127"/>
-      <c r="H2" s="127"/>
-      <c r="I2" s="127"/>
-      <c r="J2" s="127"/>
-      <c r="K2" s="127"/>
-      <c r="L2" s="127"/>
-      <c r="M2" s="127"/>
-      <c r="N2" s="127"/>
-      <c r="O2" s="127"/>
-      <c r="P2" s="127"/>
-      <c r="Q2" s="128"/>
+      <c r="B2" s="141"/>
+      <c r="C2" s="141"/>
+      <c r="D2" s="141"/>
+      <c r="E2" s="141"/>
+      <c r="F2" s="141"/>
+      <c r="G2" s="141"/>
+      <c r="H2" s="141"/>
+      <c r="I2" s="141"/>
+      <c r="J2" s="141"/>
+      <c r="K2" s="141"/>
+      <c r="L2" s="141"/>
+      <c r="M2" s="141"/>
+      <c r="N2" s="141"/>
+      <c r="O2" s="141"/>
+      <c r="P2" s="141"/>
+      <c r="Q2" s="142"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
@@ -6397,7 +6508,7 @@
       <c r="P102" s="11"/>
       <c r="Q102" s="11"/>
       <c r="R102" t="str">
-        <f t="shared" ref="R102:R124" si="3">IF($A102&lt;&gt;"",$A102,R101)</f>
+        <f t="shared" ref="R102:R126" si="3">IF($A102&lt;&gt;"",$A102,R101)</f>
         <v>E9 Data Ops</v>
       </c>
     </row>
@@ -7215,23 +7326,97 @@
         <v>E10 Deploy</v>
       </c>
     </row>
+    <row r="125" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A125" s="126" t="s">
+        <v>162</v>
+      </c>
+      <c r="B125" s="127" t="s">
+        <v>283</v>
+      </c>
+      <c r="C125" s="128" t="s">
+        <v>22</v>
+      </c>
+      <c r="D125" s="129" t="s">
+        <v>85</v>
+      </c>
+      <c r="E125" s="130">
+        <v>46238</v>
+      </c>
+      <c r="F125" s="130">
+        <v>46238</v>
+      </c>
+      <c r="G125" s="131" t="s">
+        <v>284</v>
+      </c>
+      <c r="H125" s="127"/>
+      <c r="I125" s="132"/>
+      <c r="J125" s="127"/>
+      <c r="K125" s="127"/>
+      <c r="L125" s="127"/>
+      <c r="M125" s="127"/>
+      <c r="N125" s="127"/>
+      <c r="O125" s="127"/>
+      <c r="P125" s="127"/>
+      <c r="Q125" s="127"/>
+      <c r="R125" t="str">
+        <f t="shared" si="3"/>
+        <v>E10 Deploy</v>
+      </c>
+    </row>
     <row r="126" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A126" s="25" t="s">
-        <v>283</v>
-      </c>
-      <c r="B126" s="5" t="s">
+      <c r="A126" s="133" t="s">
+        <v>162</v>
+      </c>
+      <c r="B126" s="134" t="s">
+        <v>285</v>
+      </c>
+      <c r="C126" s="135" t="s">
+        <v>128</v>
+      </c>
+      <c r="D126" s="136" t="s">
+        <v>85</v>
+      </c>
+      <c r="E126" s="137">
+        <v>46239</v>
+      </c>
+      <c r="F126" s="137">
+        <v>46239</v>
+      </c>
+      <c r="G126" s="138" t="s">
+        <v>286</v>
+      </c>
+      <c r="H126" s="134"/>
+      <c r="I126" s="139"/>
+      <c r="J126" s="134"/>
+      <c r="K126" s="134"/>
+      <c r="L126" s="134"/>
+      <c r="M126" s="134"/>
+      <c r="N126" s="134"/>
+      <c r="O126" s="134"/>
+      <c r="P126" s="134"/>
+      <c r="Q126" s="134"/>
+      <c r="R126" t="str">
+        <f t="shared" si="3"/>
+        <v>E10 Deploy</v>
+      </c>
+    </row>
+    <row r="128" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A128" s="25" t="s">
+        <v>287</v>
+      </c>
+      <c r="B128" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C126" s="17" t="s">
+      <c r="C128" s="17" t="s">
         <v>231</v>
       </c>
-      <c r="D126" s="19" t="s">
+      <c r="D128" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="E126" s="23" t="s">
+      <c r="E128" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="F126" s="21" t="s">
+      <c r="F128" s="21" t="s">
         <v>136</v>
       </c>
     </row>
@@ -7255,852 +7440,852 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="145" t="s">
-        <v>284</v>
-      </c>
-      <c r="B1" s="135"/>
-      <c r="C1" s="135"/>
-      <c r="D1" s="135"/>
-      <c r="E1" s="135"/>
-      <c r="F1" s="135"/>
-      <c r="G1" s="135"/>
-      <c r="H1" s="135"/>
-      <c r="I1" s="135"/>
-      <c r="J1" s="135"/>
-      <c r="K1" s="135"/>
-      <c r="L1" s="135"/>
-      <c r="M1" s="135"/>
-      <c r="N1" s="135"/>
-      <c r="O1" s="135"/>
-      <c r="P1" s="135"/>
-      <c r="Q1" s="135"/>
-      <c r="R1" s="135"/>
-      <c r="S1" s="135"/>
+      <c r="A1" s="159" t="s">
+        <v>288</v>
+      </c>
+      <c r="B1" s="149"/>
+      <c r="C1" s="149"/>
+      <c r="D1" s="149"/>
+      <c r="E1" s="149"/>
+      <c r="F1" s="149"/>
+      <c r="G1" s="149"/>
+      <c r="H1" s="149"/>
+      <c r="I1" s="149"/>
+      <c r="J1" s="149"/>
+      <c r="K1" s="149"/>
+      <c r="L1" s="149"/>
+      <c r="M1" s="149"/>
+      <c r="N1" s="149"/>
+      <c r="O1" s="149"/>
+      <c r="P1" s="149"/>
+      <c r="Q1" s="149"/>
+      <c r="R1" s="149"/>
+      <c r="S1" s="149"/>
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="152" t="s">
-        <v>285</v>
-      </c>
-      <c r="B2" s="135"/>
-      <c r="C2" s="135"/>
-      <c r="D2" s="135"/>
-      <c r="E2" s="135"/>
-      <c r="F2" s="135"/>
-      <c r="G2" s="135"/>
-      <c r="H2" s="135"/>
-      <c r="I2" s="135"/>
-      <c r="J2" s="135"/>
-      <c r="K2" s="135"/>
-      <c r="L2" s="135"/>
-      <c r="M2" s="135"/>
-      <c r="N2" s="135"/>
-      <c r="O2" s="135"/>
-      <c r="P2" s="135"/>
-      <c r="Q2" s="135"/>
-      <c r="R2" s="135"/>
-      <c r="S2" s="135"/>
+      <c r="A2" s="166" t="s">
+        <v>289</v>
+      </c>
+      <c r="B2" s="149"/>
+      <c r="C2" s="149"/>
+      <c r="D2" s="149"/>
+      <c r="E2" s="149"/>
+      <c r="F2" s="149"/>
+      <c r="G2" s="149"/>
+      <c r="H2" s="149"/>
+      <c r="I2" s="149"/>
+      <c r="J2" s="149"/>
+      <c r="K2" s="149"/>
+      <c r="L2" s="149"/>
+      <c r="M2" s="149"/>
+      <c r="N2" s="149"/>
+      <c r="O2" s="149"/>
+      <c r="P2" s="149"/>
+      <c r="Q2" s="149"/>
+      <c r="R2" s="149"/>
+      <c r="S2" s="149"/>
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="140" t="s">
-        <v>286</v>
-      </c>
-      <c r="B4" s="135"/>
-      <c r="C4" s="135"/>
-      <c r="D4" s="135"/>
-      <c r="E4" s="135"/>
-      <c r="F4" s="135"/>
-      <c r="G4" s="135"/>
-      <c r="H4" s="135"/>
-      <c r="I4" s="135"/>
-      <c r="J4" s="135"/>
-      <c r="K4" s="135"/>
-      <c r="L4" s="135"/>
-      <c r="M4" s="135"/>
-      <c r="N4" s="135"/>
-      <c r="O4" s="135"/>
-      <c r="P4" s="135"/>
-      <c r="Q4" s="135"/>
-      <c r="R4" s="135"/>
-      <c r="S4" s="135"/>
+      <c r="A4" s="154" t="s">
+        <v>290</v>
+      </c>
+      <c r="B4" s="149"/>
+      <c r="C4" s="149"/>
+      <c r="D4" s="149"/>
+      <c r="E4" s="149"/>
+      <c r="F4" s="149"/>
+      <c r="G4" s="149"/>
+      <c r="H4" s="149"/>
+      <c r="I4" s="149"/>
+      <c r="J4" s="149"/>
+      <c r="K4" s="149"/>
+      <c r="L4" s="149"/>
+      <c r="M4" s="149"/>
+      <c r="N4" s="149"/>
+      <c r="O4" s="149"/>
+      <c r="P4" s="149"/>
+      <c r="Q4" s="149"/>
+      <c r="R4" s="149"/>
+      <c r="S4" s="149"/>
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="37" t="s">
-        <v>287</v>
-      </c>
-      <c r="B5" s="130" t="s">
-        <v>288</v>
-      </c>
-      <c r="C5" s="131"/>
-      <c r="D5" s="132"/>
-      <c r="E5" s="133" t="s">
-        <v>289</v>
-      </c>
-      <c r="F5" s="131"/>
-      <c r="G5" s="132"/>
-      <c r="H5" s="133" t="s">
-        <v>290</v>
-      </c>
-      <c r="I5" s="131"/>
-      <c r="J5" s="132"/>
-      <c r="K5" s="130" t="s">
         <v>291</v>
       </c>
-      <c r="L5" s="131"/>
-      <c r="M5" s="132"/>
-      <c r="N5" s="137" t="s">
+      <c r="B5" s="144" t="s">
         <v>292</v>
       </c>
-      <c r="O5" s="131"/>
-      <c r="P5" s="132"/>
-      <c r="Q5" s="137" t="s">
+      <c r="C5" s="145"/>
+      <c r="D5" s="146"/>
+      <c r="E5" s="147" t="s">
         <v>293</v>
       </c>
-      <c r="R5" s="131"/>
-      <c r="S5" s="132"/>
+      <c r="F5" s="145"/>
+      <c r="G5" s="146"/>
+      <c r="H5" s="147" t="s">
+        <v>294</v>
+      </c>
+      <c r="I5" s="145"/>
+      <c r="J5" s="146"/>
+      <c r="K5" s="144" t="s">
+        <v>295</v>
+      </c>
+      <c r="L5" s="145"/>
+      <c r="M5" s="146"/>
+      <c r="N5" s="151" t="s">
+        <v>296</v>
+      </c>
+      <c r="O5" s="145"/>
+      <c r="P5" s="146"/>
+      <c r="Q5" s="151" t="s">
+        <v>297</v>
+      </c>
+      <c r="R5" s="145"/>
+      <c r="S5" s="146"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="134" t="s">
-        <v>294</v>
-      </c>
-      <c r="C6" s="135"/>
-      <c r="D6" s="135"/>
-      <c r="E6" s="135"/>
-      <c r="F6" s="135"/>
-      <c r="G6" s="135"/>
-      <c r="H6" s="135"/>
-      <c r="I6" s="135"/>
-      <c r="J6" s="135"/>
-      <c r="K6" s="135"/>
-      <c r="L6" s="135"/>
-      <c r="M6" s="135"/>
-      <c r="N6" s="135"/>
-      <c r="O6" s="135"/>
-      <c r="P6" s="135"/>
-      <c r="Q6" s="135"/>
-      <c r="R6" s="135"/>
-      <c r="S6" s="135"/>
+      <c r="B6" s="148" t="s">
+        <v>298</v>
+      </c>
+      <c r="C6" s="149"/>
+      <c r="D6" s="149"/>
+      <c r="E6" s="149"/>
+      <c r="F6" s="149"/>
+      <c r="G6" s="149"/>
+      <c r="H6" s="149"/>
+      <c r="I6" s="149"/>
+      <c r="J6" s="149"/>
+      <c r="K6" s="149"/>
+      <c r="L6" s="149"/>
+      <c r="M6" s="149"/>
+      <c r="N6" s="149"/>
+      <c r="O6" s="149"/>
+      <c r="P6" s="149"/>
+      <c r="Q6" s="149"/>
+      <c r="R6" s="149"/>
+      <c r="S6" s="149"/>
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="140" t="s">
-        <v>295</v>
-      </c>
-      <c r="B7" s="135"/>
-      <c r="C7" s="135"/>
-      <c r="D7" s="135"/>
-      <c r="E7" s="135"/>
-      <c r="F7" s="135"/>
-      <c r="G7" s="135"/>
-      <c r="H7" s="135"/>
-      <c r="I7" s="135"/>
-      <c r="J7" s="135"/>
-      <c r="K7" s="135"/>
-      <c r="L7" s="135"/>
-      <c r="M7" s="135"/>
-      <c r="N7" s="135"/>
-      <c r="O7" s="135"/>
-      <c r="P7" s="135"/>
-      <c r="Q7" s="135"/>
-      <c r="R7" s="135"/>
-      <c r="S7" s="135"/>
+      <c r="A7" s="154" t="s">
+        <v>299</v>
+      </c>
+      <c r="B7" s="149"/>
+      <c r="C7" s="149"/>
+      <c r="D7" s="149"/>
+      <c r="E7" s="149"/>
+      <c r="F7" s="149"/>
+      <c r="G7" s="149"/>
+      <c r="H7" s="149"/>
+      <c r="I7" s="149"/>
+      <c r="J7" s="149"/>
+      <c r="K7" s="149"/>
+      <c r="L7" s="149"/>
+      <c r="M7" s="149"/>
+      <c r="N7" s="149"/>
+      <c r="O7" s="149"/>
+      <c r="P7" s="149"/>
+      <c r="Q7" s="149"/>
+      <c r="R7" s="149"/>
+      <c r="S7" s="149"/>
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="37" t="s">
-        <v>296</v>
-      </c>
-      <c r="B8" s="143" t="s">
-        <v>297</v>
-      </c>
-      <c r="C8" s="131"/>
-      <c r="D8" s="131"/>
-      <c r="E8" s="131"/>
-      <c r="F8" s="131"/>
-      <c r="G8" s="131"/>
-      <c r="H8" s="131"/>
-      <c r="I8" s="131"/>
-      <c r="J8" s="132"/>
-      <c r="K8" s="143" t="s">
+        <v>300</v>
+      </c>
+      <c r="B8" s="157" t="s">
+        <v>301</v>
+      </c>
+      <c r="C8" s="145"/>
+      <c r="D8" s="145"/>
+      <c r="E8" s="145"/>
+      <c r="F8" s="145"/>
+      <c r="G8" s="145"/>
+      <c r="H8" s="145"/>
+      <c r="I8" s="145"/>
+      <c r="J8" s="146"/>
+      <c r="K8" s="157" t="s">
+        <v>302</v>
+      </c>
+      <c r="L8" s="145"/>
+      <c r="M8" s="145"/>
+      <c r="N8" s="145"/>
+      <c r="O8" s="145"/>
+      <c r="P8" s="145"/>
+      <c r="Q8" s="145"/>
+      <c r="R8" s="145"/>
+      <c r="S8" s="146"/>
+    </row>
+    <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B9" s="148" t="s">
         <v>298</v>
       </c>
-      <c r="L8" s="131"/>
-      <c r="M8" s="131"/>
-      <c r="N8" s="131"/>
-      <c r="O8" s="131"/>
-      <c r="P8" s="131"/>
-      <c r="Q8" s="131"/>
-      <c r="R8" s="131"/>
-      <c r="S8" s="132"/>
-    </row>
-    <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B9" s="134" t="s">
-        <v>294</v>
-      </c>
-      <c r="C9" s="135"/>
-      <c r="D9" s="135"/>
-      <c r="E9" s="135"/>
-      <c r="F9" s="135"/>
-      <c r="G9" s="135"/>
-      <c r="H9" s="135"/>
-      <c r="I9" s="135"/>
-      <c r="J9" s="135"/>
-      <c r="K9" s="135"/>
-      <c r="L9" s="135"/>
-      <c r="M9" s="135"/>
-      <c r="N9" s="135"/>
-      <c r="O9" s="135"/>
-      <c r="P9" s="135"/>
-      <c r="Q9" s="135"/>
-      <c r="R9" s="135"/>
-      <c r="S9" s="135"/>
+      <c r="C9" s="149"/>
+      <c r="D9" s="149"/>
+      <c r="E9" s="149"/>
+      <c r="F9" s="149"/>
+      <c r="G9" s="149"/>
+      <c r="H9" s="149"/>
+      <c r="I9" s="149"/>
+      <c r="J9" s="149"/>
+      <c r="K9" s="149"/>
+      <c r="L9" s="149"/>
+      <c r="M9" s="149"/>
+      <c r="N9" s="149"/>
+      <c r="O9" s="149"/>
+      <c r="P9" s="149"/>
+      <c r="Q9" s="149"/>
+      <c r="R9" s="149"/>
+      <c r="S9" s="149"/>
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="140" t="s">
-        <v>299</v>
-      </c>
-      <c r="B10" s="135"/>
-      <c r="C10" s="135"/>
-      <c r="D10" s="135"/>
-      <c r="E10" s="135"/>
-      <c r="F10" s="135"/>
-      <c r="G10" s="135"/>
-      <c r="H10" s="135"/>
-      <c r="I10" s="135"/>
-      <c r="J10" s="135"/>
-      <c r="K10" s="135"/>
-      <c r="L10" s="135"/>
-      <c r="M10" s="135"/>
-      <c r="N10" s="135"/>
-      <c r="O10" s="135"/>
-      <c r="P10" s="135"/>
-      <c r="Q10" s="135"/>
-      <c r="R10" s="135"/>
-      <c r="S10" s="135"/>
+      <c r="A10" s="154" t="s">
+        <v>303</v>
+      </c>
+      <c r="B10" s="149"/>
+      <c r="C10" s="149"/>
+      <c r="D10" s="149"/>
+      <c r="E10" s="149"/>
+      <c r="F10" s="149"/>
+      <c r="G10" s="149"/>
+      <c r="H10" s="149"/>
+      <c r="I10" s="149"/>
+      <c r="J10" s="149"/>
+      <c r="K10" s="149"/>
+      <c r="L10" s="149"/>
+      <c r="M10" s="149"/>
+      <c r="N10" s="149"/>
+      <c r="O10" s="149"/>
+      <c r="P10" s="149"/>
+      <c r="Q10" s="149"/>
+      <c r="R10" s="149"/>
+      <c r="S10" s="149"/>
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="37" t="s">
-        <v>300</v>
-      </c>
-      <c r="B11" s="130" t="s">
-        <v>301</v>
-      </c>
-      <c r="C11" s="131"/>
-      <c r="D11" s="132"/>
-      <c r="E11" s="130" t="s">
-        <v>302</v>
-      </c>
-      <c r="F11" s="131"/>
-      <c r="G11" s="132"/>
-      <c r="H11" s="130" t="s">
-        <v>303</v>
-      </c>
-      <c r="I11" s="131"/>
-      <c r="J11" s="132"/>
-      <c r="K11" s="133" t="s">
         <v>304</v>
       </c>
-      <c r="L11" s="131"/>
-      <c r="M11" s="132"/>
-      <c r="N11" s="130" t="s">
+      <c r="B11" s="144" t="s">
         <v>305</v>
       </c>
-      <c r="O11" s="131"/>
-      <c r="P11" s="132"/>
-      <c r="Q11" s="130" t="s">
+      <c r="C11" s="145"/>
+      <c r="D11" s="146"/>
+      <c r="E11" s="144" t="s">
         <v>306</v>
       </c>
-      <c r="R11" s="131"/>
-      <c r="S11" s="132"/>
+      <c r="F11" s="145"/>
+      <c r="G11" s="146"/>
+      <c r="H11" s="144" t="s">
+        <v>307</v>
+      </c>
+      <c r="I11" s="145"/>
+      <c r="J11" s="146"/>
+      <c r="K11" s="147" t="s">
+        <v>308</v>
+      </c>
+      <c r="L11" s="145"/>
+      <c r="M11" s="146"/>
+      <c r="N11" s="144" t="s">
+        <v>309</v>
+      </c>
+      <c r="O11" s="145"/>
+      <c r="P11" s="146"/>
+      <c r="Q11" s="144" t="s">
+        <v>310</v>
+      </c>
+      <c r="R11" s="145"/>
+      <c r="S11" s="146"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B12" s="134" t="s">
-        <v>294</v>
-      </c>
-      <c r="C12" s="135"/>
-      <c r="D12" s="135"/>
-      <c r="E12" s="135"/>
-      <c r="F12" s="135"/>
-      <c r="G12" s="135"/>
-      <c r="H12" s="135"/>
-      <c r="I12" s="135"/>
-      <c r="J12" s="135"/>
-      <c r="K12" s="135"/>
-      <c r="L12" s="135"/>
-      <c r="M12" s="135"/>
-      <c r="N12" s="135"/>
-      <c r="O12" s="135"/>
-      <c r="P12" s="135"/>
-      <c r="Q12" s="135"/>
-      <c r="R12" s="135"/>
-      <c r="S12" s="135"/>
+      <c r="B12" s="148" t="s">
+        <v>298</v>
+      </c>
+      <c r="C12" s="149"/>
+      <c r="D12" s="149"/>
+      <c r="E12" s="149"/>
+      <c r="F12" s="149"/>
+      <c r="G12" s="149"/>
+      <c r="H12" s="149"/>
+      <c r="I12" s="149"/>
+      <c r="J12" s="149"/>
+      <c r="K12" s="149"/>
+      <c r="L12" s="149"/>
+      <c r="M12" s="149"/>
+      <c r="N12" s="149"/>
+      <c r="O12" s="149"/>
+      <c r="P12" s="149"/>
+      <c r="Q12" s="149"/>
+      <c r="R12" s="149"/>
+      <c r="S12" s="149"/>
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="140" t="s">
-        <v>307</v>
-      </c>
-      <c r="B13" s="135"/>
-      <c r="C13" s="135"/>
-      <c r="D13" s="135"/>
-      <c r="E13" s="135"/>
-      <c r="F13" s="135"/>
-      <c r="G13" s="135"/>
-      <c r="H13" s="135"/>
-      <c r="I13" s="135"/>
-      <c r="J13" s="135"/>
-      <c r="K13" s="135"/>
-      <c r="L13" s="135"/>
-      <c r="M13" s="135"/>
-      <c r="N13" s="135"/>
-      <c r="O13" s="135"/>
-      <c r="P13" s="135"/>
-      <c r="Q13" s="135"/>
-      <c r="R13" s="135"/>
-      <c r="S13" s="135"/>
+      <c r="A13" s="154" t="s">
+        <v>311</v>
+      </c>
+      <c r="B13" s="149"/>
+      <c r="C13" s="149"/>
+      <c r="D13" s="149"/>
+      <c r="E13" s="149"/>
+      <c r="F13" s="149"/>
+      <c r="G13" s="149"/>
+      <c r="H13" s="149"/>
+      <c r="I13" s="149"/>
+      <c r="J13" s="149"/>
+      <c r="K13" s="149"/>
+      <c r="L13" s="149"/>
+      <c r="M13" s="149"/>
+      <c r="N13" s="149"/>
+      <c r="O13" s="149"/>
+      <c r="P13" s="149"/>
+      <c r="Q13" s="149"/>
+      <c r="R13" s="149"/>
+      <c r="S13" s="149"/>
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="37" t="s">
-        <v>308</v>
-      </c>
-      <c r="B14" s="138" t="s">
-        <v>309</v>
-      </c>
-      <c r="C14" s="131"/>
-      <c r="D14" s="131"/>
-      <c r="E14" s="131"/>
-      <c r="F14" s="131"/>
-      <c r="G14" s="132"/>
-      <c r="H14" s="138" t="s">
-        <v>310</v>
-      </c>
-      <c r="I14" s="131"/>
-      <c r="J14" s="131"/>
-      <c r="K14" s="131"/>
-      <c r="L14" s="131"/>
-      <c r="M14" s="132"/>
-      <c r="N14" s="138" t="s">
-        <v>311</v>
-      </c>
-      <c r="O14" s="131"/>
-      <c r="P14" s="132"/>
-      <c r="Q14" s="133" t="s">
         <v>312</v>
       </c>
-      <c r="R14" s="131"/>
-      <c r="S14" s="132"/>
+      <c r="B14" s="152" t="s">
+        <v>313</v>
+      </c>
+      <c r="C14" s="145"/>
+      <c r="D14" s="145"/>
+      <c r="E14" s="145"/>
+      <c r="F14" s="145"/>
+      <c r="G14" s="146"/>
+      <c r="H14" s="152" t="s">
+        <v>314</v>
+      </c>
+      <c r="I14" s="145"/>
+      <c r="J14" s="145"/>
+      <c r="K14" s="145"/>
+      <c r="L14" s="145"/>
+      <c r="M14" s="146"/>
+      <c r="N14" s="152" t="s">
+        <v>315</v>
+      </c>
+      <c r="O14" s="145"/>
+      <c r="P14" s="146"/>
+      <c r="Q14" s="147" t="s">
+        <v>316</v>
+      </c>
+      <c r="R14" s="145"/>
+      <c r="S14" s="146"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B15" s="134" t="s">
-        <v>313</v>
-      </c>
-      <c r="C15" s="135"/>
-      <c r="D15" s="135"/>
-      <c r="E15" s="135"/>
-      <c r="F15" s="135"/>
-      <c r="G15" s="135"/>
-      <c r="H15" s="135"/>
-      <c r="I15" s="135"/>
-      <c r="J15" s="135"/>
-      <c r="K15" s="135"/>
-      <c r="L15" s="135"/>
-      <c r="M15" s="135"/>
-      <c r="N15" s="135"/>
-      <c r="O15" s="135"/>
-      <c r="P15" s="135"/>
-      <c r="Q15" s="135"/>
-      <c r="R15" s="135"/>
-      <c r="S15" s="135"/>
+      <c r="B15" s="148" t="s">
+        <v>317</v>
+      </c>
+      <c r="C15" s="149"/>
+      <c r="D15" s="149"/>
+      <c r="E15" s="149"/>
+      <c r="F15" s="149"/>
+      <c r="G15" s="149"/>
+      <c r="H15" s="149"/>
+      <c r="I15" s="149"/>
+      <c r="J15" s="149"/>
+      <c r="K15" s="149"/>
+      <c r="L15" s="149"/>
+      <c r="M15" s="149"/>
+      <c r="N15" s="149"/>
+      <c r="O15" s="149"/>
+      <c r="P15" s="149"/>
+      <c r="Q15" s="149"/>
+      <c r="R15" s="149"/>
+      <c r="S15" s="149"/>
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="140" t="s">
-        <v>314</v>
-      </c>
-      <c r="B16" s="135"/>
-      <c r="C16" s="135"/>
-      <c r="D16" s="135"/>
-      <c r="E16" s="135"/>
-      <c r="F16" s="135"/>
-      <c r="G16" s="135"/>
-      <c r="H16" s="135"/>
-      <c r="I16" s="135"/>
-      <c r="J16" s="135"/>
-      <c r="K16" s="135"/>
-      <c r="L16" s="135"/>
-      <c r="M16" s="135"/>
-      <c r="N16" s="135"/>
-      <c r="O16" s="135"/>
-      <c r="P16" s="135"/>
-      <c r="Q16" s="135"/>
-      <c r="R16" s="135"/>
-      <c r="S16" s="135"/>
+      <c r="A16" s="154" t="s">
+        <v>318</v>
+      </c>
+      <c r="B16" s="149"/>
+      <c r="C16" s="149"/>
+      <c r="D16" s="149"/>
+      <c r="E16" s="149"/>
+      <c r="F16" s="149"/>
+      <c r="G16" s="149"/>
+      <c r="H16" s="149"/>
+      <c r="I16" s="149"/>
+      <c r="J16" s="149"/>
+      <c r="K16" s="149"/>
+      <c r="L16" s="149"/>
+      <c r="M16" s="149"/>
+      <c r="N16" s="149"/>
+      <c r="O16" s="149"/>
+      <c r="P16" s="149"/>
+      <c r="Q16" s="149"/>
+      <c r="R16" s="149"/>
+      <c r="S16" s="149"/>
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="37" t="s">
-        <v>315</v>
-      </c>
-      <c r="B17" s="139" t="s">
-        <v>316</v>
-      </c>
-      <c r="C17" s="131"/>
-      <c r="D17" s="131"/>
-      <c r="E17" s="131"/>
-      <c r="F17" s="131"/>
-      <c r="G17" s="132"/>
-      <c r="H17" s="139" t="s">
-        <v>317</v>
-      </c>
-      <c r="I17" s="131"/>
-      <c r="J17" s="132"/>
-      <c r="K17" s="139" t="s">
-        <v>318</v>
-      </c>
-      <c r="L17" s="131"/>
-      <c r="M17" s="132"/>
-      <c r="N17" s="139" t="s">
         <v>319</v>
       </c>
-      <c r="O17" s="131"/>
-      <c r="P17" s="132"/>
-      <c r="Q17" s="139" t="s">
+      <c r="B17" s="153" t="s">
         <v>320</v>
       </c>
-      <c r="R17" s="131"/>
-      <c r="S17" s="132"/>
+      <c r="C17" s="145"/>
+      <c r="D17" s="145"/>
+      <c r="E17" s="145"/>
+      <c r="F17" s="145"/>
+      <c r="G17" s="146"/>
+      <c r="H17" s="153" t="s">
+        <v>321</v>
+      </c>
+      <c r="I17" s="145"/>
+      <c r="J17" s="146"/>
+      <c r="K17" s="153" t="s">
+        <v>322</v>
+      </c>
+      <c r="L17" s="145"/>
+      <c r="M17" s="146"/>
+      <c r="N17" s="153" t="s">
+        <v>323</v>
+      </c>
+      <c r="O17" s="145"/>
+      <c r="P17" s="146"/>
+      <c r="Q17" s="153" t="s">
+        <v>324</v>
+      </c>
+      <c r="R17" s="145"/>
+      <c r="S17" s="146"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="134" t="s">
-        <v>294</v>
-      </c>
-      <c r="C18" s="135"/>
-      <c r="D18" s="135"/>
-      <c r="E18" s="135"/>
-      <c r="F18" s="135"/>
-      <c r="G18" s="135"/>
-      <c r="H18" s="135"/>
-      <c r="I18" s="135"/>
-      <c r="J18" s="135"/>
-      <c r="K18" s="135"/>
-      <c r="L18" s="135"/>
-      <c r="M18" s="135"/>
-      <c r="N18" s="135"/>
-      <c r="O18" s="135"/>
-      <c r="P18" s="135"/>
-      <c r="Q18" s="135"/>
-      <c r="R18" s="135"/>
-      <c r="S18" s="135"/>
+      <c r="B18" s="148" t="s">
+        <v>298</v>
+      </c>
+      <c r="C18" s="149"/>
+      <c r="D18" s="149"/>
+      <c r="E18" s="149"/>
+      <c r="F18" s="149"/>
+      <c r="G18" s="149"/>
+      <c r="H18" s="149"/>
+      <c r="I18" s="149"/>
+      <c r="J18" s="149"/>
+      <c r="K18" s="149"/>
+      <c r="L18" s="149"/>
+      <c r="M18" s="149"/>
+      <c r="N18" s="149"/>
+      <c r="O18" s="149"/>
+      <c r="P18" s="149"/>
+      <c r="Q18" s="149"/>
+      <c r="R18" s="149"/>
+      <c r="S18" s="149"/>
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="140" t="s">
-        <v>321</v>
-      </c>
-      <c r="B19" s="135"/>
-      <c r="C19" s="135"/>
-      <c r="D19" s="135"/>
-      <c r="E19" s="135"/>
-      <c r="F19" s="135"/>
-      <c r="G19" s="135"/>
-      <c r="H19" s="135"/>
-      <c r="I19" s="135"/>
-      <c r="J19" s="135"/>
-      <c r="K19" s="135"/>
-      <c r="L19" s="135"/>
-      <c r="M19" s="135"/>
-      <c r="N19" s="135"/>
-      <c r="O19" s="135"/>
-      <c r="P19" s="135"/>
-      <c r="Q19" s="135"/>
-      <c r="R19" s="135"/>
-      <c r="S19" s="135"/>
+      <c r="A19" s="154" t="s">
+        <v>325</v>
+      </c>
+      <c r="B19" s="149"/>
+      <c r="C19" s="149"/>
+      <c r="D19" s="149"/>
+      <c r="E19" s="149"/>
+      <c r="F19" s="149"/>
+      <c r="G19" s="149"/>
+      <c r="H19" s="149"/>
+      <c r="I19" s="149"/>
+      <c r="J19" s="149"/>
+      <c r="K19" s="149"/>
+      <c r="L19" s="149"/>
+      <c r="M19" s="149"/>
+      <c r="N19" s="149"/>
+      <c r="O19" s="149"/>
+      <c r="P19" s="149"/>
+      <c r="Q19" s="149"/>
+      <c r="R19" s="149"/>
+      <c r="S19" s="149"/>
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="37" t="s">
-        <v>322</v>
-      </c>
-      <c r="B20" s="141" t="s">
-        <v>323</v>
-      </c>
-      <c r="C20" s="131"/>
-      <c r="D20" s="131"/>
-      <c r="E20" s="131"/>
-      <c r="F20" s="131"/>
-      <c r="G20" s="132"/>
-      <c r="H20" s="141" t="s">
-        <v>324</v>
-      </c>
-      <c r="I20" s="131"/>
-      <c r="J20" s="131"/>
-      <c r="K20" s="131"/>
-      <c r="L20" s="131"/>
-      <c r="M20" s="132"/>
-      <c r="N20" s="141" t="s">
-        <v>325</v>
-      </c>
-      <c r="O20" s="131"/>
-      <c r="P20" s="131"/>
-      <c r="Q20" s="131"/>
-      <c r="R20" s="131"/>
-      <c r="S20" s="132"/>
+        <v>326</v>
+      </c>
+      <c r="B20" s="155" t="s">
+        <v>327</v>
+      </c>
+      <c r="C20" s="145"/>
+      <c r="D20" s="145"/>
+      <c r="E20" s="145"/>
+      <c r="F20" s="145"/>
+      <c r="G20" s="146"/>
+      <c r="H20" s="155" t="s">
+        <v>328</v>
+      </c>
+      <c r="I20" s="145"/>
+      <c r="J20" s="145"/>
+      <c r="K20" s="145"/>
+      <c r="L20" s="145"/>
+      <c r="M20" s="146"/>
+      <c r="N20" s="155" t="s">
+        <v>329</v>
+      </c>
+      <c r="O20" s="145"/>
+      <c r="P20" s="145"/>
+      <c r="Q20" s="145"/>
+      <c r="R20" s="145"/>
+      <c r="S20" s="146"/>
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B21" s="134" t="s">
-        <v>294</v>
-      </c>
-      <c r="C21" s="135"/>
-      <c r="D21" s="135"/>
-      <c r="E21" s="135"/>
-      <c r="F21" s="135"/>
-      <c r="G21" s="135"/>
-      <c r="H21" s="135"/>
-      <c r="I21" s="135"/>
-      <c r="J21" s="135"/>
-      <c r="K21" s="135"/>
-      <c r="L21" s="135"/>
-      <c r="M21" s="135"/>
-      <c r="N21" s="135"/>
-      <c r="O21" s="135"/>
-      <c r="P21" s="135"/>
-      <c r="Q21" s="135"/>
-      <c r="R21" s="135"/>
-      <c r="S21" s="135"/>
+      <c r="B21" s="148" t="s">
+        <v>298</v>
+      </c>
+      <c r="C21" s="149"/>
+      <c r="D21" s="149"/>
+      <c r="E21" s="149"/>
+      <c r="F21" s="149"/>
+      <c r="G21" s="149"/>
+      <c r="H21" s="149"/>
+      <c r="I21" s="149"/>
+      <c r="J21" s="149"/>
+      <c r="K21" s="149"/>
+      <c r="L21" s="149"/>
+      <c r="M21" s="149"/>
+      <c r="N21" s="149"/>
+      <c r="O21" s="149"/>
+      <c r="P21" s="149"/>
+      <c r="Q21" s="149"/>
+      <c r="R21" s="149"/>
+      <c r="S21" s="149"/>
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="140" t="s">
-        <v>326</v>
-      </c>
-      <c r="B22" s="135"/>
-      <c r="C22" s="135"/>
-      <c r="D22" s="135"/>
-      <c r="E22" s="135"/>
-      <c r="F22" s="135"/>
-      <c r="G22" s="135"/>
-      <c r="H22" s="135"/>
-      <c r="I22" s="135"/>
-      <c r="J22" s="135"/>
-      <c r="K22" s="135"/>
-      <c r="L22" s="135"/>
-      <c r="M22" s="135"/>
-      <c r="N22" s="135"/>
-      <c r="O22" s="135"/>
-      <c r="P22" s="135"/>
-      <c r="Q22" s="135"/>
-      <c r="R22" s="135"/>
-      <c r="S22" s="135"/>
+      <c r="A22" s="154" t="s">
+        <v>330</v>
+      </c>
+      <c r="B22" s="149"/>
+      <c r="C22" s="149"/>
+      <c r="D22" s="149"/>
+      <c r="E22" s="149"/>
+      <c r="F22" s="149"/>
+      <c r="G22" s="149"/>
+      <c r="H22" s="149"/>
+      <c r="I22" s="149"/>
+      <c r="J22" s="149"/>
+      <c r="K22" s="149"/>
+      <c r="L22" s="149"/>
+      <c r="M22" s="149"/>
+      <c r="N22" s="149"/>
+      <c r="O22" s="149"/>
+      <c r="P22" s="149"/>
+      <c r="Q22" s="149"/>
+      <c r="R22" s="149"/>
+      <c r="S22" s="149"/>
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="37" t="s">
-        <v>327</v>
-      </c>
-      <c r="B23" s="141" t="s">
-        <v>328</v>
-      </c>
-      <c r="C23" s="131"/>
-      <c r="D23" s="131"/>
-      <c r="E23" s="131"/>
-      <c r="F23" s="131"/>
-      <c r="G23" s="132"/>
-      <c r="H23" s="141" t="s">
-        <v>329</v>
-      </c>
-      <c r="I23" s="131"/>
-      <c r="J23" s="132"/>
-      <c r="K23" s="141" t="s">
-        <v>330</v>
-      </c>
-      <c r="L23" s="131"/>
-      <c r="M23" s="132"/>
-      <c r="N23" s="141" t="s">
         <v>331</v>
       </c>
-      <c r="O23" s="131"/>
-      <c r="P23" s="132"/>
-      <c r="Q23" s="137" t="s">
+      <c r="B23" s="155" t="s">
         <v>332</v>
       </c>
-      <c r="R23" s="131"/>
-      <c r="S23" s="132"/>
+      <c r="C23" s="145"/>
+      <c r="D23" s="145"/>
+      <c r="E23" s="145"/>
+      <c r="F23" s="145"/>
+      <c r="G23" s="146"/>
+      <c r="H23" s="155" t="s">
+        <v>333</v>
+      </c>
+      <c r="I23" s="145"/>
+      <c r="J23" s="146"/>
+      <c r="K23" s="155" t="s">
+        <v>334</v>
+      </c>
+      <c r="L23" s="145"/>
+      <c r="M23" s="146"/>
+      <c r="N23" s="155" t="s">
+        <v>335</v>
+      </c>
+      <c r="O23" s="145"/>
+      <c r="P23" s="146"/>
+      <c r="Q23" s="151" t="s">
+        <v>336</v>
+      </c>
+      <c r="R23" s="145"/>
+      <c r="S23" s="146"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="146" t="s">
-        <v>333</v>
-      </c>
-      <c r="B26" s="135"/>
-      <c r="C26" s="135"/>
-      <c r="D26" s="135"/>
-      <c r="E26" s="135"/>
-      <c r="F26" s="135"/>
-      <c r="G26" s="135"/>
-      <c r="H26" s="135"/>
-      <c r="I26" s="135"/>
-      <c r="J26" s="135"/>
-      <c r="K26" s="135"/>
-      <c r="L26" s="135"/>
-      <c r="M26" s="135"/>
-      <c r="N26" s="135"/>
-      <c r="O26" s="135"/>
-      <c r="P26" s="135"/>
-      <c r="Q26" s="135"/>
-      <c r="R26" s="135"/>
-      <c r="S26" s="135"/>
+      <c r="A26" s="160" t="s">
+        <v>337</v>
+      </c>
+      <c r="B26" s="149"/>
+      <c r="C26" s="149"/>
+      <c r="D26" s="149"/>
+      <c r="E26" s="149"/>
+      <c r="F26" s="149"/>
+      <c r="G26" s="149"/>
+      <c r="H26" s="149"/>
+      <c r="I26" s="149"/>
+      <c r="J26" s="149"/>
+      <c r="K26" s="149"/>
+      <c r="L26" s="149"/>
+      <c r="M26" s="149"/>
+      <c r="N26" s="149"/>
+      <c r="O26" s="149"/>
+      <c r="P26" s="149"/>
+      <c r="Q26" s="149"/>
+      <c r="R26" s="149"/>
+      <c r="S26" s="149"/>
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="37" t="s">
-        <v>334</v>
-      </c>
-      <c r="B27" s="130" t="s">
-        <v>335</v>
-      </c>
-      <c r="C27" s="131"/>
-      <c r="D27" s="132"/>
-      <c r="E27" s="130" t="s">
-        <v>336</v>
-      </c>
-      <c r="F27" s="131"/>
-      <c r="G27" s="132"/>
-      <c r="H27" s="138" t="s">
-        <v>337</v>
-      </c>
-      <c r="I27" s="131"/>
-      <c r="J27" s="132"/>
-      <c r="K27" s="139" t="s">
         <v>338</v>
       </c>
-      <c r="L27" s="131"/>
-      <c r="M27" s="132"/>
-      <c r="N27" s="139" t="s">
+      <c r="B27" s="144" t="s">
         <v>339</v>
       </c>
-      <c r="O27" s="131"/>
-      <c r="P27" s="132"/>
-      <c r="Q27" s="138" t="s">
+      <c r="C27" s="145"/>
+      <c r="D27" s="146"/>
+      <c r="E27" s="144" t="s">
         <v>340</v>
       </c>
-      <c r="R27" s="131"/>
-      <c r="S27" s="132"/>
+      <c r="F27" s="145"/>
+      <c r="G27" s="146"/>
+      <c r="H27" s="152" t="s">
+        <v>341</v>
+      </c>
+      <c r="I27" s="145"/>
+      <c r="J27" s="146"/>
+      <c r="K27" s="153" t="s">
+        <v>342</v>
+      </c>
+      <c r="L27" s="145"/>
+      <c r="M27" s="146"/>
+      <c r="N27" s="153" t="s">
+        <v>343</v>
+      </c>
+      <c r="O27" s="145"/>
+      <c r="P27" s="146"/>
+      <c r="Q27" s="152" t="s">
+        <v>344</v>
+      </c>
+      <c r="R27" s="145"/>
+      <c r="S27" s="146"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="140" t="s">
-        <v>341</v>
-      </c>
-      <c r="B30" s="135"/>
-      <c r="C30" s="135"/>
-      <c r="D30" s="135"/>
-      <c r="E30" s="135"/>
-      <c r="F30" s="135"/>
-      <c r="G30" s="135"/>
-      <c r="H30" s="135"/>
-      <c r="I30" s="135"/>
-      <c r="J30" s="135"/>
-      <c r="K30" s="135"/>
-      <c r="L30" s="135"/>
-      <c r="M30" s="135"/>
-      <c r="N30" s="135"/>
-      <c r="O30" s="135"/>
-      <c r="P30" s="135"/>
-      <c r="Q30" s="135"/>
-      <c r="R30" s="135"/>
-      <c r="S30" s="135"/>
+      <c r="A30" s="154" t="s">
+        <v>345</v>
+      </c>
+      <c r="B30" s="149"/>
+      <c r="C30" s="149"/>
+      <c r="D30" s="149"/>
+      <c r="E30" s="149"/>
+      <c r="F30" s="149"/>
+      <c r="G30" s="149"/>
+      <c r="H30" s="149"/>
+      <c r="I30" s="149"/>
+      <c r="J30" s="149"/>
+      <c r="K30" s="149"/>
+      <c r="L30" s="149"/>
+      <c r="M30" s="149"/>
+      <c r="N30" s="149"/>
+      <c r="O30" s="149"/>
+      <c r="P30" s="149"/>
+      <c r="Q30" s="149"/>
+      <c r="R30" s="149"/>
+      <c r="S30" s="149"/>
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="136" t="s">
-        <v>342</v>
-      </c>
-      <c r="B31" s="135"/>
-      <c r="C31" s="135"/>
-      <c r="D31" s="135"/>
-      <c r="E31" s="135"/>
-      <c r="F31" s="135"/>
-      <c r="G31" s="135"/>
-      <c r="H31" s="135"/>
-      <c r="I31" s="135"/>
-      <c r="J31" s="135"/>
-      <c r="K31" s="135"/>
-      <c r="L31" s="135"/>
-      <c r="M31" s="135"/>
-      <c r="N31" s="135"/>
-      <c r="O31" s="135"/>
-      <c r="P31" s="135"/>
-      <c r="Q31" s="135"/>
-      <c r="R31" s="135"/>
-      <c r="S31" s="135"/>
+      <c r="A31" s="150" t="s">
+        <v>346</v>
+      </c>
+      <c r="B31" s="149"/>
+      <c r="C31" s="149"/>
+      <c r="D31" s="149"/>
+      <c r="E31" s="149"/>
+      <c r="F31" s="149"/>
+      <c r="G31" s="149"/>
+      <c r="H31" s="149"/>
+      <c r="I31" s="149"/>
+      <c r="J31" s="149"/>
+      <c r="K31" s="149"/>
+      <c r="L31" s="149"/>
+      <c r="M31" s="149"/>
+      <c r="N31" s="149"/>
+      <c r="O31" s="149"/>
+      <c r="P31" s="149"/>
+      <c r="Q31" s="149"/>
+      <c r="R31" s="149"/>
+      <c r="S31" s="149"/>
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="136" t="s">
-        <v>343</v>
-      </c>
-      <c r="B32" s="135"/>
-      <c r="C32" s="135"/>
-      <c r="D32" s="135"/>
-      <c r="E32" s="135"/>
-      <c r="F32" s="135"/>
-      <c r="G32" s="135"/>
-      <c r="H32" s="135"/>
-      <c r="I32" s="135"/>
-      <c r="J32" s="135"/>
-      <c r="K32" s="135"/>
-      <c r="L32" s="135"/>
-      <c r="M32" s="135"/>
-      <c r="N32" s="135"/>
-      <c r="O32" s="135"/>
-      <c r="P32" s="135"/>
-      <c r="Q32" s="135"/>
-      <c r="R32" s="135"/>
-      <c r="S32" s="135"/>
+      <c r="A32" s="150" t="s">
+        <v>347</v>
+      </c>
+      <c r="B32" s="149"/>
+      <c r="C32" s="149"/>
+      <c r="D32" s="149"/>
+      <c r="E32" s="149"/>
+      <c r="F32" s="149"/>
+      <c r="G32" s="149"/>
+      <c r="H32" s="149"/>
+      <c r="I32" s="149"/>
+      <c r="J32" s="149"/>
+      <c r="K32" s="149"/>
+      <c r="L32" s="149"/>
+      <c r="M32" s="149"/>
+      <c r="N32" s="149"/>
+      <c r="O32" s="149"/>
+      <c r="P32" s="149"/>
+      <c r="Q32" s="149"/>
+      <c r="R32" s="149"/>
+      <c r="S32" s="149"/>
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="136" t="s">
-        <v>344</v>
-      </c>
-      <c r="B33" s="135"/>
-      <c r="C33" s="135"/>
-      <c r="D33" s="135"/>
-      <c r="E33" s="135"/>
-      <c r="F33" s="135"/>
-      <c r="G33" s="135"/>
-      <c r="H33" s="135"/>
-      <c r="I33" s="135"/>
-      <c r="J33" s="135"/>
-      <c r="K33" s="135"/>
-      <c r="L33" s="135"/>
-      <c r="M33" s="135"/>
-      <c r="N33" s="135"/>
-      <c r="O33" s="135"/>
-      <c r="P33" s="135"/>
-      <c r="Q33" s="135"/>
-      <c r="R33" s="135"/>
-      <c r="S33" s="135"/>
+      <c r="A33" s="150" t="s">
+        <v>348</v>
+      </c>
+      <c r="B33" s="149"/>
+      <c r="C33" s="149"/>
+      <c r="D33" s="149"/>
+      <c r="E33" s="149"/>
+      <c r="F33" s="149"/>
+      <c r="G33" s="149"/>
+      <c r="H33" s="149"/>
+      <c r="I33" s="149"/>
+      <c r="J33" s="149"/>
+      <c r="K33" s="149"/>
+      <c r="L33" s="149"/>
+      <c r="M33" s="149"/>
+      <c r="N33" s="149"/>
+      <c r="O33" s="149"/>
+      <c r="P33" s="149"/>
+      <c r="Q33" s="149"/>
+      <c r="R33" s="149"/>
+      <c r="S33" s="149"/>
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="136" t="s">
-        <v>345</v>
-      </c>
-      <c r="B34" s="135"/>
-      <c r="C34" s="135"/>
-      <c r="D34" s="135"/>
-      <c r="E34" s="135"/>
-      <c r="F34" s="135"/>
-      <c r="G34" s="135"/>
-      <c r="H34" s="135"/>
-      <c r="I34" s="135"/>
-      <c r="J34" s="135"/>
-      <c r="K34" s="135"/>
-      <c r="L34" s="135"/>
-      <c r="M34" s="135"/>
-      <c r="N34" s="135"/>
-      <c r="O34" s="135"/>
-      <c r="P34" s="135"/>
-      <c r="Q34" s="135"/>
-      <c r="R34" s="135"/>
-      <c r="S34" s="135"/>
+      <c r="A34" s="150" t="s">
+        <v>349</v>
+      </c>
+      <c r="B34" s="149"/>
+      <c r="C34" s="149"/>
+      <c r="D34" s="149"/>
+      <c r="E34" s="149"/>
+      <c r="F34" s="149"/>
+      <c r="G34" s="149"/>
+      <c r="H34" s="149"/>
+      <c r="I34" s="149"/>
+      <c r="J34" s="149"/>
+      <c r="K34" s="149"/>
+      <c r="L34" s="149"/>
+      <c r="M34" s="149"/>
+      <c r="N34" s="149"/>
+      <c r="O34" s="149"/>
+      <c r="P34" s="149"/>
+      <c r="Q34" s="149"/>
+      <c r="R34" s="149"/>
+      <c r="S34" s="149"/>
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="136" t="s">
-        <v>346</v>
-      </c>
-      <c r="B35" s="135"/>
-      <c r="C35" s="135"/>
-      <c r="D35" s="135"/>
-      <c r="E35" s="135"/>
-      <c r="F35" s="135"/>
-      <c r="G35" s="135"/>
-      <c r="H35" s="135"/>
-      <c r="I35" s="135"/>
-      <c r="J35" s="135"/>
-      <c r="K35" s="135"/>
-      <c r="L35" s="135"/>
-      <c r="M35" s="135"/>
-      <c r="N35" s="135"/>
-      <c r="O35" s="135"/>
-      <c r="P35" s="135"/>
-      <c r="Q35" s="135"/>
-      <c r="R35" s="135"/>
-      <c r="S35" s="135"/>
+      <c r="A35" s="150" t="s">
+        <v>350</v>
+      </c>
+      <c r="B35" s="149"/>
+      <c r="C35" s="149"/>
+      <c r="D35" s="149"/>
+      <c r="E35" s="149"/>
+      <c r="F35" s="149"/>
+      <c r="G35" s="149"/>
+      <c r="H35" s="149"/>
+      <c r="I35" s="149"/>
+      <c r="J35" s="149"/>
+      <c r="K35" s="149"/>
+      <c r="L35" s="149"/>
+      <c r="M35" s="149"/>
+      <c r="N35" s="149"/>
+      <c r="O35" s="149"/>
+      <c r="P35" s="149"/>
+      <c r="Q35" s="149"/>
+      <c r="R35" s="149"/>
+      <c r="S35" s="149"/>
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="136" t="s">
-        <v>347</v>
-      </c>
-      <c r="B36" s="135"/>
-      <c r="C36" s="135"/>
-      <c r="D36" s="135"/>
-      <c r="E36" s="135"/>
-      <c r="F36" s="135"/>
-      <c r="G36" s="135"/>
-      <c r="H36" s="135"/>
-      <c r="I36" s="135"/>
-      <c r="J36" s="135"/>
-      <c r="K36" s="135"/>
-      <c r="L36" s="135"/>
-      <c r="M36" s="135"/>
-      <c r="N36" s="135"/>
-      <c r="O36" s="135"/>
-      <c r="P36" s="135"/>
-      <c r="Q36" s="135"/>
-      <c r="R36" s="135"/>
-      <c r="S36" s="135"/>
+      <c r="A36" s="150" t="s">
+        <v>351</v>
+      </c>
+      <c r="B36" s="149"/>
+      <c r="C36" s="149"/>
+      <c r="D36" s="149"/>
+      <c r="E36" s="149"/>
+      <c r="F36" s="149"/>
+      <c r="G36" s="149"/>
+      <c r="H36" s="149"/>
+      <c r="I36" s="149"/>
+      <c r="J36" s="149"/>
+      <c r="K36" s="149"/>
+      <c r="L36" s="149"/>
+      <c r="M36" s="149"/>
+      <c r="N36" s="149"/>
+      <c r="O36" s="149"/>
+      <c r="P36" s="149"/>
+      <c r="Q36" s="149"/>
+      <c r="R36" s="149"/>
+      <c r="S36" s="149"/>
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="147" t="s">
-        <v>348</v>
-      </c>
-      <c r="B37" s="135"/>
-      <c r="C37" s="135"/>
-      <c r="D37" s="135"/>
-      <c r="E37" s="135"/>
-      <c r="F37" s="135"/>
-      <c r="G37" s="135"/>
-      <c r="H37" s="135"/>
-      <c r="I37" s="135"/>
-      <c r="J37" s="135"/>
-      <c r="K37" s="135"/>
-      <c r="L37" s="135"/>
-      <c r="M37" s="135"/>
-      <c r="N37" s="135"/>
-      <c r="O37" s="135"/>
-      <c r="P37" s="135"/>
-      <c r="Q37" s="135"/>
-      <c r="R37" s="135"/>
-      <c r="S37" s="135"/>
+      <c r="A37" s="161" t="s">
+        <v>352</v>
+      </c>
+      <c r="B37" s="149"/>
+      <c r="C37" s="149"/>
+      <c r="D37" s="149"/>
+      <c r="E37" s="149"/>
+      <c r="F37" s="149"/>
+      <c r="G37" s="149"/>
+      <c r="H37" s="149"/>
+      <c r="I37" s="149"/>
+      <c r="J37" s="149"/>
+      <c r="K37" s="149"/>
+      <c r="L37" s="149"/>
+      <c r="M37" s="149"/>
+      <c r="N37" s="149"/>
+      <c r="O37" s="149"/>
+      <c r="P37" s="149"/>
+      <c r="Q37" s="149"/>
+      <c r="R37" s="149"/>
+      <c r="S37" s="149"/>
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="38" t="s">
-        <v>283</v>
-      </c>
-      <c r="B39" s="150" t="s">
-        <v>349</v>
-      </c>
-      <c r="C39" s="135"/>
-      <c r="D39" s="135"/>
-      <c r="E39" s="148" t="s">
-        <v>350</v>
-      </c>
-      <c r="F39" s="135"/>
-      <c r="G39" s="135"/>
-      <c r="H39" s="151" t="s">
-        <v>351</v>
-      </c>
-      <c r="I39" s="135"/>
-      <c r="J39" s="135"/>
-      <c r="K39" s="144" t="s">
-        <v>352</v>
-      </c>
-      <c r="L39" s="135"/>
-      <c r="M39" s="135"/>
-      <c r="N39" s="142" t="s">
+        <v>287</v>
+      </c>
+      <c r="B39" s="164" t="s">
+        <v>353</v>
+      </c>
+      <c r="C39" s="149"/>
+      <c r="D39" s="149"/>
+      <c r="E39" s="162" t="s">
+        <v>354</v>
+      </c>
+      <c r="F39" s="149"/>
+      <c r="G39" s="149"/>
+      <c r="H39" s="165" t="s">
+        <v>355</v>
+      </c>
+      <c r="I39" s="149"/>
+      <c r="J39" s="149"/>
+      <c r="K39" s="158" t="s">
+        <v>356</v>
+      </c>
+      <c r="L39" s="149"/>
+      <c r="M39" s="149"/>
+      <c r="N39" s="156" t="s">
         <v>45</v>
       </c>
-      <c r="O39" s="135"/>
-      <c r="P39" s="135"/>
-      <c r="Q39" s="149" t="s">
-        <v>353</v>
-      </c>
-      <c r="R39" s="135"/>
-      <c r="S39" s="135"/>
+      <c r="O39" s="149"/>
+      <c r="P39" s="149"/>
+      <c r="Q39" s="163" t="s">
+        <v>357</v>
+      </c>
+      <c r="R39" s="149"/>
+      <c r="S39" s="149"/>
     </row>
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A16:S16"/>
     <mergeCell ref="H20:M20"/>
-    <mergeCell ref="A16:S16"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -8109,14 +8294,13 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -8125,6 +8309,7 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -8132,7 +8317,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -8180,33 +8365,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="153" t="s">
-        <v>354</v>
-      </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="128"/>
+      <c r="A1" s="167" t="s">
+        <v>358</v>
+      </c>
+      <c r="B1" s="141"/>
+      <c r="C1" s="141"/>
+      <c r="D1" s="141"/>
+      <c r="E1" s="141"/>
+      <c r="F1" s="142"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -8440,15 +8625,15 @@
       </c>
       <c r="B13" s="26">
         <f t="shared" si="0"/>
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C13" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D13" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E13" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Blocked")</f>
@@ -8456,7 +8641,7 @@
       </c>
       <c r="F13" s="27">
         <f t="shared" si="1"/>
-        <v>0.39285714285714285</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -8486,19 +8671,19 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="28" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="B16" s="29">
         <f>SUM(B4:B14)</f>
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C16" s="29">
         <f>SUM(C4:C14)</f>
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E16">
         <f>SUM(E4:E14)</f>
@@ -8506,12 +8691,12 @@
       </c>
       <c r="F16" s="30">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.65833333333333333</v>
+        <v>0.65573770491803274</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="43" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="B18" s="44">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -8520,7 +8705,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="45" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
     </row>
   </sheetData>
@@ -8552,539 +8737,539 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="153" t="s">
-        <v>361</v>
-      </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="128"/>
+      <c r="A1" s="167" t="s">
+        <v>365</v>
+      </c>
+      <c r="B1" s="141"/>
+      <c r="C1" s="141"/>
+      <c r="D1" s="141"/>
+      <c r="E1" s="142"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="31" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="D3" s="31" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="32" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="34" t="s">
+        <v>375</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>371</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>367</v>
-      </c>
       <c r="C5" s="21" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="32" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="34" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="32" t="s">
+        <v>383</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>379</v>
       </c>
-      <c r="B8" s="12" t="s">
-        <v>375</v>
-      </c>
       <c r="C8" s="19" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="34" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="32" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="34" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="32" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="34" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="32" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="34" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="32" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="34" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="32" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="34" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="32" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="34" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="32" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E22" s="33" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="34" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E23" s="35" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="32" t="s">
+        <v>425</v>
+      </c>
+      <c r="B24" s="12" t="s">
         <v>421</v>
       </c>
-      <c r="B24" s="12" t="s">
-        <v>417</v>
-      </c>
       <c r="C24" s="19" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="58" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="B25" s="55" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="C25" s="59" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D25" s="55" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E25" s="60" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="61" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="B26" s="49" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C26" s="59" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="D26" s="49" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="E26" s="62" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="58" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="B27" s="55" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="C27" s="59" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="D27" s="55" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E27" s="60" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="79" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="B28" s="66" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="C28" s="75" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="D28" s="107" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="E28" s="107" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="80" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="B29" s="72" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C29" s="77" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D29" s="106" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="E29" s="106" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="88" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="B30" s="84" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C30" s="89" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D30" s="84" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="E30" s="90" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="105" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="B31" s="94" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C31" s="103" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D31" s="94" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="E31" s="106" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="122" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="B32" s="117" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="C32" s="120" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D32" s="117" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="E32" s="123" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="124" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="B33" s="111" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="C33" s="120" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D33" s="111" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="E33" s="125" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(tracker): TheRundown Pro verified; odds quota risk closed
Closes the Critical quota risk. Also records two corrections worth keeping.

The odds cycle is fixture-gated, not league-gated: a measured run cost ZERO
requests, because _dates_with_fixtures skips a league with no fixtures in the
window. My earlier 3,360/month (67% of quota) estimate assumed every league plays
every day -- a worst case, not a forecast. Adding a league costs nothing until it
plays, which makes expansion much cheaper than budgeted.

And the upgrade does not fix a present symptom: everything playing this week is on
leagues TheRundown does not cover, already served by API-Football. Its value starts
at MLS on 08 Aug and EPL on 21 Aug.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E9620C8-618F-4334-BEBA-AEF71B9C1B3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E5B8AA7-A2CD-4C51-A215-05031B1E7366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="866" uniqueCount="462">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="471">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -933,6 +933,18 @@
   </si>
   <si>
     <t>Traded exact alignment for a badge that cannot collapse or run away</t>
+  </si>
+  <si>
+    <t>TheRundown Pro live and verified</t>
+  </si>
+  <si>
+    <t>5,000/MONTH (not per day). GET /sports 200, 36 sports, quota fresh</t>
+  </si>
+  <si>
+    <t>Measure real odds-cycle quota cost</t>
+  </si>
+  <si>
+    <t>A full cycle cost 0 requests: cost scales with fixtures played, not leagues</t>
   </si>
   <si>
     <t>Legend</t>
@@ -1494,6 +1506,21 @@
   </si>
   <si>
     <t>There is no separate test database; every suite seeds the dev one. test_watchlist.py omitted cleanup and 24 fake sports reached the app's live dropdown, and a running ingest worker computed 30 real feature vectors against them. Every other test file cleans up by convention alone - nothing enforces it. A dedicated test database, or a session-scoped truncate, would remove the whole class.</t>
+  </si>
+  <si>
+    <t>Resolved by a Pro subscription, verified live: 5,000/month, quota fresh. Note it is a MONTHLY budget, so a heavy week cannot be absorbed by waiting a day - ODDS_LOOKAHEAD_DAYS=3 stays as the ceiling that protects a busy matchday.</t>
+  </si>
+  <si>
+    <t>Odds quota cost is fixture-gated, not league-gated</t>
+  </si>
+  <si>
+    <t>A measured cycle cost ZERO requests. _dates_with_fixtures only requests dates that actually have a fixture and skips a league with none, so cost scales with matches PLAYED rather than leagues configured. An earlier estimate of 3,360/month (67% of quota) assumed every league plays every day and was a worst case, not a forecast. Adding a league costs nothing until it plays - which changes how cheap expansion is.</t>
+  </si>
+  <si>
+    <t>TheRundown value starts 21 Aug, not today</t>
+  </si>
+  <si>
+    <t>Everything playing this week (CSL, Scottish Prem, Brasileirao) is on leagues TheRundown does not cover and already has current odds from API-Football. Its coverage begins to matter at MLS on 08 Aug and properly at EPL on 21 Aug. The upgrade is correctly timed rather than fixing a present symptom - no odds are currently degrading.</t>
   </si>
 </sst>
 </file>
@@ -1503,7 +1530,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\ mmm"/>
   </numFmts>
-  <fonts count="50" x14ac:knownFonts="1">
+  <fonts count="54" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1784,8 +1811,30 @@
       <color rgb="FF6B7280"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF111827"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF111827"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF6B7280"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="45">
+  <fills count="50">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2007,8 +2056,33 @@
         <fgColor rgb="FF94A3B8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF16A34A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDC2626"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF94A3B8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -2199,11 +2273,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="188">
+  <cellXfs count="206">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2680,12 +2769,66 @@
     <xf numFmtId="0" fontId="47" fillId="40" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="50" fillId="45" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="45" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="46" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="45" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="51" fillId="45" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="45" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="46" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="47" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="47" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="47" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="51" fillId="47" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="47" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="47" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="48" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="47" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="45" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="49" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="45" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2751,7 +2894,7 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3071,7 +3214,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R134"/>
+  <dimension ref="A1:R136"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3085,46 +3228,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="163" t="s">
+      <c r="A1" s="181" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="161"/>
-      <c r="C1" s="161"/>
-      <c r="D1" s="161"/>
-      <c r="E1" s="161"/>
-      <c r="F1" s="161"/>
-      <c r="G1" s="161"/>
-      <c r="H1" s="161"/>
-      <c r="I1" s="161"/>
-      <c r="J1" s="161"/>
-      <c r="K1" s="161"/>
-      <c r="L1" s="161"/>
-      <c r="M1" s="161"/>
-      <c r="N1" s="161"/>
-      <c r="O1" s="161"/>
-      <c r="P1" s="161"/>
-      <c r="Q1" s="162"/>
+      <c r="B1" s="179"/>
+      <c r="C1" s="179"/>
+      <c r="D1" s="179"/>
+      <c r="E1" s="179"/>
+      <c r="F1" s="179"/>
+      <c r="G1" s="179"/>
+      <c r="H1" s="179"/>
+      <c r="I1" s="179"/>
+      <c r="J1" s="179"/>
+      <c r="K1" s="179"/>
+      <c r="L1" s="179"/>
+      <c r="M1" s="179"/>
+      <c r="N1" s="179"/>
+      <c r="O1" s="179"/>
+      <c r="P1" s="179"/>
+      <c r="Q1" s="180"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="160" t="s">
+      <c r="A2" s="178" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="161"/>
-      <c r="C2" s="161"/>
-      <c r="D2" s="161"/>
-      <c r="E2" s="161"/>
-      <c r="F2" s="161"/>
-      <c r="G2" s="161"/>
-      <c r="H2" s="161"/>
-      <c r="I2" s="161"/>
-      <c r="J2" s="161"/>
-      <c r="K2" s="161"/>
-      <c r="L2" s="161"/>
-      <c r="M2" s="161"/>
-      <c r="N2" s="161"/>
-      <c r="O2" s="161"/>
-      <c r="P2" s="161"/>
-      <c r="Q2" s="162"/>
+      <c r="B2" s="179"/>
+      <c r="C2" s="179"/>
+      <c r="D2" s="179"/>
+      <c r="E2" s="179"/>
+      <c r="F2" s="179"/>
+      <c r="G2" s="179"/>
+      <c r="H2" s="179"/>
+      <c r="I2" s="179"/>
+      <c r="J2" s="179"/>
+      <c r="K2" s="179"/>
+      <c r="L2" s="179"/>
+      <c r="M2" s="179"/>
+      <c r="N2" s="179"/>
+      <c r="O2" s="179"/>
+      <c r="P2" s="179"/>
+      <c r="Q2" s="180"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
@@ -6678,7 +6821,7 @@
       <c r="P102" s="11"/>
       <c r="Q102" s="11"/>
       <c r="R102" t="str">
-        <f t="shared" ref="R102:R132" si="3">IF($A102&lt;&gt;"",$A102,R101)</f>
+        <f t="shared" ref="R102:R134" si="3">IF($A102&lt;&gt;"",$A102,R101)</f>
         <v>E9 Data Ops</v>
       </c>
     </row>
@@ -7792,23 +7935,97 @@
         <v>E7 Mobile</v>
       </c>
     </row>
+    <row r="133" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A133" s="160" t="s">
+        <v>130</v>
+      </c>
+      <c r="B133" s="161" t="s">
+        <v>299</v>
+      </c>
+      <c r="C133" s="162" t="s">
+        <v>22</v>
+      </c>
+      <c r="D133" s="163" t="s">
+        <v>33</v>
+      </c>
+      <c r="E133" s="164">
+        <v>46239</v>
+      </c>
+      <c r="F133" s="164">
+        <v>46239</v>
+      </c>
+      <c r="G133" s="165" t="s">
+        <v>300</v>
+      </c>
+      <c r="H133" s="161"/>
+      <c r="I133" s="166"/>
+      <c r="J133" s="161"/>
+      <c r="K133" s="161"/>
+      <c r="L133" s="161"/>
+      <c r="M133" s="161"/>
+      <c r="N133" s="161"/>
+      <c r="O133" s="161"/>
+      <c r="P133" s="161"/>
+      <c r="Q133" s="161"/>
+      <c r="R133" t="str">
+        <f t="shared" si="3"/>
+        <v>E9 Data Ops</v>
+      </c>
+    </row>
     <row r="134" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A134" s="25" t="s">
-        <v>299</v>
-      </c>
-      <c r="B134" s="5" t="s">
+      <c r="A134" s="167" t="s">
+        <v>130</v>
+      </c>
+      <c r="B134" s="168" t="s">
+        <v>301</v>
+      </c>
+      <c r="C134" s="162" t="s">
         <v>22</v>
       </c>
-      <c r="C134" s="17" t="s">
+      <c r="D134" s="169" t="s">
+        <v>33</v>
+      </c>
+      <c r="E134" s="170">
+        <v>46239</v>
+      </c>
+      <c r="F134" s="170">
+        <v>46239</v>
+      </c>
+      <c r="G134" s="171" t="s">
+        <v>302</v>
+      </c>
+      <c r="H134" s="168"/>
+      <c r="I134" s="166"/>
+      <c r="J134" s="168"/>
+      <c r="K134" s="168"/>
+      <c r="L134" s="168"/>
+      <c r="M134" s="168"/>
+      <c r="N134" s="168"/>
+      <c r="O134" s="168"/>
+      <c r="P134" s="168"/>
+      <c r="Q134" s="168"/>
+      <c r="R134" t="str">
+        <f t="shared" si="3"/>
+        <v>E9 Data Ops</v>
+      </c>
+    </row>
+    <row r="136" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A136" s="25" t="s">
+        <v>303</v>
+      </c>
+      <c r="B136" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C136" s="17" t="s">
         <v>231</v>
       </c>
-      <c r="D134" s="19" t="s">
+      <c r="D136" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="E134" s="23" t="s">
+      <c r="E136" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="F134" s="21" t="s">
+      <c r="F136" s="21" t="s">
         <v>136</v>
       </c>
     </row>
@@ -7832,852 +8049,852 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="179" t="s">
-        <v>300</v>
-      </c>
-      <c r="B1" s="169"/>
-      <c r="C1" s="169"/>
-      <c r="D1" s="169"/>
-      <c r="E1" s="169"/>
-      <c r="F1" s="169"/>
-      <c r="G1" s="169"/>
-      <c r="H1" s="169"/>
-      <c r="I1" s="169"/>
-      <c r="J1" s="169"/>
-      <c r="K1" s="169"/>
-      <c r="L1" s="169"/>
-      <c r="M1" s="169"/>
-      <c r="N1" s="169"/>
-      <c r="O1" s="169"/>
-      <c r="P1" s="169"/>
-      <c r="Q1" s="169"/>
-      <c r="R1" s="169"/>
-      <c r="S1" s="169"/>
+      <c r="A1" s="197" t="s">
+        <v>304</v>
+      </c>
+      <c r="B1" s="187"/>
+      <c r="C1" s="187"/>
+      <c r="D1" s="187"/>
+      <c r="E1" s="187"/>
+      <c r="F1" s="187"/>
+      <c r="G1" s="187"/>
+      <c r="H1" s="187"/>
+      <c r="I1" s="187"/>
+      <c r="J1" s="187"/>
+      <c r="K1" s="187"/>
+      <c r="L1" s="187"/>
+      <c r="M1" s="187"/>
+      <c r="N1" s="187"/>
+      <c r="O1" s="187"/>
+      <c r="P1" s="187"/>
+      <c r="Q1" s="187"/>
+      <c r="R1" s="187"/>
+      <c r="S1" s="187"/>
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="186" t="s">
-        <v>301</v>
-      </c>
-      <c r="B2" s="169"/>
-      <c r="C2" s="169"/>
-      <c r="D2" s="169"/>
-      <c r="E2" s="169"/>
-      <c r="F2" s="169"/>
-      <c r="G2" s="169"/>
-      <c r="H2" s="169"/>
-      <c r="I2" s="169"/>
-      <c r="J2" s="169"/>
-      <c r="K2" s="169"/>
-      <c r="L2" s="169"/>
-      <c r="M2" s="169"/>
-      <c r="N2" s="169"/>
-      <c r="O2" s="169"/>
-      <c r="P2" s="169"/>
-      <c r="Q2" s="169"/>
-      <c r="R2" s="169"/>
-      <c r="S2" s="169"/>
+      <c r="A2" s="204" t="s">
+        <v>305</v>
+      </c>
+      <c r="B2" s="187"/>
+      <c r="C2" s="187"/>
+      <c r="D2" s="187"/>
+      <c r="E2" s="187"/>
+      <c r="F2" s="187"/>
+      <c r="G2" s="187"/>
+      <c r="H2" s="187"/>
+      <c r="I2" s="187"/>
+      <c r="J2" s="187"/>
+      <c r="K2" s="187"/>
+      <c r="L2" s="187"/>
+      <c r="M2" s="187"/>
+      <c r="N2" s="187"/>
+      <c r="O2" s="187"/>
+      <c r="P2" s="187"/>
+      <c r="Q2" s="187"/>
+      <c r="R2" s="187"/>
+      <c r="S2" s="187"/>
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="174" t="s">
-        <v>302</v>
-      </c>
-      <c r="B4" s="169"/>
-      <c r="C4" s="169"/>
-      <c r="D4" s="169"/>
-      <c r="E4" s="169"/>
-      <c r="F4" s="169"/>
-      <c r="G4" s="169"/>
-      <c r="H4" s="169"/>
-      <c r="I4" s="169"/>
-      <c r="J4" s="169"/>
-      <c r="K4" s="169"/>
-      <c r="L4" s="169"/>
-      <c r="M4" s="169"/>
-      <c r="N4" s="169"/>
-      <c r="O4" s="169"/>
-      <c r="P4" s="169"/>
-      <c r="Q4" s="169"/>
-      <c r="R4" s="169"/>
-      <c r="S4" s="169"/>
+      <c r="A4" s="192" t="s">
+        <v>306</v>
+      </c>
+      <c r="B4" s="187"/>
+      <c r="C4" s="187"/>
+      <c r="D4" s="187"/>
+      <c r="E4" s="187"/>
+      <c r="F4" s="187"/>
+      <c r="G4" s="187"/>
+      <c r="H4" s="187"/>
+      <c r="I4" s="187"/>
+      <c r="J4" s="187"/>
+      <c r="K4" s="187"/>
+      <c r="L4" s="187"/>
+      <c r="M4" s="187"/>
+      <c r="N4" s="187"/>
+      <c r="O4" s="187"/>
+      <c r="P4" s="187"/>
+      <c r="Q4" s="187"/>
+      <c r="R4" s="187"/>
+      <c r="S4" s="187"/>
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="37" t="s">
-        <v>303</v>
-      </c>
-      <c r="B5" s="164" t="s">
-        <v>304</v>
-      </c>
-      <c r="C5" s="165"/>
-      <c r="D5" s="166"/>
-      <c r="E5" s="167" t="s">
-        <v>305</v>
-      </c>
-      <c r="F5" s="165"/>
-      <c r="G5" s="166"/>
-      <c r="H5" s="167" t="s">
-        <v>306</v>
-      </c>
-      <c r="I5" s="165"/>
-      <c r="J5" s="166"/>
-      <c r="K5" s="164" t="s">
         <v>307</v>
       </c>
-      <c r="L5" s="165"/>
-      <c r="M5" s="166"/>
-      <c r="N5" s="171" t="s">
+      <c r="B5" s="182" t="s">
         <v>308</v>
       </c>
-      <c r="O5" s="165"/>
-      <c r="P5" s="166"/>
-      <c r="Q5" s="171" t="s">
+      <c r="C5" s="183"/>
+      <c r="D5" s="184"/>
+      <c r="E5" s="185" t="s">
         <v>309</v>
       </c>
-      <c r="R5" s="165"/>
-      <c r="S5" s="166"/>
+      <c r="F5" s="183"/>
+      <c r="G5" s="184"/>
+      <c r="H5" s="185" t="s">
+        <v>310</v>
+      </c>
+      <c r="I5" s="183"/>
+      <c r="J5" s="184"/>
+      <c r="K5" s="182" t="s">
+        <v>311</v>
+      </c>
+      <c r="L5" s="183"/>
+      <c r="M5" s="184"/>
+      <c r="N5" s="189" t="s">
+        <v>312</v>
+      </c>
+      <c r="O5" s="183"/>
+      <c r="P5" s="184"/>
+      <c r="Q5" s="189" t="s">
+        <v>313</v>
+      </c>
+      <c r="R5" s="183"/>
+      <c r="S5" s="184"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="168" t="s">
-        <v>310</v>
-      </c>
-      <c r="C6" s="169"/>
-      <c r="D6" s="169"/>
-      <c r="E6" s="169"/>
-      <c r="F6" s="169"/>
-      <c r="G6" s="169"/>
-      <c r="H6" s="169"/>
-      <c r="I6" s="169"/>
-      <c r="J6" s="169"/>
-      <c r="K6" s="169"/>
-      <c r="L6" s="169"/>
-      <c r="M6" s="169"/>
-      <c r="N6" s="169"/>
-      <c r="O6" s="169"/>
-      <c r="P6" s="169"/>
-      <c r="Q6" s="169"/>
-      <c r="R6" s="169"/>
-      <c r="S6" s="169"/>
+      <c r="B6" s="186" t="s">
+        <v>314</v>
+      </c>
+      <c r="C6" s="187"/>
+      <c r="D6" s="187"/>
+      <c r="E6" s="187"/>
+      <c r="F6" s="187"/>
+      <c r="G6" s="187"/>
+      <c r="H6" s="187"/>
+      <c r="I6" s="187"/>
+      <c r="J6" s="187"/>
+      <c r="K6" s="187"/>
+      <c r="L6" s="187"/>
+      <c r="M6" s="187"/>
+      <c r="N6" s="187"/>
+      <c r="O6" s="187"/>
+      <c r="P6" s="187"/>
+      <c r="Q6" s="187"/>
+      <c r="R6" s="187"/>
+      <c r="S6" s="187"/>
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="174" t="s">
-        <v>311</v>
-      </c>
-      <c r="B7" s="169"/>
-      <c r="C7" s="169"/>
-      <c r="D7" s="169"/>
-      <c r="E7" s="169"/>
-      <c r="F7" s="169"/>
-      <c r="G7" s="169"/>
-      <c r="H7" s="169"/>
-      <c r="I7" s="169"/>
-      <c r="J7" s="169"/>
-      <c r="K7" s="169"/>
-      <c r="L7" s="169"/>
-      <c r="M7" s="169"/>
-      <c r="N7" s="169"/>
-      <c r="O7" s="169"/>
-      <c r="P7" s="169"/>
-      <c r="Q7" s="169"/>
-      <c r="R7" s="169"/>
-      <c r="S7" s="169"/>
+      <c r="A7" s="192" t="s">
+        <v>315</v>
+      </c>
+      <c r="B7" s="187"/>
+      <c r="C7" s="187"/>
+      <c r="D7" s="187"/>
+      <c r="E7" s="187"/>
+      <c r="F7" s="187"/>
+      <c r="G7" s="187"/>
+      <c r="H7" s="187"/>
+      <c r="I7" s="187"/>
+      <c r="J7" s="187"/>
+      <c r="K7" s="187"/>
+      <c r="L7" s="187"/>
+      <c r="M7" s="187"/>
+      <c r="N7" s="187"/>
+      <c r="O7" s="187"/>
+      <c r="P7" s="187"/>
+      <c r="Q7" s="187"/>
+      <c r="R7" s="187"/>
+      <c r="S7" s="187"/>
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="37" t="s">
-        <v>312</v>
-      </c>
-      <c r="B8" s="177" t="s">
-        <v>313</v>
-      </c>
-      <c r="C8" s="165"/>
-      <c r="D8" s="165"/>
-      <c r="E8" s="165"/>
-      <c r="F8" s="165"/>
-      <c r="G8" s="165"/>
-      <c r="H8" s="165"/>
-      <c r="I8" s="165"/>
-      <c r="J8" s="166"/>
-      <c r="K8" s="177" t="s">
+        <v>316</v>
+      </c>
+      <c r="B8" s="195" t="s">
+        <v>317</v>
+      </c>
+      <c r="C8" s="183"/>
+      <c r="D8" s="183"/>
+      <c r="E8" s="183"/>
+      <c r="F8" s="183"/>
+      <c r="G8" s="183"/>
+      <c r="H8" s="183"/>
+      <c r="I8" s="183"/>
+      <c r="J8" s="184"/>
+      <c r="K8" s="195" t="s">
+        <v>318</v>
+      </c>
+      <c r="L8" s="183"/>
+      <c r="M8" s="183"/>
+      <c r="N8" s="183"/>
+      <c r="O8" s="183"/>
+      <c r="P8" s="183"/>
+      <c r="Q8" s="183"/>
+      <c r="R8" s="183"/>
+      <c r="S8" s="184"/>
+    </row>
+    <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B9" s="186" t="s">
         <v>314</v>
       </c>
-      <c r="L8" s="165"/>
-      <c r="M8" s="165"/>
-      <c r="N8" s="165"/>
-      <c r="O8" s="165"/>
-      <c r="P8" s="165"/>
-      <c r="Q8" s="165"/>
-      <c r="R8" s="165"/>
-      <c r="S8" s="166"/>
-    </row>
-    <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B9" s="168" t="s">
-        <v>310</v>
-      </c>
-      <c r="C9" s="169"/>
-      <c r="D9" s="169"/>
-      <c r="E9" s="169"/>
-      <c r="F9" s="169"/>
-      <c r="G9" s="169"/>
-      <c r="H9" s="169"/>
-      <c r="I9" s="169"/>
-      <c r="J9" s="169"/>
-      <c r="K9" s="169"/>
-      <c r="L9" s="169"/>
-      <c r="M9" s="169"/>
-      <c r="N9" s="169"/>
-      <c r="O9" s="169"/>
-      <c r="P9" s="169"/>
-      <c r="Q9" s="169"/>
-      <c r="R9" s="169"/>
-      <c r="S9" s="169"/>
+      <c r="C9" s="187"/>
+      <c r="D9" s="187"/>
+      <c r="E9" s="187"/>
+      <c r="F9" s="187"/>
+      <c r="G9" s="187"/>
+      <c r="H9" s="187"/>
+      <c r="I9" s="187"/>
+      <c r="J9" s="187"/>
+      <c r="K9" s="187"/>
+      <c r="L9" s="187"/>
+      <c r="M9" s="187"/>
+      <c r="N9" s="187"/>
+      <c r="O9" s="187"/>
+      <c r="P9" s="187"/>
+      <c r="Q9" s="187"/>
+      <c r="R9" s="187"/>
+      <c r="S9" s="187"/>
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="174" t="s">
-        <v>315</v>
-      </c>
-      <c r="B10" s="169"/>
-      <c r="C10" s="169"/>
-      <c r="D10" s="169"/>
-      <c r="E10" s="169"/>
-      <c r="F10" s="169"/>
-      <c r="G10" s="169"/>
-      <c r="H10" s="169"/>
-      <c r="I10" s="169"/>
-      <c r="J10" s="169"/>
-      <c r="K10" s="169"/>
-      <c r="L10" s="169"/>
-      <c r="M10" s="169"/>
-      <c r="N10" s="169"/>
-      <c r="O10" s="169"/>
-      <c r="P10" s="169"/>
-      <c r="Q10" s="169"/>
-      <c r="R10" s="169"/>
-      <c r="S10" s="169"/>
+      <c r="A10" s="192" t="s">
+        <v>319</v>
+      </c>
+      <c r="B10" s="187"/>
+      <c r="C10" s="187"/>
+      <c r="D10" s="187"/>
+      <c r="E10" s="187"/>
+      <c r="F10" s="187"/>
+      <c r="G10" s="187"/>
+      <c r="H10" s="187"/>
+      <c r="I10" s="187"/>
+      <c r="J10" s="187"/>
+      <c r="K10" s="187"/>
+      <c r="L10" s="187"/>
+      <c r="M10" s="187"/>
+      <c r="N10" s="187"/>
+      <c r="O10" s="187"/>
+      <c r="P10" s="187"/>
+      <c r="Q10" s="187"/>
+      <c r="R10" s="187"/>
+      <c r="S10" s="187"/>
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="37" t="s">
-        <v>316</v>
-      </c>
-      <c r="B11" s="164" t="s">
-        <v>317</v>
-      </c>
-      <c r="C11" s="165"/>
-      <c r="D11" s="166"/>
-      <c r="E11" s="164" t="s">
-        <v>318</v>
-      </c>
-      <c r="F11" s="165"/>
-      <c r="G11" s="166"/>
-      <c r="H11" s="164" t="s">
-        <v>319</v>
-      </c>
-      <c r="I11" s="165"/>
-      <c r="J11" s="166"/>
-      <c r="K11" s="167" t="s">
         <v>320</v>
       </c>
-      <c r="L11" s="165"/>
-      <c r="M11" s="166"/>
-      <c r="N11" s="164" t="s">
+      <c r="B11" s="182" t="s">
         <v>321</v>
       </c>
-      <c r="O11" s="165"/>
-      <c r="P11" s="166"/>
-      <c r="Q11" s="164" t="s">
+      <c r="C11" s="183"/>
+      <c r="D11" s="184"/>
+      <c r="E11" s="182" t="s">
         <v>322</v>
       </c>
-      <c r="R11" s="165"/>
-      <c r="S11" s="166"/>
+      <c r="F11" s="183"/>
+      <c r="G11" s="184"/>
+      <c r="H11" s="182" t="s">
+        <v>323</v>
+      </c>
+      <c r="I11" s="183"/>
+      <c r="J11" s="184"/>
+      <c r="K11" s="185" t="s">
+        <v>324</v>
+      </c>
+      <c r="L11" s="183"/>
+      <c r="M11" s="184"/>
+      <c r="N11" s="182" t="s">
+        <v>325</v>
+      </c>
+      <c r="O11" s="183"/>
+      <c r="P11" s="184"/>
+      <c r="Q11" s="182" t="s">
+        <v>326</v>
+      </c>
+      <c r="R11" s="183"/>
+      <c r="S11" s="184"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B12" s="168" t="s">
-        <v>310</v>
-      </c>
-      <c r="C12" s="169"/>
-      <c r="D12" s="169"/>
-      <c r="E12" s="169"/>
-      <c r="F12" s="169"/>
-      <c r="G12" s="169"/>
-      <c r="H12" s="169"/>
-      <c r="I12" s="169"/>
-      <c r="J12" s="169"/>
-      <c r="K12" s="169"/>
-      <c r="L12" s="169"/>
-      <c r="M12" s="169"/>
-      <c r="N12" s="169"/>
-      <c r="O12" s="169"/>
-      <c r="P12" s="169"/>
-      <c r="Q12" s="169"/>
-      <c r="R12" s="169"/>
-      <c r="S12" s="169"/>
+      <c r="B12" s="186" t="s">
+        <v>314</v>
+      </c>
+      <c r="C12" s="187"/>
+      <c r="D12" s="187"/>
+      <c r="E12" s="187"/>
+      <c r="F12" s="187"/>
+      <c r="G12" s="187"/>
+      <c r="H12" s="187"/>
+      <c r="I12" s="187"/>
+      <c r="J12" s="187"/>
+      <c r="K12" s="187"/>
+      <c r="L12" s="187"/>
+      <c r="M12" s="187"/>
+      <c r="N12" s="187"/>
+      <c r="O12" s="187"/>
+      <c r="P12" s="187"/>
+      <c r="Q12" s="187"/>
+      <c r="R12" s="187"/>
+      <c r="S12" s="187"/>
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="174" t="s">
-        <v>323</v>
-      </c>
-      <c r="B13" s="169"/>
-      <c r="C13" s="169"/>
-      <c r="D13" s="169"/>
-      <c r="E13" s="169"/>
-      <c r="F13" s="169"/>
-      <c r="G13" s="169"/>
-      <c r="H13" s="169"/>
-      <c r="I13" s="169"/>
-      <c r="J13" s="169"/>
-      <c r="K13" s="169"/>
-      <c r="L13" s="169"/>
-      <c r="M13" s="169"/>
-      <c r="N13" s="169"/>
-      <c r="O13" s="169"/>
-      <c r="P13" s="169"/>
-      <c r="Q13" s="169"/>
-      <c r="R13" s="169"/>
-      <c r="S13" s="169"/>
+      <c r="A13" s="192" t="s">
+        <v>327</v>
+      </c>
+      <c r="B13" s="187"/>
+      <c r="C13" s="187"/>
+      <c r="D13" s="187"/>
+      <c r="E13" s="187"/>
+      <c r="F13" s="187"/>
+      <c r="G13" s="187"/>
+      <c r="H13" s="187"/>
+      <c r="I13" s="187"/>
+      <c r="J13" s="187"/>
+      <c r="K13" s="187"/>
+      <c r="L13" s="187"/>
+      <c r="M13" s="187"/>
+      <c r="N13" s="187"/>
+      <c r="O13" s="187"/>
+      <c r="P13" s="187"/>
+      <c r="Q13" s="187"/>
+      <c r="R13" s="187"/>
+      <c r="S13" s="187"/>
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="37" t="s">
-        <v>324</v>
-      </c>
-      <c r="B14" s="172" t="s">
-        <v>325</v>
-      </c>
-      <c r="C14" s="165"/>
-      <c r="D14" s="165"/>
-      <c r="E14" s="165"/>
-      <c r="F14" s="165"/>
-      <c r="G14" s="166"/>
-      <c r="H14" s="172" t="s">
-        <v>326</v>
-      </c>
-      <c r="I14" s="165"/>
-      <c r="J14" s="165"/>
-      <c r="K14" s="165"/>
-      <c r="L14" s="165"/>
-      <c r="M14" s="166"/>
-      <c r="N14" s="172" t="s">
-        <v>327</v>
-      </c>
-      <c r="O14" s="165"/>
-      <c r="P14" s="166"/>
-      <c r="Q14" s="167" t="s">
         <v>328</v>
       </c>
-      <c r="R14" s="165"/>
-      <c r="S14" s="166"/>
+      <c r="B14" s="190" t="s">
+        <v>329</v>
+      </c>
+      <c r="C14" s="183"/>
+      <c r="D14" s="183"/>
+      <c r="E14" s="183"/>
+      <c r="F14" s="183"/>
+      <c r="G14" s="184"/>
+      <c r="H14" s="190" t="s">
+        <v>330</v>
+      </c>
+      <c r="I14" s="183"/>
+      <c r="J14" s="183"/>
+      <c r="K14" s="183"/>
+      <c r="L14" s="183"/>
+      <c r="M14" s="184"/>
+      <c r="N14" s="190" t="s">
+        <v>331</v>
+      </c>
+      <c r="O14" s="183"/>
+      <c r="P14" s="184"/>
+      <c r="Q14" s="185" t="s">
+        <v>332</v>
+      </c>
+      <c r="R14" s="183"/>
+      <c r="S14" s="184"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B15" s="168" t="s">
-        <v>329</v>
-      </c>
-      <c r="C15" s="169"/>
-      <c r="D15" s="169"/>
-      <c r="E15" s="169"/>
-      <c r="F15" s="169"/>
-      <c r="G15" s="169"/>
-      <c r="H15" s="169"/>
-      <c r="I15" s="169"/>
-      <c r="J15" s="169"/>
-      <c r="K15" s="169"/>
-      <c r="L15" s="169"/>
-      <c r="M15" s="169"/>
-      <c r="N15" s="169"/>
-      <c r="O15" s="169"/>
-      <c r="P15" s="169"/>
-      <c r="Q15" s="169"/>
-      <c r="R15" s="169"/>
-      <c r="S15" s="169"/>
+      <c r="B15" s="186" t="s">
+        <v>333</v>
+      </c>
+      <c r="C15" s="187"/>
+      <c r="D15" s="187"/>
+      <c r="E15" s="187"/>
+      <c r="F15" s="187"/>
+      <c r="G15" s="187"/>
+      <c r="H15" s="187"/>
+      <c r="I15" s="187"/>
+      <c r="J15" s="187"/>
+      <c r="K15" s="187"/>
+      <c r="L15" s="187"/>
+      <c r="M15" s="187"/>
+      <c r="N15" s="187"/>
+      <c r="O15" s="187"/>
+      <c r="P15" s="187"/>
+      <c r="Q15" s="187"/>
+      <c r="R15" s="187"/>
+      <c r="S15" s="187"/>
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="174" t="s">
-        <v>330</v>
-      </c>
-      <c r="B16" s="169"/>
-      <c r="C16" s="169"/>
-      <c r="D16" s="169"/>
-      <c r="E16" s="169"/>
-      <c r="F16" s="169"/>
-      <c r="G16" s="169"/>
-      <c r="H16" s="169"/>
-      <c r="I16" s="169"/>
-      <c r="J16" s="169"/>
-      <c r="K16" s="169"/>
-      <c r="L16" s="169"/>
-      <c r="M16" s="169"/>
-      <c r="N16" s="169"/>
-      <c r="O16" s="169"/>
-      <c r="P16" s="169"/>
-      <c r="Q16" s="169"/>
-      <c r="R16" s="169"/>
-      <c r="S16" s="169"/>
+      <c r="A16" s="192" t="s">
+        <v>334</v>
+      </c>
+      <c r="B16" s="187"/>
+      <c r="C16" s="187"/>
+      <c r="D16" s="187"/>
+      <c r="E16" s="187"/>
+      <c r="F16" s="187"/>
+      <c r="G16" s="187"/>
+      <c r="H16" s="187"/>
+      <c r="I16" s="187"/>
+      <c r="J16" s="187"/>
+      <c r="K16" s="187"/>
+      <c r="L16" s="187"/>
+      <c r="M16" s="187"/>
+      <c r="N16" s="187"/>
+      <c r="O16" s="187"/>
+      <c r="P16" s="187"/>
+      <c r="Q16" s="187"/>
+      <c r="R16" s="187"/>
+      <c r="S16" s="187"/>
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="37" t="s">
-        <v>331</v>
-      </c>
-      <c r="B17" s="173" t="s">
-        <v>332</v>
-      </c>
-      <c r="C17" s="165"/>
-      <c r="D17" s="165"/>
-      <c r="E17" s="165"/>
-      <c r="F17" s="165"/>
-      <c r="G17" s="166"/>
-      <c r="H17" s="173" t="s">
-        <v>333</v>
-      </c>
-      <c r="I17" s="165"/>
-      <c r="J17" s="166"/>
-      <c r="K17" s="173" t="s">
-        <v>334</v>
-      </c>
-      <c r="L17" s="165"/>
-      <c r="M17" s="166"/>
-      <c r="N17" s="173" t="s">
         <v>335</v>
       </c>
-      <c r="O17" s="165"/>
-      <c r="P17" s="166"/>
-      <c r="Q17" s="173" t="s">
+      <c r="B17" s="191" t="s">
         <v>336</v>
       </c>
-      <c r="R17" s="165"/>
-      <c r="S17" s="166"/>
+      <c r="C17" s="183"/>
+      <c r="D17" s="183"/>
+      <c r="E17" s="183"/>
+      <c r="F17" s="183"/>
+      <c r="G17" s="184"/>
+      <c r="H17" s="191" t="s">
+        <v>337</v>
+      </c>
+      <c r="I17" s="183"/>
+      <c r="J17" s="184"/>
+      <c r="K17" s="191" t="s">
+        <v>338</v>
+      </c>
+      <c r="L17" s="183"/>
+      <c r="M17" s="184"/>
+      <c r="N17" s="191" t="s">
+        <v>339</v>
+      </c>
+      <c r="O17" s="183"/>
+      <c r="P17" s="184"/>
+      <c r="Q17" s="191" t="s">
+        <v>340</v>
+      </c>
+      <c r="R17" s="183"/>
+      <c r="S17" s="184"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="168" t="s">
-        <v>310</v>
-      </c>
-      <c r="C18" s="169"/>
-      <c r="D18" s="169"/>
-      <c r="E18" s="169"/>
-      <c r="F18" s="169"/>
-      <c r="G18" s="169"/>
-      <c r="H18" s="169"/>
-      <c r="I18" s="169"/>
-      <c r="J18" s="169"/>
-      <c r="K18" s="169"/>
-      <c r="L18" s="169"/>
-      <c r="M18" s="169"/>
-      <c r="N18" s="169"/>
-      <c r="O18" s="169"/>
-      <c r="P18" s="169"/>
-      <c r="Q18" s="169"/>
-      <c r="R18" s="169"/>
-      <c r="S18" s="169"/>
+      <c r="B18" s="186" t="s">
+        <v>314</v>
+      </c>
+      <c r="C18" s="187"/>
+      <c r="D18" s="187"/>
+      <c r="E18" s="187"/>
+      <c r="F18" s="187"/>
+      <c r="G18" s="187"/>
+      <c r="H18" s="187"/>
+      <c r="I18" s="187"/>
+      <c r="J18" s="187"/>
+      <c r="K18" s="187"/>
+      <c r="L18" s="187"/>
+      <c r="M18" s="187"/>
+      <c r="N18" s="187"/>
+      <c r="O18" s="187"/>
+      <c r="P18" s="187"/>
+      <c r="Q18" s="187"/>
+      <c r="R18" s="187"/>
+      <c r="S18" s="187"/>
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="174" t="s">
-        <v>337</v>
-      </c>
-      <c r="B19" s="169"/>
-      <c r="C19" s="169"/>
-      <c r="D19" s="169"/>
-      <c r="E19" s="169"/>
-      <c r="F19" s="169"/>
-      <c r="G19" s="169"/>
-      <c r="H19" s="169"/>
-      <c r="I19" s="169"/>
-      <c r="J19" s="169"/>
-      <c r="K19" s="169"/>
-      <c r="L19" s="169"/>
-      <c r="M19" s="169"/>
-      <c r="N19" s="169"/>
-      <c r="O19" s="169"/>
-      <c r="P19" s="169"/>
-      <c r="Q19" s="169"/>
-      <c r="R19" s="169"/>
-      <c r="S19" s="169"/>
+      <c r="A19" s="192" t="s">
+        <v>341</v>
+      </c>
+      <c r="B19" s="187"/>
+      <c r="C19" s="187"/>
+      <c r="D19" s="187"/>
+      <c r="E19" s="187"/>
+      <c r="F19" s="187"/>
+      <c r="G19" s="187"/>
+      <c r="H19" s="187"/>
+      <c r="I19" s="187"/>
+      <c r="J19" s="187"/>
+      <c r="K19" s="187"/>
+      <c r="L19" s="187"/>
+      <c r="M19" s="187"/>
+      <c r="N19" s="187"/>
+      <c r="O19" s="187"/>
+      <c r="P19" s="187"/>
+      <c r="Q19" s="187"/>
+      <c r="R19" s="187"/>
+      <c r="S19" s="187"/>
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="37" t="s">
-        <v>338</v>
-      </c>
-      <c r="B20" s="175" t="s">
-        <v>339</v>
-      </c>
-      <c r="C20" s="165"/>
-      <c r="D20" s="165"/>
-      <c r="E20" s="165"/>
-      <c r="F20" s="165"/>
-      <c r="G20" s="166"/>
-      <c r="H20" s="175" t="s">
-        <v>340</v>
-      </c>
-      <c r="I20" s="165"/>
-      <c r="J20" s="165"/>
-      <c r="K20" s="165"/>
-      <c r="L20" s="165"/>
-      <c r="M20" s="166"/>
-      <c r="N20" s="175" t="s">
-        <v>341</v>
-      </c>
-      <c r="O20" s="165"/>
-      <c r="P20" s="165"/>
-      <c r="Q20" s="165"/>
-      <c r="R20" s="165"/>
-      <c r="S20" s="166"/>
+        <v>342</v>
+      </c>
+      <c r="B20" s="193" t="s">
+        <v>343</v>
+      </c>
+      <c r="C20" s="183"/>
+      <c r="D20" s="183"/>
+      <c r="E20" s="183"/>
+      <c r="F20" s="183"/>
+      <c r="G20" s="184"/>
+      <c r="H20" s="193" t="s">
+        <v>344</v>
+      </c>
+      <c r="I20" s="183"/>
+      <c r="J20" s="183"/>
+      <c r="K20" s="183"/>
+      <c r="L20" s="183"/>
+      <c r="M20" s="184"/>
+      <c r="N20" s="193" t="s">
+        <v>345</v>
+      </c>
+      <c r="O20" s="183"/>
+      <c r="P20" s="183"/>
+      <c r="Q20" s="183"/>
+      <c r="R20" s="183"/>
+      <c r="S20" s="184"/>
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B21" s="168" t="s">
-        <v>310</v>
-      </c>
-      <c r="C21" s="169"/>
-      <c r="D21" s="169"/>
-      <c r="E21" s="169"/>
-      <c r="F21" s="169"/>
-      <c r="G21" s="169"/>
-      <c r="H21" s="169"/>
-      <c r="I21" s="169"/>
-      <c r="J21" s="169"/>
-      <c r="K21" s="169"/>
-      <c r="L21" s="169"/>
-      <c r="M21" s="169"/>
-      <c r="N21" s="169"/>
-      <c r="O21" s="169"/>
-      <c r="P21" s="169"/>
-      <c r="Q21" s="169"/>
-      <c r="R21" s="169"/>
-      <c r="S21" s="169"/>
+      <c r="B21" s="186" t="s">
+        <v>314</v>
+      </c>
+      <c r="C21" s="187"/>
+      <c r="D21" s="187"/>
+      <c r="E21" s="187"/>
+      <c r="F21" s="187"/>
+      <c r="G21" s="187"/>
+      <c r="H21" s="187"/>
+      <c r="I21" s="187"/>
+      <c r="J21" s="187"/>
+      <c r="K21" s="187"/>
+      <c r="L21" s="187"/>
+      <c r="M21" s="187"/>
+      <c r="N21" s="187"/>
+      <c r="O21" s="187"/>
+      <c r="P21" s="187"/>
+      <c r="Q21" s="187"/>
+      <c r="R21" s="187"/>
+      <c r="S21" s="187"/>
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="174" t="s">
-        <v>342</v>
-      </c>
-      <c r="B22" s="169"/>
-      <c r="C22" s="169"/>
-      <c r="D22" s="169"/>
-      <c r="E22" s="169"/>
-      <c r="F22" s="169"/>
-      <c r="G22" s="169"/>
-      <c r="H22" s="169"/>
-      <c r="I22" s="169"/>
-      <c r="J22" s="169"/>
-      <c r="K22" s="169"/>
-      <c r="L22" s="169"/>
-      <c r="M22" s="169"/>
-      <c r="N22" s="169"/>
-      <c r="O22" s="169"/>
-      <c r="P22" s="169"/>
-      <c r="Q22" s="169"/>
-      <c r="R22" s="169"/>
-      <c r="S22" s="169"/>
+      <c r="A22" s="192" t="s">
+        <v>346</v>
+      </c>
+      <c r="B22" s="187"/>
+      <c r="C22" s="187"/>
+      <c r="D22" s="187"/>
+      <c r="E22" s="187"/>
+      <c r="F22" s="187"/>
+      <c r="G22" s="187"/>
+      <c r="H22" s="187"/>
+      <c r="I22" s="187"/>
+      <c r="J22" s="187"/>
+      <c r="K22" s="187"/>
+      <c r="L22" s="187"/>
+      <c r="M22" s="187"/>
+      <c r="N22" s="187"/>
+      <c r="O22" s="187"/>
+      <c r="P22" s="187"/>
+      <c r="Q22" s="187"/>
+      <c r="R22" s="187"/>
+      <c r="S22" s="187"/>
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="37" t="s">
-        <v>343</v>
-      </c>
-      <c r="B23" s="175" t="s">
-        <v>344</v>
-      </c>
-      <c r="C23" s="165"/>
-      <c r="D23" s="165"/>
-      <c r="E23" s="165"/>
-      <c r="F23" s="165"/>
-      <c r="G23" s="166"/>
-      <c r="H23" s="175" t="s">
-        <v>345</v>
-      </c>
-      <c r="I23" s="165"/>
-      <c r="J23" s="166"/>
-      <c r="K23" s="175" t="s">
-        <v>346</v>
-      </c>
-      <c r="L23" s="165"/>
-      <c r="M23" s="166"/>
-      <c r="N23" s="175" t="s">
         <v>347</v>
       </c>
-      <c r="O23" s="165"/>
-      <c r="P23" s="166"/>
-      <c r="Q23" s="171" t="s">
+      <c r="B23" s="193" t="s">
         <v>348</v>
       </c>
-      <c r="R23" s="165"/>
-      <c r="S23" s="166"/>
+      <c r="C23" s="183"/>
+      <c r="D23" s="183"/>
+      <c r="E23" s="183"/>
+      <c r="F23" s="183"/>
+      <c r="G23" s="184"/>
+      <c r="H23" s="193" t="s">
+        <v>349</v>
+      </c>
+      <c r="I23" s="183"/>
+      <c r="J23" s="184"/>
+      <c r="K23" s="193" t="s">
+        <v>350</v>
+      </c>
+      <c r="L23" s="183"/>
+      <c r="M23" s="184"/>
+      <c r="N23" s="193" t="s">
+        <v>351</v>
+      </c>
+      <c r="O23" s="183"/>
+      <c r="P23" s="184"/>
+      <c r="Q23" s="189" t="s">
+        <v>352</v>
+      </c>
+      <c r="R23" s="183"/>
+      <c r="S23" s="184"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="180" t="s">
-        <v>349</v>
-      </c>
-      <c r="B26" s="169"/>
-      <c r="C26" s="169"/>
-      <c r="D26" s="169"/>
-      <c r="E26" s="169"/>
-      <c r="F26" s="169"/>
-      <c r="G26" s="169"/>
-      <c r="H26" s="169"/>
-      <c r="I26" s="169"/>
-      <c r="J26" s="169"/>
-      <c r="K26" s="169"/>
-      <c r="L26" s="169"/>
-      <c r="M26" s="169"/>
-      <c r="N26" s="169"/>
-      <c r="O26" s="169"/>
-      <c r="P26" s="169"/>
-      <c r="Q26" s="169"/>
-      <c r="R26" s="169"/>
-      <c r="S26" s="169"/>
+      <c r="A26" s="198" t="s">
+        <v>353</v>
+      </c>
+      <c r="B26" s="187"/>
+      <c r="C26" s="187"/>
+      <c r="D26" s="187"/>
+      <c r="E26" s="187"/>
+      <c r="F26" s="187"/>
+      <c r="G26" s="187"/>
+      <c r="H26" s="187"/>
+      <c r="I26" s="187"/>
+      <c r="J26" s="187"/>
+      <c r="K26" s="187"/>
+      <c r="L26" s="187"/>
+      <c r="M26" s="187"/>
+      <c r="N26" s="187"/>
+      <c r="O26" s="187"/>
+      <c r="P26" s="187"/>
+      <c r="Q26" s="187"/>
+      <c r="R26" s="187"/>
+      <c r="S26" s="187"/>
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="37" t="s">
-        <v>350</v>
-      </c>
-      <c r="B27" s="164" t="s">
-        <v>351</v>
-      </c>
-      <c r="C27" s="165"/>
-      <c r="D27" s="166"/>
-      <c r="E27" s="164" t="s">
-        <v>352</v>
-      </c>
-      <c r="F27" s="165"/>
-      <c r="G27" s="166"/>
-      <c r="H27" s="172" t="s">
-        <v>353</v>
-      </c>
-      <c r="I27" s="165"/>
-      <c r="J27" s="166"/>
-      <c r="K27" s="173" t="s">
         <v>354</v>
       </c>
-      <c r="L27" s="165"/>
-      <c r="M27" s="166"/>
-      <c r="N27" s="173" t="s">
+      <c r="B27" s="182" t="s">
         <v>355</v>
       </c>
-      <c r="O27" s="165"/>
-      <c r="P27" s="166"/>
-      <c r="Q27" s="172" t="s">
+      <c r="C27" s="183"/>
+      <c r="D27" s="184"/>
+      <c r="E27" s="182" t="s">
         <v>356</v>
       </c>
-      <c r="R27" s="165"/>
-      <c r="S27" s="166"/>
+      <c r="F27" s="183"/>
+      <c r="G27" s="184"/>
+      <c r="H27" s="190" t="s">
+        <v>357</v>
+      </c>
+      <c r="I27" s="183"/>
+      <c r="J27" s="184"/>
+      <c r="K27" s="191" t="s">
+        <v>358</v>
+      </c>
+      <c r="L27" s="183"/>
+      <c r="M27" s="184"/>
+      <c r="N27" s="191" t="s">
+        <v>359</v>
+      </c>
+      <c r="O27" s="183"/>
+      <c r="P27" s="184"/>
+      <c r="Q27" s="190" t="s">
+        <v>360</v>
+      </c>
+      <c r="R27" s="183"/>
+      <c r="S27" s="184"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="174" t="s">
-        <v>357</v>
-      </c>
-      <c r="B30" s="169"/>
-      <c r="C30" s="169"/>
-      <c r="D30" s="169"/>
-      <c r="E30" s="169"/>
-      <c r="F30" s="169"/>
-      <c r="G30" s="169"/>
-      <c r="H30" s="169"/>
-      <c r="I30" s="169"/>
-      <c r="J30" s="169"/>
-      <c r="K30" s="169"/>
-      <c r="L30" s="169"/>
-      <c r="M30" s="169"/>
-      <c r="N30" s="169"/>
-      <c r="O30" s="169"/>
-      <c r="P30" s="169"/>
-      <c r="Q30" s="169"/>
-      <c r="R30" s="169"/>
-      <c r="S30" s="169"/>
+      <c r="A30" s="192" t="s">
+        <v>361</v>
+      </c>
+      <c r="B30" s="187"/>
+      <c r="C30" s="187"/>
+      <c r="D30" s="187"/>
+      <c r="E30" s="187"/>
+      <c r="F30" s="187"/>
+      <c r="G30" s="187"/>
+      <c r="H30" s="187"/>
+      <c r="I30" s="187"/>
+      <c r="J30" s="187"/>
+      <c r="K30" s="187"/>
+      <c r="L30" s="187"/>
+      <c r="M30" s="187"/>
+      <c r="N30" s="187"/>
+      <c r="O30" s="187"/>
+      <c r="P30" s="187"/>
+      <c r="Q30" s="187"/>
+      <c r="R30" s="187"/>
+      <c r="S30" s="187"/>
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="170" t="s">
-        <v>358</v>
-      </c>
-      <c r="B31" s="169"/>
-      <c r="C31" s="169"/>
-      <c r="D31" s="169"/>
-      <c r="E31" s="169"/>
-      <c r="F31" s="169"/>
-      <c r="G31" s="169"/>
-      <c r="H31" s="169"/>
-      <c r="I31" s="169"/>
-      <c r="J31" s="169"/>
-      <c r="K31" s="169"/>
-      <c r="L31" s="169"/>
-      <c r="M31" s="169"/>
-      <c r="N31" s="169"/>
-      <c r="O31" s="169"/>
-      <c r="P31" s="169"/>
-      <c r="Q31" s="169"/>
-      <c r="R31" s="169"/>
-      <c r="S31" s="169"/>
+      <c r="A31" s="188" t="s">
+        <v>362</v>
+      </c>
+      <c r="B31" s="187"/>
+      <c r="C31" s="187"/>
+      <c r="D31" s="187"/>
+      <c r="E31" s="187"/>
+      <c r="F31" s="187"/>
+      <c r="G31" s="187"/>
+      <c r="H31" s="187"/>
+      <c r="I31" s="187"/>
+      <c r="J31" s="187"/>
+      <c r="K31" s="187"/>
+      <c r="L31" s="187"/>
+      <c r="M31" s="187"/>
+      <c r="N31" s="187"/>
+      <c r="O31" s="187"/>
+      <c r="P31" s="187"/>
+      <c r="Q31" s="187"/>
+      <c r="R31" s="187"/>
+      <c r="S31" s="187"/>
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="170" t="s">
-        <v>359</v>
-      </c>
-      <c r="B32" s="169"/>
-      <c r="C32" s="169"/>
-      <c r="D32" s="169"/>
-      <c r="E32" s="169"/>
-      <c r="F32" s="169"/>
-      <c r="G32" s="169"/>
-      <c r="H32" s="169"/>
-      <c r="I32" s="169"/>
-      <c r="J32" s="169"/>
-      <c r="K32" s="169"/>
-      <c r="L32" s="169"/>
-      <c r="M32" s="169"/>
-      <c r="N32" s="169"/>
-      <c r="O32" s="169"/>
-      <c r="P32" s="169"/>
-      <c r="Q32" s="169"/>
-      <c r="R32" s="169"/>
-      <c r="S32" s="169"/>
+      <c r="A32" s="188" t="s">
+        <v>363</v>
+      </c>
+      <c r="B32" s="187"/>
+      <c r="C32" s="187"/>
+      <c r="D32" s="187"/>
+      <c r="E32" s="187"/>
+      <c r="F32" s="187"/>
+      <c r="G32" s="187"/>
+      <c r="H32" s="187"/>
+      <c r="I32" s="187"/>
+      <c r="J32" s="187"/>
+      <c r="K32" s="187"/>
+      <c r="L32" s="187"/>
+      <c r="M32" s="187"/>
+      <c r="N32" s="187"/>
+      <c r="O32" s="187"/>
+      <c r="P32" s="187"/>
+      <c r="Q32" s="187"/>
+      <c r="R32" s="187"/>
+      <c r="S32" s="187"/>
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="170" t="s">
-        <v>360</v>
-      </c>
-      <c r="B33" s="169"/>
-      <c r="C33" s="169"/>
-      <c r="D33" s="169"/>
-      <c r="E33" s="169"/>
-      <c r="F33" s="169"/>
-      <c r="G33" s="169"/>
-      <c r="H33" s="169"/>
-      <c r="I33" s="169"/>
-      <c r="J33" s="169"/>
-      <c r="K33" s="169"/>
-      <c r="L33" s="169"/>
-      <c r="M33" s="169"/>
-      <c r="N33" s="169"/>
-      <c r="O33" s="169"/>
-      <c r="P33" s="169"/>
-      <c r="Q33" s="169"/>
-      <c r="R33" s="169"/>
-      <c r="S33" s="169"/>
+      <c r="A33" s="188" t="s">
+        <v>364</v>
+      </c>
+      <c r="B33" s="187"/>
+      <c r="C33" s="187"/>
+      <c r="D33" s="187"/>
+      <c r="E33" s="187"/>
+      <c r="F33" s="187"/>
+      <c r="G33" s="187"/>
+      <c r="H33" s="187"/>
+      <c r="I33" s="187"/>
+      <c r="J33" s="187"/>
+      <c r="K33" s="187"/>
+      <c r="L33" s="187"/>
+      <c r="M33" s="187"/>
+      <c r="N33" s="187"/>
+      <c r="O33" s="187"/>
+      <c r="P33" s="187"/>
+      <c r="Q33" s="187"/>
+      <c r="R33" s="187"/>
+      <c r="S33" s="187"/>
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="170" t="s">
-        <v>361</v>
-      </c>
-      <c r="B34" s="169"/>
-      <c r="C34" s="169"/>
-      <c r="D34" s="169"/>
-      <c r="E34" s="169"/>
-      <c r="F34" s="169"/>
-      <c r="G34" s="169"/>
-      <c r="H34" s="169"/>
-      <c r="I34" s="169"/>
-      <c r="J34" s="169"/>
-      <c r="K34" s="169"/>
-      <c r="L34" s="169"/>
-      <c r="M34" s="169"/>
-      <c r="N34" s="169"/>
-      <c r="O34" s="169"/>
-      <c r="P34" s="169"/>
-      <c r="Q34" s="169"/>
-      <c r="R34" s="169"/>
-      <c r="S34" s="169"/>
+      <c r="A34" s="188" t="s">
+        <v>365</v>
+      </c>
+      <c r="B34" s="187"/>
+      <c r="C34" s="187"/>
+      <c r="D34" s="187"/>
+      <c r="E34" s="187"/>
+      <c r="F34" s="187"/>
+      <c r="G34" s="187"/>
+      <c r="H34" s="187"/>
+      <c r="I34" s="187"/>
+      <c r="J34" s="187"/>
+      <c r="K34" s="187"/>
+      <c r="L34" s="187"/>
+      <c r="M34" s="187"/>
+      <c r="N34" s="187"/>
+      <c r="O34" s="187"/>
+      <c r="P34" s="187"/>
+      <c r="Q34" s="187"/>
+      <c r="R34" s="187"/>
+      <c r="S34" s="187"/>
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="170" t="s">
-        <v>362</v>
-      </c>
-      <c r="B35" s="169"/>
-      <c r="C35" s="169"/>
-      <c r="D35" s="169"/>
-      <c r="E35" s="169"/>
-      <c r="F35" s="169"/>
-      <c r="G35" s="169"/>
-      <c r="H35" s="169"/>
-      <c r="I35" s="169"/>
-      <c r="J35" s="169"/>
-      <c r="K35" s="169"/>
-      <c r="L35" s="169"/>
-      <c r="M35" s="169"/>
-      <c r="N35" s="169"/>
-      <c r="O35" s="169"/>
-      <c r="P35" s="169"/>
-      <c r="Q35" s="169"/>
-      <c r="R35" s="169"/>
-      <c r="S35" s="169"/>
+      <c r="A35" s="188" t="s">
+        <v>366</v>
+      </c>
+      <c r="B35" s="187"/>
+      <c r="C35" s="187"/>
+      <c r="D35" s="187"/>
+      <c r="E35" s="187"/>
+      <c r="F35" s="187"/>
+      <c r="G35" s="187"/>
+      <c r="H35" s="187"/>
+      <c r="I35" s="187"/>
+      <c r="J35" s="187"/>
+      <c r="K35" s="187"/>
+      <c r="L35" s="187"/>
+      <c r="M35" s="187"/>
+      <c r="N35" s="187"/>
+      <c r="O35" s="187"/>
+      <c r="P35" s="187"/>
+      <c r="Q35" s="187"/>
+      <c r="R35" s="187"/>
+      <c r="S35" s="187"/>
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="170" t="s">
-        <v>363</v>
-      </c>
-      <c r="B36" s="169"/>
-      <c r="C36" s="169"/>
-      <c r="D36" s="169"/>
-      <c r="E36" s="169"/>
-      <c r="F36" s="169"/>
-      <c r="G36" s="169"/>
-      <c r="H36" s="169"/>
-      <c r="I36" s="169"/>
-      <c r="J36" s="169"/>
-      <c r="K36" s="169"/>
-      <c r="L36" s="169"/>
-      <c r="M36" s="169"/>
-      <c r="N36" s="169"/>
-      <c r="O36" s="169"/>
-      <c r="P36" s="169"/>
-      <c r="Q36" s="169"/>
-      <c r="R36" s="169"/>
-      <c r="S36" s="169"/>
+      <c r="A36" s="188" t="s">
+        <v>367</v>
+      </c>
+      <c r="B36" s="187"/>
+      <c r="C36" s="187"/>
+      <c r="D36" s="187"/>
+      <c r="E36" s="187"/>
+      <c r="F36" s="187"/>
+      <c r="G36" s="187"/>
+      <c r="H36" s="187"/>
+      <c r="I36" s="187"/>
+      <c r="J36" s="187"/>
+      <c r="K36" s="187"/>
+      <c r="L36" s="187"/>
+      <c r="M36" s="187"/>
+      <c r="N36" s="187"/>
+      <c r="O36" s="187"/>
+      <c r="P36" s="187"/>
+      <c r="Q36" s="187"/>
+      <c r="R36" s="187"/>
+      <c r="S36" s="187"/>
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="181" t="s">
-        <v>364</v>
-      </c>
-      <c r="B37" s="169"/>
-      <c r="C37" s="169"/>
-      <c r="D37" s="169"/>
-      <c r="E37" s="169"/>
-      <c r="F37" s="169"/>
-      <c r="G37" s="169"/>
-      <c r="H37" s="169"/>
-      <c r="I37" s="169"/>
-      <c r="J37" s="169"/>
-      <c r="K37" s="169"/>
-      <c r="L37" s="169"/>
-      <c r="M37" s="169"/>
-      <c r="N37" s="169"/>
-      <c r="O37" s="169"/>
-      <c r="P37" s="169"/>
-      <c r="Q37" s="169"/>
-      <c r="R37" s="169"/>
-      <c r="S37" s="169"/>
+      <c r="A37" s="199" t="s">
+        <v>368</v>
+      </c>
+      <c r="B37" s="187"/>
+      <c r="C37" s="187"/>
+      <c r="D37" s="187"/>
+      <c r="E37" s="187"/>
+      <c r="F37" s="187"/>
+      <c r="G37" s="187"/>
+      <c r="H37" s="187"/>
+      <c r="I37" s="187"/>
+      <c r="J37" s="187"/>
+      <c r="K37" s="187"/>
+      <c r="L37" s="187"/>
+      <c r="M37" s="187"/>
+      <c r="N37" s="187"/>
+      <c r="O37" s="187"/>
+      <c r="P37" s="187"/>
+      <c r="Q37" s="187"/>
+      <c r="R37" s="187"/>
+      <c r="S37" s="187"/>
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="38" t="s">
-        <v>299</v>
-      </c>
-      <c r="B39" s="184" t="s">
-        <v>365</v>
-      </c>
-      <c r="C39" s="169"/>
-      <c r="D39" s="169"/>
-      <c r="E39" s="182" t="s">
-        <v>366</v>
-      </c>
-      <c r="F39" s="169"/>
-      <c r="G39" s="169"/>
-      <c r="H39" s="185" t="s">
-        <v>367</v>
-      </c>
-      <c r="I39" s="169"/>
-      <c r="J39" s="169"/>
-      <c r="K39" s="178" t="s">
-        <v>368</v>
-      </c>
-      <c r="L39" s="169"/>
-      <c r="M39" s="169"/>
-      <c r="N39" s="176" t="s">
+        <v>303</v>
+      </c>
+      <c r="B39" s="202" t="s">
+        <v>369</v>
+      </c>
+      <c r="C39" s="187"/>
+      <c r="D39" s="187"/>
+      <c r="E39" s="200" t="s">
+        <v>370</v>
+      </c>
+      <c r="F39" s="187"/>
+      <c r="G39" s="187"/>
+      <c r="H39" s="203" t="s">
+        <v>371</v>
+      </c>
+      <c r="I39" s="187"/>
+      <c r="J39" s="187"/>
+      <c r="K39" s="196" t="s">
+        <v>372</v>
+      </c>
+      <c r="L39" s="187"/>
+      <c r="M39" s="187"/>
+      <c r="N39" s="194" t="s">
         <v>45</v>
       </c>
-      <c r="O39" s="169"/>
-      <c r="P39" s="169"/>
-      <c r="Q39" s="183" t="s">
-        <v>369</v>
-      </c>
-      <c r="R39" s="169"/>
-      <c r="S39" s="169"/>
+      <c r="O39" s="187"/>
+      <c r="P39" s="187"/>
+      <c r="Q39" s="201" t="s">
+        <v>373</v>
+      </c>
+      <c r="R39" s="187"/>
+      <c r="S39" s="187"/>
     </row>
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A16:S16"/>
     <mergeCell ref="H20:M20"/>
-    <mergeCell ref="A16:S16"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -8686,14 +8903,13 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -8702,6 +8918,7 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -8709,7 +8926,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -8757,33 +8974,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="187" t="s">
-        <v>370</v>
-      </c>
-      <c r="B1" s="161"/>
-      <c r="C1" s="161"/>
-      <c r="D1" s="161"/>
-      <c r="E1" s="161"/>
-      <c r="F1" s="162"/>
+      <c r="A1" s="205" t="s">
+        <v>374</v>
+      </c>
+      <c r="B1" s="179"/>
+      <c r="C1" s="179"/>
+      <c r="D1" s="179"/>
+      <c r="E1" s="179"/>
+      <c r="F1" s="180"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -8992,11 +9209,11 @@
       </c>
       <c r="B12" s="26">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C12" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D12" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -9008,7 +9225,7 @@
       </c>
       <c r="F12" s="27">
         <f t="shared" si="1"/>
-        <v>0.21052631578947367</v>
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -9063,15 +9280,15 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="28" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="B16" s="29">
         <f>SUM(B4:B14)</f>
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C16" s="29">
         <f>SUM(C4:C14)</f>
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
@@ -9083,12 +9300,12 @@
       </c>
       <c r="F16" s="30">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.6484375</v>
+        <v>0.65384615384615385</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="43" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="B18" s="44">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -9097,7 +9314,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="45" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
     </row>
   </sheetData>
@@ -9118,7 +9335,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -9129,573 +9346,624 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="187" t="s">
-        <v>377</v>
-      </c>
-      <c r="B1" s="161"/>
-      <c r="C1" s="161"/>
-      <c r="D1" s="161"/>
-      <c r="E1" s="162"/>
+      <c r="A1" s="205" t="s">
+        <v>381</v>
+      </c>
+      <c r="B1" s="179"/>
+      <c r="C1" s="179"/>
+      <c r="D1" s="179"/>
+      <c r="E1" s="180"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="31" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D3" s="31" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="32" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="34" t="s">
+        <v>391</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>383</v>
-      </c>
       <c r="C5" s="21" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="32" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="34" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="32" t="s">
+        <v>399</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>395</v>
       </c>
-      <c r="B8" s="12" t="s">
-        <v>391</v>
-      </c>
       <c r="C8" s="19" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="34" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="32" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="34" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="32" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="34" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="32" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="34" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="32" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="34" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="32" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="34" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="32" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="34" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="32" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E22" s="33" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="34" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E23" s="35" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="32" t="s">
+        <v>441</v>
+      </c>
+      <c r="B24" s="12" t="s">
         <v>437</v>
       </c>
-      <c r="B24" s="12" t="s">
-        <v>433</v>
-      </c>
       <c r="C24" s="19" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="58" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="B25" s="55" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="C25" s="59" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D25" s="55" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E25" s="60" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="61" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="B26" s="49" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="C26" s="59" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="D26" s="49" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="E26" s="62" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="58" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="B27" s="55" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="C27" s="59" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="D27" s="55" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E27" s="60" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="79" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="B28" s="66" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="C28" s="75" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="D28" s="107" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="E28" s="107" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="80" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="B29" s="72" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C29" s="77" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D29" s="106" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="E29" s="106" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="88" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B30" s="84" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C30" s="89" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D30" s="84" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E30" s="90" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="105" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="B31" s="94" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="C31" s="103" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D31" s="94" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="E31" s="106" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="122" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="B32" s="117" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="C32" s="120" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D32" s="117" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="E32" s="123" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="124" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="B33" s="111" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C33" s="120" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D33" s="111" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="E33" s="125" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="156" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="B34" s="150" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="C34" s="142" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="D34" s="150" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E34" s="157" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="158" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B35" s="143" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="C35" s="154" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="D35" s="143" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E35" s="159" t="s">
-        <v>461</v>
+        <v>465</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A36" s="172" t="s">
+        <v>399</v>
+      </c>
+      <c r="B36" s="169" t="s">
+        <v>387</v>
+      </c>
+      <c r="C36" s="173" t="s">
+        <v>388</v>
+      </c>
+      <c r="D36" s="169" t="s">
+        <v>432</v>
+      </c>
+      <c r="E36" s="174" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A37" s="175" t="s">
+        <v>467</v>
+      </c>
+      <c r="B37" s="163" t="s">
+        <v>437</v>
+      </c>
+      <c r="C37" s="176" t="s">
+        <v>400</v>
+      </c>
+      <c r="D37" s="163" t="s">
+        <v>389</v>
+      </c>
+      <c r="E37" s="177" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A38" s="172" t="s">
+        <v>469</v>
+      </c>
+      <c r="B38" s="169" t="s">
+        <v>437</v>
+      </c>
+      <c r="C38" s="176" t="s">
+        <v>412</v>
+      </c>
+      <c r="D38" s="169" t="s">
+        <v>389</v>
+      </c>
+      <c r="E38" s="174" t="s">
+        <v>470</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(tracker): trace the basic TheRundown quota; close the API-Football item
TheRundown has contributed exactly TWO rows to this database in its entire life --
both BetMGM, both the same February NBA test fixture. The other ~28,000 odds rows
are all API-Football bookmakers; Bovada and Bodog never returned anything.

The 1,000/month basic allowance went on ingest_odds running EVERY 5 MINUTES
(288x/day) from 28 Jul to 2 Aug, calling TheRundown for leagues that were either
out of season (all five European) or not covered by it at all (Brasileirao, CSL,
Scottish Prem). At 2-3 calls per run that is 600-900/day: the month gone in a day
or two. Both fixes -- 6-hourly cadence and fixture gating -- were already in place
before the Pro plan was bought.

Also closes the API-Football renewal item, which the user had already confirmed
and which I kept carrying as an open P0.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CA6CFF3-1C8F-4D89-B2C3-F8FF4B4E13BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C99C4D5-B5CB-4676-BD58-0CC4B05BC887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="476">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="481">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -951,6 +951,12 @@
   </si>
   <si>
     <t>If it flips to True, TheRundown Pro is redundant and can be dropped</t>
+  </si>
+  <si>
+    <t>Trace where the 1,000/month basic quota went</t>
+  </si>
+  <si>
+    <t>A 5-min polling loop against out-of-season leagues. Yield: 2 rows, one NBA game</t>
   </si>
   <si>
     <t>Legend</t>
@@ -1536,6 +1542,15 @@
   </si>
   <si>
     <t>UNRESOLVED, and it decides whether the TheRundown Pro subscription is needed at all. Every league reporting coverage.odds=True (MLS, Brasileirao) is currently IN SEASON; every league reporting False (all 5 European) is OUT of season. That confound is total, so the data fits 'API-Football only serves odds for a live season' exactly as well as 'these leagues are not covered'. /odds returns results=0 for EPL 2025, EPL 2026 and a specific 21 Aug fixture, while MLS 2026 returns 10 as a control - but past-season odds may simply not be retained, so that does not discriminate either. MLS is the tell: False for 2024/2025 (completed), True for 2026 (in season). Recheck on 21 Aug when EPL actually starts. Asserted as settled twice already and wrong both times - do not report it resolved before that date.</t>
+  </si>
+  <si>
+    <t>The basic quota was burned by a bug, not demand</t>
+  </si>
+  <si>
+    <t>TheRundown has contributed exactly TWO rows to this database in its entire life - both BetMGM, both the same Feb NBA test fixture. Every other odds row (~28,000) is from API-Football bookmakers. The 1,000/month basic allowance was consumed by ingest_odds running EVERY 5 MINUTES (288x/day) from 28 Jul to 2 Aug, calling TheRundown for leagues that were either out of season (all five European) or not covered by it at all (Brasileirao, CSL, Scottish Prem). At 2-3 calls per run that is 600-900/day - the month's allowance gone in a day or two. Both fixes (6-hourly cadence, fixture gating) were already in place BEFORE the Pro upgrade was bought, so the system was consuming nothing by then.</t>
+  </si>
+  <si>
+    <t>User confirmed the API-Football subscription will be renewed. This was carried as an open P0 after that had already been stated - a second instance of a stale item surviving in the list. Not a risk.</t>
   </si>
 </sst>
 </file>
@@ -1545,7 +1560,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\ mmm"/>
   </numFmts>
-  <fonts count="58" x14ac:knownFonts="1">
+  <fonts count="62" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1870,8 +1885,30 @@
       <color rgb="FF6B7280"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF111827"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF111827"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF6B7280"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="54">
+  <fills count="59">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2138,8 +2175,33 @@
         <fgColor rgb="FFB45309"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF16A34A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB45309"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF94A3B8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -2360,11 +2422,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="217">
+  <cellXfs count="231">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2928,12 +3005,54 @@
     <xf numFmtId="0" fontId="54" fillId="51" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="58" fillId="54" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="54" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="55" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="54" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="59" fillId="54" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="54" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="55" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="54" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="56" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="54" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="57" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="57" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="58" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="57" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2999,7 +3118,7 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3319,7 +3438,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R137"/>
+  <dimension ref="A1:R138"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -3333,46 +3452,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="192" t="s">
+      <c r="A1" s="206" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="190"/>
-      <c r="C1" s="190"/>
-      <c r="D1" s="190"/>
-      <c r="E1" s="190"/>
-      <c r="F1" s="190"/>
-      <c r="G1" s="190"/>
-      <c r="H1" s="190"/>
-      <c r="I1" s="190"/>
-      <c r="J1" s="190"/>
-      <c r="K1" s="190"/>
-      <c r="L1" s="190"/>
-      <c r="M1" s="190"/>
-      <c r="N1" s="190"/>
-      <c r="O1" s="190"/>
-      <c r="P1" s="190"/>
-      <c r="Q1" s="191"/>
+      <c r="B1" s="204"/>
+      <c r="C1" s="204"/>
+      <c r="D1" s="204"/>
+      <c r="E1" s="204"/>
+      <c r="F1" s="204"/>
+      <c r="G1" s="204"/>
+      <c r="H1" s="204"/>
+      <c r="I1" s="204"/>
+      <c r="J1" s="204"/>
+      <c r="K1" s="204"/>
+      <c r="L1" s="204"/>
+      <c r="M1" s="204"/>
+      <c r="N1" s="204"/>
+      <c r="O1" s="204"/>
+      <c r="P1" s="204"/>
+      <c r="Q1" s="205"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="189" t="s">
+      <c r="A2" s="203" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="190"/>
-      <c r="C2" s="190"/>
-      <c r="D2" s="190"/>
-      <c r="E2" s="190"/>
-      <c r="F2" s="190"/>
-      <c r="G2" s="190"/>
-      <c r="H2" s="190"/>
-      <c r="I2" s="190"/>
-      <c r="J2" s="190"/>
-      <c r="K2" s="190"/>
-      <c r="L2" s="190"/>
-      <c r="M2" s="190"/>
-      <c r="N2" s="190"/>
-      <c r="O2" s="190"/>
-      <c r="P2" s="190"/>
-      <c r="Q2" s="191"/>
+      <c r="B2" s="204"/>
+      <c r="C2" s="204"/>
+      <c r="D2" s="204"/>
+      <c r="E2" s="204"/>
+      <c r="F2" s="204"/>
+      <c r="G2" s="204"/>
+      <c r="H2" s="204"/>
+      <c r="I2" s="204"/>
+      <c r="J2" s="204"/>
+      <c r="K2" s="204"/>
+      <c r="L2" s="204"/>
+      <c r="M2" s="204"/>
+      <c r="N2" s="204"/>
+      <c r="O2" s="204"/>
+      <c r="P2" s="204"/>
+      <c r="Q2" s="205"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
@@ -6926,7 +7045,7 @@
       <c r="P102" s="11"/>
       <c r="Q102" s="11"/>
       <c r="R102" t="str">
-        <f t="shared" ref="R102:R135" si="3">IF($A102&lt;&gt;"",$A102,R101)</f>
+        <f t="shared" ref="R102:R136" si="3">IF($A102&lt;&gt;"",$A102,R101)</f>
         <v>E9 Data Ops</v>
       </c>
     </row>
@@ -8151,23 +8270,60 @@
         <v>E9 Data Ops</v>
       </c>
     </row>
-    <row r="137" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A137" s="25" t="s">
+    <row r="136" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A136" s="189" t="s">
+        <v>130</v>
+      </c>
+      <c r="B136" s="190" t="s">
         <v>305</v>
       </c>
-      <c r="B137" s="5" t="s">
+      <c r="C136" s="191" t="s">
         <v>22</v>
       </c>
-      <c r="C137" s="17" t="s">
+      <c r="D136" s="192" t="s">
+        <v>33</v>
+      </c>
+      <c r="E136" s="193">
+        <v>46239</v>
+      </c>
+      <c r="F136" s="193">
+        <v>46239</v>
+      </c>
+      <c r="G136" s="194" t="s">
+        <v>306</v>
+      </c>
+      <c r="H136" s="190"/>
+      <c r="I136" s="195"/>
+      <c r="J136" s="190"/>
+      <c r="K136" s="190"/>
+      <c r="L136" s="190"/>
+      <c r="M136" s="190"/>
+      <c r="N136" s="190"/>
+      <c r="O136" s="190"/>
+      <c r="P136" s="190"/>
+      <c r="Q136" s="190"/>
+      <c r="R136" t="str">
+        <f t="shared" si="3"/>
+        <v>E9 Data Ops</v>
+      </c>
+    </row>
+    <row r="138" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A138" s="25" t="s">
+        <v>307</v>
+      </c>
+      <c r="B138" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C138" s="17" t="s">
         <v>231</v>
       </c>
-      <c r="D137" s="19" t="s">
+      <c r="D138" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="E137" s="23" t="s">
+      <c r="E138" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="F137" s="21" t="s">
+      <c r="F138" s="21" t="s">
         <v>136</v>
       </c>
     </row>
@@ -8191,852 +8347,852 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="208" t="s">
-        <v>306</v>
-      </c>
-      <c r="B1" s="198"/>
-      <c r="C1" s="198"/>
-      <c r="D1" s="198"/>
-      <c r="E1" s="198"/>
-      <c r="F1" s="198"/>
-      <c r="G1" s="198"/>
-      <c r="H1" s="198"/>
-      <c r="I1" s="198"/>
-      <c r="J1" s="198"/>
-      <c r="K1" s="198"/>
-      <c r="L1" s="198"/>
-      <c r="M1" s="198"/>
-      <c r="N1" s="198"/>
-      <c r="O1" s="198"/>
-      <c r="P1" s="198"/>
-      <c r="Q1" s="198"/>
-      <c r="R1" s="198"/>
-      <c r="S1" s="198"/>
+      <c r="A1" s="222" t="s">
+        <v>308</v>
+      </c>
+      <c r="B1" s="212"/>
+      <c r="C1" s="212"/>
+      <c r="D1" s="212"/>
+      <c r="E1" s="212"/>
+      <c r="F1" s="212"/>
+      <c r="G1" s="212"/>
+      <c r="H1" s="212"/>
+      <c r="I1" s="212"/>
+      <c r="J1" s="212"/>
+      <c r="K1" s="212"/>
+      <c r="L1" s="212"/>
+      <c r="M1" s="212"/>
+      <c r="N1" s="212"/>
+      <c r="O1" s="212"/>
+      <c r="P1" s="212"/>
+      <c r="Q1" s="212"/>
+      <c r="R1" s="212"/>
+      <c r="S1" s="212"/>
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="215" t="s">
-        <v>307</v>
-      </c>
-      <c r="B2" s="198"/>
-      <c r="C2" s="198"/>
-      <c r="D2" s="198"/>
-      <c r="E2" s="198"/>
-      <c r="F2" s="198"/>
-      <c r="G2" s="198"/>
-      <c r="H2" s="198"/>
-      <c r="I2" s="198"/>
-      <c r="J2" s="198"/>
-      <c r="K2" s="198"/>
-      <c r="L2" s="198"/>
-      <c r="M2" s="198"/>
-      <c r="N2" s="198"/>
-      <c r="O2" s="198"/>
-      <c r="P2" s="198"/>
-      <c r="Q2" s="198"/>
-      <c r="R2" s="198"/>
-      <c r="S2" s="198"/>
+      <c r="A2" s="229" t="s">
+        <v>309</v>
+      </c>
+      <c r="B2" s="212"/>
+      <c r="C2" s="212"/>
+      <c r="D2" s="212"/>
+      <c r="E2" s="212"/>
+      <c r="F2" s="212"/>
+      <c r="G2" s="212"/>
+      <c r="H2" s="212"/>
+      <c r="I2" s="212"/>
+      <c r="J2" s="212"/>
+      <c r="K2" s="212"/>
+      <c r="L2" s="212"/>
+      <c r="M2" s="212"/>
+      <c r="N2" s="212"/>
+      <c r="O2" s="212"/>
+      <c r="P2" s="212"/>
+      <c r="Q2" s="212"/>
+      <c r="R2" s="212"/>
+      <c r="S2" s="212"/>
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="203" t="s">
-        <v>308</v>
-      </c>
-      <c r="B4" s="198"/>
-      <c r="C4" s="198"/>
-      <c r="D4" s="198"/>
-      <c r="E4" s="198"/>
-      <c r="F4" s="198"/>
-      <c r="G4" s="198"/>
-      <c r="H4" s="198"/>
-      <c r="I4" s="198"/>
-      <c r="J4" s="198"/>
-      <c r="K4" s="198"/>
-      <c r="L4" s="198"/>
-      <c r="M4" s="198"/>
-      <c r="N4" s="198"/>
-      <c r="O4" s="198"/>
-      <c r="P4" s="198"/>
-      <c r="Q4" s="198"/>
-      <c r="R4" s="198"/>
-      <c r="S4" s="198"/>
+      <c r="A4" s="217" t="s">
+        <v>310</v>
+      </c>
+      <c r="B4" s="212"/>
+      <c r="C4" s="212"/>
+      <c r="D4" s="212"/>
+      <c r="E4" s="212"/>
+      <c r="F4" s="212"/>
+      <c r="G4" s="212"/>
+      <c r="H4" s="212"/>
+      <c r="I4" s="212"/>
+      <c r="J4" s="212"/>
+      <c r="K4" s="212"/>
+      <c r="L4" s="212"/>
+      <c r="M4" s="212"/>
+      <c r="N4" s="212"/>
+      <c r="O4" s="212"/>
+      <c r="P4" s="212"/>
+      <c r="Q4" s="212"/>
+      <c r="R4" s="212"/>
+      <c r="S4" s="212"/>
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="37" t="s">
-        <v>309</v>
-      </c>
-      <c r="B5" s="193" t="s">
-        <v>310</v>
-      </c>
-      <c r="C5" s="194"/>
-      <c r="D5" s="195"/>
-      <c r="E5" s="196" t="s">
         <v>311</v>
       </c>
-      <c r="F5" s="194"/>
-      <c r="G5" s="195"/>
-      <c r="H5" s="196" t="s">
+      <c r="B5" s="207" t="s">
         <v>312</v>
       </c>
-      <c r="I5" s="194"/>
-      <c r="J5" s="195"/>
-      <c r="K5" s="193" t="s">
+      <c r="C5" s="208"/>
+      <c r="D5" s="209"/>
+      <c r="E5" s="210" t="s">
         <v>313</v>
       </c>
-      <c r="L5" s="194"/>
-      <c r="M5" s="195"/>
-      <c r="N5" s="200" t="s">
+      <c r="F5" s="208"/>
+      <c r="G5" s="209"/>
+      <c r="H5" s="210" t="s">
         <v>314</v>
       </c>
-      <c r="O5" s="194"/>
-      <c r="P5" s="195"/>
-      <c r="Q5" s="200" t="s">
+      <c r="I5" s="208"/>
+      <c r="J5" s="209"/>
+      <c r="K5" s="207" t="s">
         <v>315</v>
       </c>
-      <c r="R5" s="194"/>
-      <c r="S5" s="195"/>
+      <c r="L5" s="208"/>
+      <c r="M5" s="209"/>
+      <c r="N5" s="214" t="s">
+        <v>316</v>
+      </c>
+      <c r="O5" s="208"/>
+      <c r="P5" s="209"/>
+      <c r="Q5" s="214" t="s">
+        <v>317</v>
+      </c>
+      <c r="R5" s="208"/>
+      <c r="S5" s="209"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="197" t="s">
-        <v>316</v>
-      </c>
-      <c r="C6" s="198"/>
-      <c r="D6" s="198"/>
-      <c r="E6" s="198"/>
-      <c r="F6" s="198"/>
-      <c r="G6" s="198"/>
-      <c r="H6" s="198"/>
-      <c r="I6" s="198"/>
-      <c r="J6" s="198"/>
-      <c r="K6" s="198"/>
-      <c r="L6" s="198"/>
-      <c r="M6" s="198"/>
-      <c r="N6" s="198"/>
-      <c r="O6" s="198"/>
-      <c r="P6" s="198"/>
-      <c r="Q6" s="198"/>
-      <c r="R6" s="198"/>
-      <c r="S6" s="198"/>
+      <c r="B6" s="211" t="s">
+        <v>318</v>
+      </c>
+      <c r="C6" s="212"/>
+      <c r="D6" s="212"/>
+      <c r="E6" s="212"/>
+      <c r="F6" s="212"/>
+      <c r="G6" s="212"/>
+      <c r="H6" s="212"/>
+      <c r="I6" s="212"/>
+      <c r="J6" s="212"/>
+      <c r="K6" s="212"/>
+      <c r="L6" s="212"/>
+      <c r="M6" s="212"/>
+      <c r="N6" s="212"/>
+      <c r="O6" s="212"/>
+      <c r="P6" s="212"/>
+      <c r="Q6" s="212"/>
+      <c r="R6" s="212"/>
+      <c r="S6" s="212"/>
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="203" t="s">
-        <v>317</v>
-      </c>
-      <c r="B7" s="198"/>
-      <c r="C7" s="198"/>
-      <c r="D7" s="198"/>
-      <c r="E7" s="198"/>
-      <c r="F7" s="198"/>
-      <c r="G7" s="198"/>
-      <c r="H7" s="198"/>
-      <c r="I7" s="198"/>
-      <c r="J7" s="198"/>
-      <c r="K7" s="198"/>
-      <c r="L7" s="198"/>
-      <c r="M7" s="198"/>
-      <c r="N7" s="198"/>
-      <c r="O7" s="198"/>
-      <c r="P7" s="198"/>
-      <c r="Q7" s="198"/>
-      <c r="R7" s="198"/>
-      <c r="S7" s="198"/>
+      <c r="A7" s="217" t="s">
+        <v>319</v>
+      </c>
+      <c r="B7" s="212"/>
+      <c r="C7" s="212"/>
+      <c r="D7" s="212"/>
+      <c r="E7" s="212"/>
+      <c r="F7" s="212"/>
+      <c r="G7" s="212"/>
+      <c r="H7" s="212"/>
+      <c r="I7" s="212"/>
+      <c r="J7" s="212"/>
+      <c r="K7" s="212"/>
+      <c r="L7" s="212"/>
+      <c r="M7" s="212"/>
+      <c r="N7" s="212"/>
+      <c r="O7" s="212"/>
+      <c r="P7" s="212"/>
+      <c r="Q7" s="212"/>
+      <c r="R7" s="212"/>
+      <c r="S7" s="212"/>
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="37" t="s">
+        <v>320</v>
+      </c>
+      <c r="B8" s="220" t="s">
+        <v>321</v>
+      </c>
+      <c r="C8" s="208"/>
+      <c r="D8" s="208"/>
+      <c r="E8" s="208"/>
+      <c r="F8" s="208"/>
+      <c r="G8" s="208"/>
+      <c r="H8" s="208"/>
+      <c r="I8" s="208"/>
+      <c r="J8" s="209"/>
+      <c r="K8" s="220" t="s">
+        <v>322</v>
+      </c>
+      <c r="L8" s="208"/>
+      <c r="M8" s="208"/>
+      <c r="N8" s="208"/>
+      <c r="O8" s="208"/>
+      <c r="P8" s="208"/>
+      <c r="Q8" s="208"/>
+      <c r="R8" s="208"/>
+      <c r="S8" s="209"/>
+    </row>
+    <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B9" s="211" t="s">
         <v>318</v>
       </c>
-      <c r="B8" s="206" t="s">
-        <v>319</v>
-      </c>
-      <c r="C8" s="194"/>
-      <c r="D8" s="194"/>
-      <c r="E8" s="194"/>
-      <c r="F8" s="194"/>
-      <c r="G8" s="194"/>
-      <c r="H8" s="194"/>
-      <c r="I8" s="194"/>
-      <c r="J8" s="195"/>
-      <c r="K8" s="206" t="s">
-        <v>320</v>
-      </c>
-      <c r="L8" s="194"/>
-      <c r="M8" s="194"/>
-      <c r="N8" s="194"/>
-      <c r="O8" s="194"/>
-      <c r="P8" s="194"/>
-      <c r="Q8" s="194"/>
-      <c r="R8" s="194"/>
-      <c r="S8" s="195"/>
-    </row>
-    <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B9" s="197" t="s">
-        <v>316</v>
-      </c>
-      <c r="C9" s="198"/>
-      <c r="D9" s="198"/>
-      <c r="E9" s="198"/>
-      <c r="F9" s="198"/>
-      <c r="G9" s="198"/>
-      <c r="H9" s="198"/>
-      <c r="I9" s="198"/>
-      <c r="J9" s="198"/>
-      <c r="K9" s="198"/>
-      <c r="L9" s="198"/>
-      <c r="M9" s="198"/>
-      <c r="N9" s="198"/>
-      <c r="O9" s="198"/>
-      <c r="P9" s="198"/>
-      <c r="Q9" s="198"/>
-      <c r="R9" s="198"/>
-      <c r="S9" s="198"/>
+      <c r="C9" s="212"/>
+      <c r="D9" s="212"/>
+      <c r="E9" s="212"/>
+      <c r="F9" s="212"/>
+      <c r="G9" s="212"/>
+      <c r="H9" s="212"/>
+      <c r="I9" s="212"/>
+      <c r="J9" s="212"/>
+      <c r="K9" s="212"/>
+      <c r="L9" s="212"/>
+      <c r="M9" s="212"/>
+      <c r="N9" s="212"/>
+      <c r="O9" s="212"/>
+      <c r="P9" s="212"/>
+      <c r="Q9" s="212"/>
+      <c r="R9" s="212"/>
+      <c r="S9" s="212"/>
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="203" t="s">
-        <v>321</v>
-      </c>
-      <c r="B10" s="198"/>
-      <c r="C10" s="198"/>
-      <c r="D10" s="198"/>
-      <c r="E10" s="198"/>
-      <c r="F10" s="198"/>
-      <c r="G10" s="198"/>
-      <c r="H10" s="198"/>
-      <c r="I10" s="198"/>
-      <c r="J10" s="198"/>
-      <c r="K10" s="198"/>
-      <c r="L10" s="198"/>
-      <c r="M10" s="198"/>
-      <c r="N10" s="198"/>
-      <c r="O10" s="198"/>
-      <c r="P10" s="198"/>
-      <c r="Q10" s="198"/>
-      <c r="R10" s="198"/>
-      <c r="S10" s="198"/>
+      <c r="A10" s="217" t="s">
+        <v>323</v>
+      </c>
+      <c r="B10" s="212"/>
+      <c r="C10" s="212"/>
+      <c r="D10" s="212"/>
+      <c r="E10" s="212"/>
+      <c r="F10" s="212"/>
+      <c r="G10" s="212"/>
+      <c r="H10" s="212"/>
+      <c r="I10" s="212"/>
+      <c r="J10" s="212"/>
+      <c r="K10" s="212"/>
+      <c r="L10" s="212"/>
+      <c r="M10" s="212"/>
+      <c r="N10" s="212"/>
+      <c r="O10" s="212"/>
+      <c r="P10" s="212"/>
+      <c r="Q10" s="212"/>
+      <c r="R10" s="212"/>
+      <c r="S10" s="212"/>
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="37" t="s">
-        <v>322</v>
-      </c>
-      <c r="B11" s="193" t="s">
-        <v>323</v>
-      </c>
-      <c r="C11" s="194"/>
-      <c r="D11" s="195"/>
-      <c r="E11" s="193" t="s">
         <v>324</v>
       </c>
-      <c r="F11" s="194"/>
-      <c r="G11" s="195"/>
-      <c r="H11" s="193" t="s">
+      <c r="B11" s="207" t="s">
         <v>325</v>
       </c>
-      <c r="I11" s="194"/>
-      <c r="J11" s="195"/>
-      <c r="K11" s="196" t="s">
+      <c r="C11" s="208"/>
+      <c r="D11" s="209"/>
+      <c r="E11" s="207" t="s">
         <v>326</v>
       </c>
-      <c r="L11" s="194"/>
-      <c r="M11" s="195"/>
-      <c r="N11" s="193" t="s">
+      <c r="F11" s="208"/>
+      <c r="G11" s="209"/>
+      <c r="H11" s="207" t="s">
         <v>327</v>
       </c>
-      <c r="O11" s="194"/>
-      <c r="P11" s="195"/>
-      <c r="Q11" s="193" t="s">
+      <c r="I11" s="208"/>
+      <c r="J11" s="209"/>
+      <c r="K11" s="210" t="s">
         <v>328</v>
       </c>
-      <c r="R11" s="194"/>
-      <c r="S11" s="195"/>
+      <c r="L11" s="208"/>
+      <c r="M11" s="209"/>
+      <c r="N11" s="207" t="s">
+        <v>329</v>
+      </c>
+      <c r="O11" s="208"/>
+      <c r="P11" s="209"/>
+      <c r="Q11" s="207" t="s">
+        <v>330</v>
+      </c>
+      <c r="R11" s="208"/>
+      <c r="S11" s="209"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B12" s="197" t="s">
-        <v>316</v>
-      </c>
-      <c r="C12" s="198"/>
-      <c r="D12" s="198"/>
-      <c r="E12" s="198"/>
-      <c r="F12" s="198"/>
-      <c r="G12" s="198"/>
-      <c r="H12" s="198"/>
-      <c r="I12" s="198"/>
-      <c r="J12" s="198"/>
-      <c r="K12" s="198"/>
-      <c r="L12" s="198"/>
-      <c r="M12" s="198"/>
-      <c r="N12" s="198"/>
-      <c r="O12" s="198"/>
-      <c r="P12" s="198"/>
-      <c r="Q12" s="198"/>
-      <c r="R12" s="198"/>
-      <c r="S12" s="198"/>
+      <c r="B12" s="211" t="s">
+        <v>318</v>
+      </c>
+      <c r="C12" s="212"/>
+      <c r="D12" s="212"/>
+      <c r="E12" s="212"/>
+      <c r="F12" s="212"/>
+      <c r="G12" s="212"/>
+      <c r="H12" s="212"/>
+      <c r="I12" s="212"/>
+      <c r="J12" s="212"/>
+      <c r="K12" s="212"/>
+      <c r="L12" s="212"/>
+      <c r="M12" s="212"/>
+      <c r="N12" s="212"/>
+      <c r="O12" s="212"/>
+      <c r="P12" s="212"/>
+      <c r="Q12" s="212"/>
+      <c r="R12" s="212"/>
+      <c r="S12" s="212"/>
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="203" t="s">
-        <v>329</v>
-      </c>
-      <c r="B13" s="198"/>
-      <c r="C13" s="198"/>
-      <c r="D13" s="198"/>
-      <c r="E13" s="198"/>
-      <c r="F13" s="198"/>
-      <c r="G13" s="198"/>
-      <c r="H13" s="198"/>
-      <c r="I13" s="198"/>
-      <c r="J13" s="198"/>
-      <c r="K13" s="198"/>
-      <c r="L13" s="198"/>
-      <c r="M13" s="198"/>
-      <c r="N13" s="198"/>
-      <c r="O13" s="198"/>
-      <c r="P13" s="198"/>
-      <c r="Q13" s="198"/>
-      <c r="R13" s="198"/>
-      <c r="S13" s="198"/>
+      <c r="A13" s="217" t="s">
+        <v>331</v>
+      </c>
+      <c r="B13" s="212"/>
+      <c r="C13" s="212"/>
+      <c r="D13" s="212"/>
+      <c r="E13" s="212"/>
+      <c r="F13" s="212"/>
+      <c r="G13" s="212"/>
+      <c r="H13" s="212"/>
+      <c r="I13" s="212"/>
+      <c r="J13" s="212"/>
+      <c r="K13" s="212"/>
+      <c r="L13" s="212"/>
+      <c r="M13" s="212"/>
+      <c r="N13" s="212"/>
+      <c r="O13" s="212"/>
+      <c r="P13" s="212"/>
+      <c r="Q13" s="212"/>
+      <c r="R13" s="212"/>
+      <c r="S13" s="212"/>
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="37" t="s">
-        <v>330</v>
-      </c>
-      <c r="B14" s="201" t="s">
-        <v>331</v>
-      </c>
-      <c r="C14" s="194"/>
-      <c r="D14" s="194"/>
-      <c r="E14" s="194"/>
-      <c r="F14" s="194"/>
-      <c r="G14" s="195"/>
-      <c r="H14" s="201" t="s">
         <v>332</v>
       </c>
-      <c r="I14" s="194"/>
-      <c r="J14" s="194"/>
-      <c r="K14" s="194"/>
-      <c r="L14" s="194"/>
-      <c r="M14" s="195"/>
-      <c r="N14" s="201" t="s">
+      <c r="B14" s="215" t="s">
         <v>333</v>
       </c>
-      <c r="O14" s="194"/>
-      <c r="P14" s="195"/>
-      <c r="Q14" s="196" t="s">
+      <c r="C14" s="208"/>
+      <c r="D14" s="208"/>
+      <c r="E14" s="208"/>
+      <c r="F14" s="208"/>
+      <c r="G14" s="209"/>
+      <c r="H14" s="215" t="s">
         <v>334</v>
       </c>
-      <c r="R14" s="194"/>
-      <c r="S14" s="195"/>
+      <c r="I14" s="208"/>
+      <c r="J14" s="208"/>
+      <c r="K14" s="208"/>
+      <c r="L14" s="208"/>
+      <c r="M14" s="209"/>
+      <c r="N14" s="215" t="s">
+        <v>335</v>
+      </c>
+      <c r="O14" s="208"/>
+      <c r="P14" s="209"/>
+      <c r="Q14" s="210" t="s">
+        <v>336</v>
+      </c>
+      <c r="R14" s="208"/>
+      <c r="S14" s="209"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B15" s="197" t="s">
-        <v>335</v>
-      </c>
-      <c r="C15" s="198"/>
-      <c r="D15" s="198"/>
-      <c r="E15" s="198"/>
-      <c r="F15" s="198"/>
-      <c r="G15" s="198"/>
-      <c r="H15" s="198"/>
-      <c r="I15" s="198"/>
-      <c r="J15" s="198"/>
-      <c r="K15" s="198"/>
-      <c r="L15" s="198"/>
-      <c r="M15" s="198"/>
-      <c r="N15" s="198"/>
-      <c r="O15" s="198"/>
-      <c r="P15" s="198"/>
-      <c r="Q15" s="198"/>
-      <c r="R15" s="198"/>
-      <c r="S15" s="198"/>
+      <c r="B15" s="211" t="s">
+        <v>337</v>
+      </c>
+      <c r="C15" s="212"/>
+      <c r="D15" s="212"/>
+      <c r="E15" s="212"/>
+      <c r="F15" s="212"/>
+      <c r="G15" s="212"/>
+      <c r="H15" s="212"/>
+      <c r="I15" s="212"/>
+      <c r="J15" s="212"/>
+      <c r="K15" s="212"/>
+      <c r="L15" s="212"/>
+      <c r="M15" s="212"/>
+      <c r="N15" s="212"/>
+      <c r="O15" s="212"/>
+      <c r="P15" s="212"/>
+      <c r="Q15" s="212"/>
+      <c r="R15" s="212"/>
+      <c r="S15" s="212"/>
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="203" t="s">
-        <v>336</v>
-      </c>
-      <c r="B16" s="198"/>
-      <c r="C16" s="198"/>
-      <c r="D16" s="198"/>
-      <c r="E16" s="198"/>
-      <c r="F16" s="198"/>
-      <c r="G16" s="198"/>
-      <c r="H16" s="198"/>
-      <c r="I16" s="198"/>
-      <c r="J16" s="198"/>
-      <c r="K16" s="198"/>
-      <c r="L16" s="198"/>
-      <c r="M16" s="198"/>
-      <c r="N16" s="198"/>
-      <c r="O16" s="198"/>
-      <c r="P16" s="198"/>
-      <c r="Q16" s="198"/>
-      <c r="R16" s="198"/>
-      <c r="S16" s="198"/>
+      <c r="A16" s="217" t="s">
+        <v>338</v>
+      </c>
+      <c r="B16" s="212"/>
+      <c r="C16" s="212"/>
+      <c r="D16" s="212"/>
+      <c r="E16" s="212"/>
+      <c r="F16" s="212"/>
+      <c r="G16" s="212"/>
+      <c r="H16" s="212"/>
+      <c r="I16" s="212"/>
+      <c r="J16" s="212"/>
+      <c r="K16" s="212"/>
+      <c r="L16" s="212"/>
+      <c r="M16" s="212"/>
+      <c r="N16" s="212"/>
+      <c r="O16" s="212"/>
+      <c r="P16" s="212"/>
+      <c r="Q16" s="212"/>
+      <c r="R16" s="212"/>
+      <c r="S16" s="212"/>
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="37" t="s">
-        <v>337</v>
-      </c>
-      <c r="B17" s="202" t="s">
-        <v>338</v>
-      </c>
-      <c r="C17" s="194"/>
-      <c r="D17" s="194"/>
-      <c r="E17" s="194"/>
-      <c r="F17" s="194"/>
-      <c r="G17" s="195"/>
-      <c r="H17" s="202" t="s">
         <v>339</v>
       </c>
-      <c r="I17" s="194"/>
-      <c r="J17" s="195"/>
-      <c r="K17" s="202" t="s">
+      <c r="B17" s="216" t="s">
         <v>340</v>
       </c>
-      <c r="L17" s="194"/>
-      <c r="M17" s="195"/>
-      <c r="N17" s="202" t="s">
+      <c r="C17" s="208"/>
+      <c r="D17" s="208"/>
+      <c r="E17" s="208"/>
+      <c r="F17" s="208"/>
+      <c r="G17" s="209"/>
+      <c r="H17" s="216" t="s">
         <v>341</v>
       </c>
-      <c r="O17" s="194"/>
-      <c r="P17" s="195"/>
-      <c r="Q17" s="202" t="s">
+      <c r="I17" s="208"/>
+      <c r="J17" s="209"/>
+      <c r="K17" s="216" t="s">
         <v>342</v>
       </c>
-      <c r="R17" s="194"/>
-      <c r="S17" s="195"/>
+      <c r="L17" s="208"/>
+      <c r="M17" s="209"/>
+      <c r="N17" s="216" t="s">
+        <v>343</v>
+      </c>
+      <c r="O17" s="208"/>
+      <c r="P17" s="209"/>
+      <c r="Q17" s="216" t="s">
+        <v>344</v>
+      </c>
+      <c r="R17" s="208"/>
+      <c r="S17" s="209"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="197" t="s">
-        <v>316</v>
-      </c>
-      <c r="C18" s="198"/>
-      <c r="D18" s="198"/>
-      <c r="E18" s="198"/>
-      <c r="F18" s="198"/>
-      <c r="G18" s="198"/>
-      <c r="H18" s="198"/>
-      <c r="I18" s="198"/>
-      <c r="J18" s="198"/>
-      <c r="K18" s="198"/>
-      <c r="L18" s="198"/>
-      <c r="M18" s="198"/>
-      <c r="N18" s="198"/>
-      <c r="O18" s="198"/>
-      <c r="P18" s="198"/>
-      <c r="Q18" s="198"/>
-      <c r="R18" s="198"/>
-      <c r="S18" s="198"/>
+      <c r="B18" s="211" t="s">
+        <v>318</v>
+      </c>
+      <c r="C18" s="212"/>
+      <c r="D18" s="212"/>
+      <c r="E18" s="212"/>
+      <c r="F18" s="212"/>
+      <c r="G18" s="212"/>
+      <c r="H18" s="212"/>
+      <c r="I18" s="212"/>
+      <c r="J18" s="212"/>
+      <c r="K18" s="212"/>
+      <c r="L18" s="212"/>
+      <c r="M18" s="212"/>
+      <c r="N18" s="212"/>
+      <c r="O18" s="212"/>
+      <c r="P18" s="212"/>
+      <c r="Q18" s="212"/>
+      <c r="R18" s="212"/>
+      <c r="S18" s="212"/>
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="203" t="s">
-        <v>343</v>
-      </c>
-      <c r="B19" s="198"/>
-      <c r="C19" s="198"/>
-      <c r="D19" s="198"/>
-      <c r="E19" s="198"/>
-      <c r="F19" s="198"/>
-      <c r="G19" s="198"/>
-      <c r="H19" s="198"/>
-      <c r="I19" s="198"/>
-      <c r="J19" s="198"/>
-      <c r="K19" s="198"/>
-      <c r="L19" s="198"/>
-      <c r="M19" s="198"/>
-      <c r="N19" s="198"/>
-      <c r="O19" s="198"/>
-      <c r="P19" s="198"/>
-      <c r="Q19" s="198"/>
-      <c r="R19" s="198"/>
-      <c r="S19" s="198"/>
+      <c r="A19" s="217" t="s">
+        <v>345</v>
+      </c>
+      <c r="B19" s="212"/>
+      <c r="C19" s="212"/>
+      <c r="D19" s="212"/>
+      <c r="E19" s="212"/>
+      <c r="F19" s="212"/>
+      <c r="G19" s="212"/>
+      <c r="H19" s="212"/>
+      <c r="I19" s="212"/>
+      <c r="J19" s="212"/>
+      <c r="K19" s="212"/>
+      <c r="L19" s="212"/>
+      <c r="M19" s="212"/>
+      <c r="N19" s="212"/>
+      <c r="O19" s="212"/>
+      <c r="P19" s="212"/>
+      <c r="Q19" s="212"/>
+      <c r="R19" s="212"/>
+      <c r="S19" s="212"/>
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="37" t="s">
-        <v>344</v>
-      </c>
-      <c r="B20" s="204" t="s">
-        <v>345</v>
-      </c>
-      <c r="C20" s="194"/>
-      <c r="D20" s="194"/>
-      <c r="E20" s="194"/>
-      <c r="F20" s="194"/>
-      <c r="G20" s="195"/>
-      <c r="H20" s="204" t="s">
         <v>346</v>
       </c>
-      <c r="I20" s="194"/>
-      <c r="J20" s="194"/>
-      <c r="K20" s="194"/>
-      <c r="L20" s="194"/>
-      <c r="M20" s="195"/>
-      <c r="N20" s="204" t="s">
+      <c r="B20" s="218" t="s">
         <v>347</v>
       </c>
-      <c r="O20" s="194"/>
-      <c r="P20" s="194"/>
-      <c r="Q20" s="194"/>
-      <c r="R20" s="194"/>
-      <c r="S20" s="195"/>
+      <c r="C20" s="208"/>
+      <c r="D20" s="208"/>
+      <c r="E20" s="208"/>
+      <c r="F20" s="208"/>
+      <c r="G20" s="209"/>
+      <c r="H20" s="218" t="s">
+        <v>348</v>
+      </c>
+      <c r="I20" s="208"/>
+      <c r="J20" s="208"/>
+      <c r="K20" s="208"/>
+      <c r="L20" s="208"/>
+      <c r="M20" s="209"/>
+      <c r="N20" s="218" t="s">
+        <v>349</v>
+      </c>
+      <c r="O20" s="208"/>
+      <c r="P20" s="208"/>
+      <c r="Q20" s="208"/>
+      <c r="R20" s="208"/>
+      <c r="S20" s="209"/>
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B21" s="197" t="s">
-        <v>316</v>
-      </c>
-      <c r="C21" s="198"/>
-      <c r="D21" s="198"/>
-      <c r="E21" s="198"/>
-      <c r="F21" s="198"/>
-      <c r="G21" s="198"/>
-      <c r="H21" s="198"/>
-      <c r="I21" s="198"/>
-      <c r="J21" s="198"/>
-      <c r="K21" s="198"/>
-      <c r="L21" s="198"/>
-      <c r="M21" s="198"/>
-      <c r="N21" s="198"/>
-      <c r="O21" s="198"/>
-      <c r="P21" s="198"/>
-      <c r="Q21" s="198"/>
-      <c r="R21" s="198"/>
-      <c r="S21" s="198"/>
+      <c r="B21" s="211" t="s">
+        <v>318</v>
+      </c>
+      <c r="C21" s="212"/>
+      <c r="D21" s="212"/>
+      <c r="E21" s="212"/>
+      <c r="F21" s="212"/>
+      <c r="G21" s="212"/>
+      <c r="H21" s="212"/>
+      <c r="I21" s="212"/>
+      <c r="J21" s="212"/>
+      <c r="K21" s="212"/>
+      <c r="L21" s="212"/>
+      <c r="M21" s="212"/>
+      <c r="N21" s="212"/>
+      <c r="O21" s="212"/>
+      <c r="P21" s="212"/>
+      <c r="Q21" s="212"/>
+      <c r="R21" s="212"/>
+      <c r="S21" s="212"/>
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="203" t="s">
-        <v>348</v>
-      </c>
-      <c r="B22" s="198"/>
-      <c r="C22" s="198"/>
-      <c r="D22" s="198"/>
-      <c r="E22" s="198"/>
-      <c r="F22" s="198"/>
-      <c r="G22" s="198"/>
-      <c r="H22" s="198"/>
-      <c r="I22" s="198"/>
-      <c r="J22" s="198"/>
-      <c r="K22" s="198"/>
-      <c r="L22" s="198"/>
-      <c r="M22" s="198"/>
-      <c r="N22" s="198"/>
-      <c r="O22" s="198"/>
-      <c r="P22" s="198"/>
-      <c r="Q22" s="198"/>
-      <c r="R22" s="198"/>
-      <c r="S22" s="198"/>
+      <c r="A22" s="217" t="s">
+        <v>350</v>
+      </c>
+      <c r="B22" s="212"/>
+      <c r="C22" s="212"/>
+      <c r="D22" s="212"/>
+      <c r="E22" s="212"/>
+      <c r="F22" s="212"/>
+      <c r="G22" s="212"/>
+      <c r="H22" s="212"/>
+      <c r="I22" s="212"/>
+      <c r="J22" s="212"/>
+      <c r="K22" s="212"/>
+      <c r="L22" s="212"/>
+      <c r="M22" s="212"/>
+      <c r="N22" s="212"/>
+      <c r="O22" s="212"/>
+      <c r="P22" s="212"/>
+      <c r="Q22" s="212"/>
+      <c r="R22" s="212"/>
+      <c r="S22" s="212"/>
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="37" t="s">
-        <v>349</v>
-      </c>
-      <c r="B23" s="204" t="s">
-        <v>350</v>
-      </c>
-      <c r="C23" s="194"/>
-      <c r="D23" s="194"/>
-      <c r="E23" s="194"/>
-      <c r="F23" s="194"/>
-      <c r="G23" s="195"/>
-      <c r="H23" s="204" t="s">
         <v>351</v>
       </c>
-      <c r="I23" s="194"/>
-      <c r="J23" s="195"/>
-      <c r="K23" s="204" t="s">
+      <c r="B23" s="218" t="s">
         <v>352</v>
       </c>
-      <c r="L23" s="194"/>
-      <c r="M23" s="195"/>
-      <c r="N23" s="204" t="s">
+      <c r="C23" s="208"/>
+      <c r="D23" s="208"/>
+      <c r="E23" s="208"/>
+      <c r="F23" s="208"/>
+      <c r="G23" s="209"/>
+      <c r="H23" s="218" t="s">
         <v>353</v>
       </c>
-      <c r="O23" s="194"/>
-      <c r="P23" s="195"/>
-      <c r="Q23" s="200" t="s">
+      <c r="I23" s="208"/>
+      <c r="J23" s="209"/>
+      <c r="K23" s="218" t="s">
         <v>354</v>
       </c>
-      <c r="R23" s="194"/>
-      <c r="S23" s="195"/>
+      <c r="L23" s="208"/>
+      <c r="M23" s="209"/>
+      <c r="N23" s="218" t="s">
+        <v>355</v>
+      </c>
+      <c r="O23" s="208"/>
+      <c r="P23" s="209"/>
+      <c r="Q23" s="214" t="s">
+        <v>356</v>
+      </c>
+      <c r="R23" s="208"/>
+      <c r="S23" s="209"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="209" t="s">
-        <v>355</v>
-      </c>
-      <c r="B26" s="198"/>
-      <c r="C26" s="198"/>
-      <c r="D26" s="198"/>
-      <c r="E26" s="198"/>
-      <c r="F26" s="198"/>
-      <c r="G26" s="198"/>
-      <c r="H26" s="198"/>
-      <c r="I26" s="198"/>
-      <c r="J26" s="198"/>
-      <c r="K26" s="198"/>
-      <c r="L26" s="198"/>
-      <c r="M26" s="198"/>
-      <c r="N26" s="198"/>
-      <c r="O26" s="198"/>
-      <c r="P26" s="198"/>
-      <c r="Q26" s="198"/>
-      <c r="R26" s="198"/>
-      <c r="S26" s="198"/>
+      <c r="A26" s="223" t="s">
+        <v>357</v>
+      </c>
+      <c r="B26" s="212"/>
+      <c r="C26" s="212"/>
+      <c r="D26" s="212"/>
+      <c r="E26" s="212"/>
+      <c r="F26" s="212"/>
+      <c r="G26" s="212"/>
+      <c r="H26" s="212"/>
+      <c r="I26" s="212"/>
+      <c r="J26" s="212"/>
+      <c r="K26" s="212"/>
+      <c r="L26" s="212"/>
+      <c r="M26" s="212"/>
+      <c r="N26" s="212"/>
+      <c r="O26" s="212"/>
+      <c r="P26" s="212"/>
+      <c r="Q26" s="212"/>
+      <c r="R26" s="212"/>
+      <c r="S26" s="212"/>
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="37" t="s">
-        <v>356</v>
-      </c>
-      <c r="B27" s="193" t="s">
-        <v>357</v>
-      </c>
-      <c r="C27" s="194"/>
-      <c r="D27" s="195"/>
-      <c r="E27" s="193" t="s">
         <v>358</v>
       </c>
-      <c r="F27" s="194"/>
-      <c r="G27" s="195"/>
-      <c r="H27" s="201" t="s">
+      <c r="B27" s="207" t="s">
         <v>359</v>
       </c>
-      <c r="I27" s="194"/>
-      <c r="J27" s="195"/>
-      <c r="K27" s="202" t="s">
+      <c r="C27" s="208"/>
+      <c r="D27" s="209"/>
+      <c r="E27" s="207" t="s">
         <v>360</v>
       </c>
-      <c r="L27" s="194"/>
-      <c r="M27" s="195"/>
-      <c r="N27" s="202" t="s">
+      <c r="F27" s="208"/>
+      <c r="G27" s="209"/>
+      <c r="H27" s="215" t="s">
         <v>361</v>
       </c>
-      <c r="O27" s="194"/>
-      <c r="P27" s="195"/>
-      <c r="Q27" s="201" t="s">
+      <c r="I27" s="208"/>
+      <c r="J27" s="209"/>
+      <c r="K27" s="216" t="s">
         <v>362</v>
       </c>
-      <c r="R27" s="194"/>
-      <c r="S27" s="195"/>
+      <c r="L27" s="208"/>
+      <c r="M27" s="209"/>
+      <c r="N27" s="216" t="s">
+        <v>363</v>
+      </c>
+      <c r="O27" s="208"/>
+      <c r="P27" s="209"/>
+      <c r="Q27" s="215" t="s">
+        <v>364</v>
+      </c>
+      <c r="R27" s="208"/>
+      <c r="S27" s="209"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="203" t="s">
-        <v>363</v>
-      </c>
-      <c r="B30" s="198"/>
-      <c r="C30" s="198"/>
-      <c r="D30" s="198"/>
-      <c r="E30" s="198"/>
-      <c r="F30" s="198"/>
-      <c r="G30" s="198"/>
-      <c r="H30" s="198"/>
-      <c r="I30" s="198"/>
-      <c r="J30" s="198"/>
-      <c r="K30" s="198"/>
-      <c r="L30" s="198"/>
-      <c r="M30" s="198"/>
-      <c r="N30" s="198"/>
-      <c r="O30" s="198"/>
-      <c r="P30" s="198"/>
-      <c r="Q30" s="198"/>
-      <c r="R30" s="198"/>
-      <c r="S30" s="198"/>
+      <c r="A30" s="217" t="s">
+        <v>365</v>
+      </c>
+      <c r="B30" s="212"/>
+      <c r="C30" s="212"/>
+      <c r="D30" s="212"/>
+      <c r="E30" s="212"/>
+      <c r="F30" s="212"/>
+      <c r="G30" s="212"/>
+      <c r="H30" s="212"/>
+      <c r="I30" s="212"/>
+      <c r="J30" s="212"/>
+      <c r="K30" s="212"/>
+      <c r="L30" s="212"/>
+      <c r="M30" s="212"/>
+      <c r="N30" s="212"/>
+      <c r="O30" s="212"/>
+      <c r="P30" s="212"/>
+      <c r="Q30" s="212"/>
+      <c r="R30" s="212"/>
+      <c r="S30" s="212"/>
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="199" t="s">
-        <v>364</v>
-      </c>
-      <c r="B31" s="198"/>
-      <c r="C31" s="198"/>
-      <c r="D31" s="198"/>
-      <c r="E31" s="198"/>
-      <c r="F31" s="198"/>
-      <c r="G31" s="198"/>
-      <c r="H31" s="198"/>
-      <c r="I31" s="198"/>
-      <c r="J31" s="198"/>
-      <c r="K31" s="198"/>
-      <c r="L31" s="198"/>
-      <c r="M31" s="198"/>
-      <c r="N31" s="198"/>
-      <c r="O31" s="198"/>
-      <c r="P31" s="198"/>
-      <c r="Q31" s="198"/>
-      <c r="R31" s="198"/>
-      <c r="S31" s="198"/>
+      <c r="A31" s="213" t="s">
+        <v>366</v>
+      </c>
+      <c r="B31" s="212"/>
+      <c r="C31" s="212"/>
+      <c r="D31" s="212"/>
+      <c r="E31" s="212"/>
+      <c r="F31" s="212"/>
+      <c r="G31" s="212"/>
+      <c r="H31" s="212"/>
+      <c r="I31" s="212"/>
+      <c r="J31" s="212"/>
+      <c r="K31" s="212"/>
+      <c r="L31" s="212"/>
+      <c r="M31" s="212"/>
+      <c r="N31" s="212"/>
+      <c r="O31" s="212"/>
+      <c r="P31" s="212"/>
+      <c r="Q31" s="212"/>
+      <c r="R31" s="212"/>
+      <c r="S31" s="212"/>
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="199" t="s">
-        <v>365</v>
-      </c>
-      <c r="B32" s="198"/>
-      <c r="C32" s="198"/>
-      <c r="D32" s="198"/>
-      <c r="E32" s="198"/>
-      <c r="F32" s="198"/>
-      <c r="G32" s="198"/>
-      <c r="H32" s="198"/>
-      <c r="I32" s="198"/>
-      <c r="J32" s="198"/>
-      <c r="K32" s="198"/>
-      <c r="L32" s="198"/>
-      <c r="M32" s="198"/>
-      <c r="N32" s="198"/>
-      <c r="O32" s="198"/>
-      <c r="P32" s="198"/>
-      <c r="Q32" s="198"/>
-      <c r="R32" s="198"/>
-      <c r="S32" s="198"/>
+      <c r="A32" s="213" t="s">
+        <v>367</v>
+      </c>
+      <c r="B32" s="212"/>
+      <c r="C32" s="212"/>
+      <c r="D32" s="212"/>
+      <c r="E32" s="212"/>
+      <c r="F32" s="212"/>
+      <c r="G32" s="212"/>
+      <c r="H32" s="212"/>
+      <c r="I32" s="212"/>
+      <c r="J32" s="212"/>
+      <c r="K32" s="212"/>
+      <c r="L32" s="212"/>
+      <c r="M32" s="212"/>
+      <c r="N32" s="212"/>
+      <c r="O32" s="212"/>
+      <c r="P32" s="212"/>
+      <c r="Q32" s="212"/>
+      <c r="R32" s="212"/>
+      <c r="S32" s="212"/>
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="199" t="s">
-        <v>366</v>
-      </c>
-      <c r="B33" s="198"/>
-      <c r="C33" s="198"/>
-      <c r="D33" s="198"/>
-      <c r="E33" s="198"/>
-      <c r="F33" s="198"/>
-      <c r="G33" s="198"/>
-      <c r="H33" s="198"/>
-      <c r="I33" s="198"/>
-      <c r="J33" s="198"/>
-      <c r="K33" s="198"/>
-      <c r="L33" s="198"/>
-      <c r="M33" s="198"/>
-      <c r="N33" s="198"/>
-      <c r="O33" s="198"/>
-      <c r="P33" s="198"/>
-      <c r="Q33" s="198"/>
-      <c r="R33" s="198"/>
-      <c r="S33" s="198"/>
+      <c r="A33" s="213" t="s">
+        <v>368</v>
+      </c>
+      <c r="B33" s="212"/>
+      <c r="C33" s="212"/>
+      <c r="D33" s="212"/>
+      <c r="E33" s="212"/>
+      <c r="F33" s="212"/>
+      <c r="G33" s="212"/>
+      <c r="H33" s="212"/>
+      <c r="I33" s="212"/>
+      <c r="J33" s="212"/>
+      <c r="K33" s="212"/>
+      <c r="L33" s="212"/>
+      <c r="M33" s="212"/>
+      <c r="N33" s="212"/>
+      <c r="O33" s="212"/>
+      <c r="P33" s="212"/>
+      <c r="Q33" s="212"/>
+      <c r="R33" s="212"/>
+      <c r="S33" s="212"/>
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="199" t="s">
-        <v>367</v>
-      </c>
-      <c r="B34" s="198"/>
-      <c r="C34" s="198"/>
-      <c r="D34" s="198"/>
-      <c r="E34" s="198"/>
-      <c r="F34" s="198"/>
-      <c r="G34" s="198"/>
-      <c r="H34" s="198"/>
-      <c r="I34" s="198"/>
-      <c r="J34" s="198"/>
-      <c r="K34" s="198"/>
-      <c r="L34" s="198"/>
-      <c r="M34" s="198"/>
-      <c r="N34" s="198"/>
-      <c r="O34" s="198"/>
-      <c r="P34" s="198"/>
-      <c r="Q34" s="198"/>
-      <c r="R34" s="198"/>
-      <c r="S34" s="198"/>
+      <c r="A34" s="213" t="s">
+        <v>369</v>
+      </c>
+      <c r="B34" s="212"/>
+      <c r="C34" s="212"/>
+      <c r="D34" s="212"/>
+      <c r="E34" s="212"/>
+      <c r="F34" s="212"/>
+      <c r="G34" s="212"/>
+      <c r="H34" s="212"/>
+      <c r="I34" s="212"/>
+      <c r="J34" s="212"/>
+      <c r="K34" s="212"/>
+      <c r="L34" s="212"/>
+      <c r="M34" s="212"/>
+      <c r="N34" s="212"/>
+      <c r="O34" s="212"/>
+      <c r="P34" s="212"/>
+      <c r="Q34" s="212"/>
+      <c r="R34" s="212"/>
+      <c r="S34" s="212"/>
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="199" t="s">
-        <v>368</v>
-      </c>
-      <c r="B35" s="198"/>
-      <c r="C35" s="198"/>
-      <c r="D35" s="198"/>
-      <c r="E35" s="198"/>
-      <c r="F35" s="198"/>
-      <c r="G35" s="198"/>
-      <c r="H35" s="198"/>
-      <c r="I35" s="198"/>
-      <c r="J35" s="198"/>
-      <c r="K35" s="198"/>
-      <c r="L35" s="198"/>
-      <c r="M35" s="198"/>
-      <c r="N35" s="198"/>
-      <c r="O35" s="198"/>
-      <c r="P35" s="198"/>
-      <c r="Q35" s="198"/>
-      <c r="R35" s="198"/>
-      <c r="S35" s="198"/>
+      <c r="A35" s="213" t="s">
+        <v>370</v>
+      </c>
+      <c r="B35" s="212"/>
+      <c r="C35" s="212"/>
+      <c r="D35" s="212"/>
+      <c r="E35" s="212"/>
+      <c r="F35" s="212"/>
+      <c r="G35" s="212"/>
+      <c r="H35" s="212"/>
+      <c r="I35" s="212"/>
+      <c r="J35" s="212"/>
+      <c r="K35" s="212"/>
+      <c r="L35" s="212"/>
+      <c r="M35" s="212"/>
+      <c r="N35" s="212"/>
+      <c r="O35" s="212"/>
+      <c r="P35" s="212"/>
+      <c r="Q35" s="212"/>
+      <c r="R35" s="212"/>
+      <c r="S35" s="212"/>
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="199" t="s">
-        <v>369</v>
-      </c>
-      <c r="B36" s="198"/>
-      <c r="C36" s="198"/>
-      <c r="D36" s="198"/>
-      <c r="E36" s="198"/>
-      <c r="F36" s="198"/>
-      <c r="G36" s="198"/>
-      <c r="H36" s="198"/>
-      <c r="I36" s="198"/>
-      <c r="J36" s="198"/>
-      <c r="K36" s="198"/>
-      <c r="L36" s="198"/>
-      <c r="M36" s="198"/>
-      <c r="N36" s="198"/>
-      <c r="O36" s="198"/>
-      <c r="P36" s="198"/>
-      <c r="Q36" s="198"/>
-      <c r="R36" s="198"/>
-      <c r="S36" s="198"/>
+      <c r="A36" s="213" t="s">
+        <v>371</v>
+      </c>
+      <c r="B36" s="212"/>
+      <c r="C36" s="212"/>
+      <c r="D36" s="212"/>
+      <c r="E36" s="212"/>
+      <c r="F36" s="212"/>
+      <c r="G36" s="212"/>
+      <c r="H36" s="212"/>
+      <c r="I36" s="212"/>
+      <c r="J36" s="212"/>
+      <c r="K36" s="212"/>
+      <c r="L36" s="212"/>
+      <c r="M36" s="212"/>
+      <c r="N36" s="212"/>
+      <c r="O36" s="212"/>
+      <c r="P36" s="212"/>
+      <c r="Q36" s="212"/>
+      <c r="R36" s="212"/>
+      <c r="S36" s="212"/>
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="210" t="s">
-        <v>370</v>
-      </c>
-      <c r="B37" s="198"/>
-      <c r="C37" s="198"/>
-      <c r="D37" s="198"/>
-      <c r="E37" s="198"/>
-      <c r="F37" s="198"/>
-      <c r="G37" s="198"/>
-      <c r="H37" s="198"/>
-      <c r="I37" s="198"/>
-      <c r="J37" s="198"/>
-      <c r="K37" s="198"/>
-      <c r="L37" s="198"/>
-      <c r="M37" s="198"/>
-      <c r="N37" s="198"/>
-      <c r="O37" s="198"/>
-      <c r="P37" s="198"/>
-      <c r="Q37" s="198"/>
-      <c r="R37" s="198"/>
-      <c r="S37" s="198"/>
+      <c r="A37" s="224" t="s">
+        <v>372</v>
+      </c>
+      <c r="B37" s="212"/>
+      <c r="C37" s="212"/>
+      <c r="D37" s="212"/>
+      <c r="E37" s="212"/>
+      <c r="F37" s="212"/>
+      <c r="G37" s="212"/>
+      <c r="H37" s="212"/>
+      <c r="I37" s="212"/>
+      <c r="J37" s="212"/>
+      <c r="K37" s="212"/>
+      <c r="L37" s="212"/>
+      <c r="M37" s="212"/>
+      <c r="N37" s="212"/>
+      <c r="O37" s="212"/>
+      <c r="P37" s="212"/>
+      <c r="Q37" s="212"/>
+      <c r="R37" s="212"/>
+      <c r="S37" s="212"/>
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="38" t="s">
-        <v>305</v>
-      </c>
-      <c r="B39" s="213" t="s">
-        <v>371</v>
-      </c>
-      <c r="C39" s="198"/>
-      <c r="D39" s="198"/>
-      <c r="E39" s="211" t="s">
-        <v>372</v>
-      </c>
-      <c r="F39" s="198"/>
-      <c r="G39" s="198"/>
-      <c r="H39" s="214" t="s">
+        <v>307</v>
+      </c>
+      <c r="B39" s="227" t="s">
         <v>373</v>
       </c>
-      <c r="I39" s="198"/>
-      <c r="J39" s="198"/>
-      <c r="K39" s="207" t="s">
+      <c r="C39" s="212"/>
+      <c r="D39" s="212"/>
+      <c r="E39" s="225" t="s">
         <v>374</v>
       </c>
-      <c r="L39" s="198"/>
-      <c r="M39" s="198"/>
-      <c r="N39" s="205" t="s">
+      <c r="F39" s="212"/>
+      <c r="G39" s="212"/>
+      <c r="H39" s="228" t="s">
+        <v>375</v>
+      </c>
+      <c r="I39" s="212"/>
+      <c r="J39" s="212"/>
+      <c r="K39" s="221" t="s">
+        <v>376</v>
+      </c>
+      <c r="L39" s="212"/>
+      <c r="M39" s="212"/>
+      <c r="N39" s="219" t="s">
         <v>45</v>
       </c>
-      <c r="O39" s="198"/>
-      <c r="P39" s="198"/>
-      <c r="Q39" s="212" t="s">
-        <v>375</v>
-      </c>
-      <c r="R39" s="198"/>
-      <c r="S39" s="198"/>
+      <c r="O39" s="212"/>
+      <c r="P39" s="212"/>
+      <c r="Q39" s="226" t="s">
+        <v>377</v>
+      </c>
+      <c r="R39" s="212"/>
+      <c r="S39" s="212"/>
     </row>
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A16:S16"/>
     <mergeCell ref="H20:M20"/>
-    <mergeCell ref="A16:S16"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -9045,14 +9201,13 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -9061,6 +9216,7 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -9068,7 +9224,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -9116,33 +9272,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="216" t="s">
-        <v>376</v>
-      </c>
-      <c r="B1" s="190"/>
-      <c r="C1" s="190"/>
-      <c r="D1" s="190"/>
-      <c r="E1" s="190"/>
-      <c r="F1" s="191"/>
+      <c r="A1" s="230" t="s">
+        <v>378</v>
+      </c>
+      <c r="B1" s="204"/>
+      <c r="C1" s="204"/>
+      <c r="D1" s="204"/>
+      <c r="E1" s="204"/>
+      <c r="F1" s="205"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -9351,11 +9507,11 @@
       </c>
       <c r="B12" s="26">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C12" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D12" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -9367,7 +9523,7 @@
       </c>
       <c r="F12" s="27">
         <f t="shared" si="1"/>
-        <v>0.27272727272727271</v>
+        <v>0.30434782608695654</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -9422,15 +9578,15 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="28" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B16" s="29">
         <f>SUM(B4:B14)</f>
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C16" s="29">
         <f>SUM(C4:C14)</f>
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
@@ -9442,12 +9598,12 @@
       </c>
       <c r="F16" s="30">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.64885496183206104</v>
+        <v>0.65151515151515149</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="43" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B18" s="44">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -9456,7 +9612,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="45" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
   </sheetData>
@@ -9477,7 +9633,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -9488,641 +9644,675 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="216" t="s">
-        <v>383</v>
-      </c>
-      <c r="B1" s="190"/>
-      <c r="C1" s="190"/>
-      <c r="D1" s="190"/>
-      <c r="E1" s="191"/>
+      <c r="A1" s="230" t="s">
+        <v>385</v>
+      </c>
+      <c r="B1" s="204"/>
+      <c r="C1" s="204"/>
+      <c r="D1" s="204"/>
+      <c r="E1" s="205"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="31" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="D3" s="31" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="32" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="34" t="s">
+        <v>395</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>396</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>393</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>394</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>391</v>
-      </c>
       <c r="E5" s="35" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="32" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="34" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="32" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="34" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="32" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="34" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="32" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="34" t="s">
+        <v>419</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>404</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>417</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>397</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>402</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>415</v>
-      </c>
       <c r="E13" s="35" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="32" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="34" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="32" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="34" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="32" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="34" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="32" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="34" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="32" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E22" s="33" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="34" t="s">
+        <v>443</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>441</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>439</v>
-      </c>
       <c r="C23" s="19" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E23" s="35" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="32" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="58" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B25" s="55" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C25" s="59" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D25" s="55" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E25" s="60" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="61" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B26" s="49" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C26" s="59" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="D26" s="49" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="E26" s="62" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="58" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B27" s="55" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C27" s="59" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="D27" s="55" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E27" s="60" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="79" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B28" s="66" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C28" s="75" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D28" s="107" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="E28" s="107" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="80" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B29" s="72" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C29" s="77" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D29" s="106" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="E29" s="106" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="88" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B30" s="84" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C30" s="89" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D30" s="84" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E30" s="90" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="105" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B31" s="94" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C31" s="103" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D31" s="94" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="E31" s="106" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="122" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B32" s="117" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C32" s="120" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D32" s="117" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="E32" s="123" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="124" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B33" s="111" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C33" s="120" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D33" s="111" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="E33" s="125" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="156" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B34" s="150" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C34" s="142" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D34" s="150" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E34" s="157" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="158" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B35" s="143" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C35" s="154" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D35" s="143" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E35" s="159" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="74.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="172" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B36" s="169" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C36" s="173" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D36" s="178" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="E36" s="178" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="175" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B37" s="163" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C37" s="176" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D37" s="163" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E37" s="177" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="172" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B38" s="169" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C38" s="176" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="D38" s="169" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E38" s="174" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="186" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B39" s="182" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C39" s="187" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D39" s="182" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E39" s="188" t="s">
-        <v>475</v>
+        <v>477</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A40" s="196" t="s">
+        <v>478</v>
+      </c>
+      <c r="B40" s="192" t="s">
+        <v>441</v>
+      </c>
+      <c r="C40" s="197" t="s">
+        <v>396</v>
+      </c>
+      <c r="D40" s="192" t="s">
+        <v>393</v>
+      </c>
+      <c r="E40" s="198" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A41" s="199" t="s">
+        <v>140</v>
+      </c>
+      <c r="B41" s="200" t="s">
+        <v>405</v>
+      </c>
+      <c r="C41" s="201" t="s">
+        <v>404</v>
+      </c>
+      <c r="D41" s="200" t="s">
+        <v>436</v>
+      </c>
+      <c r="E41" s="202" t="s">
+        <v>480</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(tracker): no-draw guard, the player1 correction, and the stale-worker risk
Board now 197 items / 149 done, Unassigned=0.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90265004-76AB-4F7C-9EC9-82B158556ED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{199108CA-0FC2-46FB-813F-804F242BFD14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1454" uniqueCount="728">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1477" uniqueCount="736">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -1336,6 +1336,24 @@
   </si>
   <si>
     <t>Season 2026 currently holds 1,344 rows vs ~10,900 for a completed season. Promoting a 12%-complete season to TEST would make every headline metric small-sample while looking like a like-for-like comparison. Move all three windows together (train 2022-24 / val 2025 / test 2026), not just the test season. Until then, collecting current-season data cannot improve the model - only retrodiction</t>
+  </si>
+  <si>
+    <t>Impossible drawn outcomes: guarded and removed</t>
+  </si>
+  <si>
+    <t>_maybe_settle_outcome fell through to MatchResult.DRAW on any tied score, so 12 tennis rows recorded a result that cannot exist (a retirement leaves equal COMPLETED sets but still has a winner). SPORTS_WITHOUT_DRAWS now settles NOTHING on a tie - no Outcome, no draw-shaped Elo. No winner is guessed because none is available (see the player1 row). Deletion only sticks because of the guard: the first removal was undone within minutes by a stale Celery worker. Verified after restart - 2 real scheduled runs, 2 guard activations, 0 recreated. 05757c2</t>
+  </si>
+  <si>
+    <t>CORRECTED: 'player1 is always the winner' is too strong</t>
+  </si>
+  <si>
+    <t>Measured: LIST ?season=2022 100% (60/60), 2025 100% (59/59), 2026 68% (41/60), GET /matches/{id} 48% (12/25). The ordering is a property of SETTLED HISTORICAL data on the list endpoint. The leakage was real and _home_away_players is still required - training reads settled seasons - but the rule cannot be INVERTED to recover a winner, which is the case that came up. At 48% it is a coin flip. a1c52c3</t>
+  </si>
+  <si>
+    <t>Stale Celery worker hit AGAIN (2nd time in one day)</t>
+  </si>
+  <si>
+    <t>A guard written at 12:28 could not take effect in a worker started at 08:55, so ingest_live_scores re-created the deleted rows every 5 minutes. Same trap as this morning's odds gap. Restart the worker after ANY change under app/ before concluding anything from live data - the symptom is never an error, it is 'my fix did not take'</t>
   </si>
   <si>
     <t>Legend</t>
@@ -2056,6 +2074,12 @@
   </si>
   <si>
     <t>A season matching no split is assembled and then dropped, so collecting it changes nothing in the model while every surface signal (example count up, retrain runs, new artefact registered) suggests it did. Confirmed only by hashing the boosters. Hash the artefact before believing a retrain did anything</t>
+  </si>
+  <si>
+    <t>Stale workers keep masking real fixes</t>
+  </si>
+  <si>
+    <t>Hit twice on 2026-08-10: a LEAGUE_IDS change the worker never loaded (no odds for 9 leagues), then a no-draw guard the worker never loaded (deleted rows recreated every 5 minutes). Neither raised an error; both looked like the fix not working. Restart worker and beat after any change under app/, and check process start time against file mtime before believing live data</t>
   </si>
   <si>
     <t>External APIs, Quotas &amp; Expiry</t>
@@ -4499,7 +4523,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R200"/>
+  <dimension ref="A1:R203"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -10383,7 +10407,7 @@
         <v>342</v>
       </c>
       <c r="R166" t="str">
-        <f t="shared" ref="R166:R198" si="5">IF($A166&lt;&gt;"",$A166,R165)</f>
+        <f t="shared" ref="R166:R201" si="5">IF($A166&lt;&gt;"",$A166,R165)</f>
         <v>E9 Data Ops</v>
       </c>
     </row>
@@ -11161,7 +11185,7 @@
         <v>E9 Data Ops</v>
       </c>
     </row>
-    <row r="196" spans="1:18" ht="115.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="196" spans="1:18" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A196" t="s">
         <v>51</v>
       </c>
@@ -11191,7 +11215,7 @@
         <v>E4 ML Football</v>
       </c>
     </row>
-    <row r="197" spans="1:18" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="197" spans="1:18" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A197" t="s">
         <v>191</v>
       </c>
@@ -11221,7 +11245,7 @@
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="198" spans="1:18" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="198" spans="1:18" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A198" t="s">
         <v>51</v>
       </c>
@@ -11245,23 +11269,113 @@
         <v>E4 ML Football</v>
       </c>
     </row>
-    <row r="200" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A200" s="25" t="s">
+    <row r="199" spans="1:18" ht="129.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A199" t="s">
+        <v>62</v>
+      </c>
+      <c r="B199" t="s">
         <v>433</v>
       </c>
-      <c r="B200" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C200" s="17" t="s">
+      <c r="C199" t="s">
+        <v>22</v>
+      </c>
+      <c r="D199" t="s">
+        <v>75</v>
+      </c>
+      <c r="E199" s="245">
+        <v>46244</v>
+      </c>
+      <c r="F199" s="245">
+        <v>46244</v>
+      </c>
+      <c r="G199" s="250" t="s">
         <v>434</v>
       </c>
-      <c r="D200" s="19" t="s">
+      <c r="J199" t="s">
+        <v>400</v>
+      </c>
+      <c r="R199" t="str">
+        <f t="shared" si="5"/>
+        <v>E5 ML Tennis</v>
+      </c>
+    </row>
+    <row r="200" spans="1:18" ht="100.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A200" t="s">
+        <v>130</v>
+      </c>
+      <c r="B200" t="s">
+        <v>435</v>
+      </c>
+      <c r="C200" t="s">
+        <v>22</v>
+      </c>
+      <c r="D200" t="s">
+        <v>33</v>
+      </c>
+      <c r="E200" s="245">
+        <v>46244</v>
+      </c>
+      <c r="F200" s="245">
+        <v>46244</v>
+      </c>
+      <c r="G200" s="250" t="s">
+        <v>436</v>
+      </c>
+      <c r="J200" t="s">
+        <v>400</v>
+      </c>
+      <c r="R200" t="str">
+        <f t="shared" si="5"/>
+        <v>E9 Data Ops</v>
+      </c>
+    </row>
+    <row r="201" spans="1:18" ht="72" x14ac:dyDescent="0.55000000000000004">
+      <c r="A201" t="s">
+        <v>191</v>
+      </c>
+      <c r="B201" t="s">
+        <v>437</v>
+      </c>
+      <c r="C201" t="s">
+        <v>22</v>
+      </c>
+      <c r="D201" t="s">
+        <v>362</v>
+      </c>
+      <c r="E201" s="245">
+        <v>46244</v>
+      </c>
+      <c r="F201" s="245">
+        <v>46244</v>
+      </c>
+      <c r="G201" s="250" t="s">
+        <v>438</v>
+      </c>
+      <c r="J201" t="s">
+        <v>400</v>
+      </c>
+      <c r="R201" t="str">
+        <f t="shared" si="5"/>
+        <v>E11 Ops Resilience</v>
+      </c>
+    </row>
+    <row r="203" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A203" s="25" t="s">
+        <v>439</v>
+      </c>
+      <c r="B203" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C203" s="17" t="s">
+        <v>440</v>
+      </c>
+      <c r="D203" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="E200" s="23" t="s">
+      <c r="E203" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="F200" s="21" t="s">
+      <c r="F203" s="21" t="s">
         <v>138</v>
       </c>
     </row>
@@ -11286,7 +11400,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="273" t="s">
-        <v>435</v>
+        <v>441</v>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -11309,7 +11423,7 @@
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="280" t="s">
-        <v>436</v>
+        <v>442</v>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -11332,7 +11446,7 @@
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="268" t="s">
-        <v>437</v>
+        <v>443</v>
       </c>
       <c r="B4" s="262"/>
       <c r="C4" s="262"/>
@@ -11355,42 +11469,42 @@
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="37" t="s">
-        <v>438</v>
+        <v>444</v>
       </c>
       <c r="B5" s="258" t="s">
-        <v>439</v>
+        <v>445</v>
       </c>
       <c r="C5" s="259"/>
       <c r="D5" s="260"/>
       <c r="E5" s="263" t="s">
-        <v>440</v>
+        <v>446</v>
       </c>
       <c r="F5" s="259"/>
       <c r="G5" s="260"/>
       <c r="H5" s="263" t="s">
-        <v>441</v>
+        <v>447</v>
       </c>
       <c r="I5" s="259"/>
       <c r="J5" s="260"/>
       <c r="K5" s="258" t="s">
-        <v>442</v>
+        <v>448</v>
       </c>
       <c r="L5" s="259"/>
       <c r="M5" s="260"/>
       <c r="N5" s="265" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="O5" s="259"/>
       <c r="P5" s="260"/>
       <c r="Q5" s="265" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
       <c r="R5" s="259"/>
       <c r="S5" s="260"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="261" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="C6" s="262"/>
       <c r="D6" s="262"/>
@@ -11412,7 +11526,7 @@
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="268" t="s">
-        <v>446</v>
+        <v>452</v>
       </c>
       <c r="B7" s="262"/>
       <c r="C7" s="262"/>
@@ -11435,10 +11549,10 @@
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="37" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="B8" s="271" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
       <c r="C8" s="259"/>
       <c r="D8" s="259"/>
@@ -11449,7 +11563,7 @@
       <c r="I8" s="259"/>
       <c r="J8" s="260"/>
       <c r="K8" s="271" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
       <c r="L8" s="259"/>
       <c r="M8" s="259"/>
@@ -11462,7 +11576,7 @@
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="261" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="C9" s="262"/>
       <c r="D9" s="262"/>
@@ -11484,7 +11598,7 @@
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="268" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="B10" s="262"/>
       <c r="C10" s="262"/>
@@ -11507,42 +11621,42 @@
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="37" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
       <c r="B11" s="258" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
       <c r="C11" s="259"/>
       <c r="D11" s="260"/>
       <c r="E11" s="258" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="F11" s="259"/>
       <c r="G11" s="260"/>
       <c r="H11" s="258" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
       <c r="I11" s="259"/>
       <c r="J11" s="260"/>
       <c r="K11" s="263" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="L11" s="259"/>
       <c r="M11" s="260"/>
       <c r="N11" s="258" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="O11" s="259"/>
       <c r="P11" s="260"/>
       <c r="Q11" s="258" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
       <c r="R11" s="259"/>
       <c r="S11" s="260"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="261" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="C12" s="262"/>
       <c r="D12" s="262"/>
@@ -11564,7 +11678,7 @@
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="268" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
       <c r="B13" s="262"/>
       <c r="C13" s="262"/>
@@ -11587,10 +11701,10 @@
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="37" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="B14" s="266" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="C14" s="259"/>
       <c r="D14" s="259"/>
@@ -11598,7 +11712,7 @@
       <c r="F14" s="259"/>
       <c r="G14" s="260"/>
       <c r="H14" s="266" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="I14" s="259"/>
       <c r="J14" s="259"/>
@@ -11606,19 +11720,19 @@
       <c r="L14" s="259"/>
       <c r="M14" s="260"/>
       <c r="N14" s="266" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="O14" s="259"/>
       <c r="P14" s="260"/>
       <c r="Q14" s="263" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="R14" s="259"/>
       <c r="S14" s="260"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" s="261" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="C15" s="262"/>
       <c r="D15" s="262"/>
@@ -11640,7 +11754,7 @@
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="268" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="B16" s="262"/>
       <c r="C16" s="262"/>
@@ -11663,10 +11777,10 @@
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="37" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="B17" s="267" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
       <c r="C17" s="259"/>
       <c r="D17" s="259"/>
@@ -11674,29 +11788,29 @@
       <c r="F17" s="259"/>
       <c r="G17" s="260"/>
       <c r="H17" s="267" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="I17" s="259"/>
       <c r="J17" s="260"/>
       <c r="K17" s="267" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="L17" s="259"/>
       <c r="M17" s="260"/>
       <c r="N17" s="267" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
       <c r="O17" s="259"/>
       <c r="P17" s="260"/>
       <c r="Q17" s="267" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="R17" s="259"/>
       <c r="S17" s="260"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="261" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="C18" s="262"/>
       <c r="D18" s="262"/>
@@ -11718,7 +11832,7 @@
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="268" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="B19" s="262"/>
       <c r="C19" s="262"/>
@@ -11741,10 +11855,10 @@
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="37" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
       <c r="B20" s="269" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
       <c r="C20" s="259"/>
       <c r="D20" s="259"/>
@@ -11752,7 +11866,7 @@
       <c r="F20" s="259"/>
       <c r="G20" s="260"/>
       <c r="H20" s="269" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="I20" s="259"/>
       <c r="J20" s="259"/>
@@ -11760,7 +11874,7 @@
       <c r="L20" s="259"/>
       <c r="M20" s="260"/>
       <c r="N20" s="269" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
       <c r="O20" s="259"/>
       <c r="P20" s="259"/>
@@ -11770,7 +11884,7 @@
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" s="261" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="C21" s="262"/>
       <c r="D21" s="262"/>
@@ -11792,7 +11906,7 @@
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="268" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="B22" s="262"/>
       <c r="C22" s="262"/>
@@ -11815,10 +11929,10 @@
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="37" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
       <c r="B23" s="269" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
       <c r="C23" s="259"/>
       <c r="D23" s="259"/>
@@ -11826,29 +11940,29 @@
       <c r="F23" s="259"/>
       <c r="G23" s="260"/>
       <c r="H23" s="269" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="I23" s="259"/>
       <c r="J23" s="260"/>
       <c r="K23" s="269" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
       <c r="L23" s="259"/>
       <c r="M23" s="260"/>
       <c r="N23" s="269" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
       <c r="O23" s="259"/>
       <c r="P23" s="260"/>
       <c r="Q23" s="265" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
       <c r="R23" s="259"/>
       <c r="S23" s="260"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="274" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
       <c r="B26" s="262"/>
       <c r="C26" s="262"/>
@@ -11871,42 +11985,42 @@
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="37" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="B27" s="258" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="C27" s="259"/>
       <c r="D27" s="260"/>
       <c r="E27" s="258" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="F27" s="259"/>
       <c r="G27" s="260"/>
       <c r="H27" s="266" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
       <c r="I27" s="259"/>
       <c r="J27" s="260"/>
       <c r="K27" s="267" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
       <c r="L27" s="259"/>
       <c r="M27" s="260"/>
       <c r="N27" s="267" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
       <c r="O27" s="259"/>
       <c r="P27" s="260"/>
       <c r="Q27" s="266" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="R27" s="259"/>
       <c r="S27" s="260"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="268" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="B30" s="262"/>
       <c r="C30" s="262"/>
@@ -11929,7 +12043,7 @@
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="264" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="B31" s="262"/>
       <c r="C31" s="262"/>
@@ -11952,7 +12066,7 @@
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="264" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="B32" s="262"/>
       <c r="C32" s="262"/>
@@ -11975,7 +12089,7 @@
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="264" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="B33" s="262"/>
       <c r="C33" s="262"/>
@@ -11998,7 +12112,7 @@
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="264" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
       <c r="B34" s="262"/>
       <c r="C34" s="262"/>
@@ -12021,7 +12135,7 @@
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="264" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="B35" s="262"/>
       <c r="C35" s="262"/>
@@ -12044,7 +12158,7 @@
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="264" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
       <c r="B36" s="262"/>
       <c r="C36" s="262"/>
@@ -12067,7 +12181,7 @@
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="275" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="B37" s="262"/>
       <c r="C37" s="262"/>
@@ -12090,25 +12204,25 @@
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="38" t="s">
-        <v>433</v>
+        <v>439</v>
       </c>
       <c r="B39" s="278" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
       <c r="C39" s="262"/>
       <c r="D39" s="262"/>
       <c r="E39" s="276" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="F39" s="262"/>
       <c r="G39" s="262"/>
       <c r="H39" s="279" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="I39" s="262"/>
       <c r="J39" s="262"/>
       <c r="K39" s="272" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="L39" s="262"/>
       <c r="M39" s="262"/>
@@ -12118,7 +12232,7 @@
       <c r="O39" s="262"/>
       <c r="P39" s="262"/>
       <c r="Q39" s="277" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="R39" s="262"/>
       <c r="S39" s="262"/>
@@ -12126,11 +12240,11 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H14:M14"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A16:S16"/>
     <mergeCell ref="H20:M20"/>
-    <mergeCell ref="A16:S16"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -12139,13 +12253,14 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -12154,7 +12269,6 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
-    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -12162,7 +12276,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -12211,7 +12325,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="281" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
       <c r="B1" s="255"/>
       <c r="C1" s="255"/>
@@ -12224,19 +12338,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -12345,11 +12459,11 @@
       </c>
       <c r="B8" s="26">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C8" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A8,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D8" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A8,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A8,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A8,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -12361,7 +12475,7 @@
       </c>
       <c r="F8" s="27">
         <f t="shared" si="1"/>
-        <v>0.90909090909090906</v>
+        <v>0.91304347826086951</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -12445,11 +12559,11 @@
       </c>
       <c r="B12" s="26">
         <f t="shared" si="0"/>
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C12" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D12" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -12461,7 +12575,7 @@
       </c>
       <c r="F12" s="27">
         <f t="shared" si="1"/>
-        <v>0.59459459459459463</v>
+        <v>0.60526315789473684</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -12495,11 +12609,11 @@
       </c>
       <c r="B14" s="26">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C14" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D14" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -12511,20 +12625,20 @@
       </c>
       <c r="F14" s="27">
         <f t="shared" si="1"/>
-        <v>0.5625</v>
+        <v>0.58823529411764708</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="28" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="B16" s="29">
         <f>SUM(B4:B14)</f>
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C16" s="29">
         <f>SUM(C4:C14)</f>
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
@@ -12536,12 +12650,12 @@
       </c>
       <c r="F16" s="30">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.75257731958762886</v>
+        <v>0.75634517766497467</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="43" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="B18" s="44">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -12550,7 +12664,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="45" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
     </row>
   </sheetData>
@@ -12571,7 +12685,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -12583,7 +12697,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="281" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="B1" s="255"/>
       <c r="C1" s="255"/>
@@ -12592,648 +12706,648 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="31" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="D3" s="31" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="32" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="34" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="32" t="s">
+        <v>531</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>532</v>
+      </c>
+      <c r="C6" s="23" t="s">
         <v>525</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>526</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>519</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="34" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="32" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="34" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="32" t="s">
+        <v>543</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>544</v>
+      </c>
+      <c r="C10" s="19" t="s">
         <v>537</v>
       </c>
-      <c r="B10" s="12" t="s">
-        <v>538</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>531</v>
-      </c>
       <c r="D10" s="12" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="34" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="32" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="34" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="32" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="34" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="32" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="34" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="32" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="34" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="32" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="34" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="32" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E22" s="33" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="34" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E23" s="35" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="32" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="58" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
       <c r="B25" s="55" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="C25" s="59" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D25" s="55" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E25" s="60" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="61" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="B26" s="49" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="C26" s="59" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="D26" s="49" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E26" s="62" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="58" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="B27" s="55" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="C27" s="59" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="D27" s="55" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E27" s="60" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="79" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="B28" s="66" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="C28" s="75" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D28" s="107" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E28" s="107" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="80" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
       <c r="B29" s="72" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C29" s="77" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D29" s="106" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E29" s="106" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="88" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="B30" s="84" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C30" s="89" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D30" s="84" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E30" s="90" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="105" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
       <c r="B31" s="94" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="C31" s="103" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D31" s="94" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
       <c r="E31" s="106" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="122" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
       <c r="B32" s="117" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="C32" s="120" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D32" s="117" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E32" s="123" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="124" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="B33" s="111" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C33" s="120" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D33" s="111" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="E33" s="125" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="156" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="B34" s="150" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="C34" s="142" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D34" s="150" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E34" s="157" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="158" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
       <c r="B35" s="143" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C35" s="154" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D35" s="143" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E35" s="159" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="74.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="172" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="B36" s="169" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C36" s="173" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="D36" s="178" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="E36" s="178" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="175" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="B37" s="163" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="C37" s="176" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D37" s="163" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E37" s="177" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="172" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="B38" s="169" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="C38" s="176" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="D38" s="169" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E38" s="174" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="186" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="B39" s="182" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C39" s="187" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D39" s="182" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E39" s="188" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="196" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
       <c r="B40" s="192" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="C40" s="197" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D40" s="192" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E40" s="198" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -13241,356 +13355,373 @@
         <v>140</v>
       </c>
       <c r="B41" s="200" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="C41" s="201" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D41" s="200" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E41" s="202" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="219" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="B42" s="213" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="C42" s="205" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D42" s="213" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E42" s="220" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="221" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
       <c r="B43" s="206" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C43" s="217" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D43" s="206" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="E43" s="222" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="219" t="s">
-        <v>612</v>
+        <v>618</v>
       </c>
       <c r="B44" s="213" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="C44" s="217" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D44" s="213" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E44" s="220" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="221" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="B45" s="206" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="C45" s="217" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="D45" s="206" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E45" s="222" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="241" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
       <c r="B46" s="226" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="C46" s="232" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D46" s="226" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E46" s="242" t="s">
-        <v>617</v>
+        <v>623</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="243" t="s">
-        <v>618</v>
+        <v>624</v>
       </c>
       <c r="B47" s="233" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C47" s="237" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D47" s="233" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E47" s="244" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="241" t="s">
-        <v>620</v>
+        <v>626</v>
       </c>
       <c r="B48" s="226" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="C48" s="237" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D48" s="226" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E48" s="242" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
       <c r="B49" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C49" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D49" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E49" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
       <c r="B50" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C50" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D50" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E50" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
-        <v>626</v>
+        <v>632</v>
       </c>
       <c r="B51" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C51" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D51" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E51" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
       <c r="B52" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="C52" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="D52" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E52" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
       <c r="B53" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="C53" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="D53" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E53" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="250" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
       <c r="B54" s="250" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="C54" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="D54" s="250" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E54" s="250" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="250" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
       <c r="B55" s="250" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C55" s="250" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D55" s="250" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E55" s="250" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="B56" s="250" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C56" s="250" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D56" s="250" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E56" s="250" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="250" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
       <c r="B57" s="250" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C57" s="250" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D57" s="250" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E57" s="250" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="250" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
       <c r="B58" s="250" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C58" s="250" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D58" s="250" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E58" s="250" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="250" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="B59" s="250" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C59" s="250" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D59" s="250" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E59" s="250" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="250" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
       <c r="B60" s="250" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C60" s="250" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D60" s="250" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E60" s="250" t="s">
-        <v>646</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="250" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="B61" s="250" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C61" s="250" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D61" s="250" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="E61" s="250" t="s">
-        <v>648</v>
+        <v>654</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="72" x14ac:dyDescent="0.55000000000000004">
+      <c r="A62" s="250" t="s">
+        <v>655</v>
+      </c>
+      <c r="B62" s="250" t="s">
+        <v>524</v>
+      </c>
+      <c r="C62" s="250" t="s">
+        <v>537</v>
+      </c>
+      <c r="D62" s="250" t="s">
+        <v>526</v>
+      </c>
+      <c r="E62" s="250" t="s">
+        <v>656</v>
       </c>
     </row>
   </sheetData>
@@ -13619,336 +13750,336 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="246" t="s">
-        <v>649</v>
+        <v>657</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="247" t="s">
-        <v>650</v>
+        <v>658</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="248" t="s">
-        <v>651</v>
+        <v>659</v>
       </c>
       <c r="B4" s="248" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="C4" s="248" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
       <c r="D4" s="248" t="s">
-        <v>654</v>
+        <v>662</v>
       </c>
       <c r="E4" s="248" t="s">
-        <v>655</v>
+        <v>663</v>
       </c>
       <c r="F4" s="248" t="s">
-        <v>656</v>
+        <v>664</v>
       </c>
       <c r="G4" s="248" t="s">
-        <v>657</v>
+        <v>665</v>
       </c>
       <c r="H4" s="248" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="248" t="s">
-        <v>658</v>
+        <v>666</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="249" t="s">
-        <v>659</v>
+        <v>667</v>
       </c>
       <c r="B5" s="250" t="s">
-        <v>660</v>
+        <v>668</v>
       </c>
       <c r="C5" s="250" t="s">
-        <v>661</v>
+        <v>669</v>
       </c>
       <c r="D5" s="250" t="s">
-        <v>662</v>
+        <v>670</v>
       </c>
       <c r="E5" s="250" t="s">
-        <v>663</v>
+        <v>671</v>
       </c>
       <c r="F5" s="250" t="s">
-        <v>664</v>
+        <v>672</v>
       </c>
       <c r="G5" s="250" t="s">
-        <v>665</v>
+        <v>673</v>
       </c>
       <c r="H5" s="251" t="s">
-        <v>666</v>
+        <v>674</v>
       </c>
       <c r="I5" s="250" t="s">
-        <v>667</v>
+        <v>675</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="249" t="s">
-        <v>668</v>
+        <v>676</v>
       </c>
       <c r="B6" s="250" t="s">
-        <v>669</v>
+        <v>677</v>
       </c>
       <c r="C6" s="250" t="s">
-        <v>670</v>
+        <v>678</v>
       </c>
       <c r="D6" s="250" t="s">
-        <v>671</v>
+        <v>679</v>
       </c>
       <c r="E6" s="250" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="F6" s="250" t="s">
-        <v>673</v>
+        <v>681</v>
       </c>
       <c r="G6" s="250" t="s">
+        <v>682</v>
+      </c>
+      <c r="H6" s="252" t="s">
         <v>674</v>
       </c>
-      <c r="H6" s="252" t="s">
-        <v>666</v>
-      </c>
       <c r="I6" s="250" t="s">
-        <v>675</v>
+        <v>683</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="249" t="s">
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="B7" s="250" t="s">
-        <v>677</v>
+        <v>685</v>
       </c>
       <c r="C7" s="250" t="s">
-        <v>678</v>
+        <v>686</v>
       </c>
       <c r="D7" s="250" t="s">
-        <v>679</v>
+        <v>687</v>
       </c>
       <c r="E7" s="250" t="s">
-        <v>680</v>
+        <v>688</v>
       </c>
       <c r="F7" s="250" t="s">
-        <v>681</v>
+        <v>689</v>
       </c>
       <c r="G7" s="250" t="s">
-        <v>682</v>
+        <v>690</v>
       </c>
       <c r="H7" s="252" t="s">
-        <v>666</v>
+        <v>674</v>
       </c>
       <c r="I7" s="250" t="s">
-        <v>683</v>
+        <v>691</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="249" t="s">
-        <v>684</v>
+        <v>692</v>
       </c>
       <c r="B8" s="250" t="s">
-        <v>685</v>
+        <v>693</v>
       </c>
       <c r="C8" s="250" t="s">
-        <v>686</v>
+        <v>694</v>
       </c>
       <c r="D8" s="250" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
       <c r="E8" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="F8" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="G8" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="H8" s="251" t="s">
-        <v>688</v>
+        <v>696</v>
       </c>
       <c r="I8" s="250" t="s">
-        <v>689</v>
+        <v>697</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="249" t="s">
-        <v>690</v>
+        <v>698</v>
       </c>
       <c r="B9" s="250" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="C9" s="250" t="s">
-        <v>692</v>
+        <v>700</v>
       </c>
       <c r="D9" s="250" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
       <c r="E9" s="250" t="s">
-        <v>680</v>
+        <v>688</v>
       </c>
       <c r="F9" s="250" t="s">
-        <v>693</v>
+        <v>701</v>
       </c>
       <c r="G9" s="250" t="s">
-        <v>694</v>
+        <v>702</v>
       </c>
       <c r="H9" s="253" t="s">
-        <v>695</v>
+        <v>703</v>
       </c>
       <c r="I9" s="250" t="s">
-        <v>696</v>
+        <v>704</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="249" t="s">
-        <v>697</v>
+        <v>705</v>
       </c>
       <c r="B10" s="250" t="s">
-        <v>698</v>
+        <v>706</v>
       </c>
       <c r="C10" s="250" t="s">
-        <v>699</v>
+        <v>707</v>
       </c>
       <c r="D10" s="250" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="E10" s="250" t="s">
-        <v>701</v>
+        <v>709</v>
       </c>
       <c r="F10" s="250" t="s">
-        <v>702</v>
+        <v>710</v>
       </c>
       <c r="G10" s="250" t="s">
-        <v>703</v>
+        <v>711</v>
       </c>
       <c r="H10" s="253" t="s">
-        <v>704</v>
+        <v>712</v>
       </c>
       <c r="I10" s="250" t="s">
-        <v>705</v>
+        <v>713</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="249" t="s">
-        <v>706</v>
+        <v>714</v>
       </c>
       <c r="B11" s="250" t="s">
-        <v>707</v>
+        <v>715</v>
       </c>
       <c r="C11" s="250" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
       <c r="D11" s="250" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="E11" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="F11" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="G11" s="250" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="H11" s="253" t="s">
-        <v>711</v>
+        <v>719</v>
       </c>
       <c r="I11" s="250" t="s">
-        <v>712</v>
+        <v>720</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="249" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="B12" s="250" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="C12" s="250" t="s">
-        <v>715</v>
+        <v>723</v>
       </c>
       <c r="D12" s="250" t="s">
-        <v>716</v>
+        <v>724</v>
       </c>
       <c r="E12" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="F12" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="G12" s="250" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="H12" s="252" t="s">
-        <v>717</v>
+        <v>725</v>
       </c>
       <c r="I12" s="250" t="s">
-        <v>718</v>
+        <v>726</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="249" t="s">
-        <v>719</v>
+        <v>727</v>
       </c>
       <c r="B13" s="250" t="s">
-        <v>720</v>
+        <v>728</v>
       </c>
       <c r="C13" s="250" t="s">
-        <v>721</v>
+        <v>729</v>
       </c>
       <c r="D13" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="E13" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="F13" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="G13" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="H13" s="253" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="I13" s="250" t="s">
-        <v>723</v>
+        <v>731</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="249" t="s">
-        <v>724</v>
+        <v>732</v>
       </c>
       <c r="B14" s="250" t="s">
-        <v>725</v>
+        <v>733</v>
       </c>
       <c r="C14" s="250" t="s">
-        <v>721</v>
+        <v>729</v>
       </c>
       <c r="D14" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="E14" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="F14" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="G14" s="250" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="H14" s="253" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="I14" s="250" t="s">
-        <v>726</v>
+        <v>734</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="282" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
       <c r="B16" s="262"/>
       <c r="C16" s="262"/>

</xml_diff>

<commit_message>
docs(tracker): ml/ linting and the per-session test-DB truncation
Board now 198 items / 151 done, Unassigned=0.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{199108CA-0FC2-46FB-813F-804F242BFD14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B251458B-C48E-46EE-8879-D9EE85A04808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1477" uniqueCount="736">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1482" uniqueCount="738">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -1218,7 +1218,7 @@
     <t>Extend ruff/black to ml/</t>
   </si>
   <si>
-    <t>CI sets working-directory: backend, so ml/ has never been linted</t>
+    <t>DONE (4a4d6d4, CI-verified). 46 accumulated errors fixed; both trees now share backend's config. Notebooks excluded (provenance/exported artefacts). All 12 scripts import-checked after reformatting - they have no test coverage - and train_football.py AST-compared before/after: 9 functions, 99 calls, 132 assignments identical, so its 69-line drop was purely formatting</t>
   </si>
   <si>
     <t>DECIDE by 22 Sep: renew API-Football Ultra?</t>
@@ -1354,6 +1354,12 @@
   </si>
   <si>
     <t>A guard written at 12:28 could not take effect in a worker started at 08:55, so ingest_live_scores re-created the deleted rows every 5 minutes. Same trap as this morning's odds gap. Restart the worker after ANY change under app/ before concluding anything from live data - the symptom is never an error, it is 'my fix did not take'</t>
+  </si>
+  <si>
+    <t>Test DB truncated per session; teardown kept</t>
+  </si>
+  <si>
+    <t>Planned to DELETE the per-test teardown as redundant; reading it, that would have been a downgrade - it also keeps tests independent of each other, which the dedicated database does not address. Stale justifications corrected instead. The real gap was tests with NO teardown: users grew 21 per run indefinitely. conftest now truncates once per session, at the START so a failed run's rows stay inspectable. Verified 21 after both run 1 and run 2. ada6b50</t>
   </si>
   <si>
     <t>Legend</t>
@@ -4523,7 +4529,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R203"/>
+  <dimension ref="A1:R204"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -10407,7 +10413,7 @@
         <v>342</v>
       </c>
       <c r="R166" t="str">
-        <f t="shared" ref="R166:R201" si="5">IF($A166&lt;&gt;"",$A166,R165)</f>
+        <f t="shared" ref="R166:R202" si="5">IF($A166&lt;&gt;"",$A166,R165)</f>
         <v>E9 Data Ops</v>
       </c>
     </row>
@@ -10699,7 +10705,7 @@
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="179" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+    <row r="179" spans="1:18" ht="86.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A179" t="s">
         <v>191</v>
       </c>
@@ -10707,7 +10713,7 @@
         <v>392</v>
       </c>
       <c r="C179" t="s">
-        <v>128</v>
+        <v>22</v>
       </c>
       <c r="D179" t="s">
         <v>362</v>
@@ -10715,7 +10721,10 @@
       <c r="E179" s="245">
         <v>46243</v>
       </c>
-      <c r="G179" t="s">
+      <c r="F179" s="245">
+        <v>46244</v>
+      </c>
+      <c r="G179" s="250" t="s">
         <v>393</v>
       </c>
       <c r="R179" t="str">
@@ -11269,7 +11278,7 @@
         <v>E4 ML Football</v>
       </c>
     </row>
-    <row r="199" spans="1:18" ht="129.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="199" spans="1:18" ht="129.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A199" t="s">
         <v>62</v>
       </c>
@@ -11299,7 +11308,7 @@
         <v>E5 ML Tennis</v>
       </c>
     </row>
-    <row r="200" spans="1:18" ht="100.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="200" spans="1:18" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A200" t="s">
         <v>130</v>
       </c>
@@ -11329,7 +11338,7 @@
         <v>E9 Data Ops</v>
       </c>
     </row>
-    <row r="201" spans="1:18" ht="72" x14ac:dyDescent="0.55000000000000004">
+    <row r="201" spans="1:18" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A201" t="s">
         <v>191</v>
       </c>
@@ -11359,23 +11368,50 @@
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="203" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A203" s="25" t="s">
+    <row r="202" spans="1:18" ht="100.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="B202" t="s">
         <v>439</v>
       </c>
-      <c r="B203" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C203" s="17" t="s">
+      <c r="C202" t="s">
+        <v>22</v>
+      </c>
+      <c r="D202" t="s">
+        <v>362</v>
+      </c>
+      <c r="E202" s="245">
+        <v>46244</v>
+      </c>
+      <c r="F202" s="245">
+        <v>46244</v>
+      </c>
+      <c r="G202" s="250" t="s">
         <v>440</v>
       </c>
-      <c r="D203" s="19" t="s">
+      <c r="J202" t="s">
+        <v>400</v>
+      </c>
+      <c r="R202" t="str">
+        <f t="shared" si="5"/>
+        <v>E11 Ops Resilience</v>
+      </c>
+    </row>
+    <row r="204" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A204" s="25" t="s">
+        <v>441</v>
+      </c>
+      <c r="B204" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C204" s="17" t="s">
+        <v>442</v>
+      </c>
+      <c r="D204" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="E203" s="23" t="s">
+      <c r="E204" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="F203" s="21" t="s">
+      <c r="F204" s="21" t="s">
         <v>138</v>
       </c>
     </row>
@@ -11400,7 +11436,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="273" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -11423,7 +11459,7 @@
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="280" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -11446,7 +11482,7 @@
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="268" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B4" s="262"/>
       <c r="C4" s="262"/>
@@ -11469,42 +11505,42 @@
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="37" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B5" s="258" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="C5" s="259"/>
       <c r="D5" s="260"/>
       <c r="E5" s="263" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="F5" s="259"/>
       <c r="G5" s="260"/>
       <c r="H5" s="263" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="I5" s="259"/>
       <c r="J5" s="260"/>
       <c r="K5" s="258" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="L5" s="259"/>
       <c r="M5" s="260"/>
       <c r="N5" s="265" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="O5" s="259"/>
       <c r="P5" s="260"/>
       <c r="Q5" s="265" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="R5" s="259"/>
       <c r="S5" s="260"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="261" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="C6" s="262"/>
       <c r="D6" s="262"/>
@@ -11526,7 +11562,7 @@
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="268" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B7" s="262"/>
       <c r="C7" s="262"/>
@@ -11549,10 +11585,10 @@
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="37" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B8" s="271" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="C8" s="259"/>
       <c r="D8" s="259"/>
@@ -11563,7 +11599,7 @@
       <c r="I8" s="259"/>
       <c r="J8" s="260"/>
       <c r="K8" s="271" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="L8" s="259"/>
       <c r="M8" s="259"/>
@@ -11576,7 +11612,7 @@
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="261" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="C9" s="262"/>
       <c r="D9" s="262"/>
@@ -11598,7 +11634,7 @@
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="268" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B10" s="262"/>
       <c r="C10" s="262"/>
@@ -11621,42 +11657,42 @@
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="37" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B11" s="258" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="C11" s="259"/>
       <c r="D11" s="260"/>
       <c r="E11" s="258" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="F11" s="259"/>
       <c r="G11" s="260"/>
       <c r="H11" s="258" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="I11" s="259"/>
       <c r="J11" s="260"/>
       <c r="K11" s="263" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="L11" s="259"/>
       <c r="M11" s="260"/>
       <c r="N11" s="258" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="O11" s="259"/>
       <c r="P11" s="260"/>
       <c r="Q11" s="258" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="R11" s="259"/>
       <c r="S11" s="260"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="261" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="C12" s="262"/>
       <c r="D12" s="262"/>
@@ -11678,7 +11714,7 @@
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="268" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B13" s="262"/>
       <c r="C13" s="262"/>
@@ -11701,10 +11737,10 @@
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="37" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B14" s="266" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="C14" s="259"/>
       <c r="D14" s="259"/>
@@ -11712,7 +11748,7 @@
       <c r="F14" s="259"/>
       <c r="G14" s="260"/>
       <c r="H14" s="266" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="I14" s="259"/>
       <c r="J14" s="259"/>
@@ -11720,19 +11756,19 @@
       <c r="L14" s="259"/>
       <c r="M14" s="260"/>
       <c r="N14" s="266" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="O14" s="259"/>
       <c r="P14" s="260"/>
       <c r="Q14" s="263" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="R14" s="259"/>
       <c r="S14" s="260"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" s="261" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="C15" s="262"/>
       <c r="D15" s="262"/>
@@ -11754,7 +11790,7 @@
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="268" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B16" s="262"/>
       <c r="C16" s="262"/>
@@ -11777,10 +11813,10 @@
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="37" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B17" s="267" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C17" s="259"/>
       <c r="D17" s="259"/>
@@ -11788,29 +11824,29 @@
       <c r="F17" s="259"/>
       <c r="G17" s="260"/>
       <c r="H17" s="267" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="I17" s="259"/>
       <c r="J17" s="260"/>
       <c r="K17" s="267" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="L17" s="259"/>
       <c r="M17" s="260"/>
       <c r="N17" s="267" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="O17" s="259"/>
       <c r="P17" s="260"/>
       <c r="Q17" s="267" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="R17" s="259"/>
       <c r="S17" s="260"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="261" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="C18" s="262"/>
       <c r="D18" s="262"/>
@@ -11832,7 +11868,7 @@
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="268" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B19" s="262"/>
       <c r="C19" s="262"/>
@@ -11855,10 +11891,10 @@
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="37" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B20" s="269" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C20" s="259"/>
       <c r="D20" s="259"/>
@@ -11866,7 +11902,7 @@
       <c r="F20" s="259"/>
       <c r="G20" s="260"/>
       <c r="H20" s="269" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="I20" s="259"/>
       <c r="J20" s="259"/>
@@ -11874,7 +11910,7 @@
       <c r="L20" s="259"/>
       <c r="M20" s="260"/>
       <c r="N20" s="269" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="O20" s="259"/>
       <c r="P20" s="259"/>
@@ -11884,7 +11920,7 @@
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" s="261" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="C21" s="262"/>
       <c r="D21" s="262"/>
@@ -11906,7 +11942,7 @@
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="268" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B22" s="262"/>
       <c r="C22" s="262"/>
@@ -11929,10 +11965,10 @@
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="37" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B23" s="269" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="C23" s="259"/>
       <c r="D23" s="259"/>
@@ -11940,29 +11976,29 @@
       <c r="F23" s="259"/>
       <c r="G23" s="260"/>
       <c r="H23" s="269" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="I23" s="259"/>
       <c r="J23" s="260"/>
       <c r="K23" s="269" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="L23" s="259"/>
       <c r="M23" s="260"/>
       <c r="N23" s="269" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="O23" s="259"/>
       <c r="P23" s="260"/>
       <c r="Q23" s="265" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="R23" s="259"/>
       <c r="S23" s="260"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="274" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B26" s="262"/>
       <c r="C26" s="262"/>
@@ -11985,42 +12021,42 @@
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="37" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B27" s="258" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="C27" s="259"/>
       <c r="D27" s="260"/>
       <c r="E27" s="258" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="F27" s="259"/>
       <c r="G27" s="260"/>
       <c r="H27" s="266" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="I27" s="259"/>
       <c r="J27" s="260"/>
       <c r="K27" s="267" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="L27" s="259"/>
       <c r="M27" s="260"/>
       <c r="N27" s="267" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="O27" s="259"/>
       <c r="P27" s="260"/>
       <c r="Q27" s="266" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="R27" s="259"/>
       <c r="S27" s="260"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="268" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B30" s="262"/>
       <c r="C30" s="262"/>
@@ -12043,7 +12079,7 @@
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="264" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B31" s="262"/>
       <c r="C31" s="262"/>
@@ -12066,7 +12102,7 @@
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="264" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B32" s="262"/>
       <c r="C32" s="262"/>
@@ -12089,7 +12125,7 @@
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="264" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B33" s="262"/>
       <c r="C33" s="262"/>
@@ -12112,7 +12148,7 @@
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="264" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B34" s="262"/>
       <c r="C34" s="262"/>
@@ -12135,7 +12171,7 @@
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="264" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B35" s="262"/>
       <c r="C35" s="262"/>
@@ -12158,7 +12194,7 @@
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="264" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B36" s="262"/>
       <c r="C36" s="262"/>
@@ -12181,7 +12217,7 @@
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="275" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B37" s="262"/>
       <c r="C37" s="262"/>
@@ -12204,25 +12240,25 @@
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="38" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B39" s="278" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="C39" s="262"/>
       <c r="D39" s="262"/>
       <c r="E39" s="276" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="F39" s="262"/>
       <c r="G39" s="262"/>
       <c r="H39" s="279" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="I39" s="262"/>
       <c r="J39" s="262"/>
       <c r="K39" s="272" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="L39" s="262"/>
       <c r="M39" s="262"/>
@@ -12232,7 +12268,7 @@
       <c r="O39" s="262"/>
       <c r="P39" s="262"/>
       <c r="Q39" s="277" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="R39" s="262"/>
       <c r="S39" s="262"/>
@@ -12240,11 +12276,11 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="H20:M20"/>
     <mergeCell ref="A16:S16"/>
-    <mergeCell ref="H20:M20"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -12253,14 +12289,13 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -12269,6 +12304,7 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -12276,7 +12312,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -12325,7 +12361,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="281" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B1" s="255"/>
       <c r="C1" s="255"/>
@@ -12338,19 +12374,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -12609,15 +12645,15 @@
       </c>
       <c r="B14" s="26">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C14" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D14" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E14" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"Blocked")</f>
@@ -12625,24 +12661,24 @@
       </c>
       <c r="F14" s="27">
         <f t="shared" si="1"/>
-        <v>0.58823529411764708</v>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="28" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B16" s="29">
         <f>SUM(B4:B14)</f>
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C16" s="29">
         <f>SUM(C4:C14)</f>
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E16">
         <f>SUM(E4:E14)</f>
@@ -12650,12 +12686,12 @@
       </c>
       <c r="F16" s="30">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.75634517766497467</v>
+        <v>0.76262626262626265</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="43" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B18" s="44">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -12664,7 +12700,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="45" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
   </sheetData>
@@ -12697,7 +12733,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="281" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B1" s="255"/>
       <c r="C1" s="255"/>
@@ -12706,648 +12742,648 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="31" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="D3" s="31" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="32" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="34" t="s">
+        <v>530</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>526</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>531</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>528</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>529</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>526</v>
-      </c>
       <c r="E5" s="35" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="32" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="34" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="32" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="34" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="32" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="34" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="32" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="34" t="s">
+        <v>554</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>539</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>552</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>532</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>537</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>550</v>
-      </c>
       <c r="E13" s="35" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="32" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="34" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="32" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="34" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="32" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="34" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="32" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="34" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="32" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E22" s="33" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="34" t="s">
+        <v>578</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>576</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>574</v>
-      </c>
       <c r="C23" s="19" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E23" s="35" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="32" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="58" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="B25" s="55" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="C25" s="59" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D25" s="55" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E25" s="60" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="61" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="B26" s="49" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="C26" s="59" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="D26" s="49" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E26" s="62" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="58" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="B27" s="55" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="C27" s="59" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="D27" s="55" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E27" s="60" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="79" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B28" s="66" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="C28" s="75" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D28" s="107" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E28" s="107" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="80" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="B29" s="72" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C29" s="77" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D29" s="106" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E29" s="106" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="88" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="B30" s="84" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C30" s="89" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D30" s="84" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E30" s="90" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="105" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="B31" s="94" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="C31" s="103" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D31" s="94" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="E31" s="106" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="122" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="B32" s="117" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="C32" s="120" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D32" s="117" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E32" s="123" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="124" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="B33" s="111" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C33" s="120" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D33" s="111" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="E33" s="125" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="156" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="B34" s="150" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="C34" s="142" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D34" s="150" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E34" s="157" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="158" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B35" s="143" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C35" s="154" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D35" s="143" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E35" s="159" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="74.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="172" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B36" s="169" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C36" s="173" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="D36" s="178" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="E36" s="178" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="175" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="B37" s="163" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="C37" s="176" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D37" s="163" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E37" s="177" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="172" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="B38" s="169" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="C38" s="176" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="D38" s="169" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E38" s="174" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="186" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="B39" s="182" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C39" s="187" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D39" s="182" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E39" s="188" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="196" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="B40" s="192" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="C40" s="197" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D40" s="192" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E40" s="198" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -13355,373 +13391,373 @@
         <v>140</v>
       </c>
       <c r="B41" s="200" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="C41" s="201" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D41" s="200" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E41" s="202" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="219" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="B42" s="213" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="C42" s="205" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D42" s="213" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E42" s="220" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="221" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="B43" s="206" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C43" s="217" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D43" s="206" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="E43" s="222" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="219" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="B44" s="213" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="C44" s="217" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D44" s="213" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E44" s="220" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="221" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="B45" s="206" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="C45" s="217" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="D45" s="206" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E45" s="222" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="241" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="B46" s="226" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="C46" s="232" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D46" s="226" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E46" s="242" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="243" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="B47" s="233" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C47" s="237" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D47" s="233" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E47" s="244" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="241" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="B48" s="226" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="C48" s="237" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D48" s="226" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E48" s="242" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="B49" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C49" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D49" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E49" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="B50" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C50" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D50" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E50" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="B51" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C51" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D51" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E51" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="B52" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="C52" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="D52" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E52" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
+        <v>639</v>
+      </c>
+      <c r="B53" t="s">
+        <v>540</v>
+      </c>
+      <c r="C53" t="s">
         <v>637</v>
       </c>
-      <c r="B53" t="s">
-        <v>538</v>
-      </c>
-      <c r="C53" t="s">
-        <v>635</v>
-      </c>
       <c r="D53" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E53" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="250" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="B54" s="250" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="C54" s="250" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="D54" s="250" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E54" s="250" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="250" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="B55" s="250" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C55" s="250" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D55" s="250" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E55" s="250" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="250" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="B56" s="250" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C56" s="250" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D56" s="250" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E56" s="250" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="250" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="B57" s="250" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C57" s="250" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D57" s="250" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E57" s="250" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="250" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="B58" s="250" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C58" s="250" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D58" s="250" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E58" s="250" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="250" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B59" s="250" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C59" s="250" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D59" s="250" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E59" s="250" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="250" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="B60" s="250" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C60" s="250" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D60" s="250" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E60" s="250" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="250" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="B61" s="250" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C61" s="250" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D61" s="250" t="s">
+        <v>528</v>
+      </c>
+      <c r="E61" s="250" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A62" s="250" t="s">
+        <v>657</v>
+      </c>
+      <c r="B62" s="250" t="s">
         <v>526</v>
       </c>
-      <c r="E61" s="250" t="s">
-        <v>654</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" ht="72" x14ac:dyDescent="0.55000000000000004">
-      <c r="A62" s="250" t="s">
-        <v>655</v>
-      </c>
-      <c r="B62" s="250" t="s">
-        <v>524</v>
-      </c>
       <c r="C62" s="250" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D62" s="250" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E62" s="250" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
     </row>
   </sheetData>
@@ -13750,336 +13786,336 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="246" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="247" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="248" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="B4" s="248" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="C4" s="248" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="D4" s="248" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="E4" s="248" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="F4" s="248" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="G4" s="248" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="H4" s="248" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="248" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="249" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B5" s="250" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="C5" s="250" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="D5" s="250" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="E5" s="250" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="F5" s="250" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="G5" s="250" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="H5" s="251" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="I5" s="250" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="249" t="s">
+        <v>678</v>
+      </c>
+      <c r="B6" s="250" t="s">
+        <v>679</v>
+      </c>
+      <c r="C6" s="250" t="s">
+        <v>680</v>
+      </c>
+      <c r="D6" s="250" t="s">
+        <v>681</v>
+      </c>
+      <c r="E6" s="250" t="s">
+        <v>682</v>
+      </c>
+      <c r="F6" s="250" t="s">
+        <v>683</v>
+      </c>
+      <c r="G6" s="250" t="s">
+        <v>684</v>
+      </c>
+      <c r="H6" s="252" t="s">
         <v>676</v>
       </c>
-      <c r="B6" s="250" t="s">
-        <v>677</v>
-      </c>
-      <c r="C6" s="250" t="s">
-        <v>678</v>
-      </c>
-      <c r="D6" s="250" t="s">
-        <v>679</v>
-      </c>
-      <c r="E6" s="250" t="s">
-        <v>680</v>
-      </c>
-      <c r="F6" s="250" t="s">
-        <v>681</v>
-      </c>
-      <c r="G6" s="250" t="s">
-        <v>682</v>
-      </c>
-      <c r="H6" s="252" t="s">
-        <v>674</v>
-      </c>
       <c r="I6" s="250" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="249" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="B7" s="250" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="C7" s="250" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="D7" s="250" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="E7" s="250" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="F7" s="250" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="G7" s="250" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="H7" s="252" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="I7" s="250" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="249" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="B8" s="250" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="C8" s="250" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="D8" s="250" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="E8" s="250" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="F8" s="250" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="G8" s="250" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="H8" s="251" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="I8" s="250" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="249" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="B9" s="250" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="C9" s="250" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="D9" s="250" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="E9" s="250" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="F9" s="250" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="G9" s="250" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="H9" s="253" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="I9" s="250" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="249" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="B10" s="250" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="C10" s="250" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="D10" s="250" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="E10" s="250" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="F10" s="250" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="G10" s="250" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="H10" s="253" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="I10" s="250" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="249" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="B11" s="250" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="C11" s="250" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="D11" s="250" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="E11" s="250" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="F11" s="250" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="G11" s="250" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="H11" s="253" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="I11" s="250" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="249" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="B12" s="250" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="C12" s="250" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="D12" s="250" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="E12" s="250" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="F12" s="250" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="G12" s="250" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="H12" s="252" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="I12" s="250" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="249" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="B13" s="250" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="C13" s="250" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="D13" s="250" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="E13" s="250" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="F13" s="250" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="G13" s="250" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="H13" s="253" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="I13" s="250" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="249" t="s">
+        <v>734</v>
+      </c>
+      <c r="B14" s="250" t="s">
+        <v>735</v>
+      </c>
+      <c r="C14" s="250" t="s">
+        <v>731</v>
+      </c>
+      <c r="D14" s="250" t="s">
+        <v>637</v>
+      </c>
+      <c r="E14" s="250" t="s">
+        <v>637</v>
+      </c>
+      <c r="F14" s="250" t="s">
+        <v>637</v>
+      </c>
+      <c r="G14" s="250" t="s">
+        <v>637</v>
+      </c>
+      <c r="H14" s="253" t="s">
         <v>732</v>
       </c>
-      <c r="B14" s="250" t="s">
-        <v>733</v>
-      </c>
-      <c r="C14" s="250" t="s">
-        <v>729</v>
-      </c>
-      <c r="D14" s="250" t="s">
-        <v>635</v>
-      </c>
-      <c r="E14" s="250" t="s">
-        <v>635</v>
-      </c>
-      <c r="F14" s="250" t="s">
-        <v>635</v>
-      </c>
-      <c r="G14" s="250" t="s">
-        <v>635</v>
-      </c>
-      <c r="H14" s="253" t="s">
-        <v>730</v>
-      </c>
       <c r="I14" s="250" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="282" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="B16" s="262"/>
       <c r="C16" s="262"/>

</xml_diff>

<commit_message>
docs(tracker): key-player re-measurement, Polymarket decision, push receipts
Board now 201 items / 155 done, Unassigned=0.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B251458B-C48E-46EE-8879-D9EE85A04808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{310DEA81-B110-4867-9317-079474B2EC19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1482" uniqueCount="738">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1509" uniqueCount="748">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -1200,7 +1200,7 @@
     <t>Check Expo push RECEIPTS, not just tickets</t>
   </si>
   <si>
-    <t>_send_push discards the ticket id, so DeviceNotRegistered / bad FCM credential are invisible today. Fix before real users</t>
+    <t>DONE (920e897). push_tickets table + a 30-min worker. A ticket only means ACCEPTED; the receipt is the only place DeviceNotRegistered, MessageTooBig and above all InvalidCredentials appear - the last fails EVERY send for EVERY user while every ticket reports success. Checked rows are deleted (work queue, not history); a lookup FAILURE leaves them for the next run, since a failed lookup is not a failed delivery</t>
   </si>
   <si>
     <t>Purge 141 fake push tokens from the dev DB</t>
@@ -1360,6 +1360,24 @@
   </si>
   <si>
     <t>Planned to DELETE the per-test teardown as redundant; reading it, that would have been a downgrade - it also keeps tests independent of each other, which the dedicated database does not address. Stale justifications corrected instead. The real gap was tests with NO teardown: users grew 21 per run indefinitely. conftest now truncates once per session, at the START so a failed run's rows stay inspectable. Verified 21 after both run 1 and run 2. ada6b50</t>
+  </si>
+  <si>
+    <t>Key-player features re-measured, then deleted</t>
+  </si>
+  <si>
+    <t>Re-added all four and retrained on IDENTICAL splits (so the comparison is exact) rather than trusting d0a24d9's verdict, which was reached on a nine-league pool that has since doubled to eighteen with half of it lacking lineups. Result reproduced the original: accuracy 0.4857 -&gt; 0.4870 (+0.13pp, ~7 of 5,487 = noise), RPS 0.2144 -&gt; 0.2151 worse, corners MAE 2.160 -&gt; 2.166 worse, under-3.5 trend z +5.92 -&gt; +4.07 MATERIALLY worse. Bottom reliability bucket rose .604 -&gt; .655 while the top barely moved, i.e. LESS discrimination with the features. Training-time computation and lineup loading deleted; Stage 1 kept for live Stage 2 + mobile. 18-feature model repromoted. 0a62c9f</t>
+  </si>
+  <si>
+    <t>DECIDED: do not exclude Polymarket at ingest</t>
+  </si>
+  <si>
+    <t>The existing consensus test already catches 204 of Polymarket's 228 real tennis rows (89%) and is bookmaker-agnostic. A name-based blocklist would be strictly worse: HardRock inverts 20% of its own rows (42 of 209) and a Polymarket blocklist misses those entirely</t>
+  </si>
+  <si>
+    <t>Implausible prices no longer win best-odds selection</t>
+  </si>
+  <si>
+    <t>Found while investigating Polymarket. A row can be the right way round and still absurd: HardRock supplied 151.00 against a 1.97 median, 76.00 against 2.07, 61.00 against 2.90 - 25 of 100 fixture-sides had a max &gt;=15% above median. The inversion test passes them and MAX selection then picks them. Training has filtered this since an inflated ROI traced to the same rows; serving never did. Latent rather than live - MAX_EDGE_OVER_MARKET happens to reject the pick - but that drops a fixture's pick entirely rather than repricing it. 5e32146</t>
   </si>
   <si>
     <t>Legend</t>
@@ -2086,6 +2104,18 @@
   </si>
   <si>
     <t>Hit twice on 2026-08-10: a LEAGUE_IDS change the worker never loaded (no odds for 9 leagues), then a no-draw guard the worker never loaded (deleted rows recreated every 5 minutes). Neither raised an error; both looked like the fix not working. Restart worker and beat after any change under app/, and check process start time against file mtime before believing live data</t>
+  </si>
+  <si>
+    <t>Bookmaker names differ only by case</t>
+  </si>
+  <si>
+    <t>draftkings/Draftkings and fanduel/Fanduel are stored as separate books, so one book's price counts twice in the consensus median that decides which rows are inverted. Not currently changing any verdict, but it weights the median wrongly</t>
+  </si>
+  <si>
+    <t>watchlist_items.created_at model/DB drift</t>
+  </si>
+  <si>
+    <t>Autogenerate wants NOT NULL; the database has it nullable. Stripped from the push-receipts migration rather than smuggled in. Needs its own migration</t>
   </si>
   <si>
     <t>External APIs, Quotas &amp; Expiry</t>
@@ -4529,7 +4559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R204"/>
+  <dimension ref="A1:R207"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -10413,7 +10443,7 @@
         <v>342</v>
       </c>
       <c r="R166" t="str">
-        <f t="shared" ref="R166:R202" si="5">IF($A166&lt;&gt;"",$A166,R165)</f>
+        <f t="shared" ref="R166:R197" si="5">IF($A166&lt;&gt;"",$A166,R165)</f>
         <v>E9 Data Ops</v>
       </c>
     </row>
@@ -10633,7 +10663,7 @@
         <v>E9 Data Ops</v>
       </c>
     </row>
-    <row r="176" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+    <row r="176" spans="1:18" ht="100.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A176" t="s">
         <v>162</v>
       </c>
@@ -10641,7 +10671,7 @@
         <v>386</v>
       </c>
       <c r="C176" t="s">
-        <v>128</v>
+        <v>22</v>
       </c>
       <c r="D176" t="s">
         <v>75</v>
@@ -10649,7 +10679,10 @@
       <c r="E176" s="245">
         <v>46243</v>
       </c>
-      <c r="G176" t="s">
+      <c r="F176" s="245">
+        <v>46244</v>
+      </c>
+      <c r="G176" s="250" t="s">
         <v>387</v>
       </c>
       <c r="R176" t="str">
@@ -10705,7 +10738,7 @@
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="179" spans="1:18" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="179" spans="1:18" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A179" t="s">
         <v>191</v>
       </c>
@@ -11274,7 +11307,7 @@
         <v>432</v>
       </c>
       <c r="R198" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="R198:R205" si="6">IF($A198&lt;&gt;"",$A198,R197)</f>
         <v>E4 ML Football</v>
       </c>
     </row>
@@ -11304,7 +11337,7 @@
         <v>400</v>
       </c>
       <c r="R199" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>E5 ML Tennis</v>
       </c>
     </row>
@@ -11334,7 +11367,7 @@
         <v>400</v>
       </c>
       <c r="R200" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>E9 Data Ops</v>
       </c>
     </row>
@@ -11364,11 +11397,11 @@
         <v>400</v>
       </c>
       <c r="R201" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="202" spans="1:18" ht="100.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="202" spans="1:18" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B202" t="s">
         <v>439</v>
       </c>
@@ -11391,27 +11424,114 @@
         <v>400</v>
       </c>
       <c r="R202" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="204" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A204" s="25" t="s">
+    <row r="203" spans="1:18" ht="144" x14ac:dyDescent="0.55000000000000004">
+      <c r="A203" t="s">
+        <v>99</v>
+      </c>
+      <c r="B203" t="s">
         <v>441</v>
       </c>
-      <c r="B204" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C204" s="17" t="s">
+      <c r="C203" t="s">
+        <v>22</v>
+      </c>
+      <c r="D203" t="s">
+        <v>45</v>
+      </c>
+      <c r="E203" s="245">
+        <v>46244</v>
+      </c>
+      <c r="F203" s="245">
+        <v>46244</v>
+      </c>
+      <c r="G203" s="250" t="s">
         <v>442</v>
       </c>
-      <c r="D204" s="19" t="s">
+      <c r="J203" t="s">
+        <v>400</v>
+      </c>
+      <c r="R203" t="str">
+        <f t="shared" si="6"/>
+        <v>E8 Model Quality</v>
+      </c>
+    </row>
+    <row r="204" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A204" t="s">
+        <v>73</v>
+      </c>
+      <c r="B204" t="s">
+        <v>443</v>
+      </c>
+      <c r="C204" t="s">
+        <v>22</v>
+      </c>
+      <c r="D204" t="s">
+        <v>75</v>
+      </c>
+      <c r="E204" s="245">
+        <v>46244</v>
+      </c>
+      <c r="F204" s="245">
+        <v>46244</v>
+      </c>
+      <c r="G204" s="250" t="s">
+        <v>444</v>
+      </c>
+      <c r="J204" t="s">
+        <v>400</v>
+      </c>
+      <c r="R204" t="str">
+        <f t="shared" si="6"/>
+        <v>E6 Picks</v>
+      </c>
+    </row>
+    <row r="205" spans="1:18" ht="115.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="B205" t="s">
+        <v>445</v>
+      </c>
+      <c r="C205" t="s">
+        <v>22</v>
+      </c>
+      <c r="D205" t="s">
+        <v>75</v>
+      </c>
+      <c r="E205" s="245">
+        <v>46244</v>
+      </c>
+      <c r="F205" s="245">
+        <v>46244</v>
+      </c>
+      <c r="G205" s="250" t="s">
+        <v>446</v>
+      </c>
+      <c r="J205" t="s">
+        <v>400</v>
+      </c>
+      <c r="R205" t="str">
+        <f t="shared" si="6"/>
+        <v>E6 Picks</v>
+      </c>
+    </row>
+    <row r="207" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A207" s="25" t="s">
+        <v>447</v>
+      </c>
+      <c r="B207" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C207" s="17" t="s">
+        <v>448</v>
+      </c>
+      <c r="D207" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="E204" s="23" t="s">
+      <c r="E207" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="F204" s="21" t="s">
+      <c r="F207" s="21" t="s">
         <v>138</v>
       </c>
     </row>
@@ -11436,7 +11556,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="273" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="B1" s="262"/>
       <c r="C1" s="262"/>
@@ -11459,7 +11579,7 @@
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="280" t="s">
-        <v>444</v>
+        <v>450</v>
       </c>
       <c r="B2" s="262"/>
       <c r="C2" s="262"/>
@@ -11482,7 +11602,7 @@
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="268" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="B4" s="262"/>
       <c r="C4" s="262"/>
@@ -11505,42 +11625,42 @@
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="37" t="s">
-        <v>446</v>
+        <v>452</v>
       </c>
       <c r="B5" s="258" t="s">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="C5" s="259"/>
       <c r="D5" s="260"/>
       <c r="E5" s="263" t="s">
-        <v>448</v>
+        <v>454</v>
       </c>
       <c r="F5" s="259"/>
       <c r="G5" s="260"/>
       <c r="H5" s="263" t="s">
-        <v>449</v>
+        <v>455</v>
       </c>
       <c r="I5" s="259"/>
       <c r="J5" s="260"/>
       <c r="K5" s="258" t="s">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="L5" s="259"/>
       <c r="M5" s="260"/>
       <c r="N5" s="265" t="s">
-        <v>451</v>
+        <v>457</v>
       </c>
       <c r="O5" s="259"/>
       <c r="P5" s="260"/>
       <c r="Q5" s="265" t="s">
-        <v>452</v>
+        <v>458</v>
       </c>
       <c r="R5" s="259"/>
       <c r="S5" s="260"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="261" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="C6" s="262"/>
       <c r="D6" s="262"/>
@@ -11562,7 +11682,7 @@
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="268" t="s">
-        <v>454</v>
+        <v>460</v>
       </c>
       <c r="B7" s="262"/>
       <c r="C7" s="262"/>
@@ -11585,10 +11705,10 @@
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="37" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="B8" s="271" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="C8" s="259"/>
       <c r="D8" s="259"/>
@@ -11599,7 +11719,7 @@
       <c r="I8" s="259"/>
       <c r="J8" s="260"/>
       <c r="K8" s="271" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
       <c r="L8" s="259"/>
       <c r="M8" s="259"/>
@@ -11612,7 +11732,7 @@
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="261" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="C9" s="262"/>
       <c r="D9" s="262"/>
@@ -11634,7 +11754,7 @@
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="268" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
       <c r="B10" s="262"/>
       <c r="C10" s="262"/>
@@ -11657,42 +11777,42 @@
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="37" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="B11" s="258" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="C11" s="259"/>
       <c r="D11" s="260"/>
       <c r="E11" s="258" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="F11" s="259"/>
       <c r="G11" s="260"/>
       <c r="H11" s="258" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="I11" s="259"/>
       <c r="J11" s="260"/>
       <c r="K11" s="263" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="L11" s="259"/>
       <c r="M11" s="260"/>
       <c r="N11" s="258" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
       <c r="O11" s="259"/>
       <c r="P11" s="260"/>
       <c r="Q11" s="258" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="R11" s="259"/>
       <c r="S11" s="260"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="261" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="C12" s="262"/>
       <c r="D12" s="262"/>
@@ -11714,7 +11834,7 @@
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="268" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="B13" s="262"/>
       <c r="C13" s="262"/>
@@ -11737,10 +11857,10 @@
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="37" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
       <c r="B14" s="266" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="C14" s="259"/>
       <c r="D14" s="259"/>
@@ -11748,7 +11868,7 @@
       <c r="F14" s="259"/>
       <c r="G14" s="260"/>
       <c r="H14" s="266" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="I14" s="259"/>
       <c r="J14" s="259"/>
@@ -11756,19 +11876,19 @@
       <c r="L14" s="259"/>
       <c r="M14" s="260"/>
       <c r="N14" s="266" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
       <c r="O14" s="259"/>
       <c r="P14" s="260"/>
       <c r="Q14" s="263" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="R14" s="259"/>
       <c r="S14" s="260"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" s="261" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="C15" s="262"/>
       <c r="D15" s="262"/>
@@ -11790,7 +11910,7 @@
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="268" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
       <c r="B16" s="262"/>
       <c r="C16" s="262"/>
@@ -11813,10 +11933,10 @@
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="37" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
       <c r="B17" s="267" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="C17" s="259"/>
       <c r="D17" s="259"/>
@@ -11824,29 +11944,29 @@
       <c r="F17" s="259"/>
       <c r="G17" s="260"/>
       <c r="H17" s="267" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
       <c r="I17" s="259"/>
       <c r="J17" s="260"/>
       <c r="K17" s="267" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="L17" s="259"/>
       <c r="M17" s="260"/>
       <c r="N17" s="267" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
       <c r="O17" s="259"/>
       <c r="P17" s="260"/>
       <c r="Q17" s="267" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
       <c r="R17" s="259"/>
       <c r="S17" s="260"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="261" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="C18" s="262"/>
       <c r="D18" s="262"/>
@@ -11868,7 +11988,7 @@
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="268" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="B19" s="262"/>
       <c r="C19" s="262"/>
@@ -11891,10 +12011,10 @@
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="37" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
       <c r="B20" s="269" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
       <c r="C20" s="259"/>
       <c r="D20" s="259"/>
@@ -11902,7 +12022,7 @@
       <c r="F20" s="259"/>
       <c r="G20" s="260"/>
       <c r="H20" s="269" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
       <c r="I20" s="259"/>
       <c r="J20" s="259"/>
@@ -11910,7 +12030,7 @@
       <c r="L20" s="259"/>
       <c r="M20" s="260"/>
       <c r="N20" s="269" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
       <c r="O20" s="259"/>
       <c r="P20" s="259"/>
@@ -11920,7 +12040,7 @@
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" s="261" t="s">
-        <v>453</v>
+        <v>459</v>
       </c>
       <c r="C21" s="262"/>
       <c r="D21" s="262"/>
@@ -11942,7 +12062,7 @@
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="268" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="B22" s="262"/>
       <c r="C22" s="262"/>
@@ -11965,10 +12085,10 @@
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="37" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="B23" s="269" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="C23" s="259"/>
       <c r="D23" s="259"/>
@@ -11976,29 +12096,29 @@
       <c r="F23" s="259"/>
       <c r="G23" s="260"/>
       <c r="H23" s="269" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
       <c r="I23" s="259"/>
       <c r="J23" s="260"/>
       <c r="K23" s="269" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
       <c r="L23" s="259"/>
       <c r="M23" s="260"/>
       <c r="N23" s="269" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
       <c r="O23" s="259"/>
       <c r="P23" s="260"/>
       <c r="Q23" s="265" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="R23" s="259"/>
       <c r="S23" s="260"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="274" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="B26" s="262"/>
       <c r="C26" s="262"/>
@@ -12021,42 +12141,42 @@
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="37" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="B27" s="258" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="C27" s="259"/>
       <c r="D27" s="260"/>
       <c r="E27" s="258" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="F27" s="259"/>
       <c r="G27" s="260"/>
       <c r="H27" s="266" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
       <c r="I27" s="259"/>
       <c r="J27" s="260"/>
       <c r="K27" s="267" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="L27" s="259"/>
       <c r="M27" s="260"/>
       <c r="N27" s="267" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
       <c r="O27" s="259"/>
       <c r="P27" s="260"/>
       <c r="Q27" s="266" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="R27" s="259"/>
       <c r="S27" s="260"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="268" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
       <c r="B30" s="262"/>
       <c r="C30" s="262"/>
@@ -12079,7 +12199,7 @@
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="264" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="B31" s="262"/>
       <c r="C31" s="262"/>
@@ -12102,7 +12222,7 @@
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="264" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="B32" s="262"/>
       <c r="C32" s="262"/>
@@ -12125,7 +12245,7 @@
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="264" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B33" s="262"/>
       <c r="C33" s="262"/>
@@ -12148,7 +12268,7 @@
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="264" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="B34" s="262"/>
       <c r="C34" s="262"/>
@@ -12171,7 +12291,7 @@
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="264" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
       <c r="B35" s="262"/>
       <c r="C35" s="262"/>
@@ -12194,7 +12314,7 @@
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="264" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="B36" s="262"/>
       <c r="C36" s="262"/>
@@ -12217,7 +12337,7 @@
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="275" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="B37" s="262"/>
       <c r="C37" s="262"/>
@@ -12240,25 +12360,25 @@
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="38" t="s">
-        <v>441</v>
+        <v>447</v>
       </c>
       <c r="B39" s="278" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="C39" s="262"/>
       <c r="D39" s="262"/>
       <c r="E39" s="276" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="F39" s="262"/>
       <c r="G39" s="262"/>
       <c r="H39" s="279" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="I39" s="262"/>
       <c r="J39" s="262"/>
       <c r="K39" s="272" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="L39" s="262"/>
       <c r="M39" s="262"/>
@@ -12268,7 +12388,7 @@
       <c r="O39" s="262"/>
       <c r="P39" s="262"/>
       <c r="Q39" s="277" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="R39" s="262"/>
       <c r="S39" s="262"/>
@@ -12276,11 +12396,11 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H14:M14"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A16:S16"/>
     <mergeCell ref="H20:M20"/>
-    <mergeCell ref="A16:S16"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -12289,13 +12409,14 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -12304,7 +12425,6 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
-    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -12312,7 +12432,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -12361,7 +12481,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="281" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
       <c r="B1" s="255"/>
       <c r="C1" s="255"/>
@@ -12374,19 +12494,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -12520,11 +12640,11 @@
       </c>
       <c r="B9" s="26">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C9" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D9" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -12536,7 +12656,7 @@
       </c>
       <c r="F9" s="27">
         <f t="shared" si="1"/>
-        <v>0.8</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -12570,11 +12690,11 @@
       </c>
       <c r="B11" s="26">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D11" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -12586,7 +12706,7 @@
       </c>
       <c r="F11" s="27">
         <f t="shared" si="1"/>
-        <v>0.8</v>
+        <v>0.80487804878048785</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -12624,11 +12744,11 @@
       </c>
       <c r="C13" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D13" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E13" s="26">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A13,'Delivery Board'!$C$5:$C$500,"Blocked")</f>
@@ -12636,7 +12756,7 @@
       </c>
       <c r="F13" s="27">
         <f t="shared" si="1"/>
-        <v>0.6875</v>
+        <v>0.71875</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -12666,19 +12786,19 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="28" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="B16" s="29">
         <f>SUM(B4:B14)</f>
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C16" s="29">
         <f>SUM(C4:C14)</f>
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E16">
         <f>SUM(E4:E14)</f>
@@ -12686,12 +12806,12 @@
       </c>
       <c r="F16" s="30">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.76262626262626265</v>
+        <v>0.77114427860696522</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="43" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="B18" s="44">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -12700,7 +12820,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="45" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
     </row>
   </sheetData>
@@ -12721,7 +12841,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -12733,7 +12853,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="281" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="B1" s="255"/>
       <c r="C1" s="255"/>
@@ -12742,648 +12862,648 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="31" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="D3" s="31" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="32" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="34" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="32" t="s">
+        <v>539</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>540</v>
+      </c>
+      <c r="C6" s="23" t="s">
         <v>533</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>534</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>527</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="34" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="32" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="34" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="32" t="s">
+        <v>551</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>552</v>
+      </c>
+      <c r="C10" s="19" t="s">
         <v>545</v>
       </c>
-      <c r="B10" s="12" t="s">
-        <v>546</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>539</v>
-      </c>
       <c r="D10" s="12" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="34" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="32" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="34" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="32" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="34" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="32" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="34" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="32" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="34" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="32" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="34" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="32" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E22" s="33" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="34" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E23" s="35" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="32" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="58" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
       <c r="B25" s="55" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="C25" s="59" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D25" s="55" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E25" s="60" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="61" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="B26" s="49" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="C26" s="59" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="D26" s="49" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E26" s="62" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="58" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
       <c r="B27" s="55" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="C27" s="59" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="D27" s="55" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E27" s="60" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="79" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="B28" s="66" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="C28" s="75" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D28" s="107" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E28" s="107" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="80" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
       <c r="B29" s="72" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C29" s="77" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D29" s="106" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E29" s="106" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="88" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
       <c r="B30" s="84" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C30" s="89" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D30" s="84" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E30" s="90" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="105" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
       <c r="B31" s="94" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="C31" s="103" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D31" s="94" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
       <c r="E31" s="106" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="122" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="B32" s="117" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="C32" s="120" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D32" s="117" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E32" s="123" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="124" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="B33" s="111" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C33" s="120" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D33" s="111" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="E33" s="125" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="156" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="B34" s="150" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="C34" s="142" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D34" s="150" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E34" s="157" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="158" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="B35" s="143" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C35" s="154" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D35" s="143" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E35" s="159" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="74.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="172" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="B36" s="169" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C36" s="173" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="D36" s="178" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
       <c r="E36" s="178" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="175" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="B37" s="163" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="C37" s="176" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D37" s="163" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E37" s="177" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="172" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="B38" s="169" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="C38" s="176" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="D38" s="169" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E38" s="174" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="186" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
       <c r="B39" s="182" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C39" s="187" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D39" s="182" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E39" s="188" t="s">
-        <v>612</v>
+        <v>618</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="196" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
       <c r="B40" s="192" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="C40" s="197" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D40" s="192" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E40" s="198" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -13391,373 +13511,407 @@
         <v>140</v>
       </c>
       <c r="B41" s="200" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="C41" s="201" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D41" s="200" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E41" s="202" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="219" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
       <c r="B42" s="213" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="C42" s="205" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D42" s="213" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E42" s="220" t="s">
-        <v>617</v>
+        <v>623</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="221" t="s">
-        <v>618</v>
+        <v>624</v>
       </c>
       <c r="B43" s="206" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C43" s="217" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D43" s="206" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="E43" s="222" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="219" t="s">
-        <v>620</v>
+        <v>626</v>
       </c>
       <c r="B44" s="213" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="C44" s="217" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D44" s="213" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E44" s="220" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="221" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
       <c r="B45" s="206" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="C45" s="217" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="D45" s="206" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E45" s="222" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="241" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
       <c r="B46" s="226" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="C46" s="232" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D46" s="226" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E46" s="242" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="243" t="s">
-        <v>626</v>
+        <v>632</v>
       </c>
       <c r="B47" s="233" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C47" s="237" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D47" s="233" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E47" s="244" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="241" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
       <c r="B48" s="226" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="C48" s="237" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D48" s="226" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E48" s="242" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
       <c r="B49" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C49" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D49" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E49" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
       <c r="B50" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C50" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D50" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E50" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
       <c r="B51" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C51" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D51" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E51" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
       <c r="B52" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="C52" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="D52" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E52" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
       <c r="B53" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="C53" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="D53" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E53" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="250" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
       <c r="B54" s="250" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="C54" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="D54" s="250" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E54" s="250" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="250" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="B55" s="250" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C55" s="250" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D55" s="250" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E55" s="250" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="250" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
       <c r="B56" s="250" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C56" s="250" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D56" s="250" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E56" s="250" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="250" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="B57" s="250" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C57" s="250" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D57" s="250" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E57" s="250" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="250" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="B58" s="250" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C58" s="250" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D58" s="250" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E58" s="250" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="250" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
       <c r="B59" s="250" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C59" s="250" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D59" s="250" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E59" s="250" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="250" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
       <c r="B60" s="250" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C60" s="250" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D60" s="250" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E60" s="250" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="250" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="B61" s="250" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C61" s="250" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D61" s="250" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E61" s="250" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="250" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="B62" s="250" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C62" s="250" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D62" s="250" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E62" s="250" t="s">
-        <v>658</v>
+        <v>664</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A63" s="250" t="s">
+        <v>665</v>
+      </c>
+      <c r="B63" s="250" t="s">
+        <v>532</v>
+      </c>
+      <c r="C63" s="250" t="s">
+        <v>557</v>
+      </c>
+      <c r="D63" s="250" t="s">
+        <v>534</v>
+      </c>
+      <c r="E63" s="250" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A64" s="250" t="s">
+        <v>667</v>
+      </c>
+      <c r="B64" s="250" t="s">
+        <v>532</v>
+      </c>
+      <c r="C64" s="250" t="s">
+        <v>557</v>
+      </c>
+      <c r="D64" s="250" t="s">
+        <v>534</v>
+      </c>
+      <c r="E64" s="250" t="s">
+        <v>668</v>
       </c>
     </row>
   </sheetData>
@@ -13786,336 +13940,336 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="246" t="s">
-        <v>659</v>
+        <v>669</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="247" t="s">
-        <v>660</v>
+        <v>670</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="248" t="s">
-        <v>661</v>
+        <v>671</v>
       </c>
       <c r="B4" s="248" t="s">
-        <v>662</v>
+        <v>672</v>
       </c>
       <c r="C4" s="248" t="s">
-        <v>663</v>
+        <v>673</v>
       </c>
       <c r="D4" s="248" t="s">
-        <v>664</v>
+        <v>674</v>
       </c>
       <c r="E4" s="248" t="s">
-        <v>665</v>
+        <v>675</v>
       </c>
       <c r="F4" s="248" t="s">
-        <v>666</v>
+        <v>676</v>
       </c>
       <c r="G4" s="248" t="s">
-        <v>667</v>
+        <v>677</v>
       </c>
       <c r="H4" s="248" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="248" t="s">
-        <v>668</v>
+        <v>678</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="249" t="s">
-        <v>669</v>
+        <v>679</v>
       </c>
       <c r="B5" s="250" t="s">
-        <v>670</v>
+        <v>680</v>
       </c>
       <c r="C5" s="250" t="s">
-        <v>671</v>
+        <v>681</v>
       </c>
       <c r="D5" s="250" t="s">
-        <v>672</v>
+        <v>682</v>
       </c>
       <c r="E5" s="250" t="s">
-        <v>673</v>
+        <v>683</v>
       </c>
       <c r="F5" s="250" t="s">
-        <v>674</v>
+        <v>684</v>
       </c>
       <c r="G5" s="250" t="s">
-        <v>675</v>
+        <v>685</v>
       </c>
       <c r="H5" s="251" t="s">
-        <v>676</v>
+        <v>686</v>
       </c>
       <c r="I5" s="250" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="249" t="s">
-        <v>678</v>
+        <v>688</v>
       </c>
       <c r="B6" s="250" t="s">
-        <v>679</v>
+        <v>689</v>
       </c>
       <c r="C6" s="250" t="s">
-        <v>680</v>
+        <v>690</v>
       </c>
       <c r="D6" s="250" t="s">
-        <v>681</v>
+        <v>691</v>
       </c>
       <c r="E6" s="250" t="s">
-        <v>682</v>
+        <v>692</v>
       </c>
       <c r="F6" s="250" t="s">
-        <v>683</v>
+        <v>693</v>
       </c>
       <c r="G6" s="250" t="s">
-        <v>684</v>
+        <v>694</v>
       </c>
       <c r="H6" s="252" t="s">
-        <v>676</v>
+        <v>686</v>
       </c>
       <c r="I6" s="250" t="s">
-        <v>685</v>
+        <v>695</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="249" t="s">
+        <v>696</v>
+      </c>
+      <c r="B7" s="250" t="s">
+        <v>697</v>
+      </c>
+      <c r="C7" s="250" t="s">
+        <v>698</v>
+      </c>
+      <c r="D7" s="250" t="s">
+        <v>699</v>
+      </c>
+      <c r="E7" s="250" t="s">
+        <v>700</v>
+      </c>
+      <c r="F7" s="250" t="s">
+        <v>701</v>
+      </c>
+      <c r="G7" s="250" t="s">
+        <v>702</v>
+      </c>
+      <c r="H7" s="252" t="s">
         <v>686</v>
       </c>
-      <c r="B7" s="250" t="s">
-        <v>687</v>
-      </c>
-      <c r="C7" s="250" t="s">
-        <v>688</v>
-      </c>
-      <c r="D7" s="250" t="s">
-        <v>689</v>
-      </c>
-      <c r="E7" s="250" t="s">
-        <v>690</v>
-      </c>
-      <c r="F7" s="250" t="s">
-        <v>691</v>
-      </c>
-      <c r="G7" s="250" t="s">
-        <v>692</v>
-      </c>
-      <c r="H7" s="252" t="s">
-        <v>676</v>
-      </c>
       <c r="I7" s="250" t="s">
-        <v>693</v>
+        <v>703</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="249" t="s">
-        <v>694</v>
+        <v>704</v>
       </c>
       <c r="B8" s="250" t="s">
-        <v>695</v>
+        <v>705</v>
       </c>
       <c r="C8" s="250" t="s">
-        <v>696</v>
+        <v>706</v>
       </c>
       <c r="D8" s="250" t="s">
-        <v>697</v>
+        <v>707</v>
       </c>
       <c r="E8" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="F8" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="G8" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="H8" s="251" t="s">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="I8" s="250" t="s">
-        <v>699</v>
+        <v>709</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="249" t="s">
+        <v>710</v>
+      </c>
+      <c r="B9" s="250" t="s">
+        <v>711</v>
+      </c>
+      <c r="C9" s="250" t="s">
+        <v>712</v>
+      </c>
+      <c r="D9" s="250" t="s">
+        <v>707</v>
+      </c>
+      <c r="E9" s="250" t="s">
         <v>700</v>
       </c>
-      <c r="B9" s="250" t="s">
-        <v>701</v>
-      </c>
-      <c r="C9" s="250" t="s">
-        <v>702</v>
-      </c>
-      <c r="D9" s="250" t="s">
-        <v>697</v>
-      </c>
-      <c r="E9" s="250" t="s">
-        <v>690</v>
-      </c>
       <c r="F9" s="250" t="s">
-        <v>703</v>
+        <v>713</v>
       </c>
       <c r="G9" s="250" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="H9" s="253" t="s">
-        <v>705</v>
+        <v>715</v>
       </c>
       <c r="I9" s="250" t="s">
-        <v>706</v>
+        <v>716</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="249" t="s">
-        <v>707</v>
+        <v>717</v>
       </c>
       <c r="B10" s="250" t="s">
-        <v>708</v>
+        <v>718</v>
       </c>
       <c r="C10" s="250" t="s">
-        <v>709</v>
+        <v>719</v>
       </c>
       <c r="D10" s="250" t="s">
-        <v>710</v>
+        <v>720</v>
       </c>
       <c r="E10" s="250" t="s">
-        <v>711</v>
+        <v>721</v>
       </c>
       <c r="F10" s="250" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="G10" s="250" t="s">
-        <v>713</v>
+        <v>723</v>
       </c>
       <c r="H10" s="253" t="s">
-        <v>714</v>
+        <v>724</v>
       </c>
       <c r="I10" s="250" t="s">
-        <v>715</v>
+        <v>725</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="249" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="B11" s="250" t="s">
-        <v>717</v>
+        <v>727</v>
       </c>
       <c r="C11" s="250" t="s">
-        <v>718</v>
+        <v>728</v>
       </c>
       <c r="D11" s="250" t="s">
-        <v>719</v>
+        <v>729</v>
       </c>
       <c r="E11" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="F11" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="G11" s="250" t="s">
-        <v>720</v>
+        <v>730</v>
       </c>
       <c r="H11" s="253" t="s">
-        <v>721</v>
+        <v>731</v>
       </c>
       <c r="I11" s="250" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="249" t="s">
-        <v>723</v>
+        <v>733</v>
       </c>
       <c r="B12" s="250" t="s">
-        <v>724</v>
+        <v>734</v>
       </c>
       <c r="C12" s="250" t="s">
-        <v>725</v>
+        <v>735</v>
       </c>
       <c r="D12" s="250" t="s">
-        <v>726</v>
+        <v>736</v>
       </c>
       <c r="E12" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="F12" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="G12" s="250" t="s">
-        <v>720</v>
+        <v>730</v>
       </c>
       <c r="H12" s="252" t="s">
-        <v>727</v>
+        <v>737</v>
       </c>
       <c r="I12" s="250" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="249" t="s">
-        <v>729</v>
+        <v>739</v>
       </c>
       <c r="B13" s="250" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="C13" s="250" t="s">
-        <v>731</v>
+        <v>741</v>
       </c>
       <c r="D13" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="E13" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="F13" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="G13" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="H13" s="253" t="s">
-        <v>732</v>
+        <v>742</v>
       </c>
       <c r="I13" s="250" t="s">
-        <v>733</v>
+        <v>743</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="249" t="s">
-        <v>734</v>
+        <v>744</v>
       </c>
       <c r="B14" s="250" t="s">
-        <v>735</v>
+        <v>745</v>
       </c>
       <c r="C14" s="250" t="s">
-        <v>731</v>
+        <v>741</v>
       </c>
       <c r="D14" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="E14" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="F14" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="G14" s="250" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="H14" s="253" t="s">
-        <v>732</v>
+        <v>742</v>
       </c>
       <c r="I14" s="250" t="s">
-        <v>736</v>
+        <v>746</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="282" t="s">
-        <v>737</v>
+        <v>747</v>
       </c>
       <c r="B16" s="262"/>
       <c r="C16" s="262"/>

</xml_diff>

<commit_message>
docs(tracker): add an Edge Measurement sheet for the P0-P3 plan
Its own sheet rather than more Delivery Board rows, because it answers a
different question. The board tracks what has been BUILT; this tracks
whether what was built actually works. Mixing them would let delivery
progress read as evidence of product validity, which is exactly the
confusion worth avoiding: as of today there is no demonstrated edge --
football ROI -6.4% (n=38), CLV -3.58% (n=27), tennis +1.6pp over
'always back the higher-ranked player'.

P0 blocks everything, P1 builds the measurement, P2 reads it, P3 decides
on it, and HOLD records what is deliberately not being done until the
read lands.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{310DEA81-B110-4867-9317-079474B2EC19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D98EDB-5B85-4560-8EA2-8A410F3FF6F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,8 @@
     <sheet name="Architecture" sheetId="2" r:id="rId2"/>
     <sheet name="Epic Summary" sheetId="3" r:id="rId3"/>
     <sheet name="Risks &amp; Decisions" sheetId="4" r:id="rId4"/>
-    <sheet name="APIs &amp; Quotas" sheetId="5" r:id="rId5"/>
+    <sheet name="Edge Measurement" sheetId="5" r:id="rId5"/>
+    <sheet name="APIs &amp; Quotas" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1509" uniqueCount="748">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1593" uniqueCount="796">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -2116,6 +2117,150 @@
   </si>
   <si>
     <t>Autogenerate wants NOT NULL; the database has it nullable. Stripped from the push-receipts migration rather than smuggled in. Needs its own migration</t>
+  </si>
+  <si>
+    <t>SportIQ — Edge Measurement Plan (P0-P3)</t>
+  </si>
+  <si>
+    <t>Tracks whether the predictions actually work, which the Delivery Board deliberately does not: that tracks what was BUILT. As of 2026-08-10 there is no demonstrated betting edge — football ROI -6.4% (n=38), CLV -3.58% (n=27, market moving away from our picks), tennis +1.6pp over 'always back the higher-ranked player'. Green CI is not evidence the predictions are good.</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Depends on</t>
+  </si>
+  <si>
+    <t>Why it matters / what it answers</t>
+  </si>
+  <si>
+    <t>P0</t>
+  </si>
+  <si>
+    <t>Separate real pre-game forecasts from retrodictions</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>THE blocker. No schema field distinguishes them, so /history would mix hindsight with forecast and flatter the model. Every number downstream depends on this being right first.</t>
+  </si>
+  <si>
+    <t>Confirm capture_closing_odds is actually writing</t>
+  </si>
+  <si>
+    <t>Built and scheduled, but CLV still rests on n=27. Verify the sample is genuinely growing before any conclusion leans on it.</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>Spec what /history reports, before building it</t>
+  </si>
+  <si>
+    <t>Metrics (accuracy, RPS/Brier, flat-stake ROI, CLV) and slices (sport, league, market, confidence tier, completeness band). Written first so the endpoint is not shaped by whichever cut happens to look best.</t>
+  </si>
+  <si>
+    <t>Build GET /history over existing settled outcomes</t>
+  </si>
+  <si>
+    <t>P0, spec</t>
+  </si>
+  <si>
+    <t>149 football + 2,250 tennis outcomes now exist. Its documented blocker - 'no settled outcomes exist' - is gone.</t>
+  </si>
+  <si>
+    <t>Grade the pick that was SHOWN, not a recomputed one</t>
+  </si>
+  <si>
+    <t>best_pick depends on odds and guards at request time, so re-deriving it later measures a different product than users actually saw.</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>PRE-REGISTER the verdict thresholds</t>
+  </si>
+  <si>
+    <t>spec</t>
+  </si>
+  <si>
+    <t>What counts as an edge, what counts as none, and what happens in each case - written before looking at results. Same discipline that made the Tier-1 and key-player calls trustworthy rather than fitted.</t>
+  </si>
+  <si>
+    <t>First honest read: per sport, per market, per league</t>
+  </si>
+  <si>
+    <t>/history</t>
+  </si>
+  <si>
+    <t>'No edge overall' can hide a real edge in one league or market, and a headline average would bury it.</t>
+  </si>
+  <si>
+    <t>Re-read CLV at a real sample size</t>
+  </si>
+  <si>
+    <t>P0 capture check</t>
+  </si>
+  <si>
+    <t>The sharpest signal available. Currently -3.58% on n=27 - the market moving AWAY from our picks.</t>
+  </si>
+  <si>
+    <t>Do confidence tiers mean anything?</t>
+  </si>
+  <si>
+    <t>If HIGH picks are not measurably better than MEDIUM, the badge is decoration.</t>
+  </si>
+  <si>
+    <t>Re-run completeness-vs-correctness</t>
+  </si>
+  <si>
+    <t>Was n=84 and inconclusive. Tests whether the 0.25 floor sits where it should or merely looked reasonable.</t>
+  </si>
+  <si>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>Decide Over/Under's future on the evidence</t>
+  </si>
+  <si>
+    <t>P2 read</t>
+  </si>
+  <si>
+    <t>Already measured as near-base-rate (predicted xG vs actual goals r=+0.030). The open question is not how to improve it but whether to keep surfacing it as a confident pick.</t>
+  </si>
+  <si>
+    <t>Let the measurement inform the 22 Sep renewal</t>
+  </si>
+  <si>
+    <t>API-Football ends 2026-09-29. Renewing to collect more history is a different decision from renewing to serve a working product.</t>
+  </si>
+  <si>
+    <t>HOLD</t>
+  </si>
+  <si>
+    <t>No new leagues until measurement lands</t>
+  </si>
+  <si>
+    <t>Hold</t>
+  </si>
+  <si>
+    <t>Nine were added this week. More widens coverage of something whose value is unproven.</t>
+  </si>
+  <si>
+    <t>No new markets until measurement lands</t>
+  </si>
+  <si>
+    <t>Corners and O/U are already surfaced without evidence they are worth backing.</t>
+  </si>
+  <si>
+    <t>No retrains chasing accuracy</t>
+  </si>
+  <si>
+    <t>Three retrains in two days moved the headline by noise. The binding constraint is signal and evidence, not tuning.</t>
+  </si>
+  <si>
+    <t>P0 blocks everything · P1 builds the measurement · P2 reads it · P3 decides on it · HOLD = deliberately not doing until the read lands</t>
   </si>
   <si>
     <t>External APIs, Quotas &amp; Expiry</t>
@@ -2363,7 +2508,7 @@
     <numFmt numFmtId="164" formatCode="dd\ mmm"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="74" x14ac:knownFonts="1">
+  <fonts count="79" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2775,8 +2920,34 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="74">
+  <fills count="76">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3143,6 +3314,16 @@
         <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF64748B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF334155"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="19">
     <border>
@@ -3414,7 +3595,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="283">
+  <cellXfs count="293">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4167,6 +4348,29 @@
     <xf numFmtId="0" fontId="73" fillId="73" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="74" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="76" fillId="70" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="69" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="68" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="67" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="74" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="75" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="78" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -4240,6 +4444,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="75" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="71" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -4573,46 +4780,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="257" t="s">
+      <c r="A1" s="266" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="255"/>
-      <c r="C1" s="255"/>
-      <c r="D1" s="255"/>
-      <c r="E1" s="255"/>
-      <c r="F1" s="255"/>
-      <c r="G1" s="255"/>
-      <c r="H1" s="255"/>
-      <c r="I1" s="255"/>
-      <c r="J1" s="255"/>
-      <c r="K1" s="255"/>
-      <c r="L1" s="255"/>
-      <c r="M1" s="255"/>
-      <c r="N1" s="255"/>
-      <c r="O1" s="255"/>
-      <c r="P1" s="255"/>
-      <c r="Q1" s="256"/>
+      <c r="B1" s="264"/>
+      <c r="C1" s="264"/>
+      <c r="D1" s="264"/>
+      <c r="E1" s="264"/>
+      <c r="F1" s="264"/>
+      <c r="G1" s="264"/>
+      <c r="H1" s="264"/>
+      <c r="I1" s="264"/>
+      <c r="J1" s="264"/>
+      <c r="K1" s="264"/>
+      <c r="L1" s="264"/>
+      <c r="M1" s="264"/>
+      <c r="N1" s="264"/>
+      <c r="O1" s="264"/>
+      <c r="P1" s="264"/>
+      <c r="Q1" s="265"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="254" t="s">
+      <c r="A2" s="263" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="255"/>
-      <c r="C2" s="255"/>
-      <c r="D2" s="255"/>
-      <c r="E2" s="255"/>
-      <c r="F2" s="255"/>
-      <c r="G2" s="255"/>
-      <c r="H2" s="255"/>
-      <c r="I2" s="255"/>
-      <c r="J2" s="255"/>
-      <c r="K2" s="255"/>
-      <c r="L2" s="255"/>
-      <c r="M2" s="255"/>
-      <c r="N2" s="255"/>
-      <c r="O2" s="255"/>
-      <c r="P2" s="255"/>
-      <c r="Q2" s="256"/>
+      <c r="B2" s="264"/>
+      <c r="C2" s="264"/>
+      <c r="D2" s="264"/>
+      <c r="E2" s="264"/>
+      <c r="F2" s="264"/>
+      <c r="G2" s="264"/>
+      <c r="H2" s="264"/>
+      <c r="I2" s="264"/>
+      <c r="J2" s="264"/>
+      <c r="K2" s="264"/>
+      <c r="L2" s="264"/>
+      <c r="M2" s="264"/>
+      <c r="N2" s="264"/>
+      <c r="O2" s="264"/>
+      <c r="P2" s="264"/>
+      <c r="Q2" s="265"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
@@ -10663,7 +10870,7 @@
         <v>E9 Data Ops</v>
       </c>
     </row>
-    <row r="176" spans="1:18" ht="100.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="176" spans="1:18" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A176" t="s">
         <v>162</v>
       </c>
@@ -11428,7 +11635,7 @@
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="203" spans="1:18" ht="144" x14ac:dyDescent="0.55000000000000004">
+    <row r="203" spans="1:18" ht="144" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A203" t="s">
         <v>99</v>
       </c>
@@ -11458,7 +11665,7 @@
         <v>E8 Model Quality</v>
       </c>
     </row>
-    <row r="204" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="204" spans="1:18" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A204" t="s">
         <v>73</v>
       </c>
@@ -11488,7 +11695,7 @@
         <v>E6 Picks</v>
       </c>
     </row>
-    <row r="205" spans="1:18" ht="115.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="205" spans="1:18" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B205" t="s">
         <v>445</v>
       </c>
@@ -11555,852 +11762,852 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="273" t="s">
+      <c r="A1" s="282" t="s">
         <v>449</v>
       </c>
-      <c r="B1" s="262"/>
-      <c r="C1" s="262"/>
-      <c r="D1" s="262"/>
-      <c r="E1" s="262"/>
-      <c r="F1" s="262"/>
-      <c r="G1" s="262"/>
-      <c r="H1" s="262"/>
-      <c r="I1" s="262"/>
-      <c r="J1" s="262"/>
-      <c r="K1" s="262"/>
-      <c r="L1" s="262"/>
-      <c r="M1" s="262"/>
-      <c r="N1" s="262"/>
-      <c r="O1" s="262"/>
-      <c r="P1" s="262"/>
-      <c r="Q1" s="262"/>
-      <c r="R1" s="262"/>
-      <c r="S1" s="262"/>
+      <c r="B1" s="271"/>
+      <c r="C1" s="271"/>
+      <c r="D1" s="271"/>
+      <c r="E1" s="271"/>
+      <c r="F1" s="271"/>
+      <c r="G1" s="271"/>
+      <c r="H1" s="271"/>
+      <c r="I1" s="271"/>
+      <c r="J1" s="271"/>
+      <c r="K1" s="271"/>
+      <c r="L1" s="271"/>
+      <c r="M1" s="271"/>
+      <c r="N1" s="271"/>
+      <c r="O1" s="271"/>
+      <c r="P1" s="271"/>
+      <c r="Q1" s="271"/>
+      <c r="R1" s="271"/>
+      <c r="S1" s="271"/>
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="280" t="s">
+      <c r="A2" s="289" t="s">
         <v>450</v>
       </c>
-      <c r="B2" s="262"/>
-      <c r="C2" s="262"/>
-      <c r="D2" s="262"/>
-      <c r="E2" s="262"/>
-      <c r="F2" s="262"/>
-      <c r="G2" s="262"/>
-      <c r="H2" s="262"/>
-      <c r="I2" s="262"/>
-      <c r="J2" s="262"/>
-      <c r="K2" s="262"/>
-      <c r="L2" s="262"/>
-      <c r="M2" s="262"/>
-      <c r="N2" s="262"/>
-      <c r="O2" s="262"/>
-      <c r="P2" s="262"/>
-      <c r="Q2" s="262"/>
-      <c r="R2" s="262"/>
-      <c r="S2" s="262"/>
+      <c r="B2" s="271"/>
+      <c r="C2" s="271"/>
+      <c r="D2" s="271"/>
+      <c r="E2" s="271"/>
+      <c r="F2" s="271"/>
+      <c r="G2" s="271"/>
+      <c r="H2" s="271"/>
+      <c r="I2" s="271"/>
+      <c r="J2" s="271"/>
+      <c r="K2" s="271"/>
+      <c r="L2" s="271"/>
+      <c r="M2" s="271"/>
+      <c r="N2" s="271"/>
+      <c r="O2" s="271"/>
+      <c r="P2" s="271"/>
+      <c r="Q2" s="271"/>
+      <c r="R2" s="271"/>
+      <c r="S2" s="271"/>
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="268" t="s">
+      <c r="A4" s="277" t="s">
         <v>451</v>
       </c>
-      <c r="B4" s="262"/>
-      <c r="C4" s="262"/>
-      <c r="D4" s="262"/>
-      <c r="E4" s="262"/>
-      <c r="F4" s="262"/>
-      <c r="G4" s="262"/>
-      <c r="H4" s="262"/>
-      <c r="I4" s="262"/>
-      <c r="J4" s="262"/>
-      <c r="K4" s="262"/>
-      <c r="L4" s="262"/>
-      <c r="M4" s="262"/>
-      <c r="N4" s="262"/>
-      <c r="O4" s="262"/>
-      <c r="P4" s="262"/>
-      <c r="Q4" s="262"/>
-      <c r="R4" s="262"/>
-      <c r="S4" s="262"/>
+      <c r="B4" s="271"/>
+      <c r="C4" s="271"/>
+      <c r="D4" s="271"/>
+      <c r="E4" s="271"/>
+      <c r="F4" s="271"/>
+      <c r="G4" s="271"/>
+      <c r="H4" s="271"/>
+      <c r="I4" s="271"/>
+      <c r="J4" s="271"/>
+      <c r="K4" s="271"/>
+      <c r="L4" s="271"/>
+      <c r="M4" s="271"/>
+      <c r="N4" s="271"/>
+      <c r="O4" s="271"/>
+      <c r="P4" s="271"/>
+      <c r="Q4" s="271"/>
+      <c r="R4" s="271"/>
+      <c r="S4" s="271"/>
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="37" t="s">
         <v>452</v>
       </c>
-      <c r="B5" s="258" t="s">
+      <c r="B5" s="267" t="s">
         <v>453</v>
       </c>
-      <c r="C5" s="259"/>
-      <c r="D5" s="260"/>
-      <c r="E5" s="263" t="s">
+      <c r="C5" s="268"/>
+      <c r="D5" s="269"/>
+      <c r="E5" s="272" t="s">
         <v>454</v>
       </c>
-      <c r="F5" s="259"/>
-      <c r="G5" s="260"/>
-      <c r="H5" s="263" t="s">
+      <c r="F5" s="268"/>
+      <c r="G5" s="269"/>
+      <c r="H5" s="272" t="s">
         <v>455</v>
       </c>
-      <c r="I5" s="259"/>
-      <c r="J5" s="260"/>
-      <c r="K5" s="258" t="s">
+      <c r="I5" s="268"/>
+      <c r="J5" s="269"/>
+      <c r="K5" s="267" t="s">
         <v>456</v>
       </c>
-      <c r="L5" s="259"/>
-      <c r="M5" s="260"/>
-      <c r="N5" s="265" t="s">
+      <c r="L5" s="268"/>
+      <c r="M5" s="269"/>
+      <c r="N5" s="274" t="s">
         <v>457</v>
       </c>
-      <c r="O5" s="259"/>
-      <c r="P5" s="260"/>
-      <c r="Q5" s="265" t="s">
+      <c r="O5" s="268"/>
+      <c r="P5" s="269"/>
+      <c r="Q5" s="274" t="s">
         <v>458</v>
       </c>
-      <c r="R5" s="259"/>
-      <c r="S5" s="260"/>
+      <c r="R5" s="268"/>
+      <c r="S5" s="269"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="261" t="s">
+      <c r="B6" s="270" t="s">
         <v>459</v>
       </c>
-      <c r="C6" s="262"/>
-      <c r="D6" s="262"/>
-      <c r="E6" s="262"/>
-      <c r="F6" s="262"/>
-      <c r="G6" s="262"/>
-      <c r="H6" s="262"/>
-      <c r="I6" s="262"/>
-      <c r="J6" s="262"/>
-      <c r="K6" s="262"/>
-      <c r="L6" s="262"/>
-      <c r="M6" s="262"/>
-      <c r="N6" s="262"/>
-      <c r="O6" s="262"/>
-      <c r="P6" s="262"/>
-      <c r="Q6" s="262"/>
-      <c r="R6" s="262"/>
-      <c r="S6" s="262"/>
+      <c r="C6" s="271"/>
+      <c r="D6" s="271"/>
+      <c r="E6" s="271"/>
+      <c r="F6" s="271"/>
+      <c r="G6" s="271"/>
+      <c r="H6" s="271"/>
+      <c r="I6" s="271"/>
+      <c r="J6" s="271"/>
+      <c r="K6" s="271"/>
+      <c r="L6" s="271"/>
+      <c r="M6" s="271"/>
+      <c r="N6" s="271"/>
+      <c r="O6" s="271"/>
+      <c r="P6" s="271"/>
+      <c r="Q6" s="271"/>
+      <c r="R6" s="271"/>
+      <c r="S6" s="271"/>
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="268" t="s">
+      <c r="A7" s="277" t="s">
         <v>460</v>
       </c>
-      <c r="B7" s="262"/>
-      <c r="C7" s="262"/>
-      <c r="D7" s="262"/>
-      <c r="E7" s="262"/>
-      <c r="F7" s="262"/>
-      <c r="G7" s="262"/>
-      <c r="H7" s="262"/>
-      <c r="I7" s="262"/>
-      <c r="J7" s="262"/>
-      <c r="K7" s="262"/>
-      <c r="L7" s="262"/>
-      <c r="M7" s="262"/>
-      <c r="N7" s="262"/>
-      <c r="O7" s="262"/>
-      <c r="P7" s="262"/>
-      <c r="Q7" s="262"/>
-      <c r="R7" s="262"/>
-      <c r="S7" s="262"/>
+      <c r="B7" s="271"/>
+      <c r="C7" s="271"/>
+      <c r="D7" s="271"/>
+      <c r="E7" s="271"/>
+      <c r="F7" s="271"/>
+      <c r="G7" s="271"/>
+      <c r="H7" s="271"/>
+      <c r="I7" s="271"/>
+      <c r="J7" s="271"/>
+      <c r="K7" s="271"/>
+      <c r="L7" s="271"/>
+      <c r="M7" s="271"/>
+      <c r="N7" s="271"/>
+      <c r="O7" s="271"/>
+      <c r="P7" s="271"/>
+      <c r="Q7" s="271"/>
+      <c r="R7" s="271"/>
+      <c r="S7" s="271"/>
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="37" t="s">
         <v>461</v>
       </c>
-      <c r="B8" s="271" t="s">
+      <c r="B8" s="280" t="s">
         <v>462</v>
       </c>
-      <c r="C8" s="259"/>
-      <c r="D8" s="259"/>
-      <c r="E8" s="259"/>
-      <c r="F8" s="259"/>
-      <c r="G8" s="259"/>
-      <c r="H8" s="259"/>
-      <c r="I8" s="259"/>
-      <c r="J8" s="260"/>
-      <c r="K8" s="271" t="s">
+      <c r="C8" s="268"/>
+      <c r="D8" s="268"/>
+      <c r="E8" s="268"/>
+      <c r="F8" s="268"/>
+      <c r="G8" s="268"/>
+      <c r="H8" s="268"/>
+      <c r="I8" s="268"/>
+      <c r="J8" s="269"/>
+      <c r="K8" s="280" t="s">
         <v>463</v>
       </c>
-      <c r="L8" s="259"/>
-      <c r="M8" s="259"/>
-      <c r="N8" s="259"/>
-      <c r="O8" s="259"/>
-      <c r="P8" s="259"/>
-      <c r="Q8" s="259"/>
-      <c r="R8" s="259"/>
-      <c r="S8" s="260"/>
+      <c r="L8" s="268"/>
+      <c r="M8" s="268"/>
+      <c r="N8" s="268"/>
+      <c r="O8" s="268"/>
+      <c r="P8" s="268"/>
+      <c r="Q8" s="268"/>
+      <c r="R8" s="268"/>
+      <c r="S8" s="269"/>
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B9" s="261" t="s">
+      <c r="B9" s="270" t="s">
         <v>459</v>
       </c>
-      <c r="C9" s="262"/>
-      <c r="D9" s="262"/>
-      <c r="E9" s="262"/>
-      <c r="F9" s="262"/>
-      <c r="G9" s="262"/>
-      <c r="H9" s="262"/>
-      <c r="I9" s="262"/>
-      <c r="J9" s="262"/>
-      <c r="K9" s="262"/>
-      <c r="L9" s="262"/>
-      <c r="M9" s="262"/>
-      <c r="N9" s="262"/>
-      <c r="O9" s="262"/>
-      <c r="P9" s="262"/>
-      <c r="Q9" s="262"/>
-      <c r="R9" s="262"/>
-      <c r="S9" s="262"/>
+      <c r="C9" s="271"/>
+      <c r="D9" s="271"/>
+      <c r="E9" s="271"/>
+      <c r="F9" s="271"/>
+      <c r="G9" s="271"/>
+      <c r="H9" s="271"/>
+      <c r="I9" s="271"/>
+      <c r="J9" s="271"/>
+      <c r="K9" s="271"/>
+      <c r="L9" s="271"/>
+      <c r="M9" s="271"/>
+      <c r="N9" s="271"/>
+      <c r="O9" s="271"/>
+      <c r="P9" s="271"/>
+      <c r="Q9" s="271"/>
+      <c r="R9" s="271"/>
+      <c r="S9" s="271"/>
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="268" t="s">
+      <c r="A10" s="277" t="s">
         <v>464</v>
       </c>
-      <c r="B10" s="262"/>
-      <c r="C10" s="262"/>
-      <c r="D10" s="262"/>
-      <c r="E10" s="262"/>
-      <c r="F10" s="262"/>
-      <c r="G10" s="262"/>
-      <c r="H10" s="262"/>
-      <c r="I10" s="262"/>
-      <c r="J10" s="262"/>
-      <c r="K10" s="262"/>
-      <c r="L10" s="262"/>
-      <c r="M10" s="262"/>
-      <c r="N10" s="262"/>
-      <c r="O10" s="262"/>
-      <c r="P10" s="262"/>
-      <c r="Q10" s="262"/>
-      <c r="R10" s="262"/>
-      <c r="S10" s="262"/>
+      <c r="B10" s="271"/>
+      <c r="C10" s="271"/>
+      <c r="D10" s="271"/>
+      <c r="E10" s="271"/>
+      <c r="F10" s="271"/>
+      <c r="G10" s="271"/>
+      <c r="H10" s="271"/>
+      <c r="I10" s="271"/>
+      <c r="J10" s="271"/>
+      <c r="K10" s="271"/>
+      <c r="L10" s="271"/>
+      <c r="M10" s="271"/>
+      <c r="N10" s="271"/>
+      <c r="O10" s="271"/>
+      <c r="P10" s="271"/>
+      <c r="Q10" s="271"/>
+      <c r="R10" s="271"/>
+      <c r="S10" s="271"/>
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="37" t="s">
         <v>465</v>
       </c>
-      <c r="B11" s="258" t="s">
+      <c r="B11" s="267" t="s">
         <v>466</v>
       </c>
-      <c r="C11" s="259"/>
-      <c r="D11" s="260"/>
-      <c r="E11" s="258" t="s">
+      <c r="C11" s="268"/>
+      <c r="D11" s="269"/>
+      <c r="E11" s="267" t="s">
         <v>467</v>
       </c>
-      <c r="F11" s="259"/>
-      <c r="G11" s="260"/>
-      <c r="H11" s="258" t="s">
+      <c r="F11" s="268"/>
+      <c r="G11" s="269"/>
+      <c r="H11" s="267" t="s">
         <v>468</v>
       </c>
-      <c r="I11" s="259"/>
-      <c r="J11" s="260"/>
-      <c r="K11" s="263" t="s">
+      <c r="I11" s="268"/>
+      <c r="J11" s="269"/>
+      <c r="K11" s="272" t="s">
         <v>469</v>
       </c>
-      <c r="L11" s="259"/>
-      <c r="M11" s="260"/>
-      <c r="N11" s="258" t="s">
+      <c r="L11" s="268"/>
+      <c r="M11" s="269"/>
+      <c r="N11" s="267" t="s">
         <v>470</v>
       </c>
-      <c r="O11" s="259"/>
-      <c r="P11" s="260"/>
-      <c r="Q11" s="258" t="s">
+      <c r="O11" s="268"/>
+      <c r="P11" s="269"/>
+      <c r="Q11" s="267" t="s">
         <v>471</v>
       </c>
-      <c r="R11" s="259"/>
-      <c r="S11" s="260"/>
+      <c r="R11" s="268"/>
+      <c r="S11" s="269"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B12" s="261" t="s">
+      <c r="B12" s="270" t="s">
         <v>459</v>
       </c>
-      <c r="C12" s="262"/>
-      <c r="D12" s="262"/>
-      <c r="E12" s="262"/>
-      <c r="F12" s="262"/>
-      <c r="G12" s="262"/>
-      <c r="H12" s="262"/>
-      <c r="I12" s="262"/>
-      <c r="J12" s="262"/>
-      <c r="K12" s="262"/>
-      <c r="L12" s="262"/>
-      <c r="M12" s="262"/>
-      <c r="N12" s="262"/>
-      <c r="O12" s="262"/>
-      <c r="P12" s="262"/>
-      <c r="Q12" s="262"/>
-      <c r="R12" s="262"/>
-      <c r="S12" s="262"/>
+      <c r="C12" s="271"/>
+      <c r="D12" s="271"/>
+      <c r="E12" s="271"/>
+      <c r="F12" s="271"/>
+      <c r="G12" s="271"/>
+      <c r="H12" s="271"/>
+      <c r="I12" s="271"/>
+      <c r="J12" s="271"/>
+      <c r="K12" s="271"/>
+      <c r="L12" s="271"/>
+      <c r="M12" s="271"/>
+      <c r="N12" s="271"/>
+      <c r="O12" s="271"/>
+      <c r="P12" s="271"/>
+      <c r="Q12" s="271"/>
+      <c r="R12" s="271"/>
+      <c r="S12" s="271"/>
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="268" t="s">
+      <c r="A13" s="277" t="s">
         <v>472</v>
       </c>
-      <c r="B13" s="262"/>
-      <c r="C13" s="262"/>
-      <c r="D13" s="262"/>
-      <c r="E13" s="262"/>
-      <c r="F13" s="262"/>
-      <c r="G13" s="262"/>
-      <c r="H13" s="262"/>
-      <c r="I13" s="262"/>
-      <c r="J13" s="262"/>
-      <c r="K13" s="262"/>
-      <c r="L13" s="262"/>
-      <c r="M13" s="262"/>
-      <c r="N13" s="262"/>
-      <c r="O13" s="262"/>
-      <c r="P13" s="262"/>
-      <c r="Q13" s="262"/>
-      <c r="R13" s="262"/>
-      <c r="S13" s="262"/>
+      <c r="B13" s="271"/>
+      <c r="C13" s="271"/>
+      <c r="D13" s="271"/>
+      <c r="E13" s="271"/>
+      <c r="F13" s="271"/>
+      <c r="G13" s="271"/>
+      <c r="H13" s="271"/>
+      <c r="I13" s="271"/>
+      <c r="J13" s="271"/>
+      <c r="K13" s="271"/>
+      <c r="L13" s="271"/>
+      <c r="M13" s="271"/>
+      <c r="N13" s="271"/>
+      <c r="O13" s="271"/>
+      <c r="P13" s="271"/>
+      <c r="Q13" s="271"/>
+      <c r="R13" s="271"/>
+      <c r="S13" s="271"/>
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="37" t="s">
         <v>473</v>
       </c>
-      <c r="B14" s="266" t="s">
+      <c r="B14" s="275" t="s">
         <v>474</v>
       </c>
-      <c r="C14" s="259"/>
-      <c r="D14" s="259"/>
-      <c r="E14" s="259"/>
-      <c r="F14" s="259"/>
-      <c r="G14" s="260"/>
-      <c r="H14" s="266" t="s">
+      <c r="C14" s="268"/>
+      <c r="D14" s="268"/>
+      <c r="E14" s="268"/>
+      <c r="F14" s="268"/>
+      <c r="G14" s="269"/>
+      <c r="H14" s="275" t="s">
         <v>475</v>
       </c>
-      <c r="I14" s="259"/>
-      <c r="J14" s="259"/>
-      <c r="K14" s="259"/>
-      <c r="L14" s="259"/>
-      <c r="M14" s="260"/>
-      <c r="N14" s="266" t="s">
+      <c r="I14" s="268"/>
+      <c r="J14" s="268"/>
+      <c r="K14" s="268"/>
+      <c r="L14" s="268"/>
+      <c r="M14" s="269"/>
+      <c r="N14" s="275" t="s">
         <v>476</v>
       </c>
-      <c r="O14" s="259"/>
-      <c r="P14" s="260"/>
-      <c r="Q14" s="263" t="s">
+      <c r="O14" s="268"/>
+      <c r="P14" s="269"/>
+      <c r="Q14" s="272" t="s">
         <v>477</v>
       </c>
-      <c r="R14" s="259"/>
-      <c r="S14" s="260"/>
+      <c r="R14" s="268"/>
+      <c r="S14" s="269"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B15" s="261" t="s">
+      <c r="B15" s="270" t="s">
         <v>478</v>
       </c>
-      <c r="C15" s="262"/>
-      <c r="D15" s="262"/>
-      <c r="E15" s="262"/>
-      <c r="F15" s="262"/>
-      <c r="G15" s="262"/>
-      <c r="H15" s="262"/>
-      <c r="I15" s="262"/>
-      <c r="J15" s="262"/>
-      <c r="K15" s="262"/>
-      <c r="L15" s="262"/>
-      <c r="M15" s="262"/>
-      <c r="N15" s="262"/>
-      <c r="O15" s="262"/>
-      <c r="P15" s="262"/>
-      <c r="Q15" s="262"/>
-      <c r="R15" s="262"/>
-      <c r="S15" s="262"/>
+      <c r="C15" s="271"/>
+      <c r="D15" s="271"/>
+      <c r="E15" s="271"/>
+      <c r="F15" s="271"/>
+      <c r="G15" s="271"/>
+      <c r="H15" s="271"/>
+      <c r="I15" s="271"/>
+      <c r="J15" s="271"/>
+      <c r="K15" s="271"/>
+      <c r="L15" s="271"/>
+      <c r="M15" s="271"/>
+      <c r="N15" s="271"/>
+      <c r="O15" s="271"/>
+      <c r="P15" s="271"/>
+      <c r="Q15" s="271"/>
+      <c r="R15" s="271"/>
+      <c r="S15" s="271"/>
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="268" t="s">
+      <c r="A16" s="277" t="s">
         <v>479</v>
       </c>
-      <c r="B16" s="262"/>
-      <c r="C16" s="262"/>
-      <c r="D16" s="262"/>
-      <c r="E16" s="262"/>
-      <c r="F16" s="262"/>
-      <c r="G16" s="262"/>
-      <c r="H16" s="262"/>
-      <c r="I16" s="262"/>
-      <c r="J16" s="262"/>
-      <c r="K16" s="262"/>
-      <c r="L16" s="262"/>
-      <c r="M16" s="262"/>
-      <c r="N16" s="262"/>
-      <c r="O16" s="262"/>
-      <c r="P16" s="262"/>
-      <c r="Q16" s="262"/>
-      <c r="R16" s="262"/>
-      <c r="S16" s="262"/>
+      <c r="B16" s="271"/>
+      <c r="C16" s="271"/>
+      <c r="D16" s="271"/>
+      <c r="E16" s="271"/>
+      <c r="F16" s="271"/>
+      <c r="G16" s="271"/>
+      <c r="H16" s="271"/>
+      <c r="I16" s="271"/>
+      <c r="J16" s="271"/>
+      <c r="K16" s="271"/>
+      <c r="L16" s="271"/>
+      <c r="M16" s="271"/>
+      <c r="N16" s="271"/>
+      <c r="O16" s="271"/>
+      <c r="P16" s="271"/>
+      <c r="Q16" s="271"/>
+      <c r="R16" s="271"/>
+      <c r="S16" s="271"/>
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="37" t="s">
         <v>480</v>
       </c>
-      <c r="B17" s="267" t="s">
+      <c r="B17" s="276" t="s">
         <v>481</v>
       </c>
-      <c r="C17" s="259"/>
-      <c r="D17" s="259"/>
-      <c r="E17" s="259"/>
-      <c r="F17" s="259"/>
-      <c r="G17" s="260"/>
-      <c r="H17" s="267" t="s">
+      <c r="C17" s="268"/>
+      <c r="D17" s="268"/>
+      <c r="E17" s="268"/>
+      <c r="F17" s="268"/>
+      <c r="G17" s="269"/>
+      <c r="H17" s="276" t="s">
         <v>482</v>
       </c>
-      <c r="I17" s="259"/>
-      <c r="J17" s="260"/>
-      <c r="K17" s="267" t="s">
+      <c r="I17" s="268"/>
+      <c r="J17" s="269"/>
+      <c r="K17" s="276" t="s">
         <v>483</v>
       </c>
-      <c r="L17" s="259"/>
-      <c r="M17" s="260"/>
-      <c r="N17" s="267" t="s">
+      <c r="L17" s="268"/>
+      <c r="M17" s="269"/>
+      <c r="N17" s="276" t="s">
         <v>484</v>
       </c>
-      <c r="O17" s="259"/>
-      <c r="P17" s="260"/>
-      <c r="Q17" s="267" t="s">
+      <c r="O17" s="268"/>
+      <c r="P17" s="269"/>
+      <c r="Q17" s="276" t="s">
         <v>485</v>
       </c>
-      <c r="R17" s="259"/>
-      <c r="S17" s="260"/>
+      <c r="R17" s="268"/>
+      <c r="S17" s="269"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="261" t="s">
+      <c r="B18" s="270" t="s">
         <v>459</v>
       </c>
-      <c r="C18" s="262"/>
-      <c r="D18" s="262"/>
-      <c r="E18" s="262"/>
-      <c r="F18" s="262"/>
-      <c r="G18" s="262"/>
-      <c r="H18" s="262"/>
-      <c r="I18" s="262"/>
-      <c r="J18" s="262"/>
-      <c r="K18" s="262"/>
-      <c r="L18" s="262"/>
-      <c r="M18" s="262"/>
-      <c r="N18" s="262"/>
-      <c r="O18" s="262"/>
-      <c r="P18" s="262"/>
-      <c r="Q18" s="262"/>
-      <c r="R18" s="262"/>
-      <c r="S18" s="262"/>
+      <c r="C18" s="271"/>
+      <c r="D18" s="271"/>
+      <c r="E18" s="271"/>
+      <c r="F18" s="271"/>
+      <c r="G18" s="271"/>
+      <c r="H18" s="271"/>
+      <c r="I18" s="271"/>
+      <c r="J18" s="271"/>
+      <c r="K18" s="271"/>
+      <c r="L18" s="271"/>
+      <c r="M18" s="271"/>
+      <c r="N18" s="271"/>
+      <c r="O18" s="271"/>
+      <c r="P18" s="271"/>
+      <c r="Q18" s="271"/>
+      <c r="R18" s="271"/>
+      <c r="S18" s="271"/>
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="268" t="s">
+      <c r="A19" s="277" t="s">
         <v>486</v>
       </c>
-      <c r="B19" s="262"/>
-      <c r="C19" s="262"/>
-      <c r="D19" s="262"/>
-      <c r="E19" s="262"/>
-      <c r="F19" s="262"/>
-      <c r="G19" s="262"/>
-      <c r="H19" s="262"/>
-      <c r="I19" s="262"/>
-      <c r="J19" s="262"/>
-      <c r="K19" s="262"/>
-      <c r="L19" s="262"/>
-      <c r="M19" s="262"/>
-      <c r="N19" s="262"/>
-      <c r="O19" s="262"/>
-      <c r="P19" s="262"/>
-      <c r="Q19" s="262"/>
-      <c r="R19" s="262"/>
-      <c r="S19" s="262"/>
+      <c r="B19" s="271"/>
+      <c r="C19" s="271"/>
+      <c r="D19" s="271"/>
+      <c r="E19" s="271"/>
+      <c r="F19" s="271"/>
+      <c r="G19" s="271"/>
+      <c r="H19" s="271"/>
+      <c r="I19" s="271"/>
+      <c r="J19" s="271"/>
+      <c r="K19" s="271"/>
+      <c r="L19" s="271"/>
+      <c r="M19" s="271"/>
+      <c r="N19" s="271"/>
+      <c r="O19" s="271"/>
+      <c r="P19" s="271"/>
+      <c r="Q19" s="271"/>
+      <c r="R19" s="271"/>
+      <c r="S19" s="271"/>
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="37" t="s">
         <v>487</v>
       </c>
-      <c r="B20" s="269" t="s">
+      <c r="B20" s="278" t="s">
         <v>488</v>
       </c>
-      <c r="C20" s="259"/>
-      <c r="D20" s="259"/>
-      <c r="E20" s="259"/>
-      <c r="F20" s="259"/>
-      <c r="G20" s="260"/>
-      <c r="H20" s="269" t="s">
+      <c r="C20" s="268"/>
+      <c r="D20" s="268"/>
+      <c r="E20" s="268"/>
+      <c r="F20" s="268"/>
+      <c r="G20" s="269"/>
+      <c r="H20" s="278" t="s">
         <v>489</v>
       </c>
-      <c r="I20" s="259"/>
-      <c r="J20" s="259"/>
-      <c r="K20" s="259"/>
-      <c r="L20" s="259"/>
-      <c r="M20" s="260"/>
-      <c r="N20" s="269" t="s">
+      <c r="I20" s="268"/>
+      <c r="J20" s="268"/>
+      <c r="K20" s="268"/>
+      <c r="L20" s="268"/>
+      <c r="M20" s="269"/>
+      <c r="N20" s="278" t="s">
         <v>490</v>
       </c>
-      <c r="O20" s="259"/>
-      <c r="P20" s="259"/>
-      <c r="Q20" s="259"/>
-      <c r="R20" s="259"/>
-      <c r="S20" s="260"/>
+      <c r="O20" s="268"/>
+      <c r="P20" s="268"/>
+      <c r="Q20" s="268"/>
+      <c r="R20" s="268"/>
+      <c r="S20" s="269"/>
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B21" s="261" t="s">
+      <c r="B21" s="270" t="s">
         <v>459</v>
       </c>
-      <c r="C21" s="262"/>
-      <c r="D21" s="262"/>
-      <c r="E21" s="262"/>
-      <c r="F21" s="262"/>
-      <c r="G21" s="262"/>
-      <c r="H21" s="262"/>
-      <c r="I21" s="262"/>
-      <c r="J21" s="262"/>
-      <c r="K21" s="262"/>
-      <c r="L21" s="262"/>
-      <c r="M21" s="262"/>
-      <c r="N21" s="262"/>
-      <c r="O21" s="262"/>
-      <c r="P21" s="262"/>
-      <c r="Q21" s="262"/>
-      <c r="R21" s="262"/>
-      <c r="S21" s="262"/>
+      <c r="C21" s="271"/>
+      <c r="D21" s="271"/>
+      <c r="E21" s="271"/>
+      <c r="F21" s="271"/>
+      <c r="G21" s="271"/>
+      <c r="H21" s="271"/>
+      <c r="I21" s="271"/>
+      <c r="J21" s="271"/>
+      <c r="K21" s="271"/>
+      <c r="L21" s="271"/>
+      <c r="M21" s="271"/>
+      <c r="N21" s="271"/>
+      <c r="O21" s="271"/>
+      <c r="P21" s="271"/>
+      <c r="Q21" s="271"/>
+      <c r="R21" s="271"/>
+      <c r="S21" s="271"/>
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="268" t="s">
+      <c r="A22" s="277" t="s">
         <v>491</v>
       </c>
-      <c r="B22" s="262"/>
-      <c r="C22" s="262"/>
-      <c r="D22" s="262"/>
-      <c r="E22" s="262"/>
-      <c r="F22" s="262"/>
-      <c r="G22" s="262"/>
-      <c r="H22" s="262"/>
-      <c r="I22" s="262"/>
-      <c r="J22" s="262"/>
-      <c r="K22" s="262"/>
-      <c r="L22" s="262"/>
-      <c r="M22" s="262"/>
-      <c r="N22" s="262"/>
-      <c r="O22" s="262"/>
-      <c r="P22" s="262"/>
-      <c r="Q22" s="262"/>
-      <c r="R22" s="262"/>
-      <c r="S22" s="262"/>
+      <c r="B22" s="271"/>
+      <c r="C22" s="271"/>
+      <c r="D22" s="271"/>
+      <c r="E22" s="271"/>
+      <c r="F22" s="271"/>
+      <c r="G22" s="271"/>
+      <c r="H22" s="271"/>
+      <c r="I22" s="271"/>
+      <c r="J22" s="271"/>
+      <c r="K22" s="271"/>
+      <c r="L22" s="271"/>
+      <c r="M22" s="271"/>
+      <c r="N22" s="271"/>
+      <c r="O22" s="271"/>
+      <c r="P22" s="271"/>
+      <c r="Q22" s="271"/>
+      <c r="R22" s="271"/>
+      <c r="S22" s="271"/>
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="37" t="s">
         <v>492</v>
       </c>
-      <c r="B23" s="269" t="s">
+      <c r="B23" s="278" t="s">
         <v>493</v>
       </c>
-      <c r="C23" s="259"/>
-      <c r="D23" s="259"/>
-      <c r="E23" s="259"/>
-      <c r="F23" s="259"/>
-      <c r="G23" s="260"/>
-      <c r="H23" s="269" t="s">
+      <c r="C23" s="268"/>
+      <c r="D23" s="268"/>
+      <c r="E23" s="268"/>
+      <c r="F23" s="268"/>
+      <c r="G23" s="269"/>
+      <c r="H23" s="278" t="s">
         <v>494</v>
       </c>
-      <c r="I23" s="259"/>
-      <c r="J23" s="260"/>
-      <c r="K23" s="269" t="s">
+      <c r="I23" s="268"/>
+      <c r="J23" s="269"/>
+      <c r="K23" s="278" t="s">
         <v>495</v>
       </c>
-      <c r="L23" s="259"/>
-      <c r="M23" s="260"/>
-      <c r="N23" s="269" t="s">
+      <c r="L23" s="268"/>
+      <c r="M23" s="269"/>
+      <c r="N23" s="278" t="s">
         <v>496</v>
       </c>
-      <c r="O23" s="259"/>
-      <c r="P23" s="260"/>
-      <c r="Q23" s="265" t="s">
+      <c r="O23" s="268"/>
+      <c r="P23" s="269"/>
+      <c r="Q23" s="274" t="s">
         <v>497</v>
       </c>
-      <c r="R23" s="259"/>
-      <c r="S23" s="260"/>
+      <c r="R23" s="268"/>
+      <c r="S23" s="269"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="274" t="s">
+      <c r="A26" s="283" t="s">
         <v>498</v>
       </c>
-      <c r="B26" s="262"/>
-      <c r="C26" s="262"/>
-      <c r="D26" s="262"/>
-      <c r="E26" s="262"/>
-      <c r="F26" s="262"/>
-      <c r="G26" s="262"/>
-      <c r="H26" s="262"/>
-      <c r="I26" s="262"/>
-      <c r="J26" s="262"/>
-      <c r="K26" s="262"/>
-      <c r="L26" s="262"/>
-      <c r="M26" s="262"/>
-      <c r="N26" s="262"/>
-      <c r="O26" s="262"/>
-      <c r="P26" s="262"/>
-      <c r="Q26" s="262"/>
-      <c r="R26" s="262"/>
-      <c r="S26" s="262"/>
+      <c r="B26" s="271"/>
+      <c r="C26" s="271"/>
+      <c r="D26" s="271"/>
+      <c r="E26" s="271"/>
+      <c r="F26" s="271"/>
+      <c r="G26" s="271"/>
+      <c r="H26" s="271"/>
+      <c r="I26" s="271"/>
+      <c r="J26" s="271"/>
+      <c r="K26" s="271"/>
+      <c r="L26" s="271"/>
+      <c r="M26" s="271"/>
+      <c r="N26" s="271"/>
+      <c r="O26" s="271"/>
+      <c r="P26" s="271"/>
+      <c r="Q26" s="271"/>
+      <c r="R26" s="271"/>
+      <c r="S26" s="271"/>
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="37" t="s">
         <v>499</v>
       </c>
-      <c r="B27" s="258" t="s">
+      <c r="B27" s="267" t="s">
         <v>500</v>
       </c>
-      <c r="C27" s="259"/>
-      <c r="D27" s="260"/>
-      <c r="E27" s="258" t="s">
+      <c r="C27" s="268"/>
+      <c r="D27" s="269"/>
+      <c r="E27" s="267" t="s">
         <v>501</v>
       </c>
-      <c r="F27" s="259"/>
-      <c r="G27" s="260"/>
-      <c r="H27" s="266" t="s">
+      <c r="F27" s="268"/>
+      <c r="G27" s="269"/>
+      <c r="H27" s="275" t="s">
         <v>502</v>
       </c>
-      <c r="I27" s="259"/>
-      <c r="J27" s="260"/>
-      <c r="K27" s="267" t="s">
+      <c r="I27" s="268"/>
+      <c r="J27" s="269"/>
+      <c r="K27" s="276" t="s">
         <v>503</v>
       </c>
-      <c r="L27" s="259"/>
-      <c r="M27" s="260"/>
-      <c r="N27" s="267" t="s">
+      <c r="L27" s="268"/>
+      <c r="M27" s="269"/>
+      <c r="N27" s="276" t="s">
         <v>504</v>
       </c>
-      <c r="O27" s="259"/>
-      <c r="P27" s="260"/>
-      <c r="Q27" s="266" t="s">
+      <c r="O27" s="268"/>
+      <c r="P27" s="269"/>
+      <c r="Q27" s="275" t="s">
         <v>505</v>
       </c>
-      <c r="R27" s="259"/>
-      <c r="S27" s="260"/>
+      <c r="R27" s="268"/>
+      <c r="S27" s="269"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="268" t="s">
+      <c r="A30" s="277" t="s">
         <v>506</v>
       </c>
-      <c r="B30" s="262"/>
-      <c r="C30" s="262"/>
-      <c r="D30" s="262"/>
-      <c r="E30" s="262"/>
-      <c r="F30" s="262"/>
-      <c r="G30" s="262"/>
-      <c r="H30" s="262"/>
-      <c r="I30" s="262"/>
-      <c r="J30" s="262"/>
-      <c r="K30" s="262"/>
-      <c r="L30" s="262"/>
-      <c r="M30" s="262"/>
-      <c r="N30" s="262"/>
-      <c r="O30" s="262"/>
-      <c r="P30" s="262"/>
-      <c r="Q30" s="262"/>
-      <c r="R30" s="262"/>
-      <c r="S30" s="262"/>
+      <c r="B30" s="271"/>
+      <c r="C30" s="271"/>
+      <c r="D30" s="271"/>
+      <c r="E30" s="271"/>
+      <c r="F30" s="271"/>
+      <c r="G30" s="271"/>
+      <c r="H30" s="271"/>
+      <c r="I30" s="271"/>
+      <c r="J30" s="271"/>
+      <c r="K30" s="271"/>
+      <c r="L30" s="271"/>
+      <c r="M30" s="271"/>
+      <c r="N30" s="271"/>
+      <c r="O30" s="271"/>
+      <c r="P30" s="271"/>
+      <c r="Q30" s="271"/>
+      <c r="R30" s="271"/>
+      <c r="S30" s="271"/>
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="264" t="s">
+      <c r="A31" s="273" t="s">
         <v>507</v>
       </c>
-      <c r="B31" s="262"/>
-      <c r="C31" s="262"/>
-      <c r="D31" s="262"/>
-      <c r="E31" s="262"/>
-      <c r="F31" s="262"/>
-      <c r="G31" s="262"/>
-      <c r="H31" s="262"/>
-      <c r="I31" s="262"/>
-      <c r="J31" s="262"/>
-      <c r="K31" s="262"/>
-      <c r="L31" s="262"/>
-      <c r="M31" s="262"/>
-      <c r="N31" s="262"/>
-      <c r="O31" s="262"/>
-      <c r="P31" s="262"/>
-      <c r="Q31" s="262"/>
-      <c r="R31" s="262"/>
-      <c r="S31" s="262"/>
+      <c r="B31" s="271"/>
+      <c r="C31" s="271"/>
+      <c r="D31" s="271"/>
+      <c r="E31" s="271"/>
+      <c r="F31" s="271"/>
+      <c r="G31" s="271"/>
+      <c r="H31" s="271"/>
+      <c r="I31" s="271"/>
+      <c r="J31" s="271"/>
+      <c r="K31" s="271"/>
+      <c r="L31" s="271"/>
+      <c r="M31" s="271"/>
+      <c r="N31" s="271"/>
+      <c r="O31" s="271"/>
+      <c r="P31" s="271"/>
+      <c r="Q31" s="271"/>
+      <c r="R31" s="271"/>
+      <c r="S31" s="271"/>
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="264" t="s">
+      <c r="A32" s="273" t="s">
         <v>508</v>
       </c>
-      <c r="B32" s="262"/>
-      <c r="C32" s="262"/>
-      <c r="D32" s="262"/>
-      <c r="E32" s="262"/>
-      <c r="F32" s="262"/>
-      <c r="G32" s="262"/>
-      <c r="H32" s="262"/>
-      <c r="I32" s="262"/>
-      <c r="J32" s="262"/>
-      <c r="K32" s="262"/>
-      <c r="L32" s="262"/>
-      <c r="M32" s="262"/>
-      <c r="N32" s="262"/>
-      <c r="O32" s="262"/>
-      <c r="P32" s="262"/>
-      <c r="Q32" s="262"/>
-      <c r="R32" s="262"/>
-      <c r="S32" s="262"/>
+      <c r="B32" s="271"/>
+      <c r="C32" s="271"/>
+      <c r="D32" s="271"/>
+      <c r="E32" s="271"/>
+      <c r="F32" s="271"/>
+      <c r="G32" s="271"/>
+      <c r="H32" s="271"/>
+      <c r="I32" s="271"/>
+      <c r="J32" s="271"/>
+      <c r="K32" s="271"/>
+      <c r="L32" s="271"/>
+      <c r="M32" s="271"/>
+      <c r="N32" s="271"/>
+      <c r="O32" s="271"/>
+      <c r="P32" s="271"/>
+      <c r="Q32" s="271"/>
+      <c r="R32" s="271"/>
+      <c r="S32" s="271"/>
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="264" t="s">
+      <c r="A33" s="273" t="s">
         <v>509</v>
       </c>
-      <c r="B33" s="262"/>
-      <c r="C33" s="262"/>
-      <c r="D33" s="262"/>
-      <c r="E33" s="262"/>
-      <c r="F33" s="262"/>
-      <c r="G33" s="262"/>
-      <c r="H33" s="262"/>
-      <c r="I33" s="262"/>
-      <c r="J33" s="262"/>
-      <c r="K33" s="262"/>
-      <c r="L33" s="262"/>
-      <c r="M33" s="262"/>
-      <c r="N33" s="262"/>
-      <c r="O33" s="262"/>
-      <c r="P33" s="262"/>
-      <c r="Q33" s="262"/>
-      <c r="R33" s="262"/>
-      <c r="S33" s="262"/>
+      <c r="B33" s="271"/>
+      <c r="C33" s="271"/>
+      <c r="D33" s="271"/>
+      <c r="E33" s="271"/>
+      <c r="F33" s="271"/>
+      <c r="G33" s="271"/>
+      <c r="H33" s="271"/>
+      <c r="I33" s="271"/>
+      <c r="J33" s="271"/>
+      <c r="K33" s="271"/>
+      <c r="L33" s="271"/>
+      <c r="M33" s="271"/>
+      <c r="N33" s="271"/>
+      <c r="O33" s="271"/>
+      <c r="P33" s="271"/>
+      <c r="Q33" s="271"/>
+      <c r="R33" s="271"/>
+      <c r="S33" s="271"/>
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="264" t="s">
+      <c r="A34" s="273" t="s">
         <v>510</v>
       </c>
-      <c r="B34" s="262"/>
-      <c r="C34" s="262"/>
-      <c r="D34" s="262"/>
-      <c r="E34" s="262"/>
-      <c r="F34" s="262"/>
-      <c r="G34" s="262"/>
-      <c r="H34" s="262"/>
-      <c r="I34" s="262"/>
-      <c r="J34" s="262"/>
-      <c r="K34" s="262"/>
-      <c r="L34" s="262"/>
-      <c r="M34" s="262"/>
-      <c r="N34" s="262"/>
-      <c r="O34" s="262"/>
-      <c r="P34" s="262"/>
-      <c r="Q34" s="262"/>
-      <c r="R34" s="262"/>
-      <c r="S34" s="262"/>
+      <c r="B34" s="271"/>
+      <c r="C34" s="271"/>
+      <c r="D34" s="271"/>
+      <c r="E34" s="271"/>
+      <c r="F34" s="271"/>
+      <c r="G34" s="271"/>
+      <c r="H34" s="271"/>
+      <c r="I34" s="271"/>
+      <c r="J34" s="271"/>
+      <c r="K34" s="271"/>
+      <c r="L34" s="271"/>
+      <c r="M34" s="271"/>
+      <c r="N34" s="271"/>
+      <c r="O34" s="271"/>
+      <c r="P34" s="271"/>
+      <c r="Q34" s="271"/>
+      <c r="R34" s="271"/>
+      <c r="S34" s="271"/>
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="264" t="s">
+      <c r="A35" s="273" t="s">
         <v>511</v>
       </c>
-      <c r="B35" s="262"/>
-      <c r="C35" s="262"/>
-      <c r="D35" s="262"/>
-      <c r="E35" s="262"/>
-      <c r="F35" s="262"/>
-      <c r="G35" s="262"/>
-      <c r="H35" s="262"/>
-      <c r="I35" s="262"/>
-      <c r="J35" s="262"/>
-      <c r="K35" s="262"/>
-      <c r="L35" s="262"/>
-      <c r="M35" s="262"/>
-      <c r="N35" s="262"/>
-      <c r="O35" s="262"/>
-      <c r="P35" s="262"/>
-      <c r="Q35" s="262"/>
-      <c r="R35" s="262"/>
-      <c r="S35" s="262"/>
+      <c r="B35" s="271"/>
+      <c r="C35" s="271"/>
+      <c r="D35" s="271"/>
+      <c r="E35" s="271"/>
+      <c r="F35" s="271"/>
+      <c r="G35" s="271"/>
+      <c r="H35" s="271"/>
+      <c r="I35" s="271"/>
+      <c r="J35" s="271"/>
+      <c r="K35" s="271"/>
+      <c r="L35" s="271"/>
+      <c r="M35" s="271"/>
+      <c r="N35" s="271"/>
+      <c r="O35" s="271"/>
+      <c r="P35" s="271"/>
+      <c r="Q35" s="271"/>
+      <c r="R35" s="271"/>
+      <c r="S35" s="271"/>
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="264" t="s">
+      <c r="A36" s="273" t="s">
         <v>512</v>
       </c>
-      <c r="B36" s="262"/>
-      <c r="C36" s="262"/>
-      <c r="D36" s="262"/>
-      <c r="E36" s="262"/>
-      <c r="F36" s="262"/>
-      <c r="G36" s="262"/>
-      <c r="H36" s="262"/>
-      <c r="I36" s="262"/>
-      <c r="J36" s="262"/>
-      <c r="K36" s="262"/>
-      <c r="L36" s="262"/>
-      <c r="M36" s="262"/>
-      <c r="N36" s="262"/>
-      <c r="O36" s="262"/>
-      <c r="P36" s="262"/>
-      <c r="Q36" s="262"/>
-      <c r="R36" s="262"/>
-      <c r="S36" s="262"/>
+      <c r="B36" s="271"/>
+      <c r="C36" s="271"/>
+      <c r="D36" s="271"/>
+      <c r="E36" s="271"/>
+      <c r="F36" s="271"/>
+      <c r="G36" s="271"/>
+      <c r="H36" s="271"/>
+      <c r="I36" s="271"/>
+      <c r="J36" s="271"/>
+      <c r="K36" s="271"/>
+      <c r="L36" s="271"/>
+      <c r="M36" s="271"/>
+      <c r="N36" s="271"/>
+      <c r="O36" s="271"/>
+      <c r="P36" s="271"/>
+      <c r="Q36" s="271"/>
+      <c r="R36" s="271"/>
+      <c r="S36" s="271"/>
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="275" t="s">
+      <c r="A37" s="284" t="s">
         <v>513</v>
       </c>
-      <c r="B37" s="262"/>
-      <c r="C37" s="262"/>
-      <c r="D37" s="262"/>
-      <c r="E37" s="262"/>
-      <c r="F37" s="262"/>
-      <c r="G37" s="262"/>
-      <c r="H37" s="262"/>
-      <c r="I37" s="262"/>
-      <c r="J37" s="262"/>
-      <c r="K37" s="262"/>
-      <c r="L37" s="262"/>
-      <c r="M37" s="262"/>
-      <c r="N37" s="262"/>
-      <c r="O37" s="262"/>
-      <c r="P37" s="262"/>
-      <c r="Q37" s="262"/>
-      <c r="R37" s="262"/>
-      <c r="S37" s="262"/>
+      <c r="B37" s="271"/>
+      <c r="C37" s="271"/>
+      <c r="D37" s="271"/>
+      <c r="E37" s="271"/>
+      <c r="F37" s="271"/>
+      <c r="G37" s="271"/>
+      <c r="H37" s="271"/>
+      <c r="I37" s="271"/>
+      <c r="J37" s="271"/>
+      <c r="K37" s="271"/>
+      <c r="L37" s="271"/>
+      <c r="M37" s="271"/>
+      <c r="N37" s="271"/>
+      <c r="O37" s="271"/>
+      <c r="P37" s="271"/>
+      <c r="Q37" s="271"/>
+      <c r="R37" s="271"/>
+      <c r="S37" s="271"/>
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="38" t="s">
         <v>447</v>
       </c>
-      <c r="B39" s="278" t="s">
+      <c r="B39" s="287" t="s">
         <v>514</v>
       </c>
-      <c r="C39" s="262"/>
-      <c r="D39" s="262"/>
-      <c r="E39" s="276" t="s">
+      <c r="C39" s="271"/>
+      <c r="D39" s="271"/>
+      <c r="E39" s="285" t="s">
         <v>515</v>
       </c>
-      <c r="F39" s="262"/>
-      <c r="G39" s="262"/>
-      <c r="H39" s="279" t="s">
+      <c r="F39" s="271"/>
+      <c r="G39" s="271"/>
+      <c r="H39" s="288" t="s">
         <v>516</v>
       </c>
-      <c r="I39" s="262"/>
-      <c r="J39" s="262"/>
-      <c r="K39" s="272" t="s">
+      <c r="I39" s="271"/>
+      <c r="J39" s="271"/>
+      <c r="K39" s="281" t="s">
         <v>517</v>
       </c>
-      <c r="L39" s="262"/>
-      <c r="M39" s="262"/>
-      <c r="N39" s="270" t="s">
+      <c r="L39" s="271"/>
+      <c r="M39" s="271"/>
+      <c r="N39" s="279" t="s">
         <v>45</v>
       </c>
-      <c r="O39" s="262"/>
-      <c r="P39" s="262"/>
-      <c r="Q39" s="277" t="s">
+      <c r="O39" s="271"/>
+      <c r="P39" s="271"/>
+      <c r="Q39" s="286" t="s">
         <v>518</v>
       </c>
-      <c r="R39" s="262"/>
-      <c r="S39" s="262"/>
+      <c r="R39" s="271"/>
+      <c r="S39" s="271"/>
     </row>
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="H20:M20"/>
     <mergeCell ref="A16:S16"/>
-    <mergeCell ref="H20:M20"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -12409,14 +12616,13 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -12425,6 +12631,7 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -12432,7 +12639,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -12480,14 +12687,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="281" t="s">
+      <c r="A1" s="290" t="s">
         <v>519</v>
       </c>
-      <c r="B1" s="255"/>
-      <c r="C1" s="255"/>
-      <c r="D1" s="255"/>
-      <c r="E1" s="255"/>
-      <c r="F1" s="256"/>
+      <c r="B1" s="264"/>
+      <c r="C1" s="264"/>
+      <c r="D1" s="264"/>
+      <c r="E1" s="264"/>
+      <c r="F1" s="265"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
@@ -12852,13 +13059,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="281" t="s">
+      <c r="A1" s="290" t="s">
         <v>526</v>
       </c>
-      <c r="B1" s="255"/>
-      <c r="C1" s="255"/>
-      <c r="D1" s="255"/>
-      <c r="E1" s="256"/>
+      <c r="B1" s="264"/>
+      <c r="C1" s="264"/>
+      <c r="D1" s="264"/>
+      <c r="E1" s="265"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="31" t="s">
@@ -13880,7 +14087,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="250" t="s">
         <v>665</v>
       </c>
@@ -13897,7 +14104,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="250" t="s">
         <v>667</v>
       </c>
@@ -13924,6 +14131,320 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="48" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="86" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="18.3" x14ac:dyDescent="0.7">
+      <c r="A1" s="254" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="291" t="s">
+        <v>670</v>
+      </c>
+      <c r="B2" s="271"/>
+      <c r="C2" s="271"/>
+      <c r="D2" s="271"/>
+      <c r="E2" s="271"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="255" t="s">
+        <v>671</v>
+      </c>
+      <c r="B4" s="255" t="s">
+        <v>527</v>
+      </c>
+      <c r="C4" s="255" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="255" t="s">
+        <v>672</v>
+      </c>
+      <c r="E4" s="255" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="256" t="s">
+        <v>674</v>
+      </c>
+      <c r="B5" s="250" t="s">
+        <v>675</v>
+      </c>
+      <c r="C5" s="257" t="s">
+        <v>128</v>
+      </c>
+      <c r="D5" s="250" t="s">
+        <v>676</v>
+      </c>
+      <c r="E5" s="250" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="256" t="s">
+        <v>674</v>
+      </c>
+      <c r="B6" s="250" t="s">
+        <v>678</v>
+      </c>
+      <c r="C6" s="257" t="s">
+        <v>128</v>
+      </c>
+      <c r="D6" s="250" t="s">
+        <v>676</v>
+      </c>
+      <c r="E6" s="250" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="258" t="s">
+        <v>680</v>
+      </c>
+      <c r="B7" s="250" t="s">
+        <v>681</v>
+      </c>
+      <c r="C7" s="257" t="s">
+        <v>128</v>
+      </c>
+      <c r="D7" s="250" t="s">
+        <v>674</v>
+      </c>
+      <c r="E7" s="250" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="258" t="s">
+        <v>680</v>
+      </c>
+      <c r="B8" s="250" t="s">
+        <v>683</v>
+      </c>
+      <c r="C8" s="257" t="s">
+        <v>128</v>
+      </c>
+      <c r="D8" s="250" t="s">
+        <v>684</v>
+      </c>
+      <c r="E8" s="250" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="258" t="s">
+        <v>680</v>
+      </c>
+      <c r="B9" s="250" t="s">
+        <v>686</v>
+      </c>
+      <c r="C9" s="257" t="s">
+        <v>128</v>
+      </c>
+      <c r="D9" s="250" t="s">
+        <v>674</v>
+      </c>
+      <c r="E9" s="250" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="259" t="s">
+        <v>688</v>
+      </c>
+      <c r="B10" s="250" t="s">
+        <v>689</v>
+      </c>
+      <c r="C10" s="257" t="s">
+        <v>128</v>
+      </c>
+      <c r="D10" s="250" t="s">
+        <v>690</v>
+      </c>
+      <c r="E10" s="250" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="259" t="s">
+        <v>688</v>
+      </c>
+      <c r="B11" s="250" t="s">
+        <v>692</v>
+      </c>
+      <c r="C11" s="257" t="s">
+        <v>128</v>
+      </c>
+      <c r="D11" s="250" t="s">
+        <v>693</v>
+      </c>
+      <c r="E11" s="250" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="259" t="s">
+        <v>688</v>
+      </c>
+      <c r="B12" s="250" t="s">
+        <v>695</v>
+      </c>
+      <c r="C12" s="257" t="s">
+        <v>128</v>
+      </c>
+      <c r="D12" s="250" t="s">
+        <v>696</v>
+      </c>
+      <c r="E12" s="250" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="259" t="s">
+        <v>688</v>
+      </c>
+      <c r="B13" s="250" t="s">
+        <v>698</v>
+      </c>
+      <c r="C13" s="257" t="s">
+        <v>128</v>
+      </c>
+      <c r="D13" s="250" t="s">
+        <v>693</v>
+      </c>
+      <c r="E13" s="250" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="259" t="s">
+        <v>688</v>
+      </c>
+      <c r="B14" s="250" t="s">
+        <v>700</v>
+      </c>
+      <c r="C14" s="257" t="s">
+        <v>128</v>
+      </c>
+      <c r="D14" s="250" t="s">
+        <v>693</v>
+      </c>
+      <c r="E14" s="250" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="260" t="s">
+        <v>702</v>
+      </c>
+      <c r="B15" s="250" t="s">
+        <v>703</v>
+      </c>
+      <c r="C15" s="257" t="s">
+        <v>128</v>
+      </c>
+      <c r="D15" s="250" t="s">
+        <v>704</v>
+      </c>
+      <c r="E15" s="250" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="260" t="s">
+        <v>702</v>
+      </c>
+      <c r="B16" s="250" t="s">
+        <v>706</v>
+      </c>
+      <c r="C16" s="258" t="s">
+        <v>138</v>
+      </c>
+      <c r="D16" s="250" t="s">
+        <v>704</v>
+      </c>
+      <c r="E16" s="250" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="261" t="s">
+        <v>708</v>
+      </c>
+      <c r="B17" s="250" t="s">
+        <v>709</v>
+      </c>
+      <c r="C17" s="260" t="s">
+        <v>710</v>
+      </c>
+      <c r="D17" s="250" t="s">
+        <v>676</v>
+      </c>
+      <c r="E17" s="250" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="261" t="s">
+        <v>708</v>
+      </c>
+      <c r="B18" s="250" t="s">
+        <v>712</v>
+      </c>
+      <c r="C18" s="260" t="s">
+        <v>710</v>
+      </c>
+      <c r="D18" s="250" t="s">
+        <v>676</v>
+      </c>
+      <c r="E18" s="250" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="261" t="s">
+        <v>708</v>
+      </c>
+      <c r="B19" s="250" t="s">
+        <v>714</v>
+      </c>
+      <c r="C19" s="260" t="s">
+        <v>710</v>
+      </c>
+      <c r="D19" s="250" t="s">
+        <v>676</v>
+      </c>
+      <c r="E19" s="250" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21" s="262" t="s">
+        <v>447</v>
+      </c>
+      <c r="B21" s="250" t="s">
+        <v>716</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
@@ -13940,142 +14461,142 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="246" t="s">
-        <v>669</v>
+        <v>717</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="247" t="s">
-        <v>670</v>
+        <v>718</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="248" t="s">
-        <v>671</v>
+        <v>719</v>
       </c>
       <c r="B4" s="248" t="s">
-        <v>672</v>
+        <v>720</v>
       </c>
       <c r="C4" s="248" t="s">
-        <v>673</v>
+        <v>721</v>
       </c>
       <c r="D4" s="248" t="s">
-        <v>674</v>
+        <v>722</v>
       </c>
       <c r="E4" s="248" t="s">
-        <v>675</v>
+        <v>723</v>
       </c>
       <c r="F4" s="248" t="s">
-        <v>676</v>
+        <v>724</v>
       </c>
       <c r="G4" s="248" t="s">
-        <v>677</v>
+        <v>725</v>
       </c>
       <c r="H4" s="248" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="248" t="s">
-        <v>678</v>
+        <v>726</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="249" t="s">
-        <v>679</v>
+        <v>727</v>
       </c>
       <c r="B5" s="250" t="s">
-        <v>680</v>
+        <v>728</v>
       </c>
       <c r="C5" s="250" t="s">
-        <v>681</v>
+        <v>729</v>
       </c>
       <c r="D5" s="250" t="s">
-        <v>682</v>
+        <v>730</v>
       </c>
       <c r="E5" s="250" t="s">
-        <v>683</v>
+        <v>731</v>
       </c>
       <c r="F5" s="250" t="s">
-        <v>684</v>
+        <v>732</v>
       </c>
       <c r="G5" s="250" t="s">
-        <v>685</v>
+        <v>733</v>
       </c>
       <c r="H5" s="251" t="s">
-        <v>686</v>
+        <v>734</v>
       </c>
       <c r="I5" s="250" t="s">
-        <v>687</v>
+        <v>735</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="249" t="s">
-        <v>688</v>
+        <v>736</v>
       </c>
       <c r="B6" s="250" t="s">
-        <v>689</v>
+        <v>737</v>
       </c>
       <c r="C6" s="250" t="s">
-        <v>690</v>
+        <v>738</v>
       </c>
       <c r="D6" s="250" t="s">
-        <v>691</v>
+        <v>739</v>
       </c>
       <c r="E6" s="250" t="s">
-        <v>692</v>
+        <v>740</v>
       </c>
       <c r="F6" s="250" t="s">
-        <v>693</v>
+        <v>741</v>
       </c>
       <c r="G6" s="250" t="s">
-        <v>694</v>
+        <v>742</v>
       </c>
       <c r="H6" s="252" t="s">
-        <v>686</v>
+        <v>734</v>
       </c>
       <c r="I6" s="250" t="s">
-        <v>695</v>
+        <v>743</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="249" t="s">
-        <v>696</v>
+        <v>744</v>
       </c>
       <c r="B7" s="250" t="s">
-        <v>697</v>
+        <v>745</v>
       </c>
       <c r="C7" s="250" t="s">
-        <v>698</v>
+        <v>746</v>
       </c>
       <c r="D7" s="250" t="s">
-        <v>699</v>
+        <v>747</v>
       </c>
       <c r="E7" s="250" t="s">
-        <v>700</v>
+        <v>748</v>
       </c>
       <c r="F7" s="250" t="s">
-        <v>701</v>
+        <v>749</v>
       </c>
       <c r="G7" s="250" t="s">
-        <v>702</v>
+        <v>750</v>
       </c>
       <c r="H7" s="252" t="s">
-        <v>686</v>
+        <v>734</v>
       </c>
       <c r="I7" s="250" t="s">
-        <v>703</v>
+        <v>751</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="249" t="s">
-        <v>704</v>
+        <v>752</v>
       </c>
       <c r="B8" s="250" t="s">
-        <v>705</v>
+        <v>753</v>
       </c>
       <c r="C8" s="250" t="s">
-        <v>706</v>
+        <v>754</v>
       </c>
       <c r="D8" s="250" t="s">
-        <v>707</v>
+        <v>755</v>
       </c>
       <c r="E8" s="250" t="s">
         <v>643</v>
@@ -14087,82 +14608,82 @@
         <v>643</v>
       </c>
       <c r="H8" s="251" t="s">
-        <v>708</v>
+        <v>756</v>
       </c>
       <c r="I8" s="250" t="s">
-        <v>709</v>
+        <v>757</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="249" t="s">
-        <v>710</v>
+        <v>758</v>
       </c>
       <c r="B9" s="250" t="s">
-        <v>711</v>
+        <v>759</v>
       </c>
       <c r="C9" s="250" t="s">
-        <v>712</v>
+        <v>760</v>
       </c>
       <c r="D9" s="250" t="s">
-        <v>707</v>
+        <v>755</v>
       </c>
       <c r="E9" s="250" t="s">
-        <v>700</v>
+        <v>748</v>
       </c>
       <c r="F9" s="250" t="s">
-        <v>713</v>
+        <v>761</v>
       </c>
       <c r="G9" s="250" t="s">
-        <v>714</v>
+        <v>762</v>
       </c>
       <c r="H9" s="253" t="s">
-        <v>715</v>
+        <v>763</v>
       </c>
       <c r="I9" s="250" t="s">
-        <v>716</v>
+        <v>764</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="249" t="s">
-        <v>717</v>
+        <v>765</v>
       </c>
       <c r="B10" s="250" t="s">
-        <v>718</v>
+        <v>766</v>
       </c>
       <c r="C10" s="250" t="s">
-        <v>719</v>
+        <v>767</v>
       </c>
       <c r="D10" s="250" t="s">
-        <v>720</v>
+        <v>768</v>
       </c>
       <c r="E10" s="250" t="s">
-        <v>721</v>
+        <v>769</v>
       </c>
       <c r="F10" s="250" t="s">
-        <v>722</v>
+        <v>770</v>
       </c>
       <c r="G10" s="250" t="s">
-        <v>723</v>
+        <v>771</v>
       </c>
       <c r="H10" s="253" t="s">
-        <v>724</v>
+        <v>772</v>
       </c>
       <c r="I10" s="250" t="s">
-        <v>725</v>
+        <v>773</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="249" t="s">
-        <v>726</v>
+        <v>774</v>
       </c>
       <c r="B11" s="250" t="s">
-        <v>727</v>
+        <v>775</v>
       </c>
       <c r="C11" s="250" t="s">
-        <v>728</v>
+        <v>776</v>
       </c>
       <c r="D11" s="250" t="s">
-        <v>729</v>
+        <v>777</v>
       </c>
       <c r="E11" s="250" t="s">
         <v>643</v>
@@ -14171,27 +14692,27 @@
         <v>643</v>
       </c>
       <c r="G11" s="250" t="s">
-        <v>730</v>
+        <v>778</v>
       </c>
       <c r="H11" s="253" t="s">
-        <v>731</v>
+        <v>779</v>
       </c>
       <c r="I11" s="250" t="s">
-        <v>732</v>
+        <v>780</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="249" t="s">
-        <v>733</v>
+        <v>781</v>
       </c>
       <c r="B12" s="250" t="s">
-        <v>734</v>
+        <v>782</v>
       </c>
       <c r="C12" s="250" t="s">
-        <v>735</v>
+        <v>783</v>
       </c>
       <c r="D12" s="250" t="s">
-        <v>736</v>
+        <v>784</v>
       </c>
       <c r="E12" s="250" t="s">
         <v>643</v>
@@ -14200,24 +14721,24 @@
         <v>643</v>
       </c>
       <c r="G12" s="250" t="s">
-        <v>730</v>
+        <v>778</v>
       </c>
       <c r="H12" s="252" t="s">
-        <v>737</v>
+        <v>785</v>
       </c>
       <c r="I12" s="250" t="s">
-        <v>738</v>
+        <v>786</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="249" t="s">
-        <v>739</v>
+        <v>787</v>
       </c>
       <c r="B13" s="250" t="s">
-        <v>740</v>
+        <v>788</v>
       </c>
       <c r="C13" s="250" t="s">
-        <v>741</v>
+        <v>789</v>
       </c>
       <c r="D13" s="250" t="s">
         <v>643</v>
@@ -14232,21 +14753,21 @@
         <v>643</v>
       </c>
       <c r="H13" s="253" t="s">
-        <v>742</v>
+        <v>790</v>
       </c>
       <c r="I13" s="250" t="s">
-        <v>743</v>
+        <v>791</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="249" t="s">
-        <v>744</v>
+        <v>792</v>
       </c>
       <c r="B14" s="250" t="s">
-        <v>745</v>
+        <v>793</v>
       </c>
       <c r="C14" s="250" t="s">
-        <v>741</v>
+        <v>789</v>
       </c>
       <c r="D14" s="250" t="s">
         <v>643</v>
@@ -14261,24 +14782,24 @@
         <v>643</v>
       </c>
       <c r="H14" s="253" t="s">
-        <v>742</v>
+        <v>790</v>
       </c>
       <c r="I14" s="250" t="s">
-        <v>746</v>
+        <v>794</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="282" t="s">
-        <v>747</v>
-      </c>
-      <c r="B16" s="262"/>
-      <c r="C16" s="262"/>
-      <c r="D16" s="262"/>
-      <c r="E16" s="262"/>
-      <c r="F16" s="262"/>
-      <c r="G16" s="262"/>
-      <c r="H16" s="262"/>
-      <c r="I16" s="262"/>
+      <c r="A16" s="292" t="s">
+        <v>795</v>
+      </c>
+      <c r="B16" s="271"/>
+      <c r="C16" s="271"/>
+      <c r="D16" s="271"/>
+      <c r="E16" s="271"/>
+      <c r="F16" s="271"/>
+      <c r="G16" s="271"/>
+      <c r="H16" s="271"/>
+      <c r="I16" s="271"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(tracker): close P0 and record why the first read cannot be a verdict
Both P0 items are done. capture_closing_odds turned out to already be
working -- 19 runs and 1,151 closing-line candidates against the n=27
the -3.58% CLV rests on -- so CLV is a read problem, not a capture one.

The finding that matters: at 80% power, n=139 football detects only a
10.5pp edge while we believe ours is 4.1pp, needing ~891 graded
pre-match picks (6x what exists). Tennis needs ~5,406 against 79 (68x).
So /history is instrumentation that accumulates, not an immediate
verdict, and it should surface sample size and detectable effect beside
every metric so an early number cannot be mistaken for a track record.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D98EDB-5B85-4560-8EA2-8A410F3FF6F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10246592-DC18-4D7D-9365-5D641A12B4E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1593" uniqueCount="796">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1603" uniqueCount="802">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -2143,13 +2143,13 @@
     <t>—</t>
   </si>
   <si>
-    <t>THE blocker. No schema field distinguishes them, so /history would mix hindsight with forecast and flatter the model. Every number downstream depends on this being right first.</t>
+    <t>DONE (7a611e9). predictions.kind = pre_match | retrodiction | unknown, set at write time by each path, never inferred. Timestamps could NOT substitute: regenerating 91 football predictions earlier that day reset created_at to after those kickoffs. The backfill is therefore one-directional — created_at &lt; kickoff proves a forecast, the reverse proves nothing, so those rows are UNKNOWN rather than guessed. UNKNOWN is also the column default, so a future path that forgets to set it is excluded from skill measurement rather than silently claiming to be a forecast. Result: football 283 pre_match / 90 unknown, tennis 146 / 453.</t>
   </si>
   <si>
     <t>Confirm capture_closing_odds is actually writing</t>
   </si>
   <si>
-    <t>Built and scheduled, but CLV still rests on n=27. Verify the sample is genuinely growing before any conclusion leans on it.</t>
+    <t>DONE — and it was already working. 19 task runs this session and 1,151 odds rows stamped within 45 min of kickoff, against the n=27 the -3.58% CLV figure rests on. So CLV was computed on a stale slice, not a thin one: this is a READ problem, not a capture problem, and needs analysis rather than a build.</t>
   </si>
   <si>
     <t>P1</t>
@@ -2167,7 +2167,7 @@
     <t>P0, spec</t>
   </si>
   <si>
-    <t>149 football + 2,250 tennis outcomes now exist. Its documented blocker - 'no settled outcomes exist' - is gone.</t>
+    <t>149 football + 2,250 tennis outcomes exist, but only 139 football and 79 tennis are PRE_MATCH on a completed fixture — the only rows that evidence skill. See the statistical-power row: this endpoint is instrumentation, not a verdict.</t>
   </si>
   <si>
     <t>Grade the pick that was SHOWN, not a recomputed one</t>
@@ -2258,6 +2258,24 @@
   </si>
   <si>
     <t>Three retrains in two days moved the headline by noise. The binding constraint is signal and evidence, not tuning.</t>
+  </si>
+  <si>
+    <t>FINDING: the sample cannot yet answer the question</t>
+  </si>
+  <si>
+    <t>power analysis</t>
+  </si>
+  <si>
+    <t>Measured after closing P0. At 80% power, n=139 football detects only a 10.5pp edge and we believe ours is 4.1pp — 891 graded pre-match picks needed, 6x what exists. Tennis is far worse: 1.6pp believed edge needs ~5,406, against 79 (68x). CONSEQUENCE: the first /history read cannot conclude anything about edge. Build it as instrumentation that accumulates, and expect a real verdict in months, not days. Anyone reading an early number as proof either way is reading noise.</t>
+  </si>
+  <si>
+    <t>Set expectations: /history is instrumentation, not a verdict</t>
+  </si>
+  <si>
+    <t>the finding above</t>
+  </si>
+  <si>
+    <t>Follows directly. The endpoint should show sample size and detectable-effect alongside every metric, so a 55% accuracy on n=40 cannot be mistaken for a track record. This is the difference between an honest dashboard and a misleading one.</t>
   </si>
   <si>
     <t>P0 blocks everything · P1 builds the measurement · P2 reads it · P3 decides on it · HOLD = deliberately not doing until the read lands</t>
@@ -2508,7 +2526,7 @@
     <numFmt numFmtId="164" formatCode="dd\ mmm"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="79" x14ac:knownFonts="1">
+  <fonts count="80" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2944,6 +2962,12 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -3595,7 +3619,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="293">
+  <cellXfs count="297">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4371,6 +4395,18 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="78" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="79" fillId="65" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="69" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="67" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="79" fillId="68" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -4780,46 +4816,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="266" t="s">
+      <c r="A1" s="270" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="264"/>
-      <c r="C1" s="264"/>
-      <c r="D1" s="264"/>
-      <c r="E1" s="264"/>
-      <c r="F1" s="264"/>
-      <c r="G1" s="264"/>
-      <c r="H1" s="264"/>
-      <c r="I1" s="264"/>
-      <c r="J1" s="264"/>
-      <c r="K1" s="264"/>
-      <c r="L1" s="264"/>
-      <c r="M1" s="264"/>
-      <c r="N1" s="264"/>
-      <c r="O1" s="264"/>
-      <c r="P1" s="264"/>
-      <c r="Q1" s="265"/>
+      <c r="B1" s="268"/>
+      <c r="C1" s="268"/>
+      <c r="D1" s="268"/>
+      <c r="E1" s="268"/>
+      <c r="F1" s="268"/>
+      <c r="G1" s="268"/>
+      <c r="H1" s="268"/>
+      <c r="I1" s="268"/>
+      <c r="J1" s="268"/>
+      <c r="K1" s="268"/>
+      <c r="L1" s="268"/>
+      <c r="M1" s="268"/>
+      <c r="N1" s="268"/>
+      <c r="O1" s="268"/>
+      <c r="P1" s="268"/>
+      <c r="Q1" s="269"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="263" t="s">
+      <c r="A2" s="267" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="264"/>
-      <c r="C2" s="264"/>
-      <c r="D2" s="264"/>
-      <c r="E2" s="264"/>
-      <c r="F2" s="264"/>
-      <c r="G2" s="264"/>
-      <c r="H2" s="264"/>
-      <c r="I2" s="264"/>
-      <c r="J2" s="264"/>
-      <c r="K2" s="264"/>
-      <c r="L2" s="264"/>
-      <c r="M2" s="264"/>
-      <c r="N2" s="264"/>
-      <c r="O2" s="264"/>
-      <c r="P2" s="264"/>
-      <c r="Q2" s="265"/>
+      <c r="B2" s="268"/>
+      <c r="C2" s="268"/>
+      <c r="D2" s="268"/>
+      <c r="E2" s="268"/>
+      <c r="F2" s="268"/>
+      <c r="G2" s="268"/>
+      <c r="H2" s="268"/>
+      <c r="I2" s="268"/>
+      <c r="J2" s="268"/>
+      <c r="K2" s="268"/>
+      <c r="L2" s="268"/>
+      <c r="M2" s="268"/>
+      <c r="N2" s="268"/>
+      <c r="O2" s="268"/>
+      <c r="P2" s="268"/>
+      <c r="Q2" s="269"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
@@ -11762,852 +11798,852 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="282" t="s">
+      <c r="A1" s="286" t="s">
         <v>449</v>
       </c>
-      <c r="B1" s="271"/>
-      <c r="C1" s="271"/>
-      <c r="D1" s="271"/>
-      <c r="E1" s="271"/>
-      <c r="F1" s="271"/>
-      <c r="G1" s="271"/>
-      <c r="H1" s="271"/>
-      <c r="I1" s="271"/>
-      <c r="J1" s="271"/>
-      <c r="K1" s="271"/>
-      <c r="L1" s="271"/>
-      <c r="M1" s="271"/>
-      <c r="N1" s="271"/>
-      <c r="O1" s="271"/>
-      <c r="P1" s="271"/>
-      <c r="Q1" s="271"/>
-      <c r="R1" s="271"/>
-      <c r="S1" s="271"/>
+      <c r="B1" s="275"/>
+      <c r="C1" s="275"/>
+      <c r="D1" s="275"/>
+      <c r="E1" s="275"/>
+      <c r="F1" s="275"/>
+      <c r="G1" s="275"/>
+      <c r="H1" s="275"/>
+      <c r="I1" s="275"/>
+      <c r="J1" s="275"/>
+      <c r="K1" s="275"/>
+      <c r="L1" s="275"/>
+      <c r="M1" s="275"/>
+      <c r="N1" s="275"/>
+      <c r="O1" s="275"/>
+      <c r="P1" s="275"/>
+      <c r="Q1" s="275"/>
+      <c r="R1" s="275"/>
+      <c r="S1" s="275"/>
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="289" t="s">
+      <c r="A2" s="293" t="s">
         <v>450</v>
       </c>
-      <c r="B2" s="271"/>
-      <c r="C2" s="271"/>
-      <c r="D2" s="271"/>
-      <c r="E2" s="271"/>
-      <c r="F2" s="271"/>
-      <c r="G2" s="271"/>
-      <c r="H2" s="271"/>
-      <c r="I2" s="271"/>
-      <c r="J2" s="271"/>
-      <c r="K2" s="271"/>
-      <c r="L2" s="271"/>
-      <c r="M2" s="271"/>
-      <c r="N2" s="271"/>
-      <c r="O2" s="271"/>
-      <c r="P2" s="271"/>
-      <c r="Q2" s="271"/>
-      <c r="R2" s="271"/>
-      <c r="S2" s="271"/>
+      <c r="B2" s="275"/>
+      <c r="C2" s="275"/>
+      <c r="D2" s="275"/>
+      <c r="E2" s="275"/>
+      <c r="F2" s="275"/>
+      <c r="G2" s="275"/>
+      <c r="H2" s="275"/>
+      <c r="I2" s="275"/>
+      <c r="J2" s="275"/>
+      <c r="K2" s="275"/>
+      <c r="L2" s="275"/>
+      <c r="M2" s="275"/>
+      <c r="N2" s="275"/>
+      <c r="O2" s="275"/>
+      <c r="P2" s="275"/>
+      <c r="Q2" s="275"/>
+      <c r="R2" s="275"/>
+      <c r="S2" s="275"/>
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="277" t="s">
+      <c r="A4" s="281" t="s">
         <v>451</v>
       </c>
-      <c r="B4" s="271"/>
-      <c r="C4" s="271"/>
-      <c r="D4" s="271"/>
-      <c r="E4" s="271"/>
-      <c r="F4" s="271"/>
-      <c r="G4" s="271"/>
-      <c r="H4" s="271"/>
-      <c r="I4" s="271"/>
-      <c r="J4" s="271"/>
-      <c r="K4" s="271"/>
-      <c r="L4" s="271"/>
-      <c r="M4" s="271"/>
-      <c r="N4" s="271"/>
-      <c r="O4" s="271"/>
-      <c r="P4" s="271"/>
-      <c r="Q4" s="271"/>
-      <c r="R4" s="271"/>
-      <c r="S4" s="271"/>
+      <c r="B4" s="275"/>
+      <c r="C4" s="275"/>
+      <c r="D4" s="275"/>
+      <c r="E4" s="275"/>
+      <c r="F4" s="275"/>
+      <c r="G4" s="275"/>
+      <c r="H4" s="275"/>
+      <c r="I4" s="275"/>
+      <c r="J4" s="275"/>
+      <c r="K4" s="275"/>
+      <c r="L4" s="275"/>
+      <c r="M4" s="275"/>
+      <c r="N4" s="275"/>
+      <c r="O4" s="275"/>
+      <c r="P4" s="275"/>
+      <c r="Q4" s="275"/>
+      <c r="R4" s="275"/>
+      <c r="S4" s="275"/>
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="37" t="s">
         <v>452</v>
       </c>
-      <c r="B5" s="267" t="s">
+      <c r="B5" s="271" t="s">
         <v>453</v>
       </c>
-      <c r="C5" s="268"/>
-      <c r="D5" s="269"/>
-      <c r="E5" s="272" t="s">
+      <c r="C5" s="272"/>
+      <c r="D5" s="273"/>
+      <c r="E5" s="276" t="s">
         <v>454</v>
       </c>
-      <c r="F5" s="268"/>
-      <c r="G5" s="269"/>
-      <c r="H5" s="272" t="s">
+      <c r="F5" s="272"/>
+      <c r="G5" s="273"/>
+      <c r="H5" s="276" t="s">
         <v>455</v>
       </c>
-      <c r="I5" s="268"/>
-      <c r="J5" s="269"/>
-      <c r="K5" s="267" t="s">
+      <c r="I5" s="272"/>
+      <c r="J5" s="273"/>
+      <c r="K5" s="271" t="s">
         <v>456</v>
       </c>
-      <c r="L5" s="268"/>
-      <c r="M5" s="269"/>
-      <c r="N5" s="274" t="s">
+      <c r="L5" s="272"/>
+      <c r="M5" s="273"/>
+      <c r="N5" s="278" t="s">
         <v>457</v>
       </c>
-      <c r="O5" s="268"/>
-      <c r="P5" s="269"/>
-      <c r="Q5" s="274" t="s">
+      <c r="O5" s="272"/>
+      <c r="P5" s="273"/>
+      <c r="Q5" s="278" t="s">
         <v>458</v>
       </c>
-      <c r="R5" s="268"/>
-      <c r="S5" s="269"/>
+      <c r="R5" s="272"/>
+      <c r="S5" s="273"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="270" t="s">
+      <c r="B6" s="274" t="s">
         <v>459</v>
       </c>
-      <c r="C6" s="271"/>
-      <c r="D6" s="271"/>
-      <c r="E6" s="271"/>
-      <c r="F6" s="271"/>
-      <c r="G6" s="271"/>
-      <c r="H6" s="271"/>
-      <c r="I6" s="271"/>
-      <c r="J6" s="271"/>
-      <c r="K6" s="271"/>
-      <c r="L6" s="271"/>
-      <c r="M6" s="271"/>
-      <c r="N6" s="271"/>
-      <c r="O6" s="271"/>
-      <c r="P6" s="271"/>
-      <c r="Q6" s="271"/>
-      <c r="R6" s="271"/>
-      <c r="S6" s="271"/>
+      <c r="C6" s="275"/>
+      <c r="D6" s="275"/>
+      <c r="E6" s="275"/>
+      <c r="F6" s="275"/>
+      <c r="G6" s="275"/>
+      <c r="H6" s="275"/>
+      <c r="I6" s="275"/>
+      <c r="J6" s="275"/>
+      <c r="K6" s="275"/>
+      <c r="L6" s="275"/>
+      <c r="M6" s="275"/>
+      <c r="N6" s="275"/>
+      <c r="O6" s="275"/>
+      <c r="P6" s="275"/>
+      <c r="Q6" s="275"/>
+      <c r="R6" s="275"/>
+      <c r="S6" s="275"/>
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="277" t="s">
+      <c r="A7" s="281" t="s">
         <v>460</v>
       </c>
-      <c r="B7" s="271"/>
-      <c r="C7" s="271"/>
-      <c r="D7" s="271"/>
-      <c r="E7" s="271"/>
-      <c r="F7" s="271"/>
-      <c r="G7" s="271"/>
-      <c r="H7" s="271"/>
-      <c r="I7" s="271"/>
-      <c r="J7" s="271"/>
-      <c r="K7" s="271"/>
-      <c r="L7" s="271"/>
-      <c r="M7" s="271"/>
-      <c r="N7" s="271"/>
-      <c r="O7" s="271"/>
-      <c r="P7" s="271"/>
-      <c r="Q7" s="271"/>
-      <c r="R7" s="271"/>
-      <c r="S7" s="271"/>
+      <c r="B7" s="275"/>
+      <c r="C7" s="275"/>
+      <c r="D7" s="275"/>
+      <c r="E7" s="275"/>
+      <c r="F7" s="275"/>
+      <c r="G7" s="275"/>
+      <c r="H7" s="275"/>
+      <c r="I7" s="275"/>
+      <c r="J7" s="275"/>
+      <c r="K7" s="275"/>
+      <c r="L7" s="275"/>
+      <c r="M7" s="275"/>
+      <c r="N7" s="275"/>
+      <c r="O7" s="275"/>
+      <c r="P7" s="275"/>
+      <c r="Q7" s="275"/>
+      <c r="R7" s="275"/>
+      <c r="S7" s="275"/>
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="37" t="s">
         <v>461</v>
       </c>
-      <c r="B8" s="280" t="s">
+      <c r="B8" s="284" t="s">
         <v>462</v>
       </c>
-      <c r="C8" s="268"/>
-      <c r="D8" s="268"/>
-      <c r="E8" s="268"/>
-      <c r="F8" s="268"/>
-      <c r="G8" s="268"/>
-      <c r="H8" s="268"/>
-      <c r="I8" s="268"/>
-      <c r="J8" s="269"/>
-      <c r="K8" s="280" t="s">
+      <c r="C8" s="272"/>
+      <c r="D8" s="272"/>
+      <c r="E8" s="272"/>
+      <c r="F8" s="272"/>
+      <c r="G8" s="272"/>
+      <c r="H8" s="272"/>
+      <c r="I8" s="272"/>
+      <c r="J8" s="273"/>
+      <c r="K8" s="284" t="s">
         <v>463</v>
       </c>
-      <c r="L8" s="268"/>
-      <c r="M8" s="268"/>
-      <c r="N8" s="268"/>
-      <c r="O8" s="268"/>
-      <c r="P8" s="268"/>
-      <c r="Q8" s="268"/>
-      <c r="R8" s="268"/>
-      <c r="S8" s="269"/>
+      <c r="L8" s="272"/>
+      <c r="M8" s="272"/>
+      <c r="N8" s="272"/>
+      <c r="O8" s="272"/>
+      <c r="P8" s="272"/>
+      <c r="Q8" s="272"/>
+      <c r="R8" s="272"/>
+      <c r="S8" s="273"/>
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B9" s="270" t="s">
+      <c r="B9" s="274" t="s">
         <v>459</v>
       </c>
-      <c r="C9" s="271"/>
-      <c r="D9" s="271"/>
-      <c r="E9" s="271"/>
-      <c r="F9" s="271"/>
-      <c r="G9" s="271"/>
-      <c r="H9" s="271"/>
-      <c r="I9" s="271"/>
-      <c r="J9" s="271"/>
-      <c r="K9" s="271"/>
-      <c r="L9" s="271"/>
-      <c r="M9" s="271"/>
-      <c r="N9" s="271"/>
-      <c r="O9" s="271"/>
-      <c r="P9" s="271"/>
-      <c r="Q9" s="271"/>
-      <c r="R9" s="271"/>
-      <c r="S9" s="271"/>
+      <c r="C9" s="275"/>
+      <c r="D9" s="275"/>
+      <c r="E9" s="275"/>
+      <c r="F9" s="275"/>
+      <c r="G9" s="275"/>
+      <c r="H9" s="275"/>
+      <c r="I9" s="275"/>
+      <c r="J9" s="275"/>
+      <c r="K9" s="275"/>
+      <c r="L9" s="275"/>
+      <c r="M9" s="275"/>
+      <c r="N9" s="275"/>
+      <c r="O9" s="275"/>
+      <c r="P9" s="275"/>
+      <c r="Q9" s="275"/>
+      <c r="R9" s="275"/>
+      <c r="S9" s="275"/>
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="277" t="s">
+      <c r="A10" s="281" t="s">
         <v>464</v>
       </c>
-      <c r="B10" s="271"/>
-      <c r="C10" s="271"/>
-      <c r="D10" s="271"/>
-      <c r="E10" s="271"/>
-      <c r="F10" s="271"/>
-      <c r="G10" s="271"/>
-      <c r="H10" s="271"/>
-      <c r="I10" s="271"/>
-      <c r="J10" s="271"/>
-      <c r="K10" s="271"/>
-      <c r="L10" s="271"/>
-      <c r="M10" s="271"/>
-      <c r="N10" s="271"/>
-      <c r="O10" s="271"/>
-      <c r="P10" s="271"/>
-      <c r="Q10" s="271"/>
-      <c r="R10" s="271"/>
-      <c r="S10" s="271"/>
+      <c r="B10" s="275"/>
+      <c r="C10" s="275"/>
+      <c r="D10" s="275"/>
+      <c r="E10" s="275"/>
+      <c r="F10" s="275"/>
+      <c r="G10" s="275"/>
+      <c r="H10" s="275"/>
+      <c r="I10" s="275"/>
+      <c r="J10" s="275"/>
+      <c r="K10" s="275"/>
+      <c r="L10" s="275"/>
+      <c r="M10" s="275"/>
+      <c r="N10" s="275"/>
+      <c r="O10" s="275"/>
+      <c r="P10" s="275"/>
+      <c r="Q10" s="275"/>
+      <c r="R10" s="275"/>
+      <c r="S10" s="275"/>
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="37" t="s">
         <v>465</v>
       </c>
-      <c r="B11" s="267" t="s">
+      <c r="B11" s="271" t="s">
         <v>466</v>
       </c>
-      <c r="C11" s="268"/>
-      <c r="D11" s="269"/>
-      <c r="E11" s="267" t="s">
+      <c r="C11" s="272"/>
+      <c r="D11" s="273"/>
+      <c r="E11" s="271" t="s">
         <v>467</v>
       </c>
-      <c r="F11" s="268"/>
-      <c r="G11" s="269"/>
-      <c r="H11" s="267" t="s">
+      <c r="F11" s="272"/>
+      <c r="G11" s="273"/>
+      <c r="H11" s="271" t="s">
         <v>468</v>
       </c>
-      <c r="I11" s="268"/>
-      <c r="J11" s="269"/>
-      <c r="K11" s="272" t="s">
+      <c r="I11" s="272"/>
+      <c r="J11" s="273"/>
+      <c r="K11" s="276" t="s">
         <v>469</v>
       </c>
-      <c r="L11" s="268"/>
-      <c r="M11" s="269"/>
-      <c r="N11" s="267" t="s">
+      <c r="L11" s="272"/>
+      <c r="M11" s="273"/>
+      <c r="N11" s="271" t="s">
         <v>470</v>
       </c>
-      <c r="O11" s="268"/>
-      <c r="P11" s="269"/>
-      <c r="Q11" s="267" t="s">
+      <c r="O11" s="272"/>
+      <c r="P11" s="273"/>
+      <c r="Q11" s="271" t="s">
         <v>471</v>
       </c>
-      <c r="R11" s="268"/>
-      <c r="S11" s="269"/>
+      <c r="R11" s="272"/>
+      <c r="S11" s="273"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B12" s="270" t="s">
+      <c r="B12" s="274" t="s">
         <v>459</v>
       </c>
-      <c r="C12" s="271"/>
-      <c r="D12" s="271"/>
-      <c r="E12" s="271"/>
-      <c r="F12" s="271"/>
-      <c r="G12" s="271"/>
-      <c r="H12" s="271"/>
-      <c r="I12" s="271"/>
-      <c r="J12" s="271"/>
-      <c r="K12" s="271"/>
-      <c r="L12" s="271"/>
-      <c r="M12" s="271"/>
-      <c r="N12" s="271"/>
-      <c r="O12" s="271"/>
-      <c r="P12" s="271"/>
-      <c r="Q12" s="271"/>
-      <c r="R12" s="271"/>
-      <c r="S12" s="271"/>
+      <c r="C12" s="275"/>
+      <c r="D12" s="275"/>
+      <c r="E12" s="275"/>
+      <c r="F12" s="275"/>
+      <c r="G12" s="275"/>
+      <c r="H12" s="275"/>
+      <c r="I12" s="275"/>
+      <c r="J12" s="275"/>
+      <c r="K12" s="275"/>
+      <c r="L12" s="275"/>
+      <c r="M12" s="275"/>
+      <c r="N12" s="275"/>
+      <c r="O12" s="275"/>
+      <c r="P12" s="275"/>
+      <c r="Q12" s="275"/>
+      <c r="R12" s="275"/>
+      <c r="S12" s="275"/>
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="277" t="s">
+      <c r="A13" s="281" t="s">
         <v>472</v>
       </c>
-      <c r="B13" s="271"/>
-      <c r="C13" s="271"/>
-      <c r="D13" s="271"/>
-      <c r="E13" s="271"/>
-      <c r="F13" s="271"/>
-      <c r="G13" s="271"/>
-      <c r="H13" s="271"/>
-      <c r="I13" s="271"/>
-      <c r="J13" s="271"/>
-      <c r="K13" s="271"/>
-      <c r="L13" s="271"/>
-      <c r="M13" s="271"/>
-      <c r="N13" s="271"/>
-      <c r="O13" s="271"/>
-      <c r="P13" s="271"/>
-      <c r="Q13" s="271"/>
-      <c r="R13" s="271"/>
-      <c r="S13" s="271"/>
+      <c r="B13" s="275"/>
+      <c r="C13" s="275"/>
+      <c r="D13" s="275"/>
+      <c r="E13" s="275"/>
+      <c r="F13" s="275"/>
+      <c r="G13" s="275"/>
+      <c r="H13" s="275"/>
+      <c r="I13" s="275"/>
+      <c r="J13" s="275"/>
+      <c r="K13" s="275"/>
+      <c r="L13" s="275"/>
+      <c r="M13" s="275"/>
+      <c r="N13" s="275"/>
+      <c r="O13" s="275"/>
+      <c r="P13" s="275"/>
+      <c r="Q13" s="275"/>
+      <c r="R13" s="275"/>
+      <c r="S13" s="275"/>
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="37" t="s">
         <v>473</v>
       </c>
-      <c r="B14" s="275" t="s">
+      <c r="B14" s="279" t="s">
         <v>474</v>
       </c>
-      <c r="C14" s="268"/>
-      <c r="D14" s="268"/>
-      <c r="E14" s="268"/>
-      <c r="F14" s="268"/>
-      <c r="G14" s="269"/>
-      <c r="H14" s="275" t="s">
+      <c r="C14" s="272"/>
+      <c r="D14" s="272"/>
+      <c r="E14" s="272"/>
+      <c r="F14" s="272"/>
+      <c r="G14" s="273"/>
+      <c r="H14" s="279" t="s">
         <v>475</v>
       </c>
-      <c r="I14" s="268"/>
-      <c r="J14" s="268"/>
-      <c r="K14" s="268"/>
-      <c r="L14" s="268"/>
-      <c r="M14" s="269"/>
-      <c r="N14" s="275" t="s">
+      <c r="I14" s="272"/>
+      <c r="J14" s="272"/>
+      <c r="K14" s="272"/>
+      <c r="L14" s="272"/>
+      <c r="M14" s="273"/>
+      <c r="N14" s="279" t="s">
         <v>476</v>
       </c>
-      <c r="O14" s="268"/>
-      <c r="P14" s="269"/>
-      <c r="Q14" s="272" t="s">
+      <c r="O14" s="272"/>
+      <c r="P14" s="273"/>
+      <c r="Q14" s="276" t="s">
         <v>477</v>
       </c>
-      <c r="R14" s="268"/>
-      <c r="S14" s="269"/>
+      <c r="R14" s="272"/>
+      <c r="S14" s="273"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B15" s="270" t="s">
+      <c r="B15" s="274" t="s">
         <v>478</v>
       </c>
-      <c r="C15" s="271"/>
-      <c r="D15" s="271"/>
-      <c r="E15" s="271"/>
-      <c r="F15" s="271"/>
-      <c r="G15" s="271"/>
-      <c r="H15" s="271"/>
-      <c r="I15" s="271"/>
-      <c r="J15" s="271"/>
-      <c r="K15" s="271"/>
-      <c r="L15" s="271"/>
-      <c r="M15" s="271"/>
-      <c r="N15" s="271"/>
-      <c r="O15" s="271"/>
-      <c r="P15" s="271"/>
-      <c r="Q15" s="271"/>
-      <c r="R15" s="271"/>
-      <c r="S15" s="271"/>
+      <c r="C15" s="275"/>
+      <c r="D15" s="275"/>
+      <c r="E15" s="275"/>
+      <c r="F15" s="275"/>
+      <c r="G15" s="275"/>
+      <c r="H15" s="275"/>
+      <c r="I15" s="275"/>
+      <c r="J15" s="275"/>
+      <c r="K15" s="275"/>
+      <c r="L15" s="275"/>
+      <c r="M15" s="275"/>
+      <c r="N15" s="275"/>
+      <c r="O15" s="275"/>
+      <c r="P15" s="275"/>
+      <c r="Q15" s="275"/>
+      <c r="R15" s="275"/>
+      <c r="S15" s="275"/>
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="277" t="s">
+      <c r="A16" s="281" t="s">
         <v>479</v>
       </c>
-      <c r="B16" s="271"/>
-      <c r="C16" s="271"/>
-      <c r="D16" s="271"/>
-      <c r="E16" s="271"/>
-      <c r="F16" s="271"/>
-      <c r="G16" s="271"/>
-      <c r="H16" s="271"/>
-      <c r="I16" s="271"/>
-      <c r="J16" s="271"/>
-      <c r="K16" s="271"/>
-      <c r="L16" s="271"/>
-      <c r="M16" s="271"/>
-      <c r="N16" s="271"/>
-      <c r="O16" s="271"/>
-      <c r="P16" s="271"/>
-      <c r="Q16" s="271"/>
-      <c r="R16" s="271"/>
-      <c r="S16" s="271"/>
+      <c r="B16" s="275"/>
+      <c r="C16" s="275"/>
+      <c r="D16" s="275"/>
+      <c r="E16" s="275"/>
+      <c r="F16" s="275"/>
+      <c r="G16" s="275"/>
+      <c r="H16" s="275"/>
+      <c r="I16" s="275"/>
+      <c r="J16" s="275"/>
+      <c r="K16" s="275"/>
+      <c r="L16" s="275"/>
+      <c r="M16" s="275"/>
+      <c r="N16" s="275"/>
+      <c r="O16" s="275"/>
+      <c r="P16" s="275"/>
+      <c r="Q16" s="275"/>
+      <c r="R16" s="275"/>
+      <c r="S16" s="275"/>
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="37" t="s">
         <v>480</v>
       </c>
-      <c r="B17" s="276" t="s">
+      <c r="B17" s="280" t="s">
         <v>481</v>
       </c>
-      <c r="C17" s="268"/>
-      <c r="D17" s="268"/>
-      <c r="E17" s="268"/>
-      <c r="F17" s="268"/>
-      <c r="G17" s="269"/>
-      <c r="H17" s="276" t="s">
+      <c r="C17" s="272"/>
+      <c r="D17" s="272"/>
+      <c r="E17" s="272"/>
+      <c r="F17" s="272"/>
+      <c r="G17" s="273"/>
+      <c r="H17" s="280" t="s">
         <v>482</v>
       </c>
-      <c r="I17" s="268"/>
-      <c r="J17" s="269"/>
-      <c r="K17" s="276" t="s">
+      <c r="I17" s="272"/>
+      <c r="J17" s="273"/>
+      <c r="K17" s="280" t="s">
         <v>483</v>
       </c>
-      <c r="L17" s="268"/>
-      <c r="M17" s="269"/>
-      <c r="N17" s="276" t="s">
+      <c r="L17" s="272"/>
+      <c r="M17" s="273"/>
+      <c r="N17" s="280" t="s">
         <v>484</v>
       </c>
-      <c r="O17" s="268"/>
-      <c r="P17" s="269"/>
-      <c r="Q17" s="276" t="s">
+      <c r="O17" s="272"/>
+      <c r="P17" s="273"/>
+      <c r="Q17" s="280" t="s">
         <v>485</v>
       </c>
-      <c r="R17" s="268"/>
-      <c r="S17" s="269"/>
+      <c r="R17" s="272"/>
+      <c r="S17" s="273"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="270" t="s">
+      <c r="B18" s="274" t="s">
         <v>459</v>
       </c>
-      <c r="C18" s="271"/>
-      <c r="D18" s="271"/>
-      <c r="E18" s="271"/>
-      <c r="F18" s="271"/>
-      <c r="G18" s="271"/>
-      <c r="H18" s="271"/>
-      <c r="I18" s="271"/>
-      <c r="J18" s="271"/>
-      <c r="K18" s="271"/>
-      <c r="L18" s="271"/>
-      <c r="M18" s="271"/>
-      <c r="N18" s="271"/>
-      <c r="O18" s="271"/>
-      <c r="P18" s="271"/>
-      <c r="Q18" s="271"/>
-      <c r="R18" s="271"/>
-      <c r="S18" s="271"/>
+      <c r="C18" s="275"/>
+      <c r="D18" s="275"/>
+      <c r="E18" s="275"/>
+      <c r="F18" s="275"/>
+      <c r="G18" s="275"/>
+      <c r="H18" s="275"/>
+      <c r="I18" s="275"/>
+      <c r="J18" s="275"/>
+      <c r="K18" s="275"/>
+      <c r="L18" s="275"/>
+      <c r="M18" s="275"/>
+      <c r="N18" s="275"/>
+      <c r="O18" s="275"/>
+      <c r="P18" s="275"/>
+      <c r="Q18" s="275"/>
+      <c r="R18" s="275"/>
+      <c r="S18" s="275"/>
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="277" t="s">
+      <c r="A19" s="281" t="s">
         <v>486</v>
       </c>
-      <c r="B19" s="271"/>
-      <c r="C19" s="271"/>
-      <c r="D19" s="271"/>
-      <c r="E19" s="271"/>
-      <c r="F19" s="271"/>
-      <c r="G19" s="271"/>
-      <c r="H19" s="271"/>
-      <c r="I19" s="271"/>
-      <c r="J19" s="271"/>
-      <c r="K19" s="271"/>
-      <c r="L19" s="271"/>
-      <c r="M19" s="271"/>
-      <c r="N19" s="271"/>
-      <c r="O19" s="271"/>
-      <c r="P19" s="271"/>
-      <c r="Q19" s="271"/>
-      <c r="R19" s="271"/>
-      <c r="S19" s="271"/>
+      <c r="B19" s="275"/>
+      <c r="C19" s="275"/>
+      <c r="D19" s="275"/>
+      <c r="E19" s="275"/>
+      <c r="F19" s="275"/>
+      <c r="G19" s="275"/>
+      <c r="H19" s="275"/>
+      <c r="I19" s="275"/>
+      <c r="J19" s="275"/>
+      <c r="K19" s="275"/>
+      <c r="L19" s="275"/>
+      <c r="M19" s="275"/>
+      <c r="N19" s="275"/>
+      <c r="O19" s="275"/>
+      <c r="P19" s="275"/>
+      <c r="Q19" s="275"/>
+      <c r="R19" s="275"/>
+      <c r="S19" s="275"/>
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="37" t="s">
         <v>487</v>
       </c>
-      <c r="B20" s="278" t="s">
+      <c r="B20" s="282" t="s">
         <v>488</v>
       </c>
-      <c r="C20" s="268"/>
-      <c r="D20" s="268"/>
-      <c r="E20" s="268"/>
-      <c r="F20" s="268"/>
-      <c r="G20" s="269"/>
-      <c r="H20" s="278" t="s">
+      <c r="C20" s="272"/>
+      <c r="D20" s="272"/>
+      <c r="E20" s="272"/>
+      <c r="F20" s="272"/>
+      <c r="G20" s="273"/>
+      <c r="H20" s="282" t="s">
         <v>489</v>
       </c>
-      <c r="I20" s="268"/>
-      <c r="J20" s="268"/>
-      <c r="K20" s="268"/>
-      <c r="L20" s="268"/>
-      <c r="M20" s="269"/>
-      <c r="N20" s="278" t="s">
+      <c r="I20" s="272"/>
+      <c r="J20" s="272"/>
+      <c r="K20" s="272"/>
+      <c r="L20" s="272"/>
+      <c r="M20" s="273"/>
+      <c r="N20" s="282" t="s">
         <v>490</v>
       </c>
-      <c r="O20" s="268"/>
-      <c r="P20" s="268"/>
-      <c r="Q20" s="268"/>
-      <c r="R20" s="268"/>
-      <c r="S20" s="269"/>
+      <c r="O20" s="272"/>
+      <c r="P20" s="272"/>
+      <c r="Q20" s="272"/>
+      <c r="R20" s="272"/>
+      <c r="S20" s="273"/>
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B21" s="270" t="s">
+      <c r="B21" s="274" t="s">
         <v>459</v>
       </c>
-      <c r="C21" s="271"/>
-      <c r="D21" s="271"/>
-      <c r="E21" s="271"/>
-      <c r="F21" s="271"/>
-      <c r="G21" s="271"/>
-      <c r="H21" s="271"/>
-      <c r="I21" s="271"/>
-      <c r="J21" s="271"/>
-      <c r="K21" s="271"/>
-      <c r="L21" s="271"/>
-      <c r="M21" s="271"/>
-      <c r="N21" s="271"/>
-      <c r="O21" s="271"/>
-      <c r="P21" s="271"/>
-      <c r="Q21" s="271"/>
-      <c r="R21" s="271"/>
-      <c r="S21" s="271"/>
+      <c r="C21" s="275"/>
+      <c r="D21" s="275"/>
+      <c r="E21" s="275"/>
+      <c r="F21" s="275"/>
+      <c r="G21" s="275"/>
+      <c r="H21" s="275"/>
+      <c r="I21" s="275"/>
+      <c r="J21" s="275"/>
+      <c r="K21" s="275"/>
+      <c r="L21" s="275"/>
+      <c r="M21" s="275"/>
+      <c r="N21" s="275"/>
+      <c r="O21" s="275"/>
+      <c r="P21" s="275"/>
+      <c r="Q21" s="275"/>
+      <c r="R21" s="275"/>
+      <c r="S21" s="275"/>
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="277" t="s">
+      <c r="A22" s="281" t="s">
         <v>491</v>
       </c>
-      <c r="B22" s="271"/>
-      <c r="C22" s="271"/>
-      <c r="D22" s="271"/>
-      <c r="E22" s="271"/>
-      <c r="F22" s="271"/>
-      <c r="G22" s="271"/>
-      <c r="H22" s="271"/>
-      <c r="I22" s="271"/>
-      <c r="J22" s="271"/>
-      <c r="K22" s="271"/>
-      <c r="L22" s="271"/>
-      <c r="M22" s="271"/>
-      <c r="N22" s="271"/>
-      <c r="O22" s="271"/>
-      <c r="P22" s="271"/>
-      <c r="Q22" s="271"/>
-      <c r="R22" s="271"/>
-      <c r="S22" s="271"/>
+      <c r="B22" s="275"/>
+      <c r="C22" s="275"/>
+      <c r="D22" s="275"/>
+      <c r="E22" s="275"/>
+      <c r="F22" s="275"/>
+      <c r="G22" s="275"/>
+      <c r="H22" s="275"/>
+      <c r="I22" s="275"/>
+      <c r="J22" s="275"/>
+      <c r="K22" s="275"/>
+      <c r="L22" s="275"/>
+      <c r="M22" s="275"/>
+      <c r="N22" s="275"/>
+      <c r="O22" s="275"/>
+      <c r="P22" s="275"/>
+      <c r="Q22" s="275"/>
+      <c r="R22" s="275"/>
+      <c r="S22" s="275"/>
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="37" t="s">
         <v>492</v>
       </c>
-      <c r="B23" s="278" t="s">
+      <c r="B23" s="282" t="s">
         <v>493</v>
       </c>
-      <c r="C23" s="268"/>
-      <c r="D23" s="268"/>
-      <c r="E23" s="268"/>
-      <c r="F23" s="268"/>
-      <c r="G23" s="269"/>
-      <c r="H23" s="278" t="s">
+      <c r="C23" s="272"/>
+      <c r="D23" s="272"/>
+      <c r="E23" s="272"/>
+      <c r="F23" s="272"/>
+      <c r="G23" s="273"/>
+      <c r="H23" s="282" t="s">
         <v>494</v>
       </c>
-      <c r="I23" s="268"/>
-      <c r="J23" s="269"/>
-      <c r="K23" s="278" t="s">
+      <c r="I23" s="272"/>
+      <c r="J23" s="273"/>
+      <c r="K23" s="282" t="s">
         <v>495</v>
       </c>
-      <c r="L23" s="268"/>
-      <c r="M23" s="269"/>
-      <c r="N23" s="278" t="s">
+      <c r="L23" s="272"/>
+      <c r="M23" s="273"/>
+      <c r="N23" s="282" t="s">
         <v>496</v>
       </c>
-      <c r="O23" s="268"/>
-      <c r="P23" s="269"/>
-      <c r="Q23" s="274" t="s">
+      <c r="O23" s="272"/>
+      <c r="P23" s="273"/>
+      <c r="Q23" s="278" t="s">
         <v>497</v>
       </c>
-      <c r="R23" s="268"/>
-      <c r="S23" s="269"/>
+      <c r="R23" s="272"/>
+      <c r="S23" s="273"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="283" t="s">
+      <c r="A26" s="287" t="s">
         <v>498</v>
       </c>
-      <c r="B26" s="271"/>
-      <c r="C26" s="271"/>
-      <c r="D26" s="271"/>
-      <c r="E26" s="271"/>
-      <c r="F26" s="271"/>
-      <c r="G26" s="271"/>
-      <c r="H26" s="271"/>
-      <c r="I26" s="271"/>
-      <c r="J26" s="271"/>
-      <c r="K26" s="271"/>
-      <c r="L26" s="271"/>
-      <c r="M26" s="271"/>
-      <c r="N26" s="271"/>
-      <c r="O26" s="271"/>
-      <c r="P26" s="271"/>
-      <c r="Q26" s="271"/>
-      <c r="R26" s="271"/>
-      <c r="S26" s="271"/>
+      <c r="B26" s="275"/>
+      <c r="C26" s="275"/>
+      <c r="D26" s="275"/>
+      <c r="E26" s="275"/>
+      <c r="F26" s="275"/>
+      <c r="G26" s="275"/>
+      <c r="H26" s="275"/>
+      <c r="I26" s="275"/>
+      <c r="J26" s="275"/>
+      <c r="K26" s="275"/>
+      <c r="L26" s="275"/>
+      <c r="M26" s="275"/>
+      <c r="N26" s="275"/>
+      <c r="O26" s="275"/>
+      <c r="P26" s="275"/>
+      <c r="Q26" s="275"/>
+      <c r="R26" s="275"/>
+      <c r="S26" s="275"/>
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="37" t="s">
         <v>499</v>
       </c>
-      <c r="B27" s="267" t="s">
+      <c r="B27" s="271" t="s">
         <v>500</v>
       </c>
-      <c r="C27" s="268"/>
-      <c r="D27" s="269"/>
-      <c r="E27" s="267" t="s">
+      <c r="C27" s="272"/>
+      <c r="D27" s="273"/>
+      <c r="E27" s="271" t="s">
         <v>501</v>
       </c>
-      <c r="F27" s="268"/>
-      <c r="G27" s="269"/>
-      <c r="H27" s="275" t="s">
+      <c r="F27" s="272"/>
+      <c r="G27" s="273"/>
+      <c r="H27" s="279" t="s">
         <v>502</v>
       </c>
-      <c r="I27" s="268"/>
-      <c r="J27" s="269"/>
-      <c r="K27" s="276" t="s">
+      <c r="I27" s="272"/>
+      <c r="J27" s="273"/>
+      <c r="K27" s="280" t="s">
         <v>503</v>
       </c>
-      <c r="L27" s="268"/>
-      <c r="M27" s="269"/>
-      <c r="N27" s="276" t="s">
+      <c r="L27" s="272"/>
+      <c r="M27" s="273"/>
+      <c r="N27" s="280" t="s">
         <v>504</v>
       </c>
-      <c r="O27" s="268"/>
-      <c r="P27" s="269"/>
-      <c r="Q27" s="275" t="s">
+      <c r="O27" s="272"/>
+      <c r="P27" s="273"/>
+      <c r="Q27" s="279" t="s">
         <v>505</v>
       </c>
-      <c r="R27" s="268"/>
-      <c r="S27" s="269"/>
+      <c r="R27" s="272"/>
+      <c r="S27" s="273"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="277" t="s">
+      <c r="A30" s="281" t="s">
         <v>506</v>
       </c>
-      <c r="B30" s="271"/>
-      <c r="C30" s="271"/>
-      <c r="D30" s="271"/>
-      <c r="E30" s="271"/>
-      <c r="F30" s="271"/>
-      <c r="G30" s="271"/>
-      <c r="H30" s="271"/>
-      <c r="I30" s="271"/>
-      <c r="J30" s="271"/>
-      <c r="K30" s="271"/>
-      <c r="L30" s="271"/>
-      <c r="M30" s="271"/>
-      <c r="N30" s="271"/>
-      <c r="O30" s="271"/>
-      <c r="P30" s="271"/>
-      <c r="Q30" s="271"/>
-      <c r="R30" s="271"/>
-      <c r="S30" s="271"/>
+      <c r="B30" s="275"/>
+      <c r="C30" s="275"/>
+      <c r="D30" s="275"/>
+      <c r="E30" s="275"/>
+      <c r="F30" s="275"/>
+      <c r="G30" s="275"/>
+      <c r="H30" s="275"/>
+      <c r="I30" s="275"/>
+      <c r="J30" s="275"/>
+      <c r="K30" s="275"/>
+      <c r="L30" s="275"/>
+      <c r="M30" s="275"/>
+      <c r="N30" s="275"/>
+      <c r="O30" s="275"/>
+      <c r="P30" s="275"/>
+      <c r="Q30" s="275"/>
+      <c r="R30" s="275"/>
+      <c r="S30" s="275"/>
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="273" t="s">
+      <c r="A31" s="277" t="s">
         <v>507</v>
       </c>
-      <c r="B31" s="271"/>
-      <c r="C31" s="271"/>
-      <c r="D31" s="271"/>
-      <c r="E31" s="271"/>
-      <c r="F31" s="271"/>
-      <c r="G31" s="271"/>
-      <c r="H31" s="271"/>
-      <c r="I31" s="271"/>
-      <c r="J31" s="271"/>
-      <c r="K31" s="271"/>
-      <c r="L31" s="271"/>
-      <c r="M31" s="271"/>
-      <c r="N31" s="271"/>
-      <c r="O31" s="271"/>
-      <c r="P31" s="271"/>
-      <c r="Q31" s="271"/>
-      <c r="R31" s="271"/>
-      <c r="S31" s="271"/>
+      <c r="B31" s="275"/>
+      <c r="C31" s="275"/>
+      <c r="D31" s="275"/>
+      <c r="E31" s="275"/>
+      <c r="F31" s="275"/>
+      <c r="G31" s="275"/>
+      <c r="H31" s="275"/>
+      <c r="I31" s="275"/>
+      <c r="J31" s="275"/>
+      <c r="K31" s="275"/>
+      <c r="L31" s="275"/>
+      <c r="M31" s="275"/>
+      <c r="N31" s="275"/>
+      <c r="O31" s="275"/>
+      <c r="P31" s="275"/>
+      <c r="Q31" s="275"/>
+      <c r="R31" s="275"/>
+      <c r="S31" s="275"/>
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="273" t="s">
+      <c r="A32" s="277" t="s">
         <v>508</v>
       </c>
-      <c r="B32" s="271"/>
-      <c r="C32" s="271"/>
-      <c r="D32" s="271"/>
-      <c r="E32" s="271"/>
-      <c r="F32" s="271"/>
-      <c r="G32" s="271"/>
-      <c r="H32" s="271"/>
-      <c r="I32" s="271"/>
-      <c r="J32" s="271"/>
-      <c r="K32" s="271"/>
-      <c r="L32" s="271"/>
-      <c r="M32" s="271"/>
-      <c r="N32" s="271"/>
-      <c r="O32" s="271"/>
-      <c r="P32" s="271"/>
-      <c r="Q32" s="271"/>
-      <c r="R32" s="271"/>
-      <c r="S32" s="271"/>
+      <c r="B32" s="275"/>
+      <c r="C32" s="275"/>
+      <c r="D32" s="275"/>
+      <c r="E32" s="275"/>
+      <c r="F32" s="275"/>
+      <c r="G32" s="275"/>
+      <c r="H32" s="275"/>
+      <c r="I32" s="275"/>
+      <c r="J32" s="275"/>
+      <c r="K32" s="275"/>
+      <c r="L32" s="275"/>
+      <c r="M32" s="275"/>
+      <c r="N32" s="275"/>
+      <c r="O32" s="275"/>
+      <c r="P32" s="275"/>
+      <c r="Q32" s="275"/>
+      <c r="R32" s="275"/>
+      <c r="S32" s="275"/>
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="273" t="s">
+      <c r="A33" s="277" t="s">
         <v>509</v>
       </c>
-      <c r="B33" s="271"/>
-      <c r="C33" s="271"/>
-      <c r="D33" s="271"/>
-      <c r="E33" s="271"/>
-      <c r="F33" s="271"/>
-      <c r="G33" s="271"/>
-      <c r="H33" s="271"/>
-      <c r="I33" s="271"/>
-      <c r="J33" s="271"/>
-      <c r="K33" s="271"/>
-      <c r="L33" s="271"/>
-      <c r="M33" s="271"/>
-      <c r="N33" s="271"/>
-      <c r="O33" s="271"/>
-      <c r="P33" s="271"/>
-      <c r="Q33" s="271"/>
-      <c r="R33" s="271"/>
-      <c r="S33" s="271"/>
+      <c r="B33" s="275"/>
+      <c r="C33" s="275"/>
+      <c r="D33" s="275"/>
+      <c r="E33" s="275"/>
+      <c r="F33" s="275"/>
+      <c r="G33" s="275"/>
+      <c r="H33" s="275"/>
+      <c r="I33" s="275"/>
+      <c r="J33" s="275"/>
+      <c r="K33" s="275"/>
+      <c r="L33" s="275"/>
+      <c r="M33" s="275"/>
+      <c r="N33" s="275"/>
+      <c r="O33" s="275"/>
+      <c r="P33" s="275"/>
+      <c r="Q33" s="275"/>
+      <c r="R33" s="275"/>
+      <c r="S33" s="275"/>
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="273" t="s">
+      <c r="A34" s="277" t="s">
         <v>510</v>
       </c>
-      <c r="B34" s="271"/>
-      <c r="C34" s="271"/>
-      <c r="D34" s="271"/>
-      <c r="E34" s="271"/>
-      <c r="F34" s="271"/>
-      <c r="G34" s="271"/>
-      <c r="H34" s="271"/>
-      <c r="I34" s="271"/>
-      <c r="J34" s="271"/>
-      <c r="K34" s="271"/>
-      <c r="L34" s="271"/>
-      <c r="M34" s="271"/>
-      <c r="N34" s="271"/>
-      <c r="O34" s="271"/>
-      <c r="P34" s="271"/>
-      <c r="Q34" s="271"/>
-      <c r="R34" s="271"/>
-      <c r="S34" s="271"/>
+      <c r="B34" s="275"/>
+      <c r="C34" s="275"/>
+      <c r="D34" s="275"/>
+      <c r="E34" s="275"/>
+      <c r="F34" s="275"/>
+      <c r="G34" s="275"/>
+      <c r="H34" s="275"/>
+      <c r="I34" s="275"/>
+      <c r="J34" s="275"/>
+      <c r="K34" s="275"/>
+      <c r="L34" s="275"/>
+      <c r="M34" s="275"/>
+      <c r="N34" s="275"/>
+      <c r="O34" s="275"/>
+      <c r="P34" s="275"/>
+      <c r="Q34" s="275"/>
+      <c r="R34" s="275"/>
+      <c r="S34" s="275"/>
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="273" t="s">
+      <c r="A35" s="277" t="s">
         <v>511</v>
       </c>
-      <c r="B35" s="271"/>
-      <c r="C35" s="271"/>
-      <c r="D35" s="271"/>
-      <c r="E35" s="271"/>
-      <c r="F35" s="271"/>
-      <c r="G35" s="271"/>
-      <c r="H35" s="271"/>
-      <c r="I35" s="271"/>
-      <c r="J35" s="271"/>
-      <c r="K35" s="271"/>
-      <c r="L35" s="271"/>
-      <c r="M35" s="271"/>
-      <c r="N35" s="271"/>
-      <c r="O35" s="271"/>
-      <c r="P35" s="271"/>
-      <c r="Q35" s="271"/>
-      <c r="R35" s="271"/>
-      <c r="S35" s="271"/>
+      <c r="B35" s="275"/>
+      <c r="C35" s="275"/>
+      <c r="D35" s="275"/>
+      <c r="E35" s="275"/>
+      <c r="F35" s="275"/>
+      <c r="G35" s="275"/>
+      <c r="H35" s="275"/>
+      <c r="I35" s="275"/>
+      <c r="J35" s="275"/>
+      <c r="K35" s="275"/>
+      <c r="L35" s="275"/>
+      <c r="M35" s="275"/>
+      <c r="N35" s="275"/>
+      <c r="O35" s="275"/>
+      <c r="P35" s="275"/>
+      <c r="Q35" s="275"/>
+      <c r="R35" s="275"/>
+      <c r="S35" s="275"/>
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="273" t="s">
+      <c r="A36" s="277" t="s">
         <v>512</v>
       </c>
-      <c r="B36" s="271"/>
-      <c r="C36" s="271"/>
-      <c r="D36" s="271"/>
-      <c r="E36" s="271"/>
-      <c r="F36" s="271"/>
-      <c r="G36" s="271"/>
-      <c r="H36" s="271"/>
-      <c r="I36" s="271"/>
-      <c r="J36" s="271"/>
-      <c r="K36" s="271"/>
-      <c r="L36" s="271"/>
-      <c r="M36" s="271"/>
-      <c r="N36" s="271"/>
-      <c r="O36" s="271"/>
-      <c r="P36" s="271"/>
-      <c r="Q36" s="271"/>
-      <c r="R36" s="271"/>
-      <c r="S36" s="271"/>
+      <c r="B36" s="275"/>
+      <c r="C36" s="275"/>
+      <c r="D36" s="275"/>
+      <c r="E36" s="275"/>
+      <c r="F36" s="275"/>
+      <c r="G36" s="275"/>
+      <c r="H36" s="275"/>
+      <c r="I36" s="275"/>
+      <c r="J36" s="275"/>
+      <c r="K36" s="275"/>
+      <c r="L36" s="275"/>
+      <c r="M36" s="275"/>
+      <c r="N36" s="275"/>
+      <c r="O36" s="275"/>
+      <c r="P36" s="275"/>
+      <c r="Q36" s="275"/>
+      <c r="R36" s="275"/>
+      <c r="S36" s="275"/>
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="284" t="s">
+      <c r="A37" s="288" t="s">
         <v>513</v>
       </c>
-      <c r="B37" s="271"/>
-      <c r="C37" s="271"/>
-      <c r="D37" s="271"/>
-      <c r="E37" s="271"/>
-      <c r="F37" s="271"/>
-      <c r="G37" s="271"/>
-      <c r="H37" s="271"/>
-      <c r="I37" s="271"/>
-      <c r="J37" s="271"/>
-      <c r="K37" s="271"/>
-      <c r="L37" s="271"/>
-      <c r="M37" s="271"/>
-      <c r="N37" s="271"/>
-      <c r="O37" s="271"/>
-      <c r="P37" s="271"/>
-      <c r="Q37" s="271"/>
-      <c r="R37" s="271"/>
-      <c r="S37" s="271"/>
+      <c r="B37" s="275"/>
+      <c r="C37" s="275"/>
+      <c r="D37" s="275"/>
+      <c r="E37" s="275"/>
+      <c r="F37" s="275"/>
+      <c r="G37" s="275"/>
+      <c r="H37" s="275"/>
+      <c r="I37" s="275"/>
+      <c r="J37" s="275"/>
+      <c r="K37" s="275"/>
+      <c r="L37" s="275"/>
+      <c r="M37" s="275"/>
+      <c r="N37" s="275"/>
+      <c r="O37" s="275"/>
+      <c r="P37" s="275"/>
+      <c r="Q37" s="275"/>
+      <c r="R37" s="275"/>
+      <c r="S37" s="275"/>
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="38" t="s">
         <v>447</v>
       </c>
-      <c r="B39" s="287" t="s">
+      <c r="B39" s="291" t="s">
         <v>514</v>
       </c>
-      <c r="C39" s="271"/>
-      <c r="D39" s="271"/>
-      <c r="E39" s="285" t="s">
+      <c r="C39" s="275"/>
+      <c r="D39" s="275"/>
+      <c r="E39" s="289" t="s">
         <v>515</v>
       </c>
-      <c r="F39" s="271"/>
-      <c r="G39" s="271"/>
-      <c r="H39" s="288" t="s">
+      <c r="F39" s="275"/>
+      <c r="G39" s="275"/>
+      <c r="H39" s="292" t="s">
         <v>516</v>
       </c>
-      <c r="I39" s="271"/>
-      <c r="J39" s="271"/>
-      <c r="K39" s="281" t="s">
+      <c r="I39" s="275"/>
+      <c r="J39" s="275"/>
+      <c r="K39" s="285" t="s">
         <v>517</v>
       </c>
-      <c r="L39" s="271"/>
-      <c r="M39" s="271"/>
-      <c r="N39" s="279" t="s">
+      <c r="L39" s="275"/>
+      <c r="M39" s="275"/>
+      <c r="N39" s="283" t="s">
         <v>45</v>
       </c>
-      <c r="O39" s="271"/>
-      <c r="P39" s="271"/>
-      <c r="Q39" s="286" t="s">
+      <c r="O39" s="275"/>
+      <c r="P39" s="275"/>
+      <c r="Q39" s="290" t="s">
         <v>518</v>
       </c>
-      <c r="R39" s="271"/>
-      <c r="S39" s="271"/>
+      <c r="R39" s="275"/>
+      <c r="S39" s="275"/>
     </row>
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H14:M14"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A16:S16"/>
     <mergeCell ref="H20:M20"/>
-    <mergeCell ref="A16:S16"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -12616,13 +12652,14 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -12631,7 +12668,6 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
-    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -12639,7 +12675,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -12687,14 +12723,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="290" t="s">
+      <c r="A1" s="294" t="s">
         <v>519</v>
       </c>
-      <c r="B1" s="264"/>
-      <c r="C1" s="264"/>
-      <c r="D1" s="264"/>
-      <c r="E1" s="264"/>
-      <c r="F1" s="265"/>
+      <c r="B1" s="268"/>
+      <c r="C1" s="268"/>
+      <c r="D1" s="268"/>
+      <c r="E1" s="268"/>
+      <c r="F1" s="269"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
@@ -13059,13 +13095,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="290" t="s">
+      <c r="A1" s="294" t="s">
         <v>526</v>
       </c>
-      <c r="B1" s="264"/>
-      <c r="C1" s="264"/>
-      <c r="D1" s="264"/>
-      <c r="E1" s="265"/>
+      <c r="B1" s="268"/>
+      <c r="C1" s="268"/>
+      <c r="D1" s="268"/>
+      <c r="E1" s="269"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="31" t="s">
@@ -14131,7 +14167,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -14141,19 +14177,19 @@
     <col min="5" max="5" width="86" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.3" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:5" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="254" t="s">
         <v>669</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="291" t="s">
+      <c r="A2" s="295" t="s">
         <v>670</v>
       </c>
-      <c r="B2" s="271"/>
-      <c r="C2" s="271"/>
-      <c r="D2" s="271"/>
-      <c r="E2" s="271"/>
+      <c r="B2" s="275"/>
+      <c r="C2" s="275"/>
+      <c r="D2" s="275"/>
+      <c r="E2" s="275"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="255" t="s">
@@ -14179,8 +14215,8 @@
       <c r="B5" s="250" t="s">
         <v>675</v>
       </c>
-      <c r="C5" s="257" t="s">
-        <v>128</v>
+      <c r="C5" s="263" t="s">
+        <v>22</v>
       </c>
       <c r="D5" s="250" t="s">
         <v>676</v>
@@ -14196,8 +14232,8 @@
       <c r="B6" s="250" t="s">
         <v>678</v>
       </c>
-      <c r="C6" s="257" t="s">
-        <v>128</v>
+      <c r="C6" s="263" t="s">
+        <v>22</v>
       </c>
       <c r="D6" s="250" t="s">
         <v>676</v>
@@ -14427,12 +14463,46 @@
         <v>715</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="43.2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="262" t="s">
-        <v>447</v>
+    <row r="21" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21" s="264" t="s">
+        <v>674</v>
       </c>
       <c r="B21" s="250" t="s">
         <v>716</v>
+      </c>
+      <c r="C21" s="263" t="s">
+        <v>22</v>
+      </c>
+      <c r="D21" s="250" t="s">
+        <v>717</v>
+      </c>
+      <c r="E21" s="250" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A22" s="265" t="s">
+        <v>680</v>
+      </c>
+      <c r="B22" s="250" t="s">
+        <v>719</v>
+      </c>
+      <c r="C22" s="266" t="s">
+        <v>128</v>
+      </c>
+      <c r="D22" s="250" t="s">
+        <v>720</v>
+      </c>
+      <c r="E22" s="250" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A23" s="262" t="s">
+        <v>447</v>
+      </c>
+      <c r="B23" s="250" t="s">
+        <v>722</v>
       </c>
     </row>
   </sheetData>
@@ -14461,142 +14531,142 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="246" t="s">
-        <v>717</v>
+        <v>723</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="247" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="248" t="s">
-        <v>719</v>
+        <v>725</v>
       </c>
       <c r="B4" s="248" t="s">
-        <v>720</v>
+        <v>726</v>
       </c>
       <c r="C4" s="248" t="s">
-        <v>721</v>
+        <v>727</v>
       </c>
       <c r="D4" s="248" t="s">
-        <v>722</v>
+        <v>728</v>
       </c>
       <c r="E4" s="248" t="s">
-        <v>723</v>
+        <v>729</v>
       </c>
       <c r="F4" s="248" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
       <c r="G4" s="248" t="s">
-        <v>725</v>
+        <v>731</v>
       </c>
       <c r="H4" s="248" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="248" t="s">
-        <v>726</v>
+        <v>732</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="249" t="s">
-        <v>727</v>
+        <v>733</v>
       </c>
       <c r="B5" s="250" t="s">
-        <v>728</v>
+        <v>734</v>
       </c>
       <c r="C5" s="250" t="s">
-        <v>729</v>
+        <v>735</v>
       </c>
       <c r="D5" s="250" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="E5" s="250" t="s">
-        <v>731</v>
+        <v>737</v>
       </c>
       <c r="F5" s="250" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="G5" s="250" t="s">
-        <v>733</v>
+        <v>739</v>
       </c>
       <c r="H5" s="251" t="s">
-        <v>734</v>
+        <v>740</v>
       </c>
       <c r="I5" s="250" t="s">
-        <v>735</v>
+        <v>741</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="249" t="s">
-        <v>736</v>
+        <v>742</v>
       </c>
       <c r="B6" s="250" t="s">
-        <v>737</v>
+        <v>743</v>
       </c>
       <c r="C6" s="250" t="s">
-        <v>738</v>
+        <v>744</v>
       </c>
       <c r="D6" s="250" t="s">
-        <v>739</v>
+        <v>745</v>
       </c>
       <c r="E6" s="250" t="s">
+        <v>746</v>
+      </c>
+      <c r="F6" s="250" t="s">
+        <v>747</v>
+      </c>
+      <c r="G6" s="250" t="s">
+        <v>748</v>
+      </c>
+      <c r="H6" s="252" t="s">
         <v>740</v>
       </c>
-      <c r="F6" s="250" t="s">
-        <v>741</v>
-      </c>
-      <c r="G6" s="250" t="s">
-        <v>742</v>
-      </c>
-      <c r="H6" s="252" t="s">
-        <v>734</v>
-      </c>
       <c r="I6" s="250" t="s">
-        <v>743</v>
+        <v>749</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="249" t="s">
-        <v>744</v>
+        <v>750</v>
       </c>
       <c r="B7" s="250" t="s">
-        <v>745</v>
+        <v>751</v>
       </c>
       <c r="C7" s="250" t="s">
-        <v>746</v>
+        <v>752</v>
       </c>
       <c r="D7" s="250" t="s">
-        <v>747</v>
+        <v>753</v>
       </c>
       <c r="E7" s="250" t="s">
-        <v>748</v>
+        <v>754</v>
       </c>
       <c r="F7" s="250" t="s">
-        <v>749</v>
+        <v>755</v>
       </c>
       <c r="G7" s="250" t="s">
-        <v>750</v>
+        <v>756</v>
       </c>
       <c r="H7" s="252" t="s">
-        <v>734</v>
+        <v>740</v>
       </c>
       <c r="I7" s="250" t="s">
-        <v>751</v>
+        <v>757</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="249" t="s">
-        <v>752</v>
+        <v>758</v>
       </c>
       <c r="B8" s="250" t="s">
-        <v>753</v>
+        <v>759</v>
       </c>
       <c r="C8" s="250" t="s">
-        <v>754</v>
+        <v>760</v>
       </c>
       <c r="D8" s="250" t="s">
-        <v>755</v>
+        <v>761</v>
       </c>
       <c r="E8" s="250" t="s">
         <v>643</v>
@@ -14608,82 +14678,82 @@
         <v>643</v>
       </c>
       <c r="H8" s="251" t="s">
-        <v>756</v>
+        <v>762</v>
       </c>
       <c r="I8" s="250" t="s">
-        <v>757</v>
+        <v>763</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="249" t="s">
-        <v>758</v>
+        <v>764</v>
       </c>
       <c r="B9" s="250" t="s">
-        <v>759</v>
+        <v>765</v>
       </c>
       <c r="C9" s="250" t="s">
-        <v>760</v>
+        <v>766</v>
       </c>
       <c r="D9" s="250" t="s">
-        <v>755</v>
+        <v>761</v>
       </c>
       <c r="E9" s="250" t="s">
-        <v>748</v>
+        <v>754</v>
       </c>
       <c r="F9" s="250" t="s">
-        <v>761</v>
+        <v>767</v>
       </c>
       <c r="G9" s="250" t="s">
-        <v>762</v>
+        <v>768</v>
       </c>
       <c r="H9" s="253" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="I9" s="250" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="249" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="B10" s="250" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
       <c r="C10" s="250" t="s">
-        <v>767</v>
+        <v>773</v>
       </c>
       <c r="D10" s="250" t="s">
-        <v>768</v>
+        <v>774</v>
       </c>
       <c r="E10" s="250" t="s">
-        <v>769</v>
+        <v>775</v>
       </c>
       <c r="F10" s="250" t="s">
-        <v>770</v>
+        <v>776</v>
       </c>
       <c r="G10" s="250" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="H10" s="253" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
       <c r="I10" s="250" t="s">
-        <v>773</v>
+        <v>779</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="249" t="s">
-        <v>774</v>
+        <v>780</v>
       </c>
       <c r="B11" s="250" t="s">
-        <v>775</v>
+        <v>781</v>
       </c>
       <c r="C11" s="250" t="s">
-        <v>776</v>
+        <v>782</v>
       </c>
       <c r="D11" s="250" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
       <c r="E11" s="250" t="s">
         <v>643</v>
@@ -14692,27 +14762,27 @@
         <v>643</v>
       </c>
       <c r="G11" s="250" t="s">
-        <v>778</v>
+        <v>784</v>
       </c>
       <c r="H11" s="253" t="s">
-        <v>779</v>
+        <v>785</v>
       </c>
       <c r="I11" s="250" t="s">
-        <v>780</v>
+        <v>786</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="249" t="s">
-        <v>781</v>
+        <v>787</v>
       </c>
       <c r="B12" s="250" t="s">
-        <v>782</v>
+        <v>788</v>
       </c>
       <c r="C12" s="250" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="D12" s="250" t="s">
-        <v>784</v>
+        <v>790</v>
       </c>
       <c r="E12" s="250" t="s">
         <v>643</v>
@@ -14721,24 +14791,24 @@
         <v>643</v>
       </c>
       <c r="G12" s="250" t="s">
-        <v>778</v>
+        <v>784</v>
       </c>
       <c r="H12" s="252" t="s">
-        <v>785</v>
+        <v>791</v>
       </c>
       <c r="I12" s="250" t="s">
-        <v>786</v>
+        <v>792</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="249" t="s">
-        <v>787</v>
+        <v>793</v>
       </c>
       <c r="B13" s="250" t="s">
-        <v>788</v>
+        <v>794</v>
       </c>
       <c r="C13" s="250" t="s">
-        <v>789</v>
+        <v>795</v>
       </c>
       <c r="D13" s="250" t="s">
         <v>643</v>
@@ -14753,21 +14823,21 @@
         <v>643</v>
       </c>
       <c r="H13" s="253" t="s">
-        <v>790</v>
+        <v>796</v>
       </c>
       <c r="I13" s="250" t="s">
-        <v>791</v>
+        <v>797</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="249" t="s">
-        <v>792</v>
+        <v>798</v>
       </c>
       <c r="B14" s="250" t="s">
-        <v>793</v>
+        <v>799</v>
       </c>
       <c r="C14" s="250" t="s">
-        <v>789</v>
+        <v>795</v>
       </c>
       <c r="D14" s="250" t="s">
         <v>643</v>
@@ -14782,24 +14852,24 @@
         <v>643</v>
       </c>
       <c r="H14" s="253" t="s">
-        <v>790</v>
+        <v>796</v>
       </c>
       <c r="I14" s="250" t="s">
-        <v>794</v>
+        <v>800</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="292" t="s">
-        <v>795</v>
-      </c>
-      <c r="B16" s="271"/>
-      <c r="C16" s="271"/>
-      <c r="D16" s="271"/>
-      <c r="E16" s="271"/>
-      <c r="F16" s="271"/>
-      <c r="G16" s="271"/>
-      <c r="H16" s="271"/>
-      <c r="I16" s="271"/>
+      <c r="A16" s="296" t="s">
+        <v>801</v>
+      </c>
+      <c r="B16" s="275"/>
+      <c r="C16" s="275"/>
+      <c r="D16" s="275"/>
+      <c r="E16" s="275"/>
+      <c r="F16" s="275"/>
+      <c r="G16" s="275"/>
+      <c r="H16" s="275"/>
+      <c r="I16" s="275"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(tracker): close pick snapshotting on the Edge Measurement sheet
P0 fully closed; P1 now 3 of 5 done. The ROI/CLV clock started at
8f794e0 — nothing before it is recoverable, which is the reason this
was sequenced ahead of the endpoint itself.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B836150B-DB46-4C92-97FF-C4D052F77064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD61F26F-F56E-4AFF-AE90-A851D56E09C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2173,7 +2173,7 @@
     <t>Grade the pick that was SHOWN, not a recomputed one</t>
   </si>
   <si>
-    <t>best_pick depends on odds and guards at request time, so re-deriving it later measures a different product than users actually saw.</t>
+    <t>Resolved by pick_snapshots: /history will grade the stored snapshot rather than recomputing, so it measures the product users actually saw. Applies only to fixtures captured from 2026-08-10 onward.</t>
   </si>
   <si>
     <t>P2</t>
@@ -2290,7 +2290,7 @@
     <t>Persist the pick at the moment it is shown</t>
   </si>
   <si>
-    <t>Selection, market, line, odds, probability, model version, and which guards it passed. Everything in the product-skill half of /history starts accumulating from this change, not before — so the sooner it lands, the sooner the ROI/CLV clock starts.</t>
+    <t>DONE (8f794e0). pick_snapshots, captured hourly for fixtures 4-8 HOURS out — not next to the closing-odds capture, which would have made CLV meaningless by construction: taken/closing - 1 is ~0 when both prices are recorded fifteen minutes apart, so the metric would read reassuringly neutral while measuring nothing. Delegates to _bulk_best_picks, the feed's own selection, with a test asserting the delegation. One row per fixture. Verified live: an ATP pick at 2.17, p=0.536, T-7.3h. NOTE: nothing before this commit is recoverable — the ROI/CLV clock starts now.</t>
   </si>
   <si>
     <t>P0 blocks everything · P1 builds the measurement · P2 reads it · P3 decides on it · HOLD = deliberately not doing until the read lands</t>
@@ -2541,7 +2541,7 @@
     <numFmt numFmtId="164" formatCode="dd\ mmm"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="81" x14ac:knownFonts="1">
+  <fonts count="82" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2977,6 +2977,12 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -3640,7 +3646,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="300">
+  <cellXfs count="301">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4435,6 +4441,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="80" fillId="68" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="81" fillId="65" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4846,46 +4855,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="273" t="s">
+      <c r="A1" s="274" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="271"/>
-      <c r="C1" s="271"/>
-      <c r="D1" s="271"/>
-      <c r="E1" s="271"/>
-      <c r="F1" s="271"/>
-      <c r="G1" s="271"/>
-      <c r="H1" s="271"/>
-      <c r="I1" s="271"/>
-      <c r="J1" s="271"/>
-      <c r="K1" s="271"/>
-      <c r="L1" s="271"/>
-      <c r="M1" s="271"/>
-      <c r="N1" s="271"/>
-      <c r="O1" s="271"/>
-      <c r="P1" s="271"/>
-      <c r="Q1" s="272"/>
+      <c r="B1" s="272"/>
+      <c r="C1" s="272"/>
+      <c r="D1" s="272"/>
+      <c r="E1" s="272"/>
+      <c r="F1" s="272"/>
+      <c r="G1" s="272"/>
+      <c r="H1" s="272"/>
+      <c r="I1" s="272"/>
+      <c r="J1" s="272"/>
+      <c r="K1" s="272"/>
+      <c r="L1" s="272"/>
+      <c r="M1" s="272"/>
+      <c r="N1" s="272"/>
+      <c r="O1" s="272"/>
+      <c r="P1" s="272"/>
+      <c r="Q1" s="273"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="270" t="s">
+      <c r="A2" s="271" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="271"/>
-      <c r="C2" s="271"/>
-      <c r="D2" s="271"/>
-      <c r="E2" s="271"/>
-      <c r="F2" s="271"/>
-      <c r="G2" s="271"/>
-      <c r="H2" s="271"/>
-      <c r="I2" s="271"/>
-      <c r="J2" s="271"/>
-      <c r="K2" s="271"/>
-      <c r="L2" s="271"/>
-      <c r="M2" s="271"/>
-      <c r="N2" s="271"/>
-      <c r="O2" s="271"/>
-      <c r="P2" s="271"/>
-      <c r="Q2" s="272"/>
+      <c r="B2" s="272"/>
+      <c r="C2" s="272"/>
+      <c r="D2" s="272"/>
+      <c r="E2" s="272"/>
+      <c r="F2" s="272"/>
+      <c r="G2" s="272"/>
+      <c r="H2" s="272"/>
+      <c r="I2" s="272"/>
+      <c r="J2" s="272"/>
+      <c r="K2" s="272"/>
+      <c r="L2" s="272"/>
+      <c r="M2" s="272"/>
+      <c r="N2" s="272"/>
+      <c r="O2" s="272"/>
+      <c r="P2" s="272"/>
+      <c r="Q2" s="273"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
@@ -11828,852 +11837,852 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="289" t="s">
+      <c r="A1" s="290" t="s">
         <v>449</v>
       </c>
-      <c r="B1" s="278"/>
-      <c r="C1" s="278"/>
-      <c r="D1" s="278"/>
-      <c r="E1" s="278"/>
-      <c r="F1" s="278"/>
-      <c r="G1" s="278"/>
-      <c r="H1" s="278"/>
-      <c r="I1" s="278"/>
-      <c r="J1" s="278"/>
-      <c r="K1" s="278"/>
-      <c r="L1" s="278"/>
-      <c r="M1" s="278"/>
-      <c r="N1" s="278"/>
-      <c r="O1" s="278"/>
-      <c r="P1" s="278"/>
-      <c r="Q1" s="278"/>
-      <c r="R1" s="278"/>
-      <c r="S1" s="278"/>
+      <c r="B1" s="279"/>
+      <c r="C1" s="279"/>
+      <c r="D1" s="279"/>
+      <c r="E1" s="279"/>
+      <c r="F1" s="279"/>
+      <c r="G1" s="279"/>
+      <c r="H1" s="279"/>
+      <c r="I1" s="279"/>
+      <c r="J1" s="279"/>
+      <c r="K1" s="279"/>
+      <c r="L1" s="279"/>
+      <c r="M1" s="279"/>
+      <c r="N1" s="279"/>
+      <c r="O1" s="279"/>
+      <c r="P1" s="279"/>
+      <c r="Q1" s="279"/>
+      <c r="R1" s="279"/>
+      <c r="S1" s="279"/>
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="296" t="s">
+      <c r="A2" s="297" t="s">
         <v>450</v>
       </c>
-      <c r="B2" s="278"/>
-      <c r="C2" s="278"/>
-      <c r="D2" s="278"/>
-      <c r="E2" s="278"/>
-      <c r="F2" s="278"/>
-      <c r="G2" s="278"/>
-      <c r="H2" s="278"/>
-      <c r="I2" s="278"/>
-      <c r="J2" s="278"/>
-      <c r="K2" s="278"/>
-      <c r="L2" s="278"/>
-      <c r="M2" s="278"/>
-      <c r="N2" s="278"/>
-      <c r="O2" s="278"/>
-      <c r="P2" s="278"/>
-      <c r="Q2" s="278"/>
-      <c r="R2" s="278"/>
-      <c r="S2" s="278"/>
+      <c r="B2" s="279"/>
+      <c r="C2" s="279"/>
+      <c r="D2" s="279"/>
+      <c r="E2" s="279"/>
+      <c r="F2" s="279"/>
+      <c r="G2" s="279"/>
+      <c r="H2" s="279"/>
+      <c r="I2" s="279"/>
+      <c r="J2" s="279"/>
+      <c r="K2" s="279"/>
+      <c r="L2" s="279"/>
+      <c r="M2" s="279"/>
+      <c r="N2" s="279"/>
+      <c r="O2" s="279"/>
+      <c r="P2" s="279"/>
+      <c r="Q2" s="279"/>
+      <c r="R2" s="279"/>
+      <c r="S2" s="279"/>
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="284" t="s">
+      <c r="A4" s="285" t="s">
         <v>451</v>
       </c>
-      <c r="B4" s="278"/>
-      <c r="C4" s="278"/>
-      <c r="D4" s="278"/>
-      <c r="E4" s="278"/>
-      <c r="F4" s="278"/>
-      <c r="G4" s="278"/>
-      <c r="H4" s="278"/>
-      <c r="I4" s="278"/>
-      <c r="J4" s="278"/>
-      <c r="K4" s="278"/>
-      <c r="L4" s="278"/>
-      <c r="M4" s="278"/>
-      <c r="N4" s="278"/>
-      <c r="O4" s="278"/>
-      <c r="P4" s="278"/>
-      <c r="Q4" s="278"/>
-      <c r="R4" s="278"/>
-      <c r="S4" s="278"/>
+      <c r="B4" s="279"/>
+      <c r="C4" s="279"/>
+      <c r="D4" s="279"/>
+      <c r="E4" s="279"/>
+      <c r="F4" s="279"/>
+      <c r="G4" s="279"/>
+      <c r="H4" s="279"/>
+      <c r="I4" s="279"/>
+      <c r="J4" s="279"/>
+      <c r="K4" s="279"/>
+      <c r="L4" s="279"/>
+      <c r="M4" s="279"/>
+      <c r="N4" s="279"/>
+      <c r="O4" s="279"/>
+      <c r="P4" s="279"/>
+      <c r="Q4" s="279"/>
+      <c r="R4" s="279"/>
+      <c r="S4" s="279"/>
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="37" t="s">
         <v>452</v>
       </c>
-      <c r="B5" s="274" t="s">
+      <c r="B5" s="275" t="s">
         <v>453</v>
       </c>
-      <c r="C5" s="275"/>
-      <c r="D5" s="276"/>
-      <c r="E5" s="279" t="s">
+      <c r="C5" s="276"/>
+      <c r="D5" s="277"/>
+      <c r="E5" s="280" t="s">
         <v>454</v>
       </c>
-      <c r="F5" s="275"/>
-      <c r="G5" s="276"/>
-      <c r="H5" s="279" t="s">
+      <c r="F5" s="276"/>
+      <c r="G5" s="277"/>
+      <c r="H5" s="280" t="s">
         <v>455</v>
       </c>
-      <c r="I5" s="275"/>
-      <c r="J5" s="276"/>
-      <c r="K5" s="274" t="s">
+      <c r="I5" s="276"/>
+      <c r="J5" s="277"/>
+      <c r="K5" s="275" t="s">
         <v>456</v>
       </c>
-      <c r="L5" s="275"/>
-      <c r="M5" s="276"/>
-      <c r="N5" s="281" t="s">
+      <c r="L5" s="276"/>
+      <c r="M5" s="277"/>
+      <c r="N5" s="282" t="s">
         <v>457</v>
       </c>
-      <c r="O5" s="275"/>
-      <c r="P5" s="276"/>
-      <c r="Q5" s="281" t="s">
+      <c r="O5" s="276"/>
+      <c r="P5" s="277"/>
+      <c r="Q5" s="282" t="s">
         <v>458</v>
       </c>
-      <c r="R5" s="275"/>
-      <c r="S5" s="276"/>
+      <c r="R5" s="276"/>
+      <c r="S5" s="277"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="277" t="s">
+      <c r="B6" s="278" t="s">
         <v>459</v>
       </c>
-      <c r="C6" s="278"/>
-      <c r="D6" s="278"/>
-      <c r="E6" s="278"/>
-      <c r="F6" s="278"/>
-      <c r="G6" s="278"/>
-      <c r="H6" s="278"/>
-      <c r="I6" s="278"/>
-      <c r="J6" s="278"/>
-      <c r="K6" s="278"/>
-      <c r="L6" s="278"/>
-      <c r="M6" s="278"/>
-      <c r="N6" s="278"/>
-      <c r="O6" s="278"/>
-      <c r="P6" s="278"/>
-      <c r="Q6" s="278"/>
-      <c r="R6" s="278"/>
-      <c r="S6" s="278"/>
+      <c r="C6" s="279"/>
+      <c r="D6" s="279"/>
+      <c r="E6" s="279"/>
+      <c r="F6" s="279"/>
+      <c r="G6" s="279"/>
+      <c r="H6" s="279"/>
+      <c r="I6" s="279"/>
+      <c r="J6" s="279"/>
+      <c r="K6" s="279"/>
+      <c r="L6" s="279"/>
+      <c r="M6" s="279"/>
+      <c r="N6" s="279"/>
+      <c r="O6" s="279"/>
+      <c r="P6" s="279"/>
+      <c r="Q6" s="279"/>
+      <c r="R6" s="279"/>
+      <c r="S6" s="279"/>
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="284" t="s">
+      <c r="A7" s="285" t="s">
         <v>460</v>
       </c>
-      <c r="B7" s="278"/>
-      <c r="C7" s="278"/>
-      <c r="D7" s="278"/>
-      <c r="E7" s="278"/>
-      <c r="F7" s="278"/>
-      <c r="G7" s="278"/>
-      <c r="H7" s="278"/>
-      <c r="I7" s="278"/>
-      <c r="J7" s="278"/>
-      <c r="K7" s="278"/>
-      <c r="L7" s="278"/>
-      <c r="M7" s="278"/>
-      <c r="N7" s="278"/>
-      <c r="O7" s="278"/>
-      <c r="P7" s="278"/>
-      <c r="Q7" s="278"/>
-      <c r="R7" s="278"/>
-      <c r="S7" s="278"/>
+      <c r="B7" s="279"/>
+      <c r="C7" s="279"/>
+      <c r="D7" s="279"/>
+      <c r="E7" s="279"/>
+      <c r="F7" s="279"/>
+      <c r="G7" s="279"/>
+      <c r="H7" s="279"/>
+      <c r="I7" s="279"/>
+      <c r="J7" s="279"/>
+      <c r="K7" s="279"/>
+      <c r="L7" s="279"/>
+      <c r="M7" s="279"/>
+      <c r="N7" s="279"/>
+      <c r="O7" s="279"/>
+      <c r="P7" s="279"/>
+      <c r="Q7" s="279"/>
+      <c r="R7" s="279"/>
+      <c r="S7" s="279"/>
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="37" t="s">
         <v>461</v>
       </c>
-      <c r="B8" s="287" t="s">
+      <c r="B8" s="288" t="s">
         <v>462</v>
       </c>
-      <c r="C8" s="275"/>
-      <c r="D8" s="275"/>
-      <c r="E8" s="275"/>
-      <c r="F8" s="275"/>
-      <c r="G8" s="275"/>
-      <c r="H8" s="275"/>
-      <c r="I8" s="275"/>
-      <c r="J8" s="276"/>
-      <c r="K8" s="287" t="s">
+      <c r="C8" s="276"/>
+      <c r="D8" s="276"/>
+      <c r="E8" s="276"/>
+      <c r="F8" s="276"/>
+      <c r="G8" s="276"/>
+      <c r="H8" s="276"/>
+      <c r="I8" s="276"/>
+      <c r="J8" s="277"/>
+      <c r="K8" s="288" t="s">
         <v>463</v>
       </c>
-      <c r="L8" s="275"/>
-      <c r="M8" s="275"/>
-      <c r="N8" s="275"/>
-      <c r="O8" s="275"/>
-      <c r="P8" s="275"/>
-      <c r="Q8" s="275"/>
-      <c r="R8" s="275"/>
-      <c r="S8" s="276"/>
+      <c r="L8" s="276"/>
+      <c r="M8" s="276"/>
+      <c r="N8" s="276"/>
+      <c r="O8" s="276"/>
+      <c r="P8" s="276"/>
+      <c r="Q8" s="276"/>
+      <c r="R8" s="276"/>
+      <c r="S8" s="277"/>
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B9" s="277" t="s">
+      <c r="B9" s="278" t="s">
         <v>459</v>
       </c>
-      <c r="C9" s="278"/>
-      <c r="D9" s="278"/>
-      <c r="E9" s="278"/>
-      <c r="F9" s="278"/>
-      <c r="G9" s="278"/>
-      <c r="H9" s="278"/>
-      <c r="I9" s="278"/>
-      <c r="J9" s="278"/>
-      <c r="K9" s="278"/>
-      <c r="L9" s="278"/>
-      <c r="M9" s="278"/>
-      <c r="N9" s="278"/>
-      <c r="O9" s="278"/>
-      <c r="P9" s="278"/>
-      <c r="Q9" s="278"/>
-      <c r="R9" s="278"/>
-      <c r="S9" s="278"/>
+      <c r="C9" s="279"/>
+      <c r="D9" s="279"/>
+      <c r="E9" s="279"/>
+      <c r="F9" s="279"/>
+      <c r="G9" s="279"/>
+      <c r="H9" s="279"/>
+      <c r="I9" s="279"/>
+      <c r="J9" s="279"/>
+      <c r="K9" s="279"/>
+      <c r="L9" s="279"/>
+      <c r="M9" s="279"/>
+      <c r="N9" s="279"/>
+      <c r="O9" s="279"/>
+      <c r="P9" s="279"/>
+      <c r="Q9" s="279"/>
+      <c r="R9" s="279"/>
+      <c r="S9" s="279"/>
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="284" t="s">
+      <c r="A10" s="285" t="s">
         <v>464</v>
       </c>
-      <c r="B10" s="278"/>
-      <c r="C10" s="278"/>
-      <c r="D10" s="278"/>
-      <c r="E10" s="278"/>
-      <c r="F10" s="278"/>
-      <c r="G10" s="278"/>
-      <c r="H10" s="278"/>
-      <c r="I10" s="278"/>
-      <c r="J10" s="278"/>
-      <c r="K10" s="278"/>
-      <c r="L10" s="278"/>
-      <c r="M10" s="278"/>
-      <c r="N10" s="278"/>
-      <c r="O10" s="278"/>
-      <c r="P10" s="278"/>
-      <c r="Q10" s="278"/>
-      <c r="R10" s="278"/>
-      <c r="S10" s="278"/>
+      <c r="B10" s="279"/>
+      <c r="C10" s="279"/>
+      <c r="D10" s="279"/>
+      <c r="E10" s="279"/>
+      <c r="F10" s="279"/>
+      <c r="G10" s="279"/>
+      <c r="H10" s="279"/>
+      <c r="I10" s="279"/>
+      <c r="J10" s="279"/>
+      <c r="K10" s="279"/>
+      <c r="L10" s="279"/>
+      <c r="M10" s="279"/>
+      <c r="N10" s="279"/>
+      <c r="O10" s="279"/>
+      <c r="P10" s="279"/>
+      <c r="Q10" s="279"/>
+      <c r="R10" s="279"/>
+      <c r="S10" s="279"/>
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="37" t="s">
         <v>465</v>
       </c>
-      <c r="B11" s="274" t="s">
+      <c r="B11" s="275" t="s">
         <v>466</v>
       </c>
-      <c r="C11" s="275"/>
-      <c r="D11" s="276"/>
-      <c r="E11" s="274" t="s">
+      <c r="C11" s="276"/>
+      <c r="D11" s="277"/>
+      <c r="E11" s="275" t="s">
         <v>467</v>
       </c>
-      <c r="F11" s="275"/>
-      <c r="G11" s="276"/>
-      <c r="H11" s="274" t="s">
+      <c r="F11" s="276"/>
+      <c r="G11" s="277"/>
+      <c r="H11" s="275" t="s">
         <v>468</v>
       </c>
-      <c r="I11" s="275"/>
-      <c r="J11" s="276"/>
-      <c r="K11" s="279" t="s">
+      <c r="I11" s="276"/>
+      <c r="J11" s="277"/>
+      <c r="K11" s="280" t="s">
         <v>469</v>
       </c>
-      <c r="L11" s="275"/>
-      <c r="M11" s="276"/>
-      <c r="N11" s="274" t="s">
+      <c r="L11" s="276"/>
+      <c r="M11" s="277"/>
+      <c r="N11" s="275" t="s">
         <v>470</v>
       </c>
-      <c r="O11" s="275"/>
-      <c r="P11" s="276"/>
-      <c r="Q11" s="274" t="s">
+      <c r="O11" s="276"/>
+      <c r="P11" s="277"/>
+      <c r="Q11" s="275" t="s">
         <v>471</v>
       </c>
-      <c r="R11" s="275"/>
-      <c r="S11" s="276"/>
+      <c r="R11" s="276"/>
+      <c r="S11" s="277"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B12" s="277" t="s">
+      <c r="B12" s="278" t="s">
         <v>459</v>
       </c>
-      <c r="C12" s="278"/>
-      <c r="D12" s="278"/>
-      <c r="E12" s="278"/>
-      <c r="F12" s="278"/>
-      <c r="G12" s="278"/>
-      <c r="H12" s="278"/>
-      <c r="I12" s="278"/>
-      <c r="J12" s="278"/>
-      <c r="K12" s="278"/>
-      <c r="L12" s="278"/>
-      <c r="M12" s="278"/>
-      <c r="N12" s="278"/>
-      <c r="O12" s="278"/>
-      <c r="P12" s="278"/>
-      <c r="Q12" s="278"/>
-      <c r="R12" s="278"/>
-      <c r="S12" s="278"/>
+      <c r="C12" s="279"/>
+      <c r="D12" s="279"/>
+      <c r="E12" s="279"/>
+      <c r="F12" s="279"/>
+      <c r="G12" s="279"/>
+      <c r="H12" s="279"/>
+      <c r="I12" s="279"/>
+      <c r="J12" s="279"/>
+      <c r="K12" s="279"/>
+      <c r="L12" s="279"/>
+      <c r="M12" s="279"/>
+      <c r="N12" s="279"/>
+      <c r="O12" s="279"/>
+      <c r="P12" s="279"/>
+      <c r="Q12" s="279"/>
+      <c r="R12" s="279"/>
+      <c r="S12" s="279"/>
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="284" t="s">
+      <c r="A13" s="285" t="s">
         <v>472</v>
       </c>
-      <c r="B13" s="278"/>
-      <c r="C13" s="278"/>
-      <c r="D13" s="278"/>
-      <c r="E13" s="278"/>
-      <c r="F13" s="278"/>
-      <c r="G13" s="278"/>
-      <c r="H13" s="278"/>
-      <c r="I13" s="278"/>
-      <c r="J13" s="278"/>
-      <c r="K13" s="278"/>
-      <c r="L13" s="278"/>
-      <c r="M13" s="278"/>
-      <c r="N13" s="278"/>
-      <c r="O13" s="278"/>
-      <c r="P13" s="278"/>
-      <c r="Q13" s="278"/>
-      <c r="R13" s="278"/>
-      <c r="S13" s="278"/>
+      <c r="B13" s="279"/>
+      <c r="C13" s="279"/>
+      <c r="D13" s="279"/>
+      <c r="E13" s="279"/>
+      <c r="F13" s="279"/>
+      <c r="G13" s="279"/>
+      <c r="H13" s="279"/>
+      <c r="I13" s="279"/>
+      <c r="J13" s="279"/>
+      <c r="K13" s="279"/>
+      <c r="L13" s="279"/>
+      <c r="M13" s="279"/>
+      <c r="N13" s="279"/>
+      <c r="O13" s="279"/>
+      <c r="P13" s="279"/>
+      <c r="Q13" s="279"/>
+      <c r="R13" s="279"/>
+      <c r="S13" s="279"/>
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="37" t="s">
         <v>473</v>
       </c>
-      <c r="B14" s="282" t="s">
+      <c r="B14" s="283" t="s">
         <v>474</v>
       </c>
-      <c r="C14" s="275"/>
-      <c r="D14" s="275"/>
-      <c r="E14" s="275"/>
-      <c r="F14" s="275"/>
-      <c r="G14" s="276"/>
-      <c r="H14" s="282" t="s">
+      <c r="C14" s="276"/>
+      <c r="D14" s="276"/>
+      <c r="E14" s="276"/>
+      <c r="F14" s="276"/>
+      <c r="G14" s="277"/>
+      <c r="H14" s="283" t="s">
         <v>475</v>
       </c>
-      <c r="I14" s="275"/>
-      <c r="J14" s="275"/>
-      <c r="K14" s="275"/>
-      <c r="L14" s="275"/>
-      <c r="M14" s="276"/>
-      <c r="N14" s="282" t="s">
+      <c r="I14" s="276"/>
+      <c r="J14" s="276"/>
+      <c r="K14" s="276"/>
+      <c r="L14" s="276"/>
+      <c r="M14" s="277"/>
+      <c r="N14" s="283" t="s">
         <v>476</v>
       </c>
-      <c r="O14" s="275"/>
-      <c r="P14" s="276"/>
-      <c r="Q14" s="279" t="s">
+      <c r="O14" s="276"/>
+      <c r="P14" s="277"/>
+      <c r="Q14" s="280" t="s">
         <v>477</v>
       </c>
-      <c r="R14" s="275"/>
-      <c r="S14" s="276"/>
+      <c r="R14" s="276"/>
+      <c r="S14" s="277"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B15" s="277" t="s">
+      <c r="B15" s="278" t="s">
         <v>478</v>
       </c>
-      <c r="C15" s="278"/>
-      <c r="D15" s="278"/>
-      <c r="E15" s="278"/>
-      <c r="F15" s="278"/>
-      <c r="G15" s="278"/>
-      <c r="H15" s="278"/>
-      <c r="I15" s="278"/>
-      <c r="J15" s="278"/>
-      <c r="K15" s="278"/>
-      <c r="L15" s="278"/>
-      <c r="M15" s="278"/>
-      <c r="N15" s="278"/>
-      <c r="O15" s="278"/>
-      <c r="P15" s="278"/>
-      <c r="Q15" s="278"/>
-      <c r="R15" s="278"/>
-      <c r="S15" s="278"/>
+      <c r="C15" s="279"/>
+      <c r="D15" s="279"/>
+      <c r="E15" s="279"/>
+      <c r="F15" s="279"/>
+      <c r="G15" s="279"/>
+      <c r="H15" s="279"/>
+      <c r="I15" s="279"/>
+      <c r="J15" s="279"/>
+      <c r="K15" s="279"/>
+      <c r="L15" s="279"/>
+      <c r="M15" s="279"/>
+      <c r="N15" s="279"/>
+      <c r="O15" s="279"/>
+      <c r="P15" s="279"/>
+      <c r="Q15" s="279"/>
+      <c r="R15" s="279"/>
+      <c r="S15" s="279"/>
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="284" t="s">
+      <c r="A16" s="285" t="s">
         <v>479</v>
       </c>
-      <c r="B16" s="278"/>
-      <c r="C16" s="278"/>
-      <c r="D16" s="278"/>
-      <c r="E16" s="278"/>
-      <c r="F16" s="278"/>
-      <c r="G16" s="278"/>
-      <c r="H16" s="278"/>
-      <c r="I16" s="278"/>
-      <c r="J16" s="278"/>
-      <c r="K16" s="278"/>
-      <c r="L16" s="278"/>
-      <c r="M16" s="278"/>
-      <c r="N16" s="278"/>
-      <c r="O16" s="278"/>
-      <c r="P16" s="278"/>
-      <c r="Q16" s="278"/>
-      <c r="R16" s="278"/>
-      <c r="S16" s="278"/>
+      <c r="B16" s="279"/>
+      <c r="C16" s="279"/>
+      <c r="D16" s="279"/>
+      <c r="E16" s="279"/>
+      <c r="F16" s="279"/>
+      <c r="G16" s="279"/>
+      <c r="H16" s="279"/>
+      <c r="I16" s="279"/>
+      <c r="J16" s="279"/>
+      <c r="K16" s="279"/>
+      <c r="L16" s="279"/>
+      <c r="M16" s="279"/>
+      <c r="N16" s="279"/>
+      <c r="O16" s="279"/>
+      <c r="P16" s="279"/>
+      <c r="Q16" s="279"/>
+      <c r="R16" s="279"/>
+      <c r="S16" s="279"/>
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="37" t="s">
         <v>480</v>
       </c>
-      <c r="B17" s="283" t="s">
+      <c r="B17" s="284" t="s">
         <v>481</v>
       </c>
-      <c r="C17" s="275"/>
-      <c r="D17" s="275"/>
-      <c r="E17" s="275"/>
-      <c r="F17" s="275"/>
-      <c r="G17" s="276"/>
-      <c r="H17" s="283" t="s">
+      <c r="C17" s="276"/>
+      <c r="D17" s="276"/>
+      <c r="E17" s="276"/>
+      <c r="F17" s="276"/>
+      <c r="G17" s="277"/>
+      <c r="H17" s="284" t="s">
         <v>482</v>
       </c>
-      <c r="I17" s="275"/>
-      <c r="J17" s="276"/>
-      <c r="K17" s="283" t="s">
+      <c r="I17" s="276"/>
+      <c r="J17" s="277"/>
+      <c r="K17" s="284" t="s">
         <v>483</v>
       </c>
-      <c r="L17" s="275"/>
-      <c r="M17" s="276"/>
-      <c r="N17" s="283" t="s">
+      <c r="L17" s="276"/>
+      <c r="M17" s="277"/>
+      <c r="N17" s="284" t="s">
         <v>484</v>
       </c>
-      <c r="O17" s="275"/>
-      <c r="P17" s="276"/>
-      <c r="Q17" s="283" t="s">
+      <c r="O17" s="276"/>
+      <c r="P17" s="277"/>
+      <c r="Q17" s="284" t="s">
         <v>485</v>
       </c>
-      <c r="R17" s="275"/>
-      <c r="S17" s="276"/>
+      <c r="R17" s="276"/>
+      <c r="S17" s="277"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="277" t="s">
+      <c r="B18" s="278" t="s">
         <v>459</v>
       </c>
-      <c r="C18" s="278"/>
-      <c r="D18" s="278"/>
-      <c r="E18" s="278"/>
-      <c r="F18" s="278"/>
-      <c r="G18" s="278"/>
-      <c r="H18" s="278"/>
-      <c r="I18" s="278"/>
-      <c r="J18" s="278"/>
-      <c r="K18" s="278"/>
-      <c r="L18" s="278"/>
-      <c r="M18" s="278"/>
-      <c r="N18" s="278"/>
-      <c r="O18" s="278"/>
-      <c r="P18" s="278"/>
-      <c r="Q18" s="278"/>
-      <c r="R18" s="278"/>
-      <c r="S18" s="278"/>
+      <c r="C18" s="279"/>
+      <c r="D18" s="279"/>
+      <c r="E18" s="279"/>
+      <c r="F18" s="279"/>
+      <c r="G18" s="279"/>
+      <c r="H18" s="279"/>
+      <c r="I18" s="279"/>
+      <c r="J18" s="279"/>
+      <c r="K18" s="279"/>
+      <c r="L18" s="279"/>
+      <c r="M18" s="279"/>
+      <c r="N18" s="279"/>
+      <c r="O18" s="279"/>
+      <c r="P18" s="279"/>
+      <c r="Q18" s="279"/>
+      <c r="R18" s="279"/>
+      <c r="S18" s="279"/>
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="284" t="s">
+      <c r="A19" s="285" t="s">
         <v>486</v>
       </c>
-      <c r="B19" s="278"/>
-      <c r="C19" s="278"/>
-      <c r="D19" s="278"/>
-      <c r="E19" s="278"/>
-      <c r="F19" s="278"/>
-      <c r="G19" s="278"/>
-      <c r="H19" s="278"/>
-      <c r="I19" s="278"/>
-      <c r="J19" s="278"/>
-      <c r="K19" s="278"/>
-      <c r="L19" s="278"/>
-      <c r="M19" s="278"/>
-      <c r="N19" s="278"/>
-      <c r="O19" s="278"/>
-      <c r="P19" s="278"/>
-      <c r="Q19" s="278"/>
-      <c r="R19" s="278"/>
-      <c r="S19" s="278"/>
+      <c r="B19" s="279"/>
+      <c r="C19" s="279"/>
+      <c r="D19" s="279"/>
+      <c r="E19" s="279"/>
+      <c r="F19" s="279"/>
+      <c r="G19" s="279"/>
+      <c r="H19" s="279"/>
+      <c r="I19" s="279"/>
+      <c r="J19" s="279"/>
+      <c r="K19" s="279"/>
+      <c r="L19" s="279"/>
+      <c r="M19" s="279"/>
+      <c r="N19" s="279"/>
+      <c r="O19" s="279"/>
+      <c r="P19" s="279"/>
+      <c r="Q19" s="279"/>
+      <c r="R19" s="279"/>
+      <c r="S19" s="279"/>
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="37" t="s">
         <v>487</v>
       </c>
-      <c r="B20" s="285" t="s">
+      <c r="B20" s="286" t="s">
         <v>488</v>
       </c>
-      <c r="C20" s="275"/>
-      <c r="D20" s="275"/>
-      <c r="E20" s="275"/>
-      <c r="F20" s="275"/>
-      <c r="G20" s="276"/>
-      <c r="H20" s="285" t="s">
+      <c r="C20" s="276"/>
+      <c r="D20" s="276"/>
+      <c r="E20" s="276"/>
+      <c r="F20" s="276"/>
+      <c r="G20" s="277"/>
+      <c r="H20" s="286" t="s">
         <v>489</v>
       </c>
-      <c r="I20" s="275"/>
-      <c r="J20" s="275"/>
-      <c r="K20" s="275"/>
-      <c r="L20" s="275"/>
-      <c r="M20" s="276"/>
-      <c r="N20" s="285" t="s">
+      <c r="I20" s="276"/>
+      <c r="J20" s="276"/>
+      <c r="K20" s="276"/>
+      <c r="L20" s="276"/>
+      <c r="M20" s="277"/>
+      <c r="N20" s="286" t="s">
         <v>490</v>
       </c>
-      <c r="O20" s="275"/>
-      <c r="P20" s="275"/>
-      <c r="Q20" s="275"/>
-      <c r="R20" s="275"/>
-      <c r="S20" s="276"/>
+      <c r="O20" s="276"/>
+      <c r="P20" s="276"/>
+      <c r="Q20" s="276"/>
+      <c r="R20" s="276"/>
+      <c r="S20" s="277"/>
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B21" s="277" t="s">
+      <c r="B21" s="278" t="s">
         <v>459</v>
       </c>
-      <c r="C21" s="278"/>
-      <c r="D21" s="278"/>
-      <c r="E21" s="278"/>
-      <c r="F21" s="278"/>
-      <c r="G21" s="278"/>
-      <c r="H21" s="278"/>
-      <c r="I21" s="278"/>
-      <c r="J21" s="278"/>
-      <c r="K21" s="278"/>
-      <c r="L21" s="278"/>
-      <c r="M21" s="278"/>
-      <c r="N21" s="278"/>
-      <c r="O21" s="278"/>
-      <c r="P21" s="278"/>
-      <c r="Q21" s="278"/>
-      <c r="R21" s="278"/>
-      <c r="S21" s="278"/>
+      <c r="C21" s="279"/>
+      <c r="D21" s="279"/>
+      <c r="E21" s="279"/>
+      <c r="F21" s="279"/>
+      <c r="G21" s="279"/>
+      <c r="H21" s="279"/>
+      <c r="I21" s="279"/>
+      <c r="J21" s="279"/>
+      <c r="K21" s="279"/>
+      <c r="L21" s="279"/>
+      <c r="M21" s="279"/>
+      <c r="N21" s="279"/>
+      <c r="O21" s="279"/>
+      <c r="P21" s="279"/>
+      <c r="Q21" s="279"/>
+      <c r="R21" s="279"/>
+      <c r="S21" s="279"/>
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="284" t="s">
+      <c r="A22" s="285" t="s">
         <v>491</v>
       </c>
-      <c r="B22" s="278"/>
-      <c r="C22" s="278"/>
-      <c r="D22" s="278"/>
-      <c r="E22" s="278"/>
-      <c r="F22" s="278"/>
-      <c r="G22" s="278"/>
-      <c r="H22" s="278"/>
-      <c r="I22" s="278"/>
-      <c r="J22" s="278"/>
-      <c r="K22" s="278"/>
-      <c r="L22" s="278"/>
-      <c r="M22" s="278"/>
-      <c r="N22" s="278"/>
-      <c r="O22" s="278"/>
-      <c r="P22" s="278"/>
-      <c r="Q22" s="278"/>
-      <c r="R22" s="278"/>
-      <c r="S22" s="278"/>
+      <c r="B22" s="279"/>
+      <c r="C22" s="279"/>
+      <c r="D22" s="279"/>
+      <c r="E22" s="279"/>
+      <c r="F22" s="279"/>
+      <c r="G22" s="279"/>
+      <c r="H22" s="279"/>
+      <c r="I22" s="279"/>
+      <c r="J22" s="279"/>
+      <c r="K22" s="279"/>
+      <c r="L22" s="279"/>
+      <c r="M22" s="279"/>
+      <c r="N22" s="279"/>
+      <c r="O22" s="279"/>
+      <c r="P22" s="279"/>
+      <c r="Q22" s="279"/>
+      <c r="R22" s="279"/>
+      <c r="S22" s="279"/>
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="37" t="s">
         <v>492</v>
       </c>
-      <c r="B23" s="285" t="s">
+      <c r="B23" s="286" t="s">
         <v>493</v>
       </c>
-      <c r="C23" s="275"/>
-      <c r="D23" s="275"/>
-      <c r="E23" s="275"/>
-      <c r="F23" s="275"/>
-      <c r="G23" s="276"/>
-      <c r="H23" s="285" t="s">
+      <c r="C23" s="276"/>
+      <c r="D23" s="276"/>
+      <c r="E23" s="276"/>
+      <c r="F23" s="276"/>
+      <c r="G23" s="277"/>
+      <c r="H23" s="286" t="s">
         <v>494</v>
       </c>
-      <c r="I23" s="275"/>
-      <c r="J23" s="276"/>
-      <c r="K23" s="285" t="s">
+      <c r="I23" s="276"/>
+      <c r="J23" s="277"/>
+      <c r="K23" s="286" t="s">
         <v>495</v>
       </c>
-      <c r="L23" s="275"/>
-      <c r="M23" s="276"/>
-      <c r="N23" s="285" t="s">
+      <c r="L23" s="276"/>
+      <c r="M23" s="277"/>
+      <c r="N23" s="286" t="s">
         <v>496</v>
       </c>
-      <c r="O23" s="275"/>
-      <c r="P23" s="276"/>
-      <c r="Q23" s="281" t="s">
+      <c r="O23" s="276"/>
+      <c r="P23" s="277"/>
+      <c r="Q23" s="282" t="s">
         <v>497</v>
       </c>
-      <c r="R23" s="275"/>
-      <c r="S23" s="276"/>
+      <c r="R23" s="276"/>
+      <c r="S23" s="277"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="290" t="s">
+      <c r="A26" s="291" t="s">
         <v>498</v>
       </c>
-      <c r="B26" s="278"/>
-      <c r="C26" s="278"/>
-      <c r="D26" s="278"/>
-      <c r="E26" s="278"/>
-      <c r="F26" s="278"/>
-      <c r="G26" s="278"/>
-      <c r="H26" s="278"/>
-      <c r="I26" s="278"/>
-      <c r="J26" s="278"/>
-      <c r="K26" s="278"/>
-      <c r="L26" s="278"/>
-      <c r="M26" s="278"/>
-      <c r="N26" s="278"/>
-      <c r="O26" s="278"/>
-      <c r="P26" s="278"/>
-      <c r="Q26" s="278"/>
-      <c r="R26" s="278"/>
-      <c r="S26" s="278"/>
+      <c r="B26" s="279"/>
+      <c r="C26" s="279"/>
+      <c r="D26" s="279"/>
+      <c r="E26" s="279"/>
+      <c r="F26" s="279"/>
+      <c r="G26" s="279"/>
+      <c r="H26" s="279"/>
+      <c r="I26" s="279"/>
+      <c r="J26" s="279"/>
+      <c r="K26" s="279"/>
+      <c r="L26" s="279"/>
+      <c r="M26" s="279"/>
+      <c r="N26" s="279"/>
+      <c r="O26" s="279"/>
+      <c r="P26" s="279"/>
+      <c r="Q26" s="279"/>
+      <c r="R26" s="279"/>
+      <c r="S26" s="279"/>
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="37" t="s">
         <v>499</v>
       </c>
-      <c r="B27" s="274" t="s">
+      <c r="B27" s="275" t="s">
         <v>500</v>
       </c>
-      <c r="C27" s="275"/>
-      <c r="D27" s="276"/>
-      <c r="E27" s="274" t="s">
+      <c r="C27" s="276"/>
+      <c r="D27" s="277"/>
+      <c r="E27" s="275" t="s">
         <v>501</v>
       </c>
-      <c r="F27" s="275"/>
-      <c r="G27" s="276"/>
-      <c r="H27" s="282" t="s">
+      <c r="F27" s="276"/>
+      <c r="G27" s="277"/>
+      <c r="H27" s="283" t="s">
         <v>502</v>
       </c>
-      <c r="I27" s="275"/>
-      <c r="J27" s="276"/>
-      <c r="K27" s="283" t="s">
+      <c r="I27" s="276"/>
+      <c r="J27" s="277"/>
+      <c r="K27" s="284" t="s">
         <v>503</v>
       </c>
-      <c r="L27" s="275"/>
-      <c r="M27" s="276"/>
-      <c r="N27" s="283" t="s">
+      <c r="L27" s="276"/>
+      <c r="M27" s="277"/>
+      <c r="N27" s="284" t="s">
         <v>504</v>
       </c>
-      <c r="O27" s="275"/>
-      <c r="P27" s="276"/>
-      <c r="Q27" s="282" t="s">
+      <c r="O27" s="276"/>
+      <c r="P27" s="277"/>
+      <c r="Q27" s="283" t="s">
         <v>505</v>
       </c>
-      <c r="R27" s="275"/>
-      <c r="S27" s="276"/>
+      <c r="R27" s="276"/>
+      <c r="S27" s="277"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="284" t="s">
+      <c r="A30" s="285" t="s">
         <v>506</v>
       </c>
-      <c r="B30" s="278"/>
-      <c r="C30" s="278"/>
-      <c r="D30" s="278"/>
-      <c r="E30" s="278"/>
-      <c r="F30" s="278"/>
-      <c r="G30" s="278"/>
-      <c r="H30" s="278"/>
-      <c r="I30" s="278"/>
-      <c r="J30" s="278"/>
-      <c r="K30" s="278"/>
-      <c r="L30" s="278"/>
-      <c r="M30" s="278"/>
-      <c r="N30" s="278"/>
-      <c r="O30" s="278"/>
-      <c r="P30" s="278"/>
-      <c r="Q30" s="278"/>
-      <c r="R30" s="278"/>
-      <c r="S30" s="278"/>
+      <c r="B30" s="279"/>
+      <c r="C30" s="279"/>
+      <c r="D30" s="279"/>
+      <c r="E30" s="279"/>
+      <c r="F30" s="279"/>
+      <c r="G30" s="279"/>
+      <c r="H30" s="279"/>
+      <c r="I30" s="279"/>
+      <c r="J30" s="279"/>
+      <c r="K30" s="279"/>
+      <c r="L30" s="279"/>
+      <c r="M30" s="279"/>
+      <c r="N30" s="279"/>
+      <c r="O30" s="279"/>
+      <c r="P30" s="279"/>
+      <c r="Q30" s="279"/>
+      <c r="R30" s="279"/>
+      <c r="S30" s="279"/>
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="280" t="s">
+      <c r="A31" s="281" t="s">
         <v>507</v>
       </c>
-      <c r="B31" s="278"/>
-      <c r="C31" s="278"/>
-      <c r="D31" s="278"/>
-      <c r="E31" s="278"/>
-      <c r="F31" s="278"/>
-      <c r="G31" s="278"/>
-      <c r="H31" s="278"/>
-      <c r="I31" s="278"/>
-      <c r="J31" s="278"/>
-      <c r="K31" s="278"/>
-      <c r="L31" s="278"/>
-      <c r="M31" s="278"/>
-      <c r="N31" s="278"/>
-      <c r="O31" s="278"/>
-      <c r="P31" s="278"/>
-      <c r="Q31" s="278"/>
-      <c r="R31" s="278"/>
-      <c r="S31" s="278"/>
+      <c r="B31" s="279"/>
+      <c r="C31" s="279"/>
+      <c r="D31" s="279"/>
+      <c r="E31" s="279"/>
+      <c r="F31" s="279"/>
+      <c r="G31" s="279"/>
+      <c r="H31" s="279"/>
+      <c r="I31" s="279"/>
+      <c r="J31" s="279"/>
+      <c r="K31" s="279"/>
+      <c r="L31" s="279"/>
+      <c r="M31" s="279"/>
+      <c r="N31" s="279"/>
+      <c r="O31" s="279"/>
+      <c r="P31" s="279"/>
+      <c r="Q31" s="279"/>
+      <c r="R31" s="279"/>
+      <c r="S31" s="279"/>
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="280" t="s">
+      <c r="A32" s="281" t="s">
         <v>508</v>
       </c>
-      <c r="B32" s="278"/>
-      <c r="C32" s="278"/>
-      <c r="D32" s="278"/>
-      <c r="E32" s="278"/>
-      <c r="F32" s="278"/>
-      <c r="G32" s="278"/>
-      <c r="H32" s="278"/>
-      <c r="I32" s="278"/>
-      <c r="J32" s="278"/>
-      <c r="K32" s="278"/>
-      <c r="L32" s="278"/>
-      <c r="M32" s="278"/>
-      <c r="N32" s="278"/>
-      <c r="O32" s="278"/>
-      <c r="P32" s="278"/>
-      <c r="Q32" s="278"/>
-      <c r="R32" s="278"/>
-      <c r="S32" s="278"/>
+      <c r="B32" s="279"/>
+      <c r="C32" s="279"/>
+      <c r="D32" s="279"/>
+      <c r="E32" s="279"/>
+      <c r="F32" s="279"/>
+      <c r="G32" s="279"/>
+      <c r="H32" s="279"/>
+      <c r="I32" s="279"/>
+      <c r="J32" s="279"/>
+      <c r="K32" s="279"/>
+      <c r="L32" s="279"/>
+      <c r="M32" s="279"/>
+      <c r="N32" s="279"/>
+      <c r="O32" s="279"/>
+      <c r="P32" s="279"/>
+      <c r="Q32" s="279"/>
+      <c r="R32" s="279"/>
+      <c r="S32" s="279"/>
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="280" t="s">
+      <c r="A33" s="281" t="s">
         <v>509</v>
       </c>
-      <c r="B33" s="278"/>
-      <c r="C33" s="278"/>
-      <c r="D33" s="278"/>
-      <c r="E33" s="278"/>
-      <c r="F33" s="278"/>
-      <c r="G33" s="278"/>
-      <c r="H33" s="278"/>
-      <c r="I33" s="278"/>
-      <c r="J33" s="278"/>
-      <c r="K33" s="278"/>
-      <c r="L33" s="278"/>
-      <c r="M33" s="278"/>
-      <c r="N33" s="278"/>
-      <c r="O33" s="278"/>
-      <c r="P33" s="278"/>
-      <c r="Q33" s="278"/>
-      <c r="R33" s="278"/>
-      <c r="S33" s="278"/>
+      <c r="B33" s="279"/>
+      <c r="C33" s="279"/>
+      <c r="D33" s="279"/>
+      <c r="E33" s="279"/>
+      <c r="F33" s="279"/>
+      <c r="G33" s="279"/>
+      <c r="H33" s="279"/>
+      <c r="I33" s="279"/>
+      <c r="J33" s="279"/>
+      <c r="K33" s="279"/>
+      <c r="L33" s="279"/>
+      <c r="M33" s="279"/>
+      <c r="N33" s="279"/>
+      <c r="O33" s="279"/>
+      <c r="P33" s="279"/>
+      <c r="Q33" s="279"/>
+      <c r="R33" s="279"/>
+      <c r="S33" s="279"/>
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="280" t="s">
+      <c r="A34" s="281" t="s">
         <v>510</v>
       </c>
-      <c r="B34" s="278"/>
-      <c r="C34" s="278"/>
-      <c r="D34" s="278"/>
-      <c r="E34" s="278"/>
-      <c r="F34" s="278"/>
-      <c r="G34" s="278"/>
-      <c r="H34" s="278"/>
-      <c r="I34" s="278"/>
-      <c r="J34" s="278"/>
-      <c r="K34" s="278"/>
-      <c r="L34" s="278"/>
-      <c r="M34" s="278"/>
-      <c r="N34" s="278"/>
-      <c r="O34" s="278"/>
-      <c r="P34" s="278"/>
-      <c r="Q34" s="278"/>
-      <c r="R34" s="278"/>
-      <c r="S34" s="278"/>
+      <c r="B34" s="279"/>
+      <c r="C34" s="279"/>
+      <c r="D34" s="279"/>
+      <c r="E34" s="279"/>
+      <c r="F34" s="279"/>
+      <c r="G34" s="279"/>
+      <c r="H34" s="279"/>
+      <c r="I34" s="279"/>
+      <c r="J34" s="279"/>
+      <c r="K34" s="279"/>
+      <c r="L34" s="279"/>
+      <c r="M34" s="279"/>
+      <c r="N34" s="279"/>
+      <c r="O34" s="279"/>
+      <c r="P34" s="279"/>
+      <c r="Q34" s="279"/>
+      <c r="R34" s="279"/>
+      <c r="S34" s="279"/>
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="280" t="s">
+      <c r="A35" s="281" t="s">
         <v>511</v>
       </c>
-      <c r="B35" s="278"/>
-      <c r="C35" s="278"/>
-      <c r="D35" s="278"/>
-      <c r="E35" s="278"/>
-      <c r="F35" s="278"/>
-      <c r="G35" s="278"/>
-      <c r="H35" s="278"/>
-      <c r="I35" s="278"/>
-      <c r="J35" s="278"/>
-      <c r="K35" s="278"/>
-      <c r="L35" s="278"/>
-      <c r="M35" s="278"/>
-      <c r="N35" s="278"/>
-      <c r="O35" s="278"/>
-      <c r="P35" s="278"/>
-      <c r="Q35" s="278"/>
-      <c r="R35" s="278"/>
-      <c r="S35" s="278"/>
+      <c r="B35" s="279"/>
+      <c r="C35" s="279"/>
+      <c r="D35" s="279"/>
+      <c r="E35" s="279"/>
+      <c r="F35" s="279"/>
+      <c r="G35" s="279"/>
+      <c r="H35" s="279"/>
+      <c r="I35" s="279"/>
+      <c r="J35" s="279"/>
+      <c r="K35" s="279"/>
+      <c r="L35" s="279"/>
+      <c r="M35" s="279"/>
+      <c r="N35" s="279"/>
+      <c r="O35" s="279"/>
+      <c r="P35" s="279"/>
+      <c r="Q35" s="279"/>
+      <c r="R35" s="279"/>
+      <c r="S35" s="279"/>
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="280" t="s">
+      <c r="A36" s="281" t="s">
         <v>512</v>
       </c>
-      <c r="B36" s="278"/>
-      <c r="C36" s="278"/>
-      <c r="D36" s="278"/>
-      <c r="E36" s="278"/>
-      <c r="F36" s="278"/>
-      <c r="G36" s="278"/>
-      <c r="H36" s="278"/>
-      <c r="I36" s="278"/>
-      <c r="J36" s="278"/>
-      <c r="K36" s="278"/>
-      <c r="L36" s="278"/>
-      <c r="M36" s="278"/>
-      <c r="N36" s="278"/>
-      <c r="O36" s="278"/>
-      <c r="P36" s="278"/>
-      <c r="Q36" s="278"/>
-      <c r="R36" s="278"/>
-      <c r="S36" s="278"/>
+      <c r="B36" s="279"/>
+      <c r="C36" s="279"/>
+      <c r="D36" s="279"/>
+      <c r="E36" s="279"/>
+      <c r="F36" s="279"/>
+      <c r="G36" s="279"/>
+      <c r="H36" s="279"/>
+      <c r="I36" s="279"/>
+      <c r="J36" s="279"/>
+      <c r="K36" s="279"/>
+      <c r="L36" s="279"/>
+      <c r="M36" s="279"/>
+      <c r="N36" s="279"/>
+      <c r="O36" s="279"/>
+      <c r="P36" s="279"/>
+      <c r="Q36" s="279"/>
+      <c r="R36" s="279"/>
+      <c r="S36" s="279"/>
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="291" t="s">
+      <c r="A37" s="292" t="s">
         <v>513</v>
       </c>
-      <c r="B37" s="278"/>
-      <c r="C37" s="278"/>
-      <c r="D37" s="278"/>
-      <c r="E37" s="278"/>
-      <c r="F37" s="278"/>
-      <c r="G37" s="278"/>
-      <c r="H37" s="278"/>
-      <c r="I37" s="278"/>
-      <c r="J37" s="278"/>
-      <c r="K37" s="278"/>
-      <c r="L37" s="278"/>
-      <c r="M37" s="278"/>
-      <c r="N37" s="278"/>
-      <c r="O37" s="278"/>
-      <c r="P37" s="278"/>
-      <c r="Q37" s="278"/>
-      <c r="R37" s="278"/>
-      <c r="S37" s="278"/>
+      <c r="B37" s="279"/>
+      <c r="C37" s="279"/>
+      <c r="D37" s="279"/>
+      <c r="E37" s="279"/>
+      <c r="F37" s="279"/>
+      <c r="G37" s="279"/>
+      <c r="H37" s="279"/>
+      <c r="I37" s="279"/>
+      <c r="J37" s="279"/>
+      <c r="K37" s="279"/>
+      <c r="L37" s="279"/>
+      <c r="M37" s="279"/>
+      <c r="N37" s="279"/>
+      <c r="O37" s="279"/>
+      <c r="P37" s="279"/>
+      <c r="Q37" s="279"/>
+      <c r="R37" s="279"/>
+      <c r="S37" s="279"/>
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="38" t="s">
         <v>447</v>
       </c>
-      <c r="B39" s="294" t="s">
+      <c r="B39" s="295" t="s">
         <v>514</v>
       </c>
-      <c r="C39" s="278"/>
-      <c r="D39" s="278"/>
-      <c r="E39" s="292" t="s">
+      <c r="C39" s="279"/>
+      <c r="D39" s="279"/>
+      <c r="E39" s="293" t="s">
         <v>515</v>
       </c>
-      <c r="F39" s="278"/>
-      <c r="G39" s="278"/>
-      <c r="H39" s="295" t="s">
+      <c r="F39" s="279"/>
+      <c r="G39" s="279"/>
+      <c r="H39" s="296" t="s">
         <v>516</v>
       </c>
-      <c r="I39" s="278"/>
-      <c r="J39" s="278"/>
-      <c r="K39" s="288" t="s">
+      <c r="I39" s="279"/>
+      <c r="J39" s="279"/>
+      <c r="K39" s="289" t="s">
         <v>517</v>
       </c>
-      <c r="L39" s="278"/>
-      <c r="M39" s="278"/>
-      <c r="N39" s="286" t="s">
+      <c r="L39" s="279"/>
+      <c r="M39" s="279"/>
+      <c r="N39" s="287" t="s">
         <v>45</v>
       </c>
-      <c r="O39" s="278"/>
-      <c r="P39" s="278"/>
-      <c r="Q39" s="293" t="s">
+      <c r="O39" s="279"/>
+      <c r="P39" s="279"/>
+      <c r="Q39" s="294" t="s">
         <v>518</v>
       </c>
-      <c r="R39" s="278"/>
-      <c r="S39" s="278"/>
+      <c r="R39" s="279"/>
+      <c r="S39" s="279"/>
     </row>
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H14:M14"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A16:S16"/>
     <mergeCell ref="H20:M20"/>
-    <mergeCell ref="A16:S16"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -12682,13 +12691,14 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -12697,7 +12707,6 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
-    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -12705,7 +12714,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -12753,14 +12762,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="297" t="s">
+      <c r="A1" s="298" t="s">
         <v>519</v>
       </c>
-      <c r="B1" s="271"/>
-      <c r="C1" s="271"/>
-      <c r="D1" s="271"/>
-      <c r="E1" s="271"/>
-      <c r="F1" s="272"/>
+      <c r="B1" s="272"/>
+      <c r="C1" s="272"/>
+      <c r="D1" s="272"/>
+      <c r="E1" s="272"/>
+      <c r="F1" s="273"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
@@ -13125,13 +13134,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="297" t="s">
+      <c r="A1" s="298" t="s">
         <v>526</v>
       </c>
-      <c r="B1" s="271"/>
-      <c r="C1" s="271"/>
-      <c r="D1" s="271"/>
-      <c r="E1" s="272"/>
+      <c r="B1" s="272"/>
+      <c r="C1" s="272"/>
+      <c r="D1" s="272"/>
+      <c r="E1" s="273"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="31" t="s">
@@ -14213,13 +14222,13 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="298" t="s">
+      <c r="A2" s="299" t="s">
         <v>670</v>
       </c>
-      <c r="B2" s="278"/>
-      <c r="C2" s="278"/>
-      <c r="D2" s="278"/>
-      <c r="E2" s="278"/>
+      <c r="B2" s="279"/>
+      <c r="C2" s="279"/>
+      <c r="D2" s="279"/>
+      <c r="E2" s="279"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="255" t="s">
@@ -14313,8 +14322,8 @@
       <c r="B9" s="250" t="s">
         <v>686</v>
       </c>
-      <c r="C9" s="257" t="s">
-        <v>128</v>
+      <c r="C9" s="270" t="s">
+        <v>22</v>
       </c>
       <c r="D9" s="250" t="s">
         <v>674</v>
@@ -14551,8 +14560,8 @@
       <c r="B24" s="250" t="s">
         <v>725</v>
       </c>
-      <c r="C24" s="269" t="s">
-        <v>128</v>
+      <c r="C24" s="270" t="s">
+        <v>22</v>
       </c>
       <c r="D24" s="250" t="s">
         <v>720</v>
@@ -14561,7 +14570,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="262" t="s">
         <v>447</v>
       </c>
@@ -14923,17 +14932,17 @@
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="299" t="s">
+      <c r="A16" s="300" t="s">
         <v>806</v>
       </c>
-      <c r="B16" s="278"/>
-      <c r="C16" s="278"/>
-      <c r="D16" s="278"/>
-      <c r="E16" s="278"/>
-      <c r="F16" s="278"/>
-      <c r="G16" s="278"/>
-      <c r="H16" s="278"/>
-      <c r="I16" s="278"/>
+      <c r="B16" s="279"/>
+      <c r="C16" s="279"/>
+      <c r="D16" s="279"/>
+      <c r="E16" s="279"/>
+      <c r="F16" s="279"/>
+      <c r="G16" s="279"/>
+      <c r="H16" s="279"/>
+      <c r="I16" s="279"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(tracker): P1 complete on the Edge Measurement sheet
9 of 20 done. /history was never a 501 stub -- it was live and serving a
contaminated number, which is a worse starting point than the one
recorded and worth stating plainly.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD61F26F-F56E-4AFF-AE90-A851D56E09C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28923A89-6BB3-42B8-ABFA-385A0BA3B857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2167,7 +2167,7 @@
     <t>P0, spec</t>
   </si>
   <si>
-    <t>149 football + 2,250 tennis outcomes exist, but only 139 football and 79 tennis are PRE_MATCH on a completed fixture — the only rows that evidence skill. See the statistical-power row: this endpoint is instrumentation, not a verdict.</t>
+    <t>DONE (53b7d2a) — and it was never a 501 stub; CLAUDE.md was stale. The endpoint has been LIVE and serving a contaminated number: /history/summary averaged both prediction paths, which measured football at 53.3% instead of 56.1% and tennis 61.7% instead of 63.6%. DOWNWARD, the opposite of the predicted direction — retrodictions score worse, not better, because assemble_from_game_log has a leakage guard and thinner features. Now pre_match by default, retrodictions behind an explicit ?kind=, excluded rows counted rather than dropped.</t>
   </si>
   <si>
     <t>Grade the pick that was SHOWN, not a recomputed one</t>
@@ -2275,7 +2275,7 @@
     <t>the finding above</t>
   </si>
   <si>
-    <t>Follows directly. The endpoint should show sample size and detectable-effect alongside every metric, so a 55% accuracy on n=40 cannot be mistaken for a track record. This is the difference between an honest dashboard and a misleading one.</t>
+    <t>DONE. Every accuracy now carries n, a 95% Wilson interval and its minimum detectable effect. Live: football n=139 acc 0.561 CI [0.478,0.641] detectable 0.105; tennis n=77 acc 0.636 CI [0.525,0.735] detectable 0.136. The intervals are the point — football's spans 16 points and its detectable effect dwarfs the 4.1pp edge we believe in, so the number cannot settle the question either way.</t>
   </si>
   <si>
     <t>FINDING: the pick we SHOW is never persisted</t>
@@ -2284,7 +2284,7 @@
     <t>spec §2b</t>
   </si>
   <si>
-    <t>best_pick is computed per request from the prediction plus whatever odds existed at that moment, filtered by four guards and the caller's own thresholds. None of it is stored. So hit rate, ROI and CLV over SHOWN PICKS cannot be reported for anything already settled — regrading with today's odds and today's guards would measure a different product than users saw, and would be the single most misleading thing this endpoint could do. Splits /history in two: model skill (calibration/Brier/RPS) is measurable now; product skill is not, until picks are snapshotted.</t>
+    <t>RESOLVED by pick_snapshots (8f794e0). Product-skill metrics accumulate from 2026-08-10; nothing before it is recoverable.</t>
   </si>
   <si>
     <t>Persist the pick at the moment it is shown</t>
@@ -2541,7 +2541,7 @@
     <numFmt numFmtId="164" formatCode="dd\ mmm"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="82" x14ac:knownFonts="1">
+  <fonts count="83" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2977,6 +2977,12 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -3646,7 +3652,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="301">
+  <cellXfs count="300">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4431,19 +4437,16 @@
     <xf numFmtId="0" fontId="79" fillId="67" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="79" fillId="68" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="80" fillId="67" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="80" fillId="65" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="80" fillId="68" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="81" fillId="65" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="81" fillId="65" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="82" fillId="65" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4855,46 +4858,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="274" t="s">
+      <c r="A1" s="273" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="272"/>
-      <c r="C1" s="272"/>
-      <c r="D1" s="272"/>
-      <c r="E1" s="272"/>
-      <c r="F1" s="272"/>
-      <c r="G1" s="272"/>
-      <c r="H1" s="272"/>
-      <c r="I1" s="272"/>
-      <c r="J1" s="272"/>
-      <c r="K1" s="272"/>
-      <c r="L1" s="272"/>
-      <c r="M1" s="272"/>
-      <c r="N1" s="272"/>
-      <c r="O1" s="272"/>
-      <c r="P1" s="272"/>
-      <c r="Q1" s="273"/>
+      <c r="B1" s="271"/>
+      <c r="C1" s="271"/>
+      <c r="D1" s="271"/>
+      <c r="E1" s="271"/>
+      <c r="F1" s="271"/>
+      <c r="G1" s="271"/>
+      <c r="H1" s="271"/>
+      <c r="I1" s="271"/>
+      <c r="J1" s="271"/>
+      <c r="K1" s="271"/>
+      <c r="L1" s="271"/>
+      <c r="M1" s="271"/>
+      <c r="N1" s="271"/>
+      <c r="O1" s="271"/>
+      <c r="P1" s="271"/>
+      <c r="Q1" s="272"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="271" t="s">
+      <c r="A2" s="270" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="272"/>
-      <c r="C2" s="272"/>
-      <c r="D2" s="272"/>
-      <c r="E2" s="272"/>
-      <c r="F2" s="272"/>
-      <c r="G2" s="272"/>
-      <c r="H2" s="272"/>
-      <c r="I2" s="272"/>
-      <c r="J2" s="272"/>
-      <c r="K2" s="272"/>
-      <c r="L2" s="272"/>
-      <c r="M2" s="272"/>
-      <c r="N2" s="272"/>
-      <c r="O2" s="272"/>
-      <c r="P2" s="272"/>
-      <c r="Q2" s="273"/>
+      <c r="B2" s="271"/>
+      <c r="C2" s="271"/>
+      <c r="D2" s="271"/>
+      <c r="E2" s="271"/>
+      <c r="F2" s="271"/>
+      <c r="G2" s="271"/>
+      <c r="H2" s="271"/>
+      <c r="I2" s="271"/>
+      <c r="J2" s="271"/>
+      <c r="K2" s="271"/>
+      <c r="L2" s="271"/>
+      <c r="M2" s="271"/>
+      <c r="N2" s="271"/>
+      <c r="O2" s="271"/>
+      <c r="P2" s="271"/>
+      <c r="Q2" s="272"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
@@ -11837,852 +11840,852 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="290" t="s">
+      <c r="A1" s="289" t="s">
         <v>449</v>
       </c>
-      <c r="B1" s="279"/>
-      <c r="C1" s="279"/>
-      <c r="D1" s="279"/>
-      <c r="E1" s="279"/>
-      <c r="F1" s="279"/>
-      <c r="G1" s="279"/>
-      <c r="H1" s="279"/>
-      <c r="I1" s="279"/>
-      <c r="J1" s="279"/>
-      <c r="K1" s="279"/>
-      <c r="L1" s="279"/>
-      <c r="M1" s="279"/>
-      <c r="N1" s="279"/>
-      <c r="O1" s="279"/>
-      <c r="P1" s="279"/>
-      <c r="Q1" s="279"/>
-      <c r="R1" s="279"/>
-      <c r="S1" s="279"/>
+      <c r="B1" s="278"/>
+      <c r="C1" s="278"/>
+      <c r="D1" s="278"/>
+      <c r="E1" s="278"/>
+      <c r="F1" s="278"/>
+      <c r="G1" s="278"/>
+      <c r="H1" s="278"/>
+      <c r="I1" s="278"/>
+      <c r="J1" s="278"/>
+      <c r="K1" s="278"/>
+      <c r="L1" s="278"/>
+      <c r="M1" s="278"/>
+      <c r="N1" s="278"/>
+      <c r="O1" s="278"/>
+      <c r="P1" s="278"/>
+      <c r="Q1" s="278"/>
+      <c r="R1" s="278"/>
+      <c r="S1" s="278"/>
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="297" t="s">
+      <c r="A2" s="296" t="s">
         <v>450</v>
       </c>
-      <c r="B2" s="279"/>
-      <c r="C2" s="279"/>
-      <c r="D2" s="279"/>
-      <c r="E2" s="279"/>
-      <c r="F2" s="279"/>
-      <c r="G2" s="279"/>
-      <c r="H2" s="279"/>
-      <c r="I2" s="279"/>
-      <c r="J2" s="279"/>
-      <c r="K2" s="279"/>
-      <c r="L2" s="279"/>
-      <c r="M2" s="279"/>
-      <c r="N2" s="279"/>
-      <c r="O2" s="279"/>
-      <c r="P2" s="279"/>
-      <c r="Q2" s="279"/>
-      <c r="R2" s="279"/>
-      <c r="S2" s="279"/>
+      <c r="B2" s="278"/>
+      <c r="C2" s="278"/>
+      <c r="D2" s="278"/>
+      <c r="E2" s="278"/>
+      <c r="F2" s="278"/>
+      <c r="G2" s="278"/>
+      <c r="H2" s="278"/>
+      <c r="I2" s="278"/>
+      <c r="J2" s="278"/>
+      <c r="K2" s="278"/>
+      <c r="L2" s="278"/>
+      <c r="M2" s="278"/>
+      <c r="N2" s="278"/>
+      <c r="O2" s="278"/>
+      <c r="P2" s="278"/>
+      <c r="Q2" s="278"/>
+      <c r="R2" s="278"/>
+      <c r="S2" s="278"/>
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="285" t="s">
+      <c r="A4" s="284" t="s">
         <v>451</v>
       </c>
-      <c r="B4" s="279"/>
-      <c r="C4" s="279"/>
-      <c r="D4" s="279"/>
-      <c r="E4" s="279"/>
-      <c r="F4" s="279"/>
-      <c r="G4" s="279"/>
-      <c r="H4" s="279"/>
-      <c r="I4" s="279"/>
-      <c r="J4" s="279"/>
-      <c r="K4" s="279"/>
-      <c r="L4" s="279"/>
-      <c r="M4" s="279"/>
-      <c r="N4" s="279"/>
-      <c r="O4" s="279"/>
-      <c r="P4" s="279"/>
-      <c r="Q4" s="279"/>
-      <c r="R4" s="279"/>
-      <c r="S4" s="279"/>
+      <c r="B4" s="278"/>
+      <c r="C4" s="278"/>
+      <c r="D4" s="278"/>
+      <c r="E4" s="278"/>
+      <c r="F4" s="278"/>
+      <c r="G4" s="278"/>
+      <c r="H4" s="278"/>
+      <c r="I4" s="278"/>
+      <c r="J4" s="278"/>
+      <c r="K4" s="278"/>
+      <c r="L4" s="278"/>
+      <c r="M4" s="278"/>
+      <c r="N4" s="278"/>
+      <c r="O4" s="278"/>
+      <c r="P4" s="278"/>
+      <c r="Q4" s="278"/>
+      <c r="R4" s="278"/>
+      <c r="S4" s="278"/>
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="37" t="s">
         <v>452</v>
       </c>
-      <c r="B5" s="275" t="s">
+      <c r="B5" s="274" t="s">
         <v>453</v>
       </c>
-      <c r="C5" s="276"/>
-      <c r="D5" s="277"/>
-      <c r="E5" s="280" t="s">
+      <c r="C5" s="275"/>
+      <c r="D5" s="276"/>
+      <c r="E5" s="279" t="s">
         <v>454</v>
       </c>
-      <c r="F5" s="276"/>
-      <c r="G5" s="277"/>
-      <c r="H5" s="280" t="s">
+      <c r="F5" s="275"/>
+      <c r="G5" s="276"/>
+      <c r="H5" s="279" t="s">
         <v>455</v>
       </c>
-      <c r="I5" s="276"/>
-      <c r="J5" s="277"/>
-      <c r="K5" s="275" t="s">
+      <c r="I5" s="275"/>
+      <c r="J5" s="276"/>
+      <c r="K5" s="274" t="s">
         <v>456</v>
       </c>
-      <c r="L5" s="276"/>
-      <c r="M5" s="277"/>
-      <c r="N5" s="282" t="s">
+      <c r="L5" s="275"/>
+      <c r="M5" s="276"/>
+      <c r="N5" s="281" t="s">
         <v>457</v>
       </c>
-      <c r="O5" s="276"/>
-      <c r="P5" s="277"/>
-      <c r="Q5" s="282" t="s">
+      <c r="O5" s="275"/>
+      <c r="P5" s="276"/>
+      <c r="Q5" s="281" t="s">
         <v>458</v>
       </c>
-      <c r="R5" s="276"/>
-      <c r="S5" s="277"/>
+      <c r="R5" s="275"/>
+      <c r="S5" s="276"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="278" t="s">
+      <c r="B6" s="277" t="s">
         <v>459</v>
       </c>
-      <c r="C6" s="279"/>
-      <c r="D6" s="279"/>
-      <c r="E6" s="279"/>
-      <c r="F6" s="279"/>
-      <c r="G6" s="279"/>
-      <c r="H6" s="279"/>
-      <c r="I6" s="279"/>
-      <c r="J6" s="279"/>
-      <c r="K6" s="279"/>
-      <c r="L6" s="279"/>
-      <c r="M6" s="279"/>
-      <c r="N6" s="279"/>
-      <c r="O6" s="279"/>
-      <c r="P6" s="279"/>
-      <c r="Q6" s="279"/>
-      <c r="R6" s="279"/>
-      <c r="S6" s="279"/>
+      <c r="C6" s="278"/>
+      <c r="D6" s="278"/>
+      <c r="E6" s="278"/>
+      <c r="F6" s="278"/>
+      <c r="G6" s="278"/>
+      <c r="H6" s="278"/>
+      <c r="I6" s="278"/>
+      <c r="J6" s="278"/>
+      <c r="K6" s="278"/>
+      <c r="L6" s="278"/>
+      <c r="M6" s="278"/>
+      <c r="N6" s="278"/>
+      <c r="O6" s="278"/>
+      <c r="P6" s="278"/>
+      <c r="Q6" s="278"/>
+      <c r="R6" s="278"/>
+      <c r="S6" s="278"/>
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="285" t="s">
+      <c r="A7" s="284" t="s">
         <v>460</v>
       </c>
-      <c r="B7" s="279"/>
-      <c r="C7" s="279"/>
-      <c r="D7" s="279"/>
-      <c r="E7" s="279"/>
-      <c r="F7" s="279"/>
-      <c r="G7" s="279"/>
-      <c r="H7" s="279"/>
-      <c r="I7" s="279"/>
-      <c r="J7" s="279"/>
-      <c r="K7" s="279"/>
-      <c r="L7" s="279"/>
-      <c r="M7" s="279"/>
-      <c r="N7" s="279"/>
-      <c r="O7" s="279"/>
-      <c r="P7" s="279"/>
-      <c r="Q7" s="279"/>
-      <c r="R7" s="279"/>
-      <c r="S7" s="279"/>
+      <c r="B7" s="278"/>
+      <c r="C7" s="278"/>
+      <c r="D7" s="278"/>
+      <c r="E7" s="278"/>
+      <c r="F7" s="278"/>
+      <c r="G7" s="278"/>
+      <c r="H7" s="278"/>
+      <c r="I7" s="278"/>
+      <c r="J7" s="278"/>
+      <c r="K7" s="278"/>
+      <c r="L7" s="278"/>
+      <c r="M7" s="278"/>
+      <c r="N7" s="278"/>
+      <c r="O7" s="278"/>
+      <c r="P7" s="278"/>
+      <c r="Q7" s="278"/>
+      <c r="R7" s="278"/>
+      <c r="S7" s="278"/>
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="37" t="s">
         <v>461</v>
       </c>
-      <c r="B8" s="288" t="s">
+      <c r="B8" s="287" t="s">
         <v>462</v>
       </c>
-      <c r="C8" s="276"/>
-      <c r="D8" s="276"/>
-      <c r="E8" s="276"/>
-      <c r="F8" s="276"/>
-      <c r="G8" s="276"/>
-      <c r="H8" s="276"/>
-      <c r="I8" s="276"/>
-      <c r="J8" s="277"/>
-      <c r="K8" s="288" t="s">
+      <c r="C8" s="275"/>
+      <c r="D8" s="275"/>
+      <c r="E8" s="275"/>
+      <c r="F8" s="275"/>
+      <c r="G8" s="275"/>
+      <c r="H8" s="275"/>
+      <c r="I8" s="275"/>
+      <c r="J8" s="276"/>
+      <c r="K8" s="287" t="s">
         <v>463</v>
       </c>
-      <c r="L8" s="276"/>
-      <c r="M8" s="276"/>
-      <c r="N8" s="276"/>
-      <c r="O8" s="276"/>
-      <c r="P8" s="276"/>
-      <c r="Q8" s="276"/>
-      <c r="R8" s="276"/>
-      <c r="S8" s="277"/>
+      <c r="L8" s="275"/>
+      <c r="M8" s="275"/>
+      <c r="N8" s="275"/>
+      <c r="O8" s="275"/>
+      <c r="P8" s="275"/>
+      <c r="Q8" s="275"/>
+      <c r="R8" s="275"/>
+      <c r="S8" s="276"/>
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B9" s="278" t="s">
+      <c r="B9" s="277" t="s">
         <v>459</v>
       </c>
-      <c r="C9" s="279"/>
-      <c r="D9" s="279"/>
-      <c r="E9" s="279"/>
-      <c r="F9" s="279"/>
-      <c r="G9" s="279"/>
-      <c r="H9" s="279"/>
-      <c r="I9" s="279"/>
-      <c r="J9" s="279"/>
-      <c r="K9" s="279"/>
-      <c r="L9" s="279"/>
-      <c r="M9" s="279"/>
-      <c r="N9" s="279"/>
-      <c r="O9" s="279"/>
-      <c r="P9" s="279"/>
-      <c r="Q9" s="279"/>
-      <c r="R9" s="279"/>
-      <c r="S9" s="279"/>
+      <c r="C9" s="278"/>
+      <c r="D9" s="278"/>
+      <c r="E9" s="278"/>
+      <c r="F9" s="278"/>
+      <c r="G9" s="278"/>
+      <c r="H9" s="278"/>
+      <c r="I9" s="278"/>
+      <c r="J9" s="278"/>
+      <c r="K9" s="278"/>
+      <c r="L9" s="278"/>
+      <c r="M9" s="278"/>
+      <c r="N9" s="278"/>
+      <c r="O9" s="278"/>
+      <c r="P9" s="278"/>
+      <c r="Q9" s="278"/>
+      <c r="R9" s="278"/>
+      <c r="S9" s="278"/>
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="285" t="s">
+      <c r="A10" s="284" t="s">
         <v>464</v>
       </c>
-      <c r="B10" s="279"/>
-      <c r="C10" s="279"/>
-      <c r="D10" s="279"/>
-      <c r="E10" s="279"/>
-      <c r="F10" s="279"/>
-      <c r="G10" s="279"/>
-      <c r="H10" s="279"/>
-      <c r="I10" s="279"/>
-      <c r="J10" s="279"/>
-      <c r="K10" s="279"/>
-      <c r="L10" s="279"/>
-      <c r="M10" s="279"/>
-      <c r="N10" s="279"/>
-      <c r="O10" s="279"/>
-      <c r="P10" s="279"/>
-      <c r="Q10" s="279"/>
-      <c r="R10" s="279"/>
-      <c r="S10" s="279"/>
+      <c r="B10" s="278"/>
+      <c r="C10" s="278"/>
+      <c r="D10" s="278"/>
+      <c r="E10" s="278"/>
+      <c r="F10" s="278"/>
+      <c r="G10" s="278"/>
+      <c r="H10" s="278"/>
+      <c r="I10" s="278"/>
+      <c r="J10" s="278"/>
+      <c r="K10" s="278"/>
+      <c r="L10" s="278"/>
+      <c r="M10" s="278"/>
+      <c r="N10" s="278"/>
+      <c r="O10" s="278"/>
+      <c r="P10" s="278"/>
+      <c r="Q10" s="278"/>
+      <c r="R10" s="278"/>
+      <c r="S10" s="278"/>
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="37" t="s">
         <v>465</v>
       </c>
-      <c r="B11" s="275" t="s">
+      <c r="B11" s="274" t="s">
         <v>466</v>
       </c>
-      <c r="C11" s="276"/>
-      <c r="D11" s="277"/>
-      <c r="E11" s="275" t="s">
+      <c r="C11" s="275"/>
+      <c r="D11" s="276"/>
+      <c r="E11" s="274" t="s">
         <v>467</v>
       </c>
-      <c r="F11" s="276"/>
-      <c r="G11" s="277"/>
-      <c r="H11" s="275" t="s">
+      <c r="F11" s="275"/>
+      <c r="G11" s="276"/>
+      <c r="H11" s="274" t="s">
         <v>468</v>
       </c>
-      <c r="I11" s="276"/>
-      <c r="J11" s="277"/>
-      <c r="K11" s="280" t="s">
+      <c r="I11" s="275"/>
+      <c r="J11" s="276"/>
+      <c r="K11" s="279" t="s">
         <v>469</v>
       </c>
-      <c r="L11" s="276"/>
-      <c r="M11" s="277"/>
-      <c r="N11" s="275" t="s">
+      <c r="L11" s="275"/>
+      <c r="M11" s="276"/>
+      <c r="N11" s="274" t="s">
         <v>470</v>
       </c>
-      <c r="O11" s="276"/>
-      <c r="P11" s="277"/>
-      <c r="Q11" s="275" t="s">
+      <c r="O11" s="275"/>
+      <c r="P11" s="276"/>
+      <c r="Q11" s="274" t="s">
         <v>471</v>
       </c>
-      <c r="R11" s="276"/>
-      <c r="S11" s="277"/>
+      <c r="R11" s="275"/>
+      <c r="S11" s="276"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B12" s="278" t="s">
+      <c r="B12" s="277" t="s">
         <v>459</v>
       </c>
-      <c r="C12" s="279"/>
-      <c r="D12" s="279"/>
-      <c r="E12" s="279"/>
-      <c r="F12" s="279"/>
-      <c r="G12" s="279"/>
-      <c r="H12" s="279"/>
-      <c r="I12" s="279"/>
-      <c r="J12" s="279"/>
-      <c r="K12" s="279"/>
-      <c r="L12" s="279"/>
-      <c r="M12" s="279"/>
-      <c r="N12" s="279"/>
-      <c r="O12" s="279"/>
-      <c r="P12" s="279"/>
-      <c r="Q12" s="279"/>
-      <c r="R12" s="279"/>
-      <c r="S12" s="279"/>
+      <c r="C12" s="278"/>
+      <c r="D12" s="278"/>
+      <c r="E12" s="278"/>
+      <c r="F12" s="278"/>
+      <c r="G12" s="278"/>
+      <c r="H12" s="278"/>
+      <c r="I12" s="278"/>
+      <c r="J12" s="278"/>
+      <c r="K12" s="278"/>
+      <c r="L12" s="278"/>
+      <c r="M12" s="278"/>
+      <c r="N12" s="278"/>
+      <c r="O12" s="278"/>
+      <c r="P12" s="278"/>
+      <c r="Q12" s="278"/>
+      <c r="R12" s="278"/>
+      <c r="S12" s="278"/>
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="285" t="s">
+      <c r="A13" s="284" t="s">
         <v>472</v>
       </c>
-      <c r="B13" s="279"/>
-      <c r="C13" s="279"/>
-      <c r="D13" s="279"/>
-      <c r="E13" s="279"/>
-      <c r="F13" s="279"/>
-      <c r="G13" s="279"/>
-      <c r="H13" s="279"/>
-      <c r="I13" s="279"/>
-      <c r="J13" s="279"/>
-      <c r="K13" s="279"/>
-      <c r="L13" s="279"/>
-      <c r="M13" s="279"/>
-      <c r="N13" s="279"/>
-      <c r="O13" s="279"/>
-      <c r="P13" s="279"/>
-      <c r="Q13" s="279"/>
-      <c r="R13" s="279"/>
-      <c r="S13" s="279"/>
+      <c r="B13" s="278"/>
+      <c r="C13" s="278"/>
+      <c r="D13" s="278"/>
+      <c r="E13" s="278"/>
+      <c r="F13" s="278"/>
+      <c r="G13" s="278"/>
+      <c r="H13" s="278"/>
+      <c r="I13" s="278"/>
+      <c r="J13" s="278"/>
+      <c r="K13" s="278"/>
+      <c r="L13" s="278"/>
+      <c r="M13" s="278"/>
+      <c r="N13" s="278"/>
+      <c r="O13" s="278"/>
+      <c r="P13" s="278"/>
+      <c r="Q13" s="278"/>
+      <c r="R13" s="278"/>
+      <c r="S13" s="278"/>
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="37" t="s">
         <v>473</v>
       </c>
-      <c r="B14" s="283" t="s">
+      <c r="B14" s="282" t="s">
         <v>474</v>
       </c>
-      <c r="C14" s="276"/>
-      <c r="D14" s="276"/>
-      <c r="E14" s="276"/>
-      <c r="F14" s="276"/>
-      <c r="G14" s="277"/>
-      <c r="H14" s="283" t="s">
+      <c r="C14" s="275"/>
+      <c r="D14" s="275"/>
+      <c r="E14" s="275"/>
+      <c r="F14" s="275"/>
+      <c r="G14" s="276"/>
+      <c r="H14" s="282" t="s">
         <v>475</v>
       </c>
-      <c r="I14" s="276"/>
-      <c r="J14" s="276"/>
-      <c r="K14" s="276"/>
-      <c r="L14" s="276"/>
-      <c r="M14" s="277"/>
-      <c r="N14" s="283" t="s">
+      <c r="I14" s="275"/>
+      <c r="J14" s="275"/>
+      <c r="K14" s="275"/>
+      <c r="L14" s="275"/>
+      <c r="M14" s="276"/>
+      <c r="N14" s="282" t="s">
         <v>476</v>
       </c>
-      <c r="O14" s="276"/>
-      <c r="P14" s="277"/>
-      <c r="Q14" s="280" t="s">
+      <c r="O14" s="275"/>
+      <c r="P14" s="276"/>
+      <c r="Q14" s="279" t="s">
         <v>477</v>
       </c>
-      <c r="R14" s="276"/>
-      <c r="S14" s="277"/>
+      <c r="R14" s="275"/>
+      <c r="S14" s="276"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B15" s="278" t="s">
+      <c r="B15" s="277" t="s">
         <v>478</v>
       </c>
-      <c r="C15" s="279"/>
-      <c r="D15" s="279"/>
-      <c r="E15" s="279"/>
-      <c r="F15" s="279"/>
-      <c r="G15" s="279"/>
-      <c r="H15" s="279"/>
-      <c r="I15" s="279"/>
-      <c r="J15" s="279"/>
-      <c r="K15" s="279"/>
-      <c r="L15" s="279"/>
-      <c r="M15" s="279"/>
-      <c r="N15" s="279"/>
-      <c r="O15" s="279"/>
-      <c r="P15" s="279"/>
-      <c r="Q15" s="279"/>
-      <c r="R15" s="279"/>
-      <c r="S15" s="279"/>
+      <c r="C15" s="278"/>
+      <c r="D15" s="278"/>
+      <c r="E15" s="278"/>
+      <c r="F15" s="278"/>
+      <c r="G15" s="278"/>
+      <c r="H15" s="278"/>
+      <c r="I15" s="278"/>
+      <c r="J15" s="278"/>
+      <c r="K15" s="278"/>
+      <c r="L15" s="278"/>
+      <c r="M15" s="278"/>
+      <c r="N15" s="278"/>
+      <c r="O15" s="278"/>
+      <c r="P15" s="278"/>
+      <c r="Q15" s="278"/>
+      <c r="R15" s="278"/>
+      <c r="S15" s="278"/>
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="285" t="s">
+      <c r="A16" s="284" t="s">
         <v>479</v>
       </c>
-      <c r="B16" s="279"/>
-      <c r="C16" s="279"/>
-      <c r="D16" s="279"/>
-      <c r="E16" s="279"/>
-      <c r="F16" s="279"/>
-      <c r="G16" s="279"/>
-      <c r="H16" s="279"/>
-      <c r="I16" s="279"/>
-      <c r="J16" s="279"/>
-      <c r="K16" s="279"/>
-      <c r="L16" s="279"/>
-      <c r="M16" s="279"/>
-      <c r="N16" s="279"/>
-      <c r="O16" s="279"/>
-      <c r="P16" s="279"/>
-      <c r="Q16" s="279"/>
-      <c r="R16" s="279"/>
-      <c r="S16" s="279"/>
+      <c r="B16" s="278"/>
+      <c r="C16" s="278"/>
+      <c r="D16" s="278"/>
+      <c r="E16" s="278"/>
+      <c r="F16" s="278"/>
+      <c r="G16" s="278"/>
+      <c r="H16" s="278"/>
+      <c r="I16" s="278"/>
+      <c r="J16" s="278"/>
+      <c r="K16" s="278"/>
+      <c r="L16" s="278"/>
+      <c r="M16" s="278"/>
+      <c r="N16" s="278"/>
+      <c r="O16" s="278"/>
+      <c r="P16" s="278"/>
+      <c r="Q16" s="278"/>
+      <c r="R16" s="278"/>
+      <c r="S16" s="278"/>
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="37" t="s">
         <v>480</v>
       </c>
-      <c r="B17" s="284" t="s">
+      <c r="B17" s="283" t="s">
         <v>481</v>
       </c>
-      <c r="C17" s="276"/>
-      <c r="D17" s="276"/>
-      <c r="E17" s="276"/>
-      <c r="F17" s="276"/>
-      <c r="G17" s="277"/>
-      <c r="H17" s="284" t="s">
+      <c r="C17" s="275"/>
+      <c r="D17" s="275"/>
+      <c r="E17" s="275"/>
+      <c r="F17" s="275"/>
+      <c r="G17" s="276"/>
+      <c r="H17" s="283" t="s">
         <v>482</v>
       </c>
-      <c r="I17" s="276"/>
-      <c r="J17" s="277"/>
-      <c r="K17" s="284" t="s">
+      <c r="I17" s="275"/>
+      <c r="J17" s="276"/>
+      <c r="K17" s="283" t="s">
         <v>483</v>
       </c>
-      <c r="L17" s="276"/>
-      <c r="M17" s="277"/>
-      <c r="N17" s="284" t="s">
+      <c r="L17" s="275"/>
+      <c r="M17" s="276"/>
+      <c r="N17" s="283" t="s">
         <v>484</v>
       </c>
-      <c r="O17" s="276"/>
-      <c r="P17" s="277"/>
-      <c r="Q17" s="284" t="s">
+      <c r="O17" s="275"/>
+      <c r="P17" s="276"/>
+      <c r="Q17" s="283" t="s">
         <v>485</v>
       </c>
-      <c r="R17" s="276"/>
-      <c r="S17" s="277"/>
+      <c r="R17" s="275"/>
+      <c r="S17" s="276"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="278" t="s">
+      <c r="B18" s="277" t="s">
         <v>459</v>
       </c>
-      <c r="C18" s="279"/>
-      <c r="D18" s="279"/>
-      <c r="E18" s="279"/>
-      <c r="F18" s="279"/>
-      <c r="G18" s="279"/>
-      <c r="H18" s="279"/>
-      <c r="I18" s="279"/>
-      <c r="J18" s="279"/>
-      <c r="K18" s="279"/>
-      <c r="L18" s="279"/>
-      <c r="M18" s="279"/>
-      <c r="N18" s="279"/>
-      <c r="O18" s="279"/>
-      <c r="P18" s="279"/>
-      <c r="Q18" s="279"/>
-      <c r="R18" s="279"/>
-      <c r="S18" s="279"/>
+      <c r="C18" s="278"/>
+      <c r="D18" s="278"/>
+      <c r="E18" s="278"/>
+      <c r="F18" s="278"/>
+      <c r="G18" s="278"/>
+      <c r="H18" s="278"/>
+      <c r="I18" s="278"/>
+      <c r="J18" s="278"/>
+      <c r="K18" s="278"/>
+      <c r="L18" s="278"/>
+      <c r="M18" s="278"/>
+      <c r="N18" s="278"/>
+      <c r="O18" s="278"/>
+      <c r="P18" s="278"/>
+      <c r="Q18" s="278"/>
+      <c r="R18" s="278"/>
+      <c r="S18" s="278"/>
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="285" t="s">
+      <c r="A19" s="284" t="s">
         <v>486</v>
       </c>
-      <c r="B19" s="279"/>
-      <c r="C19" s="279"/>
-      <c r="D19" s="279"/>
-      <c r="E19" s="279"/>
-      <c r="F19" s="279"/>
-      <c r="G19" s="279"/>
-      <c r="H19" s="279"/>
-      <c r="I19" s="279"/>
-      <c r="J19" s="279"/>
-      <c r="K19" s="279"/>
-      <c r="L19" s="279"/>
-      <c r="M19" s="279"/>
-      <c r="N19" s="279"/>
-      <c r="O19" s="279"/>
-      <c r="P19" s="279"/>
-      <c r="Q19" s="279"/>
-      <c r="R19" s="279"/>
-      <c r="S19" s="279"/>
+      <c r="B19" s="278"/>
+      <c r="C19" s="278"/>
+      <c r="D19" s="278"/>
+      <c r="E19" s="278"/>
+      <c r="F19" s="278"/>
+      <c r="G19" s="278"/>
+      <c r="H19" s="278"/>
+      <c r="I19" s="278"/>
+      <c r="J19" s="278"/>
+      <c r="K19" s="278"/>
+      <c r="L19" s="278"/>
+      <c r="M19" s="278"/>
+      <c r="N19" s="278"/>
+      <c r="O19" s="278"/>
+      <c r="P19" s="278"/>
+      <c r="Q19" s="278"/>
+      <c r="R19" s="278"/>
+      <c r="S19" s="278"/>
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="37" t="s">
         <v>487</v>
       </c>
-      <c r="B20" s="286" t="s">
+      <c r="B20" s="285" t="s">
         <v>488</v>
       </c>
-      <c r="C20" s="276"/>
-      <c r="D20" s="276"/>
-      <c r="E20" s="276"/>
-      <c r="F20" s="276"/>
-      <c r="G20" s="277"/>
-      <c r="H20" s="286" t="s">
+      <c r="C20" s="275"/>
+      <c r="D20" s="275"/>
+      <c r="E20" s="275"/>
+      <c r="F20" s="275"/>
+      <c r="G20" s="276"/>
+      <c r="H20" s="285" t="s">
         <v>489</v>
       </c>
-      <c r="I20" s="276"/>
-      <c r="J20" s="276"/>
-      <c r="K20" s="276"/>
-      <c r="L20" s="276"/>
-      <c r="M20" s="277"/>
-      <c r="N20" s="286" t="s">
+      <c r="I20" s="275"/>
+      <c r="J20" s="275"/>
+      <c r="K20" s="275"/>
+      <c r="L20" s="275"/>
+      <c r="M20" s="276"/>
+      <c r="N20" s="285" t="s">
         <v>490</v>
       </c>
-      <c r="O20" s="276"/>
-      <c r="P20" s="276"/>
-      <c r="Q20" s="276"/>
-      <c r="R20" s="276"/>
-      <c r="S20" s="277"/>
+      <c r="O20" s="275"/>
+      <c r="P20" s="275"/>
+      <c r="Q20" s="275"/>
+      <c r="R20" s="275"/>
+      <c r="S20" s="276"/>
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B21" s="278" t="s">
+      <c r="B21" s="277" t="s">
         <v>459</v>
       </c>
-      <c r="C21" s="279"/>
-      <c r="D21" s="279"/>
-      <c r="E21" s="279"/>
-      <c r="F21" s="279"/>
-      <c r="G21" s="279"/>
-      <c r="H21" s="279"/>
-      <c r="I21" s="279"/>
-      <c r="J21" s="279"/>
-      <c r="K21" s="279"/>
-      <c r="L21" s="279"/>
-      <c r="M21" s="279"/>
-      <c r="N21" s="279"/>
-      <c r="O21" s="279"/>
-      <c r="P21" s="279"/>
-      <c r="Q21" s="279"/>
-      <c r="R21" s="279"/>
-      <c r="S21" s="279"/>
+      <c r="C21" s="278"/>
+      <c r="D21" s="278"/>
+      <c r="E21" s="278"/>
+      <c r="F21" s="278"/>
+      <c r="G21" s="278"/>
+      <c r="H21" s="278"/>
+      <c r="I21" s="278"/>
+      <c r="J21" s="278"/>
+      <c r="K21" s="278"/>
+      <c r="L21" s="278"/>
+      <c r="M21" s="278"/>
+      <c r="N21" s="278"/>
+      <c r="O21" s="278"/>
+      <c r="P21" s="278"/>
+      <c r="Q21" s="278"/>
+      <c r="R21" s="278"/>
+      <c r="S21" s="278"/>
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="285" t="s">
+      <c r="A22" s="284" t="s">
         <v>491</v>
       </c>
-      <c r="B22" s="279"/>
-      <c r="C22" s="279"/>
-      <c r="D22" s="279"/>
-      <c r="E22" s="279"/>
-      <c r="F22" s="279"/>
-      <c r="G22" s="279"/>
-      <c r="H22" s="279"/>
-      <c r="I22" s="279"/>
-      <c r="J22" s="279"/>
-      <c r="K22" s="279"/>
-      <c r="L22" s="279"/>
-      <c r="M22" s="279"/>
-      <c r="N22" s="279"/>
-      <c r="O22" s="279"/>
-      <c r="P22" s="279"/>
-      <c r="Q22" s="279"/>
-      <c r="R22" s="279"/>
-      <c r="S22" s="279"/>
+      <c r="B22" s="278"/>
+      <c r="C22" s="278"/>
+      <c r="D22" s="278"/>
+      <c r="E22" s="278"/>
+      <c r="F22" s="278"/>
+      <c r="G22" s="278"/>
+      <c r="H22" s="278"/>
+      <c r="I22" s="278"/>
+      <c r="J22" s="278"/>
+      <c r="K22" s="278"/>
+      <c r="L22" s="278"/>
+      <c r="M22" s="278"/>
+      <c r="N22" s="278"/>
+      <c r="O22" s="278"/>
+      <c r="P22" s="278"/>
+      <c r="Q22" s="278"/>
+      <c r="R22" s="278"/>
+      <c r="S22" s="278"/>
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="37" t="s">
         <v>492</v>
       </c>
-      <c r="B23" s="286" t="s">
+      <c r="B23" s="285" t="s">
         <v>493</v>
       </c>
-      <c r="C23" s="276"/>
-      <c r="D23" s="276"/>
-      <c r="E23" s="276"/>
-      <c r="F23" s="276"/>
-      <c r="G23" s="277"/>
-      <c r="H23" s="286" t="s">
+      <c r="C23" s="275"/>
+      <c r="D23" s="275"/>
+      <c r="E23" s="275"/>
+      <c r="F23" s="275"/>
+      <c r="G23" s="276"/>
+      <c r="H23" s="285" t="s">
         <v>494</v>
       </c>
-      <c r="I23" s="276"/>
-      <c r="J23" s="277"/>
-      <c r="K23" s="286" t="s">
+      <c r="I23" s="275"/>
+      <c r="J23" s="276"/>
+      <c r="K23" s="285" t="s">
         <v>495</v>
       </c>
-      <c r="L23" s="276"/>
-      <c r="M23" s="277"/>
-      <c r="N23" s="286" t="s">
+      <c r="L23" s="275"/>
+      <c r="M23" s="276"/>
+      <c r="N23" s="285" t="s">
         <v>496</v>
       </c>
-      <c r="O23" s="276"/>
-      <c r="P23" s="277"/>
-      <c r="Q23" s="282" t="s">
+      <c r="O23" s="275"/>
+      <c r="P23" s="276"/>
+      <c r="Q23" s="281" t="s">
         <v>497</v>
       </c>
-      <c r="R23" s="276"/>
-      <c r="S23" s="277"/>
+      <c r="R23" s="275"/>
+      <c r="S23" s="276"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="291" t="s">
+      <c r="A26" s="290" t="s">
         <v>498</v>
       </c>
-      <c r="B26" s="279"/>
-      <c r="C26" s="279"/>
-      <c r="D26" s="279"/>
-      <c r="E26" s="279"/>
-      <c r="F26" s="279"/>
-      <c r="G26" s="279"/>
-      <c r="H26" s="279"/>
-      <c r="I26" s="279"/>
-      <c r="J26" s="279"/>
-      <c r="K26" s="279"/>
-      <c r="L26" s="279"/>
-      <c r="M26" s="279"/>
-      <c r="N26" s="279"/>
-      <c r="O26" s="279"/>
-      <c r="P26" s="279"/>
-      <c r="Q26" s="279"/>
-      <c r="R26" s="279"/>
-      <c r="S26" s="279"/>
+      <c r="B26" s="278"/>
+      <c r="C26" s="278"/>
+      <c r="D26" s="278"/>
+      <c r="E26" s="278"/>
+      <c r="F26" s="278"/>
+      <c r="G26" s="278"/>
+      <c r="H26" s="278"/>
+      <c r="I26" s="278"/>
+      <c r="J26" s="278"/>
+      <c r="K26" s="278"/>
+      <c r="L26" s="278"/>
+      <c r="M26" s="278"/>
+      <c r="N26" s="278"/>
+      <c r="O26" s="278"/>
+      <c r="P26" s="278"/>
+      <c r="Q26" s="278"/>
+      <c r="R26" s="278"/>
+      <c r="S26" s="278"/>
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="37" t="s">
         <v>499</v>
       </c>
-      <c r="B27" s="275" t="s">
+      <c r="B27" s="274" t="s">
         <v>500</v>
       </c>
-      <c r="C27" s="276"/>
-      <c r="D27" s="277"/>
-      <c r="E27" s="275" t="s">
+      <c r="C27" s="275"/>
+      <c r="D27" s="276"/>
+      <c r="E27" s="274" t="s">
         <v>501</v>
       </c>
-      <c r="F27" s="276"/>
-      <c r="G27" s="277"/>
-      <c r="H27" s="283" t="s">
+      <c r="F27" s="275"/>
+      <c r="G27" s="276"/>
+      <c r="H27" s="282" t="s">
         <v>502</v>
       </c>
-      <c r="I27" s="276"/>
-      <c r="J27" s="277"/>
-      <c r="K27" s="284" t="s">
+      <c r="I27" s="275"/>
+      <c r="J27" s="276"/>
+      <c r="K27" s="283" t="s">
         <v>503</v>
       </c>
-      <c r="L27" s="276"/>
-      <c r="M27" s="277"/>
-      <c r="N27" s="284" t="s">
+      <c r="L27" s="275"/>
+      <c r="M27" s="276"/>
+      <c r="N27" s="283" t="s">
         <v>504</v>
       </c>
-      <c r="O27" s="276"/>
-      <c r="P27" s="277"/>
-      <c r="Q27" s="283" t="s">
+      <c r="O27" s="275"/>
+      <c r="P27" s="276"/>
+      <c r="Q27" s="282" t="s">
         <v>505</v>
       </c>
-      <c r="R27" s="276"/>
-      <c r="S27" s="277"/>
+      <c r="R27" s="275"/>
+      <c r="S27" s="276"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="285" t="s">
+      <c r="A30" s="284" t="s">
         <v>506</v>
       </c>
-      <c r="B30" s="279"/>
-      <c r="C30" s="279"/>
-      <c r="D30" s="279"/>
-      <c r="E30" s="279"/>
-      <c r="F30" s="279"/>
-      <c r="G30" s="279"/>
-      <c r="H30" s="279"/>
-      <c r="I30" s="279"/>
-      <c r="J30" s="279"/>
-      <c r="K30" s="279"/>
-      <c r="L30" s="279"/>
-      <c r="M30" s="279"/>
-      <c r="N30" s="279"/>
-      <c r="O30" s="279"/>
-      <c r="P30" s="279"/>
-      <c r="Q30" s="279"/>
-      <c r="R30" s="279"/>
-      <c r="S30" s="279"/>
+      <c r="B30" s="278"/>
+      <c r="C30" s="278"/>
+      <c r="D30" s="278"/>
+      <c r="E30" s="278"/>
+      <c r="F30" s="278"/>
+      <c r="G30" s="278"/>
+      <c r="H30" s="278"/>
+      <c r="I30" s="278"/>
+      <c r="J30" s="278"/>
+      <c r="K30" s="278"/>
+      <c r="L30" s="278"/>
+      <c r="M30" s="278"/>
+      <c r="N30" s="278"/>
+      <c r="O30" s="278"/>
+      <c r="P30" s="278"/>
+      <c r="Q30" s="278"/>
+      <c r="R30" s="278"/>
+      <c r="S30" s="278"/>
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="281" t="s">
+      <c r="A31" s="280" t="s">
         <v>507</v>
       </c>
-      <c r="B31" s="279"/>
-      <c r="C31" s="279"/>
-      <c r="D31" s="279"/>
-      <c r="E31" s="279"/>
-      <c r="F31" s="279"/>
-      <c r="G31" s="279"/>
-      <c r="H31" s="279"/>
-      <c r="I31" s="279"/>
-      <c r="J31" s="279"/>
-      <c r="K31" s="279"/>
-      <c r="L31" s="279"/>
-      <c r="M31" s="279"/>
-      <c r="N31" s="279"/>
-      <c r="O31" s="279"/>
-      <c r="P31" s="279"/>
-      <c r="Q31" s="279"/>
-      <c r="R31" s="279"/>
-      <c r="S31" s="279"/>
+      <c r="B31" s="278"/>
+      <c r="C31" s="278"/>
+      <c r="D31" s="278"/>
+      <c r="E31" s="278"/>
+      <c r="F31" s="278"/>
+      <c r="G31" s="278"/>
+      <c r="H31" s="278"/>
+      <c r="I31" s="278"/>
+      <c r="J31" s="278"/>
+      <c r="K31" s="278"/>
+      <c r="L31" s="278"/>
+      <c r="M31" s="278"/>
+      <c r="N31" s="278"/>
+      <c r="O31" s="278"/>
+      <c r="P31" s="278"/>
+      <c r="Q31" s="278"/>
+      <c r="R31" s="278"/>
+      <c r="S31" s="278"/>
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="281" t="s">
+      <c r="A32" s="280" t="s">
         <v>508</v>
       </c>
-      <c r="B32" s="279"/>
-      <c r="C32" s="279"/>
-      <c r="D32" s="279"/>
-      <c r="E32" s="279"/>
-      <c r="F32" s="279"/>
-      <c r="G32" s="279"/>
-      <c r="H32" s="279"/>
-      <c r="I32" s="279"/>
-      <c r="J32" s="279"/>
-      <c r="K32" s="279"/>
-      <c r="L32" s="279"/>
-      <c r="M32" s="279"/>
-      <c r="N32" s="279"/>
-      <c r="O32" s="279"/>
-      <c r="P32" s="279"/>
-      <c r="Q32" s="279"/>
-      <c r="R32" s="279"/>
-      <c r="S32" s="279"/>
+      <c r="B32" s="278"/>
+      <c r="C32" s="278"/>
+      <c r="D32" s="278"/>
+      <c r="E32" s="278"/>
+      <c r="F32" s="278"/>
+      <c r="G32" s="278"/>
+      <c r="H32" s="278"/>
+      <c r="I32" s="278"/>
+      <c r="J32" s="278"/>
+      <c r="K32" s="278"/>
+      <c r="L32" s="278"/>
+      <c r="M32" s="278"/>
+      <c r="N32" s="278"/>
+      <c r="O32" s="278"/>
+      <c r="P32" s="278"/>
+      <c r="Q32" s="278"/>
+      <c r="R32" s="278"/>
+      <c r="S32" s="278"/>
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="281" t="s">
+      <c r="A33" s="280" t="s">
         <v>509</v>
       </c>
-      <c r="B33" s="279"/>
-      <c r="C33" s="279"/>
-      <c r="D33" s="279"/>
-      <c r="E33" s="279"/>
-      <c r="F33" s="279"/>
-      <c r="G33" s="279"/>
-      <c r="H33" s="279"/>
-      <c r="I33" s="279"/>
-      <c r="J33" s="279"/>
-      <c r="K33" s="279"/>
-      <c r="L33" s="279"/>
-      <c r="M33" s="279"/>
-      <c r="N33" s="279"/>
-      <c r="O33" s="279"/>
-      <c r="P33" s="279"/>
-      <c r="Q33" s="279"/>
-      <c r="R33" s="279"/>
-      <c r="S33" s="279"/>
+      <c r="B33" s="278"/>
+      <c r="C33" s="278"/>
+      <c r="D33" s="278"/>
+      <c r="E33" s="278"/>
+      <c r="F33" s="278"/>
+      <c r="G33" s="278"/>
+      <c r="H33" s="278"/>
+      <c r="I33" s="278"/>
+      <c r="J33" s="278"/>
+      <c r="K33" s="278"/>
+      <c r="L33" s="278"/>
+      <c r="M33" s="278"/>
+      <c r="N33" s="278"/>
+      <c r="O33" s="278"/>
+      <c r="P33" s="278"/>
+      <c r="Q33" s="278"/>
+      <c r="R33" s="278"/>
+      <c r="S33" s="278"/>
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="281" t="s">
+      <c r="A34" s="280" t="s">
         <v>510</v>
       </c>
-      <c r="B34" s="279"/>
-      <c r="C34" s="279"/>
-      <c r="D34" s="279"/>
-      <c r="E34" s="279"/>
-      <c r="F34" s="279"/>
-      <c r="G34" s="279"/>
-      <c r="H34" s="279"/>
-      <c r="I34" s="279"/>
-      <c r="J34" s="279"/>
-      <c r="K34" s="279"/>
-      <c r="L34" s="279"/>
-      <c r="M34" s="279"/>
-      <c r="N34" s="279"/>
-      <c r="O34" s="279"/>
-      <c r="P34" s="279"/>
-      <c r="Q34" s="279"/>
-      <c r="R34" s="279"/>
-      <c r="S34" s="279"/>
+      <c r="B34" s="278"/>
+      <c r="C34" s="278"/>
+      <c r="D34" s="278"/>
+      <c r="E34" s="278"/>
+      <c r="F34" s="278"/>
+      <c r="G34" s="278"/>
+      <c r="H34" s="278"/>
+      <c r="I34" s="278"/>
+      <c r="J34" s="278"/>
+      <c r="K34" s="278"/>
+      <c r="L34" s="278"/>
+      <c r="M34" s="278"/>
+      <c r="N34" s="278"/>
+      <c r="O34" s="278"/>
+      <c r="P34" s="278"/>
+      <c r="Q34" s="278"/>
+      <c r="R34" s="278"/>
+      <c r="S34" s="278"/>
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="281" t="s">
+      <c r="A35" s="280" t="s">
         <v>511</v>
       </c>
-      <c r="B35" s="279"/>
-      <c r="C35" s="279"/>
-      <c r="D35" s="279"/>
-      <c r="E35" s="279"/>
-      <c r="F35" s="279"/>
-      <c r="G35" s="279"/>
-      <c r="H35" s="279"/>
-      <c r="I35" s="279"/>
-      <c r="J35" s="279"/>
-      <c r="K35" s="279"/>
-      <c r="L35" s="279"/>
-      <c r="M35" s="279"/>
-      <c r="N35" s="279"/>
-      <c r="O35" s="279"/>
-      <c r="P35" s="279"/>
-      <c r="Q35" s="279"/>
-      <c r="R35" s="279"/>
-      <c r="S35" s="279"/>
+      <c r="B35" s="278"/>
+      <c r="C35" s="278"/>
+      <c r="D35" s="278"/>
+      <c r="E35" s="278"/>
+      <c r="F35" s="278"/>
+      <c r="G35" s="278"/>
+      <c r="H35" s="278"/>
+      <c r="I35" s="278"/>
+      <c r="J35" s="278"/>
+      <c r="K35" s="278"/>
+      <c r="L35" s="278"/>
+      <c r="M35" s="278"/>
+      <c r="N35" s="278"/>
+      <c r="O35" s="278"/>
+      <c r="P35" s="278"/>
+      <c r="Q35" s="278"/>
+      <c r="R35" s="278"/>
+      <c r="S35" s="278"/>
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="281" t="s">
+      <c r="A36" s="280" t="s">
         <v>512</v>
       </c>
-      <c r="B36" s="279"/>
-      <c r="C36" s="279"/>
-      <c r="D36" s="279"/>
-      <c r="E36" s="279"/>
-      <c r="F36" s="279"/>
-      <c r="G36" s="279"/>
-      <c r="H36" s="279"/>
-      <c r="I36" s="279"/>
-      <c r="J36" s="279"/>
-      <c r="K36" s="279"/>
-      <c r="L36" s="279"/>
-      <c r="M36" s="279"/>
-      <c r="N36" s="279"/>
-      <c r="O36" s="279"/>
-      <c r="P36" s="279"/>
-      <c r="Q36" s="279"/>
-      <c r="R36" s="279"/>
-      <c r="S36" s="279"/>
+      <c r="B36" s="278"/>
+      <c r="C36" s="278"/>
+      <c r="D36" s="278"/>
+      <c r="E36" s="278"/>
+      <c r="F36" s="278"/>
+      <c r="G36" s="278"/>
+      <c r="H36" s="278"/>
+      <c r="I36" s="278"/>
+      <c r="J36" s="278"/>
+      <c r="K36" s="278"/>
+      <c r="L36" s="278"/>
+      <c r="M36" s="278"/>
+      <c r="N36" s="278"/>
+      <c r="O36" s="278"/>
+      <c r="P36" s="278"/>
+      <c r="Q36" s="278"/>
+      <c r="R36" s="278"/>
+      <c r="S36" s="278"/>
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="292" t="s">
+      <c r="A37" s="291" t="s">
         <v>513</v>
       </c>
-      <c r="B37" s="279"/>
-      <c r="C37" s="279"/>
-      <c r="D37" s="279"/>
-      <c r="E37" s="279"/>
-      <c r="F37" s="279"/>
-      <c r="G37" s="279"/>
-      <c r="H37" s="279"/>
-      <c r="I37" s="279"/>
-      <c r="J37" s="279"/>
-      <c r="K37" s="279"/>
-      <c r="L37" s="279"/>
-      <c r="M37" s="279"/>
-      <c r="N37" s="279"/>
-      <c r="O37" s="279"/>
-      <c r="P37" s="279"/>
-      <c r="Q37" s="279"/>
-      <c r="R37" s="279"/>
-      <c r="S37" s="279"/>
+      <c r="B37" s="278"/>
+      <c r="C37" s="278"/>
+      <c r="D37" s="278"/>
+      <c r="E37" s="278"/>
+      <c r="F37" s="278"/>
+      <c r="G37" s="278"/>
+      <c r="H37" s="278"/>
+      <c r="I37" s="278"/>
+      <c r="J37" s="278"/>
+      <c r="K37" s="278"/>
+      <c r="L37" s="278"/>
+      <c r="M37" s="278"/>
+      <c r="N37" s="278"/>
+      <c r="O37" s="278"/>
+      <c r="P37" s="278"/>
+      <c r="Q37" s="278"/>
+      <c r="R37" s="278"/>
+      <c r="S37" s="278"/>
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="38" t="s">
         <v>447</v>
       </c>
-      <c r="B39" s="295" t="s">
+      <c r="B39" s="294" t="s">
         <v>514</v>
       </c>
-      <c r="C39" s="279"/>
-      <c r="D39" s="279"/>
-      <c r="E39" s="293" t="s">
+      <c r="C39" s="278"/>
+      <c r="D39" s="278"/>
+      <c r="E39" s="292" t="s">
         <v>515</v>
       </c>
-      <c r="F39" s="279"/>
-      <c r="G39" s="279"/>
-      <c r="H39" s="296" t="s">
+      <c r="F39" s="278"/>
+      <c r="G39" s="278"/>
+      <c r="H39" s="295" t="s">
         <v>516</v>
       </c>
-      <c r="I39" s="279"/>
-      <c r="J39" s="279"/>
-      <c r="K39" s="289" t="s">
+      <c r="I39" s="278"/>
+      <c r="J39" s="278"/>
+      <c r="K39" s="288" t="s">
         <v>517</v>
       </c>
-      <c r="L39" s="279"/>
-      <c r="M39" s="279"/>
-      <c r="N39" s="287" t="s">
+      <c r="L39" s="278"/>
+      <c r="M39" s="278"/>
+      <c r="N39" s="286" t="s">
         <v>45</v>
       </c>
-      <c r="O39" s="279"/>
-      <c r="P39" s="279"/>
-      <c r="Q39" s="294" t="s">
+      <c r="O39" s="278"/>
+      <c r="P39" s="278"/>
+      <c r="Q39" s="293" t="s">
         <v>518</v>
       </c>
-      <c r="R39" s="279"/>
-      <c r="S39" s="279"/>
+      <c r="R39" s="278"/>
+      <c r="S39" s="278"/>
     </row>
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="H20:M20"/>
     <mergeCell ref="A16:S16"/>
-    <mergeCell ref="H20:M20"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -12691,14 +12694,13 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -12707,6 +12709,7 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -12714,7 +12717,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -12762,14 +12765,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="298" t="s">
+      <c r="A1" s="297" t="s">
         <v>519</v>
       </c>
-      <c r="B1" s="272"/>
-      <c r="C1" s="272"/>
-      <c r="D1" s="272"/>
-      <c r="E1" s="272"/>
-      <c r="F1" s="273"/>
+      <c r="B1" s="271"/>
+      <c r="C1" s="271"/>
+      <c r="D1" s="271"/>
+      <c r="E1" s="271"/>
+      <c r="F1" s="272"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
@@ -13134,13 +13137,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="298" t="s">
+      <c r="A1" s="297" t="s">
         <v>526</v>
       </c>
-      <c r="B1" s="272"/>
-      <c r="C1" s="272"/>
-      <c r="D1" s="272"/>
-      <c r="E1" s="273"/>
+      <c r="B1" s="271"/>
+      <c r="C1" s="271"/>
+      <c r="D1" s="271"/>
+      <c r="E1" s="272"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="31" t="s">
@@ -14222,13 +14225,13 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="299" t="s">
+      <c r="A2" s="298" t="s">
         <v>670</v>
       </c>
-      <c r="B2" s="279"/>
-      <c r="C2" s="279"/>
-      <c r="D2" s="279"/>
-      <c r="E2" s="279"/>
+      <c r="B2" s="278"/>
+      <c r="C2" s="278"/>
+      <c r="D2" s="278"/>
+      <c r="E2" s="278"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="255" t="s">
@@ -14282,13 +14285,13 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="267" t="s">
+      <c r="A7" s="266" t="s">
         <v>680</v>
       </c>
       <c r="B7" s="250" t="s">
         <v>681</v>
       </c>
-      <c r="C7" s="268" t="s">
+      <c r="C7" s="267" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="250" t="s">
@@ -14305,8 +14308,8 @@
       <c r="B8" s="250" t="s">
         <v>683</v>
       </c>
-      <c r="C8" s="257" t="s">
-        <v>128</v>
+      <c r="C8" s="269" t="s">
+        <v>22</v>
       </c>
       <c r="D8" s="250" t="s">
         <v>684</v>
@@ -14322,7 +14325,7 @@
       <c r="B9" s="250" t="s">
         <v>686</v>
       </c>
-      <c r="C9" s="270" t="s">
+      <c r="C9" s="268" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="250" t="s">
@@ -14526,8 +14529,8 @@
       <c r="B22" s="250" t="s">
         <v>719</v>
       </c>
-      <c r="C22" s="266" t="s">
-        <v>128</v>
+      <c r="C22" s="269" t="s">
+        <v>22</v>
       </c>
       <c r="D22" s="250" t="s">
         <v>720</v>
@@ -14537,14 +14540,14 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="267" t="s">
+      <c r="A23" s="266" t="s">
         <v>680</v>
       </c>
       <c r="B23" s="250" t="s">
         <v>722</v>
       </c>
       <c r="C23" s="269" t="s">
-        <v>128</v>
+        <v>22</v>
       </c>
       <c r="D23" s="250" t="s">
         <v>723</v>
@@ -14554,13 +14557,13 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="267" t="s">
+      <c r="A24" s="266" t="s">
         <v>680</v>
       </c>
       <c r="B24" s="250" t="s">
         <v>725</v>
       </c>
-      <c r="C24" s="270" t="s">
+      <c r="C24" s="268" t="s">
         <v>22</v>
       </c>
       <c r="D24" s="250" t="s">
@@ -14932,17 +14935,17 @@
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="300" t="s">
+      <c r="A16" s="299" t="s">
         <v>806</v>
       </c>
-      <c r="B16" s="279"/>
-      <c r="C16" s="279"/>
-      <c r="D16" s="279"/>
-      <c r="E16" s="279"/>
-      <c r="F16" s="279"/>
-      <c r="G16" s="279"/>
-      <c r="H16" s="279"/>
-      <c r="I16" s="279"/>
+      <c r="B16" s="278"/>
+      <c r="C16" s="278"/>
+      <c r="D16" s="278"/>
+      <c r="E16" s="278"/>
+      <c r="F16" s="278"/>
+      <c r="G16" s="278"/>
+      <c r="H16" s="278"/>
+      <c r="I16" s="278"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(tracker): P2 measurements done, 12 of 20
CLV re-read with a control (the control changed the reading), confidence
tiers answered (no, and worse than no), completeness bands measured (the
floor works, 0.35 is the real break).

Adds one decision the measurements surfaced: the push gate still selects
the worst-measured tier, left documented rather than rewritten on n=69.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28923A89-6BB3-42B8-ABFA-385A0BA3B857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BB2F352-E352-4162-B1D5-10A9EC58CB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1613" uniqueCount="807">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1618" uniqueCount="810">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -2203,19 +2203,19 @@
     <t>P0 capture check</t>
   </si>
   <si>
-    <t>The sharpest signal available. Currently -3.58% on n=27 - the market moving AWAY from our picks.</t>
+    <t>DONE — and the CONTROL changed the reading. Favoured side -3.47% vs the side NOT favoured +0.83%, a -4.30pp gap (n=81 each). But football's control is ALSO negative (-2.40%), so a real part of the raw -3.61% is systematic price drift rather than the model. The control is not clean either: for a 3-way market it is the less-likely of home/away, usually the underdog, whose prices are longer and more volatile. Directional evidence against an edge; NOT a number to quote precisely. The naive -4.00% headline would have overstated it.</t>
   </si>
   <si>
     <t>Do confidence tiers mean anything?</t>
   </si>
   <si>
-    <t>If HIGH picks are not measurably better than MEDIUM, the badge is decoration.</t>
+    <t>ANSWERED: no, and worse than no. HIGH claims 74.1% delivers 60.9% (n=69); MEDIUM claims 57.8% delivers 68.5% (n=89) — the badge pointed users at the WEAKER set. Intervals overlap so the inversion is not established; the calibration gap is. Badge hidden from mobile (7233029), field still stored as measurement data. The push gate still fires on HIGH and is knowingly left in place — n=69 is too thin to rewrite it on, and exactly one real token exists — but it MUST be resolved before push reaches real users.</t>
   </si>
   <si>
     <t>Re-run completeness-vs-correctness</t>
   </si>
   <si>
-    <t>Was n=84 and inconclusive. Tests whether the 0.25 floor sits where it should or merely looked reasonable.</t>
+    <t>DONE: &lt;0.25 33.3% (n=9), 0.25-0.35 37.5% (n=16), &gt;=0.35 69.9% (n=123). The floor works, but the real break is at 0.35 — where mobile's own LOW_CONFIDENCE_COMPLETENESS already sits. The 0.25 choice was defensible on the extremeness evidence used at the time (85% of picks below it were &gt;=0.90 confident vs 6% above); correctness points higher. NOT changed: n=16 in the middle band, and the decision belongs with the pre-registration rather than to whoever is looking at the data.</t>
   </si>
   <si>
     <t>P3</t>
@@ -2291,6 +2291,15 @@
   </si>
   <si>
     <t>DONE (8f794e0). pick_snapshots, captured hourly for fixtures 4-8 HOURS out — not next to the closing-odds capture, which would have made CLV meaningless by construction: taken/closing - 1 is ~0 when both prices are recorded fifteen minutes apart, so the metric would read reassuringly neutral while measuring nothing. Delegates to _bulk_best_picks, the feed's own selection, with a test asserting the delegation. One row per fixture. Verified live: an ATP pick at 2.17, p=0.536, T-7.3h. NOTE: nothing before this commit is recoverable — the ROI/CLV clock starts now.</t>
+  </si>
+  <si>
+    <t>DECIDE: the push gate still selects the worst-measured tier</t>
+  </si>
+  <si>
+    <t>pre-registration</t>
+  </si>
+  <si>
+    <t>notify_users fires only for HIGH, which measured 60.9% against MEDIUM's 68.5%. Left documented rather than rewritten: n=69 is too thin, and one real push token means waiting is nearly free. Must be recalibrated or replaced with a MEASURED criterion before push reaches real users — not simply widened.</t>
   </si>
   <si>
     <t>P0 blocks everything · P1 builds the measurement · P2 reads it · P3 decides on it · HOLD = deliberately not doing until the read lands</t>
@@ -2541,7 +2550,7 @@
     <numFmt numFmtId="164" formatCode="dd\ mmm"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="83" x14ac:knownFonts="1">
+  <fonts count="84" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2977,6 +2986,12 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -3652,7 +3667,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="300">
+  <cellXfs count="303">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4447,6 +4462,15 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="82" fillId="65" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="83" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="83" fillId="65" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="83" fillId="68" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4858,46 +4882,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="273" t="s">
+      <c r="A1" s="276" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="271"/>
-      <c r="C1" s="271"/>
-      <c r="D1" s="271"/>
-      <c r="E1" s="271"/>
-      <c r="F1" s="271"/>
-      <c r="G1" s="271"/>
-      <c r="H1" s="271"/>
-      <c r="I1" s="271"/>
-      <c r="J1" s="271"/>
-      <c r="K1" s="271"/>
-      <c r="L1" s="271"/>
-      <c r="M1" s="271"/>
-      <c r="N1" s="271"/>
-      <c r="O1" s="271"/>
-      <c r="P1" s="271"/>
-      <c r="Q1" s="272"/>
+      <c r="B1" s="274"/>
+      <c r="C1" s="274"/>
+      <c r="D1" s="274"/>
+      <c r="E1" s="274"/>
+      <c r="F1" s="274"/>
+      <c r="G1" s="274"/>
+      <c r="H1" s="274"/>
+      <c r="I1" s="274"/>
+      <c r="J1" s="274"/>
+      <c r="K1" s="274"/>
+      <c r="L1" s="274"/>
+      <c r="M1" s="274"/>
+      <c r="N1" s="274"/>
+      <c r="O1" s="274"/>
+      <c r="P1" s="274"/>
+      <c r="Q1" s="275"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="270" t="s">
+      <c r="A2" s="273" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="271"/>
-      <c r="C2" s="271"/>
-      <c r="D2" s="271"/>
-      <c r="E2" s="271"/>
-      <c r="F2" s="271"/>
-      <c r="G2" s="271"/>
-      <c r="H2" s="271"/>
-      <c r="I2" s="271"/>
-      <c r="J2" s="271"/>
-      <c r="K2" s="271"/>
-      <c r="L2" s="271"/>
-      <c r="M2" s="271"/>
-      <c r="N2" s="271"/>
-      <c r="O2" s="271"/>
-      <c r="P2" s="271"/>
-      <c r="Q2" s="272"/>
+      <c r="B2" s="274"/>
+      <c r="C2" s="274"/>
+      <c r="D2" s="274"/>
+      <c r="E2" s="274"/>
+      <c r="F2" s="274"/>
+      <c r="G2" s="274"/>
+      <c r="H2" s="274"/>
+      <c r="I2" s="274"/>
+      <c r="J2" s="274"/>
+      <c r="K2" s="274"/>
+      <c r="L2" s="274"/>
+      <c r="M2" s="274"/>
+      <c r="N2" s="274"/>
+      <c r="O2" s="274"/>
+      <c r="P2" s="274"/>
+      <c r="Q2" s="275"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
@@ -11840,852 +11864,852 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="289" t="s">
+      <c r="A1" s="292" t="s">
         <v>449</v>
       </c>
-      <c r="B1" s="278"/>
-      <c r="C1" s="278"/>
-      <c r="D1" s="278"/>
-      <c r="E1" s="278"/>
-      <c r="F1" s="278"/>
-      <c r="G1" s="278"/>
-      <c r="H1" s="278"/>
-      <c r="I1" s="278"/>
-      <c r="J1" s="278"/>
-      <c r="K1" s="278"/>
-      <c r="L1" s="278"/>
-      <c r="M1" s="278"/>
-      <c r="N1" s="278"/>
-      <c r="O1" s="278"/>
-      <c r="P1" s="278"/>
-      <c r="Q1" s="278"/>
-      <c r="R1" s="278"/>
-      <c r="S1" s="278"/>
+      <c r="B1" s="281"/>
+      <c r="C1" s="281"/>
+      <c r="D1" s="281"/>
+      <c r="E1" s="281"/>
+      <c r="F1" s="281"/>
+      <c r="G1" s="281"/>
+      <c r="H1" s="281"/>
+      <c r="I1" s="281"/>
+      <c r="J1" s="281"/>
+      <c r="K1" s="281"/>
+      <c r="L1" s="281"/>
+      <c r="M1" s="281"/>
+      <c r="N1" s="281"/>
+      <c r="O1" s="281"/>
+      <c r="P1" s="281"/>
+      <c r="Q1" s="281"/>
+      <c r="R1" s="281"/>
+      <c r="S1" s="281"/>
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="296" t="s">
+      <c r="A2" s="299" t="s">
         <v>450</v>
       </c>
-      <c r="B2" s="278"/>
-      <c r="C2" s="278"/>
-      <c r="D2" s="278"/>
-      <c r="E2" s="278"/>
-      <c r="F2" s="278"/>
-      <c r="G2" s="278"/>
-      <c r="H2" s="278"/>
-      <c r="I2" s="278"/>
-      <c r="J2" s="278"/>
-      <c r="K2" s="278"/>
-      <c r="L2" s="278"/>
-      <c r="M2" s="278"/>
-      <c r="N2" s="278"/>
-      <c r="O2" s="278"/>
-      <c r="P2" s="278"/>
-      <c r="Q2" s="278"/>
-      <c r="R2" s="278"/>
-      <c r="S2" s="278"/>
+      <c r="B2" s="281"/>
+      <c r="C2" s="281"/>
+      <c r="D2" s="281"/>
+      <c r="E2" s="281"/>
+      <c r="F2" s="281"/>
+      <c r="G2" s="281"/>
+      <c r="H2" s="281"/>
+      <c r="I2" s="281"/>
+      <c r="J2" s="281"/>
+      <c r="K2" s="281"/>
+      <c r="L2" s="281"/>
+      <c r="M2" s="281"/>
+      <c r="N2" s="281"/>
+      <c r="O2" s="281"/>
+      <c r="P2" s="281"/>
+      <c r="Q2" s="281"/>
+      <c r="R2" s="281"/>
+      <c r="S2" s="281"/>
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="284" t="s">
+      <c r="A4" s="287" t="s">
         <v>451</v>
       </c>
-      <c r="B4" s="278"/>
-      <c r="C4" s="278"/>
-      <c r="D4" s="278"/>
-      <c r="E4" s="278"/>
-      <c r="F4" s="278"/>
-      <c r="G4" s="278"/>
-      <c r="H4" s="278"/>
-      <c r="I4" s="278"/>
-      <c r="J4" s="278"/>
-      <c r="K4" s="278"/>
-      <c r="L4" s="278"/>
-      <c r="M4" s="278"/>
-      <c r="N4" s="278"/>
-      <c r="O4" s="278"/>
-      <c r="P4" s="278"/>
-      <c r="Q4" s="278"/>
-      <c r="R4" s="278"/>
-      <c r="S4" s="278"/>
+      <c r="B4" s="281"/>
+      <c r="C4" s="281"/>
+      <c r="D4" s="281"/>
+      <c r="E4" s="281"/>
+      <c r="F4" s="281"/>
+      <c r="G4" s="281"/>
+      <c r="H4" s="281"/>
+      <c r="I4" s="281"/>
+      <c r="J4" s="281"/>
+      <c r="K4" s="281"/>
+      <c r="L4" s="281"/>
+      <c r="M4" s="281"/>
+      <c r="N4" s="281"/>
+      <c r="O4" s="281"/>
+      <c r="P4" s="281"/>
+      <c r="Q4" s="281"/>
+      <c r="R4" s="281"/>
+      <c r="S4" s="281"/>
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="37" t="s">
         <v>452</v>
       </c>
-      <c r="B5" s="274" t="s">
+      <c r="B5" s="277" t="s">
         <v>453</v>
       </c>
-      <c r="C5" s="275"/>
-      <c r="D5" s="276"/>
-      <c r="E5" s="279" t="s">
+      <c r="C5" s="278"/>
+      <c r="D5" s="279"/>
+      <c r="E5" s="282" t="s">
         <v>454</v>
       </c>
-      <c r="F5" s="275"/>
-      <c r="G5" s="276"/>
-      <c r="H5" s="279" t="s">
+      <c r="F5" s="278"/>
+      <c r="G5" s="279"/>
+      <c r="H5" s="282" t="s">
         <v>455</v>
       </c>
-      <c r="I5" s="275"/>
-      <c r="J5" s="276"/>
-      <c r="K5" s="274" t="s">
+      <c r="I5" s="278"/>
+      <c r="J5" s="279"/>
+      <c r="K5" s="277" t="s">
         <v>456</v>
       </c>
-      <c r="L5" s="275"/>
-      <c r="M5" s="276"/>
-      <c r="N5" s="281" t="s">
+      <c r="L5" s="278"/>
+      <c r="M5" s="279"/>
+      <c r="N5" s="284" t="s">
         <v>457</v>
       </c>
-      <c r="O5" s="275"/>
-      <c r="P5" s="276"/>
-      <c r="Q5" s="281" t="s">
+      <c r="O5" s="278"/>
+      <c r="P5" s="279"/>
+      <c r="Q5" s="284" t="s">
         <v>458</v>
       </c>
-      <c r="R5" s="275"/>
-      <c r="S5" s="276"/>
+      <c r="R5" s="278"/>
+      <c r="S5" s="279"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="277" t="s">
+      <c r="B6" s="280" t="s">
         <v>459</v>
       </c>
-      <c r="C6" s="278"/>
-      <c r="D6" s="278"/>
-      <c r="E6" s="278"/>
-      <c r="F6" s="278"/>
-      <c r="G6" s="278"/>
-      <c r="H6" s="278"/>
-      <c r="I6" s="278"/>
-      <c r="J6" s="278"/>
-      <c r="K6" s="278"/>
-      <c r="L6" s="278"/>
-      <c r="M6" s="278"/>
-      <c r="N6" s="278"/>
-      <c r="O6" s="278"/>
-      <c r="P6" s="278"/>
-      <c r="Q6" s="278"/>
-      <c r="R6" s="278"/>
-      <c r="S6" s="278"/>
+      <c r="C6" s="281"/>
+      <c r="D6" s="281"/>
+      <c r="E6" s="281"/>
+      <c r="F6" s="281"/>
+      <c r="G6" s="281"/>
+      <c r="H6" s="281"/>
+      <c r="I6" s="281"/>
+      <c r="J6" s="281"/>
+      <c r="K6" s="281"/>
+      <c r="L6" s="281"/>
+      <c r="M6" s="281"/>
+      <c r="N6" s="281"/>
+      <c r="O6" s="281"/>
+      <c r="P6" s="281"/>
+      <c r="Q6" s="281"/>
+      <c r="R6" s="281"/>
+      <c r="S6" s="281"/>
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="284" t="s">
+      <c r="A7" s="287" t="s">
         <v>460</v>
       </c>
-      <c r="B7" s="278"/>
-      <c r="C7" s="278"/>
-      <c r="D7" s="278"/>
-      <c r="E7" s="278"/>
-      <c r="F7" s="278"/>
-      <c r="G7" s="278"/>
-      <c r="H7" s="278"/>
-      <c r="I7" s="278"/>
-      <c r="J7" s="278"/>
-      <c r="K7" s="278"/>
-      <c r="L7" s="278"/>
-      <c r="M7" s="278"/>
-      <c r="N7" s="278"/>
-      <c r="O7" s="278"/>
-      <c r="P7" s="278"/>
-      <c r="Q7" s="278"/>
-      <c r="R7" s="278"/>
-      <c r="S7" s="278"/>
+      <c r="B7" s="281"/>
+      <c r="C7" s="281"/>
+      <c r="D7" s="281"/>
+      <c r="E7" s="281"/>
+      <c r="F7" s="281"/>
+      <c r="G7" s="281"/>
+      <c r="H7" s="281"/>
+      <c r="I7" s="281"/>
+      <c r="J7" s="281"/>
+      <c r="K7" s="281"/>
+      <c r="L7" s="281"/>
+      <c r="M7" s="281"/>
+      <c r="N7" s="281"/>
+      <c r="O7" s="281"/>
+      <c r="P7" s="281"/>
+      <c r="Q7" s="281"/>
+      <c r="R7" s="281"/>
+      <c r="S7" s="281"/>
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="37" t="s">
         <v>461</v>
       </c>
-      <c r="B8" s="287" t="s">
+      <c r="B8" s="290" t="s">
         <v>462</v>
       </c>
-      <c r="C8" s="275"/>
-      <c r="D8" s="275"/>
-      <c r="E8" s="275"/>
-      <c r="F8" s="275"/>
-      <c r="G8" s="275"/>
-      <c r="H8" s="275"/>
-      <c r="I8" s="275"/>
-      <c r="J8" s="276"/>
-      <c r="K8" s="287" t="s">
+      <c r="C8" s="278"/>
+      <c r="D8" s="278"/>
+      <c r="E8" s="278"/>
+      <c r="F8" s="278"/>
+      <c r="G8" s="278"/>
+      <c r="H8" s="278"/>
+      <c r="I8" s="278"/>
+      <c r="J8" s="279"/>
+      <c r="K8" s="290" t="s">
         <v>463</v>
       </c>
-      <c r="L8" s="275"/>
-      <c r="M8" s="275"/>
-      <c r="N8" s="275"/>
-      <c r="O8" s="275"/>
-      <c r="P8" s="275"/>
-      <c r="Q8" s="275"/>
-      <c r="R8" s="275"/>
-      <c r="S8" s="276"/>
+      <c r="L8" s="278"/>
+      <c r="M8" s="278"/>
+      <c r="N8" s="278"/>
+      <c r="O8" s="278"/>
+      <c r="P8" s="278"/>
+      <c r="Q8" s="278"/>
+      <c r="R8" s="278"/>
+      <c r="S8" s="279"/>
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B9" s="277" t="s">
+      <c r="B9" s="280" t="s">
         <v>459</v>
       </c>
-      <c r="C9" s="278"/>
-      <c r="D9" s="278"/>
-      <c r="E9" s="278"/>
-      <c r="F9" s="278"/>
-      <c r="G9" s="278"/>
-      <c r="H9" s="278"/>
-      <c r="I9" s="278"/>
-      <c r="J9" s="278"/>
-      <c r="K9" s="278"/>
-      <c r="L9" s="278"/>
-      <c r="M9" s="278"/>
-      <c r="N9" s="278"/>
-      <c r="O9" s="278"/>
-      <c r="P9" s="278"/>
-      <c r="Q9" s="278"/>
-      <c r="R9" s="278"/>
-      <c r="S9" s="278"/>
+      <c r="C9" s="281"/>
+      <c r="D9" s="281"/>
+      <c r="E9" s="281"/>
+      <c r="F9" s="281"/>
+      <c r="G9" s="281"/>
+      <c r="H9" s="281"/>
+      <c r="I9" s="281"/>
+      <c r="J9" s="281"/>
+      <c r="K9" s="281"/>
+      <c r="L9" s="281"/>
+      <c r="M9" s="281"/>
+      <c r="N9" s="281"/>
+      <c r="O9" s="281"/>
+      <c r="P9" s="281"/>
+      <c r="Q9" s="281"/>
+      <c r="R9" s="281"/>
+      <c r="S9" s="281"/>
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="284" t="s">
+      <c r="A10" s="287" t="s">
         <v>464</v>
       </c>
-      <c r="B10" s="278"/>
-      <c r="C10" s="278"/>
-      <c r="D10" s="278"/>
-      <c r="E10" s="278"/>
-      <c r="F10" s="278"/>
-      <c r="G10" s="278"/>
-      <c r="H10" s="278"/>
-      <c r="I10" s="278"/>
-      <c r="J10" s="278"/>
-      <c r="K10" s="278"/>
-      <c r="L10" s="278"/>
-      <c r="M10" s="278"/>
-      <c r="N10" s="278"/>
-      <c r="O10" s="278"/>
-      <c r="P10" s="278"/>
-      <c r="Q10" s="278"/>
-      <c r="R10" s="278"/>
-      <c r="S10" s="278"/>
+      <c r="B10" s="281"/>
+      <c r="C10" s="281"/>
+      <c r="D10" s="281"/>
+      <c r="E10" s="281"/>
+      <c r="F10" s="281"/>
+      <c r="G10" s="281"/>
+      <c r="H10" s="281"/>
+      <c r="I10" s="281"/>
+      <c r="J10" s="281"/>
+      <c r="K10" s="281"/>
+      <c r="L10" s="281"/>
+      <c r="M10" s="281"/>
+      <c r="N10" s="281"/>
+      <c r="O10" s="281"/>
+      <c r="P10" s="281"/>
+      <c r="Q10" s="281"/>
+      <c r="R10" s="281"/>
+      <c r="S10" s="281"/>
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="37" t="s">
         <v>465</v>
       </c>
-      <c r="B11" s="274" t="s">
+      <c r="B11" s="277" t="s">
         <v>466</v>
       </c>
-      <c r="C11" s="275"/>
-      <c r="D11" s="276"/>
-      <c r="E11" s="274" t="s">
+      <c r="C11" s="278"/>
+      <c r="D11" s="279"/>
+      <c r="E11" s="277" t="s">
         <v>467</v>
       </c>
-      <c r="F11" s="275"/>
-      <c r="G11" s="276"/>
-      <c r="H11" s="274" t="s">
+      <c r="F11" s="278"/>
+      <c r="G11" s="279"/>
+      <c r="H11" s="277" t="s">
         <v>468</v>
       </c>
-      <c r="I11" s="275"/>
-      <c r="J11" s="276"/>
-      <c r="K11" s="279" t="s">
+      <c r="I11" s="278"/>
+      <c r="J11" s="279"/>
+      <c r="K11" s="282" t="s">
         <v>469</v>
       </c>
-      <c r="L11" s="275"/>
-      <c r="M11" s="276"/>
-      <c r="N11" s="274" t="s">
+      <c r="L11" s="278"/>
+      <c r="M11" s="279"/>
+      <c r="N11" s="277" t="s">
         <v>470</v>
       </c>
-      <c r="O11" s="275"/>
-      <c r="P11" s="276"/>
-      <c r="Q11" s="274" t="s">
+      <c r="O11" s="278"/>
+      <c r="P11" s="279"/>
+      <c r="Q11" s="277" t="s">
         <v>471</v>
       </c>
-      <c r="R11" s="275"/>
-      <c r="S11" s="276"/>
+      <c r="R11" s="278"/>
+      <c r="S11" s="279"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B12" s="277" t="s">
+      <c r="B12" s="280" t="s">
         <v>459</v>
       </c>
-      <c r="C12" s="278"/>
-      <c r="D12" s="278"/>
-      <c r="E12" s="278"/>
-      <c r="F12" s="278"/>
-      <c r="G12" s="278"/>
-      <c r="H12" s="278"/>
-      <c r="I12" s="278"/>
-      <c r="J12" s="278"/>
-      <c r="K12" s="278"/>
-      <c r="L12" s="278"/>
-      <c r="M12" s="278"/>
-      <c r="N12" s="278"/>
-      <c r="O12" s="278"/>
-      <c r="P12" s="278"/>
-      <c r="Q12" s="278"/>
-      <c r="R12" s="278"/>
-      <c r="S12" s="278"/>
+      <c r="C12" s="281"/>
+      <c r="D12" s="281"/>
+      <c r="E12" s="281"/>
+      <c r="F12" s="281"/>
+      <c r="G12" s="281"/>
+      <c r="H12" s="281"/>
+      <c r="I12" s="281"/>
+      <c r="J12" s="281"/>
+      <c r="K12" s="281"/>
+      <c r="L12" s="281"/>
+      <c r="M12" s="281"/>
+      <c r="N12" s="281"/>
+      <c r="O12" s="281"/>
+      <c r="P12" s="281"/>
+      <c r="Q12" s="281"/>
+      <c r="R12" s="281"/>
+      <c r="S12" s="281"/>
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="284" t="s">
+      <c r="A13" s="287" t="s">
         <v>472</v>
       </c>
-      <c r="B13" s="278"/>
-      <c r="C13" s="278"/>
-      <c r="D13" s="278"/>
-      <c r="E13" s="278"/>
-      <c r="F13" s="278"/>
-      <c r="G13" s="278"/>
-      <c r="H13" s="278"/>
-      <c r="I13" s="278"/>
-      <c r="J13" s="278"/>
-      <c r="K13" s="278"/>
-      <c r="L13" s="278"/>
-      <c r="M13" s="278"/>
-      <c r="N13" s="278"/>
-      <c r="O13" s="278"/>
-      <c r="P13" s="278"/>
-      <c r="Q13" s="278"/>
-      <c r="R13" s="278"/>
-      <c r="S13" s="278"/>
+      <c r="B13" s="281"/>
+      <c r="C13" s="281"/>
+      <c r="D13" s="281"/>
+      <c r="E13" s="281"/>
+      <c r="F13" s="281"/>
+      <c r="G13" s="281"/>
+      <c r="H13" s="281"/>
+      <c r="I13" s="281"/>
+      <c r="J13" s="281"/>
+      <c r="K13" s="281"/>
+      <c r="L13" s="281"/>
+      <c r="M13" s="281"/>
+      <c r="N13" s="281"/>
+      <c r="O13" s="281"/>
+      <c r="P13" s="281"/>
+      <c r="Q13" s="281"/>
+      <c r="R13" s="281"/>
+      <c r="S13" s="281"/>
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="37" t="s">
         <v>473</v>
       </c>
-      <c r="B14" s="282" t="s">
+      <c r="B14" s="285" t="s">
         <v>474</v>
       </c>
-      <c r="C14" s="275"/>
-      <c r="D14" s="275"/>
-      <c r="E14" s="275"/>
-      <c r="F14" s="275"/>
-      <c r="G14" s="276"/>
-      <c r="H14" s="282" t="s">
+      <c r="C14" s="278"/>
+      <c r="D14" s="278"/>
+      <c r="E14" s="278"/>
+      <c r="F14" s="278"/>
+      <c r="G14" s="279"/>
+      <c r="H14" s="285" t="s">
         <v>475</v>
       </c>
-      <c r="I14" s="275"/>
-      <c r="J14" s="275"/>
-      <c r="K14" s="275"/>
-      <c r="L14" s="275"/>
-      <c r="M14" s="276"/>
-      <c r="N14" s="282" t="s">
+      <c r="I14" s="278"/>
+      <c r="J14" s="278"/>
+      <c r="K14" s="278"/>
+      <c r="L14" s="278"/>
+      <c r="M14" s="279"/>
+      <c r="N14" s="285" t="s">
         <v>476</v>
       </c>
-      <c r="O14" s="275"/>
-      <c r="P14" s="276"/>
-      <c r="Q14" s="279" t="s">
+      <c r="O14" s="278"/>
+      <c r="P14" s="279"/>
+      <c r="Q14" s="282" t="s">
         <v>477</v>
       </c>
-      <c r="R14" s="275"/>
-      <c r="S14" s="276"/>
+      <c r="R14" s="278"/>
+      <c r="S14" s="279"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B15" s="277" t="s">
+      <c r="B15" s="280" t="s">
         <v>478</v>
       </c>
-      <c r="C15" s="278"/>
-      <c r="D15" s="278"/>
-      <c r="E15" s="278"/>
-      <c r="F15" s="278"/>
-      <c r="G15" s="278"/>
-      <c r="H15" s="278"/>
-      <c r="I15" s="278"/>
-      <c r="J15" s="278"/>
-      <c r="K15" s="278"/>
-      <c r="L15" s="278"/>
-      <c r="M15" s="278"/>
-      <c r="N15" s="278"/>
-      <c r="O15" s="278"/>
-      <c r="P15" s="278"/>
-      <c r="Q15" s="278"/>
-      <c r="R15" s="278"/>
-      <c r="S15" s="278"/>
+      <c r="C15" s="281"/>
+      <c r="D15" s="281"/>
+      <c r="E15" s="281"/>
+      <c r="F15" s="281"/>
+      <c r="G15" s="281"/>
+      <c r="H15" s="281"/>
+      <c r="I15" s="281"/>
+      <c r="J15" s="281"/>
+      <c r="K15" s="281"/>
+      <c r="L15" s="281"/>
+      <c r="M15" s="281"/>
+      <c r="N15" s="281"/>
+      <c r="O15" s="281"/>
+      <c r="P15" s="281"/>
+      <c r="Q15" s="281"/>
+      <c r="R15" s="281"/>
+      <c r="S15" s="281"/>
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="284" t="s">
+      <c r="A16" s="287" t="s">
         <v>479</v>
       </c>
-      <c r="B16" s="278"/>
-      <c r="C16" s="278"/>
-      <c r="D16" s="278"/>
-      <c r="E16" s="278"/>
-      <c r="F16" s="278"/>
-      <c r="G16" s="278"/>
-      <c r="H16" s="278"/>
-      <c r="I16" s="278"/>
-      <c r="J16" s="278"/>
-      <c r="K16" s="278"/>
-      <c r="L16" s="278"/>
-      <c r="M16" s="278"/>
-      <c r="N16" s="278"/>
-      <c r="O16" s="278"/>
-      <c r="P16" s="278"/>
-      <c r="Q16" s="278"/>
-      <c r="R16" s="278"/>
-      <c r="S16" s="278"/>
+      <c r="B16" s="281"/>
+      <c r="C16" s="281"/>
+      <c r="D16" s="281"/>
+      <c r="E16" s="281"/>
+      <c r="F16" s="281"/>
+      <c r="G16" s="281"/>
+      <c r="H16" s="281"/>
+      <c r="I16" s="281"/>
+      <c r="J16" s="281"/>
+      <c r="K16" s="281"/>
+      <c r="L16" s="281"/>
+      <c r="M16" s="281"/>
+      <c r="N16" s="281"/>
+      <c r="O16" s="281"/>
+      <c r="P16" s="281"/>
+      <c r="Q16" s="281"/>
+      <c r="R16" s="281"/>
+      <c r="S16" s="281"/>
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="37" t="s">
         <v>480</v>
       </c>
-      <c r="B17" s="283" t="s">
+      <c r="B17" s="286" t="s">
         <v>481</v>
       </c>
-      <c r="C17" s="275"/>
-      <c r="D17" s="275"/>
-      <c r="E17" s="275"/>
-      <c r="F17" s="275"/>
-      <c r="G17" s="276"/>
-      <c r="H17" s="283" t="s">
+      <c r="C17" s="278"/>
+      <c r="D17" s="278"/>
+      <c r="E17" s="278"/>
+      <c r="F17" s="278"/>
+      <c r="G17" s="279"/>
+      <c r="H17" s="286" t="s">
         <v>482</v>
       </c>
-      <c r="I17" s="275"/>
-      <c r="J17" s="276"/>
-      <c r="K17" s="283" t="s">
+      <c r="I17" s="278"/>
+      <c r="J17" s="279"/>
+      <c r="K17" s="286" t="s">
         <v>483</v>
       </c>
-      <c r="L17" s="275"/>
-      <c r="M17" s="276"/>
-      <c r="N17" s="283" t="s">
+      <c r="L17" s="278"/>
+      <c r="M17" s="279"/>
+      <c r="N17" s="286" t="s">
         <v>484</v>
       </c>
-      <c r="O17" s="275"/>
-      <c r="P17" s="276"/>
-      <c r="Q17" s="283" t="s">
+      <c r="O17" s="278"/>
+      <c r="P17" s="279"/>
+      <c r="Q17" s="286" t="s">
         <v>485</v>
       </c>
-      <c r="R17" s="275"/>
-      <c r="S17" s="276"/>
+      <c r="R17" s="278"/>
+      <c r="S17" s="279"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="277" t="s">
+      <c r="B18" s="280" t="s">
         <v>459</v>
       </c>
-      <c r="C18" s="278"/>
-      <c r="D18" s="278"/>
-      <c r="E18" s="278"/>
-      <c r="F18" s="278"/>
-      <c r="G18" s="278"/>
-      <c r="H18" s="278"/>
-      <c r="I18" s="278"/>
-      <c r="J18" s="278"/>
-      <c r="K18" s="278"/>
-      <c r="L18" s="278"/>
-      <c r="M18" s="278"/>
-      <c r="N18" s="278"/>
-      <c r="O18" s="278"/>
-      <c r="P18" s="278"/>
-      <c r="Q18" s="278"/>
-      <c r="R18" s="278"/>
-      <c r="S18" s="278"/>
+      <c r="C18" s="281"/>
+      <c r="D18" s="281"/>
+      <c r="E18" s="281"/>
+      <c r="F18" s="281"/>
+      <c r="G18" s="281"/>
+      <c r="H18" s="281"/>
+      <c r="I18" s="281"/>
+      <c r="J18" s="281"/>
+      <c r="K18" s="281"/>
+      <c r="L18" s="281"/>
+      <c r="M18" s="281"/>
+      <c r="N18" s="281"/>
+      <c r="O18" s="281"/>
+      <c r="P18" s="281"/>
+      <c r="Q18" s="281"/>
+      <c r="R18" s="281"/>
+      <c r="S18" s="281"/>
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="284" t="s">
+      <c r="A19" s="287" t="s">
         <v>486</v>
       </c>
-      <c r="B19" s="278"/>
-      <c r="C19" s="278"/>
-      <c r="D19" s="278"/>
-      <c r="E19" s="278"/>
-      <c r="F19" s="278"/>
-      <c r="G19" s="278"/>
-      <c r="H19" s="278"/>
-      <c r="I19" s="278"/>
-      <c r="J19" s="278"/>
-      <c r="K19" s="278"/>
-      <c r="L19" s="278"/>
-      <c r="M19" s="278"/>
-      <c r="N19" s="278"/>
-      <c r="O19" s="278"/>
-      <c r="P19" s="278"/>
-      <c r="Q19" s="278"/>
-      <c r="R19" s="278"/>
-      <c r="S19" s="278"/>
+      <c r="B19" s="281"/>
+      <c r="C19" s="281"/>
+      <c r="D19" s="281"/>
+      <c r="E19" s="281"/>
+      <c r="F19" s="281"/>
+      <c r="G19" s="281"/>
+      <c r="H19" s="281"/>
+      <c r="I19" s="281"/>
+      <c r="J19" s="281"/>
+      <c r="K19" s="281"/>
+      <c r="L19" s="281"/>
+      <c r="M19" s="281"/>
+      <c r="N19" s="281"/>
+      <c r="O19" s="281"/>
+      <c r="P19" s="281"/>
+      <c r="Q19" s="281"/>
+      <c r="R19" s="281"/>
+      <c r="S19" s="281"/>
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="37" t="s">
         <v>487</v>
       </c>
-      <c r="B20" s="285" t="s">
+      <c r="B20" s="288" t="s">
         <v>488</v>
       </c>
-      <c r="C20" s="275"/>
-      <c r="D20" s="275"/>
-      <c r="E20" s="275"/>
-      <c r="F20" s="275"/>
-      <c r="G20" s="276"/>
-      <c r="H20" s="285" t="s">
+      <c r="C20" s="278"/>
+      <c r="D20" s="278"/>
+      <c r="E20" s="278"/>
+      <c r="F20" s="278"/>
+      <c r="G20" s="279"/>
+      <c r="H20" s="288" t="s">
         <v>489</v>
       </c>
-      <c r="I20" s="275"/>
-      <c r="J20" s="275"/>
-      <c r="K20" s="275"/>
-      <c r="L20" s="275"/>
-      <c r="M20" s="276"/>
-      <c r="N20" s="285" t="s">
+      <c r="I20" s="278"/>
+      <c r="J20" s="278"/>
+      <c r="K20" s="278"/>
+      <c r="L20" s="278"/>
+      <c r="M20" s="279"/>
+      <c r="N20" s="288" t="s">
         <v>490</v>
       </c>
-      <c r="O20" s="275"/>
-      <c r="P20" s="275"/>
-      <c r="Q20" s="275"/>
-      <c r="R20" s="275"/>
-      <c r="S20" s="276"/>
+      <c r="O20" s="278"/>
+      <c r="P20" s="278"/>
+      <c r="Q20" s="278"/>
+      <c r="R20" s="278"/>
+      <c r="S20" s="279"/>
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B21" s="277" t="s">
+      <c r="B21" s="280" t="s">
         <v>459</v>
       </c>
-      <c r="C21" s="278"/>
-      <c r="D21" s="278"/>
-      <c r="E21" s="278"/>
-      <c r="F21" s="278"/>
-      <c r="G21" s="278"/>
-      <c r="H21" s="278"/>
-      <c r="I21" s="278"/>
-      <c r="J21" s="278"/>
-      <c r="K21" s="278"/>
-      <c r="L21" s="278"/>
-      <c r="M21" s="278"/>
-      <c r="N21" s="278"/>
-      <c r="O21" s="278"/>
-      <c r="P21" s="278"/>
-      <c r="Q21" s="278"/>
-      <c r="R21" s="278"/>
-      <c r="S21" s="278"/>
+      <c r="C21" s="281"/>
+      <c r="D21" s="281"/>
+      <c r="E21" s="281"/>
+      <c r="F21" s="281"/>
+      <c r="G21" s="281"/>
+      <c r="H21" s="281"/>
+      <c r="I21" s="281"/>
+      <c r="J21" s="281"/>
+      <c r="K21" s="281"/>
+      <c r="L21" s="281"/>
+      <c r="M21" s="281"/>
+      <c r="N21" s="281"/>
+      <c r="O21" s="281"/>
+      <c r="P21" s="281"/>
+      <c r="Q21" s="281"/>
+      <c r="R21" s="281"/>
+      <c r="S21" s="281"/>
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="284" t="s">
+      <c r="A22" s="287" t="s">
         <v>491</v>
       </c>
-      <c r="B22" s="278"/>
-      <c r="C22" s="278"/>
-      <c r="D22" s="278"/>
-      <c r="E22" s="278"/>
-      <c r="F22" s="278"/>
-      <c r="G22" s="278"/>
-      <c r="H22" s="278"/>
-      <c r="I22" s="278"/>
-      <c r="J22" s="278"/>
-      <c r="K22" s="278"/>
-      <c r="L22" s="278"/>
-      <c r="M22" s="278"/>
-      <c r="N22" s="278"/>
-      <c r="O22" s="278"/>
-      <c r="P22" s="278"/>
-      <c r="Q22" s="278"/>
-      <c r="R22" s="278"/>
-      <c r="S22" s="278"/>
+      <c r="B22" s="281"/>
+      <c r="C22" s="281"/>
+      <c r="D22" s="281"/>
+      <c r="E22" s="281"/>
+      <c r="F22" s="281"/>
+      <c r="G22" s="281"/>
+      <c r="H22" s="281"/>
+      <c r="I22" s="281"/>
+      <c r="J22" s="281"/>
+      <c r="K22" s="281"/>
+      <c r="L22" s="281"/>
+      <c r="M22" s="281"/>
+      <c r="N22" s="281"/>
+      <c r="O22" s="281"/>
+      <c r="P22" s="281"/>
+      <c r="Q22" s="281"/>
+      <c r="R22" s="281"/>
+      <c r="S22" s="281"/>
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="37" t="s">
         <v>492</v>
       </c>
-      <c r="B23" s="285" t="s">
+      <c r="B23" s="288" t="s">
         <v>493</v>
       </c>
-      <c r="C23" s="275"/>
-      <c r="D23" s="275"/>
-      <c r="E23" s="275"/>
-      <c r="F23" s="275"/>
-      <c r="G23" s="276"/>
-      <c r="H23" s="285" t="s">
+      <c r="C23" s="278"/>
+      <c r="D23" s="278"/>
+      <c r="E23" s="278"/>
+      <c r="F23" s="278"/>
+      <c r="G23" s="279"/>
+      <c r="H23" s="288" t="s">
         <v>494</v>
       </c>
-      <c r="I23" s="275"/>
-      <c r="J23" s="276"/>
-      <c r="K23" s="285" t="s">
+      <c r="I23" s="278"/>
+      <c r="J23" s="279"/>
+      <c r="K23" s="288" t="s">
         <v>495</v>
       </c>
-      <c r="L23" s="275"/>
-      <c r="M23" s="276"/>
-      <c r="N23" s="285" t="s">
+      <c r="L23" s="278"/>
+      <c r="M23" s="279"/>
+      <c r="N23" s="288" t="s">
         <v>496</v>
       </c>
-      <c r="O23" s="275"/>
-      <c r="P23" s="276"/>
-      <c r="Q23" s="281" t="s">
+      <c r="O23" s="278"/>
+      <c r="P23" s="279"/>
+      <c r="Q23" s="284" t="s">
         <v>497</v>
       </c>
-      <c r="R23" s="275"/>
-      <c r="S23" s="276"/>
+      <c r="R23" s="278"/>
+      <c r="S23" s="279"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="290" t="s">
+      <c r="A26" s="293" t="s">
         <v>498</v>
       </c>
-      <c r="B26" s="278"/>
-      <c r="C26" s="278"/>
-      <c r="D26" s="278"/>
-      <c r="E26" s="278"/>
-      <c r="F26" s="278"/>
-      <c r="G26" s="278"/>
-      <c r="H26" s="278"/>
-      <c r="I26" s="278"/>
-      <c r="J26" s="278"/>
-      <c r="K26" s="278"/>
-      <c r="L26" s="278"/>
-      <c r="M26" s="278"/>
-      <c r="N26" s="278"/>
-      <c r="O26" s="278"/>
-      <c r="P26" s="278"/>
-      <c r="Q26" s="278"/>
-      <c r="R26" s="278"/>
-      <c r="S26" s="278"/>
+      <c r="B26" s="281"/>
+      <c r="C26" s="281"/>
+      <c r="D26" s="281"/>
+      <c r="E26" s="281"/>
+      <c r="F26" s="281"/>
+      <c r="G26" s="281"/>
+      <c r="H26" s="281"/>
+      <c r="I26" s="281"/>
+      <c r="J26" s="281"/>
+      <c r="K26" s="281"/>
+      <c r="L26" s="281"/>
+      <c r="M26" s="281"/>
+      <c r="N26" s="281"/>
+      <c r="O26" s="281"/>
+      <c r="P26" s="281"/>
+      <c r="Q26" s="281"/>
+      <c r="R26" s="281"/>
+      <c r="S26" s="281"/>
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="37" t="s">
         <v>499</v>
       </c>
-      <c r="B27" s="274" t="s">
+      <c r="B27" s="277" t="s">
         <v>500</v>
       </c>
-      <c r="C27" s="275"/>
-      <c r="D27" s="276"/>
-      <c r="E27" s="274" t="s">
+      <c r="C27" s="278"/>
+      <c r="D27" s="279"/>
+      <c r="E27" s="277" t="s">
         <v>501</v>
       </c>
-      <c r="F27" s="275"/>
-      <c r="G27" s="276"/>
-      <c r="H27" s="282" t="s">
+      <c r="F27" s="278"/>
+      <c r="G27" s="279"/>
+      <c r="H27" s="285" t="s">
         <v>502</v>
       </c>
-      <c r="I27" s="275"/>
-      <c r="J27" s="276"/>
-      <c r="K27" s="283" t="s">
+      <c r="I27" s="278"/>
+      <c r="J27" s="279"/>
+      <c r="K27" s="286" t="s">
         <v>503</v>
       </c>
-      <c r="L27" s="275"/>
-      <c r="M27" s="276"/>
-      <c r="N27" s="283" t="s">
+      <c r="L27" s="278"/>
+      <c r="M27" s="279"/>
+      <c r="N27" s="286" t="s">
         <v>504</v>
       </c>
-      <c r="O27" s="275"/>
-      <c r="P27" s="276"/>
-      <c r="Q27" s="282" t="s">
+      <c r="O27" s="278"/>
+      <c r="P27" s="279"/>
+      <c r="Q27" s="285" t="s">
         <v>505</v>
       </c>
-      <c r="R27" s="275"/>
-      <c r="S27" s="276"/>
+      <c r="R27" s="278"/>
+      <c r="S27" s="279"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="284" t="s">
+      <c r="A30" s="287" t="s">
         <v>506</v>
       </c>
-      <c r="B30" s="278"/>
-      <c r="C30" s="278"/>
-      <c r="D30" s="278"/>
-      <c r="E30" s="278"/>
-      <c r="F30" s="278"/>
-      <c r="G30" s="278"/>
-      <c r="H30" s="278"/>
-      <c r="I30" s="278"/>
-      <c r="J30" s="278"/>
-      <c r="K30" s="278"/>
-      <c r="L30" s="278"/>
-      <c r="M30" s="278"/>
-      <c r="N30" s="278"/>
-      <c r="O30" s="278"/>
-      <c r="P30" s="278"/>
-      <c r="Q30" s="278"/>
-      <c r="R30" s="278"/>
-      <c r="S30" s="278"/>
+      <c r="B30" s="281"/>
+      <c r="C30" s="281"/>
+      <c r="D30" s="281"/>
+      <c r="E30" s="281"/>
+      <c r="F30" s="281"/>
+      <c r="G30" s="281"/>
+      <c r="H30" s="281"/>
+      <c r="I30" s="281"/>
+      <c r="J30" s="281"/>
+      <c r="K30" s="281"/>
+      <c r="L30" s="281"/>
+      <c r="M30" s="281"/>
+      <c r="N30" s="281"/>
+      <c r="O30" s="281"/>
+      <c r="P30" s="281"/>
+      <c r="Q30" s="281"/>
+      <c r="R30" s="281"/>
+      <c r="S30" s="281"/>
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="280" t="s">
+      <c r="A31" s="283" t="s">
         <v>507</v>
       </c>
-      <c r="B31" s="278"/>
-      <c r="C31" s="278"/>
-      <c r="D31" s="278"/>
-      <c r="E31" s="278"/>
-      <c r="F31" s="278"/>
-      <c r="G31" s="278"/>
-      <c r="H31" s="278"/>
-      <c r="I31" s="278"/>
-      <c r="J31" s="278"/>
-      <c r="K31" s="278"/>
-      <c r="L31" s="278"/>
-      <c r="M31" s="278"/>
-      <c r="N31" s="278"/>
-      <c r="O31" s="278"/>
-      <c r="P31" s="278"/>
-      <c r="Q31" s="278"/>
-      <c r="R31" s="278"/>
-      <c r="S31" s="278"/>
+      <c r="B31" s="281"/>
+      <c r="C31" s="281"/>
+      <c r="D31" s="281"/>
+      <c r="E31" s="281"/>
+      <c r="F31" s="281"/>
+      <c r="G31" s="281"/>
+      <c r="H31" s="281"/>
+      <c r="I31" s="281"/>
+      <c r="J31" s="281"/>
+      <c r="K31" s="281"/>
+      <c r="L31" s="281"/>
+      <c r="M31" s="281"/>
+      <c r="N31" s="281"/>
+      <c r="O31" s="281"/>
+      <c r="P31" s="281"/>
+      <c r="Q31" s="281"/>
+      <c r="R31" s="281"/>
+      <c r="S31" s="281"/>
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="280" t="s">
+      <c r="A32" s="283" t="s">
         <v>508</v>
       </c>
-      <c r="B32" s="278"/>
-      <c r="C32" s="278"/>
-      <c r="D32" s="278"/>
-      <c r="E32" s="278"/>
-      <c r="F32" s="278"/>
-      <c r="G32" s="278"/>
-      <c r="H32" s="278"/>
-      <c r="I32" s="278"/>
-      <c r="J32" s="278"/>
-      <c r="K32" s="278"/>
-      <c r="L32" s="278"/>
-      <c r="M32" s="278"/>
-      <c r="N32" s="278"/>
-      <c r="O32" s="278"/>
-      <c r="P32" s="278"/>
-      <c r="Q32" s="278"/>
-      <c r="R32" s="278"/>
-      <c r="S32" s="278"/>
+      <c r="B32" s="281"/>
+      <c r="C32" s="281"/>
+      <c r="D32" s="281"/>
+      <c r="E32" s="281"/>
+      <c r="F32" s="281"/>
+      <c r="G32" s="281"/>
+      <c r="H32" s="281"/>
+      <c r="I32" s="281"/>
+      <c r="J32" s="281"/>
+      <c r="K32" s="281"/>
+      <c r="L32" s="281"/>
+      <c r="M32" s="281"/>
+      <c r="N32" s="281"/>
+      <c r="O32" s="281"/>
+      <c r="P32" s="281"/>
+      <c r="Q32" s="281"/>
+      <c r="R32" s="281"/>
+      <c r="S32" s="281"/>
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="280" t="s">
+      <c r="A33" s="283" t="s">
         <v>509</v>
       </c>
-      <c r="B33" s="278"/>
-      <c r="C33" s="278"/>
-      <c r="D33" s="278"/>
-      <c r="E33" s="278"/>
-      <c r="F33" s="278"/>
-      <c r="G33" s="278"/>
-      <c r="H33" s="278"/>
-      <c r="I33" s="278"/>
-      <c r="J33" s="278"/>
-      <c r="K33" s="278"/>
-      <c r="L33" s="278"/>
-      <c r="M33" s="278"/>
-      <c r="N33" s="278"/>
-      <c r="O33" s="278"/>
-      <c r="P33" s="278"/>
-      <c r="Q33" s="278"/>
-      <c r="R33" s="278"/>
-      <c r="S33" s="278"/>
+      <c r="B33" s="281"/>
+      <c r="C33" s="281"/>
+      <c r="D33" s="281"/>
+      <c r="E33" s="281"/>
+      <c r="F33" s="281"/>
+      <c r="G33" s="281"/>
+      <c r="H33" s="281"/>
+      <c r="I33" s="281"/>
+      <c r="J33" s="281"/>
+      <c r="K33" s="281"/>
+      <c r="L33" s="281"/>
+      <c r="M33" s="281"/>
+      <c r="N33" s="281"/>
+      <c r="O33" s="281"/>
+      <c r="P33" s="281"/>
+      <c r="Q33" s="281"/>
+      <c r="R33" s="281"/>
+      <c r="S33" s="281"/>
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="280" t="s">
+      <c r="A34" s="283" t="s">
         <v>510</v>
       </c>
-      <c r="B34" s="278"/>
-      <c r="C34" s="278"/>
-      <c r="D34" s="278"/>
-      <c r="E34" s="278"/>
-      <c r="F34" s="278"/>
-      <c r="G34" s="278"/>
-      <c r="H34" s="278"/>
-      <c r="I34" s="278"/>
-      <c r="J34" s="278"/>
-      <c r="K34" s="278"/>
-      <c r="L34" s="278"/>
-      <c r="M34" s="278"/>
-      <c r="N34" s="278"/>
-      <c r="O34" s="278"/>
-      <c r="P34" s="278"/>
-      <c r="Q34" s="278"/>
-      <c r="R34" s="278"/>
-      <c r="S34" s="278"/>
+      <c r="B34" s="281"/>
+      <c r="C34" s="281"/>
+      <c r="D34" s="281"/>
+      <c r="E34" s="281"/>
+      <c r="F34" s="281"/>
+      <c r="G34" s="281"/>
+      <c r="H34" s="281"/>
+      <c r="I34" s="281"/>
+      <c r="J34" s="281"/>
+      <c r="K34" s="281"/>
+      <c r="L34" s="281"/>
+      <c r="M34" s="281"/>
+      <c r="N34" s="281"/>
+      <c r="O34" s="281"/>
+      <c r="P34" s="281"/>
+      <c r="Q34" s="281"/>
+      <c r="R34" s="281"/>
+      <c r="S34" s="281"/>
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="280" t="s">
+      <c r="A35" s="283" t="s">
         <v>511</v>
       </c>
-      <c r="B35" s="278"/>
-      <c r="C35" s="278"/>
-      <c r="D35" s="278"/>
-      <c r="E35" s="278"/>
-      <c r="F35" s="278"/>
-      <c r="G35" s="278"/>
-      <c r="H35" s="278"/>
-      <c r="I35" s="278"/>
-      <c r="J35" s="278"/>
-      <c r="K35" s="278"/>
-      <c r="L35" s="278"/>
-      <c r="M35" s="278"/>
-      <c r="N35" s="278"/>
-      <c r="O35" s="278"/>
-      <c r="P35" s="278"/>
-      <c r="Q35" s="278"/>
-      <c r="R35" s="278"/>
-      <c r="S35" s="278"/>
+      <c r="B35" s="281"/>
+      <c r="C35" s="281"/>
+      <c r="D35" s="281"/>
+      <c r="E35" s="281"/>
+      <c r="F35" s="281"/>
+      <c r="G35" s="281"/>
+      <c r="H35" s="281"/>
+      <c r="I35" s="281"/>
+      <c r="J35" s="281"/>
+      <c r="K35" s="281"/>
+      <c r="L35" s="281"/>
+      <c r="M35" s="281"/>
+      <c r="N35" s="281"/>
+      <c r="O35" s="281"/>
+      <c r="P35" s="281"/>
+      <c r="Q35" s="281"/>
+      <c r="R35" s="281"/>
+      <c r="S35" s="281"/>
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="280" t="s">
+      <c r="A36" s="283" t="s">
         <v>512</v>
       </c>
-      <c r="B36" s="278"/>
-      <c r="C36" s="278"/>
-      <c r="D36" s="278"/>
-      <c r="E36" s="278"/>
-      <c r="F36" s="278"/>
-      <c r="G36" s="278"/>
-      <c r="H36" s="278"/>
-      <c r="I36" s="278"/>
-      <c r="J36" s="278"/>
-      <c r="K36" s="278"/>
-      <c r="L36" s="278"/>
-      <c r="M36" s="278"/>
-      <c r="N36" s="278"/>
-      <c r="O36" s="278"/>
-      <c r="P36" s="278"/>
-      <c r="Q36" s="278"/>
-      <c r="R36" s="278"/>
-      <c r="S36" s="278"/>
+      <c r="B36" s="281"/>
+      <c r="C36" s="281"/>
+      <c r="D36" s="281"/>
+      <c r="E36" s="281"/>
+      <c r="F36" s="281"/>
+      <c r="G36" s="281"/>
+      <c r="H36" s="281"/>
+      <c r="I36" s="281"/>
+      <c r="J36" s="281"/>
+      <c r="K36" s="281"/>
+      <c r="L36" s="281"/>
+      <c r="M36" s="281"/>
+      <c r="N36" s="281"/>
+      <c r="O36" s="281"/>
+      <c r="P36" s="281"/>
+      <c r="Q36" s="281"/>
+      <c r="R36" s="281"/>
+      <c r="S36" s="281"/>
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="291" t="s">
+      <c r="A37" s="294" t="s">
         <v>513</v>
       </c>
-      <c r="B37" s="278"/>
-      <c r="C37" s="278"/>
-      <c r="D37" s="278"/>
-      <c r="E37" s="278"/>
-      <c r="F37" s="278"/>
-      <c r="G37" s="278"/>
-      <c r="H37" s="278"/>
-      <c r="I37" s="278"/>
-      <c r="J37" s="278"/>
-      <c r="K37" s="278"/>
-      <c r="L37" s="278"/>
-      <c r="M37" s="278"/>
-      <c r="N37" s="278"/>
-      <c r="O37" s="278"/>
-      <c r="P37" s="278"/>
-      <c r="Q37" s="278"/>
-      <c r="R37" s="278"/>
-      <c r="S37" s="278"/>
+      <c r="B37" s="281"/>
+      <c r="C37" s="281"/>
+      <c r="D37" s="281"/>
+      <c r="E37" s="281"/>
+      <c r="F37" s="281"/>
+      <c r="G37" s="281"/>
+      <c r="H37" s="281"/>
+      <c r="I37" s="281"/>
+      <c r="J37" s="281"/>
+      <c r="K37" s="281"/>
+      <c r="L37" s="281"/>
+      <c r="M37" s="281"/>
+      <c r="N37" s="281"/>
+      <c r="O37" s="281"/>
+      <c r="P37" s="281"/>
+      <c r="Q37" s="281"/>
+      <c r="R37" s="281"/>
+      <c r="S37" s="281"/>
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="38" t="s">
         <v>447</v>
       </c>
-      <c r="B39" s="294" t="s">
+      <c r="B39" s="297" t="s">
         <v>514</v>
       </c>
-      <c r="C39" s="278"/>
-      <c r="D39" s="278"/>
-      <c r="E39" s="292" t="s">
+      <c r="C39" s="281"/>
+      <c r="D39" s="281"/>
+      <c r="E39" s="295" t="s">
         <v>515</v>
       </c>
-      <c r="F39" s="278"/>
-      <c r="G39" s="278"/>
-      <c r="H39" s="295" t="s">
+      <c r="F39" s="281"/>
+      <c r="G39" s="281"/>
+      <c r="H39" s="298" t="s">
         <v>516</v>
       </c>
-      <c r="I39" s="278"/>
-      <c r="J39" s="278"/>
-      <c r="K39" s="288" t="s">
+      <c r="I39" s="281"/>
+      <c r="J39" s="281"/>
+      <c r="K39" s="291" t="s">
         <v>517</v>
       </c>
-      <c r="L39" s="278"/>
-      <c r="M39" s="278"/>
-      <c r="N39" s="286" t="s">
+      <c r="L39" s="281"/>
+      <c r="M39" s="281"/>
+      <c r="N39" s="289" t="s">
         <v>45</v>
       </c>
-      <c r="O39" s="278"/>
-      <c r="P39" s="278"/>
-      <c r="Q39" s="293" t="s">
+      <c r="O39" s="281"/>
+      <c r="P39" s="281"/>
+      <c r="Q39" s="296" t="s">
         <v>518</v>
       </c>
-      <c r="R39" s="278"/>
-      <c r="S39" s="278"/>
+      <c r="R39" s="281"/>
+      <c r="S39" s="281"/>
     </row>
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H14:M14"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A16:S16"/>
     <mergeCell ref="H20:M20"/>
-    <mergeCell ref="A16:S16"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -12694,13 +12718,14 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -12709,7 +12734,6 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
-    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -12717,7 +12741,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -12765,14 +12789,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="297" t="s">
+      <c r="A1" s="300" t="s">
         <v>519</v>
       </c>
-      <c r="B1" s="271"/>
-      <c r="C1" s="271"/>
-      <c r="D1" s="271"/>
-      <c r="E1" s="271"/>
-      <c r="F1" s="272"/>
+      <c r="B1" s="274"/>
+      <c r="C1" s="274"/>
+      <c r="D1" s="274"/>
+      <c r="E1" s="274"/>
+      <c r="F1" s="275"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
@@ -13137,13 +13161,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="297" t="s">
+      <c r="A1" s="300" t="s">
         <v>526</v>
       </c>
-      <c r="B1" s="271"/>
-      <c r="C1" s="271"/>
-      <c r="D1" s="271"/>
-      <c r="E1" s="272"/>
+      <c r="B1" s="274"/>
+      <c r="C1" s="274"/>
+      <c r="D1" s="274"/>
+      <c r="E1" s="275"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="31" t="s">
@@ -14209,7 +14233,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -14225,13 +14249,13 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="298" t="s">
+      <c r="A2" s="301" t="s">
         <v>670</v>
       </c>
-      <c r="B2" s="278"/>
-      <c r="C2" s="278"/>
-      <c r="D2" s="278"/>
-      <c r="E2" s="278"/>
+      <c r="B2" s="281"/>
+      <c r="C2" s="281"/>
+      <c r="D2" s="281"/>
+      <c r="E2" s="281"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="255" t="s">
@@ -14370,14 +14394,14 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="259" t="s">
+      <c r="A12" s="270" t="s">
         <v>688</v>
       </c>
       <c r="B12" s="250" t="s">
         <v>695</v>
       </c>
-      <c r="C12" s="257" t="s">
-        <v>128</v>
+      <c r="C12" s="271" t="s">
+        <v>22</v>
       </c>
       <c r="D12" s="250" t="s">
         <v>696</v>
@@ -14387,14 +14411,14 @@
       </c>
     </row>
     <row r="13" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="259" t="s">
+      <c r="A13" s="270" t="s">
         <v>688</v>
       </c>
       <c r="B13" s="250" t="s">
         <v>698</v>
       </c>
-      <c r="C13" s="257" t="s">
-        <v>128</v>
+      <c r="C13" s="271" t="s">
+        <v>22</v>
       </c>
       <c r="D13" s="250" t="s">
         <v>693</v>
@@ -14404,14 +14428,14 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="259" t="s">
+      <c r="A14" s="270" t="s">
         <v>688</v>
       </c>
       <c r="B14" s="250" t="s">
         <v>700</v>
       </c>
-      <c r="C14" s="257" t="s">
-        <v>128</v>
+      <c r="C14" s="271" t="s">
+        <v>22</v>
       </c>
       <c r="D14" s="250" t="s">
         <v>693</v>
@@ -14573,12 +14597,29 @@
         <v>726</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="262" t="s">
-        <v>447</v>
+    <row r="25" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A25" s="270" t="s">
+        <v>688</v>
       </c>
       <c r="B25" s="250" t="s">
         <v>727</v>
+      </c>
+      <c r="C25" s="272" t="s">
+        <v>128</v>
+      </c>
+      <c r="D25" s="250" t="s">
+        <v>728</v>
+      </c>
+      <c r="E25" s="250" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A26" s="262" t="s">
+        <v>447</v>
+      </c>
+      <c r="B26" s="250" t="s">
+        <v>730</v>
       </c>
     </row>
   </sheetData>
@@ -14607,142 +14648,142 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="246" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="247" t="s">
-        <v>729</v>
+        <v>732</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="248" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="B4" s="248" t="s">
-        <v>731</v>
+        <v>734</v>
       </c>
       <c r="C4" s="248" t="s">
-        <v>732</v>
+        <v>735</v>
       </c>
       <c r="D4" s="248" t="s">
-        <v>733</v>
+        <v>736</v>
       </c>
       <c r="E4" s="248" t="s">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="F4" s="248" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="G4" s="248" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="H4" s="248" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="248" t="s">
-        <v>737</v>
+        <v>740</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="249" t="s">
-        <v>738</v>
+        <v>741</v>
       </c>
       <c r="B5" s="250" t="s">
-        <v>739</v>
+        <v>742</v>
       </c>
       <c r="C5" s="250" t="s">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="D5" s="250" t="s">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="E5" s="250" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
       <c r="F5" s="250" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="G5" s="250" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="H5" s="251" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="I5" s="250" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="249" t="s">
-        <v>747</v>
+        <v>750</v>
       </c>
       <c r="B6" s="250" t="s">
+        <v>751</v>
+      </c>
+      <c r="C6" s="250" t="s">
+        <v>752</v>
+      </c>
+      <c r="D6" s="250" t="s">
+        <v>753</v>
+      </c>
+      <c r="E6" s="250" t="s">
+        <v>754</v>
+      </c>
+      <c r="F6" s="250" t="s">
+        <v>755</v>
+      </c>
+      <c r="G6" s="250" t="s">
+        <v>756</v>
+      </c>
+      <c r="H6" s="252" t="s">
         <v>748</v>
       </c>
-      <c r="C6" s="250" t="s">
-        <v>749</v>
-      </c>
-      <c r="D6" s="250" t="s">
-        <v>750</v>
-      </c>
-      <c r="E6" s="250" t="s">
-        <v>751</v>
-      </c>
-      <c r="F6" s="250" t="s">
-        <v>752</v>
-      </c>
-      <c r="G6" s="250" t="s">
-        <v>753</v>
-      </c>
-      <c r="H6" s="252" t="s">
-        <v>745</v>
-      </c>
       <c r="I6" s="250" t="s">
-        <v>754</v>
+        <v>757</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="249" t="s">
-        <v>755</v>
+        <v>758</v>
       </c>
       <c r="B7" s="250" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="C7" s="250" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
       <c r="D7" s="250" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="E7" s="250" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="F7" s="250" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="G7" s="250" t="s">
-        <v>761</v>
+        <v>764</v>
       </c>
       <c r="H7" s="252" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="I7" s="250" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="249" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="B8" s="250" t="s">
-        <v>764</v>
+        <v>767</v>
       </c>
       <c r="C8" s="250" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="D8" s="250" t="s">
-        <v>766</v>
+        <v>769</v>
       </c>
       <c r="E8" s="250" t="s">
         <v>643</v>
@@ -14754,82 +14795,82 @@
         <v>643</v>
       </c>
       <c r="H8" s="251" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="I8" s="250" t="s">
-        <v>768</v>
+        <v>771</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="249" t="s">
+        <v>772</v>
+      </c>
+      <c r="B9" s="250" t="s">
+        <v>773</v>
+      </c>
+      <c r="C9" s="250" t="s">
+        <v>774</v>
+      </c>
+      <c r="D9" s="250" t="s">
         <v>769</v>
       </c>
-      <c r="B9" s="250" t="s">
-        <v>770</v>
-      </c>
-      <c r="C9" s="250" t="s">
-        <v>771</v>
-      </c>
-      <c r="D9" s="250" t="s">
-        <v>766</v>
-      </c>
       <c r="E9" s="250" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="F9" s="250" t="s">
-        <v>772</v>
+        <v>775</v>
       </c>
       <c r="G9" s="250" t="s">
-        <v>773</v>
+        <v>776</v>
       </c>
       <c r="H9" s="253" t="s">
-        <v>774</v>
+        <v>777</v>
       </c>
       <c r="I9" s="250" t="s">
-        <v>775</v>
+        <v>778</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="249" t="s">
-        <v>776</v>
+        <v>779</v>
       </c>
       <c r="B10" s="250" t="s">
-        <v>777</v>
+        <v>780</v>
       </c>
       <c r="C10" s="250" t="s">
-        <v>778</v>
+        <v>781</v>
       </c>
       <c r="D10" s="250" t="s">
-        <v>779</v>
+        <v>782</v>
       </c>
       <c r="E10" s="250" t="s">
-        <v>780</v>
+        <v>783</v>
       </c>
       <c r="F10" s="250" t="s">
-        <v>781</v>
+        <v>784</v>
       </c>
       <c r="G10" s="250" t="s">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="H10" s="253" t="s">
-        <v>783</v>
+        <v>786</v>
       </c>
       <c r="I10" s="250" t="s">
-        <v>784</v>
+        <v>787</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="249" t="s">
-        <v>785</v>
+        <v>788</v>
       </c>
       <c r="B11" s="250" t="s">
-        <v>786</v>
+        <v>789</v>
       </c>
       <c r="C11" s="250" t="s">
-        <v>787</v>
+        <v>790</v>
       </c>
       <c r="D11" s="250" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="E11" s="250" t="s">
         <v>643</v>
@@ -14838,27 +14879,27 @@
         <v>643</v>
       </c>
       <c r="G11" s="250" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="H11" s="253" t="s">
-        <v>790</v>
+        <v>793</v>
       </c>
       <c r="I11" s="250" t="s">
-        <v>791</v>
+        <v>794</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="249" t="s">
-        <v>792</v>
+        <v>795</v>
       </c>
       <c r="B12" s="250" t="s">
-        <v>793</v>
+        <v>796</v>
       </c>
       <c r="C12" s="250" t="s">
-        <v>794</v>
+        <v>797</v>
       </c>
       <c r="D12" s="250" t="s">
-        <v>795</v>
+        <v>798</v>
       </c>
       <c r="E12" s="250" t="s">
         <v>643</v>
@@ -14867,24 +14908,24 @@
         <v>643</v>
       </c>
       <c r="G12" s="250" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="H12" s="252" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
       <c r="I12" s="250" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="249" t="s">
-        <v>798</v>
+        <v>801</v>
       </c>
       <c r="B13" s="250" t="s">
-        <v>799</v>
+        <v>802</v>
       </c>
       <c r="C13" s="250" t="s">
-        <v>800</v>
+        <v>803</v>
       </c>
       <c r="D13" s="250" t="s">
         <v>643</v>
@@ -14899,21 +14940,21 @@
         <v>643</v>
       </c>
       <c r="H13" s="253" t="s">
-        <v>801</v>
+        <v>804</v>
       </c>
       <c r="I13" s="250" t="s">
-        <v>802</v>
+        <v>805</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="249" t="s">
+        <v>806</v>
+      </c>
+      <c r="B14" s="250" t="s">
+        <v>807</v>
+      </c>
+      <c r="C14" s="250" t="s">
         <v>803</v>
-      </c>
-      <c r="B14" s="250" t="s">
-        <v>804</v>
-      </c>
-      <c r="C14" s="250" t="s">
-        <v>800</v>
       </c>
       <c r="D14" s="250" t="s">
         <v>643</v>
@@ -14928,24 +14969,24 @@
         <v>643</v>
       </c>
       <c r="H14" s="253" t="s">
-        <v>801</v>
+        <v>804</v>
       </c>
       <c r="I14" s="250" t="s">
-        <v>805</v>
+        <v>808</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="299" t="s">
-        <v>806</v>
-      </c>
-      <c r="B16" s="278"/>
-      <c r="C16" s="278"/>
-      <c r="D16" s="278"/>
-      <c r="E16" s="278"/>
-      <c r="F16" s="278"/>
-      <c r="G16" s="278"/>
-      <c r="H16" s="278"/>
-      <c r="I16" s="278"/>
+      <c r="A16" s="302" t="s">
+        <v>809</v>
+      </c>
+      <c r="B16" s="281"/>
+      <c r="C16" s="281"/>
+      <c r="D16" s="281"/>
+      <c r="E16" s="281"/>
+      <c r="F16" s="281"/>
+      <c r="G16" s="281"/>
+      <c r="H16" s="281"/>
+      <c r="I16" s="281"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(tracker): push gate closed, 13 of 20
Replaced with the feed's own selection rather than a new threshold, and
fixed an incoherence found on the way: the push described an h2h pick
while the card showed the best pick across markets.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BB2F352-E352-4162-B1D5-10A9EC58CB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AF29169-CF6A-4E7A-BD16-E07B75FCB5D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2293,13 +2293,13 @@
     <t>DONE (8f794e0). pick_snapshots, captured hourly for fixtures 4-8 HOURS out — not next to the closing-odds capture, which would have made CLV meaningless by construction: taken/closing - 1 is ~0 when both prices are recorded fifteen minutes apart, so the metric would read reassuringly neutral while measuring nothing. Delegates to _bulk_best_picks, the feed's own selection, with a test asserting the delegation. One row per fixture. Verified live: an ATP pick at 2.17, p=0.536, T-7.3h. NOTE: nothing before this commit is recoverable — the ROI/CLV clock starts now.</t>
   </si>
   <si>
-    <t>DECIDE: the push gate still selects the worst-measured tier</t>
+    <t>Push gate no longer uses the confidence tier</t>
   </si>
   <si>
     <t>pre-registration</t>
   </si>
   <si>
-    <t>notify_users fires only for HIGH, which measured 60.9% against MEDIUM's 68.5%. Left documented rather than rewritten: n=69 is too thin, and one real push token means waiting is nearly free. Must be recalibrated or replaced with a MEASURED criterion before push reaches real users — not simply widened.</t>
+    <t>DONE (6bd3582). Replaced with the FEED'S OWN selection (_bulk_best_picks), not a new threshold — n=69 was far too thin to invent one, and doing so was explicitly refused for the completeness floor on n=16. A push can now only be sent for a pick the app itself would surface. Removing the gate outright was not an option: best_outcome returns something for almost any priced fixture. Also fixed a real incoherence found while reading the flow — the old path used h2h-only best_outcome while the card shows the best pick ACROSS markets, so a push could say 'back home' while the app showed 'UNDER 3.5' for the same fixture.</t>
   </si>
   <si>
     <t>P0 blocks everything · P1 builds the measurement · P2 reads it · P3 decides on it · HOLD = deliberately not doing until the read lands</t>
@@ -2550,7 +2550,7 @@
     <numFmt numFmtId="164" formatCode="dd\ mmm"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="84" x14ac:knownFonts="1">
+  <fonts count="85" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2986,6 +2986,12 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -4470,7 +4476,7 @@
     <xf numFmtId="0" fontId="83" fillId="65" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="83" fillId="68" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="84" fillId="65" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -12705,11 +12711,11 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="H20:M20"/>
     <mergeCell ref="A16:S16"/>
-    <mergeCell ref="H20:M20"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -12718,14 +12724,13 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -12734,6 +12739,7 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -12741,7 +12747,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -14605,7 +14611,7 @@
         <v>727</v>
       </c>
       <c r="C25" s="272" t="s">
-        <v>128</v>
+        <v>22</v>
       </c>
       <c r="D25" s="250" t="s">
         <v>728</v>
@@ -14614,7 +14620,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="262" t="s">
         <v>447</v>
       </c>

</xml_diff>

<commit_message>
docs(tracker): close Over/Under on measurement, log the beat guards
The Over/Under decision split in two rather than resolving one way.
goals_total is barred from the headline pick (n=242, r=+0.049, 0.2% of
variance); corners_total is kept (n=234, r=+0.288, about 4.4 standard
errors from zero). Both were assumed to be the same case; measuring
first is what separated them.

Neither needed the September CLV read, which is why this moved from P3
to done now: no volume of closing-line data makes a market explaining
0.2% of variance informative.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -14527,7 +14527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="282" min="1" max="1"/>
@@ -14901,12 +14901,12 @@
       </c>
       <c r="B17" s="215" t="inlineStr">
         <is>
-          <t>Decide Over/Under's future on the evidence</t>
+          <t>Decide Over/Under's future on the evidence — DONE 2026-08-11, and it split in two: goals_total n=242 r=+0.049 (0.2% of variance) is barred from winning the headline pick; corners_total n=234 r=+0.288 (8.3%, ~4.4 SE from zero) is KEPT. Decidable without the CLV read</t>
         </is>
       </c>
       <c r="C17" s="222" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D17" s="215" t="inlineStr">
@@ -15227,6 +15227,50 @@
       <c r="D30" t="inlineStr">
         <is>
           <t>CLV sample size</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B31" s="215" t="inlineStr">
+        <is>
+          <t>Beat now publishes its own code fingerprint (beat_init) and check_stale reports it. The blind spot was exactly where the damage was: only the worker published, so a stale SCHEDULER read as "ok". Both processes moved onto dev_worker.py, which restarts on change</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>the snapshot finding</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B32" s="215" t="inlineStr">
+        <is>
+          <t>Guard: every scheduled task must belong to a module the worker imports, and the snapshot entry is pinned by name — the whole pre-registration rests on one beat_schedule line whose absence is silent</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>beat liveness</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record the observability wiring and the staleness tooling
CLAUDE.md now points at the tooling rather than restating the warning.
The stale-process failure recurred twice after being documented, so
documentation alone demonstrably does not prevent it: dev_worker.py
restarts on change, check_stale.py exits non-zero so it can gate a
verification step, and test_beat_liveness.py pins the schedule.

Also records the blind spot that made the tooling look green while the
scheduler was stale, and that check_stale caught uvicorn stale again
within minutes of covering beat.

Tracker gains the Sentry work and, deliberately, the gap it leaves: no
SENTRY_DSN_BACKEND is provisioned, so the wiring is real and inert. It
protects nothing until a DSN exists.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -14527,7 +14527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="282" min="1" max="1"/>
@@ -15271,6 +15271,72 @@
       <c r="D32" t="inlineStr">
         <is>
           <t>beat liveness</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B33" s="215" t="inlineStr">
+        <is>
+          <t>Sentry wired into the Celery worker and beat, not just the API — it had only ever been initialised in create_app(), so every silent worker failure this project has had was unreportable. One shared initialiser; events tagged with component + loaded code fingerprint</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>the snapshot finding</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B34" s="215" t="inlineStr">
+        <is>
+          <t>monitor_beat_tasks makes each beat_schedule entry a Sentry cron monitor, so a scheduled task that STOPS ARRIVING alerts. The one failure ordinary error reporting cannot catch: no exception, no failed task, no log line — the work just never happens</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Sentry wiring</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B35" s="215" t="inlineStr">
+        <is>
+          <t>GAP: no SENTRY_DSN_BACKEND is provisioned, so the above is real but inert. Needs a DSN before it protects anything — and before deployment, since the measurement currently depends on this one machine staying up</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>user action</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): tennis person-name matching, and the teams_normalized order trap
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -14527,7 +14527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="282" min="1" max="1"/>
@@ -15337,6 +15337,116 @@
       <c r="D35" t="inlineStr">
         <is>
           <t>user action</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B36" s="215" t="inlineStr">
+        <is>
+          <t>Tennis odds were stale up to 6h: the hourly job used BallDontLie only (4 matches priced) while TheRundown (31 ATP events, all unmasked) arrived only on the shared 6-hourly run. Given its own 2-hourly job — ~720 calls/mo vs ~1,440 hourly, which would not fit alongside football's expected ~3,600. One day went 4 of 28 priced -&gt; 24 of 28</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>odds coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B37" s="215" t="inlineStr">
+        <is>
+          <t>NOTE: odds make the feed SMALLER, not larger — that day went 8 fixtures to 4. min_odds can only apply where a price exists, and tennis favourites at ~0.70 price below a 1.50 floor. Those cards previously showed because the filter silently could not apply</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>odds coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B38" s="215" t="inlineStr">
+        <is>
+          <t>Football empty cards are NOT a fault: ODDS_LOOKAHEAD_DAYS=3 and no football fixture is currently inside 3 days. Recheck once the European seasons open on 21 Aug</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>odds coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B39" s="215" t="inlineStr">
+        <is>
+          <t>PERSON-name matching for tennis odds: the lookup was exact + case-sensitive, so 4 fixtures with real prices showed empty cards (SoonWoo vs Soonwoo; Wu Yibing vs Yibing Wu; Chak Lam Coleman Wong). Token-SET match needing &gt;=2 shared tokens, opt-in per sport. 24 of 28 -&gt; 28 of 28 priced; model/market agree on the favourite in 21 of 28</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>odds coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B40" s="215" t="inlineStr">
+        <is>
+          <t>TRAP: TheRundown's teams_normalized array ORDER is not home/away — read is_home. Comparing against [0] produced a false "orientation is broken" alarm that nearly became a fix; the pipeline was correct</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>odds coverage</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): vanished-fixture sweep and the Time-TBC threshold
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -14527,7 +14527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="282" min="1" max="1"/>
@@ -15447,6 +15447,50 @@
       <c r="D40" t="inlineStr">
         <is>
           <t>odds coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B41" s="215" t="inlineStr">
+        <is>
+          <t>Fixtures that vanish from the provider are now retired to POSTPONED (12h past a known kickoff, 48h past a placeholder midnight). Neither provider emits "cancelled" — BallDontLie 404s the match, API-Football omits it — so a vanished fixture kept SCHEDULED forever and its card showed an active pick days later. 3 tennis + 1 football retired</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>user report</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B42" s="215" t="inlineStr">
+        <is>
+          <t>The 48h estimated-kickoff threshold is the load-bearing half: a Time-TBC fixture is stored at midnight, so one clock for both would retire most of a live tournament every morning. 21 of 21 that day correctly untouched</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>user report</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): Sentry DSN provisioned; mobile Sentry still unwired
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -14527,7 +14527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="282" min="1" max="1"/>
@@ -15326,12 +15326,12 @@
       </c>
       <c r="B35" s="215" t="inlineStr">
         <is>
-          <t>GAP: no SENTRY_DSN_BACKEND is provisioned, so the above is real but inert. Needs a DSN before it protects anything — and before deployment, since the measurement currently depends on this one machine staying up</t>
+          <t>SENTRY_DSN_BACKEND now populated in backend/.env (gitignored). The DSN existed in keys.docx from the start — it had simply never reached the environment the app reads. Verified: init_sentry True, test event accepted, transport flushed</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -15491,6 +15491,50 @@
       <c r="D42" t="inlineStr">
         <is>
           <t>user report</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B43" s="215" t="inlineStr">
+        <is>
+          <t>GAP: keys.docx also holds SENTRY_DSN_MOBILE (project ...784, sportiq-mobile) but mobile has ZERO Sentry wiring — no dependency, no init. Crashes in the app go unreported</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>observability</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B44" s="215" t="inlineStr">
+        <is>
+          <t>TRAP: killing uvicorn by command line does not work — a --reload child is spawned via multiprocessing so its cmdline says spawn_main, not uvicorn. Two orphans served stale code through four restarts while netstat blamed dead parent PIDs. check_stale.py caught it correctly throughout</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>observability</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): mobile Sentry wired; source-map upload still unconfigured
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -14527,7 +14527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="282" min="1" max="1"/>
@@ -15502,12 +15502,12 @@
       </c>
       <c r="B43" s="215" t="inlineStr">
         <is>
-          <t>GAP: keys.docx also holds SENTRY_DSN_MOBILE (project ...784, sportiq-mobile) but mobile has ZERO Sentry wiring — no dependency, no init. Crashes in the app go unreported</t>
+          <t>Mobile crash reporting wired (@sentry/react-native, init at module level in the root layout so first-render errors are caught). Verified in a real browser: forcing one unhandled error produced exactly one envelope to the mobile project. Expo Go reports JS errors only — native crashes need an EAS build</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -15535,6 +15535,28 @@
       <c r="D44" t="inlineStr">
         <is>
           <t>observability</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B45" s="215" t="inlineStr">
+        <is>
+          <t>GAP: Sentry Expo plugin has no organization/project set, so production source maps will not upload and release stack traces would be minified. Moot until an EAS build exists</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>mobile observability</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): withdrawn fixtures hidden, and the decision that produced it
Closes the 'shown as POSTPONED' open question with the decision actually taken:
hide fixtures withdrawn from the provider's list, keep showing ones it explicitly
called off. Screenshotting the fix is what made the cost visible.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3879F0A0-A1C2-414F-9A21-E0D575606ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{012C989A-8275-46B6-90B2-138F77086AE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1870" uniqueCount="902">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1876" uniqueCount="904">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -1421,6 +1421,12 @@
   </si>
   <si>
     <t>Reported as missing odds. Cadence, quota, name matching and stale workers all measured and cleared; every real fixture was priced. The unpriced cards were matches that did not exist</t>
+  </si>
+  <si>
+    <t>Withdrawn fixtures hidden; called-off ones still shown</t>
+  </si>
+  <si>
+    <t>fixtures.withdrawn (faa1ecc4c1ac). Retiring the phantoms left 33 grey cards above the day's 2 real picks. Flag set only by the reconciliation, cleared when the provider relists - a flag that cannot be cleared hides a fixture forever. Detail still serves them</t>
   </si>
   <si>
     <t>Legend</t>
@@ -2179,10 +2185,10 @@
     <t>64 tennis fixtures carry 2 identical predictions (same model version and kind); 541 carry one. Harmless today - nothing calls scalar_one on Prediction, so this is not the MultipleResultsFound class that bit TeamFeatures - but unexplained.</t>
   </si>
   <si>
-    <t>Withdrawn fixtures show as POSTPONED</t>
-  </si>
-  <si>
-    <t>A draw entry that was never real is not the same as a match called off, but FixtureStatus has one shared bucket by design. 33 grey cards on one day is arguably its own clutter. Adding a second status is a product decision, so it was flagged rather than taken.</t>
+    <t>Withdrawn vs called-off fixtures</t>
+  </si>
+  <si>
+    <t>Decided: hide fixtures WITHDRAWN from the provider's list, keep showing ones the provider explicitly called off. Both are POSTPONED, but a called-off match was real and users asked to see it, while a withdrawn one was never scheduled. Screenshotting the fix is what made the cost visible - 33 grey cards above the day's 2 genuine picks. Hiding is scoped by fixtures.withdrawn, never by status, so it cannot swallow real postponements.</t>
   </si>
   <si>
     <t>SportIQ — Edge Measurement Plan (P0-P3)</t>
@@ -5165,7 +5171,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R214"/>
+  <dimension ref="A1:R215"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -11913,7 +11919,7 @@
         <v>432</v>
       </c>
       <c r="R198" t="str">
-        <f t="shared" ref="R198:R212" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
+        <f t="shared" ref="R198:R213" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
         <v>E4 ML Football</v>
       </c>
     </row>
@@ -12271,7 +12277,7 @@
         <v>E8 Model Quality</v>
       </c>
     </row>
-    <row r="211" spans="1:18" ht="72" x14ac:dyDescent="0.55000000000000004">
+    <row r="211" spans="1:18" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A211" t="s">
         <v>191</v>
       </c>
@@ -12301,7 +12307,7 @@
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="212" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="212" spans="1:18" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A212" t="s">
         <v>191</v>
       </c>
@@ -12331,23 +12337,53 @@
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="214" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A214" s="23" t="s">
+    <row r="213" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A213" t="s">
+        <v>191</v>
+      </c>
+      <c r="B213" t="s">
         <v>461</v>
       </c>
-      <c r="B214" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C214" s="15" t="s">
+      <c r="C213" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D213" t="s">
+        <v>75</v>
+      </c>
+      <c r="E213" s="210">
+        <v>46246</v>
+      </c>
+      <c r="F213" s="210">
+        <v>46246</v>
+      </c>
+      <c r="G213" s="215" t="s">
         <v>462</v>
       </c>
-      <c r="D214" s="17" t="s">
+      <c r="J213" t="s">
+        <v>400</v>
+      </c>
+      <c r="R213" t="str">
+        <f t="shared" si="3"/>
+        <v>E11 Ops Resilience</v>
+      </c>
+    </row>
+    <row r="215" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A215" s="23" t="s">
+        <v>463</v>
+      </c>
+      <c r="B215" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C215" s="15" t="s">
+        <v>464</v>
+      </c>
+      <c r="D215" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="E214" s="21" t="s">
+      <c r="E215" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="F214" s="19" t="s">
+      <c r="F215" s="19" t="s">
         <v>138</v>
       </c>
     </row>
@@ -12372,7 +12408,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="294" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B1" s="283"/>
       <c r="C1" s="283"/>
@@ -12395,7 +12431,7 @@
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="301" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -12418,7 +12454,7 @@
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="289" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B4" s="283"/>
       <c r="C4" s="283"/>
@@ -12441,42 +12477,42 @@
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="35" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B5" s="279" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="C5" s="280"/>
       <c r="D5" s="281"/>
       <c r="E5" s="284" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="F5" s="280"/>
       <c r="G5" s="281"/>
       <c r="H5" s="284" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="I5" s="280"/>
       <c r="J5" s="281"/>
       <c r="K5" s="279" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="L5" s="280"/>
       <c r="M5" s="281"/>
       <c r="N5" s="286" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="O5" s="280"/>
       <c r="P5" s="281"/>
       <c r="Q5" s="286" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="R5" s="280"/>
       <c r="S5" s="281"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="282" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C6" s="283"/>
       <c r="D6" s="283"/>
@@ -12498,7 +12534,7 @@
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="289" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B7" s="283"/>
       <c r="C7" s="283"/>
@@ -12521,10 +12557,10 @@
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="35" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B8" s="292" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="C8" s="280"/>
       <c r="D8" s="280"/>
@@ -12535,7 +12571,7 @@
       <c r="I8" s="280"/>
       <c r="J8" s="281"/>
       <c r="K8" s="292" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="L8" s="280"/>
       <c r="M8" s="280"/>
@@ -12548,7 +12584,7 @@
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="282" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C9" s="283"/>
       <c r="D9" s="283"/>
@@ -12570,7 +12606,7 @@
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="289" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B10" s="283"/>
       <c r="C10" s="283"/>
@@ -12593,42 +12629,42 @@
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="35" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B11" s="279" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C11" s="280"/>
       <c r="D11" s="281"/>
       <c r="E11" s="279" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F11" s="280"/>
       <c r="G11" s="281"/>
       <c r="H11" s="279" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="I11" s="280"/>
       <c r="J11" s="281"/>
       <c r="K11" s="284" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="L11" s="280"/>
       <c r="M11" s="281"/>
       <c r="N11" s="279" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="O11" s="280"/>
       <c r="P11" s="281"/>
       <c r="Q11" s="279" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="R11" s="280"/>
       <c r="S11" s="281"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="282" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C12" s="283"/>
       <c r="D12" s="283"/>
@@ -12650,7 +12686,7 @@
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="289" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B13" s="283"/>
       <c r="C13" s="283"/>
@@ -12673,10 +12709,10 @@
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="35" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B14" s="287" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="C14" s="280"/>
       <c r="D14" s="280"/>
@@ -12684,7 +12720,7 @@
       <c r="F14" s="280"/>
       <c r="G14" s="281"/>
       <c r="H14" s="287" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="I14" s="280"/>
       <c r="J14" s="280"/>
@@ -12692,19 +12728,19 @@
       <c r="L14" s="280"/>
       <c r="M14" s="281"/>
       <c r="N14" s="287" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="O14" s="280"/>
       <c r="P14" s="281"/>
       <c r="Q14" s="284" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="R14" s="280"/>
       <c r="S14" s="281"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" s="282" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="C15" s="283"/>
       <c r="D15" s="283"/>
@@ -12726,7 +12762,7 @@
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="289" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>
@@ -12749,10 +12785,10 @@
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="35" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B17" s="288" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="C17" s="280"/>
       <c r="D17" s="280"/>
@@ -12760,29 +12796,29 @@
       <c r="F17" s="280"/>
       <c r="G17" s="281"/>
       <c r="H17" s="288" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="I17" s="280"/>
       <c r="J17" s="281"/>
       <c r="K17" s="288" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="L17" s="280"/>
       <c r="M17" s="281"/>
       <c r="N17" s="288" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="O17" s="280"/>
       <c r="P17" s="281"/>
       <c r="Q17" s="288" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="R17" s="280"/>
       <c r="S17" s="281"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="282" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C18" s="283"/>
       <c r="D18" s="283"/>
@@ -12804,7 +12840,7 @@
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="289" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B19" s="283"/>
       <c r="C19" s="283"/>
@@ -12827,10 +12863,10 @@
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="35" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B20" s="290" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="C20" s="280"/>
       <c r="D20" s="280"/>
@@ -12838,7 +12874,7 @@
       <c r="F20" s="280"/>
       <c r="G20" s="281"/>
       <c r="H20" s="290" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="I20" s="280"/>
       <c r="J20" s="280"/>
@@ -12846,7 +12882,7 @@
       <c r="L20" s="280"/>
       <c r="M20" s="281"/>
       <c r="N20" s="290" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="O20" s="280"/>
       <c r="P20" s="280"/>
@@ -12856,7 +12892,7 @@
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" s="282" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C21" s="283"/>
       <c r="D21" s="283"/>
@@ -12878,7 +12914,7 @@
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="289" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B22" s="283"/>
       <c r="C22" s="283"/>
@@ -12901,10 +12937,10 @@
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="35" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B23" s="290" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="C23" s="280"/>
       <c r="D23" s="280"/>
@@ -12912,29 +12948,29 @@
       <c r="F23" s="280"/>
       <c r="G23" s="281"/>
       <c r="H23" s="290" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="I23" s="280"/>
       <c r="J23" s="281"/>
       <c r="K23" s="290" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="L23" s="280"/>
       <c r="M23" s="281"/>
       <c r="N23" s="290" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="O23" s="280"/>
       <c r="P23" s="281"/>
       <c r="Q23" s="286" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="R23" s="280"/>
       <c r="S23" s="281"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="295" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B26" s="283"/>
       <c r="C26" s="283"/>
@@ -12957,42 +12993,42 @@
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="35" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B27" s="279" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="C27" s="280"/>
       <c r="D27" s="281"/>
       <c r="E27" s="279" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="F27" s="280"/>
       <c r="G27" s="281"/>
       <c r="H27" s="287" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="I27" s="280"/>
       <c r="J27" s="281"/>
       <c r="K27" s="288" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="L27" s="280"/>
       <c r="M27" s="281"/>
       <c r="N27" s="288" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="O27" s="280"/>
       <c r="P27" s="281"/>
       <c r="Q27" s="287" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="R27" s="280"/>
       <c r="S27" s="281"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="289" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="B30" s="283"/>
       <c r="C30" s="283"/>
@@ -13015,7 +13051,7 @@
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="285" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B31" s="283"/>
       <c r="C31" s="283"/>
@@ -13038,7 +13074,7 @@
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="285" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B32" s="283"/>
       <c r="C32" s="283"/>
@@ -13061,7 +13097,7 @@
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="285" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B33" s="283"/>
       <c r="C33" s="283"/>
@@ -13084,7 +13120,7 @@
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="285" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="B34" s="283"/>
       <c r="C34" s="283"/>
@@ -13107,7 +13143,7 @@
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="285" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B35" s="283"/>
       <c r="C35" s="283"/>
@@ -13130,7 +13166,7 @@
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="285" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="B36" s="283"/>
       <c r="C36" s="283"/>
@@ -13153,7 +13189,7 @@
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="296" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B37" s="283"/>
       <c r="C37" s="283"/>
@@ -13176,25 +13212,25 @@
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="36" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B39" s="299" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="C39" s="283"/>
       <c r="D39" s="283"/>
       <c r="E39" s="297" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="F39" s="283"/>
       <c r="G39" s="283"/>
       <c r="H39" s="300" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="I39" s="283"/>
       <c r="J39" s="283"/>
       <c r="K39" s="293" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="L39" s="283"/>
       <c r="M39" s="283"/>
@@ -13204,7 +13240,7 @@
       <c r="O39" s="283"/>
       <c r="P39" s="283"/>
       <c r="Q39" s="298" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="R39" s="283"/>
       <c r="S39" s="283"/>
@@ -13212,11 +13248,11 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="H20:M20"/>
     <mergeCell ref="A16:S16"/>
-    <mergeCell ref="H20:M20"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -13225,14 +13261,13 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -13241,6 +13276,7 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -13248,7 +13284,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -13297,7 +13333,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -13310,19 +13346,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -13581,11 +13617,11 @@
       </c>
       <c r="B14" s="24">
         <f t="shared" si="0"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C14" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D14" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -13597,20 +13633,20 @@
       </c>
       <c r="F14" s="25">
         <f t="shared" si="1"/>
-        <v>0.7142857142857143</v>
+        <v>0.72727272727272729</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="26" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B16" s="27">
         <f>SUM(B4:B14)</f>
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C16" s="27">
         <f>SUM(C4:C14)</f>
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
@@ -13622,12 +13658,12 @@
       </c>
       <c r="F16" s="28">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.77884615384615385</v>
+        <v>0.77990430622009566</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="41" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="B18" s="42">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -13636,7 +13672,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="43" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
   </sheetData>
@@ -13669,7 +13705,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -13678,648 +13714,648 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="29" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D3" s="29" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="29" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="30" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="32" t="s">
+        <v>552</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>548</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>553</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>550</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>546</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>551</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>548</v>
-      </c>
       <c r="E5" s="33" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="30" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="32" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="30" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="32" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="30" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="32" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="30" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="32" t="s">
+        <v>576</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>556</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>561</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>574</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>554</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>559</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>572</v>
-      </c>
       <c r="E13" s="33" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="30" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="32" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="30" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="32" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="30" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="32" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="30" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="32" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E21" s="33" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="30" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="32" t="s">
+        <v>600</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>598</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>596</v>
-      </c>
       <c r="C23" s="17" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="30" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E24" s="31" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="53" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="B25" s="51" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C25" s="54" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E25" s="55" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="56" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="B26" s="46" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C26" s="54" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="D26" s="46" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E26" s="57" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="53" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="B27" s="51" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C27" s="54" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="D27" s="51" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E27" s="55" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="71" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B28" s="60" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C28" s="67" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D28" s="94" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E28" s="94" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="72" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="B29" s="65" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C29" s="69" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D29" s="93" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E29" s="93" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="78" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="B30" s="75" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C30" s="79" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D30" s="75" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E30" s="80" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="92" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="B31" s="83" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C31" s="90" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D31" s="83" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="E31" s="93" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="106" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="B32" s="102" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C32" s="104" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D32" s="102" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E32" s="107" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="108" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="B33" s="97" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C33" s="104" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D33" s="97" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E33" s="109" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="134" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="B34" s="129" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C34" s="123" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D34" s="129" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E34" s="135" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="136" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="B35" s="124" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C35" s="132" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D35" s="124" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E35" s="137" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="74.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="147" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="B36" s="145" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C36" s="148" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="D36" s="153" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="E36" s="153" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="150" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="B37" s="140" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C37" s="151" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D37" s="140" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E37" s="152" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="147" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="B38" s="145" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C38" s="151" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="D38" s="145" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E38" s="149" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="160" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="B39" s="157" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C39" s="161" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D39" s="157" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E39" s="162" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="168" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="B40" s="165" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C40" s="169" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D40" s="165" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E40" s="170" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -14327,475 +14363,475 @@
         <v>140</v>
       </c>
       <c r="B41" s="172" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C41" s="173" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D41" s="172" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E41" s="174" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="188" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="B42" s="183" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C42" s="177" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D42" s="183" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E42" s="189" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="190" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="B43" s="178" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C43" s="186" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D43" s="178" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E43" s="191" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="188" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B44" s="183" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C44" s="186" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D44" s="183" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E44" s="189" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="190" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="B45" s="178" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C45" s="186" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="D45" s="178" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E45" s="191" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="206" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="B46" s="194" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C46" s="199" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D46" s="194" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E46" s="207" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="208" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="B47" s="200" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C47" s="203" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D47" s="200" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E47" s="209" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="206" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="B48" s="194" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C48" s="203" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D48" s="194" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E48" s="207" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="B49" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C49" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D49" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E49" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="B50" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C50" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D50" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E50" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="B51" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C51" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D51" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E51" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="B52" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C52" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="D52" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E52" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
+        <v>661</v>
+      </c>
+      <c r="B53" t="s">
+        <v>562</v>
+      </c>
+      <c r="C53" t="s">
         <v>659</v>
       </c>
-      <c r="B53" t="s">
-        <v>560</v>
-      </c>
-      <c r="C53" t="s">
-        <v>657</v>
-      </c>
       <c r="D53" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E53" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="215" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C54" s="215" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="D54" s="215" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E54" s="215" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="215" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C55" s="215" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D55" s="215" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E55" s="215" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="215" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C56" s="215" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D56" s="215" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E56" s="215" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="215" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C57" s="215" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D57" s="215" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E57" s="215" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="215" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C58" s="215" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D58" s="215" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E58" s="215" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="215" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C59" s="215" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D59" s="215" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E59" s="215" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="215" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C60" s="215" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D60" s="215" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E60" s="215" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C61" s="215" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D61" s="215" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E61" s="215" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="215" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C62" s="215" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D62" s="215" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E62" s="215" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="215" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C63" s="215" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="D63" s="215" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E63" s="215" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="215" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C64" s="215" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="D64" s="215" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E64" s="215" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="129.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="215" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C65" s="215" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D65" s="215" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E65" s="215" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="215" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="B66" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C66" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D66" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E66" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="215" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="B67" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C67" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="D67" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E67" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="215" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="B68" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C68" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="D68" t="s">
-        <v>548</v>
+        <v>593</v>
       </c>
       <c r="E68" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
     </row>
   </sheetData>
@@ -14820,12 +14856,12 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="219" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="303" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -14834,1032 +14870,1032 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="220" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="B4" s="220" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="C4" s="220" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="220" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="E4" s="220" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="221" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="C5" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="221" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="B6" s="215" t="s">
+        <v>702</v>
+      </c>
+      <c r="C6" s="228" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="215" t="s">
         <v>700</v>
       </c>
-      <c r="C6" s="228" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="215" t="s">
-        <v>698</v>
-      </c>
       <c r="E6" s="215" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="231" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="C7" s="232" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="215" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="E7" s="215" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="223" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="C8" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="223" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B9" s="215" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="C9" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="215" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="E9" s="215" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="224" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="C10" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="C11" t="s">
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="C12" t="s">
         <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="224" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="C13" s="222" t="s">
         <v>128</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="235" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C14" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="235" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B15" s="215" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="C15" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="215" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="E15" s="215" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="235" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B16" s="215" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="C16" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="215" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="E16" s="215" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="225" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="B17" s="215" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="C17" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D17" s="215" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="E17" s="215" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="225" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="B18" s="215" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="C18" s="223" t="s">
         <v>138</v>
       </c>
       <c r="D18" s="215" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="E18" s="215" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="226" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="B19" s="215" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="C19" s="225" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="D19" s="215" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="E19" s="215" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="226" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="B20" s="215" t="s">
+        <v>739</v>
+      </c>
+      <c r="C20" s="225" t="s">
         <v>737</v>
       </c>
-      <c r="C20" s="225" t="s">
-        <v>735</v>
-      </c>
       <c r="D20" s="215" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="E20" s="215" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="226" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="B21" s="215" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="C21" s="225" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="D21" s="215" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="E21" s="215" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
     <row r="23" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="229" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="B23" s="215" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="C23" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D23" s="215" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="E23" s="215" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="230" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B24" s="215" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="C24" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D24" s="215" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="E24" s="215" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="231" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B25" s="215" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="C25" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D25" s="215" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="E25" s="215" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="231" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B26" s="215" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="C26" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D26" s="215" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="E26" s="215" t="s">
-        <v>751</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="235" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B27" s="215" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="C27" s="237" t="s">
         <v>22</v>
       </c>
       <c r="D27" s="215" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="E27" s="215" t="s">
-        <v>753</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="227" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="B28" s="215" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="C28" t="s">
         <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>755</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B29" s="215" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="C29" t="s">
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>715</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B30" s="215" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="C30" t="s">
         <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>758</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B31" s="215" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="C31" t="s">
         <v>22</v>
       </c>
       <c r="D31" t="s">
-        <v>760</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B32" s="215" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="C32" t="s">
         <v>22</v>
       </c>
       <c r="D32" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A33" t="s">
+        <v>704</v>
+      </c>
+      <c r="B33" s="215" t="s">
+        <v>765</v>
+      </c>
+      <c r="C33" t="s">
+        <v>22</v>
+      </c>
+      <c r="D33" t="s">
         <v>762</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" t="s">
-        <v>702</v>
-      </c>
-      <c r="B33" s="215" t="s">
-        <v>763</v>
-      </c>
-      <c r="C33" t="s">
-        <v>22</v>
-      </c>
-      <c r="D33" t="s">
-        <v>760</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B34" s="215" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="C34" t="s">
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>765</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B35" s="215" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="C35" t="s">
         <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>767</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B36" s="215" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="C36" t="s">
         <v>22</v>
       </c>
       <c r="D36" t="s">
-        <v>769</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B37" s="215" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="C37" t="s">
         <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>769</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="B38" s="215" t="s">
+        <v>773</v>
+      </c>
+      <c r="C38" t="s">
+        <v>22</v>
+      </c>
+      <c r="D38" t="s">
         <v>771</v>
       </c>
-      <c r="C38" t="s">
-        <v>22</v>
-      </c>
-      <c r="D38" t="s">
-        <v>769</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="39" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B39" s="215" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="C39" t="s">
         <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>769</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B40" s="215" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="C40" t="s">
         <v>22</v>
       </c>
       <c r="D40" t="s">
-        <v>769</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="100.8" x14ac:dyDescent="0.55000000000000004">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B41" s="215" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="C41" t="s">
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>775</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B42" s="215" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="C42" t="s">
         <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>775</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B43" s="215" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="C43" t="s">
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>778</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B44" s="215" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="C44" t="s">
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>778</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="B45" s="215" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="C45" t="s">
         <v>128</v>
       </c>
       <c r="D45" t="s">
-        <v>781</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B46" s="215" t="s">
-        <v>783</v>
+        <v>785</v>
       </c>
       <c r="C46" t="s">
         <v>22</v>
       </c>
       <c r="D46" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A47" s="274" t="s">
         <v>784</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
-      <c r="A47" s="274" t="s">
-        <v>782</v>
-      </c>
       <c r="B47" s="215" t="s">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>786</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B48" s="215" t="s">
-        <v>787</v>
+        <v>789</v>
       </c>
       <c r="C48" t="s">
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>786</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B49" s="215" t="s">
+        <v>790</v>
+      </c>
+      <c r="C49" t="s">
+        <v>22</v>
+      </c>
+      <c r="D49" t="s">
         <v>788</v>
       </c>
-      <c r="C49" t="s">
-        <v>22</v>
-      </c>
-      <c r="D49" t="s">
-        <v>786</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="50" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B50" s="215" t="s">
-        <v>789</v>
+        <v>791</v>
       </c>
       <c r="C50" t="s">
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>790</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="115.2" x14ac:dyDescent="0.55000000000000004">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B51" s="215" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="C51" t="s">
         <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>792</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="100.8" x14ac:dyDescent="0.55000000000000004">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B52" s="215" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="C52" t="s">
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>794</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B53" s="215" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="C53" t="s">
         <v>128</v>
       </c>
       <c r="D53" t="s">
-        <v>792</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" ht="100.8" x14ac:dyDescent="0.55000000000000004">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B54" s="215" t="s">
+        <v>798</v>
+      </c>
+      <c r="C54" t="s">
+        <v>22</v>
+      </c>
+      <c r="D54" t="s">
         <v>796</v>
       </c>
-      <c r="C54" t="s">
-        <v>22</v>
-      </c>
-      <c r="D54" t="s">
-        <v>794</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="55" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>797</v>
+        <v>799</v>
       </c>
       <c r="C55" t="s">
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>798</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>799</v>
+        <v>801</v>
       </c>
       <c r="C56" t="s">
         <v>128</v>
       </c>
       <c r="D56" t="s">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="115.2" x14ac:dyDescent="0.55000000000000004">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>801</v>
+        <v>803</v>
       </c>
       <c r="C57" t="s">
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>803</v>
+        <v>805</v>
       </c>
       <c r="C58" t="s">
         <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B59" s="215" t="s">
+        <v>806</v>
+      </c>
+      <c r="C59" t="s">
+        <v>22</v>
+      </c>
+      <c r="D59" t="s">
         <v>804</v>
       </c>
-      <c r="C59" t="s">
-        <v>22</v>
-      </c>
-      <c r="D59" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="60" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>805</v>
+        <v>807</v>
       </c>
       <c r="C60" t="s">
         <v>128</v>
       </c>
       <c r="D60" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="274" t="s">
-        <v>806</v>
+        <v>808</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>807</v>
+        <v>809</v>
       </c>
       <c r="C61" t="s">
         <v>22</v>
       </c>
       <c r="D61" t="s">
-        <v>775</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="274" t="s">
-        <v>806</v>
+        <v>808</v>
       </c>
       <c r="B62" s="215" t="s">
+        <v>810</v>
+      </c>
+      <c r="C62" t="s">
+        <v>22</v>
+      </c>
+      <c r="D62" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A63" s="274" t="s">
         <v>808</v>
       </c>
-      <c r="C62" t="s">
-        <v>22</v>
-      </c>
-      <c r="D62" t="s">
-        <v>775</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
-      <c r="A63" s="274" t="s">
-        <v>806</v>
-      </c>
       <c r="B63" s="215" t="s">
-        <v>809</v>
+        <v>811</v>
       </c>
       <c r="C63" t="s">
         <v>22</v>
       </c>
       <c r="D63" t="s">
-        <v>775</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>810</v>
+        <v>812</v>
       </c>
       <c r="C64" t="s">
         <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>812</v>
+        <v>814</v>
       </c>
       <c r="C65" t="s">
         <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B66" s="215" t="s">
+        <v>815</v>
+      </c>
+      <c r="C66" t="s">
+        <v>22</v>
+      </c>
+      <c r="D66" t="s">
         <v>813</v>
       </c>
-      <c r="C66" t="s">
-        <v>22</v>
-      </c>
-      <c r="D66" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="67" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="274" t="s">
-        <v>814</v>
+        <v>816</v>
       </c>
       <c r="B67" s="215" t="s">
-        <v>815</v>
+        <v>817</v>
       </c>
       <c r="C67" t="s">
         <v>22</v>
       </c>
       <c r="D67" t="s">
-        <v>775</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="274" t="s">
-        <v>814</v>
+        <v>816</v>
       </c>
       <c r="B68" s="215" t="s">
+        <v>818</v>
+      </c>
+      <c r="C68" t="s">
+        <v>22</v>
+      </c>
+      <c r="D68" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A69" s="274" t="s">
         <v>816</v>
       </c>
-      <c r="C68" t="s">
-        <v>22</v>
-      </c>
-      <c r="D68" t="s">
-        <v>775</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" ht="57.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A69" s="274" t="s">
-        <v>814</v>
-      </c>
       <c r="B69" s="215" t="s">
-        <v>817</v>
+        <v>819</v>
       </c>
       <c r="C69" t="s">
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>775</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B70" s="215" t="s">
-        <v>818</v>
+        <v>820</v>
       </c>
       <c r="C70" t="s">
         <v>22</v>
       </c>
       <c r="D70" t="s">
-        <v>819</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B71" s="215" t="s">
-        <v>820</v>
+        <v>822</v>
       </c>
       <c r="C71" t="s">
         <v>22</v>
       </c>
       <c r="D71" t="s">
-        <v>819</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" ht="72" x14ac:dyDescent="0.55000000000000004">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B72" s="215" t="s">
+        <v>823</v>
+      </c>
+      <c r="C72" t="s">
+        <v>22</v>
+      </c>
+      <c r="D72" t="s">
         <v>821</v>
       </c>
-      <c r="C72" t="s">
-        <v>22</v>
-      </c>
-      <c r="D72" t="s">
-        <v>819</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    </row>
+    <row r="73" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="274" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B73" s="215" t="s">
-        <v>822</v>
+        <v>824</v>
       </c>
       <c r="C73" t="s">
         <v>128</v>
       </c>
       <c r="D73" t="s">
-        <v>819</v>
+        <v>821</v>
       </c>
     </row>
   </sheetData>
@@ -15888,336 +15924,336 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="211" t="s">
-        <v>823</v>
+        <v>825</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="212" t="s">
-        <v>824</v>
+        <v>826</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="213" t="s">
-        <v>825</v>
+        <v>827</v>
       </c>
       <c r="B4" s="213" t="s">
-        <v>826</v>
+        <v>828</v>
       </c>
       <c r="C4" s="213" t="s">
-        <v>827</v>
+        <v>829</v>
       </c>
       <c r="D4" s="213" t="s">
-        <v>828</v>
+        <v>830</v>
       </c>
       <c r="E4" s="213" t="s">
-        <v>829</v>
+        <v>831</v>
       </c>
       <c r="F4" s="213" t="s">
-        <v>830</v>
+        <v>832</v>
       </c>
       <c r="G4" s="213" t="s">
-        <v>831</v>
+        <v>833</v>
       </c>
       <c r="H4" s="213" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="213" t="s">
-        <v>832</v>
+        <v>834</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="214" t="s">
-        <v>833</v>
+        <v>835</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>834</v>
+        <v>836</v>
       </c>
       <c r="C5" s="215" t="s">
-        <v>835</v>
+        <v>837</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>836</v>
+        <v>838</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>837</v>
+        <v>839</v>
       </c>
       <c r="F5" s="215" t="s">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="G5" s="215" t="s">
-        <v>839</v>
+        <v>841</v>
       </c>
       <c r="H5" s="216" t="s">
-        <v>840</v>
+        <v>842</v>
       </c>
       <c r="I5" s="215" t="s">
-        <v>841</v>
+        <v>843</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="214" t="s">
+        <v>844</v>
+      </c>
+      <c r="B6" s="215" t="s">
+        <v>845</v>
+      </c>
+      <c r="C6" s="215" t="s">
+        <v>846</v>
+      </c>
+      <c r="D6" s="215" t="s">
+        <v>847</v>
+      </c>
+      <c r="E6" s="215" t="s">
+        <v>848</v>
+      </c>
+      <c r="F6" s="215" t="s">
+        <v>849</v>
+      </c>
+      <c r="G6" s="215" t="s">
+        <v>850</v>
+      </c>
+      <c r="H6" s="217" t="s">
         <v>842</v>
       </c>
-      <c r="B6" s="215" t="s">
-        <v>843</v>
-      </c>
-      <c r="C6" s="215" t="s">
-        <v>844</v>
-      </c>
-      <c r="D6" s="215" t="s">
-        <v>845</v>
-      </c>
-      <c r="E6" s="215" t="s">
-        <v>846</v>
-      </c>
-      <c r="F6" s="215" t="s">
-        <v>847</v>
-      </c>
-      <c r="G6" s="215" t="s">
-        <v>848</v>
-      </c>
-      <c r="H6" s="217" t="s">
-        <v>840</v>
-      </c>
       <c r="I6" s="215" t="s">
-        <v>849</v>
+        <v>851</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="214" t="s">
-        <v>850</v>
+        <v>852</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>851</v>
+        <v>853</v>
       </c>
       <c r="C7" s="215" t="s">
-        <v>852</v>
+        <v>854</v>
       </c>
       <c r="D7" s="215" t="s">
-        <v>853</v>
+        <v>855</v>
       </c>
       <c r="E7" s="215" t="s">
-        <v>854</v>
+        <v>856</v>
       </c>
       <c r="F7" s="215" t="s">
-        <v>855</v>
+        <v>857</v>
       </c>
       <c r="G7" s="215" t="s">
-        <v>856</v>
+        <v>858</v>
       </c>
       <c r="H7" s="217" t="s">
-        <v>840</v>
+        <v>842</v>
       </c>
       <c r="I7" s="215" t="s">
-        <v>857</v>
+        <v>859</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="214" t="s">
-        <v>858</v>
+        <v>860</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>859</v>
+        <v>861</v>
       </c>
       <c r="C8" s="215" t="s">
-        <v>860</v>
+        <v>862</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>861</v>
+        <v>863</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="F8" s="215" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="G8" s="215" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="H8" s="216" t="s">
-        <v>862</v>
+        <v>864</v>
       </c>
       <c r="I8" s="215" t="s">
-        <v>863</v>
+        <v>865</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="214" t="s">
-        <v>864</v>
+        <v>866</v>
       </c>
       <c r="B9" s="215" t="s">
-        <v>865</v>
+        <v>867</v>
       </c>
       <c r="C9" s="215" t="s">
-        <v>866</v>
+        <v>868</v>
       </c>
       <c r="D9" s="215" t="s">
-        <v>861</v>
+        <v>863</v>
       </c>
       <c r="E9" s="215" t="s">
-        <v>854</v>
+        <v>856</v>
       </c>
       <c r="F9" s="215" t="s">
-        <v>867</v>
+        <v>869</v>
       </c>
       <c r="G9" s="215" t="s">
-        <v>868</v>
+        <v>870</v>
       </c>
       <c r="H9" s="218" t="s">
-        <v>869</v>
+        <v>871</v>
       </c>
       <c r="I9" s="215" t="s">
-        <v>870</v>
+        <v>872</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="214" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>872</v>
+        <v>874</v>
       </c>
       <c r="C10" s="215" t="s">
-        <v>873</v>
+        <v>875</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>874</v>
+        <v>876</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>875</v>
+        <v>877</v>
       </c>
       <c r="F10" s="215" t="s">
-        <v>876</v>
+        <v>878</v>
       </c>
       <c r="G10" s="215" t="s">
-        <v>877</v>
+        <v>879</v>
       </c>
       <c r="H10" s="218" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="I10" s="215" t="s">
-        <v>879</v>
+        <v>881</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="214" t="s">
-        <v>880</v>
+        <v>882</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>881</v>
+        <v>883</v>
       </c>
       <c r="C11" s="215" t="s">
-        <v>882</v>
+        <v>884</v>
       </c>
       <c r="D11" s="215" t="s">
-        <v>883</v>
+        <v>885</v>
       </c>
       <c r="E11" s="215" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="F11" s="215" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="G11" s="215" t="s">
-        <v>884</v>
+        <v>886</v>
       </c>
       <c r="H11" s="218" t="s">
-        <v>885</v>
+        <v>887</v>
       </c>
       <c r="I11" s="215" t="s">
-        <v>886</v>
+        <v>888</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="214" t="s">
-        <v>887</v>
+        <v>889</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>888</v>
+        <v>890</v>
       </c>
       <c r="C12" s="215" t="s">
-        <v>889</v>
+        <v>891</v>
       </c>
       <c r="D12" s="215" t="s">
-        <v>890</v>
+        <v>892</v>
       </c>
       <c r="E12" s="215" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="F12" s="215" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="G12" s="215" t="s">
-        <v>884</v>
+        <v>886</v>
       </c>
       <c r="H12" s="217" t="s">
-        <v>891</v>
+        <v>893</v>
       </c>
       <c r="I12" s="215" t="s">
-        <v>892</v>
+        <v>894</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="214" t="s">
-        <v>893</v>
+        <v>895</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>894</v>
+        <v>896</v>
       </c>
       <c r="C13" s="215" t="s">
-        <v>895</v>
+        <v>897</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="F13" s="215" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="G13" s="215" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="H13" s="218" t="s">
-        <v>896</v>
+        <v>898</v>
       </c>
       <c r="I13" s="215" t="s">
-        <v>897</v>
+        <v>899</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="214" t="s">
+        <v>900</v>
+      </c>
+      <c r="B14" s="215" t="s">
+        <v>901</v>
+      </c>
+      <c r="C14" s="215" t="s">
+        <v>897</v>
+      </c>
+      <c r="D14" s="215" t="s">
+        <v>659</v>
+      </c>
+      <c r="E14" s="215" t="s">
+        <v>659</v>
+      </c>
+      <c r="F14" s="215" t="s">
+        <v>659</v>
+      </c>
+      <c r="G14" s="215" t="s">
+        <v>659</v>
+      </c>
+      <c r="H14" s="218" t="s">
         <v>898</v>
       </c>
-      <c r="B14" s="215" t="s">
-        <v>899</v>
-      </c>
-      <c r="C14" s="215" t="s">
-        <v>895</v>
-      </c>
-      <c r="D14" s="215" t="s">
-        <v>657</v>
-      </c>
-      <c r="E14" s="215" t="s">
-        <v>657</v>
-      </c>
-      <c r="F14" s="215" t="s">
-        <v>657</v>
-      </c>
-      <c r="G14" s="215" t="s">
-        <v>657</v>
-      </c>
-      <c r="H14" s="218" t="s">
-        <v>896</v>
-      </c>
       <c r="I14" s="215" t="s">
-        <v>900</v>
+        <v>902</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="304" t="s">
-        <v>901</v>
+        <v>903</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>

</xml_diff>

<commit_message>
docs(tracker): corners tuning, the corners market evaluation, and the undelivered promotion
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{012C989A-8275-46B6-90B2-138F77086AE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{525A0C13-758A-4A76-ABF9-71C824732858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1876" uniqueCount="904">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1904" uniqueCount="914">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -1427,6 +1427,24 @@
   </si>
   <si>
     <t>fixtures.withdrawn (faa1ecc4c1ac). Retiring the phantoms left 33 grey cards above the day's 2 real picks. Flag set only by the reconciliation, cleared when the provider relists - a flag that cannot be cleared hides a fixture forever. Detail still serves them</t>
+  </si>
+  <si>
+    <t>Corners Poisson regressors tuned (last untuned estimator)</t>
+  </si>
+  <si>
+    <t>Pre-registered WITH tolerances. under-9.5 Brier 0.2535-&gt;0.2509, corners MAE 2.158-&gt;2.120, under-10.5 buckets inverted-&gt;monotonic. Defaults wrong again: depth 4-&gt;3/4, lr 0.3-&gt;0.032. Scoping proved by booster hashes - layer1/layer2 byte-identical. football_xgb_v20260813004745</t>
+  </si>
+  <si>
+    <t>Over/Under CORNERS held-out evaluation (never existed)</t>
+  </si>
+  <si>
+    <t>Corners was judged by MAE alone, which is not what the market sells - the same gap that let goals ship overconfident. Brier + reliability buckets per line, every run, logged to MLflow. Shows discrimination is real but weak: predicted spans 0.2-0.7, observed only 0.44-0.56</t>
+  </si>
+  <si>
+    <t>Retrains now reach the feed (stale model_version re-queue)</t>
+  </si>
+  <si>
+    <t>All 135 upcoming football fixtures were serving predictions from one of FOUR superseded versions. Guard only asked 'does a prediction exist'; promotion is a DB update so nothing logged. Re-queues on version change only, so a daily run still queues nothing</t>
   </si>
   <si>
     <t>Legend</t>
@@ -2189,6 +2207,18 @@
   </si>
   <si>
     <t>Decided: hide fixtures WITHDRAWN from the provider's list, keep showing ones the provider explicitly called off. Both are POSTPONED, but a called-off match was real and users asked to see it, while a withdrawn one was never scheduled. Screenshotting the fix is what made the cost visible - 33 grey cards above the day's 2 genuine picks. Hiding is scoped by fixtures.withdrawn, never by status, so it cannot swallow real postponements.</t>
+  </si>
+  <si>
+    <t>Corners discrimination is real but weak</t>
+  </si>
+  <si>
+    <t>Now measurable for the first time. Predicted P(under 9.5) spans 0.2-0.7 while the observed rate spans only 0.44-0.56, and the bottom two buckets are still inverted on small n. Better than goals (flat at base rate) and consistent with the r=+0.288 measured live, but corners wins ~half of all headline picks, so this is the number to watch.</t>
+  </si>
+  <si>
+    <t>A promotion did not reach any user</t>
+  </si>
+  <si>
+    <t>Found while delivering the corners tuning: every upcoming football fixture was serving a prediction from one of four superseded models. Same shape as the stale-worker and served-but-untrained traps - work completed, never delivered, with nothing failing or logging. Fixed by re-queueing on model_version change, which fires on promotion rather than on a schedule so routine runs still cost nothing.</t>
   </si>
   <si>
     <t>SportIQ — Edge Measurement Plan (P0-P3)</t>
@@ -5171,7 +5201,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R215"/>
+  <dimension ref="A1:R218"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -11919,7 +11949,7 @@
         <v>432</v>
       </c>
       <c r="R198" t="str">
-        <f t="shared" ref="R198:R213" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
+        <f t="shared" ref="R198:R216" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
         <v>E4 ML Football</v>
       </c>
     </row>
@@ -12337,7 +12367,7 @@
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="213" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="213" spans="1:18" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A213" t="s">
         <v>191</v>
       </c>
@@ -12367,23 +12397,113 @@
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="215" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A215" s="23" t="s">
+    <row r="214" spans="1:18" ht="72" x14ac:dyDescent="0.55000000000000004">
+      <c r="A214" t="s">
+        <v>99</v>
+      </c>
+      <c r="B214" t="s">
         <v>463</v>
       </c>
-      <c r="B215" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C215" s="15" t="s">
+      <c r="C214" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D214" t="s">
+        <v>45</v>
+      </c>
+      <c r="E214" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F214" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G214" s="215" t="s">
         <v>464</v>
       </c>
-      <c r="D215" s="17" t="s">
+      <c r="J214" t="s">
+        <v>400</v>
+      </c>
+      <c r="R214" t="str">
+        <f t="shared" si="3"/>
+        <v>E8 Model Quality</v>
+      </c>
+    </row>
+    <row r="215" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A215" t="s">
+        <v>99</v>
+      </c>
+      <c r="B215" t="s">
+        <v>465</v>
+      </c>
+      <c r="C215" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D215" t="s">
+        <v>45</v>
+      </c>
+      <c r="E215" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F215" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G215" s="215" t="s">
+        <v>466</v>
+      </c>
+      <c r="J215" t="s">
+        <v>400</v>
+      </c>
+      <c r="R215" t="str">
+        <f t="shared" si="3"/>
+        <v>E8 Model Quality</v>
+      </c>
+    </row>
+    <row r="216" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A216" t="s">
+        <v>191</v>
+      </c>
+      <c r="B216" t="s">
+        <v>467</v>
+      </c>
+      <c r="C216" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D216" t="s">
+        <v>75</v>
+      </c>
+      <c r="E216" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F216" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G216" s="215" t="s">
+        <v>468</v>
+      </c>
+      <c r="J216" t="s">
+        <v>400</v>
+      </c>
+      <c r="R216" t="str">
+        <f t="shared" si="3"/>
+        <v>E11 Ops Resilience</v>
+      </c>
+    </row>
+    <row r="218" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A218" s="23" t="s">
+        <v>469</v>
+      </c>
+      <c r="B218" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C218" s="15" t="s">
+        <v>470</v>
+      </c>
+      <c r="D218" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="E215" s="21" t="s">
+      <c r="E218" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="F215" s="19" t="s">
+      <c r="F218" s="19" t="s">
         <v>138</v>
       </c>
     </row>
@@ -12408,7 +12528,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="294" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="B1" s="283"/>
       <c r="C1" s="283"/>
@@ -12431,7 +12551,7 @@
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="301" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -12454,7 +12574,7 @@
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="289" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
       <c r="B4" s="283"/>
       <c r="C4" s="283"/>
@@ -12477,42 +12597,42 @@
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="35" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="B5" s="279" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="C5" s="280"/>
       <c r="D5" s="281"/>
       <c r="E5" s="284" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
       <c r="F5" s="280"/>
       <c r="G5" s="281"/>
       <c r="H5" s="284" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
       <c r="I5" s="280"/>
       <c r="J5" s="281"/>
       <c r="K5" s="279" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="L5" s="280"/>
       <c r="M5" s="281"/>
       <c r="N5" s="286" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
       <c r="O5" s="280"/>
       <c r="P5" s="281"/>
       <c r="Q5" s="286" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
       <c r="R5" s="280"/>
       <c r="S5" s="281"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="282" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="C6" s="283"/>
       <c r="D6" s="283"/>
@@ -12534,7 +12654,7 @@
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="289" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
       <c r="B7" s="283"/>
       <c r="C7" s="283"/>
@@ -12557,10 +12677,10 @@
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="35" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="B8" s="292" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
       <c r="C8" s="280"/>
       <c r="D8" s="280"/>
@@ -12571,7 +12691,7 @@
       <c r="I8" s="280"/>
       <c r="J8" s="281"/>
       <c r="K8" s="292" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
       <c r="L8" s="280"/>
       <c r="M8" s="280"/>
@@ -12584,7 +12704,7 @@
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="282" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="C9" s="283"/>
       <c r="D9" s="283"/>
@@ -12606,7 +12726,7 @@
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="289" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="B10" s="283"/>
       <c r="C10" s="283"/>
@@ -12629,42 +12749,42 @@
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="35" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
       <c r="B11" s="279" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
       <c r="C11" s="280"/>
       <c r="D11" s="281"/>
       <c r="E11" s="279" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
       <c r="F11" s="280"/>
       <c r="G11" s="281"/>
       <c r="H11" s="279" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
       <c r="I11" s="280"/>
       <c r="J11" s="281"/>
       <c r="K11" s="284" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="L11" s="280"/>
       <c r="M11" s="281"/>
       <c r="N11" s="279" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="O11" s="280"/>
       <c r="P11" s="281"/>
       <c r="Q11" s="279" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="R11" s="280"/>
       <c r="S11" s="281"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="282" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="C12" s="283"/>
       <c r="D12" s="283"/>
@@ -12686,7 +12806,7 @@
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="289" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
       <c r="B13" s="283"/>
       <c r="C13" s="283"/>
@@ -12709,10 +12829,10 @@
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="35" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
       <c r="B14" s="287" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
       <c r="C14" s="280"/>
       <c r="D14" s="280"/>
@@ -12720,7 +12840,7 @@
       <c r="F14" s="280"/>
       <c r="G14" s="281"/>
       <c r="H14" s="287" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="I14" s="280"/>
       <c r="J14" s="280"/>
@@ -12728,19 +12848,19 @@
       <c r="L14" s="280"/>
       <c r="M14" s="281"/>
       <c r="N14" s="287" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="O14" s="280"/>
       <c r="P14" s="281"/>
       <c r="Q14" s="284" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="R14" s="280"/>
       <c r="S14" s="281"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" s="282" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="C15" s="283"/>
       <c r="D15" s="283"/>
@@ -12762,7 +12882,7 @@
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="289" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>
@@ -12785,10 +12905,10 @@
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="35" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
       <c r="B17" s="288" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="C17" s="280"/>
       <c r="D17" s="280"/>
@@ -12796,29 +12916,29 @@
       <c r="F17" s="280"/>
       <c r="G17" s="281"/>
       <c r="H17" s="288" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
       <c r="I17" s="280"/>
       <c r="J17" s="281"/>
       <c r="K17" s="288" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="L17" s="280"/>
       <c r="M17" s="281"/>
       <c r="N17" s="288" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
       <c r="O17" s="280"/>
       <c r="P17" s="281"/>
       <c r="Q17" s="288" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="R17" s="280"/>
       <c r="S17" s="281"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="282" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="C18" s="283"/>
       <c r="D18" s="283"/>
@@ -12840,7 +12960,7 @@
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="289" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="B19" s="283"/>
       <c r="C19" s="283"/>
@@ -12863,10 +12983,10 @@
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="35" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B20" s="290" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="C20" s="280"/>
       <c r="D20" s="280"/>
@@ -12874,7 +12994,7 @@
       <c r="F20" s="280"/>
       <c r="G20" s="281"/>
       <c r="H20" s="290" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
       <c r="I20" s="280"/>
       <c r="J20" s="280"/>
@@ -12882,7 +13002,7 @@
       <c r="L20" s="280"/>
       <c r="M20" s="281"/>
       <c r="N20" s="290" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="O20" s="280"/>
       <c r="P20" s="280"/>
@@ -12892,7 +13012,7 @@
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" s="282" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="C21" s="283"/>
       <c r="D21" s="283"/>
@@ -12914,7 +13034,7 @@
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="289" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="B22" s="283"/>
       <c r="C22" s="283"/>
@@ -12937,10 +13057,10 @@
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="35" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="B23" s="290" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="C23" s="280"/>
       <c r="D23" s="280"/>
@@ -12948,29 +13068,29 @@
       <c r="F23" s="280"/>
       <c r="G23" s="281"/>
       <c r="H23" s="290" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="I23" s="280"/>
       <c r="J23" s="281"/>
       <c r="K23" s="290" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="L23" s="280"/>
       <c r="M23" s="281"/>
       <c r="N23" s="290" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="O23" s="280"/>
       <c r="P23" s="281"/>
       <c r="Q23" s="286" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
       <c r="R23" s="280"/>
       <c r="S23" s="281"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="295" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="B26" s="283"/>
       <c r="C26" s="283"/>
@@ -12993,42 +13113,42 @@
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="35" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="B27" s="279" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="C27" s="280"/>
       <c r="D27" s="281"/>
       <c r="E27" s="279" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="F27" s="280"/>
       <c r="G27" s="281"/>
       <c r="H27" s="287" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="I27" s="280"/>
       <c r="J27" s="281"/>
       <c r="K27" s="288" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="L27" s="280"/>
       <c r="M27" s="281"/>
       <c r="N27" s="288" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="O27" s="280"/>
       <c r="P27" s="281"/>
       <c r="Q27" s="287" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="R27" s="280"/>
       <c r="S27" s="281"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="289" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
       <c r="B30" s="283"/>
       <c r="C30" s="283"/>
@@ -13051,7 +13171,7 @@
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="285" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="B31" s="283"/>
       <c r="C31" s="283"/>
@@ -13074,7 +13194,7 @@
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="285" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="B32" s="283"/>
       <c r="C32" s="283"/>
@@ -13097,7 +13217,7 @@
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="285" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="B33" s="283"/>
       <c r="C33" s="283"/>
@@ -13120,7 +13240,7 @@
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="285" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="B34" s="283"/>
       <c r="C34" s="283"/>
@@ -13143,7 +13263,7 @@
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="285" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="B35" s="283"/>
       <c r="C35" s="283"/>
@@ -13166,7 +13286,7 @@
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="285" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="B36" s="283"/>
       <c r="C36" s="283"/>
@@ -13189,7 +13309,7 @@
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="296" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="B37" s="283"/>
       <c r="C37" s="283"/>
@@ -13212,25 +13332,25 @@
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="36" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="B39" s="299" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="C39" s="283"/>
       <c r="D39" s="283"/>
       <c r="E39" s="297" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="F39" s="283"/>
       <c r="G39" s="283"/>
       <c r="H39" s="300" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="I39" s="283"/>
       <c r="J39" s="283"/>
       <c r="K39" s="293" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
       <c r="L39" s="283"/>
       <c r="M39" s="283"/>
@@ -13240,7 +13360,7 @@
       <c r="O39" s="283"/>
       <c r="P39" s="283"/>
       <c r="Q39" s="298" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="R39" s="283"/>
       <c r="S39" s="283"/>
@@ -13248,11 +13368,11 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H14:M14"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A16:S16"/>
     <mergeCell ref="H20:M20"/>
-    <mergeCell ref="A16:S16"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -13261,13 +13381,14 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -13276,7 +13397,6 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
-    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -13284,7 +13404,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -13333,7 +13453,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -13346,19 +13466,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -13542,11 +13662,11 @@
       </c>
       <c r="B11" s="24">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C11" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D11" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -13558,7 +13678,7 @@
       </c>
       <c r="F11" s="25">
         <f t="shared" si="1"/>
-        <v>0.81395348837209303</v>
+        <v>0.82222222222222219</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -13617,11 +13737,11 @@
       </c>
       <c r="B14" s="24">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C14" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D14" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A14,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -13633,20 +13753,20 @@
       </c>
       <c r="F14" s="25">
         <f t="shared" si="1"/>
-        <v>0.72727272727272729</v>
+        <v>0.73913043478260865</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="26" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="B16" s="27">
         <f>SUM(B4:B14)</f>
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C16" s="27">
         <f>SUM(C4:C14)</f>
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
@@ -13658,12 +13778,12 @@
       </c>
       <c r="F16" s="28">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.77990430622009566</v>
+        <v>0.78301886792452835</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="41" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="B18" s="42">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -13672,7 +13792,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="43" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
   </sheetData>
@@ -13693,7 +13813,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -13705,7 +13825,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -13714,648 +13834,648 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="29" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="D3" s="29" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="29" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="30" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="32" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="30" t="s">
+        <v>561</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>562</v>
+      </c>
+      <c r="C6" s="21" t="s">
         <v>555</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>556</v>
-      </c>
-      <c r="C6" s="21" t="s">
-        <v>549</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="32" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="30" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="32" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="30" t="s">
+        <v>573</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>574</v>
+      </c>
+      <c r="C10" s="17" t="s">
         <v>567</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>568</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>561</v>
-      </c>
       <c r="D10" s="11" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="32" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="30" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="32" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="30" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="32" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="30" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="32" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="30" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="32" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="30" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="32" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="E21" s="33" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="30" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="32" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="30" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E24" s="31" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="53" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
       <c r="B25" s="51" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C25" s="54" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E25" s="55" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="56" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
       <c r="B26" s="46" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="C26" s="54" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="D26" s="46" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E26" s="57" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="53" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="B27" s="51" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C27" s="54" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="D27" s="51" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E27" s="55" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="71" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
       <c r="B28" s="60" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C28" s="67" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D28" s="94" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E28" s="94" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="72" t="s">
-        <v>612</v>
+        <v>618</v>
       </c>
       <c r="B29" s="65" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C29" s="69" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D29" s="93" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E29" s="93" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="78" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="B30" s="75" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C30" s="79" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D30" s="75" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E30" s="80" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="92" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
       <c r="B31" s="83" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="C31" s="90" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D31" s="83" t="s">
-        <v>617</v>
+        <v>623</v>
       </c>
       <c r="E31" s="93" t="s">
-        <v>618</v>
+        <v>624</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="106" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="B32" s="102" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C32" s="104" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D32" s="102" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E32" s="107" t="s">
-        <v>620</v>
+        <v>626</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="108" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
       <c r="B33" s="97" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C33" s="104" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D33" s="97" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="E33" s="109" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="134" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
       <c r="B34" s="129" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="C34" s="123" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D34" s="129" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E34" s="135" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="136" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
       <c r="B35" s="124" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C35" s="132" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D35" s="124" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E35" s="137" t="s">
-        <v>626</v>
+        <v>632</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="74.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="147" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="B36" s="145" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C36" s="148" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="D36" s="153" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
       <c r="E36" s="153" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="150" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="B37" s="140" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="C37" s="151" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D37" s="140" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E37" s="152" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="147" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
       <c r="B38" s="145" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="C38" s="151" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="D38" s="145" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E38" s="149" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="160" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
       <c r="B39" s="157" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C39" s="161" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D39" s="157" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E39" s="162" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="168" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
       <c r="B40" s="165" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="C40" s="169" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D40" s="165" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E40" s="170" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -14363,475 +14483,509 @@
         <v>140</v>
       </c>
       <c r="B41" s="172" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C41" s="173" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D41" s="172" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E41" s="174" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="188" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="B42" s="183" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="C42" s="177" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D42" s="183" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E42" s="189" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="190" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="B43" s="178" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C43" s="186" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D43" s="178" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="E43" s="191" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="188" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="B44" s="183" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="C44" s="186" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D44" s="183" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E44" s="189" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="190" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
       <c r="B45" s="178" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C45" s="186" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="D45" s="178" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E45" s="191" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="206" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
       <c r="B46" s="194" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C46" s="199" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D46" s="194" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E46" s="207" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="208" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
       <c r="B47" s="200" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C47" s="203" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D47" s="200" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E47" s="209" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="206" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="B48" s="194" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C48" s="203" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D48" s="194" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E48" s="207" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
       <c r="B49" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C49" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D49" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E49" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
       <c r="B50" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C50" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D50" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E50" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
       <c r="B51" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C51" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D51" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E51" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="B52" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C52" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="D52" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E52" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
       <c r="B53" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C53" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="D53" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E53" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="215" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C54" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="D54" s="215" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E54" s="215" t="s">
-        <v>664</v>
+        <v>670</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="215" t="s">
-        <v>665</v>
+        <v>671</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C55" s="215" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D55" s="215" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E55" s="215" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="215" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C56" s="215" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D56" s="215" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E56" s="215" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C57" s="215" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D57" s="215" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E57" s="215" t="s">
-        <v>670</v>
+        <v>676</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="215" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C58" s="215" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D58" s="215" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E58" s="215" t="s">
-        <v>672</v>
+        <v>678</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="215" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C59" s="215" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D59" s="215" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E59" s="215" t="s">
-        <v>674</v>
+        <v>680</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="215" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C60" s="215" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="D60" s="215" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E60" s="215" t="s">
-        <v>676</v>
+        <v>682</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="215" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C61" s="215" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D61" s="215" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E61" s="215" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="215" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C62" s="215" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D62" s="215" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E62" s="215" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="215" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C63" s="215" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="D63" s="215" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E63" s="215" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="215" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C64" s="215" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="D64" s="215" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E64" s="215" t="s">
-        <v>684</v>
+        <v>690</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="129.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="215" t="s">
-        <v>685</v>
+        <v>691</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C65" s="215" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D65" s="215" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E65" s="215" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="215" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="B66" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C66" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D66" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E66" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="215" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
       <c r="B67" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C67" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="D67" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="E67" t="s">
-        <v>690</v>
+        <v>696</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="215" t="s">
-        <v>691</v>
+        <v>697</v>
       </c>
       <c r="B68" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C68" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="D68" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E68" t="s">
-        <v>692</v>
+        <v>698</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A69" s="215" t="s">
+        <v>699</v>
+      </c>
+      <c r="B69" t="s">
+        <v>554</v>
+      </c>
+      <c r="C69" t="s">
+        <v>567</v>
+      </c>
+      <c r="D69" t="s">
+        <v>556</v>
+      </c>
+      <c r="E69" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A70" s="215" t="s">
+        <v>701</v>
+      </c>
+      <c r="B70" t="s">
+        <v>568</v>
+      </c>
+      <c r="C70" t="s">
+        <v>559</v>
+      </c>
+      <c r="D70" t="s">
+        <v>599</v>
+      </c>
+      <c r="E70" t="s">
+        <v>702</v>
       </c>
     </row>
   </sheetData>
@@ -14856,12 +15010,12 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="219" t="s">
-        <v>693</v>
+        <v>703</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="303" t="s">
-        <v>694</v>
+        <v>704</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -14870,1032 +15024,1032 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="220" t="s">
-        <v>695</v>
+        <v>705</v>
       </c>
       <c r="B4" s="220" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="C4" s="220" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="220" t="s">
-        <v>696</v>
+        <v>706</v>
       </c>
       <c r="E4" s="220" t="s">
-        <v>697</v>
+        <v>707</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="221" t="s">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>699</v>
+        <v>709</v>
       </c>
       <c r="C5" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>700</v>
+        <v>710</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>701</v>
+        <v>711</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="221" t="s">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>702</v>
+        <v>712</v>
       </c>
       <c r="C6" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="215" t="s">
-        <v>700</v>
+        <v>710</v>
       </c>
       <c r="E6" s="215" t="s">
-        <v>703</v>
+        <v>713</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="231" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>705</v>
+        <v>715</v>
       </c>
       <c r="C7" s="232" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="215" t="s">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="E7" s="215" t="s">
-        <v>706</v>
+        <v>716</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="223" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>707</v>
+        <v>717</v>
       </c>
       <c r="C8" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>708</v>
+        <v>718</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>709</v>
+        <v>719</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="223" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="B9" s="215" t="s">
-        <v>710</v>
+        <v>720</v>
       </c>
       <c r="C9" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="215" t="s">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="E9" s="215" t="s">
-        <v>711</v>
+        <v>721</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="224" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>713</v>
+        <v>723</v>
       </c>
       <c r="C10" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>714</v>
+        <v>724</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>715</v>
+        <v>725</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="C11" t="s">
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>717</v>
+        <v>727</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>718</v>
+        <v>728</v>
       </c>
       <c r="C12" t="s">
         <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>717</v>
+        <v>727</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="224" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>719</v>
+        <v>729</v>
       </c>
       <c r="C13" s="222" t="s">
         <v>128</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>720</v>
+        <v>730</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>721</v>
+        <v>731</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="235" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="C14" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>723</v>
+        <v>733</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>724</v>
+        <v>734</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="235" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B15" s="215" t="s">
-        <v>725</v>
+        <v>735</v>
       </c>
       <c r="C15" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="215" t="s">
-        <v>720</v>
+        <v>730</v>
       </c>
       <c r="E15" s="215" t="s">
-        <v>726</v>
+        <v>736</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="235" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B16" s="215" t="s">
-        <v>727</v>
+        <v>737</v>
       </c>
       <c r="C16" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="215" t="s">
-        <v>720</v>
+        <v>730</v>
       </c>
       <c r="E16" s="215" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="225" t="s">
-        <v>729</v>
+        <v>739</v>
       </c>
       <c r="B17" s="215" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="C17" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D17" s="215" t="s">
-        <v>731</v>
+        <v>741</v>
       </c>
       <c r="E17" s="215" t="s">
-        <v>732</v>
+        <v>742</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="225" t="s">
-        <v>729</v>
+        <v>739</v>
       </c>
       <c r="B18" s="215" t="s">
-        <v>733</v>
+        <v>743</v>
       </c>
       <c r="C18" s="223" t="s">
         <v>138</v>
       </c>
       <c r="D18" s="215" t="s">
-        <v>731</v>
+        <v>741</v>
       </c>
       <c r="E18" s="215" t="s">
-        <v>734</v>
+        <v>744</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="226" t="s">
-        <v>735</v>
+        <v>745</v>
       </c>
       <c r="B19" s="215" t="s">
-        <v>736</v>
+        <v>746</v>
       </c>
       <c r="C19" s="225" t="s">
-        <v>737</v>
+        <v>747</v>
       </c>
       <c r="D19" s="215" t="s">
-        <v>700</v>
+        <v>710</v>
       </c>
       <c r="E19" s="215" t="s">
-        <v>738</v>
+        <v>748</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="226" t="s">
-        <v>735</v>
+        <v>745</v>
       </c>
       <c r="B20" s="215" t="s">
-        <v>739</v>
+        <v>749</v>
       </c>
       <c r="C20" s="225" t="s">
-        <v>737</v>
+        <v>747</v>
       </c>
       <c r="D20" s="215" t="s">
-        <v>700</v>
+        <v>710</v>
       </c>
       <c r="E20" s="215" t="s">
-        <v>740</v>
+        <v>750</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="226" t="s">
-        <v>735</v>
+        <v>745</v>
       </c>
       <c r="B21" s="215" t="s">
-        <v>741</v>
+        <v>751</v>
       </c>
       <c r="C21" s="225" t="s">
-        <v>737</v>
+        <v>747</v>
       </c>
       <c r="D21" s="215" t="s">
-        <v>700</v>
+        <v>710</v>
       </c>
       <c r="E21" s="215" t="s">
-        <v>742</v>
+        <v>752</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
     <row r="23" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="229" t="s">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="B23" s="215" t="s">
-        <v>743</v>
+        <v>753</v>
       </c>
       <c r="C23" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D23" s="215" t="s">
-        <v>744</v>
+        <v>754</v>
       </c>
       <c r="E23" s="215" t="s">
-        <v>745</v>
+        <v>755</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="230" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="B24" s="215" t="s">
-        <v>746</v>
+        <v>756</v>
       </c>
       <c r="C24" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D24" s="215" t="s">
-        <v>747</v>
+        <v>757</v>
       </c>
       <c r="E24" s="215" t="s">
-        <v>748</v>
+        <v>758</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="231" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="B25" s="215" t="s">
-        <v>749</v>
+        <v>759</v>
       </c>
       <c r="C25" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D25" s="215" t="s">
-        <v>750</v>
+        <v>760</v>
       </c>
       <c r="E25" s="215" t="s">
-        <v>751</v>
+        <v>761</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="231" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="B26" s="215" t="s">
-        <v>752</v>
+        <v>762</v>
       </c>
       <c r="C26" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D26" s="215" t="s">
-        <v>747</v>
+        <v>757</v>
       </c>
       <c r="E26" s="215" t="s">
-        <v>753</v>
+        <v>763</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="235" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B27" s="215" t="s">
-        <v>754</v>
+        <v>764</v>
       </c>
       <c r="C27" s="237" t="s">
         <v>22</v>
       </c>
       <c r="D27" s="215" t="s">
-        <v>717</v>
+        <v>727</v>
       </c>
       <c r="E27" s="215" t="s">
-        <v>755</v>
+        <v>765</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="227" t="s">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="B28" s="215" t="s">
-        <v>756</v>
+        <v>766</v>
       </c>
       <c r="C28" t="s">
         <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>757</v>
+        <v>767</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B29" s="215" t="s">
-        <v>758</v>
+        <v>768</v>
       </c>
       <c r="C29" t="s">
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>717</v>
+        <v>727</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B30" s="215" t="s">
-        <v>759</v>
+        <v>769</v>
       </c>
       <c r="C30" t="s">
         <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>760</v>
+        <v>770</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="B31" s="215" t="s">
-        <v>761</v>
+        <v>771</v>
       </c>
       <c r="C31" t="s">
         <v>22</v>
       </c>
       <c r="D31" t="s">
-        <v>762</v>
+        <v>772</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="B32" s="215" t="s">
-        <v>763</v>
+        <v>773</v>
       </c>
       <c r="C32" t="s">
         <v>22</v>
       </c>
       <c r="D32" t="s">
-        <v>764</v>
+        <v>774</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="B33" s="215" t="s">
-        <v>765</v>
+        <v>775</v>
       </c>
       <c r="C33" t="s">
         <v>22</v>
       </c>
       <c r="D33" t="s">
-        <v>762</v>
+        <v>772</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="B34" s="215" t="s">
-        <v>766</v>
+        <v>776</v>
       </c>
       <c r="C34" t="s">
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>767</v>
+        <v>777</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B35" s="215" t="s">
-        <v>768</v>
+        <v>778</v>
       </c>
       <c r="C35" t="s">
         <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>769</v>
+        <v>779</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="B36" s="215" t="s">
-        <v>770</v>
+        <v>780</v>
       </c>
       <c r="C36" t="s">
         <v>22</v>
       </c>
       <c r="D36" t="s">
-        <v>771</v>
+        <v>781</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B37" s="215" t="s">
-        <v>772</v>
+        <v>782</v>
       </c>
       <c r="C37" t="s">
         <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>771</v>
+        <v>781</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
-        <v>729</v>
+        <v>739</v>
       </c>
       <c r="B38" s="215" t="s">
-        <v>773</v>
+        <v>783</v>
       </c>
       <c r="C38" t="s">
         <v>22</v>
       </c>
       <c r="D38" t="s">
-        <v>771</v>
+        <v>781</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="B39" s="215" t="s">
-        <v>774</v>
+        <v>784</v>
       </c>
       <c r="C39" t="s">
         <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>771</v>
+        <v>781</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B40" s="215" t="s">
-        <v>775</v>
+        <v>785</v>
       </c>
       <c r="C40" t="s">
         <v>22</v>
       </c>
       <c r="D40" t="s">
-        <v>771</v>
+        <v>781</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="B41" s="215" t="s">
-        <v>776</v>
+        <v>786</v>
       </c>
       <c r="C41" t="s">
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>777</v>
+        <v>787</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B42" s="215" t="s">
-        <v>778</v>
+        <v>788</v>
       </c>
       <c r="C42" t="s">
         <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>777</v>
+        <v>787</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B43" s="215" t="s">
-        <v>779</v>
+        <v>789</v>
       </c>
       <c r="C43" t="s">
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>780</v>
+        <v>790</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B44" s="215" t="s">
-        <v>781</v>
+        <v>791</v>
       </c>
       <c r="C44" t="s">
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>780</v>
+        <v>790</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
-        <v>729</v>
+        <v>739</v>
       </c>
       <c r="B45" s="215" t="s">
-        <v>782</v>
+        <v>792</v>
       </c>
       <c r="C45" t="s">
         <v>128</v>
       </c>
       <c r="D45" t="s">
-        <v>783</v>
+        <v>793</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B46" s="215" t="s">
-        <v>785</v>
+        <v>795</v>
       </c>
       <c r="C46" t="s">
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>786</v>
+        <v>796</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B47" s="215" t="s">
-        <v>787</v>
+        <v>797</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>788</v>
+        <v>798</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B48" s="215" t="s">
-        <v>789</v>
+        <v>799</v>
       </c>
       <c r="C48" t="s">
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>788</v>
+        <v>798</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B49" s="215" t="s">
-        <v>790</v>
+        <v>800</v>
       </c>
       <c r="C49" t="s">
         <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>788</v>
+        <v>798</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B50" s="215" t="s">
-        <v>791</v>
+        <v>801</v>
       </c>
       <c r="C50" t="s">
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>792</v>
+        <v>802</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B51" s="215" t="s">
-        <v>793</v>
+        <v>803</v>
       </c>
       <c r="C51" t="s">
         <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>794</v>
+        <v>804</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B52" s="215" t="s">
-        <v>795</v>
+        <v>805</v>
       </c>
       <c r="C52" t="s">
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>796</v>
+        <v>806</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B53" s="215" t="s">
-        <v>797</v>
+        <v>807</v>
       </c>
       <c r="C53" t="s">
         <v>128</v>
       </c>
       <c r="D53" t="s">
-        <v>794</v>
+        <v>804</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>798</v>
+        <v>808</v>
       </c>
       <c r="C54" t="s">
         <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>796</v>
+        <v>806</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>799</v>
+        <v>809</v>
       </c>
       <c r="C55" t="s">
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>800</v>
+        <v>810</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>801</v>
+        <v>811</v>
       </c>
       <c r="C56" t="s">
         <v>128</v>
       </c>
       <c r="D56" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>803</v>
+        <v>813</v>
       </c>
       <c r="C57" t="s">
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>804</v>
+        <v>814</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>805</v>
+        <v>815</v>
       </c>
       <c r="C58" t="s">
         <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>804</v>
+        <v>814</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>806</v>
+        <v>816</v>
       </c>
       <c r="C59" t="s">
         <v>22</v>
       </c>
       <c r="D59" t="s">
-        <v>804</v>
+        <v>814</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>807</v>
+        <v>817</v>
       </c>
       <c r="C60" t="s">
         <v>128</v>
       </c>
       <c r="D60" t="s">
-        <v>804</v>
+        <v>814</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="274" t="s">
-        <v>808</v>
+        <v>818</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>809</v>
+        <v>819</v>
       </c>
       <c r="C61" t="s">
         <v>22</v>
       </c>
       <c r="D61" t="s">
-        <v>777</v>
+        <v>787</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="274" t="s">
-        <v>808</v>
+        <v>818</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>810</v>
+        <v>820</v>
       </c>
       <c r="C62" t="s">
         <v>22</v>
       </c>
       <c r="D62" t="s">
-        <v>777</v>
+        <v>787</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="274" t="s">
-        <v>808</v>
+        <v>818</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>811</v>
+        <v>821</v>
       </c>
       <c r="C63" t="s">
         <v>22</v>
       </c>
       <c r="D63" t="s">
-        <v>777</v>
+        <v>787</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>812</v>
+        <v>822</v>
       </c>
       <c r="C64" t="s">
         <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>813</v>
+        <v>823</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>814</v>
+        <v>824</v>
       </c>
       <c r="C65" t="s">
         <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>813</v>
+        <v>823</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B66" s="215" t="s">
-        <v>815</v>
+        <v>825</v>
       </c>
       <c r="C66" t="s">
         <v>22</v>
       </c>
       <c r="D66" t="s">
-        <v>813</v>
+        <v>823</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="274" t="s">
-        <v>816</v>
+        <v>826</v>
       </c>
       <c r="B67" s="215" t="s">
-        <v>817</v>
+        <v>827</v>
       </c>
       <c r="C67" t="s">
         <v>22</v>
       </c>
       <c r="D67" t="s">
-        <v>777</v>
+        <v>787</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="274" t="s">
-        <v>816</v>
+        <v>826</v>
       </c>
       <c r="B68" s="215" t="s">
-        <v>818</v>
+        <v>828</v>
       </c>
       <c r="C68" t="s">
         <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>777</v>
+        <v>787</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="274" t="s">
-        <v>816</v>
+        <v>826</v>
       </c>
       <c r="B69" s="215" t="s">
-        <v>819</v>
+        <v>829</v>
       </c>
       <c r="C69" t="s">
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>777</v>
+        <v>787</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B70" s="215" t="s">
-        <v>820</v>
+        <v>830</v>
       </c>
       <c r="C70" t="s">
         <v>22</v>
       </c>
       <c r="D70" t="s">
-        <v>821</v>
+        <v>831</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B71" s="215" t="s">
-        <v>822</v>
+        <v>832</v>
       </c>
       <c r="C71" t="s">
         <v>22</v>
       </c>
       <c r="D71" t="s">
-        <v>821</v>
+        <v>831</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B72" s="215" t="s">
-        <v>823</v>
+        <v>833</v>
       </c>
       <c r="C72" t="s">
         <v>22</v>
       </c>
       <c r="D72" t="s">
-        <v>821</v>
+        <v>831</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="274" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B73" s="215" t="s">
-        <v>824</v>
+        <v>834</v>
       </c>
       <c r="C73" t="s">
         <v>128</v>
       </c>
       <c r="D73" t="s">
-        <v>821</v>
+        <v>831</v>
       </c>
     </row>
   </sheetData>
@@ -15924,336 +16078,336 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="211" t="s">
-        <v>825</v>
+        <v>835</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="212" t="s">
-        <v>826</v>
+        <v>836</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="213" t="s">
-        <v>827</v>
+        <v>837</v>
       </c>
       <c r="B4" s="213" t="s">
-        <v>828</v>
+        <v>838</v>
       </c>
       <c r="C4" s="213" t="s">
-        <v>829</v>
+        <v>839</v>
       </c>
       <c r="D4" s="213" t="s">
-        <v>830</v>
+        <v>840</v>
       </c>
       <c r="E4" s="213" t="s">
-        <v>831</v>
+        <v>841</v>
       </c>
       <c r="F4" s="213" t="s">
-        <v>832</v>
+        <v>842</v>
       </c>
       <c r="G4" s="213" t="s">
-        <v>833</v>
+        <v>843</v>
       </c>
       <c r="H4" s="213" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="213" t="s">
-        <v>834</v>
+        <v>844</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="214" t="s">
-        <v>835</v>
+        <v>845</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>836</v>
+        <v>846</v>
       </c>
       <c r="C5" s="215" t="s">
-        <v>837</v>
+        <v>847</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>838</v>
+        <v>848</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>839</v>
+        <v>849</v>
       </c>
       <c r="F5" s="215" t="s">
-        <v>840</v>
+        <v>850</v>
       </c>
       <c r="G5" s="215" t="s">
-        <v>841</v>
+        <v>851</v>
       </c>
       <c r="H5" s="216" t="s">
-        <v>842</v>
+        <v>852</v>
       </c>
       <c r="I5" s="215" t="s">
-        <v>843</v>
+        <v>853</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="214" t="s">
-        <v>844</v>
+        <v>854</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>845</v>
+        <v>855</v>
       </c>
       <c r="C6" s="215" t="s">
-        <v>846</v>
+        <v>856</v>
       </c>
       <c r="D6" s="215" t="s">
-        <v>847</v>
+        <v>857</v>
       </c>
       <c r="E6" s="215" t="s">
-        <v>848</v>
+        <v>858</v>
       </c>
       <c r="F6" s="215" t="s">
-        <v>849</v>
+        <v>859</v>
       </c>
       <c r="G6" s="215" t="s">
-        <v>850</v>
+        <v>860</v>
       </c>
       <c r="H6" s="217" t="s">
-        <v>842</v>
+        <v>852</v>
       </c>
       <c r="I6" s="215" t="s">
-        <v>851</v>
+        <v>861</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="214" t="s">
+        <v>862</v>
+      </c>
+      <c r="B7" s="215" t="s">
+        <v>863</v>
+      </c>
+      <c r="C7" s="215" t="s">
+        <v>864</v>
+      </c>
+      <c r="D7" s="215" t="s">
+        <v>865</v>
+      </c>
+      <c r="E7" s="215" t="s">
+        <v>866</v>
+      </c>
+      <c r="F7" s="215" t="s">
+        <v>867</v>
+      </c>
+      <c r="G7" s="215" t="s">
+        <v>868</v>
+      </c>
+      <c r="H7" s="217" t="s">
         <v>852</v>
       </c>
-      <c r="B7" s="215" t="s">
-        <v>853</v>
-      </c>
-      <c r="C7" s="215" t="s">
-        <v>854</v>
-      </c>
-      <c r="D7" s="215" t="s">
-        <v>855</v>
-      </c>
-      <c r="E7" s="215" t="s">
-        <v>856</v>
-      </c>
-      <c r="F7" s="215" t="s">
-        <v>857</v>
-      </c>
-      <c r="G7" s="215" t="s">
-        <v>858</v>
-      </c>
-      <c r="H7" s="217" t="s">
-        <v>842</v>
-      </c>
       <c r="I7" s="215" t="s">
-        <v>859</v>
+        <v>869</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="214" t="s">
-        <v>860</v>
+        <v>870</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>861</v>
+        <v>871</v>
       </c>
       <c r="C8" s="215" t="s">
-        <v>862</v>
+        <v>872</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>863</v>
+        <v>873</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="F8" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="G8" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="H8" s="216" t="s">
-        <v>864</v>
+        <v>874</v>
       </c>
       <c r="I8" s="215" t="s">
-        <v>865</v>
+        <v>875</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="214" t="s">
+        <v>876</v>
+      </c>
+      <c r="B9" s="215" t="s">
+        <v>877</v>
+      </c>
+      <c r="C9" s="215" t="s">
+        <v>878</v>
+      </c>
+      <c r="D9" s="215" t="s">
+        <v>873</v>
+      </c>
+      <c r="E9" s="215" t="s">
         <v>866</v>
       </c>
-      <c r="B9" s="215" t="s">
-        <v>867</v>
-      </c>
-      <c r="C9" s="215" t="s">
-        <v>868</v>
-      </c>
-      <c r="D9" s="215" t="s">
-        <v>863</v>
-      </c>
-      <c r="E9" s="215" t="s">
-        <v>856</v>
-      </c>
       <c r="F9" s="215" t="s">
-        <v>869</v>
+        <v>879</v>
       </c>
       <c r="G9" s="215" t="s">
-        <v>870</v>
+        <v>880</v>
       </c>
       <c r="H9" s="218" t="s">
-        <v>871</v>
+        <v>881</v>
       </c>
       <c r="I9" s="215" t="s">
-        <v>872</v>
+        <v>882</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="214" t="s">
-        <v>873</v>
+        <v>883</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>874</v>
+        <v>884</v>
       </c>
       <c r="C10" s="215" t="s">
-        <v>875</v>
+        <v>885</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>876</v>
+        <v>886</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>877</v>
+        <v>887</v>
       </c>
       <c r="F10" s="215" t="s">
-        <v>878</v>
+        <v>888</v>
       </c>
       <c r="G10" s="215" t="s">
-        <v>879</v>
+        <v>889</v>
       </c>
       <c r="H10" s="218" t="s">
-        <v>880</v>
+        <v>890</v>
       </c>
       <c r="I10" s="215" t="s">
-        <v>881</v>
+        <v>891</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="214" t="s">
-        <v>882</v>
+        <v>892</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>883</v>
+        <v>893</v>
       </c>
       <c r="C11" s="215" t="s">
-        <v>884</v>
+        <v>894</v>
       </c>
       <c r="D11" s="215" t="s">
-        <v>885</v>
+        <v>895</v>
       </c>
       <c r="E11" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="F11" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="G11" s="215" t="s">
-        <v>886</v>
+        <v>896</v>
       </c>
       <c r="H11" s="218" t="s">
-        <v>887</v>
+        <v>897</v>
       </c>
       <c r="I11" s="215" t="s">
-        <v>888</v>
+        <v>898</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="214" t="s">
-        <v>889</v>
+        <v>899</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>890</v>
+        <v>900</v>
       </c>
       <c r="C12" s="215" t="s">
-        <v>891</v>
+        <v>901</v>
       </c>
       <c r="D12" s="215" t="s">
-        <v>892</v>
+        <v>902</v>
       </c>
       <c r="E12" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="F12" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="G12" s="215" t="s">
-        <v>886</v>
+        <v>896</v>
       </c>
       <c r="H12" s="217" t="s">
-        <v>893</v>
+        <v>903</v>
       </c>
       <c r="I12" s="215" t="s">
-        <v>894</v>
+        <v>904</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="214" t="s">
-        <v>895</v>
+        <v>905</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>896</v>
+        <v>906</v>
       </c>
       <c r="C13" s="215" t="s">
-        <v>897</v>
+        <v>907</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="F13" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="G13" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="H13" s="218" t="s">
-        <v>898</v>
+        <v>908</v>
       </c>
       <c r="I13" s="215" t="s">
-        <v>899</v>
+        <v>909</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="214" t="s">
-        <v>900</v>
+        <v>910</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>901</v>
+        <v>911</v>
       </c>
       <c r="C14" s="215" t="s">
-        <v>897</v>
+        <v>907</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="F14" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="G14" s="215" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="H14" s="218" t="s">
-        <v>898</v>
+        <v>908</v>
       </c>
       <c r="I14" s="215" t="s">
-        <v>902</v>
+        <v>912</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="304" t="s">
-        <v>903</v>
+        <v>913</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>

</xml_diff>

<commit_message>
docs(tracker): prediction-history notebook and the row-vs-fixture counting fix
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{525A0C13-758A-4A76-ABF9-71C824732858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E69EB30D-D30E-4A13-BB0E-B94633F4A487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1904" uniqueCount="914">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1926" uniqueCount="922">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -1445,6 +1445,18 @@
   </si>
   <si>
     <t>All 135 upcoming football fixtures were serving predictions from one of FOUR superseded versions. Guard only asked 'does a prediction exist'; promotion is a DB update so nothing logged. Re-queues on version change only, so a daily run still queues nothing</t>
+  </si>
+  <si>
+    <t>Prediction-history analytics notebook</t>
+  </si>
+  <si>
+    <t>ml/notebooks/prediction_history.ipynb - daily results, cumulative accuracy with Wilson bands, reliability/Brier, confidence tier, feature completeness, per-league vs own baseline, CLV, market mix, plus a history() query helper that always returns n/CI/detectable effect. Metric helpers imported from app.history.router so it cannot drift from the endpoint</t>
+  </si>
+  <si>
+    <t>History metrics counted rows, not fixtures</t>
+  </si>
+  <si>
+    <t>Found by the notebook. run_predictions appends rather than replaces; 143 settled football rows sat on 63 fixtures (one had 25), overstating accuracy by 18.7pp (0.5524-&gt;0.3651). Now one row per fixture/kind - the last created BEFORE kickoff. Football now reads below its own baseline, which is the honest number</t>
   </si>
   <si>
     <t>Legend</t>
@@ -2219,6 +2231,18 @@
   </si>
   <si>
     <t>Found while delivering the corners tuning: every upcoming football fixture was serving a prediction from one of four superseded models. Same shape as the stale-worker and served-but-untrained traps - work completed, never delivered, with nothing failing or logging. Fixed by re-queueing on model_version change, which fires on promotion rather than on a schedule so routine runs still cost nothing.</t>
+  </si>
+  <si>
+    <t>Football pre-match accuracy is below baseline</t>
+  </si>
+  <si>
+    <t>Once each fixture counts once: n=63, accuracy 0.3651, CI [0.257, 0.489], against a ~0.47 baseline. NOT reportable (floor is 93) and the interval spans the baseline, so this is not yet evidence the model is worse than picking home - but it is the opposite direction from what was previously displayed and it is the number to watch as n grows.</t>
+  </si>
+  <si>
+    <t>Duplicate predictions were mis-triaged as harmless</t>
+  </si>
+  <si>
+    <t>They were checked for the failure mode that had bitten before (MultipleResultsFound via scalar_one) and cleared on that basis, while the defect actually present was silent inflation of a live user-facing accuracy. Checking for the last bug is not the same as checking for a bug.</t>
   </si>
   <si>
     <t>SportIQ — Edge Measurement Plan (P0-P3)</t>
@@ -5201,7 +5225,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R218"/>
+  <dimension ref="A1:R220"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -11949,7 +11973,7 @@
         <v>432</v>
       </c>
       <c r="R198" t="str">
-        <f t="shared" ref="R198:R216" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
+        <f t="shared" ref="R198:R218" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
         <v>E4 ML Football</v>
       </c>
     </row>
@@ -12397,7 +12421,7 @@
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="214" spans="1:18" ht="72" x14ac:dyDescent="0.55000000000000004">
+    <row r="214" spans="1:18" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A214" t="s">
         <v>99</v>
       </c>
@@ -12427,7 +12451,7 @@
         <v>E8 Model Quality</v>
       </c>
     </row>
-    <row r="215" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="215" spans="1:18" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A215" t="s">
         <v>99</v>
       </c>
@@ -12457,7 +12481,7 @@
         <v>E8 Model Quality</v>
       </c>
     </row>
-    <row r="216" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="216" spans="1:18" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A216" t="s">
         <v>191</v>
       </c>
@@ -12487,23 +12511,83 @@
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="218" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A218" s="23" t="s">
+    <row r="217" spans="1:18" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A217" t="s">
+        <v>99</v>
+      </c>
+      <c r="B217" t="s">
         <v>469</v>
       </c>
-      <c r="B218" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C218" s="15" t="s">
+      <c r="C217" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D217" t="s">
+        <v>45</v>
+      </c>
+      <c r="E217" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F217" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G217" s="215" t="s">
         <v>470</v>
       </c>
-      <c r="D218" s="17" t="s">
+      <c r="J217" t="s">
+        <v>400</v>
+      </c>
+      <c r="R217" t="str">
+        <f t="shared" si="3"/>
+        <v>E8 Model Quality</v>
+      </c>
+    </row>
+    <row r="218" spans="1:18" ht="72" x14ac:dyDescent="0.55000000000000004">
+      <c r="A218" t="s">
+        <v>99</v>
+      </c>
+      <c r="B218" t="s">
+        <v>471</v>
+      </c>
+      <c r="C218" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D218" t="s">
+        <v>75</v>
+      </c>
+      <c r="E218" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F218" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G218" s="215" t="s">
+        <v>472</v>
+      </c>
+      <c r="J218" t="s">
+        <v>400</v>
+      </c>
+      <c r="R218" t="str">
+        <f t="shared" si="3"/>
+        <v>E8 Model Quality</v>
+      </c>
+    </row>
+    <row r="220" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A220" s="23" t="s">
+        <v>473</v>
+      </c>
+      <c r="B220" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C220" s="15" t="s">
+        <v>474</v>
+      </c>
+      <c r="D220" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="E218" s="21" t="s">
+      <c r="E220" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="F218" s="19" t="s">
+      <c r="F220" s="19" t="s">
         <v>138</v>
       </c>
     </row>
@@ -12528,7 +12612,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="294" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="B1" s="283"/>
       <c r="C1" s="283"/>
@@ -12551,7 +12635,7 @@
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="301" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -12574,7 +12658,7 @@
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="289" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B4" s="283"/>
       <c r="C4" s="283"/>
@@ -12597,42 +12681,42 @@
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="35" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="B5" s="279" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="C5" s="280"/>
       <c r="D5" s="281"/>
       <c r="E5" s="284" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="F5" s="280"/>
       <c r="G5" s="281"/>
       <c r="H5" s="284" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="I5" s="280"/>
       <c r="J5" s="281"/>
       <c r="K5" s="279" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="L5" s="280"/>
       <c r="M5" s="281"/>
       <c r="N5" s="286" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="O5" s="280"/>
       <c r="P5" s="281"/>
       <c r="Q5" s="286" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="R5" s="280"/>
       <c r="S5" s="281"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="282" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="C6" s="283"/>
       <c r="D6" s="283"/>
@@ -12654,7 +12738,7 @@
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="289" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="B7" s="283"/>
       <c r="C7" s="283"/>
@@ -12677,10 +12761,10 @@
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="35" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="B8" s="292" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="C8" s="280"/>
       <c r="D8" s="280"/>
@@ -12691,7 +12775,7 @@
       <c r="I8" s="280"/>
       <c r="J8" s="281"/>
       <c r="K8" s="292" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="L8" s="280"/>
       <c r="M8" s="280"/>
@@ -12704,7 +12788,7 @@
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="282" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="C9" s="283"/>
       <c r="D9" s="283"/>
@@ -12726,7 +12810,7 @@
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="289" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="B10" s="283"/>
       <c r="C10" s="283"/>
@@ -12749,42 +12833,42 @@
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="35" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="B11" s="279" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="C11" s="280"/>
       <c r="D11" s="281"/>
       <c r="E11" s="279" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="F11" s="280"/>
       <c r="G11" s="281"/>
       <c r="H11" s="279" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="I11" s="280"/>
       <c r="J11" s="281"/>
       <c r="K11" s="284" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="L11" s="280"/>
       <c r="M11" s="281"/>
       <c r="N11" s="279" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="O11" s="280"/>
       <c r="P11" s="281"/>
       <c r="Q11" s="279" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="R11" s="280"/>
       <c r="S11" s="281"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="282" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="C12" s="283"/>
       <c r="D12" s="283"/>
@@ -12806,7 +12890,7 @@
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="289" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="B13" s="283"/>
       <c r="C13" s="283"/>
@@ -12829,10 +12913,10 @@
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="35" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="B14" s="287" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="C14" s="280"/>
       <c r="D14" s="280"/>
@@ -12840,7 +12924,7 @@
       <c r="F14" s="280"/>
       <c r="G14" s="281"/>
       <c r="H14" s="287" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="I14" s="280"/>
       <c r="J14" s="280"/>
@@ -12848,19 +12932,19 @@
       <c r="L14" s="280"/>
       <c r="M14" s="281"/>
       <c r="N14" s="287" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="O14" s="280"/>
       <c r="P14" s="281"/>
       <c r="Q14" s="284" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="R14" s="280"/>
       <c r="S14" s="281"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" s="282" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="C15" s="283"/>
       <c r="D15" s="283"/>
@@ -12882,7 +12966,7 @@
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="289" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>
@@ -12905,10 +12989,10 @@
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="35" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="B17" s="288" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="C17" s="280"/>
       <c r="D17" s="280"/>
@@ -12916,29 +13000,29 @@
       <c r="F17" s="280"/>
       <c r="G17" s="281"/>
       <c r="H17" s="288" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="I17" s="280"/>
       <c r="J17" s="281"/>
       <c r="K17" s="288" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="L17" s="280"/>
       <c r="M17" s="281"/>
       <c r="N17" s="288" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="O17" s="280"/>
       <c r="P17" s="281"/>
       <c r="Q17" s="288" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="R17" s="280"/>
       <c r="S17" s="281"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="282" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="C18" s="283"/>
       <c r="D18" s="283"/>
@@ -12960,7 +13044,7 @@
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="289" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="B19" s="283"/>
       <c r="C19" s="283"/>
@@ -12983,10 +13067,10 @@
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="35" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="B20" s="290" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="C20" s="280"/>
       <c r="D20" s="280"/>
@@ -12994,7 +13078,7 @@
       <c r="F20" s="280"/>
       <c r="G20" s="281"/>
       <c r="H20" s="290" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="I20" s="280"/>
       <c r="J20" s="280"/>
@@ -13002,7 +13086,7 @@
       <c r="L20" s="280"/>
       <c r="M20" s="281"/>
       <c r="N20" s="290" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="O20" s="280"/>
       <c r="P20" s="280"/>
@@ -13012,7 +13096,7 @@
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" s="282" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="C21" s="283"/>
       <c r="D21" s="283"/>
@@ -13034,7 +13118,7 @@
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="289" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
       <c r="B22" s="283"/>
       <c r="C22" s="283"/>
@@ -13057,10 +13141,10 @@
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="35" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="B23" s="290" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="C23" s="280"/>
       <c r="D23" s="280"/>
@@ -13068,29 +13152,29 @@
       <c r="F23" s="280"/>
       <c r="G23" s="281"/>
       <c r="H23" s="290" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="I23" s="280"/>
       <c r="J23" s="281"/>
       <c r="K23" s="290" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="L23" s="280"/>
       <c r="M23" s="281"/>
       <c r="N23" s="290" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="O23" s="280"/>
       <c r="P23" s="281"/>
       <c r="Q23" s="286" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="R23" s="280"/>
       <c r="S23" s="281"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="295" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="B26" s="283"/>
       <c r="C26" s="283"/>
@@ -13113,42 +13197,42 @@
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="35" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="B27" s="279" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="C27" s="280"/>
       <c r="D27" s="281"/>
       <c r="E27" s="279" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="F27" s="280"/>
       <c r="G27" s="281"/>
       <c r="H27" s="287" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="I27" s="280"/>
       <c r="J27" s="281"/>
       <c r="K27" s="288" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="L27" s="280"/>
       <c r="M27" s="281"/>
       <c r="N27" s="288" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="O27" s="280"/>
       <c r="P27" s="281"/>
       <c r="Q27" s="287" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="R27" s="280"/>
       <c r="S27" s="281"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="289" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="B30" s="283"/>
       <c r="C30" s="283"/>
@@ -13171,7 +13255,7 @@
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="285" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="B31" s="283"/>
       <c r="C31" s="283"/>
@@ -13194,7 +13278,7 @@
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="285" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="B32" s="283"/>
       <c r="C32" s="283"/>
@@ -13217,7 +13301,7 @@
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="285" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="B33" s="283"/>
       <c r="C33" s="283"/>
@@ -13240,7 +13324,7 @@
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="285" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="B34" s="283"/>
       <c r="C34" s="283"/>
@@ -13263,7 +13347,7 @@
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="285" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="B35" s="283"/>
       <c r="C35" s="283"/>
@@ -13286,7 +13370,7 @@
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="285" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="B36" s="283"/>
       <c r="C36" s="283"/>
@@ -13309,7 +13393,7 @@
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="296" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="B37" s="283"/>
       <c r="C37" s="283"/>
@@ -13332,25 +13416,25 @@
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="36" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="B39" s="299" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="C39" s="283"/>
       <c r="D39" s="283"/>
       <c r="E39" s="297" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="F39" s="283"/>
       <c r="G39" s="283"/>
       <c r="H39" s="300" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="I39" s="283"/>
       <c r="J39" s="283"/>
       <c r="K39" s="293" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="L39" s="283"/>
       <c r="M39" s="283"/>
@@ -13360,7 +13444,7 @@
       <c r="O39" s="283"/>
       <c r="P39" s="283"/>
       <c r="Q39" s="298" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="R39" s="283"/>
       <c r="S39" s="283"/>
@@ -13368,11 +13452,11 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="H20:M20"/>
     <mergeCell ref="A16:S16"/>
-    <mergeCell ref="H20:M20"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -13381,14 +13465,13 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -13397,6 +13480,7 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -13404,7 +13488,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -13453,7 +13537,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -13466,19 +13550,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -13662,11 +13746,11 @@
       </c>
       <c r="B11" s="24">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C11" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D11" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -13678,7 +13762,7 @@
       </c>
       <c r="F11" s="25">
         <f t="shared" si="1"/>
-        <v>0.82222222222222219</v>
+        <v>0.82978723404255317</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -13758,15 +13842,15 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="26" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="B16" s="27">
         <f>SUM(B4:B14)</f>
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C16" s="27">
         <f>SUM(C4:C14)</f>
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
@@ -13778,12 +13862,12 @@
       </c>
       <c r="F16" s="28">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.78301886792452835</v>
+        <v>0.78504672897196259</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="41" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="B18" s="42">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -13792,7 +13876,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="43" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
     </row>
   </sheetData>
@@ -13813,7 +13897,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -13825,7 +13909,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -13834,648 +13918,648 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="29" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="D3" s="29" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="29" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="30" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="32" t="s">
+        <v>562</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>558</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>554</v>
-      </c>
       <c r="C5" s="19" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="30" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="32" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="30" t="s">
+        <v>570</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>566</v>
       </c>
-      <c r="B8" s="11" t="s">
-        <v>562</v>
-      </c>
       <c r="C8" s="17" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="32" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="30" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="32" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="30" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="32" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="30" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="32" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="30" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="32" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="30" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="32" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="30" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="32" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="E21" s="33" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="30" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="32" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="30" t="s">
+        <v>612</v>
+      </c>
+      <c r="B24" s="11" t="s">
         <v>608</v>
       </c>
-      <c r="B24" s="11" t="s">
-        <v>604</v>
-      </c>
       <c r="C24" s="17" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E24" s="31" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="53" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="B25" s="51" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C25" s="54" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E25" s="55" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="56" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="B26" s="46" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="C26" s="54" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="D26" s="46" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E26" s="57" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="53" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="B27" s="51" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C27" s="54" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="D27" s="51" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E27" s="55" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="71" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="B28" s="60" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C28" s="67" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D28" s="94" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E28" s="94" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="72" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="B29" s="65" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C29" s="69" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D29" s="93" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E29" s="93" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="78" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="B30" s="75" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C30" s="79" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D30" s="75" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E30" s="80" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="92" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="B31" s="83" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="C31" s="90" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D31" s="83" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="E31" s="93" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="106" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="B32" s="102" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C32" s="104" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D32" s="102" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E32" s="107" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="108" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="B33" s="97" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C33" s="104" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D33" s="97" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="E33" s="109" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="134" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="B34" s="129" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="C34" s="123" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D34" s="129" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E34" s="135" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="136" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="B35" s="124" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C35" s="132" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D35" s="124" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E35" s="137" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="74.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="147" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
       <c r="B36" s="145" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C36" s="148" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="D36" s="153" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="E36" s="153" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="150" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="B37" s="140" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="C37" s="151" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D37" s="140" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E37" s="152" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="147" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="B38" s="145" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="C38" s="151" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="D38" s="145" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E38" s="149" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="160" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="B39" s="157" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C39" s="161" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D39" s="157" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E39" s="162" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="168" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="B40" s="165" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="C40" s="169" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D40" s="165" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E40" s="170" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -14483,509 +14567,543 @@
         <v>140</v>
       </c>
       <c r="B41" s="172" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C41" s="173" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D41" s="172" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E41" s="174" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="188" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="B42" s="183" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="C42" s="177" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D42" s="183" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E42" s="189" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="190" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="B43" s="178" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C43" s="186" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D43" s="178" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="E43" s="191" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="188" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="B44" s="183" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="C44" s="186" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D44" s="183" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E44" s="189" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="190" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="B45" s="178" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C45" s="186" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="D45" s="178" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E45" s="191" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="206" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="B46" s="194" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C46" s="199" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D46" s="194" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E46" s="207" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="208" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="B47" s="200" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C47" s="203" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D47" s="200" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E47" s="209" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="206" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="B48" s="194" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C48" s="203" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D48" s="194" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E48" s="207" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="B49" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C49" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D49" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E49" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="B50" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C50" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D50" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E50" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="B51" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C51" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D51" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E51" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="B52" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C52" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="D52" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E52" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="B53" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C53" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="D53" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E53" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="215" t="s">
+        <v>673</v>
+      </c>
+      <c r="B54" s="215" t="s">
+        <v>572</v>
+      </c>
+      <c r="C54" s="215" t="s">
         <v>669</v>
       </c>
-      <c r="B54" s="215" t="s">
-        <v>568</v>
-      </c>
-      <c r="C54" s="215" t="s">
-        <v>665</v>
-      </c>
       <c r="D54" s="215" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E54" s="215" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="215" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C55" s="215" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D55" s="215" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E55" s="215" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="215" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C56" s="215" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D56" s="215" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E56" s="215" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="215" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C57" s="215" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D57" s="215" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E57" s="215" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="215" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C58" s="215" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D58" s="215" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E58" s="215" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="215" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C59" s="215" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D59" s="215" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E59" s="215" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="215" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C60" s="215" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D60" s="215" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E60" s="215" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="215" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C61" s="215" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D61" s="215" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E61" s="215" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="215" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C62" s="215" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D62" s="215" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E62" s="215" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="215" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C63" s="215" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="D63" s="215" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E63" s="215" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="215" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C64" s="215" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="D64" s="215" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E64" s="215" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="129.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="215" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C65" s="215" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D65" s="215" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E65" s="215" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="215" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="B66" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C66" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D66" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E66" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="215" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="B67" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C67" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="D67" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E67" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="215" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="B68" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C68" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="D68" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E68" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="215" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="B69" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="C69" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D69" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E69" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="215" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="B70" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C70" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D70" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E70" t="s">
-        <v>702</v>
+        <v>706</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A71" s="215" t="s">
+        <v>707</v>
+      </c>
+      <c r="B71" t="s">
+        <v>558</v>
+      </c>
+      <c r="C71" t="s">
+        <v>563</v>
+      </c>
+      <c r="D71" t="s">
+        <v>560</v>
+      </c>
+      <c r="E71" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A72" s="215" t="s">
+        <v>709</v>
+      </c>
+      <c r="B72" t="s">
+        <v>572</v>
+      </c>
+      <c r="C72" t="s">
+        <v>571</v>
+      </c>
+      <c r="D72" t="s">
+        <v>603</v>
+      </c>
+      <c r="E72" t="s">
+        <v>710</v>
       </c>
     </row>
   </sheetData>
@@ -15010,12 +15128,12 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="219" t="s">
-        <v>703</v>
+        <v>711</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="303" t="s">
-        <v>704</v>
+        <v>712</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -15024,1032 +15142,1032 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="220" t="s">
-        <v>705</v>
+        <v>713</v>
       </c>
       <c r="B4" s="220" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="C4" s="220" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="220" t="s">
-        <v>706</v>
+        <v>714</v>
       </c>
       <c r="E4" s="220" t="s">
-        <v>707</v>
+        <v>715</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="221" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="C5" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>711</v>
+        <v>719</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="221" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>712</v>
+        <v>720</v>
       </c>
       <c r="C6" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="215" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="E6" s="215" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="231" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>715</v>
+        <v>723</v>
       </c>
       <c r="C7" s="232" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="215" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
       <c r="E7" s="215" t="s">
-        <v>716</v>
+        <v>724</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="223" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>717</v>
+        <v>725</v>
       </c>
       <c r="C8" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>718</v>
+        <v>726</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>719</v>
+        <v>727</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="223" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="B9" s="215" t="s">
-        <v>720</v>
+        <v>728</v>
       </c>
       <c r="C9" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="215" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
       <c r="E9" s="215" t="s">
-        <v>721</v>
+        <v>729</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="224" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>723</v>
+        <v>731</v>
       </c>
       <c r="C10" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>724</v>
+        <v>732</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>725</v>
+        <v>733</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>726</v>
+        <v>734</v>
       </c>
       <c r="C11" t="s">
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>728</v>
+        <v>736</v>
       </c>
       <c r="C12" t="s">
         <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="224" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>729</v>
+        <v>737</v>
       </c>
       <c r="C13" s="222" t="s">
         <v>128</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>730</v>
+        <v>738</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>731</v>
+        <v>739</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="235" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>732</v>
+        <v>740</v>
       </c>
       <c r="C14" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>733</v>
+        <v>741</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>734</v>
+        <v>742</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="235" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B15" s="215" t="s">
-        <v>735</v>
+        <v>743</v>
       </c>
       <c r="C15" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="215" t="s">
-        <v>730</v>
+        <v>738</v>
       </c>
       <c r="E15" s="215" t="s">
-        <v>736</v>
+        <v>744</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="235" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B16" s="215" t="s">
-        <v>737</v>
+        <v>745</v>
       </c>
       <c r="C16" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="215" t="s">
-        <v>730</v>
+        <v>738</v>
       </c>
       <c r="E16" s="215" t="s">
-        <v>738</v>
+        <v>746</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="225" t="s">
-        <v>739</v>
+        <v>747</v>
       </c>
       <c r="B17" s="215" t="s">
-        <v>740</v>
+        <v>748</v>
       </c>
       <c r="C17" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D17" s="215" t="s">
-        <v>741</v>
+        <v>749</v>
       </c>
       <c r="E17" s="215" t="s">
-        <v>742</v>
+        <v>750</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="225" t="s">
-        <v>739</v>
+        <v>747</v>
       </c>
       <c r="B18" s="215" t="s">
-        <v>743</v>
+        <v>751</v>
       </c>
       <c r="C18" s="223" t="s">
         <v>138</v>
       </c>
       <c r="D18" s="215" t="s">
-        <v>741</v>
+        <v>749</v>
       </c>
       <c r="E18" s="215" t="s">
-        <v>744</v>
+        <v>752</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="226" t="s">
-        <v>745</v>
+        <v>753</v>
       </c>
       <c r="B19" s="215" t="s">
-        <v>746</v>
+        <v>754</v>
       </c>
       <c r="C19" s="225" t="s">
-        <v>747</v>
+        <v>755</v>
       </c>
       <c r="D19" s="215" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="E19" s="215" t="s">
-        <v>748</v>
+        <v>756</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="226" t="s">
-        <v>745</v>
+        <v>753</v>
       </c>
       <c r="B20" s="215" t="s">
-        <v>749</v>
+        <v>757</v>
       </c>
       <c r="C20" s="225" t="s">
-        <v>747</v>
+        <v>755</v>
       </c>
       <c r="D20" s="215" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="E20" s="215" t="s">
-        <v>750</v>
+        <v>758</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="226" t="s">
-        <v>745</v>
+        <v>753</v>
       </c>
       <c r="B21" s="215" t="s">
-        <v>751</v>
+        <v>759</v>
       </c>
       <c r="C21" s="225" t="s">
-        <v>747</v>
+        <v>755</v>
       </c>
       <c r="D21" s="215" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="E21" s="215" t="s">
-        <v>752</v>
+        <v>760</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
     <row r="23" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="229" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
       <c r="B23" s="215" t="s">
-        <v>753</v>
+        <v>761</v>
       </c>
       <c r="C23" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D23" s="215" t="s">
-        <v>754</v>
+        <v>762</v>
       </c>
       <c r="E23" s="215" t="s">
-        <v>755</v>
+        <v>763</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="230" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="B24" s="215" t="s">
-        <v>756</v>
+        <v>764</v>
       </c>
       <c r="C24" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D24" s="215" t="s">
-        <v>757</v>
+        <v>765</v>
       </c>
       <c r="E24" s="215" t="s">
-        <v>758</v>
+        <v>766</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="231" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="B25" s="215" t="s">
-        <v>759</v>
+        <v>767</v>
       </c>
       <c r="C25" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D25" s="215" t="s">
-        <v>760</v>
+        <v>768</v>
       </c>
       <c r="E25" s="215" t="s">
-        <v>761</v>
+        <v>769</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="231" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="B26" s="215" t="s">
-        <v>762</v>
+        <v>770</v>
       </c>
       <c r="C26" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D26" s="215" t="s">
-        <v>757</v>
+        <v>765</v>
       </c>
       <c r="E26" s="215" t="s">
-        <v>763</v>
+        <v>771</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="235" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B27" s="215" t="s">
-        <v>764</v>
+        <v>772</v>
       </c>
       <c r="C27" s="237" t="s">
         <v>22</v>
       </c>
       <c r="D27" s="215" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
       <c r="E27" s="215" t="s">
-        <v>765</v>
+        <v>773</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="227" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
       <c r="B28" s="215" t="s">
-        <v>766</v>
+        <v>774</v>
       </c>
       <c r="C28" t="s">
         <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>767</v>
+        <v>775</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B29" s="215" t="s">
-        <v>768</v>
+        <v>776</v>
       </c>
       <c r="C29" t="s">
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B30" s="215" t="s">
-        <v>769</v>
+        <v>777</v>
       </c>
       <c r="C30" t="s">
         <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>770</v>
+        <v>778</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="B31" s="215" t="s">
-        <v>771</v>
+        <v>779</v>
       </c>
       <c r="C31" t="s">
         <v>22</v>
       </c>
       <c r="D31" t="s">
-        <v>772</v>
+        <v>780</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="B32" s="215" t="s">
-        <v>773</v>
+        <v>781</v>
       </c>
       <c r="C32" t="s">
         <v>22</v>
       </c>
       <c r="D32" t="s">
-        <v>774</v>
+        <v>782</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="B33" s="215" t="s">
-        <v>775</v>
+        <v>783</v>
       </c>
       <c r="C33" t="s">
         <v>22</v>
       </c>
       <c r="D33" t="s">
-        <v>772</v>
+        <v>780</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="B34" s="215" t="s">
-        <v>776</v>
+        <v>784</v>
       </c>
       <c r="C34" t="s">
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>777</v>
+        <v>785</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B35" s="215" t="s">
-        <v>778</v>
+        <v>786</v>
       </c>
       <c r="C35" t="s">
         <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>779</v>
+        <v>787</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="B36" s="215" t="s">
-        <v>780</v>
+        <v>788</v>
       </c>
       <c r="C36" t="s">
         <v>22</v>
       </c>
       <c r="D36" t="s">
-        <v>781</v>
+        <v>789</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B37" s="215" t="s">
-        <v>782</v>
+        <v>790</v>
       </c>
       <c r="C37" t="s">
         <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>781</v>
+        <v>789</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
-        <v>739</v>
+        <v>747</v>
       </c>
       <c r="B38" s="215" t="s">
-        <v>783</v>
+        <v>791</v>
       </c>
       <c r="C38" t="s">
         <v>22</v>
       </c>
       <c r="D38" t="s">
-        <v>781</v>
+        <v>789</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="B39" s="215" t="s">
-        <v>784</v>
+        <v>792</v>
       </c>
       <c r="C39" t="s">
         <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>781</v>
+        <v>789</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B40" s="215" t="s">
-        <v>785</v>
+        <v>793</v>
       </c>
       <c r="C40" t="s">
         <v>22</v>
       </c>
       <c r="D40" t="s">
-        <v>781</v>
+        <v>789</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="B41" s="215" t="s">
-        <v>786</v>
+        <v>794</v>
       </c>
       <c r="C41" t="s">
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B42" s="215" t="s">
-        <v>788</v>
+        <v>796</v>
       </c>
       <c r="C42" t="s">
         <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B43" s="215" t="s">
-        <v>789</v>
+        <v>797</v>
       </c>
       <c r="C43" t="s">
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>790</v>
+        <v>798</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B44" s="215" t="s">
-        <v>791</v>
+        <v>799</v>
       </c>
       <c r="C44" t="s">
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>790</v>
+        <v>798</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
-        <v>739</v>
+        <v>747</v>
       </c>
       <c r="B45" s="215" t="s">
-        <v>792</v>
+        <v>800</v>
       </c>
       <c r="C45" t="s">
         <v>128</v>
       </c>
       <c r="D45" t="s">
-        <v>793</v>
+        <v>801</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B46" s="215" t="s">
-        <v>795</v>
+        <v>803</v>
       </c>
       <c r="C46" t="s">
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>796</v>
+        <v>804</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B47" s="215" t="s">
-        <v>797</v>
+        <v>805</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>798</v>
+        <v>806</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B48" s="215" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="C48" t="s">
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>798</v>
+        <v>806</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B49" s="215" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
       <c r="C49" t="s">
         <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>798</v>
+        <v>806</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B50" s="215" t="s">
-        <v>801</v>
+        <v>809</v>
       </c>
       <c r="C50" t="s">
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>802</v>
+        <v>810</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B51" s="215" t="s">
-        <v>803</v>
+        <v>811</v>
       </c>
       <c r="C51" t="s">
         <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>804</v>
+        <v>812</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B52" s="215" t="s">
-        <v>805</v>
+        <v>813</v>
       </c>
       <c r="C52" t="s">
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>806</v>
+        <v>814</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B53" s="215" t="s">
-        <v>807</v>
+        <v>815</v>
       </c>
       <c r="C53" t="s">
         <v>128</v>
       </c>
       <c r="D53" t="s">
-        <v>804</v>
+        <v>812</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>808</v>
+        <v>816</v>
       </c>
       <c r="C54" t="s">
         <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>806</v>
+        <v>814</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>809</v>
+        <v>817</v>
       </c>
       <c r="C55" t="s">
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>810</v>
+        <v>818</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>811</v>
+        <v>819</v>
       </c>
       <c r="C56" t="s">
         <v>128</v>
       </c>
       <c r="D56" t="s">
-        <v>812</v>
+        <v>820</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>813</v>
+        <v>821</v>
       </c>
       <c r="C57" t="s">
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>814</v>
+        <v>822</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>815</v>
+        <v>823</v>
       </c>
       <c r="C58" t="s">
         <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>814</v>
+        <v>822</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>816</v>
+        <v>824</v>
       </c>
       <c r="C59" t="s">
         <v>22</v>
       </c>
       <c r="D59" t="s">
-        <v>814</v>
+        <v>822</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>817</v>
+        <v>825</v>
       </c>
       <c r="C60" t="s">
         <v>128</v>
       </c>
       <c r="D60" t="s">
-        <v>814</v>
+        <v>822</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="274" t="s">
-        <v>818</v>
+        <v>826</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>819</v>
+        <v>827</v>
       </c>
       <c r="C61" t="s">
         <v>22</v>
       </c>
       <c r="D61" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="274" t="s">
-        <v>818</v>
+        <v>826</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>820</v>
+        <v>828</v>
       </c>
       <c r="C62" t="s">
         <v>22</v>
       </c>
       <c r="D62" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="274" t="s">
-        <v>818</v>
+        <v>826</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>821</v>
+        <v>829</v>
       </c>
       <c r="C63" t="s">
         <v>22</v>
       </c>
       <c r="D63" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>822</v>
+        <v>830</v>
       </c>
       <c r="C64" t="s">
         <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>823</v>
+        <v>831</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>824</v>
+        <v>832</v>
       </c>
       <c r="C65" t="s">
         <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>823</v>
+        <v>831</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B66" s="215" t="s">
-        <v>825</v>
+        <v>833</v>
       </c>
       <c r="C66" t="s">
         <v>22</v>
       </c>
       <c r="D66" t="s">
-        <v>823</v>
+        <v>831</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="274" t="s">
-        <v>826</v>
+        <v>834</v>
       </c>
       <c r="B67" s="215" t="s">
-        <v>827</v>
+        <v>835</v>
       </c>
       <c r="C67" t="s">
         <v>22</v>
       </c>
       <c r="D67" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="274" t="s">
-        <v>826</v>
+        <v>834</v>
       </c>
       <c r="B68" s="215" t="s">
-        <v>828</v>
+        <v>836</v>
       </c>
       <c r="C68" t="s">
         <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="274" t="s">
-        <v>826</v>
+        <v>834</v>
       </c>
       <c r="B69" s="215" t="s">
-        <v>829</v>
+        <v>837</v>
       </c>
       <c r="C69" t="s">
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B70" s="215" t="s">
-        <v>830</v>
+        <v>838</v>
       </c>
       <c r="C70" t="s">
         <v>22</v>
       </c>
       <c r="D70" t="s">
-        <v>831</v>
+        <v>839</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B71" s="215" t="s">
-        <v>832</v>
+        <v>840</v>
       </c>
       <c r="C71" t="s">
         <v>22</v>
       </c>
       <c r="D71" t="s">
-        <v>831</v>
+        <v>839</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B72" s="215" t="s">
-        <v>833</v>
+        <v>841</v>
       </c>
       <c r="C72" t="s">
         <v>22</v>
       </c>
       <c r="D72" t="s">
-        <v>831</v>
+        <v>839</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="274" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="B73" s="215" t="s">
-        <v>834</v>
+        <v>842</v>
       </c>
       <c r="C73" t="s">
         <v>128</v>
       </c>
       <c r="D73" t="s">
-        <v>831</v>
+        <v>839</v>
       </c>
     </row>
   </sheetData>
@@ -16078,336 +16196,336 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="211" t="s">
-        <v>835</v>
+        <v>843</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="212" t="s">
-        <v>836</v>
+        <v>844</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="213" t="s">
-        <v>837</v>
+        <v>845</v>
       </c>
       <c r="B4" s="213" t="s">
-        <v>838</v>
+        <v>846</v>
       </c>
       <c r="C4" s="213" t="s">
-        <v>839</v>
+        <v>847</v>
       </c>
       <c r="D4" s="213" t="s">
-        <v>840</v>
+        <v>848</v>
       </c>
       <c r="E4" s="213" t="s">
-        <v>841</v>
+        <v>849</v>
       </c>
       <c r="F4" s="213" t="s">
-        <v>842</v>
+        <v>850</v>
       </c>
       <c r="G4" s="213" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="H4" s="213" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="213" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="214" t="s">
-        <v>845</v>
+        <v>853</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>846</v>
+        <v>854</v>
       </c>
       <c r="C5" s="215" t="s">
-        <v>847</v>
+        <v>855</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>848</v>
+        <v>856</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>849</v>
+        <v>857</v>
       </c>
       <c r="F5" s="215" t="s">
-        <v>850</v>
+        <v>858</v>
       </c>
       <c r="G5" s="215" t="s">
-        <v>851</v>
+        <v>859</v>
       </c>
       <c r="H5" s="216" t="s">
-        <v>852</v>
+        <v>860</v>
       </c>
       <c r="I5" s="215" t="s">
-        <v>853</v>
+        <v>861</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="214" t="s">
-        <v>854</v>
+        <v>862</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>855</v>
+        <v>863</v>
       </c>
       <c r="C6" s="215" t="s">
-        <v>856</v>
+        <v>864</v>
       </c>
       <c r="D6" s="215" t="s">
-        <v>857</v>
+        <v>865</v>
       </c>
       <c r="E6" s="215" t="s">
-        <v>858</v>
+        <v>866</v>
       </c>
       <c r="F6" s="215" t="s">
-        <v>859</v>
+        <v>867</v>
       </c>
       <c r="G6" s="215" t="s">
+        <v>868</v>
+      </c>
+      <c r="H6" s="217" t="s">
         <v>860</v>
       </c>
-      <c r="H6" s="217" t="s">
-        <v>852</v>
-      </c>
       <c r="I6" s="215" t="s">
-        <v>861</v>
+        <v>869</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="214" t="s">
-        <v>862</v>
+        <v>870</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>863</v>
+        <v>871</v>
       </c>
       <c r="C7" s="215" t="s">
-        <v>864</v>
+        <v>872</v>
       </c>
       <c r="D7" s="215" t="s">
-        <v>865</v>
+        <v>873</v>
       </c>
       <c r="E7" s="215" t="s">
-        <v>866</v>
+        <v>874</v>
       </c>
       <c r="F7" s="215" t="s">
-        <v>867</v>
+        <v>875</v>
       </c>
       <c r="G7" s="215" t="s">
-        <v>868</v>
+        <v>876</v>
       </c>
       <c r="H7" s="217" t="s">
-        <v>852</v>
+        <v>860</v>
       </c>
       <c r="I7" s="215" t="s">
-        <v>869</v>
+        <v>877</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="214" t="s">
-        <v>870</v>
+        <v>878</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>871</v>
+        <v>879</v>
       </c>
       <c r="C8" s="215" t="s">
-        <v>872</v>
+        <v>880</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>873</v>
+        <v>881</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="F8" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="G8" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="H8" s="216" t="s">
-        <v>874</v>
+        <v>882</v>
       </c>
       <c r="I8" s="215" t="s">
-        <v>875</v>
+        <v>883</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="214" t="s">
-        <v>876</v>
+        <v>884</v>
       </c>
       <c r="B9" s="215" t="s">
-        <v>877</v>
+        <v>885</v>
       </c>
       <c r="C9" s="215" t="s">
-        <v>878</v>
+        <v>886</v>
       </c>
       <c r="D9" s="215" t="s">
-        <v>873</v>
+        <v>881</v>
       </c>
       <c r="E9" s="215" t="s">
-        <v>866</v>
+        <v>874</v>
       </c>
       <c r="F9" s="215" t="s">
-        <v>879</v>
+        <v>887</v>
       </c>
       <c r="G9" s="215" t="s">
-        <v>880</v>
+        <v>888</v>
       </c>
       <c r="H9" s="218" t="s">
-        <v>881</v>
+        <v>889</v>
       </c>
       <c r="I9" s="215" t="s">
-        <v>882</v>
+        <v>890</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="214" t="s">
-        <v>883</v>
+        <v>891</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>884</v>
+        <v>892</v>
       </c>
       <c r="C10" s="215" t="s">
-        <v>885</v>
+        <v>893</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>886</v>
+        <v>894</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>887</v>
+        <v>895</v>
       </c>
       <c r="F10" s="215" t="s">
-        <v>888</v>
+        <v>896</v>
       </c>
       <c r="G10" s="215" t="s">
-        <v>889</v>
+        <v>897</v>
       </c>
       <c r="H10" s="218" t="s">
-        <v>890</v>
+        <v>898</v>
       </c>
       <c r="I10" s="215" t="s">
-        <v>891</v>
+        <v>899</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="214" t="s">
-        <v>892</v>
+        <v>900</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>893</v>
+        <v>901</v>
       </c>
       <c r="C11" s="215" t="s">
-        <v>894</v>
+        <v>902</v>
       </c>
       <c r="D11" s="215" t="s">
-        <v>895</v>
+        <v>903</v>
       </c>
       <c r="E11" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="F11" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="G11" s="215" t="s">
-        <v>896</v>
+        <v>904</v>
       </c>
       <c r="H11" s="218" t="s">
-        <v>897</v>
+        <v>905</v>
       </c>
       <c r="I11" s="215" t="s">
-        <v>898</v>
+        <v>906</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="214" t="s">
-        <v>899</v>
+        <v>907</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>900</v>
+        <v>908</v>
       </c>
       <c r="C12" s="215" t="s">
-        <v>901</v>
+        <v>909</v>
       </c>
       <c r="D12" s="215" t="s">
-        <v>902</v>
+        <v>910</v>
       </c>
       <c r="E12" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="F12" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="G12" s="215" t="s">
-        <v>896</v>
+        <v>904</v>
       </c>
       <c r="H12" s="217" t="s">
-        <v>903</v>
+        <v>911</v>
       </c>
       <c r="I12" s="215" t="s">
-        <v>904</v>
+        <v>912</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="214" t="s">
-        <v>905</v>
+        <v>913</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>906</v>
+        <v>914</v>
       </c>
       <c r="C13" s="215" t="s">
-        <v>907</v>
+        <v>915</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="F13" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="G13" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="H13" s="218" t="s">
-        <v>908</v>
+        <v>916</v>
       </c>
       <c r="I13" s="215" t="s">
-        <v>909</v>
+        <v>917</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="214" t="s">
-        <v>910</v>
+        <v>918</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>911</v>
+        <v>919</v>
       </c>
       <c r="C14" s="215" t="s">
-        <v>907</v>
+        <v>915</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="F14" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="G14" s="215" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="H14" s="218" t="s">
-        <v>908</v>
+        <v>916</v>
       </c>
       <c r="I14" s="215" t="s">
-        <v>912</v>
+        <v>920</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="304" t="s">
-        <v>913</v>
+        <v>921</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>

</xml_diff>

<commit_message>
docs(tracker): tennis gate removal, ranking baseline, surface whitespace fix
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E69EB30D-D30E-4A13-BB0E-B94633F4A487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28DBCC59-6373-4F91-8C16-19FC7253A05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1926" uniqueCount="922">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1954" uniqueCount="932">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -1457,6 +1457,24 @@
   </si>
   <si>
     <t>Found by the notebook. run_predictions appends rather than replaces; 143 settled football rows sat on 63 fixtures (one had 25), overstating accuracy by 18.7pp (0.5524-&gt;0.3651). Now one row per fixture/kind - the last created BEFORE kickoff. Football now reads below its own baseline, which is the honest number</t>
+  </si>
+  <si>
+    <t>Tennis base-rate gate removed (was inverting 25% of picks)</t>
+  </si>
+  <si>
+    <t>'Home' in tennis is the lower-player-id tiebreak, not a venue. The 0.6217 rate encoded 'the stronger player usually wins' (lower id = higher ranked 69% of the time), which rank_diff already prices in, and asymmetric bars 0.672/0.428 meant the away slot nearly always cleared. 167 of 669 picks recommended the side the model rated lower. Live 0 of 21 inverted, from 4 of 4</t>
+  </si>
+  <si>
+    <t>Ranking baseline reported per surface, gate pre-registered</t>
+  </si>
+  <si>
+    <t>train_tennis.py scores the model against 'back the higher-ranked player' - the strategy a user could actually run - pooled and per surface. +2.15pp pooled (Clay +2.51, Grass +5.24, Hard +1.25), below the pre-registered 3pp bar and concentrated on the smallest stratum, so no gate. Seeds pinned so the threshold is evaluable</t>
+  </si>
+  <si>
+    <t>Tennis surface whitespace bug ('Grass' vs 'Grass ')</t>
+  </si>
+  <si>
+    <t>4,296 vs 386 rows as separate categories. Not cosmetic - surface_win_rate, surface_streak and h2h_win_rate_surface all match on this string, so 8% of grass matches were compared against the wrong pool. Stripped at collection and on load</t>
   </si>
   <si>
     <t>Legend</t>
@@ -2243,6 +2261,18 @@
   </si>
   <si>
     <t>They were checked for the failure mode that had bitten before (MultipleResultsFound via scalar_one) and cleared on that basis, while the defect actually present was silent inflation of a live user-facing accuracy. Checking for the last bug is not the same as checking for a bug.</t>
+  </si>
+  <si>
+    <t>Tennis edge over a runnable baseline is 2.15pp</t>
+  </si>
+  <si>
+    <t>Against 'back the higher-ranked player' the model gains +2.15pp (n=3,900), below the 3pp bar pre-registered for reinstating a pick gate. The edge also sits on grass (+5.24pp, n=477, the smallest stratum) rather than clay where ranking is least reliable - the opposite of the stated hypothesis - and the per-surface figures move between runs that differ only by seed. Watch as data accumulates; do not act on the surface split yet.</t>
+  </si>
+  <si>
+    <t>Base rates must describe something a user could do</t>
+  </si>
+  <si>
+    <t>A base rate is the no-model alternative. Football's 'back the home team' qualifies; tennis's 'back the lower player id' does not - it is invisible to the user and is a proxy for strength the model already uses. Gating on it inverted a quarter of picks. Any future sport-specific base rate must name the strategy it represents and that strategy must be executable by someone without our database.</t>
   </si>
   <si>
     <t>SportIQ — Edge Measurement Plan (P0-P3)</t>
@@ -5225,7 +5255,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R220"/>
+  <dimension ref="A1:R223"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -11973,7 +12003,7 @@
         <v>432</v>
       </c>
       <c r="R198" t="str">
-        <f t="shared" ref="R198:R218" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
+        <f t="shared" ref="R198:R221" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
         <v>E4 ML Football</v>
       </c>
     </row>
@@ -12511,7 +12541,7 @@
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="217" spans="1:18" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="217" spans="1:18" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A217" t="s">
         <v>99</v>
       </c>
@@ -12541,7 +12571,7 @@
         <v>E8 Model Quality</v>
       </c>
     </row>
-    <row r="218" spans="1:18" ht="72" x14ac:dyDescent="0.55000000000000004">
+    <row r="218" spans="1:18" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A218" t="s">
         <v>99</v>
       </c>
@@ -12571,23 +12601,113 @@
         <v>E8 Model Quality</v>
       </c>
     </row>
-    <row r="220" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A220" s="23" t="s">
+    <row r="219" spans="1:18" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A219" t="s">
+        <v>73</v>
+      </c>
+      <c r="B219" t="s">
         <v>473</v>
       </c>
-      <c r="B220" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C220" s="15" t="s">
+      <c r="C219" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D219" t="s">
+        <v>75</v>
+      </c>
+      <c r="E219" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F219" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G219" s="215" t="s">
         <v>474</v>
       </c>
-      <c r="D220" s="17" t="s">
+      <c r="J219" t="s">
+        <v>400</v>
+      </c>
+      <c r="R219" t="str">
+        <f t="shared" si="3"/>
+        <v>E6 Picks</v>
+      </c>
+    </row>
+    <row r="220" spans="1:18" ht="72" x14ac:dyDescent="0.55000000000000004">
+      <c r="A220" t="s">
+        <v>99</v>
+      </c>
+      <c r="B220" t="s">
+        <v>475</v>
+      </c>
+      <c r="C220" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D220" t="s">
+        <v>45</v>
+      </c>
+      <c r="E220" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F220" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G220" s="215" t="s">
+        <v>476</v>
+      </c>
+      <c r="J220" t="s">
+        <v>400</v>
+      </c>
+      <c r="R220" t="str">
+        <f t="shared" si="3"/>
+        <v>E8 Model Quality</v>
+      </c>
+    </row>
+    <row r="221" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A221" t="s">
+        <v>130</v>
+      </c>
+      <c r="B221" t="s">
+        <v>477</v>
+      </c>
+      <c r="C221" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D221" t="s">
+        <v>45</v>
+      </c>
+      <c r="E221" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F221" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G221" s="215" t="s">
+        <v>478</v>
+      </c>
+      <c r="J221" t="s">
+        <v>400</v>
+      </c>
+      <c r="R221" t="str">
+        <f t="shared" si="3"/>
+        <v>E9 Data Ops</v>
+      </c>
+    </row>
+    <row r="223" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A223" s="23" t="s">
+        <v>479</v>
+      </c>
+      <c r="B223" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C223" s="15" t="s">
+        <v>480</v>
+      </c>
+      <c r="D223" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="E220" s="21" t="s">
+      <c r="E223" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="F220" s="19" t="s">
+      <c r="F223" s="19" t="s">
         <v>138</v>
       </c>
     </row>
@@ -12612,7 +12732,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="294" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="B1" s="283"/>
       <c r="C1" s="283"/>
@@ -12635,7 +12755,7 @@
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="301" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -12658,7 +12778,7 @@
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="289" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="B4" s="283"/>
       <c r="C4" s="283"/>
@@ -12681,42 +12801,42 @@
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="35" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
       <c r="B5" s="279" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
       <c r="C5" s="280"/>
       <c r="D5" s="281"/>
       <c r="E5" s="284" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="F5" s="280"/>
       <c r="G5" s="281"/>
       <c r="H5" s="284" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
       <c r="I5" s="280"/>
       <c r="J5" s="281"/>
       <c r="K5" s="279" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
       <c r="L5" s="280"/>
       <c r="M5" s="281"/>
       <c r="N5" s="286" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
       <c r="O5" s="280"/>
       <c r="P5" s="281"/>
       <c r="Q5" s="286" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
       <c r="R5" s="280"/>
       <c r="S5" s="281"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="282" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="C6" s="283"/>
       <c r="D6" s="283"/>
@@ -12738,7 +12858,7 @@
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="289" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="B7" s="283"/>
       <c r="C7" s="283"/>
@@ -12761,10 +12881,10 @@
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="35" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="B8" s="292" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
       <c r="C8" s="280"/>
       <c r="D8" s="280"/>
@@ -12775,7 +12895,7 @@
       <c r="I8" s="280"/>
       <c r="J8" s="281"/>
       <c r="K8" s="292" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
       <c r="L8" s="280"/>
       <c r="M8" s="280"/>
@@ -12788,7 +12908,7 @@
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="282" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="C9" s="283"/>
       <c r="D9" s="283"/>
@@ -12810,7 +12930,7 @@
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="289" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
       <c r="B10" s="283"/>
       <c r="C10" s="283"/>
@@ -12833,42 +12953,42 @@
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="35" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
       <c r="B11" s="279" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="C11" s="280"/>
       <c r="D11" s="281"/>
       <c r="E11" s="279" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="F11" s="280"/>
       <c r="G11" s="281"/>
       <c r="H11" s="279" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="I11" s="280"/>
       <c r="J11" s="281"/>
       <c r="K11" s="284" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="L11" s="280"/>
       <c r="M11" s="281"/>
       <c r="N11" s="279" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
       <c r="O11" s="280"/>
       <c r="P11" s="281"/>
       <c r="Q11" s="279" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="R11" s="280"/>
       <c r="S11" s="281"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="282" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="C12" s="283"/>
       <c r="D12" s="283"/>
@@ -12890,7 +13010,7 @@
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="289" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
       <c r="B13" s="283"/>
       <c r="C13" s="283"/>
@@ -12913,10 +13033,10 @@
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="35" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="B14" s="287" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
       <c r="C14" s="280"/>
       <c r="D14" s="280"/>
@@ -12924,7 +13044,7 @@
       <c r="F14" s="280"/>
       <c r="G14" s="281"/>
       <c r="H14" s="287" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="I14" s="280"/>
       <c r="J14" s="280"/>
@@ -12932,19 +13052,19 @@
       <c r="L14" s="280"/>
       <c r="M14" s="281"/>
       <c r="N14" s="287" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="O14" s="280"/>
       <c r="P14" s="281"/>
       <c r="Q14" s="284" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="R14" s="280"/>
       <c r="S14" s="281"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" s="282" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="C15" s="283"/>
       <c r="D15" s="283"/>
@@ -12966,7 +13086,7 @@
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="289" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>
@@ -12989,10 +13109,10 @@
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="35" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="B17" s="288" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C17" s="280"/>
       <c r="D17" s="280"/>
@@ -13000,29 +13120,29 @@
       <c r="F17" s="280"/>
       <c r="G17" s="281"/>
       <c r="H17" s="288" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="I17" s="280"/>
       <c r="J17" s="281"/>
       <c r="K17" s="288" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="L17" s="280"/>
       <c r="M17" s="281"/>
       <c r="N17" s="288" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="O17" s="280"/>
       <c r="P17" s="281"/>
       <c r="Q17" s="288" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="R17" s="280"/>
       <c r="S17" s="281"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="282" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="C18" s="283"/>
       <c r="D18" s="283"/>
@@ -13044,7 +13164,7 @@
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="289" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="B19" s="283"/>
       <c r="C19" s="283"/>
@@ -13067,10 +13187,10 @@
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="35" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
       <c r="B20" s="290" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="C20" s="280"/>
       <c r="D20" s="280"/>
@@ -13078,7 +13198,7 @@
       <c r="F20" s="280"/>
       <c r="G20" s="281"/>
       <c r="H20" s="290" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="I20" s="280"/>
       <c r="J20" s="280"/>
@@ -13086,7 +13206,7 @@
       <c r="L20" s="280"/>
       <c r="M20" s="281"/>
       <c r="N20" s="290" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="O20" s="280"/>
       <c r="P20" s="280"/>
@@ -13096,7 +13216,7 @@
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" s="282" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="C21" s="283"/>
       <c r="D21" s="283"/>
@@ -13118,7 +13238,7 @@
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="289" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="B22" s="283"/>
       <c r="C22" s="283"/>
@@ -13141,10 +13261,10 @@
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="35" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="B23" s="290" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="C23" s="280"/>
       <c r="D23" s="280"/>
@@ -13152,29 +13272,29 @@
       <c r="F23" s="280"/>
       <c r="G23" s="281"/>
       <c r="H23" s="290" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="I23" s="280"/>
       <c r="J23" s="281"/>
       <c r="K23" s="290" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="L23" s="280"/>
       <c r="M23" s="281"/>
       <c r="N23" s="290" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
       <c r="O23" s="280"/>
       <c r="P23" s="281"/>
       <c r="Q23" s="286" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="R23" s="280"/>
       <c r="S23" s="281"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="295" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="B26" s="283"/>
       <c r="C26" s="283"/>
@@ -13197,42 +13317,42 @@
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="35" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="B27" s="279" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C27" s="280"/>
       <c r="D27" s="281"/>
       <c r="E27" s="279" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="F27" s="280"/>
       <c r="G27" s="281"/>
       <c r="H27" s="287" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="I27" s="280"/>
       <c r="J27" s="281"/>
       <c r="K27" s="288" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="L27" s="280"/>
       <c r="M27" s="281"/>
       <c r="N27" s="288" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="O27" s="280"/>
       <c r="P27" s="281"/>
       <c r="Q27" s="287" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="R27" s="280"/>
       <c r="S27" s="281"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="289" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="B30" s="283"/>
       <c r="C30" s="283"/>
@@ -13255,7 +13375,7 @@
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="285" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
       <c r="B31" s="283"/>
       <c r="C31" s="283"/>
@@ -13278,7 +13398,7 @@
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="285" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="B32" s="283"/>
       <c r="C32" s="283"/>
@@ -13301,7 +13421,7 @@
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="285" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="B33" s="283"/>
       <c r="C33" s="283"/>
@@ -13324,7 +13444,7 @@
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="285" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="B34" s="283"/>
       <c r="C34" s="283"/>
@@ -13347,7 +13467,7 @@
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="285" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
       <c r="B35" s="283"/>
       <c r="C35" s="283"/>
@@ -13370,7 +13490,7 @@
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="285" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="B36" s="283"/>
       <c r="C36" s="283"/>
@@ -13393,7 +13513,7 @@
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="296" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="B37" s="283"/>
       <c r="C37" s="283"/>
@@ -13416,25 +13536,25 @@
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="36" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
       <c r="B39" s="299" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="C39" s="283"/>
       <c r="D39" s="283"/>
       <c r="E39" s="297" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="F39" s="283"/>
       <c r="G39" s="283"/>
       <c r="H39" s="300" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="I39" s="283"/>
       <c r="J39" s="283"/>
       <c r="K39" s="293" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="L39" s="283"/>
       <c r="M39" s="283"/>
@@ -13444,7 +13564,7 @@
       <c r="O39" s="283"/>
       <c r="P39" s="283"/>
       <c r="Q39" s="298" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="R39" s="283"/>
       <c r="S39" s="283"/>
@@ -13452,11 +13572,11 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H14:M14"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A16:S16"/>
     <mergeCell ref="H20:M20"/>
-    <mergeCell ref="A16:S16"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -13465,13 +13585,14 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -13480,7 +13601,6 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
-    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -13488,7 +13608,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -13537,7 +13657,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -13550,19 +13670,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -13696,11 +13816,11 @@
       </c>
       <c r="B9" s="24">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D9" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -13712,7 +13832,7 @@
       </c>
       <c r="F9" s="25">
         <f t="shared" si="1"/>
-        <v>0.875</v>
+        <v>0.88888888888888884</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -13746,11 +13866,11 @@
       </c>
       <c r="B11" s="24">
         <f t="shared" si="0"/>
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C11" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D11" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -13762,7 +13882,7 @@
       </c>
       <c r="F11" s="25">
         <f t="shared" si="1"/>
-        <v>0.82978723404255317</v>
+        <v>0.83333333333333337</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -13771,11 +13891,11 @@
       </c>
       <c r="B12" s="24">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C12" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D12" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -13787,7 +13907,7 @@
       </c>
       <c r="F12" s="25">
         <f t="shared" si="1"/>
-        <v>0.61538461538461542</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -13842,15 +13962,15 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="26" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="B16" s="27">
         <f>SUM(B4:B14)</f>
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C16" s="27">
         <f>SUM(C4:C14)</f>
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
@@ -13862,12 +13982,12 @@
       </c>
       <c r="F16" s="28">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.78504672897196259</v>
+        <v>0.78801843317972353</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="41" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="B18" s="42">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -13876,7 +13996,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="43" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
     </row>
   </sheetData>
@@ -13897,7 +14017,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -13909,7 +14029,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -13918,648 +14038,648 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="29" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="D3" s="29" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="29" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="30" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="32" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="30" t="s">
+        <v>571</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>572</v>
+      </c>
+      <c r="C6" s="21" t="s">
         <v>565</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>566</v>
-      </c>
-      <c r="C6" s="21" t="s">
-        <v>559</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="32" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="30" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="32" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="30" t="s">
+        <v>583</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>584</v>
+      </c>
+      <c r="C10" s="17" t="s">
         <v>577</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>578</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>571</v>
-      </c>
       <c r="D10" s="11" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="32" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="30" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="32" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="30" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="32" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="30" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="32" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="30" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="32" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="30" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="32" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E21" s="33" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="30" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="32" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="30" t="s">
-        <v>612</v>
+        <v>618</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E24" s="31" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="53" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="B25" s="51" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C25" s="54" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E25" s="55" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="56" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
       <c r="B26" s="46" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="C26" s="54" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="D26" s="46" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E26" s="57" t="s">
-        <v>617</v>
+        <v>623</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="53" t="s">
-        <v>618</v>
+        <v>624</v>
       </c>
       <c r="B27" s="51" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C27" s="54" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="D27" s="51" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E27" s="55" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="71" t="s">
-        <v>620</v>
+        <v>626</v>
       </c>
       <c r="B28" s="60" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C28" s="67" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D28" s="94" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E28" s="94" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="72" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
       <c r="B29" s="65" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C29" s="69" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D29" s="93" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E29" s="93" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="78" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
       <c r="B30" s="75" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C30" s="79" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D30" s="75" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E30" s="80" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="92" t="s">
-        <v>626</v>
+        <v>632</v>
       </c>
       <c r="B31" s="83" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="C31" s="90" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D31" s="83" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
       <c r="E31" s="93" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="106" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="B32" s="102" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C32" s="104" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D32" s="102" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E32" s="107" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="108" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
       <c r="B33" s="97" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C33" s="104" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D33" s="97" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E33" s="109" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="134" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
       <c r="B34" s="129" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="C34" s="123" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D34" s="129" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E34" s="135" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="136" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
       <c r="B35" s="124" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C35" s="132" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D35" s="124" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E35" s="137" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="74.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="147" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="B36" s="145" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C36" s="148" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="D36" s="153" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="E36" s="153" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="150" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
       <c r="B37" s="140" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="C37" s="151" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D37" s="140" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E37" s="152" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="147" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
       <c r="B38" s="145" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="C38" s="151" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="D38" s="145" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E38" s="149" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="160" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="B39" s="157" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C39" s="161" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D39" s="157" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E39" s="162" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="168" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
       <c r="B40" s="165" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="C40" s="169" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D40" s="165" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E40" s="170" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -14567,543 +14687,577 @@
         <v>140</v>
       </c>
       <c r="B41" s="172" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C41" s="173" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D41" s="172" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E41" s="174" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="188" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
       <c r="B42" s="183" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="C42" s="177" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D42" s="183" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E42" s="189" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="190" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="B43" s="178" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C43" s="186" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D43" s="178" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="E43" s="191" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="188" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
       <c r="B44" s="183" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="C44" s="186" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D44" s="183" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E44" s="189" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="190" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
       <c r="B45" s="178" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C45" s="186" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="D45" s="178" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E45" s="191" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="206" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
       <c r="B46" s="194" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C46" s="199" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D46" s="194" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E46" s="207" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="208" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="B47" s="200" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C47" s="203" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D47" s="200" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E47" s="209" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="206" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
       <c r="B48" s="194" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C48" s="203" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D48" s="194" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E48" s="207" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
       <c r="B49" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C49" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D49" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E49" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
-        <v>664</v>
+        <v>670</v>
       </c>
       <c r="B50" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C50" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D50" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E50" t="s">
-        <v>665</v>
+        <v>671</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
       <c r="B51" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C51" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D51" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E51" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
       <c r="B52" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C52" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="D52" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E52" t="s">
-        <v>670</v>
+        <v>676</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
       <c r="B53" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C53" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="D53" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E53" t="s">
-        <v>672</v>
+        <v>678</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="215" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C54" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="D54" s="215" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E54" s="215" t="s">
-        <v>674</v>
+        <v>680</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="215" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C55" s="215" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D55" s="215" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E55" s="215" t="s">
-        <v>676</v>
+        <v>682</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="215" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C56" s="215" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D56" s="215" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E56" s="215" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="215" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C57" s="215" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D57" s="215" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E57" s="215" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="215" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C58" s="215" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D58" s="215" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E58" s="215" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="215" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C59" s="215" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D59" s="215" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E59" s="215" t="s">
-        <v>684</v>
+        <v>690</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="215" t="s">
-        <v>685</v>
+        <v>691</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C60" s="215" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D60" s="215" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E60" s="215" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="215" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C61" s="215" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D61" s="215" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E61" s="215" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="215" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C62" s="215" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D62" s="215" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E62" s="215" t="s">
-        <v>690</v>
+        <v>696</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="215" t="s">
-        <v>691</v>
+        <v>697</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C63" s="215" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="D63" s="215" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E63" s="215" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="215" t="s">
-        <v>693</v>
+        <v>699</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C64" s="215" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="D64" s="215" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E64" s="215" t="s">
-        <v>694</v>
+        <v>700</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="129.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="215" t="s">
-        <v>695</v>
+        <v>701</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C65" s="215" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D65" s="215" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E65" s="215" t="s">
-        <v>696</v>
+        <v>702</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="215" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="B66" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C66" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D66" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E66" t="s">
-        <v>698</v>
+        <v>704</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="215" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="B67" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C67" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="D67" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E67" t="s">
-        <v>700</v>
+        <v>706</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="215" t="s">
-        <v>701</v>
+        <v>707</v>
       </c>
       <c r="B68" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C68" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="D68" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E68" t="s">
-        <v>702</v>
+        <v>708</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="215" t="s">
-        <v>703</v>
+        <v>709</v>
       </c>
       <c r="B69" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C69" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D69" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E69" t="s">
-        <v>704</v>
+        <v>710</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="215" t="s">
-        <v>705</v>
+        <v>711</v>
       </c>
       <c r="B70" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C70" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D70" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E70" t="s">
-        <v>706</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="215" t="s">
-        <v>707</v>
+        <v>713</v>
       </c>
       <c r="B71" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C71" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="D71" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E71" t="s">
-        <v>708</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="215" t="s">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="B72" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C72" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="D72" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="E72" t="s">
-        <v>710</v>
+        <v>716</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A73" s="215" t="s">
+        <v>717</v>
+      </c>
+      <c r="B73" t="s">
+        <v>564</v>
+      </c>
+      <c r="C73" t="s">
+        <v>577</v>
+      </c>
+      <c r="D73" t="s">
+        <v>566</v>
+      </c>
+      <c r="E73" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A74" s="215" t="s">
+        <v>719</v>
+      </c>
+      <c r="B74" t="s">
+        <v>578</v>
+      </c>
+      <c r="C74" t="s">
+        <v>577</v>
+      </c>
+      <c r="D74" t="s">
+        <v>609</v>
+      </c>
+      <c r="E74" t="s">
+        <v>720</v>
       </c>
     </row>
   </sheetData>
@@ -15128,12 +15282,12 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="219" t="s">
-        <v>711</v>
+        <v>721</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="303" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -15142,1032 +15296,1032 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="220" t="s">
-        <v>713</v>
+        <v>723</v>
       </c>
       <c r="B4" s="220" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="C4" s="220" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="220" t="s">
-        <v>714</v>
+        <v>724</v>
       </c>
       <c r="E4" s="220" t="s">
-        <v>715</v>
+        <v>725</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="221" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>717</v>
+        <v>727</v>
       </c>
       <c r="C5" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>718</v>
+        <v>728</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>719</v>
+        <v>729</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="221" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>720</v>
+        <v>730</v>
       </c>
       <c r="C6" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="215" t="s">
-        <v>718</v>
+        <v>728</v>
       </c>
       <c r="E6" s="215" t="s">
-        <v>721</v>
+        <v>731</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="231" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>723</v>
+        <v>733</v>
       </c>
       <c r="C7" s="232" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="215" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="E7" s="215" t="s">
-        <v>724</v>
+        <v>734</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="223" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>725</v>
+        <v>735</v>
       </c>
       <c r="C8" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>726</v>
+        <v>736</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>727</v>
+        <v>737</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="223" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="B9" s="215" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
       <c r="C9" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="215" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="E9" s="215" t="s">
-        <v>729</v>
+        <v>739</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="224" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>731</v>
+        <v>741</v>
       </c>
       <c r="C10" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>732</v>
+        <v>742</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>733</v>
+        <v>743</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>734</v>
+        <v>744</v>
       </c>
       <c r="C11" t="s">
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>735</v>
+        <v>745</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>736</v>
+        <v>746</v>
       </c>
       <c r="C12" t="s">
         <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>735</v>
+        <v>745</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="224" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>737</v>
+        <v>747</v>
       </c>
       <c r="C13" s="222" t="s">
         <v>128</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>738</v>
+        <v>748</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>739</v>
+        <v>749</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="235" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>740</v>
+        <v>750</v>
       </c>
       <c r="C14" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>741</v>
+        <v>751</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>742</v>
+        <v>752</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="235" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B15" s="215" t="s">
-        <v>743</v>
+        <v>753</v>
       </c>
       <c r="C15" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="215" t="s">
-        <v>738</v>
+        <v>748</v>
       </c>
       <c r="E15" s="215" t="s">
-        <v>744</v>
+        <v>754</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="235" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B16" s="215" t="s">
-        <v>745</v>
+        <v>755</v>
       </c>
       <c r="C16" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="215" t="s">
-        <v>738</v>
+        <v>748</v>
       </c>
       <c r="E16" s="215" t="s">
-        <v>746</v>
+        <v>756</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="225" t="s">
-        <v>747</v>
+        <v>757</v>
       </c>
       <c r="B17" s="215" t="s">
-        <v>748</v>
+        <v>758</v>
       </c>
       <c r="C17" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D17" s="215" t="s">
-        <v>749</v>
+        <v>759</v>
       </c>
       <c r="E17" s="215" t="s">
-        <v>750</v>
+        <v>760</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="225" t="s">
-        <v>747</v>
+        <v>757</v>
       </c>
       <c r="B18" s="215" t="s">
-        <v>751</v>
+        <v>761</v>
       </c>
       <c r="C18" s="223" t="s">
         <v>138</v>
       </c>
       <c r="D18" s="215" t="s">
-        <v>749</v>
+        <v>759</v>
       </c>
       <c r="E18" s="215" t="s">
-        <v>752</v>
+        <v>762</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="226" t="s">
-        <v>753</v>
+        <v>763</v>
       </c>
       <c r="B19" s="215" t="s">
-        <v>754</v>
+        <v>764</v>
       </c>
       <c r="C19" s="225" t="s">
-        <v>755</v>
+        <v>765</v>
       </c>
       <c r="D19" s="215" t="s">
-        <v>718</v>
+        <v>728</v>
       </c>
       <c r="E19" s="215" t="s">
-        <v>756</v>
+        <v>766</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="226" t="s">
-        <v>753</v>
+        <v>763</v>
       </c>
       <c r="B20" s="215" t="s">
-        <v>757</v>
+        <v>767</v>
       </c>
       <c r="C20" s="225" t="s">
-        <v>755</v>
+        <v>765</v>
       </c>
       <c r="D20" s="215" t="s">
-        <v>718</v>
+        <v>728</v>
       </c>
       <c r="E20" s="215" t="s">
-        <v>758</v>
+        <v>768</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="226" t="s">
-        <v>753</v>
+        <v>763</v>
       </c>
       <c r="B21" s="215" t="s">
-        <v>759</v>
+        <v>769</v>
       </c>
       <c r="C21" s="225" t="s">
-        <v>755</v>
+        <v>765</v>
       </c>
       <c r="D21" s="215" t="s">
-        <v>718</v>
+        <v>728</v>
       </c>
       <c r="E21" s="215" t="s">
-        <v>760</v>
+        <v>770</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
     <row r="23" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="229" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="B23" s="215" t="s">
-        <v>761</v>
+        <v>771</v>
       </c>
       <c r="C23" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D23" s="215" t="s">
-        <v>762</v>
+        <v>772</v>
       </c>
       <c r="E23" s="215" t="s">
-        <v>763</v>
+        <v>773</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="230" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="B24" s="215" t="s">
-        <v>764</v>
+        <v>774</v>
       </c>
       <c r="C24" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D24" s="215" t="s">
-        <v>765</v>
+        <v>775</v>
       </c>
       <c r="E24" s="215" t="s">
-        <v>766</v>
+        <v>776</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="231" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="B25" s="215" t="s">
-        <v>767</v>
+        <v>777</v>
       </c>
       <c r="C25" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D25" s="215" t="s">
-        <v>768</v>
+        <v>778</v>
       </c>
       <c r="E25" s="215" t="s">
-        <v>769</v>
+        <v>779</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="231" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="B26" s="215" t="s">
-        <v>770</v>
+        <v>780</v>
       </c>
       <c r="C26" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D26" s="215" t="s">
-        <v>765</v>
+        <v>775</v>
       </c>
       <c r="E26" s="215" t="s">
-        <v>771</v>
+        <v>781</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="235" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B27" s="215" t="s">
-        <v>772</v>
+        <v>782</v>
       </c>
       <c r="C27" s="237" t="s">
         <v>22</v>
       </c>
       <c r="D27" s="215" t="s">
-        <v>735</v>
+        <v>745</v>
       </c>
       <c r="E27" s="215" t="s">
-        <v>773</v>
+        <v>783</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="227" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="B28" s="215" t="s">
-        <v>774</v>
+        <v>784</v>
       </c>
       <c r="C28" t="s">
         <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>775</v>
+        <v>785</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B29" s="215" t="s">
-        <v>776</v>
+        <v>786</v>
       </c>
       <c r="C29" t="s">
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>735</v>
+        <v>745</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B30" s="215" t="s">
-        <v>777</v>
+        <v>787</v>
       </c>
       <c r="C30" t="s">
         <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>778</v>
+        <v>788</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="B31" s="215" t="s">
-        <v>779</v>
+        <v>789</v>
       </c>
       <c r="C31" t="s">
         <v>22</v>
       </c>
       <c r="D31" t="s">
-        <v>780</v>
+        <v>790</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="B32" s="215" t="s">
-        <v>781</v>
+        <v>791</v>
       </c>
       <c r="C32" t="s">
         <v>22</v>
       </c>
       <c r="D32" t="s">
-        <v>782</v>
+        <v>792</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="B33" s="215" t="s">
-        <v>783</v>
+        <v>793</v>
       </c>
       <c r="C33" t="s">
         <v>22</v>
       </c>
       <c r="D33" t="s">
-        <v>780</v>
+        <v>790</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="B34" s="215" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="C34" t="s">
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>785</v>
+        <v>795</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B35" s="215" t="s">
-        <v>786</v>
+        <v>796</v>
       </c>
       <c r="C35" t="s">
         <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>787</v>
+        <v>797</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="B36" s="215" t="s">
-        <v>788</v>
+        <v>798</v>
       </c>
       <c r="C36" t="s">
         <v>22</v>
       </c>
       <c r="D36" t="s">
-        <v>789</v>
+        <v>799</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B37" s="215" t="s">
-        <v>790</v>
+        <v>800</v>
       </c>
       <c r="C37" t="s">
         <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>789</v>
+        <v>799</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
-        <v>747</v>
+        <v>757</v>
       </c>
       <c r="B38" s="215" t="s">
-        <v>791</v>
+        <v>801</v>
       </c>
       <c r="C38" t="s">
         <v>22</v>
       </c>
       <c r="D38" t="s">
-        <v>789</v>
+        <v>799</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="B39" s="215" t="s">
-        <v>792</v>
+        <v>802</v>
       </c>
       <c r="C39" t="s">
         <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>789</v>
+        <v>799</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B40" s="215" t="s">
-        <v>793</v>
+        <v>803</v>
       </c>
       <c r="C40" t="s">
         <v>22</v>
       </c>
       <c r="D40" t="s">
-        <v>789</v>
+        <v>799</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="B41" s="215" t="s">
-        <v>794</v>
+        <v>804</v>
       </c>
       <c r="C41" t="s">
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>795</v>
+        <v>805</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B42" s="215" t="s">
-        <v>796</v>
+        <v>806</v>
       </c>
       <c r="C42" t="s">
         <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>795</v>
+        <v>805</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B43" s="215" t="s">
-        <v>797</v>
+        <v>807</v>
       </c>
       <c r="C43" t="s">
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>798</v>
+        <v>808</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="B44" s="215" t="s">
-        <v>799</v>
+        <v>809</v>
       </c>
       <c r="C44" t="s">
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>798</v>
+        <v>808</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
-        <v>747</v>
+        <v>757</v>
       </c>
       <c r="B45" s="215" t="s">
-        <v>800</v>
+        <v>810</v>
       </c>
       <c r="C45" t="s">
         <v>128</v>
       </c>
       <c r="D45" t="s">
-        <v>801</v>
+        <v>811</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B46" s="215" t="s">
-        <v>803</v>
+        <v>813</v>
       </c>
       <c r="C46" t="s">
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>804</v>
+        <v>814</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B47" s="215" t="s">
-        <v>805</v>
+        <v>815</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>806</v>
+        <v>816</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B48" s="215" t="s">
-        <v>807</v>
+        <v>817</v>
       </c>
       <c r="C48" t="s">
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>806</v>
+        <v>816</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B49" s="215" t="s">
-        <v>808</v>
+        <v>818</v>
       </c>
       <c r="C49" t="s">
         <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>806</v>
+        <v>816</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B50" s="215" t="s">
-        <v>809</v>
+        <v>819</v>
       </c>
       <c r="C50" t="s">
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>810</v>
+        <v>820</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B51" s="215" t="s">
-        <v>811</v>
+        <v>821</v>
       </c>
       <c r="C51" t="s">
         <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>812</v>
+        <v>822</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B52" s="215" t="s">
-        <v>813</v>
+        <v>823</v>
       </c>
       <c r="C52" t="s">
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>814</v>
+        <v>824</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B53" s="215" t="s">
-        <v>815</v>
+        <v>825</v>
       </c>
       <c r="C53" t="s">
         <v>128</v>
       </c>
       <c r="D53" t="s">
-        <v>812</v>
+        <v>822</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>816</v>
+        <v>826</v>
       </c>
       <c r="C54" t="s">
         <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>814</v>
+        <v>824</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>817</v>
+        <v>827</v>
       </c>
       <c r="C55" t="s">
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>818</v>
+        <v>828</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>819</v>
+        <v>829</v>
       </c>
       <c r="C56" t="s">
         <v>128</v>
       </c>
       <c r="D56" t="s">
-        <v>820</v>
+        <v>830</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>821</v>
+        <v>831</v>
       </c>
       <c r="C57" t="s">
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>822</v>
+        <v>832</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>823</v>
+        <v>833</v>
       </c>
       <c r="C58" t="s">
         <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>822</v>
+        <v>832</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>824</v>
+        <v>834</v>
       </c>
       <c r="C59" t="s">
         <v>22</v>
       </c>
       <c r="D59" t="s">
-        <v>822</v>
+        <v>832</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>825</v>
+        <v>835</v>
       </c>
       <c r="C60" t="s">
         <v>128</v>
       </c>
       <c r="D60" t="s">
-        <v>822</v>
+        <v>832</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="274" t="s">
-        <v>826</v>
+        <v>836</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>827</v>
+        <v>837</v>
       </c>
       <c r="C61" t="s">
         <v>22</v>
       </c>
       <c r="D61" t="s">
-        <v>795</v>
+        <v>805</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="274" t="s">
-        <v>826</v>
+        <v>836</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>828</v>
+        <v>838</v>
       </c>
       <c r="C62" t="s">
         <v>22</v>
       </c>
       <c r="D62" t="s">
-        <v>795</v>
+        <v>805</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="274" t="s">
-        <v>826</v>
+        <v>836</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>829</v>
+        <v>839</v>
       </c>
       <c r="C63" t="s">
         <v>22</v>
       </c>
       <c r="D63" t="s">
-        <v>795</v>
+        <v>805</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>830</v>
+        <v>840</v>
       </c>
       <c r="C64" t="s">
         <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>831</v>
+        <v>841</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>832</v>
+        <v>842</v>
       </c>
       <c r="C65" t="s">
         <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>831</v>
+        <v>841</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B66" s="215" t="s">
-        <v>833</v>
+        <v>843</v>
       </c>
       <c r="C66" t="s">
         <v>22</v>
       </c>
       <c r="D66" t="s">
-        <v>831</v>
+        <v>841</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="274" t="s">
-        <v>834</v>
+        <v>844</v>
       </c>
       <c r="B67" s="215" t="s">
-        <v>835</v>
+        <v>845</v>
       </c>
       <c r="C67" t="s">
         <v>22</v>
       </c>
       <c r="D67" t="s">
-        <v>795</v>
+        <v>805</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="274" t="s">
-        <v>834</v>
+        <v>844</v>
       </c>
       <c r="B68" s="215" t="s">
-        <v>836</v>
+        <v>846</v>
       </c>
       <c r="C68" t="s">
         <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>795</v>
+        <v>805</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="274" t="s">
-        <v>834</v>
+        <v>844</v>
       </c>
       <c r="B69" s="215" t="s">
-        <v>837</v>
+        <v>847</v>
       </c>
       <c r="C69" t="s">
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>795</v>
+        <v>805</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B70" s="215" t="s">
-        <v>838</v>
+        <v>848</v>
       </c>
       <c r="C70" t="s">
         <v>22</v>
       </c>
       <c r="D70" t="s">
-        <v>839</v>
+        <v>849</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B71" s="215" t="s">
-        <v>840</v>
+        <v>850</v>
       </c>
       <c r="C71" t="s">
         <v>22</v>
       </c>
       <c r="D71" t="s">
-        <v>839</v>
+        <v>849</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B72" s="215" t="s">
-        <v>841</v>
+        <v>851</v>
       </c>
       <c r="C72" t="s">
         <v>22</v>
       </c>
       <c r="D72" t="s">
-        <v>839</v>
+        <v>849</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="274" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
       <c r="B73" s="215" t="s">
-        <v>842</v>
+        <v>852</v>
       </c>
       <c r="C73" t="s">
         <v>128</v>
       </c>
       <c r="D73" t="s">
-        <v>839</v>
+        <v>849</v>
       </c>
     </row>
   </sheetData>
@@ -16196,336 +16350,336 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="211" t="s">
-        <v>843</v>
+        <v>853</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="212" t="s">
-        <v>844</v>
+        <v>854</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="213" t="s">
-        <v>845</v>
+        <v>855</v>
       </c>
       <c r="B4" s="213" t="s">
-        <v>846</v>
+        <v>856</v>
       </c>
       <c r="C4" s="213" t="s">
-        <v>847</v>
+        <v>857</v>
       </c>
       <c r="D4" s="213" t="s">
-        <v>848</v>
+        <v>858</v>
       </c>
       <c r="E4" s="213" t="s">
-        <v>849</v>
+        <v>859</v>
       </c>
       <c r="F4" s="213" t="s">
-        <v>850</v>
+        <v>860</v>
       </c>
       <c r="G4" s="213" t="s">
-        <v>851</v>
+        <v>861</v>
       </c>
       <c r="H4" s="213" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="213" t="s">
-        <v>852</v>
+        <v>862</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="214" t="s">
-        <v>853</v>
+        <v>863</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>854</v>
+        <v>864</v>
       </c>
       <c r="C5" s="215" t="s">
-        <v>855</v>
+        <v>865</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>856</v>
+        <v>866</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>857</v>
+        <v>867</v>
       </c>
       <c r="F5" s="215" t="s">
-        <v>858</v>
+        <v>868</v>
       </c>
       <c r="G5" s="215" t="s">
-        <v>859</v>
+        <v>869</v>
       </c>
       <c r="H5" s="216" t="s">
-        <v>860</v>
+        <v>870</v>
       </c>
       <c r="I5" s="215" t="s">
-        <v>861</v>
+        <v>871</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="214" t="s">
-        <v>862</v>
+        <v>872</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>863</v>
+        <v>873</v>
       </c>
       <c r="C6" s="215" t="s">
-        <v>864</v>
+        <v>874</v>
       </c>
       <c r="D6" s="215" t="s">
-        <v>865</v>
+        <v>875</v>
       </c>
       <c r="E6" s="215" t="s">
-        <v>866</v>
+        <v>876</v>
       </c>
       <c r="F6" s="215" t="s">
-        <v>867</v>
+        <v>877</v>
       </c>
       <c r="G6" s="215" t="s">
-        <v>868</v>
+        <v>878</v>
       </c>
       <c r="H6" s="217" t="s">
-        <v>860</v>
+        <v>870</v>
       </c>
       <c r="I6" s="215" t="s">
-        <v>869</v>
+        <v>879</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="214" t="s">
+        <v>880</v>
+      </c>
+      <c r="B7" s="215" t="s">
+        <v>881</v>
+      </c>
+      <c r="C7" s="215" t="s">
+        <v>882</v>
+      </c>
+      <c r="D7" s="215" t="s">
+        <v>883</v>
+      </c>
+      <c r="E7" s="215" t="s">
+        <v>884</v>
+      </c>
+      <c r="F7" s="215" t="s">
+        <v>885</v>
+      </c>
+      <c r="G7" s="215" t="s">
+        <v>886</v>
+      </c>
+      <c r="H7" s="217" t="s">
         <v>870</v>
       </c>
-      <c r="B7" s="215" t="s">
-        <v>871</v>
-      </c>
-      <c r="C7" s="215" t="s">
-        <v>872</v>
-      </c>
-      <c r="D7" s="215" t="s">
-        <v>873</v>
-      </c>
-      <c r="E7" s="215" t="s">
-        <v>874</v>
-      </c>
-      <c r="F7" s="215" t="s">
-        <v>875</v>
-      </c>
-      <c r="G7" s="215" t="s">
-        <v>876</v>
-      </c>
-      <c r="H7" s="217" t="s">
-        <v>860</v>
-      </c>
       <c r="I7" s="215" t="s">
-        <v>877</v>
+        <v>887</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="214" t="s">
-        <v>878</v>
+        <v>888</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>879</v>
+        <v>889</v>
       </c>
       <c r="C8" s="215" t="s">
-        <v>880</v>
+        <v>890</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>881</v>
+        <v>891</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="F8" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="G8" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="H8" s="216" t="s">
-        <v>882</v>
+        <v>892</v>
       </c>
       <c r="I8" s="215" t="s">
-        <v>883</v>
+        <v>893</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="214" t="s">
+        <v>894</v>
+      </c>
+      <c r="B9" s="215" t="s">
+        <v>895</v>
+      </c>
+      <c r="C9" s="215" t="s">
+        <v>896</v>
+      </c>
+      <c r="D9" s="215" t="s">
+        <v>891</v>
+      </c>
+      <c r="E9" s="215" t="s">
         <v>884</v>
       </c>
-      <c r="B9" s="215" t="s">
-        <v>885</v>
-      </c>
-      <c r="C9" s="215" t="s">
-        <v>886</v>
-      </c>
-      <c r="D9" s="215" t="s">
-        <v>881</v>
-      </c>
-      <c r="E9" s="215" t="s">
-        <v>874</v>
-      </c>
       <c r="F9" s="215" t="s">
-        <v>887</v>
+        <v>897</v>
       </c>
       <c r="G9" s="215" t="s">
-        <v>888</v>
+        <v>898</v>
       </c>
       <c r="H9" s="218" t="s">
-        <v>889</v>
+        <v>899</v>
       </c>
       <c r="I9" s="215" t="s">
-        <v>890</v>
+        <v>900</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="214" t="s">
-        <v>891</v>
+        <v>901</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>892</v>
+        <v>902</v>
       </c>
       <c r="C10" s="215" t="s">
-        <v>893</v>
+        <v>903</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>894</v>
+        <v>904</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>895</v>
+        <v>905</v>
       </c>
       <c r="F10" s="215" t="s">
-        <v>896</v>
+        <v>906</v>
       </c>
       <c r="G10" s="215" t="s">
-        <v>897</v>
+        <v>907</v>
       </c>
       <c r="H10" s="218" t="s">
-        <v>898</v>
+        <v>908</v>
       </c>
       <c r="I10" s="215" t="s">
-        <v>899</v>
+        <v>909</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="214" t="s">
-        <v>900</v>
+        <v>910</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>901</v>
+        <v>911</v>
       </c>
       <c r="C11" s="215" t="s">
-        <v>902</v>
+        <v>912</v>
       </c>
       <c r="D11" s="215" t="s">
-        <v>903</v>
+        <v>913</v>
       </c>
       <c r="E11" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="F11" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="G11" s="215" t="s">
-        <v>904</v>
+        <v>914</v>
       </c>
       <c r="H11" s="218" t="s">
-        <v>905</v>
+        <v>915</v>
       </c>
       <c r="I11" s="215" t="s">
-        <v>906</v>
+        <v>916</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="214" t="s">
-        <v>907</v>
+        <v>917</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>908</v>
+        <v>918</v>
       </c>
       <c r="C12" s="215" t="s">
-        <v>909</v>
+        <v>919</v>
       </c>
       <c r="D12" s="215" t="s">
-        <v>910</v>
+        <v>920</v>
       </c>
       <c r="E12" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="F12" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="G12" s="215" t="s">
-        <v>904</v>
+        <v>914</v>
       </c>
       <c r="H12" s="217" t="s">
-        <v>911</v>
+        <v>921</v>
       </c>
       <c r="I12" s="215" t="s">
-        <v>912</v>
+        <v>922</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="214" t="s">
-        <v>913</v>
+        <v>923</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>914</v>
+        <v>924</v>
       </c>
       <c r="C13" s="215" t="s">
-        <v>915</v>
+        <v>925</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="F13" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="G13" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="H13" s="218" t="s">
-        <v>916</v>
+        <v>926</v>
       </c>
       <c r="I13" s="215" t="s">
-        <v>917</v>
+        <v>927</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="214" t="s">
-        <v>918</v>
+        <v>928</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>919</v>
+        <v>929</v>
       </c>
       <c r="C14" s="215" t="s">
-        <v>915</v>
+        <v>925</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="F14" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="G14" s="215" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="H14" s="218" t="s">
-        <v>916</v>
+        <v>926</v>
       </c>
       <c r="I14" s="215" t="s">
-        <v>920</v>
+        <v>930</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="304" t="s">
-        <v>921</v>
+        <v>931</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>

</xml_diff>

<commit_message>
docs(tracker): completeness floor raised to 0.35, and why the stated reason was wrong
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28DBCC59-6373-4F91-8C16-19FC7253A05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8392F6BC-29ED-474C-88C7-4E2A6287EB8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1954" uniqueCount="932">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1965" uniqueCount="936">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -1475,6 +1475,12 @@
   </si>
   <si>
     <t>4,296 vs 386 rows as separate categories. Not cosmetic - surface_win_rate, surface_streak and h2h_win_rate_surface all match on this string, so 8% of grass matches were compared against the wrong pool. Stripped at collection and on load</t>
+  </si>
+  <si>
+    <t>MIN_FEATURE_COMPLETENESS raised 0.25 -&gt; 0.35</t>
+  </si>
+  <si>
+    <t>Raised for COHERENCE, not accuracy - mobile dims below 0.35, so between 0.25 and 0.35 the product recommended a pick while calling its own data limited. Accuracy bands cannot locate a cliff (every 95% CI overlaps; worst band n=5). Costs zero upcoming picks. Not 0.50, which would drop 11 picks on a six-fixture band. Re-derive at n=93</t>
   </si>
   <si>
     <t>Legend</t>
@@ -2273,6 +2279,12 @@
   </si>
   <si>
     <t>A base rate is the no-model alternative. Football's 'back the home team' qualifies; tennis's 'back the lower player id' does not - it is invisible to the user and is a proxy for strength the model already uses. Gating on it inverted a quarter of picks. Any future sport-specific base rate must name the strategy it represents and that strategy must be executable by someone without our database.</t>
+  </si>
+  <si>
+    <t>A recommendation was made on evidence not yet checked</t>
+  </si>
+  <si>
+    <t>The completeness floor was recommended on the claim that two measurements agreed the cliff was at 0.35. Measuring with intervals showed neither could locate a cliff at all, and the older one pointed at 0.50 if anywhere. The change went ahead on a different, non-statistical justification (coherence with mobile, zero cost) and the original claim is recorded as wrong rather than quietly replaced. Threshold changes should carry intervals before, not after.</t>
   </si>
   <si>
     <t>SportIQ — Edge Measurement Plan (P0-P3)</t>
@@ -5255,7 +5267,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R223"/>
+  <dimension ref="A1:R224"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -12003,7 +12015,7 @@
         <v>432</v>
       </c>
       <c r="R198" t="str">
-        <f t="shared" ref="R198:R221" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
+        <f t="shared" ref="R198:R222" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
         <v>E4 ML Football</v>
       </c>
     </row>
@@ -12601,7 +12613,7 @@
         <v>E8 Model Quality</v>
       </c>
     </row>
-    <row r="219" spans="1:18" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="219" spans="1:18" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A219" t="s">
         <v>73</v>
       </c>
@@ -12631,7 +12643,7 @@
         <v>E6 Picks</v>
       </c>
     </row>
-    <row r="220" spans="1:18" ht="72" x14ac:dyDescent="0.55000000000000004">
+    <row r="220" spans="1:18" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A220" t="s">
         <v>99</v>
       </c>
@@ -12661,7 +12673,7 @@
         <v>E8 Model Quality</v>
       </c>
     </row>
-    <row r="221" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="221" spans="1:18" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A221" t="s">
         <v>130</v>
       </c>
@@ -12691,23 +12703,53 @@
         <v>E9 Data Ops</v>
       </c>
     </row>
-    <row r="223" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A223" s="23" t="s">
+    <row r="222" spans="1:18" ht="72" x14ac:dyDescent="0.55000000000000004">
+      <c r="A222" t="s">
+        <v>73</v>
+      </c>
+      <c r="B222" t="s">
         <v>479</v>
       </c>
-      <c r="B223" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C223" s="15" t="s">
+      <c r="C222" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D222" t="s">
+        <v>75</v>
+      </c>
+      <c r="E222" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F222" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G222" s="215" t="s">
         <v>480</v>
       </c>
-      <c r="D223" s="17" t="s">
+      <c r="J222" t="s">
+        <v>400</v>
+      </c>
+      <c r="R222" t="str">
+        <f t="shared" si="3"/>
+        <v>E6 Picks</v>
+      </c>
+    </row>
+    <row r="224" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A224" s="23" t="s">
+        <v>481</v>
+      </c>
+      <c r="B224" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C224" s="15" t="s">
+        <v>482</v>
+      </c>
+      <c r="D224" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="E223" s="21" t="s">
+      <c r="E224" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="F223" s="19" t="s">
+      <c r="F224" s="19" t="s">
         <v>138</v>
       </c>
     </row>
@@ -12732,7 +12774,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="294" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B1" s="283"/>
       <c r="C1" s="283"/>
@@ -12755,7 +12797,7 @@
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="301" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -12778,7 +12820,7 @@
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="289" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B4" s="283"/>
       <c r="C4" s="283"/>
@@ -12801,42 +12843,42 @@
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="35" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B5" s="279" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="C5" s="280"/>
       <c r="D5" s="281"/>
       <c r="E5" s="284" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="F5" s="280"/>
       <c r="G5" s="281"/>
       <c r="H5" s="284" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="I5" s="280"/>
       <c r="J5" s="281"/>
       <c r="K5" s="279" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="L5" s="280"/>
       <c r="M5" s="281"/>
       <c r="N5" s="286" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="O5" s="280"/>
       <c r="P5" s="281"/>
       <c r="Q5" s="286" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="R5" s="280"/>
       <c r="S5" s="281"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="282" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="C6" s="283"/>
       <c r="D6" s="283"/>
@@ -12858,7 +12900,7 @@
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="289" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B7" s="283"/>
       <c r="C7" s="283"/>
@@ -12881,10 +12923,10 @@
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="35" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B8" s="292" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="C8" s="280"/>
       <c r="D8" s="280"/>
@@ -12895,7 +12937,7 @@
       <c r="I8" s="280"/>
       <c r="J8" s="281"/>
       <c r="K8" s="292" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="L8" s="280"/>
       <c r="M8" s="280"/>
@@ -12908,7 +12950,7 @@
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="282" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="C9" s="283"/>
       <c r="D9" s="283"/>
@@ -12930,7 +12972,7 @@
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="289" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B10" s="283"/>
       <c r="C10" s="283"/>
@@ -12953,42 +12995,42 @@
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="35" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B11" s="279" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="C11" s="280"/>
       <c r="D11" s="281"/>
       <c r="E11" s="279" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="F11" s="280"/>
       <c r="G11" s="281"/>
       <c r="H11" s="279" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="I11" s="280"/>
       <c r="J11" s="281"/>
       <c r="K11" s="284" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="L11" s="280"/>
       <c r="M11" s="281"/>
       <c r="N11" s="279" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="O11" s="280"/>
       <c r="P11" s="281"/>
       <c r="Q11" s="279" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="R11" s="280"/>
       <c r="S11" s="281"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="282" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="C12" s="283"/>
       <c r="D12" s="283"/>
@@ -13010,7 +13052,7 @@
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="289" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B13" s="283"/>
       <c r="C13" s="283"/>
@@ -13033,10 +13075,10 @@
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="35" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B14" s="287" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="C14" s="280"/>
       <c r="D14" s="280"/>
@@ -13044,7 +13086,7 @@
       <c r="F14" s="280"/>
       <c r="G14" s="281"/>
       <c r="H14" s="287" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="I14" s="280"/>
       <c r="J14" s="280"/>
@@ -13052,19 +13094,19 @@
       <c r="L14" s="280"/>
       <c r="M14" s="281"/>
       <c r="N14" s="287" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="O14" s="280"/>
       <c r="P14" s="281"/>
       <c r="Q14" s="284" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="R14" s="280"/>
       <c r="S14" s="281"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" s="282" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="C15" s="283"/>
       <c r="D15" s="283"/>
@@ -13086,7 +13128,7 @@
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="289" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>
@@ -13109,10 +13151,10 @@
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="35" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B17" s="288" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="C17" s="280"/>
       <c r="D17" s="280"/>
@@ -13120,29 +13162,29 @@
       <c r="F17" s="280"/>
       <c r="G17" s="281"/>
       <c r="H17" s="288" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="I17" s="280"/>
       <c r="J17" s="281"/>
       <c r="K17" s="288" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="L17" s="280"/>
       <c r="M17" s="281"/>
       <c r="N17" s="288" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="O17" s="280"/>
       <c r="P17" s="281"/>
       <c r="Q17" s="288" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="R17" s="280"/>
       <c r="S17" s="281"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="282" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="C18" s="283"/>
       <c r="D18" s="283"/>
@@ -13164,7 +13206,7 @@
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="289" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B19" s="283"/>
       <c r="C19" s="283"/>
@@ -13187,10 +13229,10 @@
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="35" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B20" s="290" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="C20" s="280"/>
       <c r="D20" s="280"/>
@@ -13198,7 +13240,7 @@
       <c r="F20" s="280"/>
       <c r="G20" s="281"/>
       <c r="H20" s="290" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="I20" s="280"/>
       <c r="J20" s="280"/>
@@ -13206,7 +13248,7 @@
       <c r="L20" s="280"/>
       <c r="M20" s="281"/>
       <c r="N20" s="290" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="O20" s="280"/>
       <c r="P20" s="280"/>
@@ -13216,7 +13258,7 @@
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" s="282" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="C21" s="283"/>
       <c r="D21" s="283"/>
@@ -13238,7 +13280,7 @@
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="289" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B22" s="283"/>
       <c r="C22" s="283"/>
@@ -13261,10 +13303,10 @@
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="35" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="B23" s="290" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="C23" s="280"/>
       <c r="D23" s="280"/>
@@ -13272,29 +13314,29 @@
       <c r="F23" s="280"/>
       <c r="G23" s="281"/>
       <c r="H23" s="290" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="I23" s="280"/>
       <c r="J23" s="281"/>
       <c r="K23" s="290" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="L23" s="280"/>
       <c r="M23" s="281"/>
       <c r="N23" s="290" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="O23" s="280"/>
       <c r="P23" s="281"/>
       <c r="Q23" s="286" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="R23" s="280"/>
       <c r="S23" s="281"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="295" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B26" s="283"/>
       <c r="C26" s="283"/>
@@ -13317,42 +13359,42 @@
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="35" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B27" s="279" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="C27" s="280"/>
       <c r="D27" s="281"/>
       <c r="E27" s="279" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="F27" s="280"/>
       <c r="G27" s="281"/>
       <c r="H27" s="287" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="I27" s="280"/>
       <c r="J27" s="281"/>
       <c r="K27" s="288" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="L27" s="280"/>
       <c r="M27" s="281"/>
       <c r="N27" s="288" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="O27" s="280"/>
       <c r="P27" s="281"/>
       <c r="Q27" s="287" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="R27" s="280"/>
       <c r="S27" s="281"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="289" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="B30" s="283"/>
       <c r="C30" s="283"/>
@@ -13375,7 +13417,7 @@
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="285" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="B31" s="283"/>
       <c r="C31" s="283"/>
@@ -13398,7 +13440,7 @@
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="285" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="B32" s="283"/>
       <c r="C32" s="283"/>
@@ -13421,7 +13463,7 @@
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="285" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="B33" s="283"/>
       <c r="C33" s="283"/>
@@ -13444,7 +13486,7 @@
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="285" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B34" s="283"/>
       <c r="C34" s="283"/>
@@ -13467,7 +13509,7 @@
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="285" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B35" s="283"/>
       <c r="C35" s="283"/>
@@ -13490,7 +13532,7 @@
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="285" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B36" s="283"/>
       <c r="C36" s="283"/>
@@ -13513,7 +13555,7 @@
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="296" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B37" s="283"/>
       <c r="C37" s="283"/>
@@ -13536,25 +13578,25 @@
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="36" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B39" s="299" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C39" s="283"/>
       <c r="D39" s="283"/>
       <c r="E39" s="297" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="F39" s="283"/>
       <c r="G39" s="283"/>
       <c r="H39" s="300" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="I39" s="283"/>
       <c r="J39" s="283"/>
       <c r="K39" s="293" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="L39" s="283"/>
       <c r="M39" s="283"/>
@@ -13564,7 +13606,7 @@
       <c r="O39" s="283"/>
       <c r="P39" s="283"/>
       <c r="Q39" s="298" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="R39" s="283"/>
       <c r="S39" s="283"/>
@@ -13572,11 +13614,11 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="H20:M20"/>
     <mergeCell ref="A16:S16"/>
-    <mergeCell ref="H20:M20"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -13585,14 +13627,13 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -13601,6 +13642,7 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -13608,7 +13650,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -13657,7 +13699,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -13670,19 +13712,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -13816,11 +13858,11 @@
       </c>
       <c r="B9" s="24">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C9" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D9" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -13832,7 +13874,7 @@
       </c>
       <c r="F9" s="25">
         <f t="shared" si="1"/>
-        <v>0.88888888888888884</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -13962,15 +14004,15 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="26" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B16" s="27">
         <f>SUM(B4:B14)</f>
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C16" s="27">
         <f>SUM(C4:C14)</f>
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
@@ -13982,12 +14024,12 @@
       </c>
       <c r="F16" s="28">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.78801843317972353</v>
+        <v>0.78899082568807344</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="41" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="B18" s="42">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -13996,7 +14038,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="43" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
   </sheetData>
@@ -14017,7 +14059,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -14029,7 +14071,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -14038,648 +14080,648 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="29" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="D3" s="29" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="29" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="30" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="32" t="s">
+        <v>570</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>566</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>571</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>568</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>564</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>569</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>566</v>
-      </c>
       <c r="E5" s="33" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="30" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="32" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="30" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="32" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="30" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="32" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="30" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="32" t="s">
+        <v>594</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>574</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>579</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>592</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>572</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>577</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>590</v>
-      </c>
       <c r="E13" s="33" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="30" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="32" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="30" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="32" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="30" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="32" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="30" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="32" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="E21" s="33" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="30" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="32" t="s">
+        <v>618</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>616</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>614</v>
-      </c>
       <c r="C23" s="17" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="30" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E24" s="31" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="53" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="B25" s="51" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C25" s="54" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E25" s="55" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="56" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="B26" s="46" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="C26" s="54" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="D26" s="46" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E26" s="57" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="53" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="B27" s="51" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C27" s="54" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="D27" s="51" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E27" s="55" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="71" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="B28" s="60" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C28" s="67" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D28" s="94" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E28" s="94" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="72" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="B29" s="65" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C29" s="69" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D29" s="93" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E29" s="93" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="78" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="B30" s="75" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C30" s="79" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D30" s="75" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E30" s="80" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="92" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="B31" s="83" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="C31" s="90" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D31" s="83" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="E31" s="93" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="106" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="B32" s="102" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C32" s="104" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D32" s="102" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E32" s="107" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="108" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="B33" s="97" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C33" s="104" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D33" s="97" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="E33" s="109" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="134" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="B34" s="129" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="C34" s="123" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D34" s="129" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E34" s="135" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="136" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="B35" s="124" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C35" s="132" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D35" s="124" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E35" s="137" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="74.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="147" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="B36" s="145" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C36" s="148" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D36" s="153" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="E36" s="153" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="150" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="B37" s="140" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="C37" s="151" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D37" s="140" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E37" s="152" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="147" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="B38" s="145" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="C38" s="151" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="D38" s="145" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E38" s="149" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="160" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="B39" s="157" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C39" s="161" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D39" s="157" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E39" s="162" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="168" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="B40" s="165" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="C40" s="169" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D40" s="165" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E40" s="170" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -14687,577 +14729,594 @@
         <v>140</v>
       </c>
       <c r="B41" s="172" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C41" s="173" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D41" s="172" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E41" s="174" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="188" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="B42" s="183" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="C42" s="177" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D42" s="183" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E42" s="189" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="190" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="B43" s="178" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C43" s="186" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D43" s="178" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="E43" s="191" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="188" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="B44" s="183" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="C44" s="186" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D44" s="183" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E44" s="189" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="190" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="B45" s="178" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C45" s="186" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="D45" s="178" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E45" s="191" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="206" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="B46" s="194" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C46" s="199" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D46" s="194" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E46" s="207" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="208" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="B47" s="200" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C47" s="203" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D47" s="200" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E47" s="209" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="206" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="B48" s="194" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C48" s="203" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D48" s="194" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E48" s="207" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="B49" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C49" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D49" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E49" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="B50" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C50" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D50" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E50" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="B51" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C51" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D51" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E51" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="B52" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C52" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="D52" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E52" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
+        <v>679</v>
+      </c>
+      <c r="B53" t="s">
+        <v>580</v>
+      </c>
+      <c r="C53" t="s">
         <v>677</v>
       </c>
-      <c r="B53" t="s">
-        <v>578</v>
-      </c>
-      <c r="C53" t="s">
-        <v>675</v>
-      </c>
       <c r="D53" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E53" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="215" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C54" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="D54" s="215" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E54" s="215" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="215" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C55" s="215" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D55" s="215" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E55" s="215" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="215" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C56" s="215" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D56" s="215" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E56" s="215" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="215" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C57" s="215" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D57" s="215" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E57" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="215" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C58" s="215" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D58" s="215" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E58" s="215" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="215" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C59" s="215" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D59" s="215" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E59" s="215" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="215" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C60" s="215" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D60" s="215" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E60" s="215" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="215" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C61" s="215" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D61" s="215" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E61" s="215" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="215" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C62" s="215" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D62" s="215" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E62" s="215" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="215" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C63" s="215" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="D63" s="215" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E63" s="215" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="215" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C64" s="215" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="D64" s="215" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E64" s="215" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="129.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="215" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C65" s="215" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D65" s="215" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E65" s="215" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="215" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="B66" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C66" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D66" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E66" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="215" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="B67" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C67" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="D67" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E67" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="215" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="B68" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C68" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="D68" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E68" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="215" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="B69" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C69" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D69" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E69" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="215" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="B70" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C70" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D70" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E70" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="215" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="B71" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C71" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D71" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E71" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="215" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="B72" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C72" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D72" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E72" t="s">
-        <v>716</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="215" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="B73" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C73" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D73" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E73" t="s">
-        <v>718</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" s="215" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="B74" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C74" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D74" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E74" t="s">
-        <v>720</v>
+        <v>722</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A75" s="215" t="s">
+        <v>723</v>
+      </c>
+      <c r="B75" t="s">
+        <v>580</v>
+      </c>
+      <c r="C75" t="s">
+        <v>591</v>
+      </c>
+      <c r="D75" t="s">
+        <v>611</v>
+      </c>
+      <c r="E75" t="s">
+        <v>724</v>
       </c>
     </row>
   </sheetData>
@@ -15282,12 +15341,12 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="219" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="303" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -15296,1032 +15355,1032 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="220" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="B4" s="220" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="C4" s="220" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="220" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="E4" s="220" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="221" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="C5" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="221" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="C6" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="215" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="E6" s="215" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="231" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="C7" s="232" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="215" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="E7" s="215" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="223" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="C8" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="223" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B9" s="215" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
       <c r="C9" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="215" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="E9" s="215" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="224" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="C10" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="C11" t="s">
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="C12" t="s">
         <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="224" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
       <c r="C13" s="222" t="s">
         <v>128</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="235" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="C14" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="235" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B15" s="215" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="C15" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="215" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="E15" s="215" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="235" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B16" s="215" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="C16" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="215" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="E16" s="215" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="225" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B17" s="215" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="C17" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D17" s="215" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="E17" s="215" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="225" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B18" s="215" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="C18" s="223" t="s">
         <v>138</v>
       </c>
       <c r="D18" s="215" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="E18" s="215" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="226" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="B19" s="215" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="C19" s="225" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="D19" s="215" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="E19" s="215" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="226" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="B20" s="215" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="C20" s="225" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="D20" s="215" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="E20" s="215" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="226" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="B21" s="215" t="s">
+        <v>773</v>
+      </c>
+      <c r="C21" s="225" t="s">
         <v>769</v>
       </c>
-      <c r="C21" s="225" t="s">
-        <v>765</v>
-      </c>
       <c r="D21" s="215" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="E21" s="215" t="s">
-        <v>770</v>
+        <v>774</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
     <row r="23" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="229" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="B23" s="215" t="s">
-        <v>771</v>
+        <v>775</v>
       </c>
       <c r="C23" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D23" s="215" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="E23" s="215" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="230" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B24" s="215" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="C24" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D24" s="215" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
       <c r="E24" s="215" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="231" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B25" s="215" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
       <c r="C25" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D25" s="215" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
       <c r="E25" s="215" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="231" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B26" s="215" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="C26" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D26" s="215" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
       <c r="E26" s="215" t="s">
-        <v>781</v>
+        <v>785</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="235" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B27" s="215" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="C27" s="237" t="s">
         <v>22</v>
       </c>
       <c r="D27" s="215" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="E27" s="215" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="227" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="B28" s="215" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="C28" t="s">
         <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B29" s="215" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
       <c r="C29" t="s">
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B30" s="215" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="C30" t="s">
         <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B31" s="215" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="C31" t="s">
         <v>22</v>
       </c>
       <c r="D31" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B32" s="215" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="C32" t="s">
         <v>22</v>
       </c>
       <c r="D32" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B33" s="215" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
       <c r="C33" t="s">
         <v>22</v>
       </c>
       <c r="D33" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B34" s="215" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
       <c r="C34" t="s">
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B35" s="215" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
       <c r="C35" t="s">
         <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>797</v>
+        <v>801</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B36" s="215" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
       <c r="C36" t="s">
         <v>22</v>
       </c>
       <c r="D36" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B37" s="215" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C37" t="s">
         <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B38" s="215" t="s">
-        <v>801</v>
+        <v>805</v>
       </c>
       <c r="C38" t="s">
         <v>22</v>
       </c>
       <c r="D38" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B39" s="215" t="s">
-        <v>802</v>
+        <v>806</v>
       </c>
       <c r="C39" t="s">
         <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B40" s="215" t="s">
+        <v>807</v>
+      </c>
+      <c r="C40" t="s">
+        <v>22</v>
+      </c>
+      <c r="D40" t="s">
         <v>803</v>
-      </c>
-      <c r="C40" t="s">
-        <v>22</v>
-      </c>
-      <c r="D40" t="s">
-        <v>799</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="B41" s="215" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C41" t="s">
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B42" s="215" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="C42" t="s">
         <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B43" s="215" t="s">
-        <v>807</v>
+        <v>811</v>
       </c>
       <c r="C43" t="s">
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>808</v>
+        <v>812</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B44" s="215" t="s">
-        <v>809</v>
+        <v>813</v>
       </c>
       <c r="C44" t="s">
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>808</v>
+        <v>812</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B45" s="215" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
       <c r="C45" t="s">
         <v>128</v>
       </c>
       <c r="D45" t="s">
-        <v>811</v>
+        <v>815</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B46" s="215" t="s">
-        <v>813</v>
+        <v>817</v>
       </c>
       <c r="C46" t="s">
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>814</v>
+        <v>818</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B47" s="215" t="s">
-        <v>815</v>
+        <v>819</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B48" s="215" t="s">
-        <v>817</v>
+        <v>821</v>
       </c>
       <c r="C48" t="s">
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B49" s="215" t="s">
-        <v>818</v>
+        <v>822</v>
       </c>
       <c r="C49" t="s">
         <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B50" s="215" t="s">
-        <v>819</v>
+        <v>823</v>
       </c>
       <c r="C50" t="s">
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>820</v>
+        <v>824</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B51" s="215" t="s">
-        <v>821</v>
+        <v>825</v>
       </c>
       <c r="C51" t="s">
         <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B52" s="215" t="s">
-        <v>823</v>
+        <v>827</v>
       </c>
       <c r="C52" t="s">
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>824</v>
+        <v>828</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B53" s="215" t="s">
-        <v>825</v>
+        <v>829</v>
       </c>
       <c r="C53" t="s">
         <v>128</v>
       </c>
       <c r="D53" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>826</v>
+        <v>830</v>
       </c>
       <c r="C54" t="s">
         <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>824</v>
+        <v>828</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>827</v>
+        <v>831</v>
       </c>
       <c r="C55" t="s">
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>828</v>
+        <v>832</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="C56" t="s">
         <v>128</v>
       </c>
       <c r="D56" t="s">
-        <v>830</v>
+        <v>834</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>831</v>
+        <v>835</v>
       </c>
       <c r="C57" t="s">
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>832</v>
+        <v>836</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
       <c r="C58" t="s">
         <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>832</v>
+        <v>836</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>834</v>
+        <v>838</v>
       </c>
       <c r="C59" t="s">
         <v>22</v>
       </c>
       <c r="D59" t="s">
-        <v>832</v>
+        <v>836</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>835</v>
+        <v>839</v>
       </c>
       <c r="C60" t="s">
         <v>128</v>
       </c>
       <c r="D60" t="s">
-        <v>832</v>
+        <v>836</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="274" t="s">
-        <v>836</v>
+        <v>840</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>837</v>
+        <v>841</v>
       </c>
       <c r="C61" t="s">
         <v>22</v>
       </c>
       <c r="D61" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="274" t="s">
-        <v>836</v>
+        <v>840</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>838</v>
+        <v>842</v>
       </c>
       <c r="C62" t="s">
         <v>22</v>
       </c>
       <c r="D62" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="274" t="s">
-        <v>836</v>
+        <v>840</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>839</v>
+        <v>843</v>
       </c>
       <c r="C63" t="s">
         <v>22</v>
       </c>
       <c r="D63" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="C64" t="s">
         <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>841</v>
+        <v>845</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>842</v>
+        <v>846</v>
       </c>
       <c r="C65" t="s">
         <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>841</v>
+        <v>845</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B66" s="215" t="s">
-        <v>843</v>
+        <v>847</v>
       </c>
       <c r="C66" t="s">
         <v>22</v>
       </c>
       <c r="D66" t="s">
-        <v>841</v>
+        <v>845</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="274" t="s">
-        <v>844</v>
+        <v>848</v>
       </c>
       <c r="B67" s="215" t="s">
-        <v>845</v>
+        <v>849</v>
       </c>
       <c r="C67" t="s">
         <v>22</v>
       </c>
       <c r="D67" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="274" t="s">
-        <v>844</v>
+        <v>848</v>
       </c>
       <c r="B68" s="215" t="s">
-        <v>846</v>
+        <v>850</v>
       </c>
       <c r="C68" t="s">
         <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="274" t="s">
-        <v>844</v>
+        <v>848</v>
       </c>
       <c r="B69" s="215" t="s">
-        <v>847</v>
+        <v>851</v>
       </c>
       <c r="C69" t="s">
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B70" s="215" t="s">
-        <v>848</v>
+        <v>852</v>
       </c>
       <c r="C70" t="s">
         <v>22</v>
       </c>
       <c r="D70" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B71" s="215" t="s">
-        <v>850</v>
+        <v>854</v>
       </c>
       <c r="C71" t="s">
         <v>22</v>
       </c>
       <c r="D71" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B72" s="215" t="s">
-        <v>851</v>
+        <v>855</v>
       </c>
       <c r="C72" t="s">
         <v>22</v>
       </c>
       <c r="D72" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="274" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="B73" s="215" t="s">
-        <v>852</v>
+        <v>856</v>
       </c>
       <c r="C73" t="s">
         <v>128</v>
       </c>
       <c r="D73" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
     </row>
   </sheetData>
@@ -16350,336 +16409,336 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="211" t="s">
-        <v>853</v>
+        <v>857</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="212" t="s">
-        <v>854</v>
+        <v>858</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="213" t="s">
-        <v>855</v>
+        <v>859</v>
       </c>
       <c r="B4" s="213" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C4" s="213" t="s">
-        <v>857</v>
+        <v>861</v>
       </c>
       <c r="D4" s="213" t="s">
-        <v>858</v>
+        <v>862</v>
       </c>
       <c r="E4" s="213" t="s">
-        <v>859</v>
+        <v>863</v>
       </c>
       <c r="F4" s="213" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="G4" s="213" t="s">
-        <v>861</v>
+        <v>865</v>
       </c>
       <c r="H4" s="213" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="213" t="s">
-        <v>862</v>
+        <v>866</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="214" t="s">
-        <v>863</v>
+        <v>867</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C5" s="215" t="s">
-        <v>865</v>
+        <v>869</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="F5" s="215" t="s">
-        <v>868</v>
+        <v>872</v>
       </c>
       <c r="G5" s="215" t="s">
-        <v>869</v>
+        <v>873</v>
       </c>
       <c r="H5" s="216" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
       <c r="I5" s="215" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="214" t="s">
-        <v>872</v>
+        <v>876</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>873</v>
+        <v>877</v>
       </c>
       <c r="C6" s="215" t="s">
+        <v>878</v>
+      </c>
+      <c r="D6" s="215" t="s">
+        <v>879</v>
+      </c>
+      <c r="E6" s="215" t="s">
+        <v>880</v>
+      </c>
+      <c r="F6" s="215" t="s">
+        <v>881</v>
+      </c>
+      <c r="G6" s="215" t="s">
+        <v>882</v>
+      </c>
+      <c r="H6" s="217" t="s">
         <v>874</v>
       </c>
-      <c r="D6" s="215" t="s">
-        <v>875</v>
-      </c>
-      <c r="E6" s="215" t="s">
-        <v>876</v>
-      </c>
-      <c r="F6" s="215" t="s">
-        <v>877</v>
-      </c>
-      <c r="G6" s="215" t="s">
-        <v>878</v>
-      </c>
-      <c r="H6" s="217" t="s">
-        <v>870</v>
-      </c>
       <c r="I6" s="215" t="s">
-        <v>879</v>
+        <v>883</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="214" t="s">
-        <v>880</v>
+        <v>884</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>881</v>
+        <v>885</v>
       </c>
       <c r="C7" s="215" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="D7" s="215" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="E7" s="215" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="F7" s="215" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="G7" s="215" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
       <c r="H7" s="217" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
       <c r="I7" s="215" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="214" t="s">
-        <v>888</v>
+        <v>892</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>889</v>
+        <v>893</v>
       </c>
       <c r="C8" s="215" t="s">
-        <v>890</v>
+        <v>894</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>891</v>
+        <v>895</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="F8" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="G8" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="H8" s="216" t="s">
-        <v>892</v>
+        <v>896</v>
       </c>
       <c r="I8" s="215" t="s">
-        <v>893</v>
+        <v>897</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="214" t="s">
-        <v>894</v>
+        <v>898</v>
       </c>
       <c r="B9" s="215" t="s">
+        <v>899</v>
+      </c>
+      <c r="C9" s="215" t="s">
+        <v>900</v>
+      </c>
+      <c r="D9" s="215" t="s">
         <v>895</v>
       </c>
-      <c r="C9" s="215" t="s">
-        <v>896</v>
-      </c>
-      <c r="D9" s="215" t="s">
-        <v>891</v>
-      </c>
       <c r="E9" s="215" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="F9" s="215" t="s">
-        <v>897</v>
+        <v>901</v>
       </c>
       <c r="G9" s="215" t="s">
-        <v>898</v>
+        <v>902</v>
       </c>
       <c r="H9" s="218" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="I9" s="215" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="214" t="s">
-        <v>901</v>
+        <v>905</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>902</v>
+        <v>906</v>
       </c>
       <c r="C10" s="215" t="s">
-        <v>903</v>
+        <v>907</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>904</v>
+        <v>908</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>905</v>
+        <v>909</v>
       </c>
       <c r="F10" s="215" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
       <c r="G10" s="215" t="s">
-        <v>907</v>
+        <v>911</v>
       </c>
       <c r="H10" s="218" t="s">
-        <v>908</v>
+        <v>912</v>
       </c>
       <c r="I10" s="215" t="s">
-        <v>909</v>
+        <v>913</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="214" t="s">
-        <v>910</v>
+        <v>914</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="C11" s="215" t="s">
-        <v>912</v>
+        <v>916</v>
       </c>
       <c r="D11" s="215" t="s">
-        <v>913</v>
+        <v>917</v>
       </c>
       <c r="E11" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="F11" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="G11" s="215" t="s">
-        <v>914</v>
+        <v>918</v>
       </c>
       <c r="H11" s="218" t="s">
-        <v>915</v>
+        <v>919</v>
       </c>
       <c r="I11" s="215" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="214" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
       <c r="B12" s="215" t="s">
+        <v>922</v>
+      </c>
+      <c r="C12" s="215" t="s">
+        <v>923</v>
+      </c>
+      <c r="D12" s="215" t="s">
+        <v>924</v>
+      </c>
+      <c r="E12" s="215" t="s">
+        <v>677</v>
+      </c>
+      <c r="F12" s="215" t="s">
+        <v>677</v>
+      </c>
+      <c r="G12" s="215" t="s">
         <v>918</v>
       </c>
-      <c r="C12" s="215" t="s">
-        <v>919</v>
-      </c>
-      <c r="D12" s="215" t="s">
-        <v>920</v>
-      </c>
-      <c r="E12" s="215" t="s">
-        <v>675</v>
-      </c>
-      <c r="F12" s="215" t="s">
-        <v>675</v>
-      </c>
-      <c r="G12" s="215" t="s">
-        <v>914</v>
-      </c>
       <c r="H12" s="217" t="s">
-        <v>921</v>
+        <v>925</v>
       </c>
       <c r="I12" s="215" t="s">
-        <v>922</v>
+        <v>926</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="214" t="s">
-        <v>923</v>
+        <v>927</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>924</v>
+        <v>928</v>
       </c>
       <c r="C13" s="215" t="s">
-        <v>925</v>
+        <v>929</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="F13" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="G13" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="H13" s="218" t="s">
-        <v>926</v>
+        <v>930</v>
       </c>
       <c r="I13" s="215" t="s">
-        <v>927</v>
+        <v>931</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="214" t="s">
-        <v>928</v>
+        <v>932</v>
       </c>
       <c r="B14" s="215" t="s">
+        <v>933</v>
+      </c>
+      <c r="C14" s="215" t="s">
         <v>929</v>
       </c>
-      <c r="C14" s="215" t="s">
-        <v>925</v>
-      </c>
       <c r="D14" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="F14" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="G14" s="215" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="H14" s="218" t="s">
-        <v>926</v>
+        <v>930</v>
       </c>
       <c r="I14" s="215" t="s">
-        <v>930</v>
+        <v>934</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="304" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>

</xml_diff>

<commit_message>
docs(tracker): corners backfill, the four-league gate bug, and the corrected API plan
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8392F6BC-29ED-474C-88C7-4E2A6287EB8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70448276-8F51-49E3-A6F8-037F033893BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1965" uniqueCount="936">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1999" uniqueCount="949">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -1481,6 +1481,33 @@
   </si>
   <si>
     <t>Raised for COHERENCE, not accuracy - mobile dims below 0.35, so between 0.25 and 0.35 the product recommended a pick while calling its own data limited. Accuracy bands cannot locate a cliff (every 95% CI overlaps; worst band n=5). Costs zero upcoming picks. Not 0.50, which would drop 11 picks on a six-fixture band. Re-derive at n=93</t>
+  </si>
+  <si>
+    <t>Corners coverage backfilled 66% -&gt; 91%</t>
+  </si>
+  <si>
+    <t>+6,913 fixtures, 50,540 rows. The date bound was a 7,500/day budget decision; the plan is Ultra at 75,000/day. Sampled 12 gaps first - 8 returned real data, so most were collection misses. Corners training rows 10,877 -&gt; 14,745</t>
+  </si>
+  <si>
+    <t>collect_league silently skipped 4 leagues incl. EPL</t>
+  </si>
+  <si>
+    <t>Gated on games_path AND names_path existing, so the four leagues with no team_names parquet returned immediately for every non-gamelog stage, logging 'no game log yet' about a 3,800-row file. Found only because the backfill measured per league and those four gained exactly zero</t>
+  </si>
+  <si>
+    <t>Football retrained on fuller corners data</t>
+  </si>
+  <si>
+    <t>football_xgb_v20260813134423. layer1/layer2 byte-identical by hash, only corners changed. MAE 2.120 both sides but the test set grew 35% so not like-for-like; under-10.5 bucket spread 0.149 -&gt; 0.277 and still monotonic, which is the structural read</t>
+  </si>
+  <si>
+    <t>API-Football plan facts corrected in CLAUDE.md</t>
+  </si>
+  <si>
+    <t>Docs</t>
+  </si>
+  <si>
+    <t>Documented as Pro/7,500/day ending 2026-08-29; actually Ultra/75,000/day ending 2026-09-29. Several 'cannot afford' decisions were sized against the old ceiling</t>
   </si>
   <si>
     <t>Legend</t>
@@ -2285,6 +2312,18 @@
   </si>
   <si>
     <t>The completeness floor was recommended on the claim that two measurements agreed the cliff was at 0.35. Measuring with intervals showed neither could locate a cliff at all, and the older one pointed at 0.50 if anywhere. The change went ahead on a different, non-statistical justification (coherence with mobile, zero cost) and the original claim is recorded as wrong rather than quietly replaced. Threshold changes should carry intervals before, not after.</t>
+  </si>
+  <si>
+    <t>Budget-shaped decisions outlive the budget</t>
+  </si>
+  <si>
+    <t>The corners date bound, and the choice not to collect several leagues at all, were correct under 7,500 requests/day and were still being honoured under 75,000. Constraints recorded as engineering decisions should name the budget they assumed, so they can be re-opened when it changes rather than inherited as permanent.</t>
+  </si>
+  <si>
+    <t>Veikkausliiga corners genuinely absent</t>
+  </si>
+  <si>
+    <t>44% coverage after the backfill (from 35%), the worst by a wide margin. Direct re-requests for its 2021 fixtures return empty, so this is provider absence rather than a collection miss. Left as a real gap, not zero-filled.</t>
   </si>
   <si>
     <t>SportIQ — Edge Measurement Plan (P0-P3)</t>
@@ -5267,7 +5306,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R224"/>
+  <dimension ref="A1:R228"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -12015,7 +12054,7 @@
         <v>432</v>
       </c>
       <c r="R198" t="str">
-        <f t="shared" ref="R198:R222" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
+        <f t="shared" ref="R198:R226" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
         <v>E4 ML Football</v>
       </c>
     </row>
@@ -12703,7 +12742,7 @@
         <v>E9 Data Ops</v>
       </c>
     </row>
-    <row r="222" spans="1:18" ht="72" x14ac:dyDescent="0.55000000000000004">
+    <row r="222" spans="1:18" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A222" t="s">
         <v>73</v>
       </c>
@@ -12733,23 +12772,143 @@
         <v>E6 Picks</v>
       </c>
     </row>
-    <row r="224" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A224" s="23" t="s">
+    <row r="223" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A223" t="s">
+        <v>130</v>
+      </c>
+      <c r="B223" t="s">
         <v>481</v>
       </c>
-      <c r="B224" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C224" s="15" t="s">
+      <c r="C223" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D223" t="s">
+        <v>45</v>
+      </c>
+      <c r="E223" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F223" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G223" s="215" t="s">
         <v>482</v>
       </c>
-      <c r="D224" s="17" t="s">
+      <c r="J223" t="s">
+        <v>400</v>
+      </c>
+      <c r="R223" t="str">
+        <f t="shared" si="3"/>
+        <v>E9 Data Ops</v>
+      </c>
+    </row>
+    <row r="224" spans="1:18" ht="72" x14ac:dyDescent="0.55000000000000004">
+      <c r="A224" t="s">
+        <v>130</v>
+      </c>
+      <c r="B224" t="s">
+        <v>483</v>
+      </c>
+      <c r="C224" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D224" t="s">
+        <v>45</v>
+      </c>
+      <c r="E224" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F224" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G224" s="215" t="s">
+        <v>484</v>
+      </c>
+      <c r="J224" t="s">
+        <v>400</v>
+      </c>
+      <c r="R224" t="str">
+        <f t="shared" si="3"/>
+        <v>E9 Data Ops</v>
+      </c>
+    </row>
+    <row r="225" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A225" t="s">
+        <v>99</v>
+      </c>
+      <c r="B225" t="s">
+        <v>485</v>
+      </c>
+      <c r="C225" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D225" t="s">
+        <v>45</v>
+      </c>
+      <c r="E225" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F225" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G225" s="215" t="s">
+        <v>486</v>
+      </c>
+      <c r="J225" t="s">
+        <v>400</v>
+      </c>
+      <c r="R225" t="str">
+        <f t="shared" si="3"/>
+        <v>E8 Model Quality</v>
+      </c>
+    </row>
+    <row r="226" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A226" t="s">
+        <v>130</v>
+      </c>
+      <c r="B226" t="s">
+        <v>487</v>
+      </c>
+      <c r="C226" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D226" t="s">
+        <v>488</v>
+      </c>
+      <c r="E226" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F226" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G226" s="215" t="s">
+        <v>489</v>
+      </c>
+      <c r="J226" t="s">
+        <v>400</v>
+      </c>
+      <c r="R226" t="str">
+        <f t="shared" si="3"/>
+        <v>E9 Data Ops</v>
+      </c>
+    </row>
+    <row r="228" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A228" s="23" t="s">
+        <v>490</v>
+      </c>
+      <c r="B228" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C228" s="15" t="s">
+        <v>491</v>
+      </c>
+      <c r="D228" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="E224" s="21" t="s">
+      <c r="E228" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="F224" s="19" t="s">
+      <c r="F228" s="19" t="s">
         <v>138</v>
       </c>
     </row>
@@ -12774,7 +12933,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="294" t="s">
-        <v>483</v>
+        <v>492</v>
       </c>
       <c r="B1" s="283"/>
       <c r="C1" s="283"/>
@@ -12797,7 +12956,7 @@
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="301" t="s">
-        <v>484</v>
+        <v>493</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -12820,7 +12979,7 @@
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="289" t="s">
-        <v>485</v>
+        <v>494</v>
       </c>
       <c r="B4" s="283"/>
       <c r="C4" s="283"/>
@@ -12843,42 +13002,42 @@
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="35" t="s">
-        <v>486</v>
+        <v>495</v>
       </c>
       <c r="B5" s="279" t="s">
-        <v>487</v>
+        <v>496</v>
       </c>
       <c r="C5" s="280"/>
       <c r="D5" s="281"/>
       <c r="E5" s="284" t="s">
-        <v>488</v>
+        <v>497</v>
       </c>
       <c r="F5" s="280"/>
       <c r="G5" s="281"/>
       <c r="H5" s="284" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="I5" s="280"/>
       <c r="J5" s="281"/>
       <c r="K5" s="279" t="s">
-        <v>490</v>
+        <v>499</v>
       </c>
       <c r="L5" s="280"/>
       <c r="M5" s="281"/>
       <c r="N5" s="286" t="s">
-        <v>491</v>
+        <v>500</v>
       </c>
       <c r="O5" s="280"/>
       <c r="P5" s="281"/>
       <c r="Q5" s="286" t="s">
-        <v>492</v>
+        <v>501</v>
       </c>
       <c r="R5" s="280"/>
       <c r="S5" s="281"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="282" t="s">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="C6" s="283"/>
       <c r="D6" s="283"/>
@@ -12900,7 +13059,7 @@
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="289" t="s">
-        <v>494</v>
+        <v>503</v>
       </c>
       <c r="B7" s="283"/>
       <c r="C7" s="283"/>
@@ -12923,10 +13082,10 @@
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="35" t="s">
-        <v>495</v>
+        <v>504</v>
       </c>
       <c r="B8" s="292" t="s">
-        <v>496</v>
+        <v>505</v>
       </c>
       <c r="C8" s="280"/>
       <c r="D8" s="280"/>
@@ -12937,7 +13096,7 @@
       <c r="I8" s="280"/>
       <c r="J8" s="281"/>
       <c r="K8" s="292" t="s">
-        <v>497</v>
+        <v>506</v>
       </c>
       <c r="L8" s="280"/>
       <c r="M8" s="280"/>
@@ -12950,7 +13109,7 @@
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="282" t="s">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="C9" s="283"/>
       <c r="D9" s="283"/>
@@ -12972,7 +13131,7 @@
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="289" t="s">
-        <v>498</v>
+        <v>507</v>
       </c>
       <c r="B10" s="283"/>
       <c r="C10" s="283"/>
@@ -12995,42 +13154,42 @@
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="35" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="B11" s="279" t="s">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="C11" s="280"/>
       <c r="D11" s="281"/>
       <c r="E11" s="279" t="s">
-        <v>501</v>
+        <v>510</v>
       </c>
       <c r="F11" s="280"/>
       <c r="G11" s="281"/>
       <c r="H11" s="279" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="I11" s="280"/>
       <c r="J11" s="281"/>
       <c r="K11" s="284" t="s">
-        <v>503</v>
+        <v>512</v>
       </c>
       <c r="L11" s="280"/>
       <c r="M11" s="281"/>
       <c r="N11" s="279" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="O11" s="280"/>
       <c r="P11" s="281"/>
       <c r="Q11" s="279" t="s">
-        <v>505</v>
+        <v>514</v>
       </c>
       <c r="R11" s="280"/>
       <c r="S11" s="281"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="282" t="s">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="C12" s="283"/>
       <c r="D12" s="283"/>
@@ -13052,7 +13211,7 @@
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="289" t="s">
-        <v>506</v>
+        <v>515</v>
       </c>
       <c r="B13" s="283"/>
       <c r="C13" s="283"/>
@@ -13075,10 +13234,10 @@
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="35" t="s">
-        <v>507</v>
+        <v>516</v>
       </c>
       <c r="B14" s="287" t="s">
-        <v>508</v>
+        <v>517</v>
       </c>
       <c r="C14" s="280"/>
       <c r="D14" s="280"/>
@@ -13086,7 +13245,7 @@
       <c r="F14" s="280"/>
       <c r="G14" s="281"/>
       <c r="H14" s="287" t="s">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="I14" s="280"/>
       <c r="J14" s="280"/>
@@ -13094,19 +13253,19 @@
       <c r="L14" s="280"/>
       <c r="M14" s="281"/>
       <c r="N14" s="287" t="s">
-        <v>510</v>
+        <v>519</v>
       </c>
       <c r="O14" s="280"/>
       <c r="P14" s="281"/>
       <c r="Q14" s="284" t="s">
-        <v>511</v>
+        <v>520</v>
       </c>
       <c r="R14" s="280"/>
       <c r="S14" s="281"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" s="282" t="s">
-        <v>512</v>
+        <v>521</v>
       </c>
       <c r="C15" s="283"/>
       <c r="D15" s="283"/>
@@ -13128,7 +13287,7 @@
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="289" t="s">
-        <v>513</v>
+        <v>522</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>
@@ -13151,10 +13310,10 @@
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="35" t="s">
-        <v>514</v>
+        <v>523</v>
       </c>
       <c r="B17" s="288" t="s">
-        <v>515</v>
+        <v>524</v>
       </c>
       <c r="C17" s="280"/>
       <c r="D17" s="280"/>
@@ -13162,29 +13321,29 @@
       <c r="F17" s="280"/>
       <c r="G17" s="281"/>
       <c r="H17" s="288" t="s">
-        <v>516</v>
+        <v>525</v>
       </c>
       <c r="I17" s="280"/>
       <c r="J17" s="281"/>
       <c r="K17" s="288" t="s">
-        <v>517</v>
+        <v>526</v>
       </c>
       <c r="L17" s="280"/>
       <c r="M17" s="281"/>
       <c r="N17" s="288" t="s">
-        <v>518</v>
+        <v>527</v>
       </c>
       <c r="O17" s="280"/>
       <c r="P17" s="281"/>
       <c r="Q17" s="288" t="s">
-        <v>519</v>
+        <v>528</v>
       </c>
       <c r="R17" s="280"/>
       <c r="S17" s="281"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="282" t="s">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="C18" s="283"/>
       <c r="D18" s="283"/>
@@ -13206,7 +13365,7 @@
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="289" t="s">
-        <v>520</v>
+        <v>529</v>
       </c>
       <c r="B19" s="283"/>
       <c r="C19" s="283"/>
@@ -13229,10 +13388,10 @@
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="35" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="B20" s="290" t="s">
-        <v>522</v>
+        <v>531</v>
       </c>
       <c r="C20" s="280"/>
       <c r="D20" s="280"/>
@@ -13240,7 +13399,7 @@
       <c r="F20" s="280"/>
       <c r="G20" s="281"/>
       <c r="H20" s="290" t="s">
-        <v>523</v>
+        <v>532</v>
       </c>
       <c r="I20" s="280"/>
       <c r="J20" s="280"/>
@@ -13248,7 +13407,7 @@
       <c r="L20" s="280"/>
       <c r="M20" s="281"/>
       <c r="N20" s="290" t="s">
-        <v>524</v>
+        <v>533</v>
       </c>
       <c r="O20" s="280"/>
       <c r="P20" s="280"/>
@@ -13258,7 +13417,7 @@
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" s="282" t="s">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="C21" s="283"/>
       <c r="D21" s="283"/>
@@ -13280,7 +13439,7 @@
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="289" t="s">
-        <v>525</v>
+        <v>534</v>
       </c>
       <c r="B22" s="283"/>
       <c r="C22" s="283"/>
@@ -13303,10 +13462,10 @@
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="35" t="s">
-        <v>526</v>
+        <v>535</v>
       </c>
       <c r="B23" s="290" t="s">
-        <v>527</v>
+        <v>536</v>
       </c>
       <c r="C23" s="280"/>
       <c r="D23" s="280"/>
@@ -13314,29 +13473,29 @@
       <c r="F23" s="280"/>
       <c r="G23" s="281"/>
       <c r="H23" s="290" t="s">
-        <v>528</v>
+        <v>537</v>
       </c>
       <c r="I23" s="280"/>
       <c r="J23" s="281"/>
       <c r="K23" s="290" t="s">
-        <v>529</v>
+        <v>538</v>
       </c>
       <c r="L23" s="280"/>
       <c r="M23" s="281"/>
       <c r="N23" s="290" t="s">
-        <v>530</v>
+        <v>539</v>
       </c>
       <c r="O23" s="280"/>
       <c r="P23" s="281"/>
       <c r="Q23" s="286" t="s">
-        <v>531</v>
+        <v>540</v>
       </c>
       <c r="R23" s="280"/>
       <c r="S23" s="281"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="295" t="s">
-        <v>532</v>
+        <v>541</v>
       </c>
       <c r="B26" s="283"/>
       <c r="C26" s="283"/>
@@ -13359,42 +13518,42 @@
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="35" t="s">
-        <v>533</v>
+        <v>542</v>
       </c>
       <c r="B27" s="279" t="s">
-        <v>534</v>
+        <v>543</v>
       </c>
       <c r="C27" s="280"/>
       <c r="D27" s="281"/>
       <c r="E27" s="279" t="s">
-        <v>535</v>
+        <v>544</v>
       </c>
       <c r="F27" s="280"/>
       <c r="G27" s="281"/>
       <c r="H27" s="287" t="s">
-        <v>536</v>
+        <v>545</v>
       </c>
       <c r="I27" s="280"/>
       <c r="J27" s="281"/>
       <c r="K27" s="288" t="s">
-        <v>537</v>
+        <v>546</v>
       </c>
       <c r="L27" s="280"/>
       <c r="M27" s="281"/>
       <c r="N27" s="288" t="s">
-        <v>538</v>
+        <v>547</v>
       </c>
       <c r="O27" s="280"/>
       <c r="P27" s="281"/>
       <c r="Q27" s="287" t="s">
-        <v>539</v>
+        <v>548</v>
       </c>
       <c r="R27" s="280"/>
       <c r="S27" s="281"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="289" t="s">
-        <v>540</v>
+        <v>549</v>
       </c>
       <c r="B30" s="283"/>
       <c r="C30" s="283"/>
@@ -13417,7 +13576,7 @@
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="285" t="s">
-        <v>541</v>
+        <v>550</v>
       </c>
       <c r="B31" s="283"/>
       <c r="C31" s="283"/>
@@ -13440,7 +13599,7 @@
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="285" t="s">
-        <v>542</v>
+        <v>551</v>
       </c>
       <c r="B32" s="283"/>
       <c r="C32" s="283"/>
@@ -13463,7 +13622,7 @@
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="285" t="s">
-        <v>543</v>
+        <v>552</v>
       </c>
       <c r="B33" s="283"/>
       <c r="C33" s="283"/>
@@ -13486,7 +13645,7 @@
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="285" t="s">
-        <v>544</v>
+        <v>553</v>
       </c>
       <c r="B34" s="283"/>
       <c r="C34" s="283"/>
@@ -13509,7 +13668,7 @@
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="285" t="s">
-        <v>545</v>
+        <v>554</v>
       </c>
       <c r="B35" s="283"/>
       <c r="C35" s="283"/>
@@ -13532,7 +13691,7 @@
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="285" t="s">
-        <v>546</v>
+        <v>555</v>
       </c>
       <c r="B36" s="283"/>
       <c r="C36" s="283"/>
@@ -13555,7 +13714,7 @@
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="296" t="s">
-        <v>547</v>
+        <v>556</v>
       </c>
       <c r="B37" s="283"/>
       <c r="C37" s="283"/>
@@ -13578,25 +13737,25 @@
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="36" t="s">
-        <v>481</v>
+        <v>490</v>
       </c>
       <c r="B39" s="299" t="s">
-        <v>548</v>
+        <v>557</v>
       </c>
       <c r="C39" s="283"/>
       <c r="D39" s="283"/>
       <c r="E39" s="297" t="s">
-        <v>549</v>
+        <v>558</v>
       </c>
       <c r="F39" s="283"/>
       <c r="G39" s="283"/>
       <c r="H39" s="300" t="s">
-        <v>550</v>
+        <v>559</v>
       </c>
       <c r="I39" s="283"/>
       <c r="J39" s="283"/>
       <c r="K39" s="293" t="s">
-        <v>551</v>
+        <v>560</v>
       </c>
       <c r="L39" s="283"/>
       <c r="M39" s="283"/>
@@ -13606,7 +13765,7 @@
       <c r="O39" s="283"/>
       <c r="P39" s="283"/>
       <c r="Q39" s="298" t="s">
-        <v>552</v>
+        <v>561</v>
       </c>
       <c r="R39" s="283"/>
       <c r="S39" s="283"/>
@@ -13614,11 +13773,11 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H14:M14"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A16:S16"/>
     <mergeCell ref="H20:M20"/>
-    <mergeCell ref="A16:S16"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -13627,13 +13786,14 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -13642,7 +13802,6 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
-    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -13650,7 +13809,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -13699,7 +13858,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>553</v>
+        <v>562</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -13712,19 +13871,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>554</v>
+        <v>563</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>555</v>
+        <v>564</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>556</v>
+        <v>565</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -13908,11 +14067,11 @@
       </c>
       <c r="B11" s="24">
         <f t="shared" si="0"/>
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C11" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D11" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -13924,7 +14083,7 @@
       </c>
       <c r="F11" s="25">
         <f t="shared" si="1"/>
-        <v>0.83333333333333337</v>
+        <v>0.83673469387755106</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -13933,11 +14092,11 @@
       </c>
       <c r="B12" s="24">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C12" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D12" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -13949,7 +14108,7 @@
       </c>
       <c r="F12" s="25">
         <f t="shared" si="1"/>
-        <v>0.625</v>
+        <v>0.65116279069767447</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -14004,15 +14163,15 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="26" t="s">
-        <v>557</v>
+        <v>566</v>
       </c>
       <c r="B16" s="27">
         <f>SUM(B4:B14)</f>
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C16" s="27">
         <f>SUM(C4:C14)</f>
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
@@ -14024,12 +14183,12 @@
       </c>
       <c r="F16" s="28">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.78899082568807344</v>
+        <v>0.7927927927927928</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="41" t="s">
-        <v>558</v>
+        <v>567</v>
       </c>
       <c r="B18" s="42">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -14038,7 +14197,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="43" t="s">
-        <v>559</v>
+        <v>568</v>
       </c>
     </row>
   </sheetData>
@@ -14059,7 +14218,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -14071,7 +14230,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>560</v>
+        <v>569</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -14080,648 +14239,648 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="29" t="s">
-        <v>561</v>
+        <v>570</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>562</v>
+        <v>571</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>563</v>
+        <v>572</v>
       </c>
       <c r="D3" s="29" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="29" t="s">
-        <v>564</v>
+        <v>573</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="30" t="s">
-        <v>565</v>
+        <v>574</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="32" t="s">
-        <v>570</v>
+        <v>579</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="30" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>574</v>
+        <v>583</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>575</v>
+        <v>584</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="32" t="s">
-        <v>576</v>
+        <v>585</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>577</v>
+        <v>586</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="30" t="s">
-        <v>578</v>
+        <v>587</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>574</v>
+        <v>583</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>581</v>
+        <v>590</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="32" t="s">
-        <v>582</v>
+        <v>591</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>583</v>
+        <v>592</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>584</v>
+        <v>593</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="30" t="s">
-        <v>585</v>
+        <v>594</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>586</v>
+        <v>595</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>587</v>
+        <v>596</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="32" t="s">
-        <v>588</v>
+        <v>597</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>574</v>
+        <v>583</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>589</v>
+        <v>598</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="30" t="s">
-        <v>590</v>
+        <v>599</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>574</v>
+        <v>583</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>591</v>
+        <v>600</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>592</v>
+        <v>601</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>593</v>
+        <v>602</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="32" t="s">
-        <v>594</v>
+        <v>603</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>574</v>
+        <v>583</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>592</v>
+        <v>601</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>595</v>
+        <v>604</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="30" t="s">
-        <v>596</v>
+        <v>605</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>597</v>
+        <v>606</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="32" t="s">
-        <v>598</v>
+        <v>607</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>599</v>
+        <v>608</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="30" t="s">
-        <v>600</v>
+        <v>609</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>601</v>
+        <v>610</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>602</v>
+        <v>611</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="32" t="s">
-        <v>603</v>
+        <v>612</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>604</v>
+        <v>613</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="30" t="s">
-        <v>605</v>
+        <v>614</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>574</v>
+        <v>583</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>606</v>
+        <v>615</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="32" t="s">
-        <v>607</v>
+        <v>616</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>608</v>
+        <v>617</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="30" t="s">
-        <v>609</v>
+        <v>618</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>610</v>
+        <v>619</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>612</v>
+        <v>621</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="32" t="s">
-        <v>613</v>
+        <v>622</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>601</v>
+        <v>610</v>
       </c>
       <c r="E21" s="33" t="s">
-        <v>614</v>
+        <v>623</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="30" t="s">
-        <v>615</v>
+        <v>624</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>616</v>
+        <v>625</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>617</v>
+        <v>626</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="32" t="s">
-        <v>618</v>
+        <v>627</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>616</v>
+        <v>625</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>619</v>
+        <v>628</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="30" t="s">
-        <v>620</v>
+        <v>629</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>616</v>
+        <v>625</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E24" s="31" t="s">
-        <v>621</v>
+        <v>630</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="53" t="s">
-        <v>622</v>
+        <v>631</v>
       </c>
       <c r="B25" s="51" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C25" s="54" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E25" s="55" t="s">
-        <v>623</v>
+        <v>632</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="56" t="s">
-        <v>624</v>
+        <v>633</v>
       </c>
       <c r="B26" s="46" t="s">
-        <v>616</v>
+        <v>625</v>
       </c>
       <c r="C26" s="54" t="s">
-        <v>591</v>
+        <v>600</v>
       </c>
       <c r="D26" s="46" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E26" s="57" t="s">
-        <v>625</v>
+        <v>634</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="53" t="s">
-        <v>626</v>
+        <v>635</v>
       </c>
       <c r="B27" s="51" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C27" s="54" t="s">
-        <v>591</v>
+        <v>600</v>
       </c>
       <c r="D27" s="51" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E27" s="55" t="s">
-        <v>627</v>
+        <v>636</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="71" t="s">
-        <v>628</v>
+        <v>637</v>
       </c>
       <c r="B28" s="60" t="s">
+        <v>589</v>
+      </c>
+      <c r="C28" s="67" t="s">
         <v>580</v>
       </c>
-      <c r="C28" s="67" t="s">
-        <v>571</v>
-      </c>
       <c r="D28" s="94" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E28" s="94" t="s">
-        <v>629</v>
+        <v>638</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="72" t="s">
-        <v>630</v>
+        <v>639</v>
       </c>
       <c r="B29" s="65" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C29" s="69" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D29" s="93" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E29" s="93" t="s">
-        <v>631</v>
+        <v>640</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="78" t="s">
-        <v>632</v>
+        <v>641</v>
       </c>
       <c r="B30" s="75" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C30" s="79" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D30" s="75" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E30" s="80" t="s">
-        <v>633</v>
+        <v>642</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="92" t="s">
-        <v>634</v>
+        <v>643</v>
       </c>
       <c r="B31" s="83" t="s">
-        <v>616</v>
+        <v>625</v>
       </c>
       <c r="C31" s="90" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D31" s="83" t="s">
-        <v>635</v>
+        <v>644</v>
       </c>
       <c r="E31" s="93" t="s">
-        <v>636</v>
+        <v>645</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="106" t="s">
-        <v>637</v>
+        <v>646</v>
       </c>
       <c r="B32" s="102" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C32" s="104" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D32" s="102" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E32" s="107" t="s">
-        <v>638</v>
+        <v>647</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="108" t="s">
-        <v>639</v>
+        <v>648</v>
       </c>
       <c r="B33" s="97" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C33" s="104" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D33" s="97" t="s">
-        <v>601</v>
+        <v>610</v>
       </c>
       <c r="E33" s="109" t="s">
-        <v>640</v>
+        <v>649</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="134" t="s">
-        <v>641</v>
+        <v>650</v>
       </c>
       <c r="B34" s="129" t="s">
-        <v>616</v>
+        <v>625</v>
       </c>
       <c r="C34" s="123" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D34" s="129" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E34" s="135" t="s">
-        <v>642</v>
+        <v>651</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="136" t="s">
-        <v>643</v>
+        <v>652</v>
       </c>
       <c r="B35" s="124" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C35" s="132" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D35" s="124" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E35" s="137" t="s">
-        <v>644</v>
+        <v>653</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="74.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="147" t="s">
-        <v>578</v>
+        <v>587</v>
       </c>
       <c r="B36" s="145" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C36" s="148" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="D36" s="153" t="s">
-        <v>645</v>
+        <v>654</v>
       </c>
       <c r="E36" s="153" t="s">
-        <v>646</v>
+        <v>655</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="150" t="s">
-        <v>647</v>
+        <v>656</v>
       </c>
       <c r="B37" s="140" t="s">
-        <v>616</v>
+        <v>625</v>
       </c>
       <c r="C37" s="151" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D37" s="140" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E37" s="152" t="s">
-        <v>648</v>
+        <v>657</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="147" t="s">
-        <v>649</v>
+        <v>658</v>
       </c>
       <c r="B38" s="145" t="s">
-        <v>616</v>
+        <v>625</v>
       </c>
       <c r="C38" s="151" t="s">
-        <v>591</v>
+        <v>600</v>
       </c>
       <c r="D38" s="145" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E38" s="149" t="s">
-        <v>650</v>
+        <v>659</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="160" t="s">
-        <v>651</v>
+        <v>660</v>
       </c>
       <c r="B39" s="157" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C39" s="161" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D39" s="157" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E39" s="162" t="s">
-        <v>652</v>
+        <v>661</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="168" t="s">
-        <v>653</v>
+        <v>662</v>
       </c>
       <c r="B40" s="165" t="s">
-        <v>616</v>
+        <v>625</v>
       </c>
       <c r="C40" s="169" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D40" s="165" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E40" s="170" t="s">
-        <v>654</v>
+        <v>663</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -14729,594 +14888,628 @@
         <v>140</v>
       </c>
       <c r="B41" s="172" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C41" s="173" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D41" s="172" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E41" s="174" t="s">
-        <v>655</v>
+        <v>664</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="188" t="s">
-        <v>656</v>
+        <v>665</v>
       </c>
       <c r="B42" s="183" t="s">
-        <v>616</v>
+        <v>625</v>
       </c>
       <c r="C42" s="177" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D42" s="183" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E42" s="189" t="s">
-        <v>657</v>
+        <v>666</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="190" t="s">
-        <v>658</v>
+        <v>667</v>
       </c>
       <c r="B43" s="178" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C43" s="186" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D43" s="178" t="s">
-        <v>601</v>
+        <v>610</v>
       </c>
       <c r="E43" s="191" t="s">
-        <v>659</v>
+        <v>668</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="188" t="s">
-        <v>660</v>
+        <v>669</v>
       </c>
       <c r="B44" s="183" t="s">
-        <v>616</v>
+        <v>625</v>
       </c>
       <c r="C44" s="186" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D44" s="183" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E44" s="189" t="s">
-        <v>661</v>
+        <v>670</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="190" t="s">
-        <v>662</v>
+        <v>671</v>
       </c>
       <c r="B45" s="178" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C45" s="186" t="s">
-        <v>591</v>
+        <v>600</v>
       </c>
       <c r="D45" s="178" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E45" s="191" t="s">
-        <v>663</v>
+        <v>672</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="206" t="s">
-        <v>664</v>
+        <v>673</v>
       </c>
       <c r="B46" s="194" t="s">
+        <v>589</v>
+      </c>
+      <c r="C46" s="199" t="s">
         <v>580</v>
       </c>
-      <c r="C46" s="199" t="s">
-        <v>571</v>
-      </c>
       <c r="D46" s="194" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E46" s="207" t="s">
-        <v>665</v>
+        <v>674</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="208" t="s">
-        <v>666</v>
+        <v>675</v>
       </c>
       <c r="B47" s="200" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C47" s="203" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D47" s="200" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E47" s="209" t="s">
-        <v>667</v>
+        <v>676</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="206" t="s">
-        <v>668</v>
+        <v>677</v>
       </c>
       <c r="B48" s="194" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C48" s="203" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D48" s="194" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E48" s="207" t="s">
-        <v>669</v>
+        <v>678</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
-        <v>670</v>
+        <v>679</v>
       </c>
       <c r="B49" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C49" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D49" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E49" t="s">
-        <v>671</v>
+        <v>680</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
-        <v>672</v>
+        <v>681</v>
       </c>
       <c r="B50" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C50" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D50" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E50" t="s">
-        <v>673</v>
+        <v>682</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
-        <v>674</v>
+        <v>683</v>
       </c>
       <c r="B51" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C51" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D51" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E51" t="s">
-        <v>675</v>
+        <v>684</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
-        <v>676</v>
+        <v>685</v>
       </c>
       <c r="B52" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C52" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="D52" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E52" t="s">
-        <v>678</v>
+        <v>687</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
-        <v>679</v>
+        <v>688</v>
       </c>
       <c r="B53" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C53" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="D53" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E53" t="s">
-        <v>680</v>
+        <v>689</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="215" t="s">
-        <v>681</v>
+        <v>690</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C54" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="D54" s="215" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E54" s="215" t="s">
-        <v>682</v>
+        <v>691</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="215" t="s">
-        <v>683</v>
+        <v>692</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C55" s="215" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D55" s="215" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E55" s="215" t="s">
-        <v>684</v>
+        <v>693</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="215" t="s">
-        <v>685</v>
+        <v>694</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C56" s="215" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D56" s="215" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E56" s="215" t="s">
-        <v>686</v>
+        <v>695</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="215" t="s">
-        <v>687</v>
+        <v>696</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C57" s="215" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D57" s="215" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E57" s="215" t="s">
-        <v>688</v>
+        <v>697</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="215" t="s">
-        <v>689</v>
+        <v>698</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C58" s="215" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D58" s="215" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E58" s="215" t="s">
-        <v>690</v>
+        <v>699</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="215" t="s">
-        <v>691</v>
+        <v>700</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C59" s="215" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D59" s="215" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E59" s="215" t="s">
-        <v>692</v>
+        <v>701</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="215" t="s">
-        <v>693</v>
+        <v>702</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C60" s="215" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D60" s="215" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E60" s="215" t="s">
-        <v>694</v>
+        <v>703</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="215" t="s">
-        <v>695</v>
+        <v>704</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C61" s="215" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D61" s="215" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E61" s="215" t="s">
-        <v>696</v>
+        <v>705</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="215" t="s">
-        <v>697</v>
+        <v>706</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C62" s="215" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D62" s="215" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E62" s="215" t="s">
-        <v>698</v>
+        <v>707</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="215" t="s">
-        <v>699</v>
+        <v>708</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C63" s="215" t="s">
-        <v>591</v>
+        <v>600</v>
       </c>
       <c r="D63" s="215" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E63" s="215" t="s">
-        <v>700</v>
+        <v>709</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="215" t="s">
-        <v>701</v>
+        <v>710</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C64" s="215" t="s">
-        <v>591</v>
+        <v>600</v>
       </c>
       <c r="D64" s="215" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E64" s="215" t="s">
-        <v>702</v>
+        <v>711</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="129.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="215" t="s">
-        <v>703</v>
+        <v>712</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C65" s="215" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D65" s="215" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E65" s="215" t="s">
-        <v>704</v>
+        <v>713</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="215" t="s">
-        <v>705</v>
+        <v>714</v>
       </c>
       <c r="B66" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C66" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D66" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E66" t="s">
-        <v>706</v>
+        <v>715</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="215" t="s">
-        <v>707</v>
+        <v>716</v>
       </c>
       <c r="B67" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C67" t="s">
-        <v>591</v>
+        <v>600</v>
       </c>
       <c r="D67" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E67" t="s">
-        <v>708</v>
+        <v>717</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="215" t="s">
-        <v>709</v>
+        <v>718</v>
       </c>
       <c r="B68" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C68" t="s">
-        <v>591</v>
+        <v>600</v>
       </c>
       <c r="D68" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E68" t="s">
-        <v>710</v>
+        <v>719</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="215" t="s">
-        <v>711</v>
+        <v>720</v>
       </c>
       <c r="B69" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C69" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D69" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E69" t="s">
-        <v>712</v>
+        <v>721</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="215" t="s">
-        <v>713</v>
+        <v>722</v>
       </c>
       <c r="B70" t="s">
+        <v>589</v>
+      </c>
+      <c r="C70" t="s">
         <v>580</v>
       </c>
-      <c r="C70" t="s">
-        <v>571</v>
-      </c>
       <c r="D70" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E70" t="s">
-        <v>714</v>
+        <v>723</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="215" t="s">
-        <v>715</v>
+        <v>724</v>
       </c>
       <c r="B71" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C71" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="D71" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E71" t="s">
-        <v>716</v>
+        <v>725</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="215" t="s">
-        <v>717</v>
+        <v>726</v>
       </c>
       <c r="B72" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C72" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D72" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E72" t="s">
-        <v>718</v>
+        <v>727</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="215" t="s">
-        <v>719</v>
+        <v>728</v>
       </c>
       <c r="B73" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="C73" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D73" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
       <c r="E73" t="s">
-        <v>720</v>
+        <v>729</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" s="215" t="s">
-        <v>721</v>
+        <v>730</v>
       </c>
       <c r="B74" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C74" t="s">
-        <v>579</v>
+        <v>588</v>
       </c>
       <c r="D74" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E74" t="s">
-        <v>722</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" s="215" t="s">
-        <v>723</v>
+        <v>732</v>
       </c>
       <c r="B75" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C75" t="s">
-        <v>591</v>
+        <v>600</v>
       </c>
       <c r="D75" t="s">
-        <v>611</v>
+        <v>620</v>
       </c>
       <c r="E75" t="s">
-        <v>724</v>
+        <v>733</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A76" s="215" t="s">
+        <v>734</v>
+      </c>
+      <c r="B76" t="s">
+        <v>589</v>
+      </c>
+      <c r="C76" t="s">
+        <v>588</v>
+      </c>
+      <c r="D76" t="s">
+        <v>620</v>
+      </c>
+      <c r="E76" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A77" s="215" t="s">
+        <v>736</v>
+      </c>
+      <c r="B77" t="s">
+        <v>575</v>
+      </c>
+      <c r="C77" t="s">
+        <v>600</v>
+      </c>
+      <c r="D77" t="s">
+        <v>577</v>
+      </c>
+      <c r="E77" t="s">
+        <v>737</v>
       </c>
     </row>
   </sheetData>
@@ -15341,12 +15534,12 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="219" t="s">
-        <v>725</v>
+        <v>738</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="303" t="s">
-        <v>726</v>
+        <v>739</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -15355,1032 +15548,1032 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="220" t="s">
-        <v>727</v>
+        <v>740</v>
       </c>
       <c r="B4" s="220" t="s">
-        <v>561</v>
+        <v>570</v>
       </c>
       <c r="C4" s="220" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="220" t="s">
-        <v>728</v>
+        <v>741</v>
       </c>
       <c r="E4" s="220" t="s">
-        <v>729</v>
+        <v>742</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="221" t="s">
-        <v>730</v>
+        <v>743</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>731</v>
+        <v>744</v>
       </c>
       <c r="C5" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>732</v>
+        <v>745</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>733</v>
+        <v>746</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="221" t="s">
-        <v>730</v>
+        <v>743</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>734</v>
+        <v>747</v>
       </c>
       <c r="C6" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="215" t="s">
-        <v>732</v>
+        <v>745</v>
       </c>
       <c r="E6" s="215" t="s">
-        <v>735</v>
+        <v>748</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="231" t="s">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>737</v>
+        <v>750</v>
       </c>
       <c r="C7" s="232" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="215" t="s">
-        <v>730</v>
+        <v>743</v>
       </c>
       <c r="E7" s="215" t="s">
-        <v>738</v>
+        <v>751</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="223" t="s">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>739</v>
+        <v>752</v>
       </c>
       <c r="C8" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>740</v>
+        <v>753</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>741</v>
+        <v>754</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="223" t="s">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="B9" s="215" t="s">
-        <v>742</v>
+        <v>755</v>
       </c>
       <c r="C9" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="215" t="s">
-        <v>730</v>
+        <v>743</v>
       </c>
       <c r="E9" s="215" t="s">
-        <v>743</v>
+        <v>756</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="224" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>745</v>
+        <v>758</v>
       </c>
       <c r="C10" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>746</v>
+        <v>759</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>747</v>
+        <v>760</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>748</v>
+        <v>761</v>
       </c>
       <c r="C11" t="s">
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>749</v>
+        <v>762</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>750</v>
+        <v>763</v>
       </c>
       <c r="C12" t="s">
         <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>749</v>
+        <v>762</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="224" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>751</v>
+        <v>764</v>
       </c>
       <c r="C13" s="222" t="s">
         <v>128</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>752</v>
+        <v>765</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>753</v>
+        <v>766</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="235" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>754</v>
+        <v>767</v>
       </c>
       <c r="C14" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>755</v>
+        <v>768</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>756</v>
+        <v>769</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="235" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B15" s="215" t="s">
-        <v>757</v>
+        <v>770</v>
       </c>
       <c r="C15" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="215" t="s">
-        <v>752</v>
+        <v>765</v>
       </c>
       <c r="E15" s="215" t="s">
-        <v>758</v>
+        <v>771</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="235" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B16" s="215" t="s">
-        <v>759</v>
+        <v>772</v>
       </c>
       <c r="C16" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="215" t="s">
-        <v>752</v>
+        <v>765</v>
       </c>
       <c r="E16" s="215" t="s">
-        <v>760</v>
+        <v>773</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="225" t="s">
-        <v>761</v>
+        <v>774</v>
       </c>
       <c r="B17" s="215" t="s">
-        <v>762</v>
+        <v>775</v>
       </c>
       <c r="C17" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D17" s="215" t="s">
-        <v>763</v>
+        <v>776</v>
       </c>
       <c r="E17" s="215" t="s">
-        <v>764</v>
+        <v>777</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="225" t="s">
-        <v>761</v>
+        <v>774</v>
       </c>
       <c r="B18" s="215" t="s">
-        <v>765</v>
+        <v>778</v>
       </c>
       <c r="C18" s="223" t="s">
         <v>138</v>
       </c>
       <c r="D18" s="215" t="s">
-        <v>763</v>
+        <v>776</v>
       </c>
       <c r="E18" s="215" t="s">
-        <v>766</v>
+        <v>779</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="226" t="s">
-        <v>767</v>
+        <v>780</v>
       </c>
       <c r="B19" s="215" t="s">
-        <v>768</v>
+        <v>781</v>
       </c>
       <c r="C19" s="225" t="s">
-        <v>769</v>
+        <v>782</v>
       </c>
       <c r="D19" s="215" t="s">
-        <v>732</v>
+        <v>745</v>
       </c>
       <c r="E19" s="215" t="s">
-        <v>770</v>
+        <v>783</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="226" t="s">
-        <v>767</v>
+        <v>780</v>
       </c>
       <c r="B20" s="215" t="s">
-        <v>771</v>
+        <v>784</v>
       </c>
       <c r="C20" s="225" t="s">
-        <v>769</v>
+        <v>782</v>
       </c>
       <c r="D20" s="215" t="s">
-        <v>732</v>
+        <v>745</v>
       </c>
       <c r="E20" s="215" t="s">
-        <v>772</v>
+        <v>785</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="226" t="s">
-        <v>767</v>
+        <v>780</v>
       </c>
       <c r="B21" s="215" t="s">
-        <v>773</v>
+        <v>786</v>
       </c>
       <c r="C21" s="225" t="s">
-        <v>769</v>
+        <v>782</v>
       </c>
       <c r="D21" s="215" t="s">
-        <v>732</v>
+        <v>745</v>
       </c>
       <c r="E21" s="215" t="s">
-        <v>774</v>
+        <v>787</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
     <row r="23" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="229" t="s">
-        <v>730</v>
+        <v>743</v>
       </c>
       <c r="B23" s="215" t="s">
-        <v>775</v>
+        <v>788</v>
       </c>
       <c r="C23" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D23" s="215" t="s">
-        <v>776</v>
+        <v>789</v>
       </c>
       <c r="E23" s="215" t="s">
-        <v>777</v>
+        <v>790</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="230" t="s">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="B24" s="215" t="s">
-        <v>778</v>
+        <v>791</v>
       </c>
       <c r="C24" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D24" s="215" t="s">
-        <v>779</v>
+        <v>792</v>
       </c>
       <c r="E24" s="215" t="s">
-        <v>780</v>
+        <v>793</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="231" t="s">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="B25" s="215" t="s">
-        <v>781</v>
+        <v>794</v>
       </c>
       <c r="C25" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D25" s="215" t="s">
-        <v>782</v>
+        <v>795</v>
       </c>
       <c r="E25" s="215" t="s">
-        <v>783</v>
+        <v>796</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="231" t="s">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="B26" s="215" t="s">
-        <v>784</v>
+        <v>797</v>
       </c>
       <c r="C26" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D26" s="215" t="s">
-        <v>779</v>
+        <v>792</v>
       </c>
       <c r="E26" s="215" t="s">
-        <v>785</v>
+        <v>798</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="235" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B27" s="215" t="s">
-        <v>786</v>
+        <v>799</v>
       </c>
       <c r="C27" s="237" t="s">
         <v>22</v>
       </c>
       <c r="D27" s="215" t="s">
-        <v>749</v>
+        <v>762</v>
       </c>
       <c r="E27" s="215" t="s">
-        <v>787</v>
+        <v>800</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="227" t="s">
-        <v>730</v>
+        <v>743</v>
       </c>
       <c r="B28" s="215" t="s">
-        <v>788</v>
+        <v>801</v>
       </c>
       <c r="C28" t="s">
         <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>789</v>
+        <v>802</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B29" s="215" t="s">
-        <v>790</v>
+        <v>803</v>
       </c>
       <c r="C29" t="s">
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>749</v>
+        <v>762</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B30" s="215" t="s">
-        <v>791</v>
+        <v>804</v>
       </c>
       <c r="C30" t="s">
         <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>792</v>
+        <v>805</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="B31" s="215" t="s">
-        <v>793</v>
+        <v>806</v>
       </c>
       <c r="C31" t="s">
         <v>22</v>
       </c>
       <c r="D31" t="s">
-        <v>794</v>
+        <v>807</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="B32" s="215" t="s">
-        <v>795</v>
+        <v>808</v>
       </c>
       <c r="C32" t="s">
         <v>22</v>
       </c>
       <c r="D32" t="s">
-        <v>796</v>
+        <v>809</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="B33" s="215" t="s">
-        <v>797</v>
+        <v>810</v>
       </c>
       <c r="C33" t="s">
         <v>22</v>
       </c>
       <c r="D33" t="s">
-        <v>794</v>
+        <v>807</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="B34" s="215" t="s">
-        <v>798</v>
+        <v>811</v>
       </c>
       <c r="C34" t="s">
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>799</v>
+        <v>812</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B35" s="215" t="s">
-        <v>800</v>
+        <v>813</v>
       </c>
       <c r="C35" t="s">
         <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>801</v>
+        <v>814</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="B36" s="215" t="s">
-        <v>802</v>
+        <v>815</v>
       </c>
       <c r="C36" t="s">
         <v>22</v>
       </c>
       <c r="D36" t="s">
-        <v>803</v>
+        <v>816</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B37" s="215" t="s">
-        <v>804</v>
+        <v>817</v>
       </c>
       <c r="C37" t="s">
         <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>803</v>
+        <v>816</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
-        <v>761</v>
+        <v>774</v>
       </c>
       <c r="B38" s="215" t="s">
-        <v>805</v>
+        <v>818</v>
       </c>
       <c r="C38" t="s">
         <v>22</v>
       </c>
       <c r="D38" t="s">
-        <v>803</v>
+        <v>816</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="B39" s="215" t="s">
-        <v>806</v>
+        <v>819</v>
       </c>
       <c r="C39" t="s">
         <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>803</v>
+        <v>816</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B40" s="215" t="s">
-        <v>807</v>
+        <v>820</v>
       </c>
       <c r="C40" t="s">
         <v>22</v>
       </c>
       <c r="D40" t="s">
-        <v>803</v>
+        <v>816</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="B41" s="215" t="s">
-        <v>808</v>
+        <v>821</v>
       </c>
       <c r="C41" t="s">
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>809</v>
+        <v>822</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B42" s="215" t="s">
-        <v>810</v>
+        <v>823</v>
       </c>
       <c r="C42" t="s">
         <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>809</v>
+        <v>822</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B43" s="215" t="s">
-        <v>811</v>
+        <v>824</v>
       </c>
       <c r="C43" t="s">
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>812</v>
+        <v>825</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
-        <v>744</v>
+        <v>757</v>
       </c>
       <c r="B44" s="215" t="s">
-        <v>813</v>
+        <v>826</v>
       </c>
       <c r="C44" t="s">
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>812</v>
+        <v>825</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
-        <v>761</v>
+        <v>774</v>
       </c>
       <c r="B45" s="215" t="s">
-        <v>814</v>
+        <v>827</v>
       </c>
       <c r="C45" t="s">
         <v>128</v>
       </c>
       <c r="D45" t="s">
-        <v>815</v>
+        <v>828</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B46" s="215" t="s">
-        <v>817</v>
+        <v>830</v>
       </c>
       <c r="C46" t="s">
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>818</v>
+        <v>831</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B47" s="215" t="s">
-        <v>819</v>
+        <v>832</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>820</v>
+        <v>833</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B48" s="215" t="s">
-        <v>821</v>
+        <v>834</v>
       </c>
       <c r="C48" t="s">
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>820</v>
+        <v>833</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B49" s="215" t="s">
-        <v>822</v>
+        <v>835</v>
       </c>
       <c r="C49" t="s">
         <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>820</v>
+        <v>833</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B50" s="215" t="s">
-        <v>823</v>
+        <v>836</v>
       </c>
       <c r="C50" t="s">
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>824</v>
+        <v>837</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B51" s="215" t="s">
-        <v>825</v>
+        <v>838</v>
       </c>
       <c r="C51" t="s">
         <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>826</v>
+        <v>839</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B52" s="215" t="s">
-        <v>827</v>
+        <v>840</v>
       </c>
       <c r="C52" t="s">
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>828</v>
+        <v>841</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B53" s="215" t="s">
-        <v>829</v>
+        <v>842</v>
       </c>
       <c r="C53" t="s">
         <v>128</v>
       </c>
       <c r="D53" t="s">
-        <v>826</v>
+        <v>839</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>830</v>
+        <v>843</v>
       </c>
       <c r="C54" t="s">
         <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>828</v>
+        <v>841</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>831</v>
+        <v>844</v>
       </c>
       <c r="C55" t="s">
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>832</v>
+        <v>845</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>833</v>
+        <v>846</v>
       </c>
       <c r="C56" t="s">
         <v>128</v>
       </c>
       <c r="D56" t="s">
-        <v>834</v>
+        <v>847</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>835</v>
+        <v>848</v>
       </c>
       <c r="C57" t="s">
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>836</v>
+        <v>849</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>837</v>
+        <v>850</v>
       </c>
       <c r="C58" t="s">
         <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>836</v>
+        <v>849</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>838</v>
+        <v>851</v>
       </c>
       <c r="C59" t="s">
         <v>22</v>
       </c>
       <c r="D59" t="s">
-        <v>836</v>
+        <v>849</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>839</v>
+        <v>852</v>
       </c>
       <c r="C60" t="s">
         <v>128</v>
       </c>
       <c r="D60" t="s">
-        <v>836</v>
+        <v>849</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="274" t="s">
-        <v>840</v>
+        <v>853</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>841</v>
+        <v>854</v>
       </c>
       <c r="C61" t="s">
         <v>22</v>
       </c>
       <c r="D61" t="s">
-        <v>809</v>
+        <v>822</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="274" t="s">
-        <v>840</v>
+        <v>853</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>842</v>
+        <v>855</v>
       </c>
       <c r="C62" t="s">
         <v>22</v>
       </c>
       <c r="D62" t="s">
-        <v>809</v>
+        <v>822</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="274" t="s">
-        <v>840</v>
+        <v>853</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>843</v>
+        <v>856</v>
       </c>
       <c r="C63" t="s">
         <v>22</v>
       </c>
       <c r="D63" t="s">
-        <v>809</v>
+        <v>822</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>844</v>
+        <v>857</v>
       </c>
       <c r="C64" t="s">
         <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>845</v>
+        <v>858</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>846</v>
+        <v>859</v>
       </c>
       <c r="C65" t="s">
         <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>845</v>
+        <v>858</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B66" s="215" t="s">
-        <v>847</v>
+        <v>860</v>
       </c>
       <c r="C66" t="s">
         <v>22</v>
       </c>
       <c r="D66" t="s">
-        <v>845</v>
+        <v>858</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="274" t="s">
-        <v>848</v>
+        <v>861</v>
       </c>
       <c r="B67" s="215" t="s">
-        <v>849</v>
+        <v>862</v>
       </c>
       <c r="C67" t="s">
         <v>22</v>
       </c>
       <c r="D67" t="s">
-        <v>809</v>
+        <v>822</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="274" t="s">
-        <v>848</v>
+        <v>861</v>
       </c>
       <c r="B68" s="215" t="s">
-        <v>850</v>
+        <v>863</v>
       </c>
       <c r="C68" t="s">
         <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>809</v>
+        <v>822</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="274" t="s">
-        <v>848</v>
+        <v>861</v>
       </c>
       <c r="B69" s="215" t="s">
-        <v>851</v>
+        <v>864</v>
       </c>
       <c r="C69" t="s">
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>809</v>
+        <v>822</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B70" s="215" t="s">
-        <v>852</v>
+        <v>865</v>
       </c>
       <c r="C70" t="s">
         <v>22</v>
       </c>
       <c r="D70" t="s">
-        <v>853</v>
+        <v>866</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B71" s="215" t="s">
-        <v>854</v>
+        <v>867</v>
       </c>
       <c r="C71" t="s">
         <v>22</v>
       </c>
       <c r="D71" t="s">
-        <v>853</v>
+        <v>866</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B72" s="215" t="s">
-        <v>855</v>
+        <v>868</v>
       </c>
       <c r="C72" t="s">
         <v>22</v>
       </c>
       <c r="D72" t="s">
-        <v>853</v>
+        <v>866</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="274" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B73" s="215" t="s">
-        <v>856</v>
+        <v>869</v>
       </c>
       <c r="C73" t="s">
         <v>128</v>
       </c>
       <c r="D73" t="s">
-        <v>853</v>
+        <v>866</v>
       </c>
     </row>
   </sheetData>
@@ -16409,336 +16602,336 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="211" t="s">
-        <v>857</v>
+        <v>870</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="212" t="s">
-        <v>858</v>
+        <v>871</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="213" t="s">
-        <v>859</v>
+        <v>872</v>
       </c>
       <c r="B4" s="213" t="s">
-        <v>860</v>
+        <v>873</v>
       </c>
       <c r="C4" s="213" t="s">
-        <v>861</v>
+        <v>874</v>
       </c>
       <c r="D4" s="213" t="s">
-        <v>862</v>
+        <v>875</v>
       </c>
       <c r="E4" s="213" t="s">
-        <v>863</v>
+        <v>876</v>
       </c>
       <c r="F4" s="213" t="s">
-        <v>864</v>
+        <v>877</v>
       </c>
       <c r="G4" s="213" t="s">
-        <v>865</v>
+        <v>878</v>
       </c>
       <c r="H4" s="213" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="213" t="s">
-        <v>866</v>
+        <v>879</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="214" t="s">
-        <v>867</v>
+        <v>880</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>868</v>
+        <v>881</v>
       </c>
       <c r="C5" s="215" t="s">
-        <v>869</v>
+        <v>882</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>870</v>
+        <v>883</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>871</v>
+        <v>884</v>
       </c>
       <c r="F5" s="215" t="s">
-        <v>872</v>
+        <v>885</v>
       </c>
       <c r="G5" s="215" t="s">
-        <v>873</v>
+        <v>886</v>
       </c>
       <c r="H5" s="216" t="s">
-        <v>874</v>
+        <v>887</v>
       </c>
       <c r="I5" s="215" t="s">
-        <v>875</v>
+        <v>888</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="214" t="s">
-        <v>876</v>
+        <v>889</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>877</v>
+        <v>890</v>
       </c>
       <c r="C6" s="215" t="s">
-        <v>878</v>
+        <v>891</v>
       </c>
       <c r="D6" s="215" t="s">
-        <v>879</v>
+        <v>892</v>
       </c>
       <c r="E6" s="215" t="s">
-        <v>880</v>
+        <v>893</v>
       </c>
       <c r="F6" s="215" t="s">
-        <v>881</v>
+        <v>894</v>
       </c>
       <c r="G6" s="215" t="s">
-        <v>882</v>
+        <v>895</v>
       </c>
       <c r="H6" s="217" t="s">
-        <v>874</v>
+        <v>887</v>
       </c>
       <c r="I6" s="215" t="s">
-        <v>883</v>
+        <v>896</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="214" t="s">
-        <v>884</v>
+        <v>897</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>885</v>
+        <v>898</v>
       </c>
       <c r="C7" s="215" t="s">
-        <v>886</v>
+        <v>899</v>
       </c>
       <c r="D7" s="215" t="s">
+        <v>900</v>
+      </c>
+      <c r="E7" s="215" t="s">
+        <v>901</v>
+      </c>
+      <c r="F7" s="215" t="s">
+        <v>902</v>
+      </c>
+      <c r="G7" s="215" t="s">
+        <v>903</v>
+      </c>
+      <c r="H7" s="217" t="s">
         <v>887</v>
       </c>
-      <c r="E7" s="215" t="s">
-        <v>888</v>
-      </c>
-      <c r="F7" s="215" t="s">
-        <v>889</v>
-      </c>
-      <c r="G7" s="215" t="s">
-        <v>890</v>
-      </c>
-      <c r="H7" s="217" t="s">
-        <v>874</v>
-      </c>
       <c r="I7" s="215" t="s">
-        <v>891</v>
+        <v>904</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="214" t="s">
-        <v>892</v>
+        <v>905</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>893</v>
+        <v>906</v>
       </c>
       <c r="C8" s="215" t="s">
-        <v>894</v>
+        <v>907</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>895</v>
+        <v>908</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="F8" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="G8" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="H8" s="216" t="s">
-        <v>896</v>
+        <v>909</v>
       </c>
       <c r="I8" s="215" t="s">
-        <v>897</v>
+        <v>910</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="214" t="s">
-        <v>898</v>
+        <v>911</v>
       </c>
       <c r="B9" s="215" t="s">
-        <v>899</v>
+        <v>912</v>
       </c>
       <c r="C9" s="215" t="s">
-        <v>900</v>
+        <v>913</v>
       </c>
       <c r="D9" s="215" t="s">
-        <v>895</v>
+        <v>908</v>
       </c>
       <c r="E9" s="215" t="s">
-        <v>888</v>
+        <v>901</v>
       </c>
       <c r="F9" s="215" t="s">
-        <v>901</v>
+        <v>914</v>
       </c>
       <c r="G9" s="215" t="s">
-        <v>902</v>
+        <v>915</v>
       </c>
       <c r="H9" s="218" t="s">
-        <v>903</v>
+        <v>916</v>
       </c>
       <c r="I9" s="215" t="s">
-        <v>904</v>
+        <v>917</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="214" t="s">
-        <v>905</v>
+        <v>918</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>906</v>
+        <v>919</v>
       </c>
       <c r="C10" s="215" t="s">
-        <v>907</v>
+        <v>920</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>908</v>
+        <v>921</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>909</v>
+        <v>922</v>
       </c>
       <c r="F10" s="215" t="s">
-        <v>910</v>
+        <v>923</v>
       </c>
       <c r="G10" s="215" t="s">
-        <v>911</v>
+        <v>924</v>
       </c>
       <c r="H10" s="218" t="s">
-        <v>912</v>
+        <v>925</v>
       </c>
       <c r="I10" s="215" t="s">
-        <v>913</v>
+        <v>926</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="214" t="s">
-        <v>914</v>
+        <v>927</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>915</v>
+        <v>928</v>
       </c>
       <c r="C11" s="215" t="s">
-        <v>916</v>
+        <v>929</v>
       </c>
       <c r="D11" s="215" t="s">
-        <v>917</v>
+        <v>930</v>
       </c>
       <c r="E11" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="F11" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="G11" s="215" t="s">
-        <v>918</v>
+        <v>931</v>
       </c>
       <c r="H11" s="218" t="s">
-        <v>919</v>
+        <v>932</v>
       </c>
       <c r="I11" s="215" t="s">
-        <v>920</v>
+        <v>933</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="214" t="s">
-        <v>921</v>
+        <v>934</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>922</v>
+        <v>935</v>
       </c>
       <c r="C12" s="215" t="s">
-        <v>923</v>
+        <v>936</v>
       </c>
       <c r="D12" s="215" t="s">
-        <v>924</v>
+        <v>937</v>
       </c>
       <c r="E12" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="F12" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="G12" s="215" t="s">
-        <v>918</v>
+        <v>931</v>
       </c>
       <c r="H12" s="217" t="s">
-        <v>925</v>
+        <v>938</v>
       </c>
       <c r="I12" s="215" t="s">
-        <v>926</v>
+        <v>939</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="214" t="s">
-        <v>927</v>
+        <v>940</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>928</v>
+        <v>941</v>
       </c>
       <c r="C13" s="215" t="s">
-        <v>929</v>
+        <v>942</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="F13" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="G13" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="H13" s="218" t="s">
-        <v>930</v>
+        <v>943</v>
       </c>
       <c r="I13" s="215" t="s">
-        <v>931</v>
+        <v>944</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="214" t="s">
-        <v>932</v>
+        <v>945</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>933</v>
+        <v>946</v>
       </c>
       <c r="C14" s="215" t="s">
-        <v>929</v>
+        <v>942</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="F14" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="G14" s="215" t="s">
-        <v>677</v>
+        <v>686</v>
       </c>
       <c r="H14" s="218" t="s">
-        <v>930</v>
+        <v>943</v>
       </c>
       <c r="I14" s="215" t="s">
-        <v>934</v>
+        <v>947</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="304" t="s">
-        <v>935</v>
+        <v>948</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>

</xml_diff>

<commit_message>
docs(tracker): budget audit closed; season-2021 xG gap logged as a standing risk
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70448276-8F51-49E3-A6F8-037F033893BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{319D927B-F203-4C76-9FBD-C06E186678B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1999" uniqueCount="949">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2010" uniqueCount="953">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -1508,6 +1508,12 @@
   </si>
   <si>
     <t>Documented as Pro/7,500/day ending 2026-08-29; actually Ultra/75,000/day ending 2026-09-29. Several 'cannot afford' decisions were sized against the old ceiling</t>
+  </si>
+  <si>
+    <t>Budget audit: no further cheap data wins remain</t>
+  </si>
+  <si>
+    <t>Re-checked every budget-shaped decision after the Pro-&gt;Ultra correction. Corners was the only real opportunity (done). Odds cadences are TheRundown/month (unchanged); xG is a different provider with upstream gaps (2021 absent across all 18 leagues); injuries could widen but feed features pruned in d0a24d9. La Liga 24/25 at 70/380 confirmed upstream, not a collection failure</t>
   </si>
   <si>
     <t>Legend</t>
@@ -2324,6 +2330,12 @@
   </si>
   <si>
     <t>44% coverage after the backfill (from 35%), the worst by a wide margin. Direct re-requests for its 2021 fixtures return empty, so this is provider absence rather than a collection miss. Left as a real gap, not zero-filled.</t>
+  </si>
+  <si>
+    <t>Season 2021 has no xG in any league</t>
+  </si>
+  <si>
+    <t>5,413 fixtures in a TRAIN season carry no xG upstream, and 2022 is only 57% covered. xg_for_5/xg_against_5 are Layer 1 features, so roughly a third of the training data scores them as missing. Not fixable by collection - the provider does not have it. Relevant to goals_total being barred for no demonstrated signal: the feature most likely to carry that signal is the one most incomplete in training.</t>
   </si>
   <si>
     <t>SportIQ — Edge Measurement Plan (P0-P3)</t>
@@ -5306,7 +5318,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R228"/>
+  <dimension ref="A1:R229"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -12054,7 +12066,7 @@
         <v>432</v>
       </c>
       <c r="R198" t="str">
-        <f t="shared" ref="R198:R226" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
+        <f t="shared" ref="R198:R227" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
         <v>E4 ML Football</v>
       </c>
     </row>
@@ -12772,7 +12784,7 @@
         <v>E6 Picks</v>
       </c>
     </row>
-    <row r="223" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="223" spans="1:18" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A223" t="s">
         <v>130</v>
       </c>
@@ -12802,7 +12814,7 @@
         <v>E9 Data Ops</v>
       </c>
     </row>
-    <row r="224" spans="1:18" ht="72" x14ac:dyDescent="0.55000000000000004">
+    <row r="224" spans="1:18" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A224" t="s">
         <v>130</v>
       </c>
@@ -12832,7 +12844,7 @@
         <v>E9 Data Ops</v>
       </c>
     </row>
-    <row r="225" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="225" spans="1:18" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A225" t="s">
         <v>99</v>
       </c>
@@ -12862,7 +12874,7 @@
         <v>E8 Model Quality</v>
       </c>
     </row>
-    <row r="226" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="226" spans="1:18" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A226" t="s">
         <v>130</v>
       </c>
@@ -12892,23 +12904,53 @@
         <v>E9 Data Ops</v>
       </c>
     </row>
-    <row r="228" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A228" s="23" t="s">
+    <row r="227" spans="1:18" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A227" t="s">
+        <v>130</v>
+      </c>
+      <c r="B227" t="s">
         <v>490</v>
       </c>
-      <c r="B228" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C228" s="15" t="s">
+      <c r="C227" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D227" t="s">
+        <v>45</v>
+      </c>
+      <c r="E227" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F227" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G227" s="215" t="s">
         <v>491</v>
       </c>
-      <c r="D228" s="17" t="s">
+      <c r="J227" t="s">
+        <v>400</v>
+      </c>
+      <c r="R227" t="str">
+        <f t="shared" si="3"/>
+        <v>E9 Data Ops</v>
+      </c>
+    </row>
+    <row r="229" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A229" s="23" t="s">
+        <v>492</v>
+      </c>
+      <c r="B229" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C229" s="15" t="s">
+        <v>493</v>
+      </c>
+      <c r="D229" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="E228" s="21" t="s">
+      <c r="E229" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="F228" s="19" t="s">
+      <c r="F229" s="19" t="s">
         <v>138</v>
       </c>
     </row>
@@ -12933,7 +12975,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="294" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B1" s="283"/>
       <c r="C1" s="283"/>
@@ -12956,7 +12998,7 @@
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="301" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -12979,7 +13021,7 @@
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="289" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B4" s="283"/>
       <c r="C4" s="283"/>
@@ -13002,42 +13044,42 @@
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="35" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B5" s="279" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="C5" s="280"/>
       <c r="D5" s="281"/>
       <c r="E5" s="284" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="F5" s="280"/>
       <c r="G5" s="281"/>
       <c r="H5" s="284" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="I5" s="280"/>
       <c r="J5" s="281"/>
       <c r="K5" s="279" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="L5" s="280"/>
       <c r="M5" s="281"/>
       <c r="N5" s="286" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="O5" s="280"/>
       <c r="P5" s="281"/>
       <c r="Q5" s="286" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="R5" s="280"/>
       <c r="S5" s="281"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="282" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="C6" s="283"/>
       <c r="D6" s="283"/>
@@ -13059,7 +13101,7 @@
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="289" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B7" s="283"/>
       <c r="C7" s="283"/>
@@ -13082,10 +13124,10 @@
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="35" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B8" s="292" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="C8" s="280"/>
       <c r="D8" s="280"/>
@@ -13096,7 +13138,7 @@
       <c r="I8" s="280"/>
       <c r="J8" s="281"/>
       <c r="K8" s="292" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="L8" s="280"/>
       <c r="M8" s="280"/>
@@ -13109,7 +13151,7 @@
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="282" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="C9" s="283"/>
       <c r="D9" s="283"/>
@@ -13131,7 +13173,7 @@
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="289" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B10" s="283"/>
       <c r="C10" s="283"/>
@@ -13154,42 +13196,42 @@
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="35" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B11" s="279" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="C11" s="280"/>
       <c r="D11" s="281"/>
       <c r="E11" s="279" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="F11" s="280"/>
       <c r="G11" s="281"/>
       <c r="H11" s="279" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="I11" s="280"/>
       <c r="J11" s="281"/>
       <c r="K11" s="284" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="L11" s="280"/>
       <c r="M11" s="281"/>
       <c r="N11" s="279" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="O11" s="280"/>
       <c r="P11" s="281"/>
       <c r="Q11" s="279" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="R11" s="280"/>
       <c r="S11" s="281"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="282" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="C12" s="283"/>
       <c r="D12" s="283"/>
@@ -13211,7 +13253,7 @@
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="289" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B13" s="283"/>
       <c r="C13" s="283"/>
@@ -13234,10 +13276,10 @@
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="35" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B14" s="287" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C14" s="280"/>
       <c r="D14" s="280"/>
@@ -13245,7 +13287,7 @@
       <c r="F14" s="280"/>
       <c r="G14" s="281"/>
       <c r="H14" s="287" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="I14" s="280"/>
       <c r="J14" s="280"/>
@@ -13253,19 +13295,19 @@
       <c r="L14" s="280"/>
       <c r="M14" s="281"/>
       <c r="N14" s="287" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="O14" s="280"/>
       <c r="P14" s="281"/>
       <c r="Q14" s="284" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="R14" s="280"/>
       <c r="S14" s="281"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" s="282" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="C15" s="283"/>
       <c r="D15" s="283"/>
@@ -13287,7 +13329,7 @@
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="289" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>
@@ -13310,10 +13352,10 @@
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="35" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B17" s="288" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C17" s="280"/>
       <c r="D17" s="280"/>
@@ -13321,29 +13363,29 @@
       <c r="F17" s="280"/>
       <c r="G17" s="281"/>
       <c r="H17" s="288" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="I17" s="280"/>
       <c r="J17" s="281"/>
       <c r="K17" s="288" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="L17" s="280"/>
       <c r="M17" s="281"/>
       <c r="N17" s="288" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="O17" s="280"/>
       <c r="P17" s="281"/>
       <c r="Q17" s="288" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="R17" s="280"/>
       <c r="S17" s="281"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="282" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="C18" s="283"/>
       <c r="D18" s="283"/>
@@ -13365,7 +13407,7 @@
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="289" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B19" s="283"/>
       <c r="C19" s="283"/>
@@ -13388,10 +13430,10 @@
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="35" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B20" s="290" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="C20" s="280"/>
       <c r="D20" s="280"/>
@@ -13399,7 +13441,7 @@
       <c r="F20" s="280"/>
       <c r="G20" s="281"/>
       <c r="H20" s="290" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="I20" s="280"/>
       <c r="J20" s="280"/>
@@ -13407,7 +13449,7 @@
       <c r="L20" s="280"/>
       <c r="M20" s="281"/>
       <c r="N20" s="290" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="O20" s="280"/>
       <c r="P20" s="280"/>
@@ -13417,7 +13459,7 @@
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" s="282" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="C21" s="283"/>
       <c r="D21" s="283"/>
@@ -13439,7 +13481,7 @@
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="289" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="B22" s="283"/>
       <c r="C22" s="283"/>
@@ -13462,10 +13504,10 @@
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="35" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B23" s="290" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="C23" s="280"/>
       <c r="D23" s="280"/>
@@ -13473,29 +13515,29 @@
       <c r="F23" s="280"/>
       <c r="G23" s="281"/>
       <c r="H23" s="290" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="I23" s="280"/>
       <c r="J23" s="281"/>
       <c r="K23" s="290" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="L23" s="280"/>
       <c r="M23" s="281"/>
       <c r="N23" s="290" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="O23" s="280"/>
       <c r="P23" s="281"/>
       <c r="Q23" s="286" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="R23" s="280"/>
       <c r="S23" s="281"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="295" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="B26" s="283"/>
       <c r="C26" s="283"/>
@@ -13518,42 +13560,42 @@
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="35" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B27" s="279" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="C27" s="280"/>
       <c r="D27" s="281"/>
       <c r="E27" s="279" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="F27" s="280"/>
       <c r="G27" s="281"/>
       <c r="H27" s="287" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="I27" s="280"/>
       <c r="J27" s="281"/>
       <c r="K27" s="288" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="L27" s="280"/>
       <c r="M27" s="281"/>
       <c r="N27" s="288" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="O27" s="280"/>
       <c r="P27" s="281"/>
       <c r="Q27" s="287" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="R27" s="280"/>
       <c r="S27" s="281"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="289" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="B30" s="283"/>
       <c r="C30" s="283"/>
@@ -13576,7 +13618,7 @@
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="285" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="B31" s="283"/>
       <c r="C31" s="283"/>
@@ -13599,7 +13641,7 @@
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="285" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="B32" s="283"/>
       <c r="C32" s="283"/>
@@ -13622,7 +13664,7 @@
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="285" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="B33" s="283"/>
       <c r="C33" s="283"/>
@@ -13645,7 +13687,7 @@
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="285" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="B34" s="283"/>
       <c r="C34" s="283"/>
@@ -13668,7 +13710,7 @@
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="285" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="B35" s="283"/>
       <c r="C35" s="283"/>
@@ -13691,7 +13733,7 @@
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="285" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B36" s="283"/>
       <c r="C36" s="283"/>
@@ -13714,7 +13756,7 @@
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="296" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="B37" s="283"/>
       <c r="C37" s="283"/>
@@ -13737,25 +13779,25 @@
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="36" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B39" s="299" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="C39" s="283"/>
       <c r="D39" s="283"/>
       <c r="E39" s="297" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="F39" s="283"/>
       <c r="G39" s="283"/>
       <c r="H39" s="300" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="I39" s="283"/>
       <c r="J39" s="283"/>
       <c r="K39" s="293" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="L39" s="283"/>
       <c r="M39" s="283"/>
@@ -13765,7 +13807,7 @@
       <c r="O39" s="283"/>
       <c r="P39" s="283"/>
       <c r="Q39" s="298" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="R39" s="283"/>
       <c r="S39" s="283"/>
@@ -13773,11 +13815,11 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="H20:M20"/>
     <mergeCell ref="A16:S16"/>
-    <mergeCell ref="H20:M20"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -13786,14 +13828,13 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -13802,6 +13843,7 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -13809,7 +13851,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -13858,7 +13900,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -13871,19 +13913,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -14092,11 +14134,11 @@
       </c>
       <c r="B12" s="24">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C12" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D12" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A12,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -14108,7 +14150,7 @@
       </c>
       <c r="F12" s="25">
         <f t="shared" si="1"/>
-        <v>0.65116279069767447</v>
+        <v>0.65909090909090906</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -14163,15 +14205,15 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="26" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="B16" s="27">
         <f>SUM(B4:B14)</f>
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C16" s="27">
         <f>SUM(C4:C14)</f>
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
@@ -14183,12 +14225,12 @@
       </c>
       <c r="F16" s="28">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.7927927927927928</v>
+        <v>0.79372197309417036</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="41" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="B18" s="42">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -14197,7 +14239,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="43" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
     </row>
   </sheetData>
@@ -14218,7 +14260,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -14230,7 +14272,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -14239,648 +14281,648 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="29" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="D3" s="29" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="29" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="30" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="32" t="s">
+        <v>581</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>577</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>582</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>579</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>575</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>580</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>577</v>
-      </c>
       <c r="E5" s="33" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="30" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="32" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="30" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="32" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="30" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="32" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="30" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="32" t="s">
+        <v>605</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>585</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>590</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>603</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>583</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>588</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>601</v>
-      </c>
       <c r="E13" s="33" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="30" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="32" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="30" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="32" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="30" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="32" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="30" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="32" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="E21" s="33" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="30" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="32" t="s">
+        <v>629</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>627</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>625</v>
-      </c>
       <c r="C23" s="17" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="30" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E24" s="31" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="53" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="B25" s="51" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C25" s="54" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E25" s="55" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="56" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="B26" s="46" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C26" s="54" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D26" s="46" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E26" s="57" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="53" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="B27" s="51" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C27" s="54" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D27" s="51" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E27" s="55" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="71" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="B28" s="60" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C28" s="67" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D28" s="94" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E28" s="94" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="72" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="B29" s="65" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C29" s="69" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D29" s="93" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E29" s="93" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="78" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="B30" s="75" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C30" s="79" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D30" s="75" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E30" s="80" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="92" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="B31" s="83" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C31" s="90" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D31" s="83" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="E31" s="93" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="106" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="B32" s="102" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C32" s="104" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D32" s="102" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E32" s="107" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="108" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="B33" s="97" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C33" s="104" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D33" s="97" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="E33" s="109" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="134" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="B34" s="129" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C34" s="123" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D34" s="129" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E34" s="135" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="136" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="B35" s="124" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C35" s="132" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D35" s="124" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E35" s="137" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="74.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="147" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="B36" s="145" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C36" s="148" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="D36" s="153" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="E36" s="153" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="150" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="B37" s="140" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C37" s="151" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D37" s="140" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E37" s="152" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="147" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="B38" s="145" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C38" s="151" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D38" s="145" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E38" s="149" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="160" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="B39" s="157" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C39" s="161" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D39" s="157" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E39" s="162" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="168" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="B40" s="165" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C40" s="169" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D40" s="165" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E40" s="170" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -14888,628 +14930,645 @@
         <v>140</v>
       </c>
       <c r="B41" s="172" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C41" s="173" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D41" s="172" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E41" s="174" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="188" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="B42" s="183" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C42" s="177" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D42" s="183" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E42" s="189" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="190" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="B43" s="178" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C43" s="186" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D43" s="178" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="E43" s="191" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="188" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="B44" s="183" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C44" s="186" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D44" s="183" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E44" s="189" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="190" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="B45" s="178" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C45" s="186" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D45" s="178" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E45" s="191" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="206" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="B46" s="194" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C46" s="199" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D46" s="194" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E46" s="207" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="208" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="B47" s="200" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C47" s="203" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D47" s="200" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E47" s="209" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="206" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="B48" s="194" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C48" s="203" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D48" s="194" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E48" s="207" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="B49" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C49" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D49" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E49" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="B50" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C50" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D50" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E50" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="B51" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C51" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D51" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E51" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="B52" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C52" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="D52" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E52" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
+        <v>690</v>
+      </c>
+      <c r="B53" t="s">
+        <v>591</v>
+      </c>
+      <c r="C53" t="s">
         <v>688</v>
       </c>
-      <c r="B53" t="s">
-        <v>589</v>
-      </c>
-      <c r="C53" t="s">
-        <v>686</v>
-      </c>
       <c r="D53" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E53" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="215" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C54" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="D54" s="215" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E54" s="215" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="215" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C55" s="215" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D55" s="215" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E55" s="215" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="215" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C56" s="215" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D56" s="215" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E56" s="215" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="215" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C57" s="215" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D57" s="215" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E57" s="215" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="215" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C58" s="215" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D58" s="215" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E58" s="215" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="215" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C59" s="215" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D59" s="215" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E59" s="215" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="215" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C60" s="215" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D60" s="215" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E60" s="215" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="215" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C61" s="215" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D61" s="215" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E61" s="215" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="215" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C62" s="215" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D62" s="215" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E62" s="215" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="215" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C63" s="215" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D63" s="215" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E63" s="215" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="215" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C64" s="215" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D64" s="215" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E64" s="215" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="129.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="215" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C65" s="215" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D65" s="215" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E65" s="215" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="215" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="B66" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C66" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D66" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E66" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="215" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="B67" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C67" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D67" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E67" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="215" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="B68" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C68" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D68" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E68" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="215" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="B69" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C69" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D69" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E69" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="215" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="B70" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C70" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D70" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E70" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="215" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="B71" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C71" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D71" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E71" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="215" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="B72" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C72" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D72" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E72" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="215" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="B73" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C73" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D73" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E73" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" s="215" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="B74" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C74" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D74" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E74" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" s="215" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="B75" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C75" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D75" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E75" t="s">
-        <v>733</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A76" s="215" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="B76" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C76" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D76" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E76" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A77" s="215" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="B77" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C77" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D77" t="s">
+        <v>579</v>
+      </c>
+      <c r="E77" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A78" s="215" t="s">
+        <v>740</v>
+      </c>
+      <c r="B78" t="s">
         <v>577</v>
       </c>
-      <c r="E77" t="s">
-        <v>737</v>
+      <c r="C78" t="s">
+        <v>590</v>
+      </c>
+      <c r="D78" t="s">
+        <v>579</v>
+      </c>
+      <c r="E78" t="s">
+        <v>741</v>
       </c>
     </row>
   </sheetData>
@@ -15534,12 +15593,12 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="219" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="303" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -15548,1032 +15607,1032 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="220" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B4" s="220" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="C4" s="220" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="220" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="E4" s="220" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="221" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="C5" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="221" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
       <c r="C6" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="215" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="E6" s="215" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="231" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="C7" s="232" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="215" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="E7" s="215" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="223" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="C8" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="223" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B9" s="215" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="C9" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="215" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="E9" s="215" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="224" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="C10" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="C11" t="s">
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="C12" t="s">
         <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="224" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="C13" s="222" t="s">
         <v>128</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="235" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="C14" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>769</v>
+        <v>773</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="235" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B15" s="215" t="s">
-        <v>770</v>
+        <v>774</v>
       </c>
       <c r="C15" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="215" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="E15" s="215" t="s">
-        <v>771</v>
+        <v>775</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="235" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B16" s="215" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="C16" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="215" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="E16" s="215" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="225" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="B17" s="215" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
       <c r="C17" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D17" s="215" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="E17" s="215" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="225" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="B18" s="215" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
       <c r="C18" s="223" t="s">
         <v>138</v>
       </c>
       <c r="D18" s="215" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="E18" s="215" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="226" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="B19" s="215" t="s">
-        <v>781</v>
+        <v>785</v>
       </c>
       <c r="C19" s="225" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="D19" s="215" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="E19" s="215" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="226" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="B20" s="215" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="C20" s="225" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="D20" s="215" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="E20" s="215" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="226" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="B21" s="215" t="s">
+        <v>790</v>
+      </c>
+      <c r="C21" s="225" t="s">
         <v>786</v>
       </c>
-      <c r="C21" s="225" t="s">
-        <v>782</v>
-      </c>
       <c r="D21" s="215" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="E21" s="215" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
     <row r="23" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="229" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="B23" s="215" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="C23" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D23" s="215" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="E23" s="215" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="230" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B24" s="215" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="C24" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D24" s="215" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="E24" s="215" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="231" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B25" s="215" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
       <c r="C25" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D25" s="215" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
       <c r="E25" s="215" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="231" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B26" s="215" t="s">
-        <v>797</v>
+        <v>801</v>
       </c>
       <c r="C26" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D26" s="215" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="E26" s="215" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="235" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B27" s="215" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
       <c r="C27" s="237" t="s">
         <v>22</v>
       </c>
       <c r="D27" s="215" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
       <c r="E27" s="215" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="227" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="B28" s="215" t="s">
-        <v>801</v>
+        <v>805</v>
       </c>
       <c r="C28" t="s">
         <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>802</v>
+        <v>806</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B29" s="215" t="s">
-        <v>803</v>
+        <v>807</v>
       </c>
       <c r="C29" t="s">
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B30" s="215" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C30" t="s">
         <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B31" s="215" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="C31" t="s">
         <v>22</v>
       </c>
       <c r="D31" t="s">
-        <v>807</v>
+        <v>811</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B32" s="215" t="s">
-        <v>808</v>
+        <v>812</v>
       </c>
       <c r="C32" t="s">
         <v>22</v>
       </c>
       <c r="D32" t="s">
-        <v>809</v>
+        <v>813</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B33" s="215" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
       <c r="C33" t="s">
         <v>22</v>
       </c>
       <c r="D33" t="s">
-        <v>807</v>
+        <v>811</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B34" s="215" t="s">
-        <v>811</v>
+        <v>815</v>
       </c>
       <c r="C34" t="s">
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B35" s="215" t="s">
-        <v>813</v>
+        <v>817</v>
       </c>
       <c r="C35" t="s">
         <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>814</v>
+        <v>818</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B36" s="215" t="s">
-        <v>815</v>
+        <v>819</v>
       </c>
       <c r="C36" t="s">
         <v>22</v>
       </c>
       <c r="D36" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B37" s="215" t="s">
-        <v>817</v>
+        <v>821</v>
       </c>
       <c r="C37" t="s">
         <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="B38" s="215" t="s">
-        <v>818</v>
+        <v>822</v>
       </c>
       <c r="C38" t="s">
         <v>22</v>
       </c>
       <c r="D38" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B39" s="215" t="s">
-        <v>819</v>
+        <v>823</v>
       </c>
       <c r="C39" t="s">
         <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B40" s="215" t="s">
+        <v>824</v>
+      </c>
+      <c r="C40" t="s">
+        <v>22</v>
+      </c>
+      <c r="D40" t="s">
         <v>820</v>
-      </c>
-      <c r="C40" t="s">
-        <v>22</v>
-      </c>
-      <c r="D40" t="s">
-        <v>816</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B41" s="215" t="s">
-        <v>821</v>
+        <v>825</v>
       </c>
       <c r="C41" t="s">
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B42" s="215" t="s">
-        <v>823</v>
+        <v>827</v>
       </c>
       <c r="C42" t="s">
         <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B43" s="215" t="s">
-        <v>824</v>
+        <v>828</v>
       </c>
       <c r="C43" t="s">
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>825</v>
+        <v>829</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="B44" s="215" t="s">
-        <v>826</v>
+        <v>830</v>
       </c>
       <c r="C44" t="s">
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>825</v>
+        <v>829</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="B45" s="215" t="s">
-        <v>827</v>
+        <v>831</v>
       </c>
       <c r="C45" t="s">
         <v>128</v>
       </c>
       <c r="D45" t="s">
-        <v>828</v>
+        <v>832</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B46" s="215" t="s">
-        <v>830</v>
+        <v>834</v>
       </c>
       <c r="C46" t="s">
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>831</v>
+        <v>835</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B47" s="215" t="s">
-        <v>832</v>
+        <v>836</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B48" s="215" t="s">
-        <v>834</v>
+        <v>838</v>
       </c>
       <c r="C48" t="s">
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B49" s="215" t="s">
-        <v>835</v>
+        <v>839</v>
       </c>
       <c r="C49" t="s">
         <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B50" s="215" t="s">
-        <v>836</v>
+        <v>840</v>
       </c>
       <c r="C50" t="s">
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>837</v>
+        <v>841</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B51" s="215" t="s">
-        <v>838</v>
+        <v>842</v>
       </c>
       <c r="C51" t="s">
         <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>839</v>
+        <v>843</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B52" s="215" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="C52" t="s">
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>841</v>
+        <v>845</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B53" s="215" t="s">
-        <v>842</v>
+        <v>846</v>
       </c>
       <c r="C53" t="s">
         <v>128</v>
       </c>
       <c r="D53" t="s">
-        <v>839</v>
+        <v>843</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>843</v>
+        <v>847</v>
       </c>
       <c r="C54" t="s">
         <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>841</v>
+        <v>845</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>844</v>
+        <v>848</v>
       </c>
       <c r="C55" t="s">
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>845</v>
+        <v>849</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>846</v>
+        <v>850</v>
       </c>
       <c r="C56" t="s">
         <v>128</v>
       </c>
       <c r="D56" t="s">
-        <v>847</v>
+        <v>851</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>848</v>
+        <v>852</v>
       </c>
       <c r="C57" t="s">
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>850</v>
+        <v>854</v>
       </c>
       <c r="C58" t="s">
         <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>851</v>
+        <v>855</v>
       </c>
       <c r="C59" t="s">
         <v>22</v>
       </c>
       <c r="D59" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>852</v>
+        <v>856</v>
       </c>
       <c r="C60" t="s">
         <v>128</v>
       </c>
       <c r="D60" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="274" t="s">
-        <v>853</v>
+        <v>857</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>854</v>
+        <v>858</v>
       </c>
       <c r="C61" t="s">
         <v>22</v>
       </c>
       <c r="D61" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="274" t="s">
-        <v>853</v>
+        <v>857</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>855</v>
+        <v>859</v>
       </c>
       <c r="C62" t="s">
         <v>22</v>
       </c>
       <c r="D62" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="274" t="s">
-        <v>853</v>
+        <v>857</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C63" t="s">
         <v>22</v>
       </c>
       <c r="D63" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>857</v>
+        <v>861</v>
       </c>
       <c r="C64" t="s">
         <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>858</v>
+        <v>862</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>859</v>
+        <v>863</v>
       </c>
       <c r="C65" t="s">
         <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>858</v>
+        <v>862</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B66" s="215" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C66" t="s">
         <v>22</v>
       </c>
       <c r="D66" t="s">
-        <v>858</v>
+        <v>862</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="274" t="s">
-        <v>861</v>
+        <v>865</v>
       </c>
       <c r="B67" s="215" t="s">
-        <v>862</v>
+        <v>866</v>
       </c>
       <c r="C67" t="s">
         <v>22</v>
       </c>
       <c r="D67" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="274" t="s">
-        <v>861</v>
+        <v>865</v>
       </c>
       <c r="B68" s="215" t="s">
-        <v>863</v>
+        <v>867</v>
       </c>
       <c r="C68" t="s">
         <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="274" t="s">
-        <v>861</v>
+        <v>865</v>
       </c>
       <c r="B69" s="215" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C69" t="s">
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B70" s="215" t="s">
-        <v>865</v>
+        <v>869</v>
       </c>
       <c r="C70" t="s">
         <v>22</v>
       </c>
       <c r="D70" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B71" s="215" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="C71" t="s">
         <v>22</v>
       </c>
       <c r="D71" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B72" s="215" t="s">
-        <v>868</v>
+        <v>872</v>
       </c>
       <c r="C72" t="s">
         <v>22</v>
       </c>
       <c r="D72" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="274" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
       <c r="B73" s="215" t="s">
-        <v>869</v>
+        <v>873</v>
       </c>
       <c r="C73" t="s">
         <v>128</v>
       </c>
       <c r="D73" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
     </row>
   </sheetData>
@@ -16602,336 +16661,336 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="211" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="212" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="213" t="s">
-        <v>872</v>
+        <v>876</v>
       </c>
       <c r="B4" s="213" t="s">
-        <v>873</v>
+        <v>877</v>
       </c>
       <c r="C4" s="213" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="D4" s="213" t="s">
-        <v>875</v>
+        <v>879</v>
       </c>
       <c r="E4" s="213" t="s">
-        <v>876</v>
+        <v>880</v>
       </c>
       <c r="F4" s="213" t="s">
-        <v>877</v>
+        <v>881</v>
       </c>
       <c r="G4" s="213" t="s">
-        <v>878</v>
+        <v>882</v>
       </c>
       <c r="H4" s="213" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="213" t="s">
-        <v>879</v>
+        <v>883</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="214" t="s">
-        <v>880</v>
+        <v>884</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>881</v>
+        <v>885</v>
       </c>
       <c r="C5" s="215" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="F5" s="215" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="G5" s="215" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
       <c r="H5" s="216" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="I5" s="215" t="s">
-        <v>888</v>
+        <v>892</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="214" t="s">
-        <v>889</v>
+        <v>893</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>890</v>
+        <v>894</v>
       </c>
       <c r="C6" s="215" t="s">
+        <v>895</v>
+      </c>
+      <c r="D6" s="215" t="s">
+        <v>896</v>
+      </c>
+      <c r="E6" s="215" t="s">
+        <v>897</v>
+      </c>
+      <c r="F6" s="215" t="s">
+        <v>898</v>
+      </c>
+      <c r="G6" s="215" t="s">
+        <v>899</v>
+      </c>
+      <c r="H6" s="217" t="s">
         <v>891</v>
       </c>
-      <c r="D6" s="215" t="s">
-        <v>892</v>
-      </c>
-      <c r="E6" s="215" t="s">
-        <v>893</v>
-      </c>
-      <c r="F6" s="215" t="s">
-        <v>894</v>
-      </c>
-      <c r="G6" s="215" t="s">
-        <v>895</v>
-      </c>
-      <c r="H6" s="217" t="s">
-        <v>887</v>
-      </c>
       <c r="I6" s="215" t="s">
-        <v>896</v>
+        <v>900</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="214" t="s">
-        <v>897</v>
+        <v>901</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>898</v>
+        <v>902</v>
       </c>
       <c r="C7" s="215" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="D7" s="215" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="E7" s="215" t="s">
-        <v>901</v>
+        <v>905</v>
       </c>
       <c r="F7" s="215" t="s">
-        <v>902</v>
+        <v>906</v>
       </c>
       <c r="G7" s="215" t="s">
-        <v>903</v>
+        <v>907</v>
       </c>
       <c r="H7" s="217" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="I7" s="215" t="s">
-        <v>904</v>
+        <v>908</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="214" t="s">
-        <v>905</v>
+        <v>909</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
       <c r="C8" s="215" t="s">
-        <v>907</v>
+        <v>911</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>908</v>
+        <v>912</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="F8" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="G8" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="H8" s="216" t="s">
-        <v>909</v>
+        <v>913</v>
       </c>
       <c r="I8" s="215" t="s">
-        <v>910</v>
+        <v>914</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="214" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="B9" s="215" t="s">
+        <v>916</v>
+      </c>
+      <c r="C9" s="215" t="s">
+        <v>917</v>
+      </c>
+      <c r="D9" s="215" t="s">
         <v>912</v>
       </c>
-      <c r="C9" s="215" t="s">
-        <v>913</v>
-      </c>
-      <c r="D9" s="215" t="s">
-        <v>908</v>
-      </c>
       <c r="E9" s="215" t="s">
-        <v>901</v>
+        <v>905</v>
       </c>
       <c r="F9" s="215" t="s">
-        <v>914</v>
+        <v>918</v>
       </c>
       <c r="G9" s="215" t="s">
-        <v>915</v>
+        <v>919</v>
       </c>
       <c r="H9" s="218" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
       <c r="I9" s="215" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="214" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
       <c r="C10" s="215" t="s">
-        <v>920</v>
+        <v>924</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>921</v>
+        <v>925</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>922</v>
+        <v>926</v>
       </c>
       <c r="F10" s="215" t="s">
-        <v>923</v>
+        <v>927</v>
       </c>
       <c r="G10" s="215" t="s">
-        <v>924</v>
+        <v>928</v>
       </c>
       <c r="H10" s="218" t="s">
-        <v>925</v>
+        <v>929</v>
       </c>
       <c r="I10" s="215" t="s">
-        <v>926</v>
+        <v>930</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="214" t="s">
-        <v>927</v>
+        <v>931</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>928</v>
+        <v>932</v>
       </c>
       <c r="C11" s="215" t="s">
-        <v>929</v>
+        <v>933</v>
       </c>
       <c r="D11" s="215" t="s">
-        <v>930</v>
+        <v>934</v>
       </c>
       <c r="E11" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="F11" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="G11" s="215" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="H11" s="218" t="s">
-        <v>932</v>
+        <v>936</v>
       </c>
       <c r="I11" s="215" t="s">
-        <v>933</v>
+        <v>937</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="214" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="B12" s="215" t="s">
+        <v>939</v>
+      </c>
+      <c r="C12" s="215" t="s">
+        <v>940</v>
+      </c>
+      <c r="D12" s="215" t="s">
+        <v>941</v>
+      </c>
+      <c r="E12" s="215" t="s">
+        <v>688</v>
+      </c>
+      <c r="F12" s="215" t="s">
+        <v>688</v>
+      </c>
+      <c r="G12" s="215" t="s">
         <v>935</v>
       </c>
-      <c r="C12" s="215" t="s">
-        <v>936</v>
-      </c>
-      <c r="D12" s="215" t="s">
-        <v>937</v>
-      </c>
-      <c r="E12" s="215" t="s">
-        <v>686</v>
-      </c>
-      <c r="F12" s="215" t="s">
-        <v>686</v>
-      </c>
-      <c r="G12" s="215" t="s">
-        <v>931</v>
-      </c>
       <c r="H12" s="217" t="s">
-        <v>938</v>
+        <v>942</v>
       </c>
       <c r="I12" s="215" t="s">
-        <v>939</v>
+        <v>943</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="214" t="s">
-        <v>940</v>
+        <v>944</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>941</v>
+        <v>945</v>
       </c>
       <c r="C13" s="215" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="F13" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="G13" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="H13" s="218" t="s">
-        <v>943</v>
+        <v>947</v>
       </c>
       <c r="I13" s="215" t="s">
-        <v>944</v>
+        <v>948</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="214" t="s">
-        <v>945</v>
+        <v>949</v>
       </c>
       <c r="B14" s="215" t="s">
+        <v>950</v>
+      </c>
+      <c r="C14" s="215" t="s">
         <v>946</v>
       </c>
-      <c r="C14" s="215" t="s">
-        <v>942</v>
-      </c>
       <c r="D14" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="F14" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="G14" s="215" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="H14" s="218" t="s">
-        <v>943</v>
+        <v>947</v>
       </c>
       <c r="I14" s="215" t="s">
-        <v>947</v>
+        <v>951</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="304" t="s">
-        <v>948</v>
+        <v>952</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>

</xml_diff>

<commit_message>
docs(tracker): 1X2 calibration instruments, per-fixture outputs, settled-card fix
Three Delivery Board rows and four Risks & Decisions entries: the history
rewrite and its measured bias direction, isotonic calibration on 1X2 showing
no held-out benefit, the model's inability to discriminate draws, and the
xG train/test availability mismatch.

Recalculated through Excel COM so Epic Summary caches values (Unassigned 0,
overall 180/226). PowerShell's COM binding failed with "Interface not
registered" and printed a success line anyway; late-bound pywin32 works.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{319D927B-F203-4C76-9FBD-C06E186678B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{594F2C9E-6E00-4AD0-B1ED-413FA26F489F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2010" uniqueCount="953">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2045" uniqueCount="964">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -1514,6 +1514,15 @@
   </si>
   <si>
     <t>Re-checked every budget-shaped decision after the Pro-&gt;Ultra correction. Corners was the only real opportunity (done). Odds cadences are TheRundown/month (unchanged); xG is a different provider with upstream gaps (2021 absent across all 18 leagues); injuries could widen but feed features pruned in d0a24d9. La Liga 24/25 at 70/380 confirmed upstream, not a collection failure</t>
+  </si>
+  <si>
+    <t>1X2 held-out log loss / Brier / ECE / reliability</t>
+  </si>
+  <si>
+    <t>Per-fixture test outputs saved (comparisons now joinable)</t>
+  </si>
+  <si>
+    <t>Settled cards no longer re-gated by a tightened floor</t>
   </si>
   <si>
     <t>Legend</t>
@@ -2336,6 +2345,30 @@
   </si>
   <si>
     <t>5,413 fixtures in a TRAIN season carry no xG upstream, and 2022 is only 57% covered. xg_for_5/xg_against_5 are Layer 1 features, so roughly a third of the training data scores them as missing. Not fixable by collection - the provider does not have it. Relevant to goals_total being barred for no demonstrated signal: the feature most likely to carry that signal is the one most incomplete in training.</t>
+  </si>
+  <si>
+    <t>A tightening guard rewrote published history</t>
+  </si>
+  <si>
+    <t>MIN_FEATURE_COMPLETENESS 0.25 -&gt; 0.35 deleted 21 already-published picks from past cards (9 Scottish Prem), because best_pick is recomputed per request rather than stored. The measurement that justified the raise said 'zero upcoming picks lost' - true, and the wrong population. Not neutral: sub-0.35 picks run 0.2857 accuracy vs 0.5263 above, so filtering them made the visible record better than the real one. Settled fixtures are now exempt from that one guard only - exempting the others ADDED picks never shown, which is the same defect. pick_snapshots (nothing before 2026-08-10) is the only real fix.</t>
+  </si>
+  <si>
+    <t>Isotonic calibration on 1X2 may not be earning its place</t>
+  </si>
+  <si>
+    <t>First held-out measurement after months in the pipeline: log loss 1.0179 calibrated vs 1.0148 raw, multiclass Brier identical to 4dp, ECE 0.0143. Not harmful at this size, but no evidence it helps. Re-measure before treating the step as load-bearing.</t>
+  </si>
+  <si>
+    <t>The model cannot discriminate draws</t>
+  </si>
+  <si>
+    <t>92% of test fixtures (5,023 of 5,487) receive a draw probability between 0.2 and 0.3, observed 0.257 - correct on average and carrying no per-fixture information. The 1X2 analogue of the goals_total finding, invisible until per-class reliability existed because RPS averages it away. Home is monotonic across nine buckets and within ~0.02 of the diagonal.</t>
+  </si>
+  <si>
+    <t>xG availability differs between train and test</t>
+  </si>
+  <si>
+    <t>Coverage by season: 2021 0%, 2022 57%, 2023 91% (TRAIN), 2024 86% (VAL), 2025 98% (TEST). Train is ~49% covered against a test set at 98%, so held-out metrics are measured on a feature-availability regime the model largely did not learn under. A distribution mismatch, not a metrics gap. Corners is flat at 89-92% across every season and is unaffected.</t>
   </si>
   <si>
     <t>SportIQ — Edge Measurement Plan (P0-P3)</t>
@@ -5318,7 +5351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R229"/>
+  <dimension ref="A1:R232"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -12066,7 +12099,7 @@
         <v>432</v>
       </c>
       <c r="R198" t="str">
-        <f t="shared" ref="R198:R227" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
+        <f t="shared" ref="R198:R230" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
         <v>E4 ML Football</v>
       </c>
     </row>
@@ -12904,7 +12937,7 @@
         <v>E9 Data Ops</v>
       </c>
     </row>
-    <row r="227" spans="1:18" ht="86.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="227" spans="1:18" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A227" t="s">
         <v>130</v>
       </c>
@@ -12934,23 +12967,107 @@
         <v>E9 Data Ops</v>
       </c>
     </row>
+    <row r="228" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A228" t="s">
+        <v>99</v>
+      </c>
+      <c r="B228" t="s">
+        <v>492</v>
+      </c>
+      <c r="C228" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D228" t="s">
+        <v>45</v>
+      </c>
+      <c r="E228" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F228" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G228" s="215"/>
+      <c r="J228" t="s">
+        <v>400</v>
+      </c>
+      <c r="R228" t="str">
+        <f t="shared" si="3"/>
+        <v>E8 Model Quality</v>
+      </c>
+    </row>
     <row r="229" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A229" s="23" t="s">
-        <v>492</v>
-      </c>
-      <c r="B229" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C229" s="15" t="s">
+      <c r="A229" t="s">
+        <v>99</v>
+      </c>
+      <c r="B229" t="s">
         <v>493</v>
       </c>
-      <c r="D229" s="17" t="s">
+      <c r="C229" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D229" t="s">
+        <v>45</v>
+      </c>
+      <c r="E229" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F229" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G229" s="215"/>
+      <c r="J229" t="s">
+        <v>400</v>
+      </c>
+      <c r="R229" t="str">
+        <f t="shared" si="3"/>
+        <v>E8 Model Quality</v>
+      </c>
+    </row>
+    <row r="230" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A230" t="s">
+        <v>73</v>
+      </c>
+      <c r="B230" t="s">
+        <v>494</v>
+      </c>
+      <c r="C230" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D230" t="s">
+        <v>75</v>
+      </c>
+      <c r="E230" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F230" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G230" s="215"/>
+      <c r="J230" t="s">
+        <v>400</v>
+      </c>
+      <c r="R230" t="str">
+        <f t="shared" si="3"/>
+        <v>E6 Picks</v>
+      </c>
+    </row>
+    <row r="232" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A232" s="23" t="s">
+        <v>495</v>
+      </c>
+      <c r="B232" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C232" s="15" t="s">
+        <v>496</v>
+      </c>
+      <c r="D232" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="E229" s="21" t="s">
+      <c r="E232" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="F229" s="19" t="s">
+      <c r="F232" s="19" t="s">
         <v>138</v>
       </c>
     </row>
@@ -12975,7 +13092,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="294" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="B1" s="283"/>
       <c r="C1" s="283"/>
@@ -12998,7 +13115,7 @@
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="301" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -13021,7 +13138,7 @@
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="289" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="B4" s="283"/>
       <c r="C4" s="283"/>
@@ -13044,42 +13161,42 @@
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="35" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="B5" s="279" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="C5" s="280"/>
       <c r="D5" s="281"/>
       <c r="E5" s="284" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="F5" s="280"/>
       <c r="G5" s="281"/>
       <c r="H5" s="284" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="I5" s="280"/>
       <c r="J5" s="281"/>
       <c r="K5" s="279" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="L5" s="280"/>
       <c r="M5" s="281"/>
       <c r="N5" s="286" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="O5" s="280"/>
       <c r="P5" s="281"/>
       <c r="Q5" s="286" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="R5" s="280"/>
       <c r="S5" s="281"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="282" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C6" s="283"/>
       <c r="D6" s="283"/>
@@ -13101,7 +13218,7 @@
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="289" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B7" s="283"/>
       <c r="C7" s="283"/>
@@ -13124,10 +13241,10 @@
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="35" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="B8" s="292" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="C8" s="280"/>
       <c r="D8" s="280"/>
@@ -13138,7 +13255,7 @@
       <c r="I8" s="280"/>
       <c r="J8" s="281"/>
       <c r="K8" s="292" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="L8" s="280"/>
       <c r="M8" s="280"/>
@@ -13151,7 +13268,7 @@
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="282" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C9" s="283"/>
       <c r="D9" s="283"/>
@@ -13173,7 +13290,7 @@
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="289" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="B10" s="283"/>
       <c r="C10" s="283"/>
@@ -13196,42 +13313,42 @@
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="35" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="B11" s="279" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="C11" s="280"/>
       <c r="D11" s="281"/>
       <c r="E11" s="279" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="F11" s="280"/>
       <c r="G11" s="281"/>
       <c r="H11" s="279" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="I11" s="280"/>
       <c r="J11" s="281"/>
       <c r="K11" s="284" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="L11" s="280"/>
       <c r="M11" s="281"/>
       <c r="N11" s="279" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="O11" s="280"/>
       <c r="P11" s="281"/>
       <c r="Q11" s="279" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="R11" s="280"/>
       <c r="S11" s="281"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="282" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C12" s="283"/>
       <c r="D12" s="283"/>
@@ -13253,7 +13370,7 @@
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="289" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="B13" s="283"/>
       <c r="C13" s="283"/>
@@ -13276,10 +13393,10 @@
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="35" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B14" s="287" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="C14" s="280"/>
       <c r="D14" s="280"/>
@@ -13287,7 +13404,7 @@
       <c r="F14" s="280"/>
       <c r="G14" s="281"/>
       <c r="H14" s="287" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="I14" s="280"/>
       <c r="J14" s="280"/>
@@ -13295,19 +13412,19 @@
       <c r="L14" s="280"/>
       <c r="M14" s="281"/>
       <c r="N14" s="287" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="O14" s="280"/>
       <c r="P14" s="281"/>
       <c r="Q14" s="284" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="R14" s="280"/>
       <c r="S14" s="281"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" s="282" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="C15" s="283"/>
       <c r="D15" s="283"/>
@@ -13329,7 +13446,7 @@
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="289" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>
@@ -13352,10 +13469,10 @@
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="35" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="B17" s="288" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="C17" s="280"/>
       <c r="D17" s="280"/>
@@ -13363,29 +13480,29 @@
       <c r="F17" s="280"/>
       <c r="G17" s="281"/>
       <c r="H17" s="288" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="I17" s="280"/>
       <c r="J17" s="281"/>
       <c r="K17" s="288" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="L17" s="280"/>
       <c r="M17" s="281"/>
       <c r="N17" s="288" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="O17" s="280"/>
       <c r="P17" s="281"/>
       <c r="Q17" s="288" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="R17" s="280"/>
       <c r="S17" s="281"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="282" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C18" s="283"/>
       <c r="D18" s="283"/>
@@ -13407,7 +13524,7 @@
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="289" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="B19" s="283"/>
       <c r="C19" s="283"/>
@@ -13430,10 +13547,10 @@
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="35" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="B20" s="290" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="C20" s="280"/>
       <c r="D20" s="280"/>
@@ -13441,7 +13558,7 @@
       <c r="F20" s="280"/>
       <c r="G20" s="281"/>
       <c r="H20" s="290" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="I20" s="280"/>
       <c r="J20" s="280"/>
@@ -13449,7 +13566,7 @@
       <c r="L20" s="280"/>
       <c r="M20" s="281"/>
       <c r="N20" s="290" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="O20" s="280"/>
       <c r="P20" s="280"/>
@@ -13459,7 +13576,7 @@
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" s="282" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C21" s="283"/>
       <c r="D21" s="283"/>
@@ -13481,7 +13598,7 @@
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="289" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="B22" s="283"/>
       <c r="C22" s="283"/>
@@ -13504,10 +13621,10 @@
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="35" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="B23" s="290" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="C23" s="280"/>
       <c r="D23" s="280"/>
@@ -13515,29 +13632,29 @@
       <c r="F23" s="280"/>
       <c r="G23" s="281"/>
       <c r="H23" s="290" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="I23" s="280"/>
       <c r="J23" s="281"/>
       <c r="K23" s="290" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="L23" s="280"/>
       <c r="M23" s="281"/>
       <c r="N23" s="290" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="O23" s="280"/>
       <c r="P23" s="281"/>
       <c r="Q23" s="286" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="R23" s="280"/>
       <c r="S23" s="281"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="295" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="B26" s="283"/>
       <c r="C26" s="283"/>
@@ -13560,42 +13677,42 @@
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="35" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="B27" s="279" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="C27" s="280"/>
       <c r="D27" s="281"/>
       <c r="E27" s="279" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="F27" s="280"/>
       <c r="G27" s="281"/>
       <c r="H27" s="287" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="I27" s="280"/>
       <c r="J27" s="281"/>
       <c r="K27" s="288" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="L27" s="280"/>
       <c r="M27" s="281"/>
       <c r="N27" s="288" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="O27" s="280"/>
       <c r="P27" s="281"/>
       <c r="Q27" s="287" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="R27" s="280"/>
       <c r="S27" s="281"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="289" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="B30" s="283"/>
       <c r="C30" s="283"/>
@@ -13618,7 +13735,7 @@
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="285" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="B31" s="283"/>
       <c r="C31" s="283"/>
@@ -13641,7 +13758,7 @@
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="285" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="B32" s="283"/>
       <c r="C32" s="283"/>
@@ -13664,7 +13781,7 @@
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="285" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="B33" s="283"/>
       <c r="C33" s="283"/>
@@ -13687,7 +13804,7 @@
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="285" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="B34" s="283"/>
       <c r="C34" s="283"/>
@@ -13710,7 +13827,7 @@
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="285" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="B35" s="283"/>
       <c r="C35" s="283"/>
@@ -13733,7 +13850,7 @@
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="285" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="B36" s="283"/>
       <c r="C36" s="283"/>
@@ -13756,7 +13873,7 @@
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="296" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="B37" s="283"/>
       <c r="C37" s="283"/>
@@ -13779,25 +13896,25 @@
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="36" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="B39" s="299" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="C39" s="283"/>
       <c r="D39" s="283"/>
       <c r="E39" s="297" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="F39" s="283"/>
       <c r="G39" s="283"/>
       <c r="H39" s="300" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="I39" s="283"/>
       <c r="J39" s="283"/>
       <c r="K39" s="293" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="L39" s="283"/>
       <c r="M39" s="283"/>
@@ -13807,7 +13924,7 @@
       <c r="O39" s="283"/>
       <c r="P39" s="283"/>
       <c r="Q39" s="298" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="R39" s="283"/>
       <c r="S39" s="283"/>
@@ -13815,11 +13932,11 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H14:M14"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A16:S16"/>
     <mergeCell ref="H20:M20"/>
-    <mergeCell ref="A16:S16"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -13828,13 +13945,14 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -13843,7 +13961,6 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
-    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -13851,7 +13968,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -13900,7 +14017,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -13913,19 +14030,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -14059,11 +14176,11 @@
       </c>
       <c r="B9" s="24">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C9" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D9" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A9,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -14075,7 +14192,7 @@
       </c>
       <c r="F9" s="25">
         <f t="shared" si="1"/>
-        <v>0.9</v>
+        <v>0.90909090909090906</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -14109,11 +14226,11 @@
       </c>
       <c r="B11" s="24">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C11" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D11" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -14125,7 +14242,7 @@
       </c>
       <c r="F11" s="25">
         <f t="shared" si="1"/>
-        <v>0.83673469387755106</v>
+        <v>0.84313725490196079</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -14205,15 +14322,15 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="26" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="B16" s="27">
         <f>SUM(B4:B14)</f>
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C16" s="27">
         <f>SUM(C4:C14)</f>
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
@@ -14225,12 +14342,12 @@
       </c>
       <c r="F16" s="28">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.79372197309417036</v>
+        <v>0.79646017699115046</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="41" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="B18" s="42">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -14239,7 +14356,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="43" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
     </row>
   </sheetData>
@@ -14260,7 +14377,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -14272,7 +14389,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -14281,648 +14398,648 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="29" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="D3" s="29" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="29" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="30" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="32" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C5" s="19" t="s">
+        <v>585</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>582</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>579</v>
-      </c>
       <c r="E5" s="33" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="30" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="32" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="30" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="32" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="30" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="32" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="B11" s="6" t="s">
+        <v>588</v>
+      </c>
+      <c r="C11" s="19" t="s">
         <v>585</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>582</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="30" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="32" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="30" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="32" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="30" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="32" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="30" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="32" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="30" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="32" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="E21" s="33" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="30" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="32" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="30" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E24" s="31" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="53" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="B25" s="51" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C25" s="54" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E25" s="55" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="56" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="B26" s="46" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="C26" s="54" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D26" s="46" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E26" s="57" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="53" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="B27" s="51" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C27" s="54" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D27" s="51" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E27" s="55" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="71" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="B28" s="60" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C28" s="67" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="D28" s="94" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E28" s="94" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="72" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
       <c r="B29" s="65" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C29" s="69" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D29" s="93" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E29" s="93" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="78" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="B30" s="75" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C30" s="79" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D30" s="75" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E30" s="80" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="92" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="B31" s="83" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="C31" s="90" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D31" s="83" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="E31" s="93" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="106" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="B32" s="102" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C32" s="104" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D32" s="102" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E32" s="107" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="108" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="B33" s="97" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C33" s="104" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D33" s="97" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="E33" s="109" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="134" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="B34" s="129" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="C34" s="123" t="s">
+        <v>585</v>
+      </c>
+      <c r="D34" s="129" t="s">
         <v>582</v>
       </c>
-      <c r="D34" s="129" t="s">
-        <v>579</v>
-      </c>
       <c r="E34" s="135" t="s">
-        <v>653</v>
+        <v>656</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="136" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="B35" s="124" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C35" s="132" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D35" s="124" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E35" s="137" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="74.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="147" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="B36" s="145" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C36" s="148" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="D36" s="153" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="E36" s="153" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="150" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="B37" s="140" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="C37" s="151" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D37" s="140" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E37" s="152" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="147" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="B38" s="145" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="C38" s="151" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D38" s="145" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E38" s="149" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="160" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="B39" s="157" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C39" s="161" t="s">
+        <v>585</v>
+      </c>
+      <c r="D39" s="157" t="s">
         <v>582</v>
       </c>
-      <c r="D39" s="157" t="s">
-        <v>579</v>
-      </c>
       <c r="E39" s="162" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="168" t="s">
-        <v>664</v>
+        <v>667</v>
       </c>
       <c r="B40" s="165" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="C40" s="169" t="s">
+        <v>585</v>
+      </c>
+      <c r="D40" s="165" t="s">
         <v>582</v>
       </c>
-      <c r="D40" s="165" t="s">
-        <v>579</v>
-      </c>
       <c r="E40" s="170" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -14930,645 +15047,713 @@
         <v>140</v>
       </c>
       <c r="B41" s="172" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C41" s="173" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D41" s="172" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E41" s="174" t="s">
-        <v>666</v>
+        <v>669</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="188" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
       <c r="B42" s="183" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="C42" s="177" t="s">
+        <v>585</v>
+      </c>
+      <c r="D42" s="183" t="s">
         <v>582</v>
       </c>
-      <c r="D42" s="183" t="s">
-        <v>579</v>
-      </c>
       <c r="E42" s="189" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="190" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="B43" s="178" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C43" s="186" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D43" s="178" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="E43" s="191" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="188" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="B44" s="183" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="C44" s="186" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D44" s="183" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E44" s="189" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="190" t="s">
-        <v>673</v>
+        <v>676</v>
       </c>
       <c r="B45" s="178" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C45" s="186" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D45" s="178" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E45" s="191" t="s">
-        <v>674</v>
+        <v>677</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="206" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="B46" s="194" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C46" s="199" t="s">
+        <v>585</v>
+      </c>
+      <c r="D46" s="194" t="s">
         <v>582</v>
       </c>
-      <c r="D46" s="194" t="s">
-        <v>579</v>
-      </c>
       <c r="E46" s="207" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="208" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
       <c r="B47" s="200" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C47" s="203" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D47" s="200" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E47" s="209" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="206" t="s">
-        <v>679</v>
+        <v>682</v>
       </c>
       <c r="B48" s="194" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C48" s="203" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D48" s="194" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E48" s="207" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="B49" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C49" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D49" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E49" t="s">
-        <v>682</v>
+        <v>685</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
-        <v>683</v>
+        <v>686</v>
       </c>
       <c r="B50" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C50" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D50" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E50" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="B51" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C51" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D51" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E51" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="B52" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C52" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="D52" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E52" t="s">
-        <v>689</v>
+        <v>692</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
-        <v>690</v>
+        <v>693</v>
       </c>
       <c r="B53" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C53" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="D53" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E53" t="s">
-        <v>691</v>
+        <v>694</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="215" t="s">
-        <v>692</v>
+        <v>695</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C54" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="D54" s="215" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E54" s="215" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="215" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C55" s="215" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="D55" s="215" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E55" s="215" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="215" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C56" s="215" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D56" s="215" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E56" s="215" t="s">
-        <v>697</v>
+        <v>700</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="215" t="s">
-        <v>698</v>
+        <v>701</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C57" s="215" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D57" s="215" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E57" s="215" t="s">
-        <v>699</v>
+        <v>702</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="215" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C58" s="215" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D58" s="215" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E58" s="215" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="215" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C59" s="215" t="s">
+        <v>585</v>
+      </c>
+      <c r="D59" s="215" t="s">
         <v>582</v>
       </c>
-      <c r="D59" s="215" t="s">
-        <v>579</v>
-      </c>
       <c r="E59" s="215" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="215" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C60" s="215" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="D60" s="215" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E60" s="215" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="215" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C61" s="215" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D61" s="215" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E61" s="215" t="s">
-        <v>707</v>
+        <v>710</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="215" t="s">
-        <v>708</v>
+        <v>711</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C62" s="215" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D62" s="215" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E62" s="215" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="215" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C63" s="215" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D63" s="215" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E63" s="215" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="215" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C64" s="215" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D64" s="215" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E64" s="215" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="129.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="215" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C65" s="215" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D65" s="215" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E65" s="215" t="s">
-        <v>715</v>
+        <v>718</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="215" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
       <c r="B66" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C66" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D66" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E66" t="s">
-        <v>717</v>
+        <v>720</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="215" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
       <c r="B67" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C67" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D67" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E67" t="s">
-        <v>719</v>
+        <v>722</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="215" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="B68" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C68" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D68" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E68" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="215" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="B69" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C69" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D69" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E69" t="s">
-        <v>723</v>
+        <v>726</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="215" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="B70" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C70" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="D70" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E70" t="s">
-        <v>725</v>
+        <v>728</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="215" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="B71" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C71" t="s">
+        <v>585</v>
+      </c>
+      <c r="D71" t="s">
         <v>582</v>
       </c>
-      <c r="D71" t="s">
-        <v>579</v>
-      </c>
       <c r="E71" t="s">
-        <v>727</v>
+        <v>730</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="215" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="B72" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C72" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D72" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E72" t="s">
-        <v>729</v>
+        <v>732</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="215" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="B73" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C73" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D73" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E73" t="s">
-        <v>731</v>
+        <v>734</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" s="215" t="s">
-        <v>732</v>
+        <v>735</v>
       </c>
       <c r="B74" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C74" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D74" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E74" t="s">
-        <v>733</v>
+        <v>736</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" s="215" t="s">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="B75" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C75" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D75" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E75" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A76" s="215" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="B76" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C76" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D76" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="E76" t="s">
-        <v>737</v>
+        <v>740</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A77" s="215" t="s">
-        <v>738</v>
+        <v>741</v>
       </c>
       <c r="B77" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C77" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D77" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E77" t="s">
-        <v>739</v>
+        <v>742</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A78" s="215" t="s">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="B78" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="C78" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D78" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E78" t="s">
-        <v>741</v>
+        <v>744</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A79" s="215" t="s">
+        <v>745</v>
+      </c>
+      <c r="B79" t="s">
+        <v>594</v>
+      </c>
+      <c r="C79" t="s">
+        <v>585</v>
+      </c>
+      <c r="D79" t="s">
+        <v>625</v>
+      </c>
+      <c r="E79" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A80" s="215" t="s">
+        <v>747</v>
+      </c>
+      <c r="B80" t="s">
+        <v>580</v>
+      </c>
+      <c r="C80" t="s">
+        <v>593</v>
+      </c>
+      <c r="D80" t="s">
+        <v>582</v>
+      </c>
+      <c r="E80" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A81" s="215" t="s">
+        <v>749</v>
+      </c>
+      <c r="B81" t="s">
+        <v>580</v>
+      </c>
+      <c r="C81" t="s">
+        <v>593</v>
+      </c>
+      <c r="D81" t="s">
+        <v>582</v>
+      </c>
+      <c r="E81" t="s">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A82" s="215" t="s">
+        <v>751</v>
+      </c>
+      <c r="B82" t="s">
+        <v>580</v>
+      </c>
+      <c r="C82" t="s">
+        <v>593</v>
+      </c>
+      <c r="D82" t="s">
+        <v>582</v>
+      </c>
+      <c r="E82" t="s">
+        <v>752</v>
       </c>
     </row>
   </sheetData>
@@ -15593,12 +15778,12 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="219" t="s">
-        <v>742</v>
+        <v>753</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="303" t="s">
-        <v>743</v>
+        <v>754</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -15607,1032 +15792,1032 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="220" t="s">
-        <v>744</v>
+        <v>755</v>
       </c>
       <c r="B4" s="220" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="C4" s="220" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="220" t="s">
-        <v>745</v>
+        <v>756</v>
       </c>
       <c r="E4" s="220" t="s">
-        <v>746</v>
+        <v>757</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="221" t="s">
-        <v>747</v>
+        <v>758</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>748</v>
+        <v>759</v>
       </c>
       <c r="C5" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>749</v>
+        <v>760</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>750</v>
+        <v>761</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="221" t="s">
-        <v>747</v>
+        <v>758</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>751</v>
+        <v>762</v>
       </c>
       <c r="C6" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="215" t="s">
-        <v>749</v>
+        <v>760</v>
       </c>
       <c r="E6" s="215" t="s">
-        <v>752</v>
+        <v>763</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="231" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>754</v>
+        <v>765</v>
       </c>
       <c r="C7" s="232" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="215" t="s">
-        <v>747</v>
+        <v>758</v>
       </c>
       <c r="E7" s="215" t="s">
-        <v>755</v>
+        <v>766</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="223" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>756</v>
+        <v>767</v>
       </c>
       <c r="C8" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>757</v>
+        <v>768</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>758</v>
+        <v>769</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="223" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="B9" s="215" t="s">
-        <v>759</v>
+        <v>770</v>
       </c>
       <c r="C9" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="215" t="s">
-        <v>747</v>
+        <v>758</v>
       </c>
       <c r="E9" s="215" t="s">
-        <v>760</v>
+        <v>771</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="224" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>762</v>
+        <v>773</v>
       </c>
       <c r="C10" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>763</v>
+        <v>774</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>764</v>
+        <v>775</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>765</v>
+        <v>776</v>
       </c>
       <c r="C11" t="s">
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>766</v>
+        <v>777</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>767</v>
+        <v>778</v>
       </c>
       <c r="C12" t="s">
         <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>766</v>
+        <v>777</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="224" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>768</v>
+        <v>779</v>
       </c>
       <c r="C13" s="222" t="s">
         <v>128</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>769</v>
+        <v>780</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>770</v>
+        <v>781</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="235" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>771</v>
+        <v>782</v>
       </c>
       <c r="C14" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>772</v>
+        <v>783</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>773</v>
+        <v>784</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="235" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B15" s="215" t="s">
-        <v>774</v>
+        <v>785</v>
       </c>
       <c r="C15" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="215" t="s">
-        <v>769</v>
+        <v>780</v>
       </c>
       <c r="E15" s="215" t="s">
-        <v>775</v>
+        <v>786</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="235" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B16" s="215" t="s">
-        <v>776</v>
+        <v>787</v>
       </c>
       <c r="C16" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="215" t="s">
-        <v>769</v>
+        <v>780</v>
       </c>
       <c r="E16" s="215" t="s">
-        <v>777</v>
+        <v>788</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="225" t="s">
-        <v>778</v>
+        <v>789</v>
       </c>
       <c r="B17" s="215" t="s">
-        <v>779</v>
+        <v>790</v>
       </c>
       <c r="C17" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D17" s="215" t="s">
-        <v>780</v>
+        <v>791</v>
       </c>
       <c r="E17" s="215" t="s">
-        <v>781</v>
+        <v>792</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="225" t="s">
-        <v>778</v>
+        <v>789</v>
       </c>
       <c r="B18" s="215" t="s">
-        <v>782</v>
+        <v>793</v>
       </c>
       <c r="C18" s="223" t="s">
         <v>138</v>
       </c>
       <c r="D18" s="215" t="s">
-        <v>780</v>
+        <v>791</v>
       </c>
       <c r="E18" s="215" t="s">
-        <v>783</v>
+        <v>794</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="226" t="s">
-        <v>784</v>
+        <v>795</v>
       </c>
       <c r="B19" s="215" t="s">
-        <v>785</v>
+        <v>796</v>
       </c>
       <c r="C19" s="225" t="s">
-        <v>786</v>
+        <v>797</v>
       </c>
       <c r="D19" s="215" t="s">
-        <v>749</v>
+        <v>760</v>
       </c>
       <c r="E19" s="215" t="s">
-        <v>787</v>
+        <v>798</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="226" t="s">
-        <v>784</v>
+        <v>795</v>
       </c>
       <c r="B20" s="215" t="s">
-        <v>788</v>
+        <v>799</v>
       </c>
       <c r="C20" s="225" t="s">
-        <v>786</v>
+        <v>797</v>
       </c>
       <c r="D20" s="215" t="s">
-        <v>749</v>
+        <v>760</v>
       </c>
       <c r="E20" s="215" t="s">
-        <v>789</v>
+        <v>800</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="226" t="s">
-        <v>784</v>
+        <v>795</v>
       </c>
       <c r="B21" s="215" t="s">
-        <v>790</v>
+        <v>801</v>
       </c>
       <c r="C21" s="225" t="s">
-        <v>786</v>
+        <v>797</v>
       </c>
       <c r="D21" s="215" t="s">
-        <v>749</v>
+        <v>760</v>
       </c>
       <c r="E21" s="215" t="s">
-        <v>791</v>
+        <v>802</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
     <row r="23" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="229" t="s">
-        <v>747</v>
+        <v>758</v>
       </c>
       <c r="B23" s="215" t="s">
-        <v>792</v>
+        <v>803</v>
       </c>
       <c r="C23" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D23" s="215" t="s">
-        <v>793</v>
+        <v>804</v>
       </c>
       <c r="E23" s="215" t="s">
-        <v>794</v>
+        <v>805</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="230" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="B24" s="215" t="s">
-        <v>795</v>
+        <v>806</v>
       </c>
       <c r="C24" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D24" s="215" t="s">
-        <v>796</v>
+        <v>807</v>
       </c>
       <c r="E24" s="215" t="s">
-        <v>797</v>
+        <v>808</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="231" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="B25" s="215" t="s">
-        <v>798</v>
+        <v>809</v>
       </c>
       <c r="C25" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D25" s="215" t="s">
-        <v>799</v>
+        <v>810</v>
       </c>
       <c r="E25" s="215" t="s">
-        <v>800</v>
+        <v>811</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="231" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="B26" s="215" t="s">
-        <v>801</v>
+        <v>812</v>
       </c>
       <c r="C26" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D26" s="215" t="s">
-        <v>796</v>
+        <v>807</v>
       </c>
       <c r="E26" s="215" t="s">
-        <v>802</v>
+        <v>813</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="235" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B27" s="215" t="s">
-        <v>803</v>
+        <v>814</v>
       </c>
       <c r="C27" s="237" t="s">
         <v>22</v>
       </c>
       <c r="D27" s="215" t="s">
-        <v>766</v>
+        <v>777</v>
       </c>
       <c r="E27" s="215" t="s">
-        <v>804</v>
+        <v>815</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="227" t="s">
-        <v>747</v>
+        <v>758</v>
       </c>
       <c r="B28" s="215" t="s">
-        <v>805</v>
+        <v>816</v>
       </c>
       <c r="C28" t="s">
         <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>806</v>
+        <v>817</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B29" s="215" t="s">
-        <v>807</v>
+        <v>818</v>
       </c>
       <c r="C29" t="s">
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>766</v>
+        <v>777</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B30" s="215" t="s">
-        <v>808</v>
+        <v>819</v>
       </c>
       <c r="C30" t="s">
         <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>809</v>
+        <v>820</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="B31" s="215" t="s">
-        <v>810</v>
+        <v>821</v>
       </c>
       <c r="C31" t="s">
         <v>22</v>
       </c>
       <c r="D31" t="s">
-        <v>811</v>
+        <v>822</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="B32" s="215" t="s">
-        <v>812</v>
+        <v>823</v>
       </c>
       <c r="C32" t="s">
         <v>22</v>
       </c>
       <c r="D32" t="s">
-        <v>813</v>
+        <v>824</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="B33" s="215" t="s">
-        <v>814</v>
+        <v>825</v>
       </c>
       <c r="C33" t="s">
         <v>22</v>
       </c>
       <c r="D33" t="s">
-        <v>811</v>
+        <v>822</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="B34" s="215" t="s">
-        <v>815</v>
+        <v>826</v>
       </c>
       <c r="C34" t="s">
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>816</v>
+        <v>827</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B35" s="215" t="s">
-        <v>817</v>
+        <v>828</v>
       </c>
       <c r="C35" t="s">
         <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>818</v>
+        <v>829</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="B36" s="215" t="s">
-        <v>819</v>
+        <v>830</v>
       </c>
       <c r="C36" t="s">
         <v>22</v>
       </c>
       <c r="D36" t="s">
-        <v>820</v>
+        <v>831</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B37" s="215" t="s">
-        <v>821</v>
+        <v>832</v>
       </c>
       <c r="C37" t="s">
         <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>820</v>
+        <v>831</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
-        <v>778</v>
+        <v>789</v>
       </c>
       <c r="B38" s="215" t="s">
-        <v>822</v>
+        <v>833</v>
       </c>
       <c r="C38" t="s">
         <v>22</v>
       </c>
       <c r="D38" t="s">
-        <v>820</v>
+        <v>831</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="B39" s="215" t="s">
-        <v>823</v>
+        <v>834</v>
       </c>
       <c r="C39" t="s">
         <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>820</v>
+        <v>831</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B40" s="215" t="s">
-        <v>824</v>
+        <v>835</v>
       </c>
       <c r="C40" t="s">
         <v>22</v>
       </c>
       <c r="D40" t="s">
-        <v>820</v>
+        <v>831</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="B41" s="215" t="s">
-        <v>825</v>
+        <v>836</v>
       </c>
       <c r="C41" t="s">
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>826</v>
+        <v>837</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B42" s="215" t="s">
-        <v>827</v>
+        <v>838</v>
       </c>
       <c r="C42" t="s">
         <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>826</v>
+        <v>837</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B43" s="215" t="s">
-        <v>828</v>
+        <v>839</v>
       </c>
       <c r="C43" t="s">
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>829</v>
+        <v>840</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
-        <v>761</v>
+        <v>772</v>
       </c>
       <c r="B44" s="215" t="s">
-        <v>830</v>
+        <v>841</v>
       </c>
       <c r="C44" t="s">
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>829</v>
+        <v>840</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
-        <v>778</v>
+        <v>789</v>
       </c>
       <c r="B45" s="215" t="s">
-        <v>831</v>
+        <v>842</v>
       </c>
       <c r="C45" t="s">
         <v>128</v>
       </c>
       <c r="D45" t="s">
-        <v>832</v>
+        <v>843</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B46" s="215" t="s">
-        <v>834</v>
+        <v>845</v>
       </c>
       <c r="C46" t="s">
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>835</v>
+        <v>846</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B47" s="215" t="s">
-        <v>836</v>
+        <v>847</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>837</v>
+        <v>848</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B48" s="215" t="s">
-        <v>838</v>
+        <v>849</v>
       </c>
       <c r="C48" t="s">
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>837</v>
+        <v>848</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B49" s="215" t="s">
-        <v>839</v>
+        <v>850</v>
       </c>
       <c r="C49" t="s">
         <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>837</v>
+        <v>848</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B50" s="215" t="s">
-        <v>840</v>
+        <v>851</v>
       </c>
       <c r="C50" t="s">
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>841</v>
+        <v>852</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B51" s="215" t="s">
-        <v>842</v>
+        <v>853</v>
       </c>
       <c r="C51" t="s">
         <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>843</v>
+        <v>854</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B52" s="215" t="s">
-        <v>844</v>
+        <v>855</v>
       </c>
       <c r="C52" t="s">
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>845</v>
+        <v>856</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B53" s="215" t="s">
-        <v>846</v>
+        <v>857</v>
       </c>
       <c r="C53" t="s">
         <v>128</v>
       </c>
       <c r="D53" t="s">
-        <v>843</v>
+        <v>854</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>847</v>
+        <v>858</v>
       </c>
       <c r="C54" t="s">
         <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>845</v>
+        <v>856</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>848</v>
+        <v>859</v>
       </c>
       <c r="C55" t="s">
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>849</v>
+        <v>860</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>850</v>
+        <v>861</v>
       </c>
       <c r="C56" t="s">
         <v>128</v>
       </c>
       <c r="D56" t="s">
-        <v>851</v>
+        <v>862</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>852</v>
+        <v>863</v>
       </c>
       <c r="C57" t="s">
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>853</v>
+        <v>864</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>854</v>
+        <v>865</v>
       </c>
       <c r="C58" t="s">
         <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>853</v>
+        <v>864</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>855</v>
+        <v>866</v>
       </c>
       <c r="C59" t="s">
         <v>22</v>
       </c>
       <c r="D59" t="s">
-        <v>853</v>
+        <v>864</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>856</v>
+        <v>867</v>
       </c>
       <c r="C60" t="s">
         <v>128</v>
       </c>
       <c r="D60" t="s">
-        <v>853</v>
+        <v>864</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="274" t="s">
-        <v>857</v>
+        <v>868</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>858</v>
+        <v>869</v>
       </c>
       <c r="C61" t="s">
         <v>22</v>
       </c>
       <c r="D61" t="s">
-        <v>826</v>
+        <v>837</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="274" t="s">
-        <v>857</v>
+        <v>868</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>859</v>
+        <v>870</v>
       </c>
       <c r="C62" t="s">
         <v>22</v>
       </c>
       <c r="D62" t="s">
-        <v>826</v>
+        <v>837</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="274" t="s">
-        <v>857</v>
+        <v>868</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>860</v>
+        <v>871</v>
       </c>
       <c r="C63" t="s">
         <v>22</v>
       </c>
       <c r="D63" t="s">
-        <v>826</v>
+        <v>837</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>861</v>
+        <v>872</v>
       </c>
       <c r="C64" t="s">
         <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>862</v>
+        <v>873</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>863</v>
+        <v>874</v>
       </c>
       <c r="C65" t="s">
         <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>862</v>
+        <v>873</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B66" s="215" t="s">
-        <v>864</v>
+        <v>875</v>
       </c>
       <c r="C66" t="s">
         <v>22</v>
       </c>
       <c r="D66" t="s">
-        <v>862</v>
+        <v>873</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="274" t="s">
-        <v>865</v>
+        <v>876</v>
       </c>
       <c r="B67" s="215" t="s">
-        <v>866</v>
+        <v>877</v>
       </c>
       <c r="C67" t="s">
         <v>22</v>
       </c>
       <c r="D67" t="s">
-        <v>826</v>
+        <v>837</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="274" t="s">
-        <v>865</v>
+        <v>876</v>
       </c>
       <c r="B68" s="215" t="s">
-        <v>867</v>
+        <v>878</v>
       </c>
       <c r="C68" t="s">
         <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>826</v>
+        <v>837</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="274" t="s">
-        <v>865</v>
+        <v>876</v>
       </c>
       <c r="B69" s="215" t="s">
-        <v>868</v>
+        <v>879</v>
       </c>
       <c r="C69" t="s">
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>826</v>
+        <v>837</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B70" s="215" t="s">
-        <v>869</v>
+        <v>880</v>
       </c>
       <c r="C70" t="s">
         <v>22</v>
       </c>
       <c r="D70" t="s">
-        <v>870</v>
+        <v>881</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B71" s="215" t="s">
-        <v>871</v>
+        <v>882</v>
       </c>
       <c r="C71" t="s">
         <v>22</v>
       </c>
       <c r="D71" t="s">
-        <v>870</v>
+        <v>881</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B72" s="215" t="s">
-        <v>872</v>
+        <v>883</v>
       </c>
       <c r="C72" t="s">
         <v>22</v>
       </c>
       <c r="D72" t="s">
-        <v>870</v>
+        <v>881</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="274" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
       <c r="B73" s="215" t="s">
-        <v>873</v>
+        <v>884</v>
       </c>
       <c r="C73" t="s">
         <v>128</v>
       </c>
       <c r="D73" t="s">
-        <v>870</v>
+        <v>881</v>
       </c>
     </row>
   </sheetData>
@@ -16661,336 +16846,336 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="211" t="s">
-        <v>874</v>
+        <v>885</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="212" t="s">
-        <v>875</v>
+        <v>886</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="213" t="s">
-        <v>876</v>
+        <v>887</v>
       </c>
       <c r="B4" s="213" t="s">
-        <v>877</v>
+        <v>888</v>
       </c>
       <c r="C4" s="213" t="s">
-        <v>878</v>
+        <v>889</v>
       </c>
       <c r="D4" s="213" t="s">
-        <v>879</v>
+        <v>890</v>
       </c>
       <c r="E4" s="213" t="s">
-        <v>880</v>
+        <v>891</v>
       </c>
       <c r="F4" s="213" t="s">
-        <v>881</v>
+        <v>892</v>
       </c>
       <c r="G4" s="213" t="s">
-        <v>882</v>
+        <v>893</v>
       </c>
       <c r="H4" s="213" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="213" t="s">
-        <v>883</v>
+        <v>894</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="214" t="s">
-        <v>884</v>
+        <v>895</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>885</v>
+        <v>896</v>
       </c>
       <c r="C5" s="215" t="s">
-        <v>886</v>
+        <v>897</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>887</v>
+        <v>898</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>888</v>
+        <v>899</v>
       </c>
       <c r="F5" s="215" t="s">
-        <v>889</v>
+        <v>900</v>
       </c>
       <c r="G5" s="215" t="s">
-        <v>890</v>
+        <v>901</v>
       </c>
       <c r="H5" s="216" t="s">
-        <v>891</v>
+        <v>902</v>
       </c>
       <c r="I5" s="215" t="s">
-        <v>892</v>
+        <v>903</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="214" t="s">
-        <v>893</v>
+        <v>904</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>894</v>
+        <v>905</v>
       </c>
       <c r="C6" s="215" t="s">
-        <v>895</v>
+        <v>906</v>
       </c>
       <c r="D6" s="215" t="s">
-        <v>896</v>
+        <v>907</v>
       </c>
       <c r="E6" s="215" t="s">
-        <v>897</v>
+        <v>908</v>
       </c>
       <c r="F6" s="215" t="s">
-        <v>898</v>
+        <v>909</v>
       </c>
       <c r="G6" s="215" t="s">
-        <v>899</v>
+        <v>910</v>
       </c>
       <c r="H6" s="217" t="s">
-        <v>891</v>
+        <v>902</v>
       </c>
       <c r="I6" s="215" t="s">
-        <v>900</v>
+        <v>911</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="214" t="s">
-        <v>901</v>
+        <v>912</v>
       </c>
       <c r="B7" s="215" t="s">
+        <v>913</v>
+      </c>
+      <c r="C7" s="215" t="s">
+        <v>914</v>
+      </c>
+      <c r="D7" s="215" t="s">
+        <v>915</v>
+      </c>
+      <c r="E7" s="215" t="s">
+        <v>916</v>
+      </c>
+      <c r="F7" s="215" t="s">
+        <v>917</v>
+      </c>
+      <c r="G7" s="215" t="s">
+        <v>918</v>
+      </c>
+      <c r="H7" s="217" t="s">
         <v>902</v>
       </c>
-      <c r="C7" s="215" t="s">
-        <v>903</v>
-      </c>
-      <c r="D7" s="215" t="s">
-        <v>904</v>
-      </c>
-      <c r="E7" s="215" t="s">
-        <v>905</v>
-      </c>
-      <c r="F7" s="215" t="s">
-        <v>906</v>
-      </c>
-      <c r="G7" s="215" t="s">
-        <v>907</v>
-      </c>
-      <c r="H7" s="217" t="s">
-        <v>891</v>
-      </c>
       <c r="I7" s="215" t="s">
-        <v>908</v>
+        <v>919</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="214" t="s">
-        <v>909</v>
+        <v>920</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>910</v>
+        <v>921</v>
       </c>
       <c r="C8" s="215" t="s">
-        <v>911</v>
+        <v>922</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>912</v>
+        <v>923</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="F8" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="G8" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="H8" s="216" t="s">
-        <v>913</v>
+        <v>924</v>
       </c>
       <c r="I8" s="215" t="s">
-        <v>914</v>
+        <v>925</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="214" t="s">
-        <v>915</v>
+        <v>926</v>
       </c>
       <c r="B9" s="215" t="s">
+        <v>927</v>
+      </c>
+      <c r="C9" s="215" t="s">
+        <v>928</v>
+      </c>
+      <c r="D9" s="215" t="s">
+        <v>923</v>
+      </c>
+      <c r="E9" s="215" t="s">
         <v>916</v>
       </c>
-      <c r="C9" s="215" t="s">
-        <v>917</v>
-      </c>
-      <c r="D9" s="215" t="s">
-        <v>912</v>
-      </c>
-      <c r="E9" s="215" t="s">
-        <v>905</v>
-      </c>
       <c r="F9" s="215" t="s">
-        <v>918</v>
+        <v>929</v>
       </c>
       <c r="G9" s="215" t="s">
-        <v>919</v>
+        <v>930</v>
       </c>
       <c r="H9" s="218" t="s">
-        <v>920</v>
+        <v>931</v>
       </c>
       <c r="I9" s="215" t="s">
-        <v>921</v>
+        <v>932</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="214" t="s">
-        <v>922</v>
+        <v>933</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>923</v>
+        <v>934</v>
       </c>
       <c r="C10" s="215" t="s">
-        <v>924</v>
+        <v>935</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>925</v>
+        <v>936</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>926</v>
+        <v>937</v>
       </c>
       <c r="F10" s="215" t="s">
-        <v>927</v>
+        <v>938</v>
       </c>
       <c r="G10" s="215" t="s">
-        <v>928</v>
+        <v>939</v>
       </c>
       <c r="H10" s="218" t="s">
-        <v>929</v>
+        <v>940</v>
       </c>
       <c r="I10" s="215" t="s">
-        <v>930</v>
+        <v>941</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="214" t="s">
-        <v>931</v>
+        <v>942</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>932</v>
+        <v>943</v>
       </c>
       <c r="C11" s="215" t="s">
-        <v>933</v>
+        <v>944</v>
       </c>
       <c r="D11" s="215" t="s">
-        <v>934</v>
+        <v>945</v>
       </c>
       <c r="E11" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="F11" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="G11" s="215" t="s">
-        <v>935</v>
+        <v>946</v>
       </c>
       <c r="H11" s="218" t="s">
-        <v>936</v>
+        <v>947</v>
       </c>
       <c r="I11" s="215" t="s">
-        <v>937</v>
+        <v>948</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="214" t="s">
-        <v>938</v>
+        <v>949</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>939</v>
+        <v>950</v>
       </c>
       <c r="C12" s="215" t="s">
-        <v>940</v>
+        <v>951</v>
       </c>
       <c r="D12" s="215" t="s">
-        <v>941</v>
+        <v>952</v>
       </c>
       <c r="E12" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="F12" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="G12" s="215" t="s">
-        <v>935</v>
+        <v>946</v>
       </c>
       <c r="H12" s="217" t="s">
-        <v>942</v>
+        <v>953</v>
       </c>
       <c r="I12" s="215" t="s">
-        <v>943</v>
+        <v>954</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="214" t="s">
-        <v>944</v>
+        <v>955</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>945</v>
+        <v>956</v>
       </c>
       <c r="C13" s="215" t="s">
-        <v>946</v>
+        <v>957</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="F13" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="G13" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="H13" s="218" t="s">
-        <v>947</v>
+        <v>958</v>
       </c>
       <c r="I13" s="215" t="s">
-        <v>948</v>
+        <v>959</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="214" t="s">
-        <v>949</v>
+        <v>960</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>950</v>
+        <v>961</v>
       </c>
       <c r="C14" s="215" t="s">
-        <v>946</v>
+        <v>957</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="F14" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="G14" s="215" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="H14" s="218" t="s">
-        <v>947</v>
+        <v>958</v>
       </c>
       <c r="I14" s="215" t="s">
-        <v>951</v>
+        <v>962</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="304" t="s">
-        <v>952</v>
+        <v>963</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>

</xml_diff>

<commit_message>
docs(tracker): card-pick grading, and the snapshot coverage gap
Board row for the notebook change plus two Risks & Decisions entries: the
published accuracy having measured the 1X2 argmax rather than the card, and
pick_snapshots capturing tennis only (0 of 6 football fixtures since 08-10).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{594F2C9E-6E00-4AD0-B1ED-413FA26F489F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AA50724-AAD4-4015-8FAD-937B962CEA63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2045" uniqueCount="964">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2060" uniqueCount="969">
   <si>
     <t>SportIQ — Delivery Board &amp; Roadmap</t>
   </si>
@@ -1523,6 +1523,9 @@
   </si>
   <si>
     <t>Settled cards no longer re-gated by a tightened floor</t>
+  </si>
+  <si>
+    <t>Notebook grades the CARD's pick across all four markets</t>
   </si>
   <si>
     <t>Legend</t>
@@ -2369,6 +2372,18 @@
   </si>
   <si>
     <t>Coverage by season: 2021 0%, 2022 57%, 2023 91% (TRAIN), 2024 86% (VAL), 2025 98% (TEST). Train is ~49% covered against a test set at 98%, so held-out metrics are measured on a feature-availability regime the model largely did not learn under. A distribution mismatch, not a metrics gap. Corners is flat at 89-92% across every season and is unaffected.</t>
+  </si>
+  <si>
+    <t>Published accuracy measured a different object from the product</t>
+  </si>
+  <si>
+    <t>/history and the notebook graded the 1X2 argmax while the card shows best_pick across four markets. Football card picks are 43 double chance + 19 corners and ZERO h2h, so the published football accuracy described a market football cards never show. Grading the card instead moves it 0.3651 -&gt; 0.7258 (n=62), but the no-skill baseline rises with it to 0.6391, so the honest figure is +8.67pp against a 14.09pp detectable effect - not conclusive. The grading rule existed only in TypeScript and is now ported to app/predictions/grading.py with parity tests.</t>
+  </si>
+  <si>
+    <t>pick_snapshots is capturing tennis only</t>
+  </si>
+  <si>
+    <t>59 snapshots since 2026-08-10, all tennis h2h; 0 of the 6 football fixtures that passed through the 4-8h window were captured. Snapshots are the only true record of what was displayed - everything else is recomputed against today's odds - so a gap here is a permanent hole in the trust record. n=6 is too small to call it a bug yet; diagnose before the football season opens.</t>
   </si>
   <si>
     <t>SportIQ — Edge Measurement Plan (P0-P3)</t>
@@ -5351,7 +5366,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R232"/>
+  <dimension ref="A1:R233"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -12099,7 +12114,7 @@
         <v>432</v>
       </c>
       <c r="R198" t="str">
-        <f t="shared" ref="R198:R230" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
+        <f t="shared" ref="R198:R231" si="3">IF($A198&lt;&gt;"",$A198,R197)</f>
         <v>E4 ML Football</v>
       </c>
     </row>
@@ -13051,23 +13066,51 @@
         <v>E6 Picks</v>
       </c>
     </row>
-    <row r="232" spans="1:18" x14ac:dyDescent="0.55000000000000004">
-      <c r="A232" s="23" t="s">
+    <row r="231" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A231" t="s">
+        <v>99</v>
+      </c>
+      <c r="B231" t="s">
         <v>495</v>
       </c>
-      <c r="B232" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C232" s="15" t="s">
+      <c r="C231" s="273" t="s">
+        <v>22</v>
+      </c>
+      <c r="D231" t="s">
+        <v>45</v>
+      </c>
+      <c r="E231" s="210">
+        <v>46247</v>
+      </c>
+      <c r="F231" s="210">
+        <v>46247</v>
+      </c>
+      <c r="G231" s="215"/>
+      <c r="J231" t="s">
+        <v>400</v>
+      </c>
+      <c r="R231" t="str">
+        <f t="shared" si="3"/>
+        <v>E8 Model Quality</v>
+      </c>
+    </row>
+    <row r="233" spans="1:18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A233" s="23" t="s">
         <v>496</v>
       </c>
-      <c r="D232" s="17" t="s">
+      <c r="B233" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C233" s="15" t="s">
+        <v>497</v>
+      </c>
+      <c r="D233" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="E232" s="21" t="s">
+      <c r="E233" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="F232" s="19" t="s">
+      <c r="F233" s="19" t="s">
         <v>138</v>
       </c>
     </row>
@@ -13092,7 +13135,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="294" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B1" s="283"/>
       <c r="C1" s="283"/>
@@ -13115,7 +13158,7 @@
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="301" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -13138,7 +13181,7 @@
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="289" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B4" s="283"/>
       <c r="C4" s="283"/>
@@ -13161,42 +13204,42 @@
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="35" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B5" s="279" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="C5" s="280"/>
       <c r="D5" s="281"/>
       <c r="E5" s="284" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F5" s="280"/>
       <c r="G5" s="281"/>
       <c r="H5" s="284" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="I5" s="280"/>
       <c r="J5" s="281"/>
       <c r="K5" s="279" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="L5" s="280"/>
       <c r="M5" s="281"/>
       <c r="N5" s="286" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="O5" s="280"/>
       <c r="P5" s="281"/>
       <c r="Q5" s="286" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="R5" s="280"/>
       <c r="S5" s="281"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="282" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="C6" s="283"/>
       <c r="D6" s="283"/>
@@ -13218,7 +13261,7 @@
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="289" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B7" s="283"/>
       <c r="C7" s="283"/>
@@ -13241,10 +13284,10 @@
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="35" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B8" s="292" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C8" s="280"/>
       <c r="D8" s="280"/>
@@ -13255,7 +13298,7 @@
       <c r="I8" s="280"/>
       <c r="J8" s="281"/>
       <c r="K8" s="292" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="L8" s="280"/>
       <c r="M8" s="280"/>
@@ -13268,7 +13311,7 @@
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="282" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="C9" s="283"/>
       <c r="D9" s="283"/>
@@ -13290,7 +13333,7 @@
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="289" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B10" s="283"/>
       <c r="C10" s="283"/>
@@ -13313,42 +13356,42 @@
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="35" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B11" s="279" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C11" s="280"/>
       <c r="D11" s="281"/>
       <c r="E11" s="279" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F11" s="280"/>
       <c r="G11" s="281"/>
       <c r="H11" s="279" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="I11" s="280"/>
       <c r="J11" s="281"/>
       <c r="K11" s="284" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="L11" s="280"/>
       <c r="M11" s="281"/>
       <c r="N11" s="279" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="O11" s="280"/>
       <c r="P11" s="281"/>
       <c r="Q11" s="279" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="R11" s="280"/>
       <c r="S11" s="281"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" s="282" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="C12" s="283"/>
       <c r="D12" s="283"/>
@@ -13370,7 +13413,7 @@
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="289" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B13" s="283"/>
       <c r="C13" s="283"/>
@@ -13393,10 +13436,10 @@
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="35" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B14" s="287" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="C14" s="280"/>
       <c r="D14" s="280"/>
@@ -13404,7 +13447,7 @@
       <c r="F14" s="280"/>
       <c r="G14" s="281"/>
       <c r="H14" s="287" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="I14" s="280"/>
       <c r="J14" s="280"/>
@@ -13412,19 +13455,19 @@
       <c r="L14" s="280"/>
       <c r="M14" s="281"/>
       <c r="N14" s="287" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="O14" s="280"/>
       <c r="P14" s="281"/>
       <c r="Q14" s="284" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="R14" s="280"/>
       <c r="S14" s="281"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" s="282" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="C15" s="283"/>
       <c r="D15" s="283"/>
@@ -13446,7 +13489,7 @@
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="289" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>
@@ -13469,10 +13512,10 @@
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="35" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B17" s="288" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="C17" s="280"/>
       <c r="D17" s="280"/>
@@ -13480,29 +13523,29 @@
       <c r="F17" s="280"/>
       <c r="G17" s="281"/>
       <c r="H17" s="288" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="I17" s="280"/>
       <c r="J17" s="281"/>
       <c r="K17" s="288" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="L17" s="280"/>
       <c r="M17" s="281"/>
       <c r="N17" s="288" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="O17" s="280"/>
       <c r="P17" s="281"/>
       <c r="Q17" s="288" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="R17" s="280"/>
       <c r="S17" s="281"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="282" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="C18" s="283"/>
       <c r="D18" s="283"/>
@@ -13524,7 +13567,7 @@
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="289" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B19" s="283"/>
       <c r="C19" s="283"/>
@@ -13547,10 +13590,10 @@
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="35" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B20" s="290" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="C20" s="280"/>
       <c r="D20" s="280"/>
@@ -13558,7 +13601,7 @@
       <c r="F20" s="280"/>
       <c r="G20" s="281"/>
       <c r="H20" s="290" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="I20" s="280"/>
       <c r="J20" s="280"/>
@@ -13566,7 +13609,7 @@
       <c r="L20" s="280"/>
       <c r="M20" s="281"/>
       <c r="N20" s="290" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="O20" s="280"/>
       <c r="P20" s="280"/>
@@ -13576,7 +13619,7 @@
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" s="282" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="C21" s="283"/>
       <c r="D21" s="283"/>
@@ -13598,7 +13641,7 @@
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="289" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B22" s="283"/>
       <c r="C22" s="283"/>
@@ -13621,10 +13664,10 @@
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="35" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B23" s="290" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C23" s="280"/>
       <c r="D23" s="280"/>
@@ -13632,29 +13675,29 @@
       <c r="F23" s="280"/>
       <c r="G23" s="281"/>
       <c r="H23" s="290" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="I23" s="280"/>
       <c r="J23" s="281"/>
       <c r="K23" s="290" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="L23" s="280"/>
       <c r="M23" s="281"/>
       <c r="N23" s="290" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="O23" s="280"/>
       <c r="P23" s="281"/>
       <c r="Q23" s="286" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="R23" s="280"/>
       <c r="S23" s="281"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="295" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B26" s="283"/>
       <c r="C26" s="283"/>
@@ -13677,42 +13720,42 @@
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="35" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B27" s="279" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C27" s="280"/>
       <c r="D27" s="281"/>
       <c r="E27" s="279" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="F27" s="280"/>
       <c r="G27" s="281"/>
       <c r="H27" s="287" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="I27" s="280"/>
       <c r="J27" s="281"/>
       <c r="K27" s="288" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="L27" s="280"/>
       <c r="M27" s="281"/>
       <c r="N27" s="288" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="O27" s="280"/>
       <c r="P27" s="281"/>
       <c r="Q27" s="287" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="R27" s="280"/>
       <c r="S27" s="281"/>
     </row>
     <row r="30" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="289" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="B30" s="283"/>
       <c r="C30" s="283"/>
@@ -13735,7 +13778,7 @@
     </row>
     <row r="31" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="285" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B31" s="283"/>
       <c r="C31" s="283"/>
@@ -13758,7 +13801,7 @@
     </row>
     <row r="32" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="285" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B32" s="283"/>
       <c r="C32" s="283"/>
@@ -13781,7 +13824,7 @@
     </row>
     <row r="33" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="285" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B33" s="283"/>
       <c r="C33" s="283"/>
@@ -13804,7 +13847,7 @@
     </row>
     <row r="34" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="285" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B34" s="283"/>
       <c r="C34" s="283"/>
@@ -13827,7 +13870,7 @@
     </row>
     <row r="35" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="285" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B35" s="283"/>
       <c r="C35" s="283"/>
@@ -13850,7 +13893,7 @@
     </row>
     <row r="36" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="285" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B36" s="283"/>
       <c r="C36" s="283"/>
@@ -13873,7 +13916,7 @@
     </row>
     <row r="37" spans="1:19" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="296" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B37" s="283"/>
       <c r="C37" s="283"/>
@@ -13896,25 +13939,25 @@
     </row>
     <row r="39" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="36" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B39" s="299" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="C39" s="283"/>
       <c r="D39" s="283"/>
       <c r="E39" s="297" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="F39" s="283"/>
       <c r="G39" s="283"/>
       <c r="H39" s="300" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="I39" s="283"/>
       <c r="J39" s="283"/>
       <c r="K39" s="293" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="L39" s="283"/>
       <c r="M39" s="283"/>
@@ -13924,7 +13967,7 @@
       <c r="O39" s="283"/>
       <c r="P39" s="283"/>
       <c r="Q39" s="298" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="R39" s="283"/>
       <c r="S39" s="283"/>
@@ -13932,11 +13975,11 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="H20:M20"/>
     <mergeCell ref="A16:S16"/>
-    <mergeCell ref="H20:M20"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -13945,14 +13988,13 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -13961,6 +14003,7 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -13968,7 +14011,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -14017,7 +14060,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -14030,19 +14073,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>145</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -14226,11 +14269,11 @@
       </c>
       <c r="B11" s="24">
         <f t="shared" si="0"/>
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Done")</f>
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D11" s="24">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,$A11,'Delivery Board'!$C$5:$C$500,"Milestone")</f>
@@ -14242,7 +14285,7 @@
       </c>
       <c r="F11" s="25">
         <f t="shared" si="1"/>
-        <v>0.84313725490196079</v>
+        <v>0.84615384615384615</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -14322,15 +14365,15 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="26" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="B16" s="27">
         <f>SUM(B4:B14)</f>
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C16" s="27">
         <f>SUM(C4:C14)</f>
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D16">
         <f>SUM(D4:D14)</f>
@@ -14342,12 +14385,12 @@
       </c>
       <c r="F16" s="28">
         <f>IF(B16=0,0,C16/B16)</f>
-        <v>0.79646017699115046</v>
+        <v>0.79735682819383258</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="41" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B18" s="42">
         <f>COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Done")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Planned")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"In progress")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Milestone")+COUNTIFS('Delivery Board'!$R$5:$R$500,"&lt;&gt;",'Delivery Board'!$C$5:$C$500,"Blocked")-B16</f>
@@ -14356,7 +14399,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="43" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
     </row>
   </sheetData>
@@ -14377,7 +14420,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E84"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -14389,7 +14432,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="302" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B1" s="276"/>
       <c r="C1" s="276"/>
@@ -14398,648 +14441,648 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="29" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="D3" s="29" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="29" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="30" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="32" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="30" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="32" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="30" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="32" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="30" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="32" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="30" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C12" s="34" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="32" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="30" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>128</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="32" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="30" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="32" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="30" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="32" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="30" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="32" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E21" s="33" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="30" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="32" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="30" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E24" s="31" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="53" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B25" s="51" t="s">
+        <v>595</v>
+      </c>
+      <c r="C25" s="54" t="s">
         <v>594</v>
       </c>
-      <c r="C25" s="54" t="s">
-        <v>593</v>
-      </c>
       <c r="D25" s="51" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E25" s="55" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="56" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B26" s="46" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C26" s="54" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D26" s="46" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E26" s="57" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="53" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B27" s="51" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C27" s="54" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D27" s="51" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E27" s="55" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="71" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="B28" s="60" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C28" s="67" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D28" s="94" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E28" s="94" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="72" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="B29" s="65" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C29" s="69" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D29" s="93" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E29" s="93" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="78" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B30" s="75" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C30" s="79" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D30" s="75" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E30" s="80" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="92" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B31" s="83" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C31" s="90" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D31" s="83" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="E31" s="93" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="106" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="B32" s="102" t="s">
+        <v>595</v>
+      </c>
+      <c r="C32" s="104" t="s">
         <v>594</v>
       </c>
-      <c r="C32" s="104" t="s">
-        <v>593</v>
-      </c>
       <c r="D32" s="102" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E32" s="107" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="108" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B33" s="97" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C33" s="104" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D33" s="97" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E33" s="109" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="134" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B34" s="129" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C34" s="123" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D34" s="129" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E34" s="135" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="136" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B35" s="124" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C35" s="132" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D35" s="124" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E35" s="137" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="74.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="147" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B36" s="145" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C36" s="148" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="D36" s="153" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="E36" s="153" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="150" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="B37" s="140" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C37" s="151" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D37" s="140" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E37" s="152" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="147" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="B38" s="145" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C38" s="151" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D38" s="145" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E38" s="149" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="160" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B39" s="157" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C39" s="161" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D39" s="157" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E39" s="162" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="168" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B40" s="165" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C40" s="169" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D40" s="165" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E40" s="170" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -15047,713 +15090,747 @@
         <v>140</v>
       </c>
       <c r="B41" s="172" t="s">
+        <v>595</v>
+      </c>
+      <c r="C41" s="173" t="s">
         <v>594</v>
       </c>
-      <c r="C41" s="173" t="s">
-        <v>593</v>
-      </c>
       <c r="D41" s="172" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E41" s="174" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="188" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B42" s="183" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C42" s="177" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D42" s="183" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E42" s="189" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="190" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B43" s="178" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C43" s="186" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D43" s="178" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E43" s="191" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="188" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B44" s="183" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C44" s="186" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D44" s="183" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E44" s="189" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="190" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B45" s="178" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C45" s="186" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D45" s="178" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E45" s="191" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="206" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B46" s="194" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C46" s="199" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D46" s="194" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E46" s="207" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="208" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B47" s="200" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C47" s="203" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D47" s="200" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E47" s="209" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="32.049999999999997" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="206" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="B48" s="194" t="s">
+        <v>595</v>
+      </c>
+      <c r="C48" s="203" t="s">
         <v>594</v>
       </c>
-      <c r="C48" s="203" t="s">
-        <v>593</v>
-      </c>
       <c r="D48" s="194" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E48" s="207" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="B49" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C49" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D49" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E49" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="B50" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C50" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D50" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E50" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B51" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C51" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D51" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E51" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B52" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C52" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="D52" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E52" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="B53" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C53" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="D53" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E53" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="215" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C54" s="215" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="D54" s="215" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E54" s="215" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="215" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C55" s="215" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D55" s="215" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E55" s="215" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="215" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C56" s="215" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D56" s="215" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E56" s="215" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="215" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C57" s="215" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D57" s="215" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E57" s="215" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="215" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C58" s="215" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D58" s="215" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E58" s="215" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="215" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C59" s="215" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D59" s="215" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E59" s="215" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="215" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C60" s="215" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D60" s="215" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E60" s="215" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="215" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C61" s="215" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D61" s="215" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E61" s="215" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="215" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C62" s="215" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D62" s="215" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E62" s="215" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="215" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C63" s="215" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D63" s="215" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E63" s="215" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="215" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C64" s="215" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D64" s="215" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E64" s="215" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="129.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="215" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C65" s="215" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D65" s="215" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E65" s="215" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="215" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B66" t="s">
+        <v>595</v>
+      </c>
+      <c r="C66" t="s">
         <v>594</v>
       </c>
-      <c r="C66" t="s">
-        <v>593</v>
-      </c>
       <c r="D66" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E66" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="215" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B67" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C67" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D67" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E67" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="215" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B68" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C68" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D68" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E68" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="215" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B69" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C69" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D69" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E69" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="215" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B70" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C70" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D70" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E70" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="215" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B71" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C71" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D71" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E71" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="215" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="B72" t="s">
+        <v>595</v>
+      </c>
+      <c r="C72" t="s">
         <v>594</v>
       </c>
-      <c r="C72" t="s">
-        <v>593</v>
-      </c>
       <c r="D72" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E72" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="215" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B73" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C73" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D73" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E73" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" s="215" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B74" t="s">
+        <v>595</v>
+      </c>
+      <c r="C74" t="s">
         <v>594</v>
       </c>
-      <c r="C74" t="s">
-        <v>593</v>
-      </c>
       <c r="D74" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E74" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" s="215" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B75" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="C75" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D75" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E75" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A76" s="215" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B76" t="s">
+        <v>595</v>
+      </c>
+      <c r="C76" t="s">
         <v>594</v>
       </c>
-      <c r="C76" t="s">
-        <v>593</v>
-      </c>
       <c r="D76" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E76" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A77" s="215" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B77" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C77" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D77" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E77" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A78" s="215" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B78" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C78" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D78" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E78" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A79" s="215" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B79" t="s">
+        <v>595</v>
+      </c>
+      <c r="C79" t="s">
+        <v>586</v>
+      </c>
+      <c r="D79" t="s">
+        <v>626</v>
+      </c>
+      <c r="E79" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A80" s="215" t="s">
+        <v>748</v>
+      </c>
+      <c r="B80" t="s">
+        <v>581</v>
+      </c>
+      <c r="C80" t="s">
         <v>594</v>
       </c>
-      <c r="C79" t="s">
-        <v>585</v>
-      </c>
-      <c r="D79" t="s">
-        <v>625</v>
-      </c>
-      <c r="E79" t="s">
-        <v>746</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A80" s="215" t="s">
-        <v>747</v>
-      </c>
-      <c r="B80" t="s">
-        <v>580</v>
-      </c>
-      <c r="C80" t="s">
-        <v>593</v>
-      </c>
       <c r="D80" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E80" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A81" s="215" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B81" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C81" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D81" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E81" t="s">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A82" s="215" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="B82" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C82" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D82" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E82" t="s">
-        <v>752</v>
+        <v>753</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A83" s="215" t="s">
+        <v>754</v>
+      </c>
+      <c r="B83" t="s">
+        <v>595</v>
+      </c>
+      <c r="C83" t="s">
+        <v>586</v>
+      </c>
+      <c r="D83" t="s">
+        <v>626</v>
+      </c>
+      <c r="E83" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A84" s="215" t="s">
+        <v>756</v>
+      </c>
+      <c r="B84" t="s">
+        <v>581</v>
+      </c>
+      <c r="C84" t="s">
+        <v>594</v>
+      </c>
+      <c r="D84" t="s">
+        <v>583</v>
+      </c>
+      <c r="E84" t="s">
+        <v>757</v>
       </c>
     </row>
   </sheetData>
@@ -15778,12 +15855,12 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="219" t="s">
-        <v>753</v>
+        <v>758</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="303" t="s">
-        <v>754</v>
+        <v>759</v>
       </c>
       <c r="B2" s="283"/>
       <c r="C2" s="283"/>
@@ -15792,1032 +15869,1032 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="220" t="s">
-        <v>755</v>
+        <v>760</v>
       </c>
       <c r="B4" s="220" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C4" s="220" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="220" t="s">
-        <v>756</v>
+        <v>761</v>
       </c>
       <c r="E4" s="220" t="s">
-        <v>757</v>
+        <v>762</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="221" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>759</v>
+        <v>764</v>
       </c>
       <c r="C5" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>761</v>
+        <v>766</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="221" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>762</v>
+        <v>767</v>
       </c>
       <c r="C6" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="215" t="s">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="E6" s="215" t="s">
-        <v>763</v>
+        <v>768</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="231" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>765</v>
+        <v>770</v>
       </c>
       <c r="C7" s="232" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="215" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="E7" s="215" t="s">
-        <v>766</v>
+        <v>771</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="223" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>767</v>
+        <v>772</v>
       </c>
       <c r="C8" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>768</v>
+        <v>773</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>769</v>
+        <v>774</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="223" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B9" s="215" t="s">
-        <v>770</v>
+        <v>775</v>
       </c>
       <c r="C9" s="233" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="215" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="E9" s="215" t="s">
-        <v>771</v>
+        <v>776</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="224" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>773</v>
+        <v>778</v>
       </c>
       <c r="C10" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>774</v>
+        <v>779</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>775</v>
+        <v>780</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>776</v>
+        <v>781</v>
       </c>
       <c r="C11" t="s">
         <v>22</v>
       </c>
       <c r="D11" t="s">
-        <v>777</v>
+        <v>782</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>778</v>
+        <v>783</v>
       </c>
       <c r="C12" t="s">
         <v>22</v>
       </c>
       <c r="D12" t="s">
-        <v>777</v>
+        <v>782</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="224" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>779</v>
+        <v>784</v>
       </c>
       <c r="C13" s="222" t="s">
         <v>128</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>780</v>
+        <v>785</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>781</v>
+        <v>786</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="235" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>782</v>
+        <v>787</v>
       </c>
       <c r="C14" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>783</v>
+        <v>788</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>784</v>
+        <v>789</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="235" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B15" s="215" t="s">
+        <v>790</v>
+      </c>
+      <c r="C15" s="236" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" s="215" t="s">
         <v>785</v>
       </c>
-      <c r="C15" s="236" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="215" t="s">
-        <v>780</v>
-      </c>
       <c r="E15" s="215" t="s">
-        <v>786</v>
+        <v>791</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="235" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B16" s="215" t="s">
-        <v>787</v>
+        <v>792</v>
       </c>
       <c r="C16" s="236" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="215" t="s">
-        <v>780</v>
+        <v>785</v>
       </c>
       <c r="E16" s="215" t="s">
-        <v>788</v>
+        <v>793</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="225" t="s">
-        <v>789</v>
+        <v>794</v>
       </c>
       <c r="B17" s="215" t="s">
-        <v>790</v>
+        <v>795</v>
       </c>
       <c r="C17" s="222" t="s">
         <v>22</v>
       </c>
       <c r="D17" s="215" t="s">
-        <v>791</v>
+        <v>796</v>
       </c>
       <c r="E17" s="215" t="s">
-        <v>792</v>
+        <v>797</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="225" t="s">
-        <v>789</v>
+        <v>794</v>
       </c>
       <c r="B18" s="215" t="s">
-        <v>793</v>
+        <v>798</v>
       </c>
       <c r="C18" s="223" t="s">
         <v>138</v>
       </c>
       <c r="D18" s="215" t="s">
-        <v>791</v>
+        <v>796</v>
       </c>
       <c r="E18" s="215" t="s">
-        <v>794</v>
+        <v>799</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="44.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="226" t="s">
-        <v>795</v>
+        <v>800</v>
       </c>
       <c r="B19" s="215" t="s">
-        <v>796</v>
+        <v>801</v>
       </c>
       <c r="C19" s="225" t="s">
-        <v>797</v>
+        <v>802</v>
       </c>
       <c r="D19" s="215" t="s">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="E19" s="215" t="s">
-        <v>798</v>
+        <v>803</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="226" t="s">
-        <v>795</v>
+        <v>800</v>
       </c>
       <c r="B20" s="215" t="s">
-        <v>799</v>
+        <v>804</v>
       </c>
       <c r="C20" s="225" t="s">
-        <v>797</v>
+        <v>802</v>
       </c>
       <c r="D20" s="215" t="s">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="E20" s="215" t="s">
-        <v>800</v>
+        <v>805</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="226" t="s">
-        <v>795</v>
+        <v>800</v>
       </c>
       <c r="B21" s="215" t="s">
-        <v>801</v>
+        <v>806</v>
       </c>
       <c r="C21" s="225" t="s">
-        <v>797</v>
+        <v>802</v>
       </c>
       <c r="D21" s="215" t="s">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="E21" s="215" t="s">
-        <v>802</v>
+        <v>807</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004"/>
     <row r="23" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="229" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="B23" s="215" t="s">
-        <v>803</v>
+        <v>808</v>
       </c>
       <c r="C23" s="228" t="s">
         <v>22</v>
       </c>
       <c r="D23" s="215" t="s">
-        <v>804</v>
+        <v>809</v>
       </c>
       <c r="E23" s="215" t="s">
-        <v>805</v>
+        <v>810</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="230" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B24" s="215" t="s">
-        <v>806</v>
+        <v>811</v>
       </c>
       <c r="C24" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D24" s="215" t="s">
-        <v>807</v>
+        <v>812</v>
       </c>
       <c r="E24" s="215" t="s">
-        <v>808</v>
+        <v>813</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="231" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B25" s="215" t="s">
-        <v>809</v>
+        <v>814</v>
       </c>
       <c r="C25" s="234" t="s">
         <v>22</v>
       </c>
       <c r="D25" s="215" t="s">
-        <v>810</v>
+        <v>815</v>
       </c>
       <c r="E25" s="215" t="s">
-        <v>811</v>
+        <v>816</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="231" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B26" s="215" t="s">
+        <v>817</v>
+      </c>
+      <c r="C26" s="233" t="s">
+        <v>22</v>
+      </c>
+      <c r="D26" s="215" t="s">
         <v>812</v>
       </c>
-      <c r="C26" s="233" t="s">
-        <v>22</v>
-      </c>
-      <c r="D26" s="215" t="s">
-        <v>807</v>
-      </c>
       <c r="E26" s="215" t="s">
-        <v>813</v>
+        <v>818</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="235" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B27" s="215" t="s">
-        <v>814</v>
+        <v>819</v>
       </c>
       <c r="C27" s="237" t="s">
         <v>22</v>
       </c>
       <c r="D27" s="215" t="s">
-        <v>777</v>
+        <v>782</v>
       </c>
       <c r="E27" s="215" t="s">
-        <v>815</v>
+        <v>820</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="227" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="B28" s="215" t="s">
-        <v>816</v>
+        <v>821</v>
       </c>
       <c r="C28" t="s">
         <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>817</v>
+        <v>822</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B29" s="215" t="s">
-        <v>818</v>
+        <v>823</v>
       </c>
       <c r="C29" t="s">
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>777</v>
+        <v>782</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B30" s="215" t="s">
-        <v>819</v>
+        <v>824</v>
       </c>
       <c r="C30" t="s">
         <v>22</v>
       </c>
       <c r="D30" t="s">
-        <v>820</v>
+        <v>825</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B31" s="215" t="s">
-        <v>821</v>
+        <v>826</v>
       </c>
       <c r="C31" t="s">
         <v>22</v>
       </c>
       <c r="D31" t="s">
-        <v>822</v>
+        <v>827</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B32" s="215" t="s">
-        <v>823</v>
+        <v>828</v>
       </c>
       <c r="C32" t="s">
         <v>22</v>
       </c>
       <c r="D32" t="s">
-        <v>824</v>
+        <v>829</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B33" s="215" t="s">
-        <v>825</v>
+        <v>830</v>
       </c>
       <c r="C33" t="s">
         <v>22</v>
       </c>
       <c r="D33" t="s">
-        <v>822</v>
+        <v>827</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B34" s="215" t="s">
-        <v>826</v>
+        <v>831</v>
       </c>
       <c r="C34" t="s">
         <v>22</v>
       </c>
       <c r="D34" t="s">
-        <v>827</v>
+        <v>832</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B35" s="215" t="s">
-        <v>828</v>
+        <v>833</v>
       </c>
       <c r="C35" t="s">
         <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>829</v>
+        <v>834</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B36" s="215" t="s">
-        <v>830</v>
+        <v>835</v>
       </c>
       <c r="C36" t="s">
         <v>22</v>
       </c>
       <c r="D36" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B37" s="215" t="s">
-        <v>832</v>
+        <v>837</v>
       </c>
       <c r="C37" t="s">
         <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
-        <v>789</v>
+        <v>794</v>
       </c>
       <c r="B38" s="215" t="s">
-        <v>833</v>
+        <v>838</v>
       </c>
       <c r="C38" t="s">
         <v>22</v>
       </c>
       <c r="D38" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B39" s="215" t="s">
-        <v>834</v>
+        <v>839</v>
       </c>
       <c r="C39" t="s">
         <v>22</v>
       </c>
       <c r="D39" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B40" s="215" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
       <c r="C40" t="s">
         <v>22</v>
       </c>
       <c r="D40" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B41" s="215" t="s">
-        <v>836</v>
+        <v>841</v>
       </c>
       <c r="C41" t="s">
         <v>22</v>
       </c>
       <c r="D41" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B42" s="215" t="s">
-        <v>838</v>
+        <v>843</v>
       </c>
       <c r="C42" t="s">
         <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B43" s="215" t="s">
-        <v>839</v>
+        <v>844</v>
       </c>
       <c r="C43" t="s">
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="B44" s="215" t="s">
-        <v>841</v>
+        <v>846</v>
       </c>
       <c r="C44" t="s">
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
-        <v>789</v>
+        <v>794</v>
       </c>
       <c r="B45" s="215" t="s">
-        <v>842</v>
+        <v>847</v>
       </c>
       <c r="C45" t="s">
         <v>128</v>
       </c>
       <c r="D45" t="s">
-        <v>843</v>
+        <v>848</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B46" s="215" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
       <c r="C46" t="s">
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>846</v>
+        <v>851</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B47" s="215" t="s">
-        <v>847</v>
+        <v>852</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>848</v>
+        <v>853</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B48" s="215" t="s">
-        <v>849</v>
+        <v>854</v>
       </c>
       <c r="C48" t="s">
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>848</v>
+        <v>853</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B49" s="215" t="s">
-        <v>850</v>
+        <v>855</v>
       </c>
       <c r="C49" t="s">
         <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>848</v>
+        <v>853</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B50" s="215" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="C50" t="s">
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>852</v>
+        <v>857</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B51" s="215" t="s">
-        <v>853</v>
+        <v>858</v>
       </c>
       <c r="C51" t="s">
         <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>854</v>
+        <v>859</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B52" s="215" t="s">
-        <v>855</v>
+        <v>860</v>
       </c>
       <c r="C52" t="s">
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>856</v>
+        <v>861</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B53" s="215" t="s">
-        <v>857</v>
+        <v>862</v>
       </c>
       <c r="C53" t="s">
         <v>128</v>
       </c>
       <c r="D53" t="s">
-        <v>854</v>
+        <v>859</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B54" s="215" t="s">
-        <v>858</v>
+        <v>863</v>
       </c>
       <c r="C54" t="s">
         <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>856</v>
+        <v>861</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B55" s="215" t="s">
-        <v>859</v>
+        <v>864</v>
       </c>
       <c r="C55" t="s">
         <v>22</v>
       </c>
       <c r="D55" t="s">
-        <v>860</v>
+        <v>865</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B56" s="215" t="s">
-        <v>861</v>
+        <v>866</v>
       </c>
       <c r="C56" t="s">
         <v>128</v>
       </c>
       <c r="D56" t="s">
-        <v>862</v>
+        <v>867</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="115.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B57" s="215" t="s">
-        <v>863</v>
+        <v>868</v>
       </c>
       <c r="C57" t="s">
         <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>864</v>
+        <v>869</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B58" s="215" t="s">
-        <v>865</v>
+        <v>870</v>
       </c>
       <c r="C58" t="s">
         <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>864</v>
+        <v>869</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B59" s="215" t="s">
-        <v>866</v>
+        <v>871</v>
       </c>
       <c r="C59" t="s">
         <v>22</v>
       </c>
       <c r="D59" t="s">
-        <v>864</v>
+        <v>869</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B60" s="215" t="s">
-        <v>867</v>
+        <v>872</v>
       </c>
       <c r="C60" t="s">
         <v>128</v>
       </c>
       <c r="D60" t="s">
-        <v>864</v>
+        <v>869</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="274" t="s">
-        <v>868</v>
+        <v>873</v>
       </c>
       <c r="B61" s="215" t="s">
-        <v>869</v>
+        <v>874</v>
       </c>
       <c r="C61" t="s">
         <v>22</v>
       </c>
       <c r="D61" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="274" t="s">
-        <v>868</v>
+        <v>873</v>
       </c>
       <c r="B62" s="215" t="s">
-        <v>870</v>
+        <v>875</v>
       </c>
       <c r="C62" t="s">
         <v>22</v>
       </c>
       <c r="D62" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="274" t="s">
-        <v>868</v>
+        <v>873</v>
       </c>
       <c r="B63" s="215" t="s">
-        <v>871</v>
+        <v>876</v>
       </c>
       <c r="C63" t="s">
         <v>22</v>
       </c>
       <c r="D63" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B64" s="215" t="s">
-        <v>872</v>
+        <v>877</v>
       </c>
       <c r="C64" t="s">
         <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>873</v>
+        <v>878</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B65" s="215" t="s">
-        <v>874</v>
+        <v>879</v>
       </c>
       <c r="C65" t="s">
         <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>873</v>
+        <v>878</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B66" s="215" t="s">
-        <v>875</v>
+        <v>880</v>
       </c>
       <c r="C66" t="s">
         <v>22</v>
       </c>
       <c r="D66" t="s">
-        <v>873</v>
+        <v>878</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="274" t="s">
-        <v>876</v>
+        <v>881</v>
       </c>
       <c r="B67" s="215" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
       <c r="C67" t="s">
         <v>22</v>
       </c>
       <c r="D67" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" s="274" t="s">
-        <v>876</v>
+        <v>881</v>
       </c>
       <c r="B68" s="215" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
       <c r="C68" t="s">
         <v>22</v>
       </c>
       <c r="D68" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
     </row>
     <row r="69" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" s="274" t="s">
-        <v>876</v>
+        <v>881</v>
       </c>
       <c r="B69" s="215" t="s">
-        <v>879</v>
+        <v>884</v>
       </c>
       <c r="C69" t="s">
         <v>22</v>
       </c>
       <c r="D69" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="86.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B70" s="215" t="s">
-        <v>880</v>
+        <v>885</v>
       </c>
       <c r="C70" t="s">
         <v>22</v>
       </c>
       <c r="D70" t="s">
-        <v>881</v>
+        <v>886</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B71" s="215" t="s">
-        <v>882</v>
+        <v>887</v>
       </c>
       <c r="C71" t="s">
         <v>22</v>
       </c>
       <c r="D71" t="s">
-        <v>881</v>
+        <v>886</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B72" s="215" t="s">
-        <v>883</v>
+        <v>888</v>
       </c>
       <c r="C72" t="s">
         <v>22</v>
       </c>
       <c r="D72" t="s">
-        <v>881</v>
+        <v>886</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" s="274" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="B73" s="215" t="s">
-        <v>884</v>
+        <v>889</v>
       </c>
       <c r="C73" t="s">
         <v>128</v>
       </c>
       <c r="D73" t="s">
-        <v>881</v>
+        <v>886</v>
       </c>
     </row>
   </sheetData>
@@ -16846,336 +16923,336 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.3" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="211" t="s">
-        <v>885</v>
+        <v>890</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="212" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="213" t="s">
-        <v>887</v>
+        <v>892</v>
       </c>
       <c r="B4" s="213" t="s">
-        <v>888</v>
+        <v>893</v>
       </c>
       <c r="C4" s="213" t="s">
-        <v>889</v>
+        <v>894</v>
       </c>
       <c r="D4" s="213" t="s">
-        <v>890</v>
+        <v>895</v>
       </c>
       <c r="E4" s="213" t="s">
-        <v>891</v>
+        <v>896</v>
       </c>
       <c r="F4" s="213" t="s">
-        <v>892</v>
+        <v>897</v>
       </c>
       <c r="G4" s="213" t="s">
-        <v>893</v>
+        <v>898</v>
       </c>
       <c r="H4" s="213" t="s">
         <v>4</v>
       </c>
       <c r="I4" s="213" t="s">
-        <v>894</v>
+        <v>899</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="214" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="B5" s="215" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
       <c r="C5" s="215" t="s">
-        <v>897</v>
+        <v>902</v>
       </c>
       <c r="D5" s="215" t="s">
-        <v>898</v>
+        <v>903</v>
       </c>
       <c r="E5" s="215" t="s">
-        <v>899</v>
+        <v>904</v>
       </c>
       <c r="F5" s="215" t="s">
-        <v>900</v>
+        <v>905</v>
       </c>
       <c r="G5" s="215" t="s">
-        <v>901</v>
+        <v>906</v>
       </c>
       <c r="H5" s="216" t="s">
-        <v>902</v>
+        <v>907</v>
       </c>
       <c r="I5" s="215" t="s">
-        <v>903</v>
+        <v>908</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="214" t="s">
-        <v>904</v>
+        <v>909</v>
       </c>
       <c r="B6" s="215" t="s">
-        <v>905</v>
+        <v>910</v>
       </c>
       <c r="C6" s="215" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
       <c r="D6" s="215" t="s">
+        <v>912</v>
+      </c>
+      <c r="E6" s="215" t="s">
+        <v>913</v>
+      </c>
+      <c r="F6" s="215" t="s">
+        <v>914</v>
+      </c>
+      <c r="G6" s="215" t="s">
+        <v>915</v>
+      </c>
+      <c r="H6" s="217" t="s">
         <v>907</v>
       </c>
-      <c r="E6" s="215" t="s">
-        <v>908</v>
-      </c>
-      <c r="F6" s="215" t="s">
-        <v>909</v>
-      </c>
-      <c r="G6" s="215" t="s">
-        <v>910</v>
-      </c>
-      <c r="H6" s="217" t="s">
-        <v>902</v>
-      </c>
       <c r="I6" s="215" t="s">
-        <v>911</v>
+        <v>916</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="214" t="s">
-        <v>912</v>
+        <v>917</v>
       </c>
       <c r="B7" s="215" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="C7" s="215" t="s">
-        <v>914</v>
+        <v>919</v>
       </c>
       <c r="D7" s="215" t="s">
-        <v>915</v>
+        <v>920</v>
       </c>
       <c r="E7" s="215" t="s">
-        <v>916</v>
+        <v>921</v>
       </c>
       <c r="F7" s="215" t="s">
-        <v>917</v>
+        <v>922</v>
       </c>
       <c r="G7" s="215" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
       <c r="H7" s="217" t="s">
-        <v>902</v>
+        <v>907</v>
       </c>
       <c r="I7" s="215" t="s">
-        <v>919</v>
+        <v>924</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="214" t="s">
-        <v>920</v>
+        <v>925</v>
       </c>
       <c r="B8" s="215" t="s">
-        <v>921</v>
+        <v>926</v>
       </c>
       <c r="C8" s="215" t="s">
-        <v>922</v>
+        <v>927</v>
       </c>
       <c r="D8" s="215" t="s">
-        <v>923</v>
+        <v>928</v>
       </c>
       <c r="E8" s="215" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="F8" s="215" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="G8" s="215" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="H8" s="216" t="s">
-        <v>924</v>
+        <v>929</v>
       </c>
       <c r="I8" s="215" t="s">
-        <v>925</v>
+        <v>930</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="214" t="s">
-        <v>926</v>
+        <v>931</v>
       </c>
       <c r="B9" s="215" t="s">
-        <v>927</v>
+        <v>932</v>
       </c>
       <c r="C9" s="215" t="s">
+        <v>933</v>
+      </c>
+      <c r="D9" s="215" t="s">
         <v>928</v>
       </c>
-      <c r="D9" s="215" t="s">
-        <v>923</v>
-      </c>
       <c r="E9" s="215" t="s">
-        <v>916</v>
+        <v>921</v>
       </c>
       <c r="F9" s="215" t="s">
-        <v>929</v>
+        <v>934</v>
       </c>
       <c r="G9" s="215" t="s">
-        <v>930</v>
+        <v>935</v>
       </c>
       <c r="H9" s="218" t="s">
-        <v>931</v>
+        <v>936</v>
       </c>
       <c r="I9" s="215" t="s">
-        <v>932</v>
+        <v>937</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="214" t="s">
-        <v>933</v>
+        <v>938</v>
       </c>
       <c r="B10" s="215" t="s">
-        <v>934</v>
+        <v>939</v>
       </c>
       <c r="C10" s="215" t="s">
-        <v>935</v>
+        <v>940</v>
       </c>
       <c r="D10" s="215" t="s">
-        <v>936</v>
+        <v>941</v>
       </c>
       <c r="E10" s="215" t="s">
-        <v>937</v>
+        <v>942</v>
       </c>
       <c r="F10" s="215" t="s">
-        <v>938</v>
+        <v>943</v>
       </c>
       <c r="G10" s="215" t="s">
-        <v>939</v>
+        <v>944</v>
       </c>
       <c r="H10" s="218" t="s">
-        <v>940</v>
+        <v>945</v>
       </c>
       <c r="I10" s="215" t="s">
-        <v>941</v>
+        <v>946</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="214" t="s">
-        <v>942</v>
+        <v>947</v>
       </c>
       <c r="B11" s="215" t="s">
-        <v>943</v>
+        <v>948</v>
       </c>
       <c r="C11" s="215" t="s">
-        <v>944</v>
+        <v>949</v>
       </c>
       <c r="D11" s="215" t="s">
-        <v>945</v>
+        <v>950</v>
       </c>
       <c r="E11" s="215" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="F11" s="215" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="G11" s="215" t="s">
-        <v>946</v>
+        <v>951</v>
       </c>
       <c r="H11" s="218" t="s">
-        <v>947</v>
+        <v>952</v>
       </c>
       <c r="I11" s="215" t="s">
-        <v>948</v>
+        <v>953</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="214" t="s">
-        <v>949</v>
+        <v>954</v>
       </c>
       <c r="B12" s="215" t="s">
-        <v>950</v>
+        <v>955</v>
       </c>
       <c r="C12" s="215" t="s">
+        <v>956</v>
+      </c>
+      <c r="D12" s="215" t="s">
+        <v>957</v>
+      </c>
+      <c r="E12" s="215" t="s">
+        <v>692</v>
+      </c>
+      <c r="F12" s="215" t="s">
+        <v>692</v>
+      </c>
+      <c r="G12" s="215" t="s">
         <v>951</v>
       </c>
-      <c r="D12" s="215" t="s">
-        <v>952</v>
-      </c>
-      <c r="E12" s="215" t="s">
-        <v>691</v>
-      </c>
-      <c r="F12" s="215" t="s">
-        <v>691</v>
-      </c>
-      <c r="G12" s="215" t="s">
-        <v>946</v>
-      </c>
       <c r="H12" s="217" t="s">
-        <v>953</v>
+        <v>958</v>
       </c>
       <c r="I12" s="215" t="s">
-        <v>954</v>
+        <v>959</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="214" t="s">
-        <v>955</v>
+        <v>960</v>
       </c>
       <c r="B13" s="215" t="s">
-        <v>956</v>
+        <v>961</v>
       </c>
       <c r="C13" s="215" t="s">
-        <v>957</v>
+        <v>962</v>
       </c>
       <c r="D13" s="215" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="E13" s="215" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="F13" s="215" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="G13" s="215" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="H13" s="218" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
       <c r="I13" s="215" t="s">
-        <v>959</v>
+        <v>964</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="214" t="s">
-        <v>960</v>
+        <v>965</v>
       </c>
       <c r="B14" s="215" t="s">
-        <v>961</v>
+        <v>966</v>
       </c>
       <c r="C14" s="215" t="s">
-        <v>957</v>
+        <v>962</v>
       </c>
       <c r="D14" s="215" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="E14" s="215" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="F14" s="215" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="G14" s="215" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="H14" s="218" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
       <c r="I14" s="215" t="s">
-        <v>962</v>
+        <v>967</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="304" t="s">
-        <v>963</v>
+        <v>968</v>
       </c>
       <c r="B16" s="283"/>
       <c r="C16" s="283"/>

</xml_diff>

<commit_message>
docs(tracker): history card verdict and the snapshot coverage risk
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AA50724-AAD4-4015-8FAD-937B962CEA63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D914C86-542C-49C7-A23F-7191F4A8DC26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4979,68 +4979,68 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -13134,846 +13134,897 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="294" t="s">
+      <c r="A1" s="279" t="s">
         <v>498</v>
       </c>
-      <c r="B1" s="283"/>
-      <c r="C1" s="283"/>
-      <c r="D1" s="283"/>
-      <c r="E1" s="283"/>
-      <c r="F1" s="283"/>
-      <c r="G1" s="283"/>
-      <c r="H1" s="283"/>
-      <c r="I1" s="283"/>
-      <c r="J1" s="283"/>
-      <c r="K1" s="283"/>
-      <c r="L1" s="283"/>
-      <c r="M1" s="283"/>
-      <c r="N1" s="283"/>
-      <c r="O1" s="283"/>
-      <c r="P1" s="283"/>
-      <c r="Q1" s="283"/>
-      <c r="R1" s="283"/>
-      <c r="S1" s="283"/>
+      <c r="B1" s="280"/>
+      <c r="C1" s="280"/>
+      <c r="D1" s="280"/>
+      <c r="E1" s="280"/>
+      <c r="F1" s="280"/>
+      <c r="G1" s="280"/>
+      <c r="H1" s="280"/>
+      <c r="I1" s="280"/>
+      <c r="J1" s="280"/>
+      <c r="K1" s="280"/>
+      <c r="L1" s="280"/>
+      <c r="M1" s="280"/>
+      <c r="N1" s="280"/>
+      <c r="O1" s="280"/>
+      <c r="P1" s="280"/>
+      <c r="Q1" s="280"/>
+      <c r="R1" s="280"/>
+      <c r="S1" s="280"/>
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="301" t="s">
+      <c r="A2" s="290" t="s">
         <v>499</v>
       </c>
-      <c r="B2" s="283"/>
-      <c r="C2" s="283"/>
-      <c r="D2" s="283"/>
-      <c r="E2" s="283"/>
-      <c r="F2" s="283"/>
-      <c r="G2" s="283"/>
-      <c r="H2" s="283"/>
-      <c r="I2" s="283"/>
-      <c r="J2" s="283"/>
-      <c r="K2" s="283"/>
-      <c r="L2" s="283"/>
-      <c r="M2" s="283"/>
-      <c r="N2" s="283"/>
-      <c r="O2" s="283"/>
-      <c r="P2" s="283"/>
-      <c r="Q2" s="283"/>
-      <c r="R2" s="283"/>
-      <c r="S2" s="283"/>
+      <c r="B2" s="280"/>
+      <c r="C2" s="280"/>
+      <c r="D2" s="280"/>
+      <c r="E2" s="280"/>
+      <c r="F2" s="280"/>
+      <c r="G2" s="280"/>
+      <c r="H2" s="280"/>
+      <c r="I2" s="280"/>
+      <c r="J2" s="280"/>
+      <c r="K2" s="280"/>
+      <c r="L2" s="280"/>
+      <c r="M2" s="280"/>
+      <c r="N2" s="280"/>
+      <c r="O2" s="280"/>
+      <c r="P2" s="280"/>
+      <c r="Q2" s="280"/>
+      <c r="R2" s="280"/>
+      <c r="S2" s="280"/>
     </row>
     <row r="4" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="289" t="s">
+      <c r="A4" s="287" t="s">
         <v>500</v>
       </c>
-      <c r="B4" s="283"/>
-      <c r="C4" s="283"/>
-      <c r="D4" s="283"/>
-      <c r="E4" s="283"/>
-      <c r="F4" s="283"/>
-      <c r="G4" s="283"/>
-      <c r="H4" s="283"/>
-      <c r="I4" s="283"/>
-      <c r="J4" s="283"/>
-      <c r="K4" s="283"/>
-      <c r="L4" s="283"/>
-      <c r="M4" s="283"/>
-      <c r="N4" s="283"/>
-      <c r="O4" s="283"/>
-      <c r="P4" s="283"/>
-      <c r="Q4" s="283"/>
-      <c r="R4" s="283"/>
-      <c r="S4" s="283"/>
+      <c r="B4" s="280"/>
+      <c r="C4" s="280"/>
+      <c r="D4" s="280"/>
+      <c r="E4" s="280"/>
+      <c r="F4" s="280"/>
+      <c r="G4" s="280"/>
+      <c r="H4" s="280"/>
+      <c r="I4" s="280"/>
+      <c r="J4" s="280"/>
+      <c r="K4" s="280"/>
+      <c r="L4" s="280"/>
+      <c r="M4" s="280"/>
+      <c r="N4" s="280"/>
+      <c r="O4" s="280"/>
+      <c r="P4" s="280"/>
+      <c r="Q4" s="280"/>
+      <c r="R4" s="280"/>
+      <c r="S4" s="280"/>
     </row>
     <row r="5" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="35" t="s">
         <v>501</v>
       </c>
-      <c r="B5" s="279" t="s">
+      <c r="B5" s="288" t="s">
         <v>502</v>
       </c>
-      <c r="C5" s="280"/>
-      <c r="D5" s="281"/>
-      <c r="E5" s="284" t="s">
+      <c r="C5" s="282"/>
+      <c r="D5" s="283"/>
+      <c r="E5" s="289" t="s">
         <v>503</v>
       </c>
-      <c r="F5" s="280"/>
-      <c r="G5" s="281"/>
-      <c r="H5" s="284" t="s">
+      <c r="F5" s="282"/>
+      <c r="G5" s="283"/>
+      <c r="H5" s="289" t="s">
         <v>504</v>
       </c>
-      <c r="I5" s="280"/>
-      <c r="J5" s="281"/>
-      <c r="K5" s="279" t="s">
+      <c r="I5" s="282"/>
+      <c r="J5" s="283"/>
+      <c r="K5" s="288" t="s">
         <v>505</v>
       </c>
-      <c r="L5" s="280"/>
-      <c r="M5" s="281"/>
-      <c r="N5" s="286" t="s">
+      <c r="L5" s="282"/>
+      <c r="M5" s="283"/>
+      <c r="N5" s="301" t="s">
         <v>506</v>
       </c>
-      <c r="O5" s="280"/>
-      <c r="P5" s="281"/>
-      <c r="Q5" s="286" t="s">
+      <c r="O5" s="282"/>
+      <c r="P5" s="283"/>
+      <c r="Q5" s="301" t="s">
         <v>507</v>
       </c>
-      <c r="R5" s="280"/>
-      <c r="S5" s="281"/>
+      <c r="R5" s="282"/>
+      <c r="S5" s="283"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="282" t="s">
+      <c r="B6" s="291" t="s">
         <v>508</v>
       </c>
-      <c r="C6" s="283"/>
-      <c r="D6" s="283"/>
-      <c r="E6" s="283"/>
-      <c r="F6" s="283"/>
-      <c r="G6" s="283"/>
-      <c r="H6" s="283"/>
-      <c r="I6" s="283"/>
-      <c r="J6" s="283"/>
-      <c r="K6" s="283"/>
-      <c r="L6" s="283"/>
-      <c r="M6" s="283"/>
-      <c r="N6" s="283"/>
-      <c r="O6" s="283"/>
-      <c r="P6" s="283"/>
-      <c r="Q6" s="283"/>
-      <c r="R6" s="283"/>
-      <c r="S6" s="283"/>
+      <c r="C6" s="280"/>
+      <c r="D6" s="280"/>
+      <c r="E6" s="280"/>
+      <c r="F6" s="280"/>
+      <c r="G6" s="280"/>
+      <c r="H6" s="280"/>
+      <c r="I6" s="280"/>
+      <c r="J6" s="280"/>
+      <c r="K6" s="280"/>
+      <c r="L6" s="280"/>
+      <c r="M6" s="280"/>
+      <c r="N6" s="280"/>
+      <c r="O6" s="280"/>
+      <c r="P6" s="280"/>
+      <c r="Q6" s="280"/>
+      <c r="R6" s="280"/>
+      <c r="S6" s="280"/>
     </row>
     <row r="7" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="289" t="s">
+      <c r="A7" s="287" t="s">
         <v>509</v>
       </c>
-      <c r="B7" s="283"/>
-      <c r="C7" s="283"/>
-      <c r="D7" s="283"/>
-      <c r="E7" s="283"/>
-      <c r="F7" s="283"/>
-      <c r="G7" s="283"/>
-      <c r="H7" s="283"/>
-      <c r="I7" s="283"/>
-      <c r="J7" s="283"/>
-      <c r="K7" s="283"/>
-      <c r="L7" s="283"/>
-      <c r="M7" s="283"/>
-      <c r="N7" s="283"/>
-      <c r="O7" s="283"/>
-      <c r="P7" s="283"/>
-      <c r="Q7" s="283"/>
-      <c r="R7" s="283"/>
-      <c r="S7" s="283"/>
+      <c r="B7" s="280"/>
+      <c r="C7" s="280"/>
+      <c r="D7" s="280"/>
+      <c r="E7" s="280"/>
+      <c r="F7" s="280"/>
+      <c r="G7" s="280"/>
+      <c r="H7" s="280"/>
+      <c r="I7" s="280"/>
+      <c r="J7" s="280"/>
+      <c r="K7" s="280"/>
+      <c r="L7" s="280"/>
+      <c r="M7" s="280"/>
+      <c r="N7" s="280"/>
+      <c r="O7" s="280"/>
+      <c r="P7" s="280"/>
+      <c r="Q7" s="280"/>
+      <c r="R7" s="280"/>
+      <c r="S7" s="280"/>
     </row>
     <row r="8" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="35" t="s">
         <v>510</v>
       </c>
-      <c r="B8" s="292" t="s">
+      <c r="B8" s="300" t="s">
         <v>511</v>
       </c>
-      <c r="C8" s="280"/>
-      <c r="D8" s="280"/>
-      <c r="E8" s="280"/>
-      <c r="F8" s="280"/>
-      <c r="G8" s="280"/>
-      <c r="H8" s="280"/>
-      <c r="I8" s="280"/>
-      <c r="J8" s="281"/>
-      <c r="K8" s="292" t="s">
+      <c r="C8" s="282"/>
+      <c r="D8" s="282"/>
+      <c r="E8" s="282"/>
+      <c r="F8" s="282"/>
+      <c r="G8" s="282"/>
+      <c r="H8" s="282"/>
+      <c r="I8" s="282"/>
+      <c r="J8" s="283"/>
+      <c r="K8" s="300" t="s">
         <v>512</v>
       </c>
-      <c r="L8" s="280"/>
-      <c r="M8" s="280"/>
-      <c r="N8" s="280"/>
-      <c r="O8" s="280"/>
-      <c r="P8" s="280"/>
-      <c r="Q8" s="280"/>
-      <c r="R8" s="280"/>
-      <c r="S8" s="281"/>
+      <c r="L8" s="282"/>
+      <c r="M8" s="282"/>
+      <c r="N8" s="282"/>
+      <c r="O8" s="282"/>
+      <c r="P8" s="282"/>
+      <c r="Q8" s="282"/>
+      <c r="R8" s="282"/>
+      <c r="S8" s="283"/>
     </row>
     <row r="9" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B9" s="282" t="s">
+      <c r="B9" s="291" t="s">
         <v>508</v>
       </c>
-      <c r="C9" s="283"/>
-      <c r="D9" s="283"/>
-      <c r="E9" s="283"/>
-      <c r="F9" s="283"/>
-      <c r="G9" s="283"/>
-      <c r="H9" s="283"/>
-      <c r="I9" s="283"/>
-      <c r="J9" s="283"/>
-      <c r="K9" s="283"/>
-      <c r="L9" s="283"/>
-      <c r="M9" s="283"/>
-      <c r="N9" s="283"/>
-      <c r="O9" s="283"/>
-      <c r="P9" s="283"/>
-      <c r="Q9" s="283"/>
-      <c r="R9" s="283"/>
-      <c r="S9" s="283"/>
+      <c r="C9" s="280"/>
+      <c r="D9" s="280"/>
+      <c r="E9" s="280"/>
+      <c r="F9" s="280"/>
+      <c r="G9" s="280"/>
+      <c r="H9" s="280"/>
+      <c r="I9" s="280"/>
+      <c r="J9" s="280"/>
+      <c r="K9" s="280"/>
+      <c r="L9" s="280"/>
+      <c r="M9" s="280"/>
+      <c r="N9" s="280"/>
+      <c r="O9" s="280"/>
+      <c r="P9" s="280"/>
+      <c r="Q9" s="280"/>
+      <c r="R9" s="280"/>
+      <c r="S9" s="280"/>
     </row>
     <row r="10" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="289" t="s">
+      <c r="A10" s="287" t="s">
         <v>513</v>
       </c>
-      <c r="B10" s="283"/>
-      <c r="C10" s="283"/>
-      <c r="D10" s="283"/>
-      <c r="E10" s="283"/>
-      <c r="F10" s="283"/>
-      <c r="G10" s="283"/>
-      <c r="H10" s="283"/>
-      <c r="I10" s="283"/>
-      <c r="J10" s="283"/>
-      <c r="K10" s="283"/>
-      <c r="L10" s="283"/>
-      <c r="M10" s="283"/>
-      <c r="N10" s="283"/>
-      <c r="O10" s="283"/>
-      <c r="P10" s="283"/>
-      <c r="Q10" s="283"/>
-      <c r="R10" s="283"/>
-      <c r="S10" s="283"/>
+      <c r="B10" s="280"/>
+      <c r="C10" s="280"/>
+      <c r="D10" s="280"/>
+      <c r="E10" s="280"/>
+      <c r="F10" s="280"/>
+      <c r="G10" s="280"/>
+      <c r="H10" s="280"/>
+      <c r="I10" s="280"/>
+      <c r="J10" s="280"/>
+      <c r="K10" s="280"/>
+      <c r="L10" s="280"/>
+      <c r="M10" s="280"/>
+      <c r="N10" s="280"/>
+      <c r="O10" s="280"/>
+      <c r="P10" s="280"/>
+      <c r="Q10" s="280"/>
+      <c r="R10" s="280"/>
+      <c r="S10" s="280"/>
     </row>
     <row r="11" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="35" t="s">
         <v>514</v>
       </c>
-      <c r="B11" s="279" t="s">
+      <c r="B11" s="288" t="s">
         <v>515</v>
       </c>
-      <c r="C11" s="280"/>
-      <c r="D11" s="281"/>
-      <c r="E11" s="279" t="s">
+      <c r="C11" s="282"/>
+      <c r="D11" s="283"/>
+      <c r="E11" s="288" t="s">
         <v>516</v>
       </c>
-      <c r="F11" s="280"/>
-      <c r="G11" s="281"/>
-      <c r="H11" s="279" t="s">
+      <c r="F11" s="282"/>
+      <c r="G11" s="283"/>
+      <c r="H11" s="288" t="s">
         <v>517</v>
       </c>
-      <c r="I11" s="280"/>
-      <c r="J11" s="281"/>
-      <c r="K11" s="284" t="s">
+      <c r="I11" s="282"/>
+      <c r="J11" s="283"/>
+      <c r="K11" s="289" t="s">
         <v>518</v>
       </c>
-      <c r="L11" s="280"/>
-      <c r="M11" s="281"/>
-      <c r="N11" s="279" t="s">
+      <c r="L11" s="282"/>
+      <c r="M11" s="283"/>
+      <c r="N11" s="288" t="s">
         <v>519</v>
       </c>
-      <c r="O11" s="280"/>
-      <c r="P11" s="281"/>
-      <c r="Q11" s="279" t="s">
+      <c r="O11" s="282"/>
+      <c r="P11" s="283"/>
+      <c r="Q11" s="288" t="s">
         <v>520</v>
       </c>
-      <c r="R11" s="280"/>
-      <c r="S11" s="281"/>
+      <c r="R11" s="282"/>
+      <c r="S11" s="283"/>
     </row>
     <row r="12" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B12" s="282" t="s">
+      <c r="B12" s="291" t="s">
         <v>508</v>
       </c>
-      <c r="C12" s="283"/>
-      <c r="D12" s="283"/>
-      <c r="E12" s="283"/>
-      <c r="F12" s="283"/>
-      <c r="G12" s="283"/>
-      <c r="H12" s="283"/>
-      <c r="I12" s="283"/>
-      <c r="J12" s="283"/>
-      <c r="K12" s="283"/>
-      <c r="L12" s="283"/>
-      <c r="M12" s="283"/>
-      <c r="N12" s="283"/>
-      <c r="O12" s="283"/>
-      <c r="P12" s="283"/>
-      <c r="Q12" s="283"/>
-      <c r="R12" s="283"/>
-      <c r="S12" s="283"/>
+      <c r="C12" s="280"/>
+      <c r="D12" s="280"/>
+      <c r="E12" s="280"/>
+      <c r="F12" s="280"/>
+      <c r="G12" s="280"/>
+      <c r="H12" s="280"/>
+      <c r="I12" s="280"/>
+      <c r="J12" s="280"/>
+      <c r="K12" s="280"/>
+      <c r="L12" s="280"/>
+      <c r="M12" s="280"/>
+      <c r="N12" s="280"/>
+      <c r="O12" s="280"/>
+      <c r="P12" s="280"/>
+      <c r="Q12" s="280"/>
+      <c r="R12" s="280"/>
+      <c r="S12" s="280"/>
     </row>
     <row r="13" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="289" t="s">
+      <c r="A13" s="287" t="s">
         <v>521</v>
       </c>
-      <c r="B13" s="283"/>
-      <c r="C13" s="283"/>
-      <c r="D13" s="283"/>
-      <c r="E13" s="283"/>
-      <c r="F13" s="283"/>
-      <c r="G13" s="283"/>
-      <c r="H13" s="283"/>
-      <c r="I13" s="283"/>
-      <c r="J13" s="283"/>
-      <c r="K13" s="283"/>
-      <c r="L13" s="283"/>
-      <c r="M13" s="283"/>
-      <c r="N13" s="283"/>
-      <c r="O13" s="283"/>
-      <c r="P13" s="283"/>
-      <c r="Q13" s="283"/>
-      <c r="R13" s="283"/>
-      <c r="S13" s="283"/>
+      <c r="B13" s="280"/>
+      <c r="C13" s="280"/>
+      <c r="D13" s="280"/>
+      <c r="E13" s="280"/>
+      <c r="F13" s="280"/>
+      <c r="G13" s="280"/>
+      <c r="H13" s="280"/>
+      <c r="I13" s="280"/>
+      <c r="J13" s="280"/>
+      <c r="K13" s="280"/>
+      <c r="L13" s="280"/>
+      <c r="M13" s="280"/>
+      <c r="N13" s="280"/>
+      <c r="O13" s="280"/>
+      <c r="P13" s="280"/>
+      <c r="Q13" s="280"/>
+      <c r="R13" s="280"/>
+      <c r="S13" s="280"/>
     </row>
     <row r="14" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="35" t="s">
         <v>522</v>
       </c>
-      <c r="B14" s="287" t="s">
+      <c r="B14" s="281" t="s">
         <v>523</v>
       </c>
-      <c r="C14" s="280"/>
-      <c r="D14" s="280"/>
-      <c r="E14" s="280"/>
-      <c r="F14" s="280"/>
-      <c r="G14" s="281"/>
-      <c r="H14" s="287" t="s">
+      <c r="C14" s="282"/>
+      <c r="D14" s="282"/>
+      <c r="E14" s="282"/>
+      <c r="F14" s="282"/>
+      <c r="G14" s="283"/>
+      <c r="H14" s="281" t="s">
         <v>524</v>
       </c>
-      <c r="I14" s="280"/>
-      <c r="J14" s="280"/>
-      <c r="K14" s="280"/>
-      <c r="L14" s="280"/>
-      <c r="M14" s="281"/>
-      <c r="N14" s="287" t="s">
+      <c r="I14" s="282"/>
+      <c r="J14" s="282"/>
+      <c r="K14" s="282"/>
+      <c r="L14" s="282"/>
+      <c r="M14" s="283"/>
+      <c r="N14" s="281" t="s">
         <v>525</v>
       </c>
-      <c r="O14" s="280"/>
-      <c r="P14" s="281"/>
-      <c r="Q14" s="284" t="s">
+      <c r="O14" s="282"/>
+      <c r="P14" s="283"/>
+      <c r="Q14" s="289" t="s">
         <v>526</v>
       </c>
-      <c r="R14" s="280"/>
-      <c r="S14" s="281"/>
+      <c r="R14" s="282"/>
+      <c r="S14" s="283"/>
     </row>
     <row r="15" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B15" s="282" t="s">
+      <c r="B15" s="291" t="s">
         <v>527</v>
       </c>
-      <c r="C15" s="283"/>
-      <c r="D15" s="283"/>
-      <c r="E15" s="283"/>
-      <c r="F15" s="283"/>
-      <c r="G15" s="283"/>
-      <c r="H15" s="283"/>
-      <c r="I15" s="283"/>
-      <c r="J15" s="283"/>
-      <c r="K15" s="283"/>
-      <c r="L15" s="283"/>
-      <c r="M15" s="283"/>
-      <c r="N15" s="283"/>
-      <c r="O15" s="283"/>
-      <c r="P15" s="283"/>
-      <c r="Q15" s="283"/>
-      <c r="R15" s="283"/>
-      <c r="S15" s="283"/>
+      <c r="C15" s="280"/>
+      <c r="D15" s="280"/>
+      <c r="E15" s="280"/>
+      <c r="F15" s="280"/>
+      <c r="G15" s="280"/>
+      <c r="H15" s="280"/>
+      <c r="I15" s="280"/>
+      <c r="J15" s="280"/>
+      <c r="K15" s="280"/>
+      <c r="L15" s="280"/>
+      <c r="M15" s="280"/>
+      <c r="N15" s="280"/>
+      <c r="O15" s="280"/>
+      <c r="P15" s="280"/>
+      <c r="Q15" s="280"/>
+      <c r="R15" s="280"/>
+      <c r="S15" s="280"/>
     </row>
     <row r="16" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="289" t="s">
+      <c r="A16" s="287" t="s">
         <v>528</v>
       </c>
-      <c r="B16" s="283"/>
-      <c r="C16" s="283"/>
-      <c r="D16" s="283"/>
-      <c r="E16" s="283"/>
-      <c r="F16" s="283"/>
-      <c r="G16" s="283"/>
-      <c r="H16" s="283"/>
-      <c r="I16" s="283"/>
-      <c r="J16" s="283"/>
-      <c r="K16" s="283"/>
-      <c r="L16" s="283"/>
-      <c r="M16" s="283"/>
-      <c r="N16" s="283"/>
-      <c r="O16" s="283"/>
-      <c r="P16" s="283"/>
-      <c r="Q16" s="283"/>
-      <c r="R16" s="283"/>
-      <c r="S16" s="283"/>
+      <c r="B16" s="280"/>
+      <c r="C16" s="280"/>
+      <c r="D16" s="280"/>
+      <c r="E16" s="280"/>
+      <c r="F16" s="280"/>
+      <c r="G16" s="280"/>
+      <c r="H16" s="280"/>
+      <c r="I16" s="280"/>
+      <c r="J16" s="280"/>
+      <c r="K16" s="280"/>
+      <c r="L16" s="280"/>
+      <c r="M16" s="280"/>
+      <c r="N16" s="280"/>
+      <c r="O16" s="280"/>
+      <c r="P16" s="280"/>
+      <c r="Q16" s="280"/>
+      <c r="R16" s="280"/>
+      <c r="S16" s="280"/>
     </row>
     <row r="17" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="35" t="s">
         <v>529</v>
       </c>
-      <c r="B17" s="288" t="s">
+      <c r="B17" s="284" t="s">
         <v>530</v>
       </c>
-      <c r="C17" s="280"/>
-      <c r="D17" s="280"/>
-      <c r="E17" s="280"/>
-      <c r="F17" s="280"/>
-      <c r="G17" s="281"/>
-      <c r="H17" s="288" t="s">
+      <c r="C17" s="282"/>
+      <c r="D17" s="282"/>
+      <c r="E17" s="282"/>
+      <c r="F17" s="282"/>
+      <c r="G17" s="283"/>
+      <c r="H17" s="284" t="s">
         <v>531</v>
       </c>
-      <c r="I17" s="280"/>
-      <c r="J17" s="281"/>
-      <c r="K17" s="288" t="s">
+      <c r="I17" s="282"/>
+      <c r="J17" s="283"/>
+      <c r="K17" s="284" t="s">
         <v>532</v>
       </c>
-      <c r="L17" s="280"/>
-      <c r="M17" s="281"/>
-      <c r="N17" s="288" t="s">
+      <c r="L17" s="282"/>
+      <c r="M17" s="283"/>
+      <c r="N17" s="284" t="s">
         <v>533</v>
       </c>
-      <c r="O17" s="280"/>
-      <c r="P17" s="281"/>
-      <c r="Q17" s="288" t="s">
+      <c r="O17" s="282"/>
+      <c r="P17" s="283"/>
+      <c r="Q17" s="284" t="s">
         <v>534</v>
       </c>
-      <c r="R17" s="280"/>
-      <c r="S17" s="281"/>
+      <c r="R17" s="282"/>
+      <c r="S17" s="283"/>
     </row>
     <row r="18" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B18" s="282" t="s">
+      <c r="B18" s="291" t="s">
         <v>508</v>
       </c>
-      <c r="C18" s="283"/>
-      <c r="D18" s="283"/>
-      <c r="E18" s="283"/>
-      <c r="F18" s="283"/>
-      <c r="G18" s="283"/>
-      <c r="H18" s="283"/>
-      <c r="I18" s="283"/>
-      <c r="J18" s="283"/>
-      <c r="K18" s="283"/>
-      <c r="L18" s="283"/>
-      <c r="M18" s="283"/>
-      <c r="N18" s="283"/>
-      <c r="O18" s="283"/>
-      <c r="P18" s="283"/>
-      <c r="Q18" s="283"/>
-      <c r="R18" s="283"/>
-      <c r="S18" s="283"/>
+      <c r="C18" s="280"/>
+      <c r="D18" s="280"/>
+      <c r="E18" s="280"/>
+      <c r="F18" s="280"/>
+      <c r="G18" s="280"/>
+      <c r="H18" s="280"/>
+      <c r="I18" s="280"/>
+      <c r="J18" s="280"/>
+      <c r="K18" s="280"/>
+      <c r="L18" s="280"/>
+      <c r="M18" s="280"/>
+      <c r="N18" s="280"/>
+      <c r="O18" s="280"/>
+      <c r="P18" s="280"/>
+      <c r="Q18" s="280"/>
+      <c r="R18" s="280"/>
+      <c r="S18" s="280"/>
     </row>
     <row r="19" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="289" t="s">
+      <c r="A19" s="287" t="s">
         <v>535</v>
       </c>
-      <c r="B19" s="283"/>
-      <c r="C19" s="283"/>
-      <c r="D19" s="283"/>
-      <c r="E19" s="283"/>
-      <c r="F19" s="283"/>
-      <c r="G19" s="283"/>
-      <c r="H19" s="283"/>
-      <c r="I19" s="283"/>
-      <c r="J19" s="283"/>
-      <c r="K19" s="283"/>
-      <c r="L19" s="283"/>
-      <c r="M19" s="283"/>
-      <c r="N19" s="283"/>
-      <c r="O19" s="283"/>
-      <c r="P19" s="283"/>
-      <c r="Q19" s="283"/>
-      <c r="R19" s="283"/>
-      <c r="S19" s="283"/>
+      <c r="B19" s="280"/>
+      <c r="C19" s="280"/>
+      <c r="D19" s="280"/>
+      <c r="E19" s="280"/>
+      <c r="F19" s="280"/>
+      <c r="G19" s="280"/>
+      <c r="H19" s="280"/>
+      <c r="I19" s="280"/>
+      <c r="J19" s="280"/>
+      <c r="K19" s="280"/>
+      <c r="L19" s="280"/>
+      <c r="M19" s="280"/>
+      <c r="N19" s="280"/>
+      <c r="O19" s="280"/>
+      <c r="P19" s="280"/>
+      <c r="Q19" s="280"/>
+      <c r="R19" s="280"/>
+      <c r="S19" s="280"/>
     </row>
     <row r="20" spans="1:19" ht="46" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="35" t="s">
         <v>536</v>
       </c>
-      <c r="B20" s="290" t="s">
+      <c r="B20" s="286" t="s">
         <v>537</v>
       </c>
-      <c r="C20" s="280"/>
-      <c r="D20" s="280"/>
-      <c r="E20" s="280"/>
-      <c r="F20" s="280"/>
-      <c r="G20" s="281"/>
-      <c r="H20" s="290" t="s">
+      <c r="C20" s="282"/>
+      <c r="D20" s="282"/>
+      <c r="E20" s="282"/>
+      <c r="F20" s="282"/>
+      <c r="G20" s="283"/>
+      <c r="H20" s="286" t="s">
         <v>538</v>
       </c>
-      <c r="I20" s="280"/>
-      <c r="J20" s="280"/>
-      <c r="K20" s="280"/>
-      <c r="L20" s="280"/>
-      <c r="M20" s="281"/>
-      <c r="N20" s="290" t="s">
+      <c r="I20" s="282"/>
+      <c r="J20" s="282"/>
+      <c r="K20" s="282"/>
+      <c r="L20" s="282"/>
+      <c r="M20" s="283"/>
+      <c r="N20" s="286" t="s">
         <v>539</v>
       </c>
-      <c r="O20" s="280"/>
-      <c r="P20" s="280"/>
-      <c r="Q20" s="280"/>
-      <c r="R20" s="280"/>
-      <c r="S20" s="281"/>
+      <c r="O20" s="282"/>
+      <c r="P20" s="282"/>
+      <c r="Q20" s="282"/>
+      <c r="R20" s="282"/>
+      <c r="S20" s="283"/>
     </row>
     <row r="21" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B21" s="282" t="s">
+      <c r="B21" s="291" t="s">
         <v>508</v>
       </c>
-      <c r="C21" s="283"/>
-      <c r="D21" s="283"/>
-      <c r="E21" s="283"/>
-      <c r="F21" s="283"/>
-      <c r="G21" s="283"/>
-      <c r="H21" s="283"/>
-      <c r="I21" s="283"/>
-      <c r="J21" s="283"/>
-      <c r="K21" s="283"/>
-      <c r="L21" s="283"/>
-      <c r="M21" s="283"/>
-      <c r="N21" s="283"/>
-      <c r="O21" s="283"/>
-      <c r="P21" s="283"/>
-      <c r="Q21" s="283"/>
-      <c r="R21" s="283"/>
-      <c r="S21" s="283"/>
+      <c r="C21" s="280"/>
+      <c r="D21" s="280"/>
+      <c r="E21" s="280"/>
+      <c r="F21" s="280"/>
+      <c r="G21" s="280"/>
+      <c r="H21" s="280"/>
+      <c r="I21" s="280"/>
+      <c r="J21" s="280"/>
+      <c r="K21" s="280"/>
+      <c r="L21" s="280"/>
+      <c r="M21" s="280"/>
+      <c r="N21" s="280"/>
+      <c r="O21" s="280"/>
+      <c r="P21" s="280"/>
+      <c r="Q21" s="280"/>
+      <c r="R21" s="280"/>
+      <c r="S21" s="280"/>
     </row>
     <row r="22" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="289" t="s">
+      <c r="A22" s="287" t="s">
         <v>540</v>
       </c>
-      <c r="B22" s="283"/>
-      <c r="C22" s="283"/>
-      <c r="D22" s="283"/>
-      <c r="E22" s="283"/>
-      <c r="F22" s="283"/>
-      <c r="G22" s="283"/>
-      <c r="H22" s="283"/>
-      <c r="I22" s="283"/>
-      <c r="J22" s="283"/>
-      <c r="K22" s="283"/>
-      <c r="L22" s="283"/>
-      <c r="M22" s="283"/>
-      <c r="N22" s="283"/>
-      <c r="O22" s="283"/>
-      <c r="P22" s="283"/>
-      <c r="Q22" s="283"/>
-      <c r="R22" s="283"/>
-      <c r="S22" s="283"/>
+      <c r="B22" s="280"/>
+      <c r="C22" s="280"/>
+      <c r="D22" s="280"/>
+      <c r="E22" s="280"/>
+      <c r="F22" s="280"/>
+      <c r="G22" s="280"/>
+      <c r="H22" s="280"/>
+      <c r="I22" s="280"/>
+      <c r="J22" s="280"/>
+      <c r="K22" s="280"/>
+      <c r="L22" s="280"/>
+      <c r="M22" s="280"/>
+      <c r="N22" s="280"/>
+      <c r="O22" s="280"/>
+      <c r="P22" s="280"/>
+      <c r="Q22" s="280"/>
+      <c r="R22" s="280"/>
+      <c r="S22" s="280"/>
     </row>
     <row r="23" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="35" t="s">
         <v>541</v>
       </c>
-      <c r="B23" s="290" t="s">
+      <c r="B23" s="286" t="s">
         <v>542</v>
       </c>
-      <c r="C23" s="280"/>
-      <c r="D23" s="280"/>
-      <c r="E23" s="280"/>
-      <c r="F23" s="280"/>
-      <c r="G23" s="281"/>
-      <c r="H23" s="290" t="s">
+      <c r="C23" s="282"/>
+      <c r="D23" s="282"/>
+      <c r="E23" s="282"/>
+      <c r="F23" s="282"/>
+      <c r="G23" s="283"/>
+      <c r="H23" s="286" t="s">
         <v>543</v>
       </c>
-      <c r="I23" s="280"/>
-      <c r="J23" s="281"/>
-      <c r="K23" s="290" t="s">
+      <c r="I23" s="282"/>
+      <c r="J23" s="283"/>
+      <c r="K23" s="286" t="s">
         <v>544</v>
       </c>
-      <c r="L23" s="280"/>
-      <c r="M23" s="281"/>
-      <c r="N23" s="290" t="s">
+      <c r="L23" s="282"/>
+      <c r="M23" s="283"/>
+      <c r="N23" s="286" t="s">
         <v>545</v>
       </c>
-      <c r="O23" s="280"/>
-      <c r="P23" s="281"/>
-      <c r="Q23" s="286" t="s">
+      <c r="O23" s="282"/>
+      <c r="P23" s="283"/>
+      <c r="Q23" s="301" t="s">
         <v>546</v>
       </c>
-      <c r="R23" s="280"/>
-      <c r="S23" s="281"/>
+      <c r="R23" s="282"/>
+      <c r="S23" s="283"/>
     </row>
     <row r="26" spans="1:19" ht="20.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="295" t="s">
+      <c r="A26" s="285" t="s">
         <v>547</v>
       </c>
-      <c r="B26" s="283"/>
-      <c r="C26" s="283"/>
-      <c r="D26" s="283"/>
-      <c r="E26" s="283"/>
-      <c r="F26" s="283"/>
-      <c r="G26" s="283"/>
-      <c r="H26" s="283"/>
-      <c r="I26" s="283"/>
-      <c r="J26" s="283"/>
-      <c r="K26" s="283"/>
-      <c r="L26" s="283"/>
-      <c r="M26" s="283"/>
-      <c r="N26" s="283"/>
-      <c r="O26" s="283"/>
-      <c r="P26" s="283"/>
-      <c r="Q26" s="283"/>
-      <c r="R26" s="283"/>
-      <c r="S26" s="283"/>
+      <c r="B26" s="280"/>
+      <c r="C26" s="280"/>
+      <c r="D26" s="280"/>
+      <c r="E26" s="280"/>
+      <c r="F26" s="280"/>
+      <c r="G26" s="280"/>
+      <c r="H26" s="280"/>
+      <c r="I26" s="280"/>
+      <c r="J26" s="280"/>
+      <c r="K26" s="280"/>
+      <c r="L26" s="280"/>
+      <c r="M26" s="280"/>
+      <c r="N26" s="280"/>
+      <c r="O26" s="280"/>
+      <c r="P26" s="280"/>
+      <c r="Q26" s="280"/>
+      <c r="R26" s="280"/>
+      <c r="S26" s="280"/>
     </row>
     <row r="27" spans="1:19" ht="52" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="35" t="s">
         <v>548</v>
       </c>
-      <c r="B27" s="279" t="s">
+      <c r="B27" s="288" t="s">
         <v>549</v>
       </c>
-      <c r="C27" s="280"/>
-      <c r="D27" s="281"/>
-      <c r="E27" s="279" t="s">
+      <c r="C27" s="282"/>
+      <c r="D27" s="283"/>
+      <c r="E27" s="288" t="s">
         <v>550</v>
       </c>
-      <c r="F27" s="280"/>
-      <c r="G27" s="281"/>
-      <c r="H27" s="287" t="s">
+      <c r="F27" s="282"/>
+      <c r="G27" s="283"/>
+      <c r="H27" s="281" t="s">
         <v>551</v>
       </c>
-      <c r="I27" s="280"/>
-      <c r="J27" s="281"/>
-      <c r="K27" s="288" t="s">
+      <c r="I27" s="282"/>
+      <c r="J27" s="283"/>
+      <c r="K27" s="284" t="s">
         <v>552</v>
       </c>
-      <c r="L27" s="280"/>
-      <c r="M27" s="281"/>
-      <c r="N27" s="288" t="s">
+      <c r="L27" s="282"/>
+      <c r="M27" s="283"/>
+      <c r="N27" s="284" t="s">
         <v>553</v>
       </c>
-      <c r="O27" s="280"/>
-      <c r="P27" s="281"/>
-      <c r="Q27" s="28